<commit_message>
Chot hai diem spec §13 truoc khi lam Ban doc sau
(1) Phan tat-ach GIU muc an toan spec dat: nhip nang luong, kieu qua tai,
    vung co the de phan ung o muc XU HUONG. Cam dinh benh, cam noi tho
    yeu, bat buoc co disclaimer y te.
(2) Free mo DUNG MOT phan chuyen sau TU CHON, khong dung phuong an mo dan.
    Nguoi dung chon dung phan ho dang dau thi cam giac 'dung voi toi' manh
    nhat, va ho tu suy ra 11 phan con lai cung sau nhu vay.

Ghi vao PRODUCT-BACKLOG CEL-092 de tang sau khong phai hoi lai.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Backlog'!$A$1:$O$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Logic chi tiết'!$A$1:$G$103</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Nhật ký thay đổi'!$A$1:$F$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Nhật ký thay đổi'!$A$1:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="M93" s="8" t="inlineStr">
         <is>
-          <t>Spec Luận Giải 12 Cung §11 items 10–15. Cần: bảng Supabase `bao_luan_giai` (CHẠY SQL TAY), đổi contract POST /api/luan-giai bỏ Markdown, ba tuyến mới, mười component, và FREE_DEEP_SECTIONS ở entitlements. HAI ĐIỂM SPEC ĐÒI CHỐT TRƯỚC KHI CODE (§13): (1) mức an toàn của phần tat-ach — hiện đặt ở "nhịp năng lượng + xu hướng quá tải", không định bệnh; (2) free mở 1 phần chuyên sâu TỰ CHỌN (~500 từ nội dung đắt nhất) hay chỉ cho xem 3 tiêu chí đầu rồi mờ dần.</t>
+          <t>Spec Luận Giải 12 Cung §11 items 10–15. Cần: bảng Supabase `bao_luan_giai` (CHẠY SQL TAY), đổi contract POST /api/luan-giai bỏ Markdown, ba tuyến mới, mười component, và FREE_DEEP_SECTIONS ở entitlements. HAI ĐIỂM §13 ĐÃ CHỐT ngày 19/09/2026: (1) phần tat-ach GIỮ mức an toàn spec đặt — nhịp năng lượng, kiểu quá tải, vùng cơ thể dễ phản ứng ở mức XU HƯỚNG, cấm định bệnh, bắt buộc có disclaimer y tế; (2) free mở ĐÚNG MỘT phần chuyên sâu TỰ CHỌN, không dùng phương án mờ dần — người dùng chọn đúng phần họ đang đau thì cảm giác "đúng với tôi" mạnh nhất, và họ tự suy ra 11 phần còn lại cũng sâu như vậy.</t>
         </is>
       </c>
       <c r="N93" s="8" t="inlineStr">
@@ -12059,7 +12059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12934,8 +12934,40 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>CEL-092</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Chốt hai điểm spec Luận Giải 12 Cung §13 đòi quyết trước khi code tầng Bản đọc sâu.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án chốt: giữ mức an toàn spec đặt cho phần sức khoẻ, và free mở đúng một phần tự chọn.</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F27"/>
+  <autoFilter ref="A1:F28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
to mau ten sao trong ban doc sau, sua loi rung phan
Ten sao va ten cach cuc duoc to mau o tang hien thi (ChuSao.tsx), chu
khong bang ky hieu Markdown trong chu. Bang 12 phan ve bang the <p> tran
nen dau sao se hien nguyen van truoc mat nguoi doc.

Chi to nhung ten CO THAT tren la so dang doc, do may chu gui kem. Khong
quet bang tu dien sao day du: lam vay thi mot ngoi sao khong co tren la
so cung duoc to dep nhu that, va mau bien thanh loi bao dam cho mot thu
chua duoc kiem.

Kem theo: sua loi bo nghiem thu bao 10/12 phan. Danh sach sao duoc phep
nhac truoc day dung tu goi bang chung, nen nhung cau nhac dung ngoi sao
co tren la so van bi loc. Nay dung tu toan bo la so.

Chay lai bang model that: 12/12 phan, 12/12 co khoi guong, 100% tieu chi
co luc nguoc, 148 giay.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -8328,7 +8328,9 @@
         <is>
           <t>Tầng sâu nhất sản phẩm có. Mười hai phần, mỗi phần 6–7 tiêu chí ở thang L1→L5, khoảng 500–650 từ một phần — tổng gần 7.000 từ.
 Bảng 77 tiêu chí BÓC BẰNG MÁY từ spec mục 4, không chép tay: chép chừng ấy dòng là chắc chắn sai ở đâu đó, và sai ở đây không báo lỗi — nó chỉ làm một phần đời bị luận thiếu một góc mà không ai biết góc nào đã mất.
-KHỐI GƯƠNG là thứ không được bỏ: mỗi phần có đúng một tiêu chí đọc phần này QUA cung đối diện, render đảo màu #2D0334. Đó là cơ chế làm bài không tuyến tính — không phần nào đọc một mình — và là USP spec mục 12 nêu. Thiếu nó thì bản đọc sâu chỉ là bức tranh đầy đủ viết dài ra, mà dài hơn không phải sâu hơn.</t>
+KHỐI GƯƠNG là thứ không được bỏ: mỗi phần có đúng một tiêu chí đọc phần này QUA cung đối diện, render đảo màu #2D0334. Đó là cơ chế làm bài không tuyến tính — không phần nào đọc một mình — và là USP spec mục 12 nêu. Thiếu nó thì bản đọc sâu chỉ là bức tranh đầy đủ viết dài ra, mà dài hơn không phải sâu hơn.
+TÊN SAO ĐƯỢC TÔ MÀU Ở TẦNG HIỂN THỊ, KHÔNG BẰNG KÝ HIỆU TRONG CHỮ. Model viết chữ trơn; ChuSao.tsx nhận danh sách tên CÓ THẬT trên lá số do máy chủ gửi kèm rồi bọc chúng bằng thẻ đậm có màu. Lý do không bảo model viết **Tham Lang**: bảng 12 phần vẽ bằng thẻ &lt;p&gt; trần nên dấu sao hiện nguyên xi — đã trả giá một lần.
+Chỉ tô tên lấy từ chính lá số đang đọc, không quét bằng từ điển sao đầy đủ: quét từ điển thì một ngôi sao KHÔNG có trên lá số cũng được tô đẹp như thật, và màu biến thành lời bảo đảm cho thứ chưa kiểm. Khối gương đảo nền nên dùng màu khác (#F58FD0) — cùng một màu đọc rất khác trên nền tím đậm và trên nền kem.</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -8363,7 +8365,7 @@
       </c>
       <c r="K93" s="8" t="inlineStr">
         <is>
-          <t>lib/tuvi/tieu-chi-sau.ts, lib/rag/ban-doc-sau.ts, app/api/ban-doc-sau/route.ts, app/luan-giai/sau/page.tsx, components/luangiai/{MucDeepSection,KhoiGuong,SoDoBonChang}.tsx, scripts/test-ban-doc-sau.ts</t>
+          <t>lib/tuvi/tieu-chi-sau.ts, lib/rag/ban-doc-sau.ts, app/api/ban-doc-sau/route.ts, app/luan-giai/sau/page.tsx, components/luangiai/{MucDeepSection,KhoiGuong,SoDoBonChang,ChuSao}.tsx, scripts/test-ban-doc-sau.ts</t>
         </is>
       </c>
       <c r="L93" s="8" t="inlineStr">
@@ -8389,7 +8391,7 @@
       </c>
       <c r="O93" s="8" t="inlineStr">
         <is>
-          <t>ban-doc-sau</t>
+          <t>to-mau-ten-sao</t>
         </is>
       </c>
     </row>
@@ -13133,7 +13135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14231,6 +14233,38 @@
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="50" t="inlineStr">
+        <is>
+          <t>to-mau-ten-sao</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>CEL-092</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Tô màu tên sao và tên cách cục trong bản đọc sâu. Sửa lỗi rụng phần: danh sách sao được phép nhắc trước đây dựng từ gói bằng chứng, nay dựng từ TOÀN BỘ lá số.</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án so với một sản phẩm khác và yêu cầu tô màu tên sao. Việc này lộ luôn lỗi thứ hai: bộ nghiệm thu đang báo 10/12 phần dựng được, truy ra là lớp lọc đang gạch những câu nhắc đúng ngôi sao CÓ trên lá số, chỉ vì ngôi sao ấy không nằm trong gói bằng chứng của phần đó. Sau khi nới, chạy lại bằng model thật: 12/12 phần, 12/12 có khối gương, 100% tiêu chí có lực ngược, 148 giây.</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
hien so luot doc sau con lai truoc khi bam
Han muc mot bai moi ngay co tu truoc, nhung nguoi dung chi biet minh da
het khi da bam va bi chan. Chan sau khi bam la dang tu choi te nhat: ho
da quyet dinh doc, da cho trang chuyen, roi moi biet hom nay khong duoc.

luotBaiSauConLai tach han khoi datChoBaiSau du hai ben dem cung mot thu.
Ham kia GHI mot dong truoc khi dem - do la cach no chong mo hai tab -
nen goi no de hien thi thi moi lan mo trang la tieu mat mot luot.

Ham moi chi doc nen KHONG chong duoc dua. Chap nhan duoc: con so o day de
nguoi dung biet minh dang con gi truoc khi bam, con viec chan that van do
datChoBaiSau lam luc bam.

Dem hong thi tra "chua ro" va giao dien hien lai cau tinh cu, KHONG doan
mot con so. Hua "con 1 luot" roi chan o buoc sau te hon han khong hua gi.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -8690,7 +8690,7 @@
       </c>
       <c r="K97" s="8" t="inlineStr">
         <is>
-          <t>lib/support/quota-bai-sau.ts, app/api/luan-giai/route.ts, lib/support/config.ts</t>
+          <t>lib/support/quota-bai-sau.ts, app/api/luan-giai/route.ts, lib/support/config.ts, app/api/luot-bai-sau/route.ts, components/support/LuotBaiSau.tsx</t>
         </is>
       </c>
       <c r="L97" s="8" t="inlineStr">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="M97" s="8" t="inlineStr">
         <is>
-          <t>Chưa có chỗ nào hiện "còn mấy lượt hôm nay" trước khi bấm — người dùng chỉ biết khi đã hết. Số dư supporter trừ bằng update có điều kiện chứ không bằng hàm Postgres, nên nếu sau này có nhiều đường tiêu cùng lúc thì nên chuyển vào SQL.</t>
+          <t>ĐÃ LÀM 20/09/2026 — thẻ CTA trên trang Lá số hiện số lượt còn lại, đọc từ /api/luot-bai-sau. Hàm luotBaiSauConLai tách hẳn khỏi datChoBaiSau dù hai bên đếm cùng một thứ: hàm kia GHI một dòng trước khi đếm (đó là cách nó chống mở hai tab), nên gọi nó để hiển thị thì mỗi lần mở trang là tiêu mất một lượt. Hàm mới chỉ đọc nên không chống được đua — chấp nhận được, vì việc chặn thật vẫn do datChoBaiSau làm lúc bấm. Đếm hỏng thì trả "chưa rõ" và giao diện hiện lại câu tĩnh, KHÔNG đoán một con số: hứa "còn 1 lượt" rồi chặn ở bước sau tệ hơn hẳn không hứa gì. Số dư supporter trừ bằng update có điều kiện chứ không bằng hàm Postgres, nên nếu sau này có nhiều đường tiêu cùng lúc thì nên chuyển vào SQL.</t>
         </is>
       </c>
       <c r="N97" s="8" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="O97" s="8" t="inlineStr">
         <is>
-          <t>han-muc-bai-sau</t>
+          <t>luot-con-lai</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
them net doi song cho 48 phu tinh con lai
Engine bo qua moi sao khong co net viet san. Do la luat dung: dua mot cai
ten khong giai nghia duoc vao prompt la mo duong cho model tu nghi nghia.
Nhung he qua khong ai thay la 48 ngoi sao CO tren la so ma chua bao gio
duoc doc toi - engine khong giau chung, no chua tung doc duoc chung.

Nang nhat la VONG THAI TUE: ca muoi hai sao deu trong, tuc la nen cua
moi cau luan theo NAM chua tung doc duoc - Thai Tue, Tang Mon, Tue Pha,
Bach Ho, Dieu Khach, Quan Phu...

Nay 83/83 phu tinh doc duoc. Ghi chu cu trong backlog noi "khoang 20";
con so that la 48.

Hai bo kiem moi de khong tut lai: moi sao trong tu dien phai co net, va
net khong duoc dung chu truu tuong. Khong co phep dem thi chuyen nay im
lang mai - bai van ra, van dung ngu phap, chi la mong hon muc la so cho
phep.

Bang tieng Anh van 35 net. Thieu net thi engine bo qua nen khong sai,
chi mong hon ban Viet.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -8541,17 +8541,19 @@
       </c>
       <c r="M95" s="8" t="inlineStr">
         <is>
-          <t>Còn khoảng 20 phụ tinh nữa chưa có nét (Bát Tọa, Tam Thai, Thai Phụ, Phong Cáo, Thiên Trù…). Chúng ít ảnh hưởng tới các chủ đề đang hỏi nhiều nhất, nên xếp sau.</t>
+          <t>XONG 20/09/2026 — thêm 48 nét còn lại, nay 83/83 phụ tinh đọc được, và có bộ kiểm chặn việc tụt lại.
+Con số thật là 48 chứ không phải 20 như ghi chú cũ. Nặng nhất là VÒNG THÁI TUẾ: cả mười hai sao đều trống, tức là nền của mọi câu luận theo NĂM chưa từng đọc được — Thái Tuế, Tang Môn, Tuế Phá, Bạch Hổ, Điếu Khách...
+CÒN LẠI: bảng tiếng Anh vẫn 35 nét. Thiếu nét thì engine bỏ qua, nên bản tiếng Anh không sai, chỉ mỏng hơn bản Việt.</t>
         </is>
       </c>
       <c r="N95" s="8" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="O95" s="8" t="inlineStr">
         <is>
-          <t>du-kien-co-ten</t>
+          <t>net-phu-tinh</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
them net doi song tieng Anh cho 48 phu tinh
Khop voi ban tieng Viet cung ngay: 83/83 o ca hai ngon ngu. Them bo kiem
rieng cho bang tieng Anh - mot bang du va mot bang thieu thi hai ngon
ngu cung san pham doc ra hai do day khac nhau, ma khong co phep dem nao
noi ra dieu do.

Nghiem thu ban doc sau sau khi them 48 net tieng Viet: 12/12 phan, moi
phep do xanh.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -8543,7 +8543,7 @@
         <is>
           <t>XONG 20/09/2026 — thêm 48 nét còn lại, nay 83/83 phụ tinh đọc được, và có bộ kiểm chặn việc tụt lại.
 Con số thật là 48 chứ không phải 20 như ghi chú cũ. Nặng nhất là VÒNG THÁI TUẾ: cả mười hai sao đều trống, tức là nền của mọi câu luận theo NĂM chưa từng đọc được — Thái Tuế, Tang Môn, Tuế Phá, Bạch Hổ, Điếu Khách...
-CÒN LẠI: bảng tiếng Anh vẫn 35 nét. Thiếu nét thì engine bỏ qua, nên bản tiếng Anh không sai, chỉ mỏng hơn bản Việt.</t>
+Tiếng Anh cũng đã đủ 83/83 cùng ngày, có bộ kiểm riêng.</t>
         </is>
       </c>
       <c r="N95" s="8" t="inlineStr">
@@ -8553,7 +8553,7 @@
       </c>
       <c r="O95" s="8" t="inlineStr">
         <is>
-          <t>net-phu-tinh</t>
+          <t>net-phu-tinh-en</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bo sung backlog cho CEL-107
Commit truoc (e0bbb76) di ma khong kem backlog: script ghi Excel bao loi
IllegalCharacterError vi chinh cai bay backslash vua sua trong ma cung
lot vao o Excel, nen file khong duoc luu, con lenh commit van chay.

Quy cua du an la backlog cap nhat trong CUNG commit. Lan nay khong giu
duoc vi commit kia da push; ghi ro o day thay vi sua lich su.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O107"/>
+  <dimension ref="A1:O108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9584,6 +9584,87 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="13" t="inlineStr">
+        <is>
+          <t>CEL-107</t>
+        </is>
+      </c>
+      <c r="B108" s="14" t="inlineStr">
+        <is>
+          <t>F. Giao diện &amp; thiết kế</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>Thang khoảng cách sáu bậc</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="inlineStr">
+        <is>
+          <t>Mã dùng 20 giá trị khoảng cách rời nhau: 1 2 3 4 5 6 7 8 10 12 14 16 18 20 22 24 28 32 36 40.
+Mắt không gọi tên được chuyện đó, nhưng cảm nhận được: hai khối lẽ ra cùng một nhịp lại lệch nhau 2px, và cả trang đọc như hơi rung. Không lỗi nào báo, không ai sửa, và mỗi lần thêm màn mới là thêm một giá trị nữa.
+Sáu bậc: 4 dính · 8 sát · 12 thường · 16 rời · 24 khối · 32 chương. Đổi 132 chỗ trong 40 tệp.
+MỆNH BÀN MIỄN TRỪ, và đó là ngoại lệ duy nhất: nó là sơ đồ hình học có tỉ lệ riêng, thu nhỏ theo bề ngang màn, nơi 1-3px là khoảng cách thật sự cần giữa các dòng sao. Thang này dành cho bố cục trang.</t>
+        </is>
+      </c>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>Token --space-1..6 trong globals.css; bộ kiểm quét mã nguồn trong test-chuan-ngon-ngu.ts.</t>
+        </is>
+      </c>
+      <c r="F108" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="inlineStr">
+        <is>
+          <t>Thiết kế (không AI)</t>
+        </is>
+      </c>
+      <c r="H108" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J108" s="8" t="inlineStr">
+        <is>
+          <t>Toàn sản phẩm</t>
+        </is>
+      </c>
+      <c r="K108" s="8" t="inlineStr">
+        <is>
+          <t>app/globals.css, 40 tệp trong app/ và components/, scripts/test-chuan-ngon-ngu.ts</t>
+        </is>
+      </c>
+      <c r="L108" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M108" s="8" t="inlineStr">
+        <is>
+          <t>BỘ KIỂM BAN ĐẦU RỖNG và suýt lọt: biểu thức chính quy bị nuốt mất dấu gạch chéo khi chèn qua shell — ranh giới từ (\b) biến thành ký tự backspace — nên nó không khớp gì và báo xanh cả khi có vi phạm. Phát hiện bằng cách CỐ Ý gây lỗi rồi thấy bộ kiểm vẫn xanh. Sau khi sửa, nó bắt đúng "components/SiteFooter.tsx: gap-[20px]". Đã quét cả kho, không còn tệp nào dính ký tự điều khiển kiểu này.
+Mới quy chuẩn GAP. Padding và margin vẫn còn nhiều giá trị rời nhau, chưa đụng tới.</t>
+        </is>
+      </c>
+      <c r="N108" s="8" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="O108" s="8" t="inlineStr">
+        <is>
+          <t>thang-khoang-cach</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -14006,7 +14087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15336,6 +15417,39 @@
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="B42" s="50" t="inlineStr">
+        <is>
+          <t>thang-khoang-cach</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>CEL-107, CEL-103, CEL-105, CEL-106</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Thang khoảng cách sáu bậc cho toàn bộ bố cục trang. Kèm bộ kiểm quét mã nguồn.</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu tiếp tục theo plan review UIUX; đây là mục cuối của bảng ưu tiên.
+Bài học đáng giữ: bộ kiểm đầu tiên RỖNG và suýt được commit. Chỉ phát hiện vì tôi cố ý gây lỗi để xem nó có đỏ không. Từ nay mọi bộ kiểm mới đều phải qua bước ấy trước khi tin.</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Giao dien luan giai v3: tong quan cho khach, chuyen sau 14 chu de
Chu du an chot 23/09/2026: tong quan mo cho khach, chuyen sau can dang nhap,
khong tru han muc.

/la-so doc tong quan v3 (11 cau). Bang linh vuc cu khong go: no la duong lui,
chi tai khi v3 hong hoac giao dien khong phai tieng Viet (v3 chi viet tieng
Viet). Tai ca hai la ton gap doi luot goi cho cung mot cho.

/luan-giai/sau thanh 14 chu de chuyen sau, moi chu de mot luot goi va chi goi
khi nguoi doc mo toi. Ban doc sau 4 chang (CEL-092) tam dung o giao dien; route
va thu vien giu nguyen.

Route dat han chot 52 giay: do bang trinh duyet that, nhom tong quan 11 cau lan
dau xong o giay 47, sat tran 60 giay cua Vercel. Con duoi 20 giay thi bo vong
sua, giu ban dau.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -8344,7 +8344,7 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Tạm dừng</t>
         </is>
       </c>
       <c r="G93" s="8" t="inlineStr">
@@ -8379,19 +8379,12 @@
       </c>
       <c r="M93" s="8" t="inlineStr">
         <is>
-          <t>CHƯA LÀM, nói rõ để khỏi tưởng đã xong:
-· Chương mở trả lời mối bận tâm của người dùng (spec mục 10.18). CHẶN BỞI ONBOARDING: hiện KHÔNG có chỗ nào hỏi và lưu mối bận tâm, nên chưa có dữ liệu để truyền. Tham số banKhoan từng khai báo sẵn cho việc này đã được GỠ ngày 20/09/2026 — nó chưa bao giờ vào prompt, và một tham số đứng đó mà không làm gì tệ hơn là không có: người đọc mã thấy dungChang({banKhoan}) sẽ tin rằng bài đã đọc mối bận tâm ấy. Làm thật thì phải thêm câu hỏi ở onboarding trước.
-· Ba chương khâu cuối bài: "Hai điều kéo ngược nhau", "Giai đoạn bạn đang đi qua", "Nếu ghép tất cả lại" (spec mục 5 BaiLuanGiai).
-· EvidenceLedger (phụ lục Nhận định · Dữ kiện · Mức) và ReadingProgress.
-· Lưu vị trí đọc dở ("Lần trước bạn dừng ở chặng 3").
-· "Làm mới bài" giữ lịch sử — cần bảng riêng, đệm hiện tại chỉ giữ một bản.
-ĐÃ CHỐT 20/09/2026 — gate "free mở 1 phần tự chọn" của spec mục 13 BỊ BỎ HẲN, không giữ song song. Chỉ còn một luật: 1 bài/ngày, hết thì ủng hộ để mở thêm (CEL-096). Gate cũ chưa từng có trong mã, nên bỏ nó là việc của tài liệu — không có dòng nào phải gỡ.
-ĐÃ SỬA 20/09/2026 — mất câu kết luận không còn làm mất cả phần. Trước đây câu kết luận bị lọc là phần bị vứt luôn: câu "Bạn nên có cộng sự trong việc lớn..." là câu ra lệnh, bị gạt đúng luật, kết luận chỉ có một câu nên gạt xong là rỗng, và sáu tiêu chí đã viết xong ở dưới chết theo. Nay phần vẫn được giữ, giao diện không vẽ thẻ trống. Prompt cũng cấm câu kết luận viết thành lời khuyên.</t>
+          <t>TẠM DỪNG 23/09/2026: /luan-giai/sau chuyển sang luận giải v3 (CEL-119) theo quyết định của chủ dự án bỏ mô hình 4 chặng. Route /api/ban-doc-sau và lib/rag/ban-doc-sau.ts GIỮ NGUYÊN, không còn màn nào gọi.</t>
         </is>
       </c>
       <c r="N93" s="8" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="O93" s="8" t="inlineStr">
@@ -10340,7 +10333,7 @@
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>Chưa phát triển</t>
+          <t>Tạm dừng</t>
         </is>
       </c>
       <c r="G117" s="8" t="inlineStr">
@@ -10375,7 +10368,7 @@
       </c>
       <c r="M117" s="8" t="inlineStr">
         <is>
-          <t>HỎNG NGẪU NHIÊN nên dễ bị bỏ qua: ba lần chạy trong một ngày thì hai lần xanh. Người dùng gặp nó thì thấy bài mất một chặng, không thấy lỗi. Cần đếm tỉ lệ hỏng trước khi chọn hướng sửa — sửa theo hướng 3 mà thật ra chỉ cần hướng 1 là trả giá bằng gấp đôi chi phí model cho mọi lá số.</t>
+          <t>Không còn màn nào gọi bản đọc sâu 4 chặng (xem CEL-092). Bài học trần 60 giây áp vào CEL-119: mỗi câu độc lập + hạn chót trong route.</t>
         </is>
       </c>
       <c r="N117" s="8" t="inlineStr">
@@ -10455,7 +10448,7 @@
       </c>
       <c r="M118" s="8" t="inlineStr">
         <is>
-          <t>KHÔNG TỐN THÊM LƯỢT GỌI MODEL NÀO — đó là điều kiện để mở được: nhánh gọi model chỉ chạy khi deepMap đúng, mà khách thì không. Ai sau này định cho khách thấy bản AI viết thì phải cân lại: mỗi ngày sinh gõ bừa là hai lượt gọi model, và không có tài khoản nào để đặt hạn mức. || ĐÃ KIỂM như một khách thật (Supabase bật, hồ sơ Chrome sạch): tổng quan 200 với 12 phần; bản đọc sâu, bài dài, luận hạn đều 401; mệnh bàn đủ 12 cung ở bốn cỡ màn. || PHÁT HIỆN KÈM: thanh điều hướng tràn 404px trên iPhone cho khách — lỗi sẵn có, nằm im vì mọi lần đo trước đều chạy với Supabase tắt. Đã sửa trong cùng nhánh. || components/laso/KhoiChuyenDoi.tsx giờ không còn chỗ nào dùng; để nguyên, chưa xoá.</t>
+          <t>CẬP NHẬT 23/09/2026: phần tổng quan tiếng Việt giờ là luận giải v3 (CEL-119) và CÓ gọi model cho cả khách — chủ dự án chốt không áp hạn mức. Bảng lĩnh vực ở đây chỉ còn là đường lùi (tiếng Anh, hoặc v3 hỏng).</t>
         </is>
       </c>
       <c r="N118" s="8" t="inlineStr">
@@ -10501,7 +10494,7 @@
       </c>
       <c r="F119" s="9" t="inlineStr">
         <is>
-          <t>Đang phát triển</t>
+          <t>Đang chạy</t>
         </is>
       </c>
       <c r="G119" s="8" t="inlineStr">
@@ -10516,27 +10509,27 @@
       </c>
       <c r="I119" s="8" t="inlineStr">
         <is>
-          <t>Đã đăng nhập (tạm)</t>
+          <t>Tổng quan: khách trở lên · Chuyên sâu: đã đăng nhập · KHÔNG trừ hạn mức (chủ dự án chốt 23/09/2026)</t>
         </is>
       </c>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>/api/luan-giai-v3 (chưa có giao diện)</t>
+          <t>/la-so (khối "Bức tranh chung của lá số"), /luan-giai/sau (14 chủ đề), /api/luan-giai-v3</t>
         </is>
       </c>
       <c r="K119" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/v3/*, app/api/luan-giai-v3/route.ts, scripts/test-luan-giai-v3.ts, scripts/cham-luan-giai-v3.ts</t>
+          <t>lib/rag/v3/*, app/api/luan-giai-v3/route.ts, components/luangiai/TongQuanV3.tsx, components/luangiai/CauTraLoiV3.tsx, app/luan-giai/sau/page.tsx, app/la-so/page.tsx</t>
         </is>
       </c>
       <c r="L119" s="8" t="inlineStr">
         <is>
-          <t>Chưa nối giao diện</t>
+          <t>Giao diện tiếng Việt. Tiếng Anh hoặc v3 hỏng → /la-so tự lùi về bảng lĩnh vực cũ (CEL-118)</t>
         </is>
       </c>
       <c r="M119" s="8" t="inlineStr">
         <is>
-          <t>CHỜ CHỦ DỰ ÁN: (1) hạn mức — route chưa trừ lượt; (2) khách có được đọc tổng quan v3 không (tổng quan v3 gọi model, CEL-118 thì không). Chưa làm: giao diện; chuyên gia duyệt trọng số chấm Mạnh/Bình/Cần gắng; lưu Hồng Loan/Thiên Hỷ theo năm. Điểm đo hiện là luna tự chấm (giám khảo gemini dính 429).</t>
+          <t>Lần đầu một lá số: nhóm tổng quan 11 câu mất ~47s (đo trên máy) — sát trần 60s nên route đặt hạn chót 52s và bỏ vòng sửa khi còn &lt;20s. Khách mở lá số mới là 11+ lượt gọi model (không hạn mức, theo quyết định). Chưa làm: chuyên gia duyệt trọng số chấm Mạnh/Bình/Cần gắng; lưu Hồng Loan/Thiên Hỷ theo năm; bản tiếng Anh. Điểm đo phần lớn do luna tự chấm (gemini 429).</t>
         </is>
       </c>
       <c r="N119" s="8" t="inlineStr">
@@ -10567,7 +10560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G136"/>
+  <dimension ref="A1:G137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15478,6 +15471,43 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="30" t="inlineStr">
+        <is>
+          <t>L16</t>
+        </is>
+      </c>
+      <c r="B137" s="31" t="inlineStr">
+        <is>
+          <t>Luận giải v3 (Tổng quan + Chuyên sâu)</t>
+        </is>
+      </c>
+      <c r="C137" s="31" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện + quyền</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>/la-so: TongQuanV3 gọi nhom=tong-quan (không cần đăng nhập). /luan-giai/sau: 14 chủ đề, mỗi chủ đề một lượt gọi, chỉ gọi khi mở tới. Mỗi câu: bài luận → "Độ rõ" → nút "Muốn biết vì sao không?" (ẩn mặc định). Route đặt hạn chót 52s.</t>
+        </is>
+      </c>
+      <c r="F137" s="32" t="inlineStr">
+        <is>
+          <t>Bảng lĩnh vực cũ chỉ tải khi v3 hỏng hoặc giao diện không phải tiếng Việt — tải cả hai là tốn gấp đôi lượt gọi cho cùng một chỗ. Mọi setState trong callback bất đồng bộ, không trong thân effect (giữ mốc 7 lỗi lint).</t>
+        </is>
+      </c>
+      <c r="G137" s="8" t="inlineStr">
+        <is>
+          <t>components/luangiai/TongQuanV3.tsx, components/luangiai/CauTraLoiV3.tsx, app/luan-giai/sau/page.tsx, app/la-so/page.tsx, app/api/luan-giai-v3/route.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15490,7 +15520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17050,6 +17080,38 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="49" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="B49" s="50" t="inlineStr">
+        <is>
+          <t>luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>CEL-119, CEL-118, CEL-092, CEL-117</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Lên production: sửa truy hồi (hnsw, tìm nguyên cụm, bỏ bản chép, phân cấp nguồn) + luận giải v3 có giao diện. /la-so đọc tổng quan v3 cho cả khách; /luan-giai/sau thành 14 chủ đề chuyên sâu (cần đăng nhập). Không hạn mức.</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án chạy SQL truy hồi, chốt quyền (tổng quan mở cho khách, chuyên sâu cần đăng nhập, không trừ lượt) và yêu cầu gộp main, công khai tất cả phần đã chốt. Đo sau SQL: RAG recall 90%, MRR 0,608 (trước 0,695); luận giải v3 lá A 3,97 → 4,05.</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17062,7 +17124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18775,6 +18837,50 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="51" t="inlineStr">
+        <is>
+          <t>Nghiệm thu RAG</t>
+        </is>
+      </c>
+      <c r="B79" s="51" t="inlineStr">
+        <is>
+          <t>Recall / MRR sau SQL hnsw + tìm cụm (23/09/2026)</t>
+        </is>
+      </c>
+      <c r="C79" s="52" t="inlineStr">
+        <is>
+          <t>90% / 0,608</t>
+        </is>
+      </c>
+      <c r="D79" s="51" t="inlineStr">
+        <is>
+          <t>Recall giữ nguyên, MRR giảm từ 0,695 — đoạn đúng vẫn có nhưng xếp hạng thấp hơn. Bộ vàng chỉ 10 câu; luận giải v3 không tụt (lá A 3,97 → 4,05). Nên mở rộng bộ vàng trước khi chỉnh trọng số cụm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="51" t="inlineStr">
+        <is>
+          <t>Luận giải v3</t>
+        </is>
+      </c>
+      <c r="B80" s="51" t="inlineStr">
+        <is>
+          <t>Thời gian nhóm tổng quan lần đầu</t>
+        </is>
+      </c>
+      <c r="C80" s="52" t="inlineStr">
+        <is>
+          <t>~47 giây (11 câu song song)</t>
+        </is>
+      </c>
+      <c r="D80" s="51" t="inlineStr">
+        <is>
+          <t>Đo 23/09/2026 bằng trình duyệt thật ở máy; đã đệm thì 0,4 giây. Route đặt hạn chót 52s.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Giao dien luan giai v3: ba the dau, tong quan danh so, trang chuyen sau
- /la-so: ba the dau (Diem noi bat / Dieu can luu y / Giai doan hien tai)
  lay tu TQ02/TQ03/TQ08 cua v3; the khuon cu chi con la duong lui khi v3 hong.
  Cau da len the khong lap o danh sach; tong quan thanh the danh so.
- Nut chinh "Doc luan giai chuyen sau" -> /luan-giai/sau; link phu
  "Kham pha tung chu de" -> /luan-giai. Bo dong han muc (LuotBaiSau).
- /luan-giai/sau: tag nam xem noi bat, bo mo ta va nhan "Do ro", muc luc
  moi (so, so cau, da doc x/14, chip cuon ngang tren dien thoai),
  cuoi bai "Doc lai: chu de truoc" + "Doc tiep".
- Backlog: CEL-119, L16 buoc 7, nhat ky.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -10514,12 +10514,12 @@
       </c>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>/la-so (khối "Bức tranh chung của lá số"), /luan-giai/sau (14 chủ đề), /api/luan-giai-v3</t>
+          <t>/la-so (ba thẻ đầu "Điểm nổi bật / Điều cần lưu ý / Giai đoạn hiện tại" + khối "Bức tranh chung của lá số"), /luan-giai/sau (14 chủ đề)</t>
         </is>
       </c>
       <c r="K119" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/v3/*, app/api/luan-giai-v3/route.ts, components/luangiai/TongQuanV3.tsx, components/luangiai/CauTraLoiV3.tsx, app/luan-giai/sau/page.tsx, app/la-so/page.tsx</t>
+          <t>lib/rag/v3/*, app/api/luan-giai-v3/route.ts, components/luangiai/TongQuanV3.tsx, components/luangiai/CauTraLoiV3.tsx, app/luan-giai/sau/page.tsx, app/la-so/page.tsx, components/luangiai/TongQuanV3.tsx (useTongQuanV3, BaTheDauV3), app/luan-giai/sau/page.tsx</t>
         </is>
       </c>
       <c r="L119" s="8" t="inlineStr">
@@ -10529,17 +10529,20 @@
       </c>
       <c r="M119" s="8" t="inlineStr">
         <is>
-          <t>Lần đầu một lá số: nhóm tổng quan 11 câu mất ~47s (đo trên máy) — sát trần 60s nên route đặt hạn chót 52s và bỏ vòng sửa khi còn &lt;20s. Khách mở lá số mới là 11+ lượt gọi model (không hạn mức, theo quyết định). Chưa làm: chuyên gia duyệt trọng số chấm Mạnh/Bình/Cần gắng; lưu Hồng Loan/Thiên Hỷ theo năm; bản tiếng Anh. Điểm đo phần lớn do luna tự chấm (gemini 429).</t>
+          <t>Lần đầu một lá số: nhóm tổng quan 11 câu mất ~47s (đo trên máy) — sát trần 60s nên route đặt hạn chót 52s và bỏ vòng sửa khi còn &lt;20s. Khách mở lá số mới là 11+ lượt gọi model (không hạn mức, theo quyết định). Chưa làm: chuyên gia duyệt trọng số chấm Mạnh/Bình/Cần gắng; lưu Hồng Loan/Thiên Hỷ theo năm; bản tiếng Anh. Điểm đo phần lớn do luna tự chấm (gemini 429).
+CẬP NHẬT 24/09/2026 (giao diện): ba thẻ đầu /la-so lấy từ TQ02/TQ03/TQ08 của v3 (thẻ khuôn cũ chỉ còn là đường lùi khi v3 hỏng); câu đã lên thẻ không lặp ở danh sách; danh sách tổng quan thành thẻ đánh số. Nút chính "Đọc luận giải chuyên sâu" → /luan-giai/sau; link phụ "Khám phá từng chủ đề" → /luan-giai. Bỏ dòng hạn mức (LuotBaiSau) và nhãn "Độ rõ". /luan-giai/sau: tag năm xem nổi bật, bỏ mô tả, mục lục thẻ có số + số câu + "Đã đọc x/14" (điện thoại: chip cuộn ngang), cuối bài "← Đọc lại: chủ đề trước" + "Đọc tiếp".
+CHƯA LÊN PROD (nhánh viec/chong-lap-chuyen-sau): chống lặp ý giữa các câu chuyên sâu + chặn chữ lạ (production có "აღარ" ở TQ02). Chờ OpenAI nạp credit để Celes chạy đo lại — đổi phiên bản prompt/dữ kiện làm mọi bài đệm phải sinh lại.
+SỰ CỐ 24/09/2026: OpenAI báo hết credit — gpt-5.6-luna và embedding RAG đều hỏng; bài chưa đệm sẽ lỗi hoặc lùi về bảng cũ.</t>
         </is>
       </c>
       <c r="N119" s="8" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="O119" s="8" t="inlineStr">
         <is>
-          <t>luan-giai-v3</t>
+          <t>giao-dien-luan-giai-v3</t>
         </is>
       </c>
     </row>
@@ -15494,12 +15497,14 @@
       </c>
       <c r="E137" s="8" t="inlineStr">
         <is>
-          <t>/la-so: TongQuanV3 gọi nhom=tong-quan (không cần đăng nhập). /luan-giai/sau: 14 chủ đề, mỗi chủ đề một lượt gọi, chỉ gọi khi mở tới. Mỗi câu: bài luận → "Độ rõ" → nút "Muốn biết vì sao không?" (ẩn mặc định). Route đặt hạn chót 52s.</t>
+          <t>/la-so: TongQuanV3 gọi nhom=tong-quan (không cần đăng nhập). /luan-giai/sau: 14 chủ đề, mỗi chủ đề một lượt gọi, chỉ gọi khi mở tới. Mỗi câu: bài luận → "Độ rõ" → nút "Muốn biết vì sao không?" (ẩn mặc định). Route đặt hạn chót 52s.
+24/09/2026: useTongQuanV3 tải nhóm tổng quan MỘT lần cho cả trang; BaTheDauV3 dựng ba thẻ đầu từ TQ02/TQ03/TQ08, TongQuanV3 hiện các câu còn lại thành thẻ đánh số. /luan-giai/sau: nút "Đọc lại" chủ đề liền trước, "Đọc tiếp" là nút chính duy nhất.</t>
         </is>
       </c>
       <c r="F137" s="32" t="inlineStr">
         <is>
-          <t>Bảng lĩnh vực cũ chỉ tải khi v3 hỏng hoặc giao diện không phải tiếng Việt — tải cả hai là tốn gấp đôi lượt gọi cho cùng một chỗ. Mọi setState trong callback bất đồng bộ, không trong thân effect (giữ mốc 7 lỗi lint).</t>
+          <t>Bảng lĩnh vực cũ chỉ tải khi v3 hỏng hoặc giao diện không phải tiếng Việt — tải cả hai là tốn gấp đôi lượt gọi cho cùng một chỗ. Mọi setState trong callback bất đồng bộ, không trong thân effect (giữ mốc 7 lỗi lint).
+Dải thẻ đầu chỉ lùi về GocNhinCard khi v3 hỏng cho đúng lá số đang xem — hiện cả hai là lặp nội dung. GocNhinCard còn dùng ở trang chủ và /hanh-trinh, đừng sửa nó cho /la-so.</t>
         </is>
       </c>
       <c r="G137" s="8" t="inlineStr">
@@ -15520,7 +15525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17107,6 +17112,38 @@
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="49" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="50" t="inlineStr">
+        <is>
+          <t>giao-dien-luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>CEL-119</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>/la-so: ba thẻ đầu lấy từ luận giải v3, khối tổng quan thành thẻ đánh số, nút chính dẫn thẳng vào luận giải chuyên sâu, link phụ sang khám phá từng chủ đề, bỏ dòng hạn mức. /luan-giai/sau: tag năm xem nổi bật, bỏ mô tả và nhãn "Độ rõ", mục lục mới, nút "Đọc lại" chủ đề trước.</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án chỉnh sửa 6 điểm giao diện theo ảnh chụp (thẻ khuôn cũ lặp câu, khó nhìn, link sai chỗ).</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Chuyen sau: bat ket bang loi khuyen rieng + do lai sau khi co credit
Luot 8 (sau chong lap): ba cau ket bai khong khuyen gi, giam khao
loiKhuyen 4.00 -> 3.47. Cam loi khuyen chung ma khong bat thay bang loi
khuyen rieng thi model bo luon loi khuyen.

- index: pham vi chuyen sau bat ket bang mot loi khuyen hanh dong cu the.
- prompt: luat 10 noi ro thay loi khuyen chung, khong bo trong (2026.09.5).
- kiem: khong-loi-khuyen (chan) khi doan cuoi khong co chu khuyen nao.
- Backlog: CEL-119, L16 buoc 2/4/5, nhat ky.

Do la so A, 19 cau chuyen sau, Celes chay that (gpt-5.6-luna):
luot 7 -> luot 9: giam khao 4.06 -> 4.15, loiKhuyen 4.00 -> 4.21,
moc tuoi o cau khong hoi thoi diem 7 -> 0, "truoc 30 tuoi" 8 -> 3 cau,
"25-34 tuoi" 10 -> 4 cau. Tong quan 11/11 dat, 48s.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -10531,8 +10531,9 @@
         <is>
           <t>Lần đầu một lá số: nhóm tổng quan 11 câu mất ~47s (đo trên máy) — sát trần 60s nên route đặt hạn chót 52s và bỏ vòng sửa khi còn &lt;20s. Khách mở lá số mới là 11+ lượt gọi model (không hạn mức, theo quyết định). Chưa làm: chuyên gia duyệt trọng số chấm Mạnh/Bình/Cần gắng; lưu Hồng Loan/Thiên Hỷ theo năm; bản tiếng Anh. Điểm đo phần lớn do luna tự chấm (gemini 429).
 CẬP NHẬT 24/09/2026 (giao diện): ba thẻ đầu /la-so lấy từ TQ02/TQ03/TQ08 của v3 (thẻ khuôn cũ chỉ còn là đường lùi khi v3 hỏng); câu đã lên thẻ không lặp ở danh sách; danh sách tổng quan thành thẻ đánh số. Nút chính "Đọc luận giải chuyên sâu" → /luan-giai/sau; link phụ "Khám phá từng chủ đề" → /luan-giai. Bỏ dòng hạn mức (LuotBaiSau) và nhãn "Độ rõ". /luan-giai/sau: tag năm xem nổi bật, bỏ mô tả, mục lục thẻ có số + số câu + "Đã đọc x/14" (điện thoại: chip cuộn ngang), cuối bài "← Đọc lại: chủ đề trước" + "Đọc tiếp".
-CHƯA LÊN PROD (nhánh viec/chong-lap-chuyen-sau): chống lặp ý giữa các câu chuyên sâu + chặn chữ lạ (production có "აღარ" ở TQ02). Chờ OpenAI nạp credit để Celes chạy đo lại — đổi phiên bản prompt/dữ kiện làm mọi bài đệm phải sinh lại.
-SỰ CỐ 24/09/2026: OpenAI báo hết credit — gpt-5.6-luna và embedding RAG đều hỏng; bài chưa đệm sẽ lỗi hoặc lùi về bảng cũ.</t>
+ĐÃ LÊN PROD 24/09/2026 (nhánh viec/chong-lap-chuyen-sau, trước đó chờ credit): chống lặp ý giữa các câu chuyên sâu + chặn chữ lạ (production có "აღარ" ở TQ02). Chờ OpenAI nạp credit để Celes chạy đo lại — đổi phiên bản prompt/dữ kiện làm mọi bài đệm phải sinh lại.
+SỰ CỐ 24/09/2026 (ĐÃ XỬ LÝ — chủ dự án nạp credit): OpenAI báo hết credit — gpt-5.6-luna và embedding RAG đều hỏng; bài chưa đệm sẽ lỗi hoặc lùi về bảng cũ.
+CHỐNG LẶP Ý (24/09/2026): câu không hỏi thời điểm thì dữ kiện không kèm mốc tuổi; mỗi câu chuyên sâu biết các câu cùng chủ đề lo phần nào; bộ kiểm chặn mốc tuổi ở câu không hỏi thời điểm, chặn chữ không phải tiếng Việt, chặn bài chuyên sâu không có lời khuyên ở đoạn cuối. Đo lá số A, 19 câu chuyên sâu: câu gắn mốc tuổi sai chỗ 7 → 0, "trước 30 tuổi" 8 → 3 câu, "25–34 tuổi" 10 → 4 câu; giám khảo 4,06 → 4,15. Đổi phiên bản prompt/dữ kiện → mọi bài đệm sinh lại lần đầu.</t>
         </is>
       </c>
       <c r="N119" s="8" t="inlineStr">
@@ -10542,7 +10543,7 @@
       </c>
       <c r="O119" s="8" t="inlineStr">
         <is>
-          <t>giao-dien-luan-giai-v3</t>
+          <t>chong-lap-chuyen-sau</t>
         </is>
       </c>
     </row>
@@ -15312,12 +15313,14 @@
       </c>
       <c r="E132" s="8" t="inlineStr">
         <is>
-          <t>dungDuKien(): cung chính + xung chiếu + tam hợp + phụ trợ (chỉ chuyên sâu) + sao toàn cục + cách cục trên cung đang đọc + lớp vận (đại vận, chuỗi đại vận, tiểu hạn, lưu tứ hóa tính từ TU_HOA theo can năm, lưu tinh, nguyệt hạn, điểm 12 cung). Mỗi cung kèm nghĩa sao lấy từ KHUON.vi.netPhuTinh / netSao.</t>
+          <t>dungDuKien(): cung chính + xung chiếu + tam hợp + phụ trợ (chỉ chuyên sâu) + sao toàn cục + cách cục trên cung đang đọc + lớp vận (đại vận, chuỗi đại vận, tiểu hạn, lưu tứ hóa tính từ TU_HOA theo can năm, lưu tinh, nguyệt hạn, điểm 12 cung). Mỗi cung kèm nghĩa sao lấy từ KHUON.vi.netPhuTinh / netSao.
+24/09/2026: hoiThoiDiem(q) — câu không hỏi thời điểm thì mô tả cung KHÔNG kèm "đại vận X–Y tuổi" và Tuần/Triệt không kèm mốc tuổi.</t>
         </is>
       </c>
       <c r="F132" s="32" t="inlineStr">
         <is>
-          <t>Cấp NGHĨA SAO do engine giữ — thiếu nó model tự nhớ nghĩa (lượt 5: 135 nhận định không căn cứ / 30 bài). "Nghĩa nền" (manhCau) chỉ cho Mệnh/Thân: gắn vào cung khác thì ra "Tử Vi ở Tài Bạch khiến tiền cần tự quyết".</t>
+          <t>Cấp NGHĨA SAO do engine giữ — thiếu nó model tự nhớ nghĩa (lượt 5: 135 nhận định không căn cứ / 30 bài). "Nghĩa nền" (manhCau) chỉ cho Mệnh/Thân: gắn vào cung khác thì ra "Tử Vi ở Tài Bạch khiến tiền cần tự quyết".
+Mọi cung mang nhãn đại vận làm model gắn mốc tuổi vào cả câu "tôi hợp nghề gì" — cùng một mốc lặp ở bảy câu.</t>
         </is>
       </c>
       <c r="G132" s="8" t="inlineStr">
@@ -15386,12 +15389,14 @@
       </c>
       <c r="E134" s="8" t="inlineStr">
         <is>
-          <t>SYSTEM_V3 = nguyên văn quy tắc viết + hai bài mẫu của chủ dự án + luật căn cứ + luật trình bày. Đầu ra JSON: danY (mỗi ý có mã F/E) → luanGiai → viSao. Tổng quan có PHẠM VI riêng từng câu.</t>
+          <t>SYSTEM_V3 = nguyên văn quy tắc viết + hai bài mẫu của chủ dự án + luật căn cứ + luật trình bày. Đầu ra JSON: danY (mỗi ý có mã F/E) → luanGiai → viSao. Tổng quan có PHẠM VI riêng từng câu.
+24/09/2026: phamViChuyenSau(q) dựng từ khung — liệt kê các câu cùng chủ đề (không lấn sang), cấm tả lại tính cách ngoài chủ đề Tính cách, bắt kết bằng lời khuyên riêng. Luật 10 trong LUAT_CAN_CU: không lặp giữa các câu.</t>
         </is>
       </c>
       <c r="F134" s="32" t="inlineStr">
         <is>
-          <t>Đừng tóm gọn quy tắc của chủ dự án: bản rút gọn trước đó làm bài dài gấp ba mức cho phép. Tổng quan sinh song song nên phải chia phạm vi bằng mã (lượt 2: 5/11 câu cùng kết "đừng làm một mình").</t>
+          <t>Đừng tóm gọn quy tắc của chủ dự án: bản rút gọn trước đó làm bài dài gấp ba mức cho phép. Tổng quan sinh song song nên phải chia phạm vi bằng mã (lượt 2: 5/11 câu cùng kết "đừng làm một mình").
+Cấm lời khuyên chung mà không bắt kết bằng lời khuyên riêng thì model BỎ luôn lời khuyên (lượt 8: ba câu, giám khảo 4 → 1).</t>
         </is>
       </c>
       <c r="G134" s="8" t="inlineStr">
@@ -15423,12 +15428,14 @@
       </c>
       <c r="E135" s="8" t="inlineStr">
         <is>
-          <t>kiemBai(): độ dài (lệch ≤15% chỉ ghi nhận), số đoạn, gạch ý, lộ tên sao/cung/thuật ngữ trong bài luận, từ cấm, mã nội bộ, viết tắt, sao ngoài dữ kiện ở viSao (so CÓ DẤU), mở câu "Bạn" quá nhiều, lặp từ nối. Lỗi chặn → MỘT vòng sửa có chỉ đích; chỉ nhận bản sửa không tệ hơn. Câu an toàn sức khỏe / tài chính do mã chèn.</t>
+          <t>kiemBai(): độ dài (lệch ≤15% chỉ ghi nhận), số đoạn, gạch ý, lộ tên sao/cung/thuật ngữ trong bài luận, từ cấm, mã nội bộ, viết tắt, sao ngoài dữ kiện ở viSao (so CÓ DẤU), mở câu "Bạn" quá nhiều, lặp từ nối. Lỗi chặn → MỘT vòng sửa có chỉ đích; chỉ nhận bản sửa không tệ hơn. Câu an toàn sức khỏe / tài chính do mã chèn.
+24/09/2026: thêm moc-tuoi (chặn), ky-tu-la (chặn), khong-loi-khuyen (chặn, chuyên sâu), khuyen-chung (ghi nhận).</t>
         </is>
       </c>
       <c r="F135" s="32" t="inlineStr">
         <is>
-          <t>So tên sao phải có dấu: bỏ dấu thì "Tử Phủ" trùng "Tử Phù" và bắt oan (lượt 3).</t>
+          <t>So tên sao phải có dấu: bỏ dấu thì "Tử Phủ" trùng "Tử Phù" và bắt oan (lượt 3).
+Production từng hiện "cách làm cũ აღარ còn thuyết phục" (chữ Georgia) — model lẫn ngôn ngữ, phải chặn bằng mã.</t>
         </is>
       </c>
       <c r="G135" s="8" t="inlineStr">
@@ -15525,7 +15532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17144,6 +17151,38 @@
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="49" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B51" s="50" t="inlineStr">
+        <is>
+          <t>chong-lap-chuyen-sau</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>CEL-119</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Chống lặp ý giữa các câu chuyên sâu (bỏ mốc tuổi khỏi dữ kiện câu không hỏi thời điểm, chia phạm vi theo các câu cùng chủ đề, luật 10) + chặn chữ lạ + bắt kết bằng lời khuyên. Giám khảo 4,06 → 4,15; mốc tuổi sai chỗ 7 → 0.</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "hạn chế tình trạng trùng lặp nội dung (1 nội dung được nhắc lại nhiều lần qua nhiều câu hỏi)".</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Sua an sao sau doi chieu tuvivietnam (CEL-121)
- Do sang Thien Khoc/Thien Hu: dac Ty Ngo Mao Dau Mui (truoc nham
  Mao Dau thanh Dan Than; Thien Hu khong co do sang).
- Hoa Ky dac tu mo Thin Tuat Suu Mui (truoc luon Ham).
- Them Luu Tang Mon (Thai Tue +2), Luu Bach Ho (Thai Tue +8), co nghia vi/en.
- PHUONG_PHAP 2026.09.2, dua phien ban phuong phap vao PHIEN_BAN_CHU
  de moi bai dem (ke ca v3) sinh lai theo do sang moi.
- test-ansao: phep kiem hoi quy. Backlog CEL-121.

Khoi/Viet nam Canh GIU (Khoi Ngo, Viet Dan) - cho chu du an chot.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O120"/>
+  <dimension ref="A1:O121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10628,6 +10628,86 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" s="13" t="inlineStr">
+        <is>
+          <t>CEL-121</t>
+        </is>
+      </c>
+      <c r="B121" s="14" t="inlineStr">
+        <is>
+          <t>A. Engine lá số</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>Sửa an sao sau đối chiếu với tuvivietnam.vn: độ sáng Khốc/Hư, Hóa Kỵ, thêm Lưu Tang Môn/Bạch Hổ</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án đối chiếu một lá số với tuvivietnam.vn (24/09/2026). 10/12 cung khớp. Lệch: (1) độ sáng Thiên Khốc sai bảng, Thiên Hư không có độ sáng; (2) Hóa Kỵ luôn Hãm; (3) thiếu Lưu Tang Môn, Lưu Bạch Hổ; (4) Thiên Khôi/Thiên Việt năm Canh đảo nhau — GIỮ, xem cột rủi ro.</t>
+        </is>
+      </c>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t>1. dosang.ts: Khốc/Hư đắc Tý Ngọ Mão Dậu Mùi (trước: Tý Dần Ngọ Thân); Hóa Kỵ đắc tứ mộ Thìn Tuất Sửu Mùi.
+2. ansao.ts luuTinhTheoNam: + Lưu Tang Môn (Thái Tuế +2), Lưu Bạch Hổ (Thái Tuế +8); nghieng-ve.ts có nghĩa vi/en.
+3. PHUONG_PHAP 2026.09.2 và đưa phiên bản phương pháp vào PHIEN_BAN_CHU → mọi bài đệm (kể cả v3) sinh lại theo độ sáng mới.
+4. scripts/test-ansao.ts thêm phép kiểm hồi quy (không dùng ngày sinh thật).</t>
+        </is>
+      </c>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G121" s="8" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="H121" s="8" t="inlineStr">
+        <is>
+          <t>Tính lại mỗi lần lập</t>
+        </is>
+      </c>
+      <c r="I121" s="8" t="inlineStr">
+        <is>
+          <t>Khách trở lên</t>
+        </is>
+      </c>
+      <c r="J121" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, mọi màn luận giải</t>
+        </is>
+      </c>
+      <c r="K121" s="8" t="inlineStr">
+        <is>
+          <t>lib/tuvi/dosang.ts, lib/tuvi/ansao.ts, lib/tuvi/phuong-phap.ts, lib/rag/phien-ban-chu.ts, lib/rag/nghieng-ve.ts</t>
+        </is>
+      </c>
+      <c r="L121" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="M121" s="8" t="inlineStr">
+        <is>
+          <t>KHÔI/VIỆT: engine dùng Canh/Tân → Khôi Ngọ, Việt Dần (constants.ts, "Nam phái"; tracuutuvi và đa số nguồn tra được cùng bảng này). tuvivietnam.vn đảo lại (Khôi Dần, Việt Ngọ) — hai cách đọc câu "Canh Tân phùng Mã Hổ". Chưa đổi, chờ chủ dự án chốt trường phái. Chưa làm: hiện độ sáng cho Tứ Hóa/Lộc Tồn như tuvivietnam (Lộc B, Quyền V…) — quy ước riêng của trang đó. Đổi phương pháp → lần mở đầu mọi lá số phải sinh lại bài.</t>
+        </is>
+      </c>
+      <c r="N121" s="8" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="O121" s="8" t="inlineStr">
+        <is>
+          <t>sua-an-sao</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15724,7 +15804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17407,6 +17487,38 @@
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="49" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B53" s="50" t="inlineStr">
+        <is>
+          <t>sua-an-sao</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>CEL-121</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Sửa độ sáng Thiên Khốc/Thiên Hư (nhầm Mão Dậu thành Dần Thân, Hư không có độ sáng), Hóa Kỵ đắc tứ mộ, thêm Lưu Tang Môn/Bạch Hổ; phiên bản phương pháp vào khoá đệm.</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án đối chiếu lá số với tuvivietnam.vn và thấy vài sao lệch.</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Luan giai la so chi sinh mot lan moi la so + nam + nhom (CEL-122)
Khoa dem cu gan phien ban cua moi thu (prompt, du kien, RAG, chuan ngon
ngu, planner, validator, phuong phap) -> moi lan deploy la moi la so sinh
lai. Do trong bang: cung la so, chu de Tinh cach sinh 3 lan trong 8 tieng.

- Khoa = nam|nhom (+THE_HE_DEM khi muon lam moi toan bo bang tay).
- Khong thay khoa moi -> dung lai ban moi nhat duoi khoa kieu cu va chuyen
  sang khoa moi (docNoiDungMoiNhat).
- Cau chua viet duoc thi chi sinh dung cau do roi ghep vao.
- luuNoiDung ghi log khi upsert loi (truoc bi nuot im lang).
- DangDocV3: chi noi "lan dau mat khoang nua phut" khi cho qua 3 giay.
- test-chuan-ngon-ngu: ngoai le co khai bao cho khoa v3. Backlog CEL-122.

Do tren may noi DB that: la so da co bai 0.26s khong goi model; la so moi
lan dau 37s, cac lan sau 0.12-0.14s.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O121"/>
+  <dimension ref="A1:O122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10708,6 +10708,87 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="13" t="inlineStr">
+        <is>
+          <t>CEL-122</t>
+        </is>
+      </c>
+      <c r="B122" s="14" t="inlineStr">
+        <is>
+          <t>D. Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>Luận giải lá số (tổng quan + chuyên sâu) chỉ sinh MỘT lần mỗi lá số + năm + nhóm</t>
+        </is>
+      </c>
+      <c r="D122" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án (24/09/2026): lá số đã xem chuyên sâu mà lần sau vào vẫn sinh lại. Soi bảng noi_dung_ai: ghi đệm vẫn chạy, nhưng khoá gắn phiên bản của mọi thứ (prompt, dữ kiện, RAG, chuẩn ngôn ngữ, planner, validator, phương pháp) nên mỗi lần deploy là mọi lá số sinh lại — cùng lá số, chủ đề Tính cách sinh 3 lần trong 8 tiếng.</t>
+        </is>
+      </c>
+      <c r="E122" s="8" t="inlineStr">
+        <is>
+          <t>1. /api/luan-giai-v3: khoá = nam:&lt;năm&gt;|nhom:&lt;nhóm&gt; (+|th:&lt;THE_HE_DEM&gt; khi &gt;1). Không còn phiên bản trong khoá.
+2. Không thấy khoá mới → đọc bản MỚI NHẤT dưới khoá kiểu cũ (…|s:…) bằng docNoiDungMoiNhat và chuyển sang khoá mới — không ai phải sinh lại thêm lần nào.
+3. Câu nào lần trước chưa viết được thì chỉ sinh đúng câu đó rồi ghép vào.
+4. luuNoiDung ghi log khi upsert lỗi (trước: bị nuốt im lặng).
+5. Giao diện: DangDocV3 — "Celes đang mở bài", chỉ nói "lần đầu mất khoảng nửa phút" khi chờ quá 3 giây.</t>
+        </is>
+      </c>
+      <c r="F122" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G122" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H122" s="8" t="inlineStr">
+        <is>
+          <t>Một lần mỗi lá số + năm xem + nhóm</t>
+        </is>
+      </c>
+      <c r="I122" s="8" t="inlineStr">
+        <is>
+          <t>Tổng quan: khách · Chuyên sâu: đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="J122" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, /luan-giai/sau, /api/luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="K122" s="8" t="inlineStr">
+        <is>
+          <t>app/api/luan-giai-v3/route.ts, lib/rag/noi-dung-ai.ts, components/luangiai/CauTraLoiV3.tsx</t>
+        </is>
+      </c>
+      <c r="L122" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M122" s="8" t="inlineStr">
+        <is>
+          <t>Đo trên máy nối DB thật: lá số đã có bài → 0,26s không gọi model; lá số mới → lần đầu 37s, các lần sau 0,12–0,14s. Đánh đổi: sửa prompt/an sao KHÔNG còn tự làm mới bài cũ — lá số đã có bài giữ bài đó (kể cả bài sinh trước khi sửa độ sáng Khốc/Hư/Hóa Kỵ, CEL-121). Muốn làm mới toàn bộ thì tăng THE_HE_DEM trong route. Các bề mặt khác (hành trình, điểm nổi bật, bảng lĩnh vực) vẫn khoá theo kyCoPhienBan.</t>
+        </is>
+      </c>
+      <c r="N122" s="8" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="O122" s="8" t="inlineStr">
+        <is>
+          <t>dem-mot-lan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15804,7 +15885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17519,6 +17600,38 @@
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="49" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B54" s="50" t="inlineStr">
+        <is>
+          <t>dem-mot-lan</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>CEL-122</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Luận giải lá số sinh một lần mỗi lá số + năm + nhóm: bỏ phiên bản khỏi khoá, dùng lại bài dưới khoá cũ, chỉ sinh câu còn thiếu, ghi log khi cất lỗi, chữ chờ không còn nói "lần đầu" khi đọc từ đệm.</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "1 lá số đã xem... các lần sau vào vẫn gen lại =&gt; sửa mỗi lá chỉ gen 1 lần và lưu lại".</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Backlog: dot toi uu 3 (CEL-124, CEL-125), don muc loi thoi
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O123"/>
+  <dimension ref="A1:O125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1632,12 +1632,13 @@
       </c>
       <c r="M7" s="8" t="inlineStr">
         <is>
-          <t>Hàng chọn chế độ đã gỡ theo yêu cầu (c36b43a). Mã ba chế độ vẫn còn — quyết định xem giữ hay xoá hẳn.</t>
+          <t>Hàng chọn chế độ đã gỡ theo yêu cầu (c36b43a). Mã ba chế độ vẫn còn — quyết định xem giữ hay xoá hẳn.
+Cần chủ dự án quyết: xoá hẳn mã ba chế độ (không còn nút chọn) hay giữ.</t>
         </is>
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
@@ -6078,7 +6079,7 @@
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Đang chạy</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
@@ -6113,17 +6114,18 @@
       </c>
       <c r="M64" s="8" t="inlineStr">
         <is>
-          <t>CHƯA nối dịch vụ analytics nào. Khi chọn được nhà cung cấp chỉ sửa hàm ghiSuKien, không phải rải lại khắp app — xem CEL-082.</t>
+          <t>CHƯA nối dịch vụ analytics nào. Khi chọn được nhà cung cấp chỉ sửa hàm ghiSuKien, không phải rải lại khắp app — xem CEL-082.
+XONG (25/09/2026): sự kiện gửi về /api/su-kien → bảng su_kien (không dịch vụ ngoài), phễu ở trang quản trị. CẦN CHẠY supabase/va-su-kien.sql.</t>
         </is>
       </c>
       <c r="N64" s="8" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="O64" s="8" t="inlineStr">
         <is>
-          <t>a04efc7</t>
+          <t>toi-uu-dot-3</t>
         </is>
       </c>
     </row>
@@ -6619,7 +6621,7 @@
       </c>
       <c r="F71" s="28" t="inlineStr">
         <is>
-          <t>Chưa phát triển</t>
+          <t>Đang chạy</t>
         </is>
       </c>
       <c r="G71" s="8" t="inlineStr">
@@ -6654,12 +6656,13 @@
       </c>
       <c r="M71" s="8" t="inlineStr">
         <is>
-          <t>Việc này do rà soát ngày 19/09 phát hiện, chưa nằm trong roadmap gốc. Ưu tiên cao: hiện mỗi lần đổi prompt phải nhớ chạy tay scripts/chay-lai-luan-giai.ts, quên là người dùng đọc bài cũ suốt kỳ.</t>
+          <t>Việc này do rà soát ngày 19/09 phát hiện, chưa nằm trong roadmap gốc. Ưu tiên cao: hiện mỗi lần đổi prompt phải nhớ chạy tay scripts/chay-lai-luan-giai.ts, quên là người dùng đọc bài cũ suốt kỳ.
+XONG (25/09/2026): mọi bề mặt khoá đệm theo PHIEN_BAN_CHU (băm bộ luật + phương pháp an sao); riêng luận giải lá số v3 CỐ Ý sinh một lần (CEL-122, THE_HE_DEM).</t>
         </is>
       </c>
       <c r="N71" s="8" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="O71" s="8" t="inlineStr">
@@ -6773,7 +6776,7 @@
       </c>
       <c r="F73" s="28" t="inlineStr">
         <is>
-          <t>Chưa phát triển</t>
+          <t>Đang chạy</t>
         </is>
       </c>
       <c r="G73" s="8" t="inlineStr">
@@ -6808,17 +6811,18 @@
       </c>
       <c r="M73" s="8" t="inlineStr">
         <is>
-          <t>Là một trong ba việc lớn nhất còn lại.</t>
+          <t>Là một trong ba việc lớn nhất còn lại.
+XONG (25/09/2026): màn hẹp có "Danh sách 12 cung" (components/laso/DanhSachCung.tsx) bên cạnh lưới — chữ nhỏ nhất 12px thay vì ~9px, đủ sao, chạm mở ngăn chi tiết, nhớ lựa chọn.</t>
         </is>
       </c>
       <c r="N73" s="8" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="O73" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>toi-uu-dot-3</t>
         </is>
       </c>
     </row>
@@ -7543,7 +7547,7 @@
       </c>
       <c r="F83" s="28" t="inlineStr">
         <is>
-          <t>Chưa phát triển</t>
+          <t>Đang chạy</t>
         </is>
       </c>
       <c r="G83" s="8" t="inlineStr">
@@ -7578,17 +7582,18 @@
       </c>
       <c r="M83" s="8" t="inlineStr">
         <is>
-          <t>Chỉ phải sửa hàm ghiSuKien, các điểm gọi đã rải sẵn khắp app. Liên quan CEL-063.</t>
+          <t>Chỉ phải sửa hàm ghiSuKien, các điểm gọi đã rải sẵn khắp app. Liên quan CEL-063.
+Làm theo hướng TỰ GHI VÀO DB thay cho GA4/Plausible/PostHog (ngân sách 0, chưa chốt nhà cung cấp) — xem CEL-063. Chọn được nhà cung cấp thì chỉ sửa ghiSuKien.</t>
         </is>
       </c>
       <c r="N83" s="8" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="O83" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>toi-uu-dot-3</t>
         </is>
       </c>
     </row>
@@ -10872,6 +10877,166 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" s="13" t="inlineStr">
+        <is>
+          <t>CEL-124</t>
+        </is>
+      </c>
+      <c r="B124" s="14" t="inlineStr">
+        <is>
+          <t>D. Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="inlineStr">
+        <is>
+          <t>Cảnh báo sự cố AI: ghi lý do, cron sức khoẻ hằng ngày, webhook tuỳ chọn</t>
+        </is>
+      </c>
+      <c r="D124" s="8" t="inlineStr">
+        <is>
+          <t>24/09/2026 OpenAI hết credit, model viết và embedding cùng hỏng mà không ai được báo; ai_usage_logs không giữ lý do.</t>
+        </is>
+      </c>
+      <c r="E124" s="8" t="inlineStr">
+        <is>
+          <t>1. lib/ai/su-co.ts: ghi sự cố kèm loại (quota/auth = nặng → webhook; rate-limit/server/network = nhẹ), giãn cách 1 giờ / 10 phút.
+2. Nối vào goiVoiFallback và embedding của RAG; 429 insufficient_quota của embedding nay là "hết credit".
+3. /api/cron/suc-khoe-ai 01:00 hằng ngày: gọi thử từng model + embedding.
+4. Trang quản trị: dải cảnh báo 24 giờ (SuCoAi).</t>
+        </is>
+      </c>
+      <c r="F124" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G124" s="8" t="inlineStr">
+        <is>
+          <t>Luật cứng</t>
+        </is>
+      </c>
+      <c r="H124" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi ngày + theo sự kiện</t>
+        </is>
+      </c>
+      <c r="I124" s="8" t="inlineStr">
+        <is>
+          <t>Quản trị</t>
+        </is>
+      </c>
+      <c r="J124" s="8" t="inlineStr">
+        <is>
+          <t>/admin, /api/cron/suc-khoe-ai, /api/admin/su-co</t>
+        </is>
+      </c>
+      <c r="K124" s="8" t="inlineStr">
+        <is>
+          <t>lib/ai/su-co.ts, lib/ai/fallback.ts, lib/ai/embedding.ts, lib/rag/truy-hoi.ts, app/api/cron/suc-khoe-ai, components/admin/SuCoAi.tsx</t>
+        </is>
+      </c>
+      <c r="L124" s="8" t="inlineStr">
+        <is>
+          <t>Cần chạy supabase/va-su-co-ai.sql; webhook: CANH_BAO_WEBHOOK_URL</t>
+        </is>
+      </c>
+      <c r="M124" s="8" t="inlineStr">
+        <is>
+          <t>Chạy thử 25/09/2026 bắt được Cerebras "Payment required" — model chết trong chuỗi dự phòng từ trước. Groq báo nhầm khi maxTokens 16 (model suy luận) → cron dùng 256.</t>
+        </is>
+      </c>
+      <c r="N124" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O124" s="8" t="inlineStr">
+        <is>
+          <t>toi-uu-dot-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="13" t="inlineStr">
+        <is>
+          <t>CEL-125</t>
+        </is>
+      </c>
+      <c r="B125" s="14" t="inlineStr">
+        <is>
+          <t>D. Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t>Tốc độ: tổng quan ba thẻ đầu trước + tăng tốc nhánh từ khoá RAG</t>
+        </is>
+      </c>
+      <c r="D125" s="8" t="inlineStr">
+        <is>
+          <t>Tổng quan lần đầu 35–48 giây; một truy vấn RAG 2,7–4,3 giây, nhánh từ khoá không chạy song song được (15 truy vấn = 15 giây).</t>
+        </is>
+      </c>
+      <c r="E125" s="8" t="inlineStr">
+        <is>
+          <t>1. /api/luan-giai-v3 nhận `chi` (chỉ lấy/chỉ sinh một phần nhóm) và đọc lại bản mới nhất trước khi ghi.
+2. useTongQuanV3: lượt 1 ba thẻ đầu, lượt 2 tám câu còn lại, NỐI TIẾP.
+3. supabase/va-rag-toc-do.sql: cột tsv tính sẵn + GIN; tim_kien_thuc_tu_khoa_cum dùng c.tsv.
+4. truy-hoi-v3: đệm truy hồi dùng chung giữa request (30 phút).</t>
+        </is>
+      </c>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G125" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H125" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I125" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J125" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, /api/luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="K125" s="8" t="inlineStr">
+        <is>
+          <t>app/api/luan-giai-v3/route.ts, components/luangiai/TongQuanV3.tsx, lib/rag/v3/truy-hoi-v3.ts, supabase/va-rag-toc-do.sql</t>
+        </is>
+      </c>
+      <c r="L125" s="8" t="inlineStr">
+        <is>
+          <t>Cần chạy supabase/va-rag-toc-do.sql để có phần tăng tốc RAG</t>
+        </is>
+      </c>
+      <c r="M125" s="8" t="inlineStr">
+        <is>
+          <t>Đo trên lá số chưa có bài: ba thẻ đầu 33–37s → ~20s; cả trang ~37s → ~50s (danh sách nằm dưới, nạp sau). Song song hai lượt chậm hơn (33s) vì tranh nhau ở nhánh từ khoá — chạy SQL xong nên đo lại, có thể chuyển về song song.</t>
+        </is>
+      </c>
+      <c r="N125" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O125" s="8" t="inlineStr">
+        <is>
+          <t>toi-uu-dot-3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15968,7 +16133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17747,6 +17912,38 @@
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B56" s="50" t="inlineStr">
+        <is>
+          <t>toi-uu-dot-3</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>CEL-124, CEL-125, CEL-063, CEL-082, CEL-072, CEL-070</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Cảnh báo sự cố AI + cron sức khoẻ; phễu sự kiện tự ghi DB; tổng quan ba thẻ đầu hiện trước; tăng tốc RAG (SQL + đệm); Kết nối có lớp sửa tiếng lóng; mệnh bàn mobile dạng danh sách; Hỏi Celes dùng lá số vừa lập; dọn backlog lỗi thời.</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "làm các phần đang dang dở và cần tối ưu" sau buổi review toàn bộ tính năng.</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Ban do manh - yeu 12 mat doi o /la-so va ap ban C (luan sau hon)
- du-kien: chiTietDiemTungCung (sao do/keo trong cung + cung soi vao), hung tinh dac dia chi tru nua
- BanDoManhYeu: The manh / Binh / Can gang, thanh do manh chay khi cuon toi, mo "vi sao", loi sang doc sau dung chu de
- /luan-giai/sau nhan ?chuDe, chip muc luc tu cuon toi
- TQ04 lam tom tat trong ban do, bo khoi danh sach tong quan
- prompt v3: khoi LUAN_SAU, do dai tong quan 60-140, chuyen sau 180-360 (thu nghiem mu: C thang 11/18)
- Backlog: CEL-126, CEL-127

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O125"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11037,6 +11037,166 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="13" t="inlineStr">
+        <is>
+          <t>CEL-126</t>
+        </is>
+      </c>
+      <c r="B126" s="14" t="inlineStr">
+        <is>
+          <t>B. Luận giải AI</t>
+        </is>
+      </c>
+      <c r="C126" s="8" t="inlineStr">
+        <is>
+          <t>Luận sâu hơn ("bản C"): biểu hiện + tình huống + điều kiện, độ dài ~1,3 lần</t>
+        </is>
+      </c>
+      <c r="D126" s="8" t="inlineStr">
+        <is>
+          <t>Góp ý "Celes trung dung". Thử nghiệm mù 3 lá số × 6 câu (scripts/thu-nghiem-do-ro.ts): C thắng 11/18, rõ ràng 4,83 vs 4,28; đổi luật cho "thẳng thắn" (B) không thắng lần nào, ghép với C (D) làm bám căn cứ tụt 4,83 → 4,50.</t>
+        </is>
+      </c>
+      <c r="E126" s="8" t="inlineStr">
+        <is>
+          <t>1. prompt-v3: khối LUAN_SAU vào khoiDoDai cho cả tổng quan và chuyên sâu.
+2. DO_DAI_V3: tổng quan 60–140 từ, chuyên sâu 180–360 từ (TỔNG ~230–300).
+3. Quy tắc viết của chủ dự án KHÔNG đổi.</t>
+        </is>
+      </c>
+      <c r="F126" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G126" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H126" s="8" t="inlineStr">
+        <is>
+          <t>Một lần mỗi lá số + năm + nhóm</t>
+        </is>
+      </c>
+      <c r="I126" s="8" t="inlineStr">
+        <is>
+          <t>Theo CEL-118</t>
+        </is>
+      </c>
+      <c r="J126" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, /luan-giai/sau</t>
+        </is>
+      </c>
+      <c r="K126" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/prompt-v3.ts, scripts/thu-nghiem-do-ro.ts</t>
+        </is>
+      </c>
+      <c r="L126" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M126" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ áp cho lá số CHƯA có bài (đệm sinh một lần, CEL-122) — muốn áp cho cả lá số cũ thì tăng THE_HE_DEM. Giám khảo là AI (gemini chấm luna viết) — cần 5–10 người thật đọc mù xác nhận. Đo: 6 câu song song xong 24s, 6/6 đạt luật.</t>
+        </is>
+      </c>
+      <c r="N126" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O126" s="8" t="inlineStr">
+        <is>
+          <t>ban-do-manh-yeu</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="13" t="inlineStr">
+        <is>
+          <t>CEL-127</t>
+        </is>
+      </c>
+      <c r="B127" s="14" t="inlineStr">
+        <is>
+          <t>G. Trải nghiệm &amp; giao diện</t>
+        </is>
+      </c>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>Bản đồ mạnh – yếu 12 mặt đời ở /la-so</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="inlineStr">
+        <is>
+          <t>Luận giải thiếu THỨ BẬC (3/30 bài nói mạnh nhất/yếu nhất) và đưa thứ bậc qua prompt thì model gần như bỏ qua → hiện bằng engine, tất định.</t>
+        </is>
+      </c>
+      <c r="E127" s="8" t="inlineStr">
+        <is>
+          <t>1. du-kien: chiTietDiemTungCung — điểm kèm sao đỡ/kéo trong cung + các cung soi vào; hung tinh ĐẮC ĐỊA chỉ trừ nửa (Hóa Kỵ ở tứ mộ, Kình Đà đắc…).
+2. components/luangiai/BanDoManhYeu.tsx: Thế mạnh / Bình (gập) / Cần gắng; thanh độ mạnh tương đối chạy khi cuộn tới; chạm một dòng mở "vì sao" (Đang đỡ / Đang kéo / mặt đời soi vào) + "Đọc sâu về …" sang /luan-giai/sau?chuDe=…; nhãn "Đang đi qua" / "Năm …".
+3. Đoạn TQ04 của Celes làm tóm tắt (3 dòng + Đọc tiếp); TQ04 bỏ khỏi danh sách tổng quan.
+4. /luan-giai/sau nhận ?chuDe, chip mục lục tự cuộn tới chủ đề đang mở.
+5. Token màu --tier-manh / --tier-binh / --tier-gang (hổ phách, không đỏ) cho hai theme.</t>
+        </is>
+      </c>
+      <c r="F127" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G127" s="8" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="H127" s="8" t="inlineStr">
+        <is>
+          <t>Tính lại mỗi lần lập</t>
+        </is>
+      </c>
+      <c r="I127" s="8" t="inlineStr">
+        <is>
+          <t>Khách trở lên (đọc sâu cần đăng nhập)</t>
+        </is>
+      </c>
+      <c r="J127" s="8" t="inlineStr">
+        <is>
+          <t>/la-so</t>
+        </is>
+      </c>
+      <c r="K127" s="8" t="inlineStr">
+        <is>
+          <t>components/luangiai/BanDoManhYeu.tsx, lib/rag/v3/du-kien.ts, app/la-so/page.tsx, app/luan-giai/sau/page.tsx, app/globals.css</t>
+        </is>
+      </c>
+      <c r="L127" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện tiếng Việt</t>
+        </is>
+      </c>
+      <c r="M127" s="8" t="inlineStr">
+        <is>
+          <t>Không hiện điểm thô (xếp hạng tương đối, không phải thang tốt–xấu); dòng Sức khỏe kèm "không phải chẩn đoán". Trọng số điểm là luật cố định CHƯA được người xem tử vi kiểm — nên nhờ chuyên gia đối chiếu vài lá số. Đo: nút ≥44px, không tràn ngang, CLS /la-so desktop 0,066 (trước 0,109), mobile 0.</t>
+        </is>
+      </c>
+      <c r="N127" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O127" s="8" t="inlineStr">
+        <is>
+          <t>ban-do-manh-yeu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16133,7 +16293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17944,6 +18104,38 @@
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="50" t="inlineStr">
+        <is>
+          <t>ban-do-manh-yeu</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>CEL-126, CEL-127</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Áp "bản C" (luận sâu hơn) vào prompt v3; thêm Bản đồ mạnh – yếu 12 mặt đời trên /la-so (engine, tất định) với phần "vì sao" và lối sang đọc sâu đúng chủ đề; hung tinh đắc địa chỉ trừ nửa điểm.</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt sau thử nghiệm mù độ rõ: "áp bản C, làm bản đồ mạnh-yếu".</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Thiet ke lai Ban do manh - yeu va viet lai chu cho de hieu
- Thanh lech hai phia quanh muc giua (trung vi) cua la so, mot thuoc chung; bo chuan hoa min-max
- Hien du 12 dong, hai o "Thuan loi nhat / Can cham chut nhat", thanh cung hang ca tren dien thoai
- Nhom Thuan loi / On dinh / Can cham chut dung chung cho prompt TQ04 va du kien (TEN_MUC)
- Ly do viet bang loi thuong, ten sao de sau; GopDiem them loai/sao/doSang
- PHIEN_BAN_DU_KIEN_V3 2026.09.6

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -11143,7 +11143,9 @@
 2. components/luangiai/BanDoManhYeu.tsx: Thế mạnh / Bình (gập) / Cần gắng; thanh độ mạnh tương đối chạy khi cuộn tới; chạm một dòng mở "vì sao" (Đang đỡ / Đang kéo / mặt đời soi vào) + "Đọc sâu về …" sang /luan-giai/sau?chuDe=…; nhãn "Đang đi qua" / "Năm …".
 3. Đoạn TQ04 của Celes làm tóm tắt (3 dòng + Đọc tiếp); TQ04 bỏ khỏi danh sách tổng quan.
 4. /luan-giai/sau nhận ?chuDe, chip mục lục tự cuộn tới chủ đề đang mở.
-5. Token màu --tier-manh / --tier-binh / --tier-gang (hổ phách, không đỏ) cho hai theme.</t>
+5. Token màu --tier-manh / --tier-binh / --tier-gang (hổ phách, không đỏ) cho hai theme.
+6. Thiết kế lại (25/09): thanh LỆCH HAI PHÍA quanh mức giữa (trung vị) của lá số, một thước chung — bỏ chuẩn hoá min–max vốn phóng đại khoảng cách; hiện đủ 12 dòng (nhóm giữa không gập); hai ô "Thuận lợi nhất / Cần chăm chút nhất" ở đầu; thanh cùng hàng với tên cả trên điện thoại.
+7. Đổi lời: nhóm Thuận lợi / Ổn định / Cần chăm chút (prompt TQ04 và dữ kiện dùng cùng tên — TEN_MUC); phần lý do viết bằng lời thường ("Điều giúp bạn", "Điều gây trở ngại", tên sao để sau); "Vận hiện tại" thay "Đang đi qua"; bỏ chữ "engine", "soi vào", "đang kéo".</t>
         </is>
       </c>
       <c r="F127" s="9" t="inlineStr">
@@ -16293,7 +16295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18136,6 +18138,38 @@
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B58" s="50" t="inlineStr">
+        <is>
+          <t>ban-do-thiet-ke-lai</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>CEL-127</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Thiết kế lại Bản đồ mạnh – yếu: thanh lệch hai phía quanh mức giữa, đủ 12 dòng, ô tóm tắt mạnh nhất / cần chăm chút nhất; viết lại toàn bộ chữ cho dễ hiểu, giải nghĩa sao bằng lời thường.</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "xem lại giải pháp thiết kế… đẹp hơn" và "từ ngữ còn thô, khó hiểu, reword lại".</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Trang la so chia tab va bieu do radar cho ban do manh - yeu
- Tab Tong quan / Chuyen sau / Manh - yeu / La so (chi dien thoai), dinh duoi thanh dieu huong, kem so phan, nho tab tren URL
- Tong quan chi con danh gia chung + luan tong quan + mot loi moi tiep
- Tab Chuyen sau hien du 14 chu de kem nhan manh - yeu cua cung chinh
- Ban do manh - yeu them bieu do radar 12 cung theo vong la so
- Bo the doc dai cu, lien ket kham pha chu de, the hoi Celes lon (trung lap)
- Backlog: CEL-128

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O127"/>
+  <dimension ref="A1:O128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11199,6 +11199,89 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="13" t="inlineStr">
+        <is>
+          <t>CEL-128</t>
+        </is>
+      </c>
+      <c r="B128" s="14" t="inlineStr">
+        <is>
+          <t>G. Trải nghiệm &amp; giao diện</t>
+        </is>
+      </c>
+      <c r="C128" s="8" t="inlineStr">
+        <is>
+          <t>Trang lá số chia tab: Tổng quan · Chuyên sâu · Mạnh – yếu · Lá số</t>
+        </is>
+      </c>
+      <c r="D128" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: trang lá số nhồi quá nhiều khối xếp dọc (ba thẻ đánh giá → bản đồ mạnh–yếu → thẻ mời chuyên sâu → luận tổng quan → đọc dài → hỏi Celes), luận tổng quan nằm tít dưới, luận chuyên sâu không nổi bật; người đọc không biết trang có bao nhiêu nội dung.</t>
+        </is>
+      </c>
+      <c r="E128" s="8" t="inlineStr">
+        <is>
+          <t>1. Thanh tab dính dưới thanh điều hướng, mỗi tab kèm số phần (10 / 14 / 12), nhớ tab trên URL (?tab=), phím mũi tên chuyển tab (ARIA tablist).
+2. Tổng quan = Đánh giá chung (3 thẻ) + Luận giải tổng quan (7 câu) + MỘT lời mời tiếp (sang Chuyên sâu) + dòng Hỏi Celes nhỏ.
+3. Chuyên sâu = đủ 14 chủ đề dạng thẻ trên chính trang lá số, mỗi thẻ có số câu và nhãn mạnh–yếu của cung chính (gợi ý đọc gì trước) → /luan-giai/sau?chuDe=.
+4. Mạnh – yếu = biểu đồ RADAR 12 cung (xếp theo vòng lá số: trục đối diện là cung xung chiếu) + ô mạnh nhất/cần chăm chút nhất + danh sách chi tiết.
+5. Lá số (chỉ điện thoại) = mệnh bàn; máy tính giữ mệnh bàn dính cột trái.
+6. Bỏ khỏi trang: thẻ "Cùng Celes nhìn kỹ hơn" (đọc dài cũ, trùng tổng quan v3 — chỉ còn ở đường lùi tiếng Anh), liên kết "Khám phá từng chủ đề" (/luan-giai cũ, trùng chuyên sâu), thẻ Hỏi Celes cỡ lớn.
+7. Tiêu đề trang: "Lá số của bạn" thay "Có một điều khá rõ ở bạn…".</t>
+        </is>
+      </c>
+      <c r="F128" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G128" s="8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="H128" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I128" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người (chuyên sâu cần đăng nhập)</t>
+        </is>
+      </c>
+      <c r="J128" s="8" t="inlineStr">
+        <is>
+          <t>/la-so</t>
+        </is>
+      </c>
+      <c r="K128" s="8" t="inlineStr">
+        <is>
+          <t>app/la-so/page.tsx, components/laso/TabLaSo.tsx, components/laso/HoiCelesDong.tsx, components/luangiai/ChuyenSauChuDe.tsx, components/luangiai/BanDoManhYeu.tsx, lib/i18n/vi.ts, lib/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L128" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện vi + en (en chỉ có Tổng quan và Lá số — v3 chỉ viết tiếng Việt)</t>
+        </is>
+      </c>
+      <c r="M128" s="8" t="inlineStr">
+        <is>
+          <t>Tham khảo: Ashtakavarga/VedAstro "Life Map" (chấm điểm 12 nhà, tô màu theo độ mạnh), app bát tự dùng radar ngũ hành. Sự kiện mới chart_tab_opened để đo tab nào được mở. Đo: không tràn ngang ở 390px, mọi tab ≥44px. Cần theo dõi: tỉ lệ bấm sang Chuyên sâu trước/sau (deep_read_cta theo viTri).</t>
+        </is>
+      </c>
+      <c r="N128" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O128" s="8" t="inlineStr">
+        <is>
+          <t>la-so-chia-tab</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16295,7 +16378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18170,6 +18253,38 @@
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B59" s="50" t="inlineStr">
+        <is>
+          <t>la-so-chia-tab</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>CEL-128, CEL-127</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Chia trang lá số thành 4 tab có số phần; tab Chuyên sâu hiện đủ 14 chủ đề; Bản đồ mạnh – yếu thêm biểu đồ radar theo vòng lá số; bỏ các khối trùng (đọc dài cũ, khám phá chủ đề, thẻ hỏi Celes lớn).</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "phần luận giải lá số nên chỉ có đánh giá và luận tổng quan… chức năng khác tách ra" + "biểu đồ làm nổi bật hơn, tham khảo loại biểu đồ khác".</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Sinh lai luan v3 cho la so cu theo ban C (THE_HE_DEM 2)
- Moi la so cu duoc viet lai mot lan khi mo
- Cau sinh lai hong thi tam tra bai the he truoc, khong ghi vao khoa moi
- Backlog: CEL-126

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16378,7 +16378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18285,6 +18285,38 @@
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B60" s="50" t="inlineStr">
+        <is>
+          <t>sinh-lai-ban-c</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>CEL-126</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Tăng thế hệ đệm luận v3 (THE_HE_DEM 1 → 2): mọi lá số cũ được viết lại theo bản C khi mở; câu sinh lại hỏng thì tạm trả bài thế hệ trước, không ghi vào khoá mới.</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "chạy lại với các lá cũ".</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Nut quay lai dung chung cho cac trang con
- QuayLai: uu tien ?ve=, roi trang vua roi trong phien, roi duong mac dinh
- Gan vao luan giai chuyen sau, kham pha chu de, dang nhap, hoi Celes
- La so gan duong ve kem tab cho moi loi sang trang con
- Hop giu lai la so khong chan lien ket dang nhap
- Backlog: CEL-129

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O128"/>
+  <dimension ref="A1:O129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11282,6 +11282,86 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" s="13" t="inlineStr">
+        <is>
+          <t>CEL-129</t>
+        </is>
+      </c>
+      <c r="B129" s="14" t="inlineStr">
+        <is>
+          <t>G. Trải nghiệm &amp; giao diện</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>Nút quay lại cho các trang con</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: bấm sang luận giải chuyên sâu thì không có chỗ quay lại màn cũ.</t>
+        </is>
+      </c>
+      <c r="E129" s="8" t="inlineStr">
+        <is>
+          <t>1. components/QuayLai.tsx: nút "← Về …" dùng chung — ưu tiên ?ve= (trang trước dặn đường về, kèm đúng tab), rồi trang vừa rời trong phiên (GhiTrangTruoc ở layout ghi khi bấm liên kết nội bộ), rồi đường mặc định.
+2. Gắn vào: /luan-giai/sau (mọi trạng thái; không có ve thì dựng lại /la-so?…&amp;tab=chuyen-sau từ thông tin sinh trên URL), /luan-giai, /dang-nhap, /hoi-dap (chỉ khi đến từ lá số).
+3. /la-so gắn ve kèm tab cho: thẻ chủ đề chuyên sâu, "Đọc phân tích chi tiết" ở mạnh–yếu, Hỏi Celes.
+4. Hộp "giữ lại lá số" không chặn liên kết sang /dang-nhap nữa (người bấm đã chọn đăng nhập).</t>
+        </is>
+      </c>
+      <c r="F129" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G129" s="8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="H129" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I129" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người</t>
+        </is>
+      </c>
+      <c r="J129" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau, /luan-giai, /dang-nhap, /hoi-dap</t>
+        </is>
+      </c>
+      <c r="K129" s="8" t="inlineStr">
+        <is>
+          <t>components/QuayLai.tsx, app/layout.tsx, app/luan-giai/sau/page.tsx, app/luan-giai/page.tsx, app/dang-nhap/page.tsx, app/hoi-dap/page.tsx, app/la-so/page.tsx, components/laso/CanhBaoRoiTrang.tsx</t>
+        </is>
+      </c>
+      <c r="L129" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện tiếng Việt</t>
+        </is>
+      </c>
+      <c r="M129" s="8" t="inlineStr">
+        <is>
+          <t>Đã rà: /hanh-trinh/chi-tiet, /support/checkout, các bước nhập sinh đã có nút lùi sẵn. `ve` chỉ nhận đường nội bộ (chặn // và /\) — không thành lối chuyển hướng ra ngoài. Thử luồng khách: la-so tab Chuyên sâu → chủ đề → đăng nhập → Quay lại = đúng tab; /luan-giai/sau có ve → Về lá số = đúng tab Mạnh – yếu.</t>
+        </is>
+      </c>
+      <c r="N129" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O129" s="8" t="inlineStr">
+        <is>
+          <t>nut-quay-lai</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16378,7 +16458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18317,6 +18397,38 @@
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B61" s="50" t="inlineStr">
+        <is>
+          <t>nut-quay-lai</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>CEL-129</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Thêm nút quay lại dùng chung cho luận giải chuyên sâu, khám phá chủ đề, đăng nhập, hỏi Celes; về đúng lá số và đúng tab vừa rời.</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "khi bấm sang luận giải sâu, ko có chỗ back lại màn cũ, check vs tất cả các nút khác".</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Chong lap noi dung giua cac phan luan cua cung la so
- Phan quyen du kien: cung tam phuong khong kem doan dien nghia, cach cuc chi vao chu de lien quan
- So y (so-y.ts): cau sau biet phan truoc da noi gi, kiem lap gan nguyen van
- Mot cau giu moc thoi gian moi chu de; TQ10 chi ke ba chang
- Diem noi bat xoay 7 goc theo ngay, tranh y 3 ngay truoc
- Hanh trinh khong ke lai tinh cach goc
- Bo do chat luong theo phien doc (scripts/do-chat-luong-v3.ts)
- THE_HE_DEM 3
- Backlog: CEL-130

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O129"/>
+  <dimension ref="A1:O130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11362,6 +11362,88 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="13" t="inlineStr">
+        <is>
+          <t>CEL-130</t>
+        </is>
+      </c>
+      <c r="B130" s="14" t="inlineStr">
+        <is>
+          <t>B. Luận giải AI</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t>Chống lặp nội dung giữa các phần luận của cùng lá số</t>
+        </is>
+      </c>
+      <c r="D130" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án rà lá số của mình: "đã đọc cái này rồi, sao xuất hiện nhiều thế". Rà 46 câu v3 + 7 thẻ điểm nổi bật + hành trình: "khó chịu âm ỉ, phản ứng nhanh" 15 lần, "thấy thiếu dù đủ" 9 lần, "trước 30 tuổi bị chặn" 15 lần, lời khuyên "tìm người cùng gánh" gần mọi câu; điểm nổi bật 7 ngày liền cùng một ý.</t>
+        </is>
+      </c>
+      <c r="E130" s="8" t="inlineStr">
+        <is>
+          <t>1. Phân quyền dữ kiện (du-kien): cung chỉ ở tam phương không kèm đoạn diễn nghĩa (Nghĩa nền/Nét chung/nghĩa phụ tinh); cách cục của cung tam phương chỉ vào chủ đề liên quan (CACH_CUC_CHU_DE).
+2. Sổ ý (lib/rag/v3/so-y.ts): mỗi câu nhận ý chính + lời khuyên các phần đã sinh của cùng lá số + năm (route đọc từ đệm, lưu dàn ý yChinh); kiểm lặp gần nguyên văn (cụm 4 chữ) → vòng sửa.
+3. Một câu giữ dòng thời gian mỗi chủ đề (CAU_GIU_MOC); TQ10 chỉ kể ba chặng tiền–trung–hậu vận.
+4. Điểm nổi bật: xoay 7 góc theo ngày (GOC_THEO_NGAY) + tránh ý của 3 ngày gần nhất.
+5. Hành trình: không kể lại tính cách gốc/cách cục Mệnh.
+6. THE_HE_DEM 2 → 3 để lá số cũ sinh lại.</t>
+        </is>
+      </c>
+      <c r="F130" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G130" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H130" s="8" t="inlineStr">
+        <is>
+          <t>Một lần mỗi lá số + năm + nhóm</t>
+        </is>
+      </c>
+      <c r="I130" s="8" t="inlineStr">
+        <is>
+          <t>Theo CEL-118</t>
+        </is>
+      </c>
+      <c r="J130" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, /luan-giai/sau, /home, /hanh-trinh</t>
+        </is>
+      </c>
+      <c r="K130" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/so-y.ts, lib/rag/v3/du-kien.ts, lib/rag/v3/index.ts, app/api/luan-giai-v3/route.ts, lib/rag/noi-dung-ai.ts, lib/rag/be-mat-ngan.ts, app/api/diem-noi-bat/route.ts, scripts/do-chat-luong-v3.ts</t>
+        </is>
+      </c>
+      <c r="L130" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M130" s="8" t="inlineStr">
+        <is>
+          <t>Đo (scripts/do-chat-luong-v3.ts, lá số A, 39 câu tổng quan + 4 chủ đề): câu lặp ý với câu đã đọc (embedding ≥0,70) 16% → 12%, ≥0,75 5% → 3%; giám khảo đếm lần lặp thừa 158 → 103, điểm "mới" 3,67 → 3,90, tự nhiên/cụ thể không giảm; ý có trích nguồn RAG 18% → 27%. Giám khảo gemini 503 lúc đo → lùi về model viết (chỉ tham khảo). Sổ ý phụ thuộc thứ tự mở: phần mở trước giữ ý, phần sau né.</t>
+        </is>
+      </c>
+      <c r="N130" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O130" s="8" t="inlineStr">
+        <is>
+          <t>chong-lap-giua-phan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16458,7 +16540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18429,6 +18511,38 @@
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B62" s="50" t="inlineStr">
+        <is>
+          <t>chong-lap-giua-phan</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>CEL-130</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Chống lặp nội dung giữa các phần luận: phân quyền dữ kiện, sổ ý đã nói, một câu giữ mốc mỗi chủ đề; điểm nổi bật xoay góc theo ngày; hành trình không kể lại tính cách gốc; bộ đo chất lượng theo phiên đọc.</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "rà soát tất cả nội dung xung quanh 1 lá số… hạn chế nội dung trùng lặp".</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Backlog: CEL-131 dot 1 cai thien chat luong luan giai
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O130"/>
+  <dimension ref="A1:O131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11444,6 +11444,87 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="13" t="inlineStr">
+        <is>
+          <t>CEL-131</t>
+        </is>
+      </c>
+      <c r="B131" s="14" t="inlineStr">
+        <is>
+          <t>B. Luận giải AI</t>
+        </is>
+      </c>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t>Vòng cải thiện chất lượng luận giải (prompt + RAG), đo bằng so mù</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: chạy phiên 2 giờ liên tục chấm điểm và cải thiện — lời văn mượt như người đang xem lá số, cụ thể, có giá trị, tận dụng tối đa tài liệu RAG.</t>
+        </is>
+      </c>
+      <c r="E131" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 1 (25/09): 1. Truy hồi v3 2026.09.5 — cung chính của chủ đề đứng trước, hai lượt chọn mỗi vòng; bỏ bí danh "phu" (trùng Thiên Phủ); loại đoạn sai giới tính; cộng điểm đoạn đúng chủ đề.
+2. TQ04 không kể lại danh sách nhóm (bản đồ đã hiện), nói vì sao hai đầu thang, có dữ kiện "vì sao" từ engine chấm.
+3. Chuyên sâu: luật DÙNG NGUỒN (≥2 ý dựa nguồn khi có đoạn [KHỚP CUNG CHÍNH]).
+4. Tổng quan: luật lời khuyên nói như người thật. (Đã thử và BỎ: "dám nói rõ" — model chép cụm "Nói thẳng"; lời khuyên "một việc" ở chuyên sâu — mất biện pháp thực tế.)
+5. Bộ đo: scripts/do-chat-luong-v3.ts (phiên đọc, lặp bằng embedding, RAG bằng mã) + scripts/so-sanh-v3.ts (so mù từng cặp).</t>
+        </is>
+      </c>
+      <c r="F131" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G131" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H131" s="8" t="inlineStr">
+        <is>
+          <t>Một lần mỗi lá số + năm + nhóm</t>
+        </is>
+      </c>
+      <c r="I131" s="8" t="inlineStr">
+        <is>
+          <t>Theo CEL-118</t>
+        </is>
+      </c>
+      <c r="J131" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, /luan-giai/sau</t>
+        </is>
+      </c>
+      <c r="K131" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/truy-hoi-v3.ts, lib/rag/v3/prompt-v3.ts, lib/rag/v3/index.ts, lib/rag/v3/du-kien.ts, scripts/so-sanh-v3.ts</t>
+        </is>
+      </c>
+      <c r="L131" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M131" s="8" t="inlineStr">
+        <is>
+          <t>Mốc kiểm tra trên lá số C + 3 chủ đề KHÔNG dùng để tối ưu (tiền bạc, sức khỏe, gia đình): bản mới thắng production 69% chuyên sâu, 64% tổng quan (so mù); ý có trích nguồn 27% → 58%. Giám khảo: gemini 503 suốt phiên → lùi về model viết (luna) — so cặp giảm thiên lệch nhưng vẫn nên có người đọc xác nhận.</t>
+        </is>
+      </c>
+      <c r="N131" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O131" s="8" t="inlineStr">
+        <is>
+          <t>chat-luong-luan-giai</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16540,7 +16621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18543,6 +18624,38 @@
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="50" t="inlineStr">
+        <is>
+          <t>chat-luong-luan-giai</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>CEL-131</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 1 phiên cải thiện chất lượng: truy hồi ưu tiên cung chính chủ đề, TQ04 nói vì sao, chuyên sâu dùng nguồn RAG, bộ so mù từng cặp.</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "tiếp tục chạy session 2 giờ … liên tục cải thiện chất lượng luận giải".</t>
+        </is>
+      </c>
+      <c r="F63" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Chuyen sau: viec lam duoc ngay o doan cuoi; THE_HE_DEM 4
- VIEC_LAM_NGAY: 2-3 viec cu the trong tuan toi, khong neu so tien (so mu 3 giam khao x 2 la so: ~68%)
- Prompt 2026.09.10
- THE_HE_DEM 3 -> 4: la so cu sinh lai mot lan voi toan bo cai thien cua phien
- Backlog: CEL-131 dot 2

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -11471,7 +11471,13 @@
 2. TQ04 không kể lại danh sách nhóm (bản đồ đã hiện), nói vì sao hai đầu thang, có dữ kiện "vì sao" từ engine chấm.
 3. Chuyên sâu: luật DÙNG NGUỒN (≥2 ý dựa nguồn khi có đoạn [KHỚP CUNG CHÍNH]).
 4. Tổng quan: luật lời khuyên nói như người thật. (Đã thử và BỎ: "dám nói rõ" — model chép cụm "Nói thẳng"; lời khuyên "một việc" ở chuyên sâu — mất biện pháp thực tế.)
-5. Bộ đo: scripts/do-chat-luong-v3.ts (phiên đọc, lặp bằng embedding, RAG bằng mã) + scripts/so-sanh-v3.ts (so mù từng cặp).</t>
+5. Bộ đo: scripts/do-chat-luong-v3.ts (phiên đọc, lặp bằng embedding, RAG bằng mã) + scripts/so-sanh-v3.ts (so mù từng cặp).
+Đợt 2 (25/09): 6. Trang chuyên sâu gọi HAI lượt nối tiếp mỗi chủ đề (nửa đầu hiện trước; nửa sau nhận sổ ý của nửa đầu) — câu lặp ý 5–6% → 1–3%.
+7. Chặn tên sách lọt vào bài: bỏ tên tài liệu khỏi nhãn nguồn + kiểm bằng mã.
+8. TQ04 mở bằng tên hai mặt mạnh nhất / hai mặt cần chăm chút nhất.
+9. Chuyên sâu: VIỆC LÀM ĐƯỢC NGAY — đoạn cuối 2–3 việc cụ thể trong tuần tới, không nêu số tiền.
+10. Bỏ luật lời khuyên "một việc" ở chuyên sâu. Đã thử và BỎ: chỉ vào lá số bằng lời thường; tổng quan dài 80–170 từ.
+11. THE_HE_DEM 3 → 4.</t>
         </is>
       </c>
       <c r="F131" s="9" t="inlineStr">
@@ -11516,7 +11522,7 @@
       </c>
       <c r="N131" s="8" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>Đánh giá cuối (3 giám khảo luna / groq gpt-oss-120b / gpt-4o-mini, 74 cặp × 3 = 222 lượt): bản sau đợt 1 thắng bản gốc ~58% (chuyên sâu ~58%, tổng quan ~57% — gpt-4o-mini không thích TQ04 cũ-mới); sau khi TQ04 nêu tên hai đầu thang: tổng quan ~63%. Vòng 9 (việc làm được ngay): thắng ~68% trên 78 lượt, cả 3 giám khảo &gt; 50%. RAG: ý có trích nguồn ở chuyên sâu ~27% → ~60%. BÀI HỌC ĐO: một giám khảo (model viết tự chấm) dao động tới ±30% chỉ vì đổi chữ tiêu chí; ≤25 cặp có khoảng tin cậy ±20–26% — phải dùng ≥3 giám khảo và ≥60 cặp trước khi kết luận. Gemini 503 suốt phiên.</t>
         </is>
       </c>
       <c r="O131" s="8" t="inlineStr">
@@ -16621,7 +16627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18656,6 +18662,38 @@
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="50" t="inlineStr">
+        <is>
+          <t>chat-luong-luan-giai</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>CEL-131</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 2: chuyên sâu hai lượt nối tiếp, chặn tên sách, TQ04 nêu hai đầu thang, việc làm được ngay ở chuyên sâu; THE_HE_DEM 4; đánh giá 3 giám khảo.</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: phiên 2 giờ cải thiện chất lượng luận giải.</t>
+        </is>
+      </c>
+      <c r="F64" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Tach loi khuyen khoi tung cau: gom thanh "Goi y cua Celes"; bo do tiet kiem token
- Bai luan v3 khong ket bang loi khuyen; truong goiY rieng (giong goi y, khong dat han); kiem ket-loi-khuyen + giao-viec
- Bo luat viec lam duoc ngay
- GoiYCeles cuoi tong quan va cuoi moi chu de chuyen sau
- THE_HE_DEM 5
- do-chat-luong-v3: --chi, --tu, dem token; so-sanh-v3: giam khao re truoc, dung som, chi tra ma chon
- Backlog: CEL-132, CEL-133

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O131"/>
+  <dimension ref="A1:O133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11531,6 +11531,166 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" s="13" t="inlineStr">
+        <is>
+          <t>CEL-132</t>
+        </is>
+      </c>
+      <c r="B132" s="14" t="inlineStr">
+        <is>
+          <t>B. Luận giải AI</t>
+        </is>
+      </c>
+      <c r="C132" s="8" t="inlineStr">
+        <is>
+          <t>Tách lời khuyên khỏi từng câu luận — gom thành phần "Gợi ý của Celes"</t>
+        </is>
+      </c>
+      <c r="D132" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "trong tuần tới…" nghe như ép buộc; "không nên mỗi câu hỏi đều có lời khuyên, có thể tổng hợp thành một phần riêng".</t>
+        </is>
+      </c>
+      <c r="E132" s="8" t="inlineStr">
+        <is>
+          <t>1. Bài luận v3 KHÔNG kết bằng lời khuyên — kết bằng điểm cần lưu ý / câu khép ý; kiểm bằng mã (ket-loi-khuyen) thay luật cũ bắt buộc có lời khuyên.
+2. Model trả thêm trường goiY (≤30 từ, giọng gợi ý "bạn có thể…", không đặt hạn); kiểm giao-viec chặn "trong tuần tới / ngay hôm nay".
+3. Bỏ luật VIỆC LÀM ĐƯỢC NGAY.
+4. Giao diện GoiYCeles: cuối phần tổng quan và cuối mỗi chủ đề chuyên sâu, tối đa 5 gợi ý, bỏ trùng, ghi câu hỏi nguồn — không tốn thêm lượt gọi model.
+5. Sổ ý dùng goiY làm "gợi ý đã dùng". THE_HE_DEM 4 → 5.</t>
+        </is>
+      </c>
+      <c r="F132" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G132" s="8" t="inlineStr">
+        <is>
+          <t>AI + UI</t>
+        </is>
+      </c>
+      <c r="H132" s="8" t="inlineStr">
+        <is>
+          <t>Một lần mỗi lá số + năm + nhóm</t>
+        </is>
+      </c>
+      <c r="I132" s="8" t="inlineStr">
+        <is>
+          <t>Theo CEL-118</t>
+        </is>
+      </c>
+      <c r="J132" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, /luan-giai/sau</t>
+        </is>
+      </c>
+      <c r="K132" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/prompt-v3.ts, lib/rag/v3/index.ts, lib/rag/v3/kiem-v3.ts, lib/rag/v3/so-y.ts, app/api/luan-giai-v3/route.ts, components/luangiai/GoiYCeles.tsx, components/luangiai/TongQuanV3.tsx, app/luan-giai/sau/page.tsx</t>
+        </is>
+      </c>
+      <c r="L132" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện tiếng Việt</t>
+        </is>
+      </c>
+      <c r="M132" s="8" t="inlineStr">
+        <is>
+          <t>Đo lá số C (17 câu): 17/17 có goiY, 0 câu kết bằng lời khuyên, 0 câu đặt hạn. Bộ quy tắc gốc (quy-tac-luan-giai.ts, dùng chung các màn khác) giữ nguyên — Bước 8 "điểm cần lưu ý hoặc lời khuyên" chọn vế đầu cho v3.</t>
+        </is>
+      </c>
+      <c r="N132" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O132" s="8" t="inlineStr">
+        <is>
+          <t>bo-giao-viec-tiet-kiem-test</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="13" t="inlineStr">
+        <is>
+          <t>CEL-133</t>
+        </is>
+      </c>
+      <c r="B133" s="14" t="inlineStr">
+        <is>
+          <t>H. Vận hành &amp; đo lường</t>
+        </is>
+      </c>
+      <c r="C133" s="8" t="inlineStr">
+        <is>
+          <t>Bộ đo chất lượng luận giải tiết kiệm token</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: phần test tốn quá nhiều token. Ngày 25/09 luna 1.773 lượt gọi, ~13,6 triệu token vào / 1,5 triệu ra (phần lớn là bộ đo); mỗi câu ~14–15 nghìn token vào (prompt hệ thống ~10 nghìn ký tự + dữ kiện + 8 đoạn nguồn + sổ ý; câu phải sửa gửi lại toàn bộ); chỉ ~32% được đệm.</t>
+        </is>
+      </c>
+      <c r="E133" s="8" t="inlineStr">
+        <is>
+          <t>1. do-chat-luong-v3.ts: --chi (chỉ sinh câu thay đổi chạm tới), --tu (lấy câu còn lại từ lượt đã lưu, không sinh lại bản mốc), in token vào/ra/đệm.
+2. so-sanh-v3.ts: chuỗi giám khảo rẻ → đắt (groq → gpt-4o-mini → luna), dừng sớm khi hai giám khảo cùng chiều (≥60% hoặc ≤40%), chỉ trả mã chọn không lý do (maxTokens 400), bỏ cặp trùng nguyên văn, --chi.
+3. Quy trình: sinh bản mốc MỘT lần cho mỗi phiên bản prompt rồi dùng lại; đo lặp/RAG bằng mã (gần như miễn phí) trước, chỉ gọi giám khảo khi cần.</t>
+        </is>
+      </c>
+      <c r="F133" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G133" s="8" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="H133" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I133" s="8" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="J133" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K133" s="8" t="inlineStr">
+        <is>
+          <t>scripts/do-chat-luong-v3.ts, scripts/so-sanh-v3.ts</t>
+        </is>
+      </c>
+      <c r="L133" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M133" s="8" t="inlineStr">
+        <is>
+          <t>Ước tính mỗi vòng thử: trước ~1,5 triệu token (sinh 2 lá × 25 câu + sinh lại bản mốc + luna chấm có lý do) → sau ~100–300 nghìn (6–18 câu thay đổi + giám khảo rẻ, dừng sớm), giảm ~80–90%. Đo thật: chấm 13 cặp bằng 2 giám khảo rẻ = 22,6 nghìn vào / 1,1 nghìn ra. Giám khảo vẫn nhiễu (cùng hai tệp: groq 38% khi viết lý do, 62% khi chỉ chọn) — chỉ tin khi ≥2 giám khảo cùng chiều.</t>
+        </is>
+      </c>
+      <c r="N133" s="8" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="O133" s="8" t="inlineStr">
+        <is>
+          <t>bo-giao-viec-tiet-kiem-test</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16627,7 +16787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18694,6 +18854,38 @@
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="49" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="50" t="inlineStr">
+        <is>
+          <t>bo-giao-viec-tiet-kiem-test</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>CEL-132, CEL-133</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Tách lời khuyên khỏi từng câu, gom thành "Gợi ý của Celes"; bỏ "việc làm được ngay"; bộ đo tiết kiệm token (--chi, --tu, giám khảo rẻ dừng sớm).</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "bỏ phần lời khuyên… tổng hợp thành 1 phần riêng" + "phần test tốn quá nhiều token".</t>
+        </is>
+      </c>
+      <c r="F65" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Chuyen sau thanh mot mach doc: khung Su nghiep moi, cong thuc viet, Tom lai moi chu de
- Khung Su nghiep 8 cau theo mach (tao gia tri -> vi tri -> nghe -> mo hinh -> nut that -> quy nhan -> duong len va dinh -> dang o dau)
- Cong thuc chuyen sau: tra loi thang, mo lop moi, khong chung chung, ban chat truoc ten nganh, moc co dieu kien, mot khoanh khac dung qua khong dan nhan
- Tom lai moi chu de (tom-lai.ts), cau dan 14 chu de
- Kiem: chep nguyen mot cau dai, nhan luat lot vao bai
- so-sanh-phien-v3.ts; THE_HE_DEM 6
- Backlog: CEL-134

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O133"/>
+  <dimension ref="A1:O134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11691,6 +11691,88 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="13" t="inlineStr">
+        <is>
+          <t>CEL-134</t>
+        </is>
+      </c>
+      <c r="B134" s="14" t="inlineStr">
+        <is>
+          <t>B. Luận giải AI</t>
+        </is>
+      </c>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>Chuyên sâu thành một mạch đọc: khung Sự nghiệp mới, công thức viết, "Tóm lại" mỗi chủ đề</t>
+        </is>
+      </c>
+      <c r="D134" s="8" t="inlineStr">
+        <is>
+          <t>Review của chủ dự án về chủ đề Sự nghiệp (7/10): "Celes hiểu tôi từ 2–3 ý rồi diễn giải lại theo 8 câu hỏi"; đọc giống career coaching; "hợp nghề nào" mở bằng tên ngành; mốc "đỉnh 45–54" quá tuyệt đối; "Trong tuần tới…" máy móc; thiếu khoảnh khắc "đúng quá"; cần phần tóm lại ghép thành một con đường. Kèm bản thiết kế luồng Pain point → Narrative → Prediction → Summary cho 14 chủ đề.</t>
+        </is>
+      </c>
+      <c r="E134" s="8" t="inlineStr">
+        <is>
+          <t>1. Khung Sự nghiệp viết lại (8 câu): tạo giá trị bằng cách nào → vị trí trong tổ chức → nhóm nghề (bản chất trước, ngành là ví dụ) → làm công / tự do / tự làm → nút thắt → quý nhân / đối thủ → kiểu đi lên &amp; đỉnh của cái gì → đang ở đâu. Bỏ "môi trường" (gộp SN02) và "xa quê" (trùng RN02).
+2. Công thức chuyên sâu (prompt 2026.09.14): trả lời thẳng câu đầu → biểu hiện → điều kiện/thời điểm → mức chắc chắn; mở lớp mới, không lấy nét chung của chủ đề làm trọng tâm; tự kiểm "bỏ lá số đi có đúng với ai cũng được không"; mốc thời gian có điều kiện; một khoảnh khắc "đúng quá" không dán nhãn.
+3. "Tóm lại" mỗi chủ đề (lib/rag/v3/tom-lai.ts): một lượt gọi ngắn, ghép các câu theo mạch riêng từng chủ đề, 100–150 từ, đệm khoá …|tom-lai; trang gọi sau khi đủ câu.
+4. Câu dẫn nỗi băn khoăn cho 14 chủ đề (tĩnh).
+5. Kiểm bằng mã: chép gần nguyên một câu dài (≥70%) chặn; nhãn luật lọt vào bài ("đúng quá", "cảm giác rất đúng với bạn là") chặn.
+6. Bộ so sánh cả phiên (scripts/so-sanh-phien-v3.ts). THE_HE_DEM 5 → 6; đường lùi thế hệ trước chỉ nhận bài cùng câu hỏi.</t>
+        </is>
+      </c>
+      <c r="F134" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G134" s="8" t="inlineStr">
+        <is>
+          <t>AI + UI</t>
+        </is>
+      </c>
+      <c r="H134" s="8" t="inlineStr">
+        <is>
+          <t>Một lần mỗi lá số + năm + nhóm (+ tóm lại)</t>
+        </is>
+      </c>
+      <c r="I134" s="8" t="inlineStr">
+        <is>
+          <t>Theo CEL-118</t>
+        </is>
+      </c>
+      <c r="J134" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau</t>
+        </is>
+      </c>
+      <c r="K134" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/khung.ts, lib/rag/v3/prompt-v3.ts, lib/rag/v3/tom-lai.ts, lib/rag/v3/index.ts, lib/rag/v3/so-y.ts, app/api/luan-giai-v3/route.ts, app/luan-giai/sau/page.tsx, scripts/so-sanh-phien-v3.ts</t>
+        </is>
+      </c>
+      <c r="L134" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện tiếng Việt</t>
+        </is>
+      </c>
+      <c r="M134" s="8" t="inlineStr">
+        <is>
+          <t>Đo Sự nghiệp (lá A, C): câu lặp ý trong chủ đề 15–19% → 7–10% (embedding ≥0,70), ≥0,80: 5–9% → 0–1%. So cả phiên với bản cũ: lá A bản mới thắng 100% (2 giám khảo), lá C ~67%. Bài học: câu VÍ DỤ trong prompt bị chép vào 7/8 câu — không đưa câu mẫu cho yêu cầu kiểu "khoảnh khắc đúng quá". CHƯA áp khung mới cho 13 chủ đề còn lại, chưa có "Bức tranh lớn" toàn lá số, chưa có "Muốn đi sâu hơn"; sức khỏe gọi tên nhóm cơ quan cần chủ dự án quyết (đụng luật "không chẩn đoán").</t>
+        </is>
+      </c>
+      <c r="N134" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O134" s="8" t="inlineStr">
+        <is>
+          <t>luan-chuyen-sau-mach-truyen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16787,7 +16869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18886,6 +18968,38 @@
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B66" s="50" t="inlineStr">
+        <is>
+          <t>luan-chuyen-sau-mach-truyen</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>CEL-134</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Khung Sự nghiệp mới theo mạch đọc, công thức viết chuyên sâu, phần "Tóm lại" cuối mỗi chủ đề, câu dẫn 14 chủ đề; THE_HE_DEM 6.</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án gửi review Sự nghiệp + bản thiết kế luồng chuyên sâu.</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Khung chuyen sau moi cho 13 chu de, Buc tranh lon, Muon di sau hon, du doan suc khoe
- Khung 2026.09.3 theo luong cua chu du an (87 cau chuyen sau)
- An toan: suc khoe duoc neu nhom co quan dang xu huong, khong khang dinh; con cai / hon nhan noi xu huong
- Buc tranh lon (buc-tranh.ts, BucTranhLon) va Muon di sau hon (DiSauHon)
- Chan chu noi bo trong bai; loc doc de theo the he; chi nhan bai cung cau hoi
- THE_HE_DEM 7
- Backlog: CEL-135

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O134"/>
+  <dimension ref="A1:O135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11773,6 +11773,87 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" s="13" t="inlineStr">
+        <is>
+          <t>CEL-135</t>
+        </is>
+      </c>
+      <c r="B135" s="14" t="inlineStr">
+        <is>
+          <t>B. Luận giải AI</t>
+        </is>
+      </c>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t>Khung chuyên sâu mới cho 13 chủ đề + Bức tranh lớn + Muốn đi sâu hơn + dự đoán sức khỏe</t>
+        </is>
+      </c>
+      <c r="D135" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "làm tất cả các phần chưa làm"; sức khỏe "có thể nêu dự đoán — mục tiêu tử vi là dự đoán vận mệnh, miễn là không áp đặt, khẳng định".</t>
+        </is>
+      </c>
+      <c r="E135" s="8" t="inlineStr">
+        <is>
+          <t>1. Khung 2026.09.3: 13 chủ đề viết lại theo luồng Pain point → Narrative → Prediction của chủ dự án (tổng 87 câu chuyên sâu, trước 61); gộp các cặp sát nghĩa để không quá dài (Tình duyên 10→8, Vận hạn 10→8, chủ đề ngắn gộp câu cùng ý).
+2. Luật an toàn mới: sức khỏe được nêu nhóm cơ quan / vùng đáng lưu ý và kiểu vấn đề, xếp theo mức, bằng lời xu hướng — không khẳng định mắc bệnh, không chẩn đoán; con cái được nói xu hướng ít/đông (không con số); hôn nhân được nói xu hướng biến động, rủi ro người thứ ba như khả năng (không khẳng định). Bỏ câu an toàn gắn vào từng câu sức khỏe → một dòng lưu ý đầu chủ đề.
+3. Bức tranh lớn (lib/rag/v3/buc-tranh.ts, components/luangiai/BucTranhLon.tsx): mục cuối mục lục chuyên sâu, ghép "Tóm lại" các chủ đề đã đọc + tổng quan, 6 điều, ~300–450 từ; cần ≥3 chủ đề; khoá kèm danh sách chủ đề.
+4. Muốn đi sâu hơn (components/luangiai/DiSauHon.tsx): 2–4 câu tò mò mỗi chủ đề dẫn sang Hỏi Celes, có đường về.
+5. Chặn chữ nội bộ trong bài ("dữ kiện", "tín hiệu phụ trợ"). CAU_GIU_MOC theo id mới. docNhieuTheoTienTo lọc theo thế hệ ngay trong truy vấn. Route chỉ nhận bài đã cất khi cùng câu hỏi. THE_HE_DEM 6 → 7.</t>
+        </is>
+      </c>
+      <c r="F135" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G135" s="8" t="inlineStr">
+        <is>
+          <t>AI + UI</t>
+        </is>
+      </c>
+      <c r="H135" s="8" t="inlineStr">
+        <is>
+          <t>Một lần mỗi lá số + năm + nhóm (+ tóm lại, + bức tranh theo danh sách chủ đề)</t>
+        </is>
+      </c>
+      <c r="I135" s="8" t="inlineStr">
+        <is>
+          <t>Theo CEL-118</t>
+        </is>
+      </c>
+      <c r="J135" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau</t>
+        </is>
+      </c>
+      <c r="K135" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/khung.ts, lib/rag/v3/prompt-v3.ts, lib/rag/v3/index.ts, lib/rag/v3/buc-tranh.ts, lib/rag/noi-dung-ai.ts, app/api/luan-giai-v3/route.ts, app/luan-giai/sau/page.tsx, components/luangiai/BucTranhLon.tsx, components/luangiai/DiSauHon.tsx</t>
+        </is>
+      </c>
+      <c r="L135" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện tiếng Việt</t>
+        </is>
+      </c>
+      <c r="M135" s="8" t="inlineStr">
+        <is>
+          <t>Đo lá số C (Sức khỏe + Tiền bạc, 13 câu): 13/13 đạt; câu lặp ý 9% (≥0,70); sức khỏe nêu vùng đầu – mắt, tai – giác quan, da theo thứ bậc + kiểu âm ỉ/tái phát + giai đoạn, không khẳng định. Bức tranh lớn (3 chủ đề) 435 từ. Chi phí đo ~165 nghìn token vào cho 13 câu + tóm lại. CHƯA đo so mù từng chủ đề mới với khung cũ; "Bức tranh lớn" chưa có lối vào từ /la-so.</t>
+        </is>
+      </c>
+      <c r="N135" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O135" s="8" t="inlineStr">
+        <is>
+          <t>khung-chuyen-sau-toan-bo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16869,7 +16950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19000,6 +19081,38 @@
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B67" s="50" t="inlineStr">
+        <is>
+          <t>khung-chuyen-sau-toan-bo</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>CEL-135</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Khung chuyên sâu mới cho 13 chủ đề, dự đoán sức khỏe theo nhóm cơ quan, Bức tranh lớn, Muốn đi sâu hơn; THE_HE_DEM 7.</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "làm tất cả các phần chưa làm" + duyệt dự đoán sức khỏe.</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Lang kinh tung chu de, chong lap cum tu, Tinh cach ba tang
- LANG_KINH 12 chu de: Tinh cach noi ve con nguoi ngoai vai tro, cong viec toi da mot vi du phu
- Khung Tinh cach 2026.09.4 theo ba tang (ben trong / va vao doi / trong mat nguoi khac)
- Chong lap cum 3-4 am tiet va cum quen tay (tinh huong roi, giu trat tu...)
- Khoa tom lai / buc tranh lon kem phien ban khung; khong tang THE_HE_DEM
- Backlog: CEL-136

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O135"/>
+  <dimension ref="A1:O136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11854,6 +11854,86 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" s="13" t="inlineStr">
+        <is>
+          <t>CEL-136</t>
+        </is>
+      </c>
+      <c r="B136" s="14" t="inlineStr">
+        <is>
+          <t>B. Luận giải AI</t>
+        </is>
+      </c>
+      <c r="C136" s="8" t="inlineStr">
+        <is>
+          <t>Lăng kính riêng từng chủ đề + chống lặp cụm từ; Tính cách viết lại theo ba tầng</t>
+        </is>
+      </c>
+      <c r="D136" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: lá số Hiếu lặp "tình huống rối" 5 lần trong chủ đề Tính cách; review chương Tính cách: ~40% trượt sang năng lực / phong cách làm việc ("đồng nghiệp nhìn tôi", gợi ý thành tư vấn nghề).</t>
+        </is>
+      </c>
+      <c r="E136" s="8" t="inlineStr">
+        <is>
+          <t>1. LANG_KINH cho 12 chủ đề (index.ts): mỗi chủ đề giữ đúng phần đời; Tính cách: con người khi bỏ vai trò ra ngoài, ví dụ ở gia đình / bạn bè / tình yêu / tiền / lúc một mình / biến cố, công việc tối đa một ví dụ phụ, cấm từ vựng quản lý; áp cả trường goiY. TQ01–TQ03 thêm cùng lăng kính.
+2. Khung Tính cách 2026.09.4 — ba tầng: bên trong (bản chất, nổi bật, cần gì – sợ gì) → khi va vào đời (bị tổn thương / hiểu lầm, áp lực – biến cố, người thân vs người ngoài, tự làm khó mình) → trong mắt người khác &amp; theo tuổi. Bỏ "quyết định sai ở đâu".
+3. Chống lặp cụm từ (so-y.ts): sổ cụm 3–4 âm tiết đã dùng ở ≥2 câu cùng chủ đề đưa vào prompt; chặn khi dùng lại ≥2 cụm, tự lặp một cụm ≥3 lần, hoặc dùng lại "cụm quen tay" (tình huống rối, giữ trật tự, tự xoay xở, giữ nhịp, âm ỉ…).
+4. Khoá tóm lại / bức tranh lớn kèm phiên bản khung; KHÔNG tăng THE_HE_DEM — route chỉ nhận bài cùng câu hỏi nên chỉ các câu đổi nghĩa sinh lại.</t>
+        </is>
+      </c>
+      <c r="F136" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G136" s="8" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H136" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ câu đổi nghĩa sinh lại</t>
+        </is>
+      </c>
+      <c r="I136" s="8" t="inlineStr">
+        <is>
+          <t>Theo CEL-118</t>
+        </is>
+      </c>
+      <c r="J136" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau, /la-so</t>
+        </is>
+      </c>
+      <c r="K136" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/index.ts, lib/rag/v3/so-y.ts, lib/rag/v3/khung.ts, lib/rag/v3/prompt-v3.ts, app/api/luan-giai-v3/route.ts, scripts/so-sanh-phien-v3.ts</t>
+        </is>
+      </c>
+      <c r="L136" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M136" s="8" t="inlineStr">
+        <is>
+          <t>Đo Tính cách lá số Hiếu (bài cũ trong DB vs sinh lại): từ công sở 8,0 → 0,4 /1000 chữ; từ đời sống 0 → 7,3 /1000; "tình huống rối" 2 → 0 trong bài luận; câu lặp ý 3%; so cả phiên theo tiêu chí review: bản mới thắng ~83% (luna 100% ×2, gpt-4o-mini 50%). Các chủ đề khác (từ lượt đo đã lưu): mật độ từ công sở Tình duyên 8,0, Tiền 7,0, Sức khỏe 5,2 /1000 (Sự nghiệp 26,1 là đúng chủ đề). Còn lại: hai câu cùng đợt sinh đầu (song song) vẫn có thể trùng một cụm.</t>
+        </is>
+      </c>
+      <c r="N136" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O136" s="8" t="inlineStr">
+        <is>
+          <t>lang-kinh-chu-de-va-lap-cum</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16950,7 +17030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19113,6 +19193,38 @@
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="50" t="inlineStr">
+        <is>
+          <t>lang-kinh-chu-de-va-lap-cum</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>CEL-136</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Lăng kính từng chủ đề, chống lặp cụm từ và cụm quen tay, khung Tính cách ba tầng.</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: lỗi lặp "tình huống rối" + review chương Tính cách.</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Xuat luan giai chuyen sau ra Excel/PDF cho quan tri vien
- Nut Xuat du lieu o /luan-giai/sau, chi hien voi admin (ADMIN_EMAILS)
- Xuat chu de dang xem hoac toan bo 14 chu de + Buc tranh lon
- Route /api/admin/xuat-luan-giai kiem quyen, dung tep bang exceljs / pdfkit
- Nhung font Be Vietnam Pro (OFL) cho PDF tieng Viet
- Backlog: CEL-137

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O136"/>
+  <dimension ref="A1:O137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11934,6 +11934,87 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="13" t="inlineStr">
+        <is>
+          <t>CEL-137</t>
+        </is>
+      </c>
+      <c r="B137" s="14" t="inlineStr">
+        <is>
+          <t>D. Quản trị</t>
+        </is>
+      </c>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>Xuất luận giải chuyên sâu ra Excel / PDF — chỉ quản trị viên</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: cần xuất dữ liệu luận giải chuyên sâu để đọc, soát và lưu ngoài app; chỉ tài khoản admin.</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>1. Nút "Xuất dữ liệu" ở đầu bài /luan-giai/sau, chỉ hiện khi GET /api/admin/xuat-luan-giai trả laAdmin (ADMIN_EMAILS).
+2. Chọn phạm vi: chủ đề đang xem hoặc toàn bộ 14 chủ đề (kèm Bức tranh lớn); chọn định dạng Excel hoặc PDF.
+3. Chủ đề đã đọc xong dùng luôn bài đang hiện; chủ đề chưa mở gọi đúng /api/luan-giai-v3 (hai nửa + tóm lại), có dòng tiến độ.
+4. POST dựng tệp ở máy chủ, kiểm lại quyền admin (403 nếu không), làm sạch dữ liệu, chặn 3 MB.
+5. Excel (exceljs): 3 trang Tổng quan / Luận giải (mỗi câu một dòng: chủ đề, mã câu, câu hỏi, luận giải, vì sao, gợi ý; có lọc) / Tóm lại (+ Bức tranh lớn). PDF (pdfkit + font Be Vietnam Pro nhúng): bìa, mục lục, mỗi chủ đề một trang mới, vì sao, tóm lại, gợi ý, số trang.</t>
+        </is>
+      </c>
+      <c r="F137" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G137" s="8" t="inlineStr">
+        <is>
+          <t>Quản trị</t>
+        </is>
+      </c>
+      <c r="H137" s="8" t="inlineStr">
+        <is>
+          <t>Không tốn thêm lượt AI với chủ đề đã đệm</t>
+        </is>
+      </c>
+      <c r="I137" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J137" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau</t>
+        </is>
+      </c>
+      <c r="K137" s="8" t="inlineStr">
+        <is>
+          <t>app/api/admin/xuat-luan-giai/route.ts, lib/xuat/luan-giai.ts, lib/xuat/fonts/*, components/luangiai/XuatLuanGiai.tsx, app/luan-giai/sau/page.tsx, next.config.ts</t>
+        </is>
+      </c>
+      <c r="L137" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ admin</t>
+        </is>
+      </c>
+      <c r="M137" s="8" t="inlineStr">
+        <is>
+          <t>Dựng thử bằng dữ liệu giả: Excel đủ 3 trang; PDF 8 trang cho 2 chủ đề, dấu tiếng Việt đúng. Chưa đăng nhập: GET laAdmin=false, POST 403. next build: font theo route (nft).</t>
+        </is>
+      </c>
+      <c r="N137" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O137" s="8" t="inlineStr">
+        <is>
+          <t>xuat-luan-giai-admin</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17030,7 +17111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19225,6 +19306,38 @@
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B69" s="50" t="inlineStr">
+        <is>
+          <t>xuat-luan-giai-admin</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>CEL-137</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Nút xuất luận giải chuyên sâu (Excel/PDF, từng chủ đề hoặc toàn bộ) cho quản trị viên.</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu.</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Dem luan giai v3 theo khung gio sinh, gioi han la so moi theo IP cho khach
- Khoa dem bam theo khung gio (veGioLaSo) de cung la so tren may khac khong sinh lai; doc lui khoa gio tho
- Khach chua dang nhap: toi da 3 la so phai viet moi/ngay/IP (GUEST_NEW_CHARTS_DAILY_LIMIT), IP bam HMAC, dem trong noi_dung_ai
- /la-so: het luot thi lui ve ban doc nhanh tat dinh + the dang nhap
- CEL-138, CEL-139

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O137"/>
+  <dimension ref="A1:O139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12015,6 +12015,165 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" s="13" t="inlineStr">
+        <is>
+          <t>CEL-138</t>
+        </is>
+      </c>
+      <c r="B138" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>Đệm luận giải v3 theo khung giờ sinh — cùng lá số không sinh lại ở máy khác</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án báo 26/09/2026: mở một tài khoản trên nhiều thiết bị thì bài vẫn "load lại". Đo trong noi_dung_ai: lá số của chủ dự án bị sinh lại 8 lần trong 24–25/09 — nguyên nhân chính là các lần tăng THE_HE_DEM (th:2 → th:6 → th:7) và đổi kiểu khoá, KHÔNG phải thiết bị. Đệm theo lá số đúng như thiết kế (đo trên production: lần đầu 23,7 giây, lần hai 1,2 giây). Lỗ hổng thật còn lại: khoá băm GIỜ THÔ, nên cùng người lưu giờ 6 ở máy này và 5 ở máy kia là hai khoá.</t>
+        </is>
+      </c>
+      <c r="E138" s="8" t="inlineStr">
+        <is>
+          <t>1. veGioLaSo(): giờ chẵn 2–22 gộp về giờ lẻ liền trước; 0 và 23 giữ nguyên (Tý muộn đổi ngày). Kiểm: 4 ngày sinh × 24 giờ × 2 giới — lá số khớp engine 100%
+2. /api/luan-giai-v3 băm theo khung giờ; docCoLui đọc bài cũ dưới khoá giờ thô rồi chép sang khoá mới
+3. Ghi chú tại THE_HE_DEM: không tăng khi chưa hỏi chủ dự án, gom thay đổi vào một lần tăng</t>
+        </is>
+      </c>
+      <c r="F138" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G138" s="8" t="inlineStr">
+        <is>
+          <t>AI (có đệm)</t>
+        </is>
+      </c>
+      <c r="H138" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lá số + năm + nhóm</t>
+        </is>
+      </c>
+      <c r="I138" s="8" t="inlineStr">
+        <is>
+          <t>Khách trở lên</t>
+        </is>
+      </c>
+      <c r="J138" s="8" t="inlineStr">
+        <is>
+          <t>/api/luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="K138" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/nhat-ky.ts, app/api/luan-giai-v3/route.ts</t>
+        </is>
+      </c>
+      <c r="L138" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M138" s="8" t="inlineStr">
+        <is>
+          <t>Sổ ý và Bức tranh lớn đọc theo tiền tố khoá MỚI: lá số giờ chẵn chỉ thấy các chủ đề đã mở lại sau 26/09 (mở lại chủ đề là tự chuyển khoá). Nút "Tạo bản mới" (thay cho việc tăng thế hệ) vẫn chờ làm.</t>
+        </is>
+      </c>
+      <c r="N138" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O138" s="8" t="inlineStr">
+        <is>
+          <t>dem-da-thiet-bi-gioi-han-khach</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="13" t="inlineStr">
+        <is>
+          <t>CEL-139</t>
+        </is>
+      </c>
+      <c r="B139" s="14" t="inlineStr">
+        <is>
+          <t>E. Tài khoản &amp; quyền</t>
+        </is>
+      </c>
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t>Giới hạn lá số mới mỗi ngày theo IP cho khách chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="D139" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu 26/09/2026. Tổng quan v3 mở cho khách (CEL-118) và mỗi lá số chưa có bài tốn ~12 lượt gọi model — rủi ro chi phí lớn nhất hiện tại. Giờ mỗi IP được tối đa 3 lá số PHẢI VIẾT MỚI mỗi ngày (giờ VN); lá số đã có bài, mở lại, hay lượt thứ hai của cùng trang đều không đếm. Đã đăng nhập: không giới hạn.</t>
+        </is>
+      </c>
+      <c r="E139" s="8" t="inlineStr">
+        <is>
+          <t>1. lib/auth/gioi-han-khach.ts: xinLuotLaSoMoi — IP băm HMAC (không cất IP thô), đếm trong noi_dung_ai bề mặt gioi-han-khach (không cần SQL mới)
+2. Route trả 429 gioiHanKhach chỉ khi đệm thiếu bài và là khách
+3. /la-so: hết lượt thì lùi về bản đọc nhanh tất định (không gọi model) + thẻ "Đăng nhập để đọc tiếp"
+4. Trần đổi qua biến môi trường GUEST_NEW_CHARTS_DAILY_LIMIT (mặc định 3)</t>
+        </is>
+      </c>
+      <c r="F139" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G139" s="8" t="inlineStr">
+        <is>
+          <t>Máy chủ</t>
+        </is>
+      </c>
+      <c r="H139" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi ngày</t>
+        </is>
+      </c>
+      <c r="I139" s="8" t="inlineStr">
+        <is>
+          <t>Khách</t>
+        </is>
+      </c>
+      <c r="J139" s="8" t="inlineStr">
+        <is>
+          <t>/api/luan-giai-v3, /la-so</t>
+        </is>
+      </c>
+      <c r="K139" s="8" t="inlineStr">
+        <is>
+          <t>lib/auth/gioi-han-khach.ts, app/api/luan-giai-v3/route.ts, components/luangiai/TongQuanV3.tsx, app/la-so/page.tsx, lib/rag/noi-dung-ai.ts</t>
+        </is>
+      </c>
+      <c r="L139" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M139" s="8" t="inlineStr">
+        <is>
+          <t>Hỏng thì cho qua (không đọc được IP, bảng lỗi) — chặn nhầm khách thật tệ hơn lọt vài lượt. Nhiều người chung một IP (văn phòng, 4G nhà mạng) chia chung 3 lượt. Hai lá số mới gọi song song có thể lọt quá trần một lượt. ĐÃ KIỂM bằng server thật (trần 1): lá số mới thứ hai 429, lá số đã đếm mở lại được, Chrome 390px hiện thẻ đăng nhập, không tràn ngang.</t>
+        </is>
+      </c>
+      <c r="N139" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O139" s="8" t="inlineStr">
+        <is>
+          <t>dem-da-thiet-bi-gioi-han-khach</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17111,7 +17270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19338,6 +19497,38 @@
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B70" s="50" t="inlineStr">
+        <is>
+          <t>dem-da-thiet-bi-gioi-han-khach</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>CEL-138, CEL-139</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Khoá đệm luận giải v3 theo khung giờ sinh (kèm đọc lùi khoá cũ); giới hạn 3 lá số mới/ngày/IP cho khách, hết lượt lùi về bản đọc nhanh + mời đăng nhập.</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án báo bài load lại khi đổi thiết bị và yêu cầu giới hạn IP cho khách. Đo ra nguyên nhân chính là các lần tăng thế hệ đệm, không phải thiết bị.</t>
+        </is>
+      </c>
+      <c r="F70" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
RAG: muc tin cay co tac dung that, admin gan lai; luat ngam; luat ghep sao; nut Tao ban moi
- PATCH /api/admin/knowledge + o chon muc tin cay / loai nguon, ghi nhat ky quan tri
- tai-lieu-meta.ts doc muc tin cay tuoi tu kho, dau phien ban kho
- Truy hoi v3 2026.09.6 cong diem theo muc tin cay sau cong khop; prompt 2026.09.17 gan nhan tin cay
- Kiem chi-bo-tro, lo-luat-ngam; ghi chu chuyen gia / noi bo la luat ngam
- Ghep nghia hai sao duoc phep tru khi nguon noi nguoc; y ghep gan co ghep
- Tao ban moi: dang nhap, moi la so mot lan moi phien ban kho
- CEL-140, CEL-141, CEL-142

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O139"/>
+  <dimension ref="A1:O142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12174,6 +12174,246 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" s="13" t="inlineStr">
+        <is>
+          <t>CEL-140</t>
+        </is>
+      </c>
+      <c r="B140" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C140" s="8" t="inlineStr">
+        <is>
+          <t>Mức tin cậy nguồn có tác dụng thật + admin gán lại được</t>
+        </is>
+      </c>
+      <c r="D140" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 26/09/2026: "Tài liệu đã tải lên cũng phải cho Admin gán lại mức độ tin cậy, và mức độ tin cậy có value thực sự". Trước đó mức tin cậy chỉ chọn lúc tải lên, và luận giải v3 bỏ qua hẳn nó.</t>
+        </is>
+      </c>
+      <c r="E140" s="8" t="inlineStr">
+        <is>
+          <t>1. PATCH /api/admin/knowledge + hai ô chọn (loại nguồn, mức tin cậy) cho từng tài liệu ở /admin/knowledge; ghi admin_audit_log trước/sau
+2. lib/rag/tai-lieu-meta.ts: đọc mức tin cậy / loại nguồn thẳng từ kho, tươi sau ≤1 phút (truy hồi đệm 30 phút)
+3. Truy hồi v3 (2026.09.6): cộng điểm SAU cổng khớp sao–cung — cốt lõi +0,02, chuyên gia duyệt +0,012, tham khảo 0, bổ trợ −0,012
+4. Prompt 2026.09.17: nhãn [tin cậy: …] ở mỗi đoạn; hai đoạn ngược nhau theo đoạn tin cậy cao hơn, ngang mức thì nói cả hai
+5. Bộ kiểm chi-bo-tro: ý có căn cứ duy nhất là đoạn bổ trợ phải sửa</t>
+        </is>
+      </c>
+      <c r="F140" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G140" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H140" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt luận giải</t>
+        </is>
+      </c>
+      <c r="I140" s="8" t="inlineStr">
+        <is>
+          <t>Quản trị viên (gán) · mọi người đọc (tác dụng)</t>
+        </is>
+      </c>
+      <c r="J140" s="8" t="inlineStr">
+        <is>
+          <t>/admin/knowledge, /api/admin/knowledge, /api/luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="K140" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/tai-lieu-meta.ts, lib/rag/v3/truy-hoi-v3.ts, lib/rag/v3/index.ts, lib/rag/v3/prompt-v3.ts, app/api/admin/knowledge/route.ts, app/admin/knowledge/page.tsx</t>
+        </is>
+      </c>
+      <c r="L140" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M140" s="8" t="inlineStr">
+        <is>
+          <t>ĐO (21 câu × 3 lá số tổng hợp, chỉ truy hồi): 5% đoạn được chọn đổi, đoạn cốt lõi 12 → 18, đoạn khớp đúng cung 164 → 160. Kho hiện chỉ có MỘT tài liệu cốt lõi (Tử vi hàm số), 14 tài liệu tham khảo, chưa có bổ trợ / ghi chú chuyên gia — tác dụng thật tuỳ chủ dự án xếp lại 15 tài liệu. Hồ sơ README vẫn đang xuất bản (3 đoạn) — nên lưu trữ. Hỏi Celes / bài dài (bang-chung.ts) vẫn dùng mức tin cậy kiểu cũ (băng dung sai 5%).</t>
+        </is>
+      </c>
+      <c r="N140" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O140" s="8" t="inlineStr">
+        <is>
+          <t>rag-tin-cay</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="13" t="inlineStr">
+        <is>
+          <t>CEL-141</t>
+        </is>
+      </c>
+      <c r="B141" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C141" s="8" t="inlineStr">
+        <is>
+          <t>Luật ngầm (nguồn chuyên gia) và luật ghép nghĩa hai sao</t>
+        </is>
+      </c>
+      <c r="D141" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 26/09/2026: "Nguồn chuyên gia Celes là luật ngầm, không ghi trên lá số"; ghép nghĩa hai sao "không cấm, nếu tài liệu RAG không đề cập nội dung mâu thuẫn, ngược lại thì vẫn có thể ghép".</t>
+        </is>
+      </c>
+      <c r="E141" s="8" t="inlineStr">
+        <is>
+          <t>1. Loại nguồn "Ghi chú chuyên gia" và "Nội bộ" = luật ngầm: đoạn gắn nhãn [LUẬT NGẦM] (không mang đề mục), prompt cấm nhắc tới; bộ kiểm lo-luat-ngam bắt kiểu viện dẫn ("theo chuyên gia", "ghi chú của…")
+2. Luật 12 của prompt: được ghép, trừ khi nguồn nói tổ hợp ấy mang nghĩa khác / ngược (phản vi kỳ cách, phá cách) — khi đó theo nguồn
+3. Ý ghép chưa có nguồn cho tổ hợp: model gắn "ghep": true; route cất vào trường ghep của câu (sổ khuyết để bổ sung kho)</t>
+        </is>
+      </c>
+      <c r="F141" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G141" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H141" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt luận giải</t>
+        </is>
+      </c>
+      <c r="I141" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người đọc</t>
+        </is>
+      </c>
+      <c r="J141" s="8" t="inlineStr">
+        <is>
+          <t>/api/luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="K141" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/index.ts, lib/rag/v3/prompt-v3.ts, lib/rag/v3/kiem-v3.ts, lib/rag/tai-lieu-meta.ts, app/api/luan-giai-v3/route.ts</t>
+        </is>
+      </c>
+      <c r="L141" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M141" s="8" t="inlineStr">
+        <is>
+          <t>ĐÃ THỬ 8 bài (2 lá số tổng hợp × 4 câu), giả lập 2 tài liệu thành ghi chú chuyên gia: 2 bài dùng đoạn luật ngầm, 0 bài lộ; 4/8 bài có ý gắn ghep. So cùng 8 bài với bản cũ: đạt 7/8 so với 8/8, lỗi còn lại cùng loại có sẵn (độ dài, chữ nội bộ) — mẫu nhỏ, CHƯA so mù ≥3 giám khảo × ≥60 cặp. Chưa có trang tổng hợp sổ khuyết ghép (dữ liệu đã cất trong noi_dung_ai).</t>
+        </is>
+      </c>
+      <c r="N141" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O141" s="8" t="inlineStr">
+        <is>
+          <t>rag-tin-cay</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="13" t="inlineStr">
+        <is>
+          <t>CEL-142</t>
+        </is>
+      </c>
+      <c r="B142" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C142" s="8" t="inlineStr">
+        <is>
+          <t>Nút "Tạo bản mới" khi kho tri thức cập nhật</t>
+        </is>
+      </c>
+      <c r="D142" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án chốt phương án C (26/09/2026): người đã đăng nhập tự bấm viết lại, mỗi lá số một lần cho mỗi phiên bản kho — thay cho việc tăng THE_HE_DEM làm mọi lá số sinh lại (CEL-138).</t>
+        </is>
+      </c>
+      <c r="E142" s="8" t="inlineStr">
+        <is>
+          <t>1. phienBanKho(): dấu vân tay các tài liệu đang xuất bản (id, bản xuất bản, mức tin cậy, loại nguồn)
+2. Mỗi câu cất kèm kho; bài cũ không dấu coi như kho 40749bb09806 (đo lúc deploy) để nút không bật hàng loạt
+3. /api/luan-giai-v3 taoMoi: cần đăng nhập (401 cho khách), chỉ viết lại câu viết với kho cũ; tóm lại / bức tranh lớn cũng viết lại theo kho
+4. Nút ở cuối tổng quan (/la-so) và cuối mỗi chủ đề (/luan-giai/sau), chỉ hiện khi có câu viết với kho cũ</t>
+        </is>
+      </c>
+      <c r="F142" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G142" s="8" t="inlineStr">
+        <is>
+          <t>AI (có đệm)</t>
+        </is>
+      </c>
+      <c r="H142" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi phiên bản kho</t>
+        </is>
+      </c>
+      <c r="I142" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="J142" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, /luan-giai/sau, /api/luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="K142" s="8" t="inlineStr">
+        <is>
+          <t>app/api/luan-giai-v3/route.ts, components/luangiai/TongQuanV3.tsx, app/la-so/page.tsx, app/luan-giai/sau/page.tsx, lib/rag/tai-lieu-meta.ts</t>
+        </is>
+      </c>
+      <c r="L142" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M142" s="8" t="inlineStr">
+        <is>
+          <t>Mọi thay đổi kho (xuất bản, lưu trữ, đổi mức tin cậy) đều bật nút cho MỌI lá số — gom thay đổi kho thành đợt. Đã kiểm bằng server thật: khách 401, bài cũ banMoi=false. CHƯA kiểm được luồng viết lại khi đã đăng nhập bằng trình duyệt (cần tài khoản thật).</t>
+        </is>
+      </c>
+      <c r="N142" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O142" s="8" t="inlineStr">
+        <is>
+          <t>rag-tin-cay</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17270,7 +17510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19529,6 +19769,38 @@
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="50" t="inlineStr">
+        <is>
+          <t>rag-tin-cay</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>CEL-140, CEL-141, CEL-142</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Mức tin cậy có tác dụng thật + admin gán lại; luật ngầm cho nguồn chuyên gia; luật ghép nghĩa hai sao; nút Tạo bản mới theo phiên bản kho.</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Bốn quyết định của chủ dự án ngày 26/09/2026 về RAG.</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Kien truc luan giai v2 va thu vien tri thuc: lat cat Su nghiep luot 1 (chua bat)
- KIEN-TRUC-LUAN-GIAI.md v2: hien trang / dich, kiem ke du kien engine, quan he neo vao cung, 10 nguyen tac, nhat ky quyet dinh co cot xet lai, nguong lat cat chot truoc; v1 lam phu luc
- lib/rag/thu-vien: kieu muc, bo khop, kiem tat dinh, khoi T### cho prompt v3
- scripts/dung-thu-vien.ts (trich offline, luu Supabase), do-thu-vien.ts, test-thu-vien.ts; so-sanh-v3 --du
- Luot 1: 1091 muc; tieu chi 1,2,3,5 dat, so mu ~47% truot -> CAU_THU_VIEN rong, chua bat
- CEL-143

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O142"/>
+  <dimension ref="A1:O143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12414,6 +12414,86 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" s="13" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B143" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C143" s="8" t="inlineStr">
+        <is>
+          <t>Kiến trúc luận giải v2 + Thư viện tri thức: lát cắt "Sự nghiệp — lá số gốc" (lượt 1, CHƯA bật)</t>
+        </is>
+      </c>
+      <c r="D143" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt chi phí và yêu cầu làm hết phần đã chốt (26/09/2026). KIEN-TRUC-LUAN-GIAI.md viết lại thành v2 (hiện trạng / đích, kiểm kê dữ kiện engine, hợp đồng quan hệ neo vào cung, 10 nguyên tắc, nhật ký quyết định có cột "xét lại khi", ngưỡng lát cắt chốt trước), bản v1 giữ làm phụ lục. Dựng thư viện sự nghiệp và đo A/B.</t>
+        </is>
+      </c>
+      <c r="E143" s="8" t="inlineStr">
+        <is>
+          <t>1. lib/rag/thu-vien/: kiểu mục, bộ khớp (o-cung, xung, tam-hop, tam-phuong, giáp hai bên, mượn sao vô chính diệu, độ sáng, Tuần/Triệt, Tràng Sinh, chi), kiểm tất định, gom tổ hợp + lật/hoá giải + ngược chiều cho prompt
+2. scripts/dung-thu-vien.ts: trích offline → kiểm → gộp → mâu thuẫn → đích; lưu tạm noi_dung_ai bề mặt thu-vien (QĐ-13)
+3. Luồng v3 nhận khối T### (trần 14 mục, bớt đoạn sách khi thư viện đủ); route có CAU_THU_VIEN — đang RỖNG
+4. scripts/do-thu-vien.ts (tiêu chí 1,2,3,5) + so-sanh-v3.ts --du (chấm đủ, tỉ lệ bỏ hoà); scripts/test-thu-vien.ts 27 kiểm</t>
+        </is>
+      </c>
+      <c r="F143" s="9" t="inlineStr">
+        <is>
+          <t>Chờ quyết định</t>
+        </is>
+      </c>
+      <c r="G143" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H143" s="8" t="inlineStr">
+        <is>
+          <t>Offline (dựng) · mỗi lượt (khi bật)</t>
+        </is>
+      </c>
+      <c r="I143" s="8" t="inlineStr">
+        <is>
+          <t>Chưa ai (cờ tắt)</t>
+        </is>
+      </c>
+      <c r="J143" s="8" t="inlineStr">
+        <is>
+          <t>/api/luan-giai-v3 (khi bật)</t>
+        </is>
+      </c>
+      <c r="K143" s="8" t="inlineStr">
+        <is>
+          <t>KIEN-TRUC-LUAN-GIAI.md, lib/rag/thu-vien/*, lib/rag/v3/index.ts, lib/rag/v3/kiem-v3.ts, lib/rag/v3/truy-hoi-v3.ts, app/api/luan-giai-v3/route.ts, scripts/dung-thu-vien.ts, scripts/do-thu-vien.ts, scripts/test-thu-vien.ts, scripts/so-sanh-v3.ts</t>
+        </is>
+      </c>
+      <c r="L143" s="8" t="inlineStr">
+        <is>
+          <t>Tắt (CAU_THU_VIEN rỗng)</t>
+        </is>
+      </c>
+      <c r="M143" s="8" t="inlineStr">
+        <is>
+          <t>KẾT QUẢ LƯỢT 1: 1.091 mục (741 tổ hợp) từ 997 đoạn, 74% ứng viên qua kiểm tất định, tốn 0,64 tr token vào / 0,37 tr ra. Tiêu chí: #1 ghép bỏ qua 0,4% ĐẠT · #2 ý có nguồn 51% → 78% ĐẠT · #3 độ phủ 100% ĐẠT · #5 p95 30,2 → 22,4 giây ĐẠT · #4 so mù ~47% (luna 48/42, gpt-4o-mini 50/46) TRƯỢT → không bật (QĐ-15). Chỉ gọi được 2 model giám khảo khác nhau. Chẩn đoán: văn ngang nhau, thư viện tăng độ có căn cứ nhưng giám khảo máy không chấm độ đúng. Độ đúng trích ~80% trên 40 mẫu, lỗi chính: bỏ sót điều kiện cung; ~6,5 cặp ngược chiều mỗi bài. Chủ dự án chọn hướng: tự đọc mù chấm độ đúng / sửa khâu trích rồi đo lại / đổi ngưỡng.</t>
+        </is>
+      </c>
+      <c r="N143" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O143" s="8" t="inlineStr">
+        <is>
+          <t>thu-vien-su-nghiep</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17510,7 +17590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19801,6 +19881,38 @@
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="50" t="inlineStr">
+        <is>
+          <t>thu-vien-su-nghiep</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Tài liệu kiến trúc v2; thư viện tri thức sự nghiệp (1.091 mục, lưu Supabase); đo lát cắt — trượt so mù, chưa bật.</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt chi phí, yêu cầu làm hết phần đã chốt. Ngưỡng chốt trước khi chạy nên không dời.</t>
+        </is>
+      </c>
+      <c r="F72" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Bo do do dung (nhan dien la so) va do lai lat cat Su nghiep: khong co bang chung thu vien dung hon
- scripts/do-do-dung.ts: xep loai nhan dinh tren goi bang chung chung, kiem giam khao (luot 1: giam khao khong hop le)
- scripts/do-nhan-dien.ts: nhan dien la so co dap an + dem sao la bang ma; --chi-bai-luan
- scripts/lat-cat-su-nghiep.ts: bo la so dung chung
- Ket qua luot 3: luna A 93,3 / B 90; gpt-4o-mini A 70 / B 75 -> thu vien giu tat
- CEL-144

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O143"/>
+  <dimension ref="A1:O144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12480,7 +12480,7 @@
       </c>
       <c r="M143" s="8" t="inlineStr">
         <is>
-          <t>KẾT QUẢ LƯỢT 1: 1.091 mục (741 tổ hợp) từ 997 đoạn, 74% ứng viên qua kiểm tất định, tốn 0,64 tr token vào / 0,37 tr ra. Tiêu chí: #1 ghép bỏ qua 0,4% ĐẠT · #2 ý có nguồn 51% → 78% ĐẠT · #3 độ phủ 100% ĐẠT · #5 p95 30,2 → 22,4 giây ĐẠT · #4 so mù ~47% (luna 48/42, gpt-4o-mini 50/46) TRƯỢT → không bật (QĐ-15). Chỉ gọi được 2 model giám khảo khác nhau. Chẩn đoán: văn ngang nhau, thư viện tăng độ có căn cứ nhưng giám khảo máy không chấm độ đúng. Độ đúng trích ~80% trên 40 mẫu, lỗi chính: bỏ sót điều kiện cung; ~6,5 cặp ngược chiều mỗi bài. Chủ dự án chọn hướng: tự đọc mù chấm độ đúng / sửa khâu trích rồi đo lại / đổi ngưỡng.</t>
+          <t>KẾT QUẢ LƯỢT 1: 1.091 mục (741 tổ hợp) từ 997 đoạn, 74% ứng viên qua kiểm tất định, tốn 0,64 tr token vào / 0,37 tr ra. Tiêu chí: #1 ghép bỏ qua 0,4% ĐẠT · #2 ý có nguồn 51% → 78% ĐẠT · #3 độ phủ 100% ĐẠT · #5 p95 30,2 → 22,4 giây ĐẠT · #4 so mù ~47% (luna 48/42, gpt-4o-mini 50/46) TRƯỢT → không bật (QĐ-15). Chỉ gọi được 2 model giám khảo khác nhau. Chẩn đoán: văn ngang nhau, thư viện tăng độ có căn cứ nhưng giám khảo máy không chấm độ đúng. Độ đúng trích ~80% trên 40 mẫu, lỗi chính: bỏ sót điều kiện cung; ~6,5 cặp ngược chiều mỗi bài. Chủ dự án chọn hướng: tự đọc mù chấm độ đúng / sửa khâu trích rồi đo lại / đổi ngưỡng. || 26/09: bộ đo độ đúng (CEL-144) cũng không thấy B đúng hơn A → giữ tắt.</t>
         </is>
       </c>
       <c r="N143" s="8" t="inlineStr">
@@ -12491,6 +12491,85 @@
       <c r="O143" s="8" t="inlineStr">
         <is>
           <t>thu-vien-su-nghiep</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="13" t="inlineStr">
+        <is>
+          <t>CEL-144</t>
+        </is>
+      </c>
+      <c r="B144" s="14" t="inlineStr">
+        <is>
+          <t>H. Đo lường</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t>Bộ đo ĐỘ ĐÚNG luận giải (nhận diện lá số) + đo lại lát cắt Sự nghiệp</t>
+        </is>
+      </c>
+      <c r="D144" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu 26/09/2026: tự xây bộ tiêu chí đo độ đúng và test lại (so mù chỉ đo độ hay). Ngưỡng chốt vào KIEN-TRUC-LUAN-GIAI.md 11.5–11.6 TRƯỚC mỗi lượt chạy.</t>
+        </is>
+      </c>
+      <c r="E144" s="8" t="inlineStr">
+        <is>
+          <t>1. scripts/do-do-dung.ts: tách nhận định, xếp 4 loại trên gói bằng chứng chung, kèm kiểm giám khảo (cài lỗi, lệch lá)
+2. scripts/do-nhan-dien.ts: nhận diện lá số (lá thật vs lá mồi, có đáp án) + đếm sao lạ trong phần vì sao bằng mã; --chi-bai-luan
+3. scripts/lat-cat-su-nghiep.ts: bộ 12 lá số tổng hợp + 5 câu dùng chung</t>
+        </is>
+      </c>
+      <c r="F144" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G144" s="8" t="inlineStr">
+        <is>
+          <t>Công cụ đo</t>
+        </is>
+      </c>
+      <c r="H144" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi thay đổi prompt / RAG</t>
+        </is>
+      </c>
+      <c r="I144" s="8" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="J144" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K144" s="8" t="inlineStr">
+        <is>
+          <t>scripts/do-do-dung.ts, scripts/do-nhan-dien.ts, scripts/lat-cat-su-nghiep.ts, scripts/do-thu-vien.ts, KIEN-TRUC-LUAN-GIAI.md</t>
+        </is>
+      </c>
+      <c r="L144" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M144" s="8" t="inlineStr">
+        <is>
+          <t>Lượt 1 (xếp loại nhận định): KHÔNG DÙNG ĐƯỢC — bài của lá khác vẫn được chấm "có căn cứ" ~95% như bài thật. Lượt 2 (nhận diện, có phần vì sao): luna chạm trần 100/100. Lượt 3 (chỉ bài luận): luna A 93,3 / B 90,0; gpt-4o-mini A 70 / B 75 — ngược chiều, trong sai số → không có bằng chứng thư viện làm bài đúng hơn. Sao lạ 0/0. Phát hiện: bài hiện tại bám lá số tốt (93% nhận diện chỉ từ văn). Tốn ~1,6 tr token chấm.</t>
+        </is>
+      </c>
+      <c r="N144" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O144" s="8" t="inlineStr">
+        <is>
+          <t>do-do-dung</t>
         </is>
       </c>
     </row>
@@ -17590,7 +17669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19913,6 +19992,38 @@
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B73" s="50" t="inlineStr">
+        <is>
+          <t>do-do-dung</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>CEL-144, CEL-143</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Bộ đo độ đúng (nhận diện lá số) và đo lại lát cắt: không có bằng chứng thư viện làm bài đúng hơn.</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu tự xây tiêu chí đo độ đúng.</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Nguyen nhan goc thu vien va nghiem thu kien thuc bang dap an
- scripts/do-kien-thuc.ts: dap an kien thuc doc lap, cham dat/thieu/sai, kiem giam khao (cai loi, cham lai)
- cho-prompt.ts: xep tang chinh tinh tai cung chinh -> to hop co sao lon -> sao lon -> sao nho
- Ket qua: giam khao hop le, KT phang (A 58,5 / B2 56,9); thu vien chi phu 15% diem dap an (3% co do sang)
- CEL-145

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O144"/>
+  <dimension ref="A1:O145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12573,6 +12573,85 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="13" t="inlineStr">
+        <is>
+          <t>CEL-145</t>
+        </is>
+      </c>
+      <c r="B145" s="14" t="inlineStr">
+        <is>
+          <t>H. Đo lường</t>
+        </is>
+      </c>
+      <c r="C145" s="8" t="inlineStr">
+        <is>
+          <t>Phân tích nguyên nhân gốc thư viện + nghiệm thu KIẾN THỨC bằng đáp án chuyên gia</t>
+        </is>
+      </c>
+      <c r="D145" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu 26/09/2026: tìm rõ vì sao thư viện không cải thiện (kỹ thuật / giám khảo / thư viện), tìm tiêu chí nghiệm thu, chấm kiến thức tách khỏi cách viết bằng đáp án nạp cho giám khảo.</t>
+        </is>
+      </c>
+      <c r="E145" s="8" t="inlineStr">
+        <is>
+          <t>1. scripts/do-kien-thuc.ts: đáp án kiến thức mỗi (lá, câu) dựng độc lập từ cấu hình trọng yếu (engine) + kiến thức model + hợp đoạn sách; chấm dat/thieu/sai + vi phạm; kiểm giám khảo (cài lỗi đảo nghĩa, chấm lại)
+2. Sửa khâu chọn mục thư viện (cho-prompt.ts): xếp tầng chính tinh tại cung chính → tổ hợp có sao lớn → sao lớn → sao nhỏ; tối đa 3 mục / bộ sao
+3. do-thu-vien.ts --chi-b: sinh lại riêng bản có thư viện</t>
+        </is>
+      </c>
+      <c r="F145" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G145" s="8" t="inlineStr">
+        <is>
+          <t>Công cụ đo</t>
+        </is>
+      </c>
+      <c r="H145" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt sửa thư viện / prompt</t>
+        </is>
+      </c>
+      <c r="I145" s="8" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="J145" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K145" s="8" t="inlineStr">
+        <is>
+          <t>scripts/do-kien-thuc.ts, scripts/do-thu-vien.ts, lib/rag/thu-vien/cho-prompt.ts, KIEN-TRUC-LUAN-GIAI.md</t>
+        </is>
+      </c>
+      <c r="L145" s="8" t="inlineStr">
+        <is>
+          <t>Thư viện vẫn tắt</t>
+        </is>
+      </c>
+      <c r="M145" s="8" t="inlineStr">
+        <is>
+          <t>Giám khảo kiến thức HỢP LỆ (luna cài lỗi 12/12, nhất quán 87,5%; gpt-4o-mini 10/12, 92,6%). KT: luna A 58,5 / B 58,3 / B2 56,9; gpt-4o-mini 51 / 53,2 / 51 → phẳng. Nguyên nhân gốc: điểm đáp án trung bình 4,6 yếu tố, 94% cần độ sáng, 42% có sát tinh, 48% kết hợp ≥2 cung; thư viện chỉ phủ 15% điểm (3% có độ sáng). Kết luận: chính = thư viện chưa đủ chi tiết (khâu trích bỏ trống độ sáng / cung / sao đi cùng); phụ = khâu chọn (đã sửa, không quyết định); giám khảo trước đo sai thứ. Liêm Phủ + lục cát: 0 mục. Đề xuất nghiệm thu: cổng tất định phủ đáp án ≥50% (≥30% có độ sáng) → KT ≥ A+10 → cách viết ≥45% → chủ dự án duyệt 10 đáp án mẫu. Tốn ~1 tr token vào chấm + 0,4 tr sinh B2.</t>
+        </is>
+      </c>
+      <c r="N145" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O145" s="8" t="inlineStr">
+        <is>
+          <t>rootcause-thu-vien</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17669,7 +17748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20024,6 +20103,38 @@
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B74" s="50" t="inlineStr">
+        <is>
+          <t>rootcause-thu-vien</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>CEL-145</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Nguyên nhân gốc thư viện: thiếu chi tiết (độ sáng, tổ hợp nhiều yếu tố), không phải giám khảo; bộ nghiệm thu kiến thức bằng đáp án.</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu phân tích nguyên nhân gốc và tiêu chí nghiệm thu.</t>
+        </is>
+      </c>
+      <c r="F74" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Backlog: CEL-146 thu vien luot 2
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O145"/>
+  <dimension ref="A1:O146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12652,6 +12652,87 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="13" t="inlineStr">
+        <is>
+          <t>CEL-146</t>
+        </is>
+      </c>
+      <c r="B146" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C146" s="8" t="inlineStr">
+        <is>
+          <t>Thư viện Sự nghiệp lượt 2 — trích chi tiết (độ sáng, nhóm "ít nhất k", tổ hợp) + đo lại</t>
+        </is>
+      </c>
+      <c r="D146" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 26/09/2026: "làm lại thật chi tiết phần thư viện". Đợt sn-2 + sn-2b (2.499 mục), thư viện vẫn tắt.</t>
+        </is>
+      </c>
+      <c r="E146" s="8" t="inlineStr">
+        <is>
+          <t>1. Trích: tập tổ hợp chính tinh + sao lớn trên toàn kho, tập "sao + độ sáng", ngữ cảnh đoạn trước; prompt bắt độ sáng / cung / sao đi cùng / cách cục có tên
+2. Lược đồ: nhóm "ít nhất k trong số" (nhom) — bộ khớp, kiểm, khoá gộp
+3. Kiểm tất định: cặp chính tinh đồng cung phải có thật (dựng từ engine), không bỏ độ sáng, khớp gần nguyên văn, từ chỉ nhóm, tìm lại đoạn thật, độ sáng theo đề mục / ngữ cảnh trên văn CÓ DẤU
+4. Khâu chọn: ưu tiên sao lớn tại cung chính có độ sáng khớp, trần 18
+5. scripts/do-phu-dap-an.ts (cổng), scripts/do-tran-kien-thuc.ts (đo trần); 47 kiểm trong test-thu-vien</t>
+        </is>
+      </c>
+      <c r="F146" s="9" t="inlineStr">
+        <is>
+          <t>Chờ quyết định</t>
+        </is>
+      </c>
+      <c r="G146" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H146" s="8" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="I146" s="8" t="inlineStr">
+        <is>
+          <t>Chưa ai (cờ tắt)</t>
+        </is>
+      </c>
+      <c r="J146" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K146" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/*, scripts/dung-thu-vien.ts, scripts/do-phu-dap-an.ts, scripts/do-tran-kien-thuc.ts, scripts/do-thu-vien.ts, scripts/test-thu-vien.ts, KIEN-TRUC-LUAN-GIAI.md</t>
+        </is>
+      </c>
+      <c r="L146" s="8" t="inlineStr">
+        <is>
+          <t>Tắt</t>
+        </is>
+      </c>
+      <c r="M146" s="8" t="inlineStr">
+        <is>
+          <t>Qua kiểm tất định 38–54% → 87% (lượt thử), 71% / 76% (đủ). Độ sáng 8% → 33% mục. Phủ đáp án 26,6% → 49,4%; phủ có độ sáng 5,2% → 21% (cổng 30% đặt sai cấu trúc: đáp án gộp 3–7 sao/điểm). Nghiệm thu B3: KT luna 59,0 → 60,0, gpt-4o-mini 52,2 → 53,7; cách viết 49–50% → KHÔNG đạt. Đo trần (đưa thẳng đáp án cho người viết) CHƯA chạy được: OpenAI hết credit giữa chừng. Tốn lượt này: ~2,1 tr token vào dựng + ~2 tr sinh/chấm.</t>
+        </is>
+      </c>
+      <c r="N146" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O146" s="8" t="inlineStr">
+        <is>
+          <t>thu-vien-chi-tiet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17748,7 +17829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20135,6 +20216,38 @@
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B75" s="50" t="inlineStr">
+        <is>
+          <t>thu-vien-chi-tiet</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>CEL-146</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Thư viện lượt 2 chi tiết (2.499 mục, 33% có độ sáng); kiến thức vẫn phẳng; OpenAI hết credit.</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu làm lại thật chi tiết.</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Bat thu vien tri thuc cho 5 cau Su nghiep, doc theo goi, chi phi do lai
- CAU_THU_VIEN = SN01 SN02 SN03 SN05 SN06, dot sn-2,sn-2b (QD-16: chu du an tu nghiem thu)
- Dau kho theo cau: cau Su nghiep cu hien Tao ban moi, chi 5 cau + tom lai viet lai
- Thu vien doc theo goi moi dot: 11,6 s -> 0,6 s
- KIEN-TRUC muc 15: chi phi moi la so do lai
- CEL-147

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O146"/>
+  <dimension ref="A1:O147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12445,7 +12445,7 @@
       </c>
       <c r="F143" s="9" t="inlineStr">
         <is>
-          <t>Chờ quyết định</t>
+          <t>Đang chạy (bật 26/09, CEL-147)</t>
         </is>
       </c>
       <c r="G143" s="8" t="inlineStr">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="F146" s="9" t="inlineStr">
         <is>
-          <t>Chờ quyết định</t>
+          <t>Đang chạy (bật 26/09, CEL-147)</t>
         </is>
       </c>
       <c r="G146" s="8" t="inlineStr">
@@ -12730,6 +12730,86 @@
       <c r="O146" s="8" t="inlineStr">
         <is>
           <t>thu-vien-chi-tiet</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="13" t="inlineStr">
+        <is>
+          <t>CEL-147</t>
+        </is>
+      </c>
+      <c r="B147" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C147" s="8" t="inlineStr">
+        <is>
+          <t>BẬT thư viện tri thức cho 5 câu Sự nghiệp (chủ dự án tự nghiệm thu)</t>
+        </is>
+      </c>
+      <c r="D147" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 26/09/2026: "tính lại chi phí token của từng lá số, không thực hiện test nữa, đẩy thư viện lên và tôi sẽ tự check trên lá số". Bật dù lát cắt chưa đạt ngưỡng máy (QĐ-16).</t>
+        </is>
+      </c>
+      <c r="E147" s="8" t="inlineStr">
+        <is>
+          <t>1. Route: CAU_THU_VIEN = SN01, SN02, SN03, SN05, SN06; DOT_THU_VIEN = sn-2,sn-2b (2.499 mục)
+2. Dấu kho theo câu (khoMongDoi): câu Sự nghiệp viết trước khi bật hiện nút "Tạo bản mới"; chỉ 5 câu + tóm lại Sự nghiệp được viết lại
+3. Thư viện đọc theo GÓI mỗi đợt (một dòng noi_dung_ai khoá goi:&lt;đợt&gt;): 11,6 giây → 0,6 giây; dongGoi() dựng lại gói sau mỗi lần lưu
+4. Chi phí đo lại (KIEN-TRUC mục 15): mỗi câu 11.678 vào / 1.429 ra; cả lá số ~1,24 tr vào / ~150 nghìn ra (~8% ngày 25/09); thư viện làm Sự nghiệp +9% vào</t>
+        </is>
+      </c>
+      <c r="F147" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G147" s="8" t="inlineStr">
+        <is>
+          <t>AI + RAG</t>
+        </is>
+      </c>
+      <c r="H147" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt Sự nghiệp</t>
+        </is>
+      </c>
+      <c r="I147" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập (chuyên sâu)</t>
+        </is>
+      </c>
+      <c r="J147" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau (Sự nghiệp), /api/luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="K147" s="8" t="inlineStr">
+        <is>
+          <t>app/api/luan-giai-v3/route.ts, lib/rag/thu-vien/kho.ts, KIEN-TRUC-LUAN-GIAI.md</t>
+        </is>
+      </c>
+      <c r="L147" s="8" t="inlineStr">
+        <is>
+          <t>Bật (5 câu)</t>
+        </is>
+      </c>
+      <c r="M147" s="8" t="inlineStr">
+        <is>
+          <t>OpenAI đang HẾT CREDIT — chưa sinh được bài mới nào cho tới khi nạp. Cách tắt: xoá mã câu khỏi CAU_THU_VIEN. Máy đo trước đó: kiến thức +1 điểm, cách viết ngang — chủ dự án tự đánh giá. Lá số đã có bài Sự nghiệp: bấm "Tạo bản mới" ở cuối chủ đề để xem bản có thư viện (mỗi lá một lần).</t>
+        </is>
+      </c>
+      <c r="N147" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O147" s="8" t="inlineStr">
+        <is>
+          <t>bat-thu-vien-su-nghiep</t>
         </is>
       </c>
     </row>
@@ -17829,7 +17909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20248,6 +20328,38 @@
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B76" s="50" t="inlineStr">
+        <is>
+          <t>bat-thu-vien-su-nghiep</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>CEL-147</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Bật thư viện Sự nghiệp (sn-2, sn-2b) cho 5 câu; đọc theo gói; chi phí đo lại theo lá số.</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án tự nghiệm thu trên lá số thật.</t>
+        </is>
+      </c>
+      <c r="F76" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Giam chi phi goi API khong doi dau ra va giam chi phi test
- Sua cuc bo: loi khoanh duoc vao cau chi gui cac cau do (vong sua dang chiem 22% token ra)
- prompt_cache_key theo cau hoi / theo bam phan luat; khoi co dinh theo cau hoi dung truoc so y (prompt 2026.09.18)
- Ghi token dem + token suy nghi (usage v2, SQL va-chi-phi-token chua chay, tu lui)
- Test: tran ngan sach 1 tr + nhan @test, khong lui ngam sang luna, giam khao mac dinh gpt-4o-mini, dem phieu cham, dung som, mau tham do 6x3, Batch API, trich tang dan
- CEL-148

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O147"/>
+  <dimension ref="A1:O148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12813,6 +12813,87 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="13" t="inlineStr">
+        <is>
+          <t>CEL-148</t>
+        </is>
+      </c>
+      <c r="B148" s="14" t="inlineStr">
+        <is>
+          <t>I. Chi phí &amp; vận hành</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>Giảm chi phí gọi API (không đổi đầu ra) và chi phí test</t>
+        </is>
+      </c>
+      <c r="D148" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 26/09/2026: một lá số đọc trọn ~9 nghìn đồng, nhiều user không thu phí sẽ lỗ; test tốn quá nhiều token. Yêu cầu làm mọi giải pháp giảm chi phí mà không ảnh hưởng đầu ra.</t>
+        </is>
+      </c>
+      <c r="E148" s="8" t="inlineStr">
+        <is>
+          <t>SẢN PHẨM: 1. Sửa cục bộ — lỗi khoanh được vào câu chỉ gửi các câu ấy (sua-cuc-bo.ts; LoiV3.cum)
+2. prompt_cache_key: theo câu hỏi cho v3, theo băm phần luật cho mọi bề mặt (providers.ts); tự bỏ nếu cổng không nhận
+3. Thứ tự tiền tố: khối cố định theo câu hỏi trước sổ ý / dữ kiện (prompt 2026.09.18)
+4. Ghi token đệm + token suy nghĩ (usage.ts v2, supabase/va-chi-phi-token.sql — CHƯA chạy, mã tự lùi)
+TEST: trần ngân sách 1 tr / lượt + nhãn @test (thu-chung.ts); giám khảo không lùi ngầm sang luna; giám khảo mặc định gpt-4o-mini; đệm phiếu chấm; dừng sớm theo đợt 20 cặp; mẫu thăm dò 6×3 (--nghiem-thu cho 60 cặp); Batch API (batch-openai.ts, --batch); trích tăng dần (--bo-qua)</t>
+        </is>
+      </c>
+      <c r="F148" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G148" s="8" t="inlineStr">
+        <is>
+          <t>Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="H148" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt gọi</t>
+        </is>
+      </c>
+      <c r="I148" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J148" s="8" t="inlineStr">
+        <is>
+          <t>/api/luan-giai-v3 và mọi bề mặt gọi AI</t>
+        </is>
+      </c>
+      <c r="K148" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/sua-cuc-bo.ts, lib/rag/v3/index.ts, lib/rag/v3/kiem-v3.ts, lib/ai/providers.ts, lib/ai/types.ts, lib/ai/fallback.ts, lib/ai/usage.ts, lib/ai/batch-openai.ts, supabase/va-chi-phi-token.sql, scripts/thu-chung.ts, scripts/do-kien-thuc.ts, scripts/so-sanh-v3.ts, scripts/do-thu-vien.ts, scripts/dung-thu-vien.ts, scripts/test-sua-cuc-bo.ts</t>
+        </is>
+      </c>
+      <c r="L148" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M148" s="8" t="inlineStr">
+        <is>
+          <t>Số đo nền (60 câu): mỗi câu 1,25 lượt, 11.678 vào (41% đệm), 1.429 ra; token ra ~61% tiền, vòng sửa 22% token ra (30/37 ca lỗi một câu). Ước giảm ~20–25% mỗi câu (9 nghìn → ~7 nghìn / lá đọc trọn) — CHƯA đo được vì OpenAI hết credit; đo lại bằng 6 câu (~0,1 tr token). Test: một vòng A/B nghiệm thu ~3 tr → ~0,5 tr token (~0,25 tr với Batch). Sửa cục bộ chưa chạy thật với model — có đường lùi về sửa cả bài.</t>
+        </is>
+      </c>
+      <c r="N148" s="8" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="O148" s="8" t="inlineStr">
+        <is>
+          <t>giam-chi-phi-token</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17909,7 +17990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20360,6 +20441,38 @@
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B77" s="50" t="inlineStr">
+        <is>
+          <t>giam-chi-phi-token</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>CEL-148</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Sửa cục bộ, khoá đệm prompt, thứ tự tiền tố, sổ chi phí đủ; công cụ test tiết kiệm (ngân sách, đệm, dừng sớm, Batch).</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu giảm chi phí API và test mà không đổi đầu ra.</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Cau hinh AI Agent cho Claude Code
- .claude/agents: researcher (chi doc), celes-domain (tham dinh Tu Vi), qa (chay cong kiem, PASS/FAIL theo AC)
- .claude/skills/build-feature: Spec -> Research -> Domain -> Plan (dung cho duyet) -> Code -> QA
- specs/: README + mau spec
- .claude/settings.json: chan doc .env*.local, chan force push
- Khong doi ma chay

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -17990,7 +17990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20473,6 +20473,38 @@
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="49" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B78" s="50" t="inlineStr">
+        <is>
+          <t>agent-setup</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Cấu hình AI Agent cho Claude Code: .claude/agents (researcher, celes-domain, qa), skill /build-feature, specs/ (mẫu spec), .claude/settings.json chặn đọc .env và force push. Không đổi mã chạy.</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án chuyển sang phát triển theo spec + agent chuyên trách để giảm ngữ cảnh phiên chính và có cổng duyệt trước khi code.</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Giam token Claude Code
- AGENTS.md 28KB -> 9.3KB: bay da gap tach nguyen van sang docs/bay/*.md theo vung
- .claude/rules/*.md nap theo thu muc (paths), tro toi docs/bay
- .claude/settings.json: autoCompactWindow 200000, bashOutputMaxChars 12000 (da doi chieu schema Claude Code 2.1.283)
- Muc Tiet kiem ngu canh trong AGENTS.md cho moi AI

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -17990,7 +17990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20505,6 +20505,38 @@
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="49" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B79" s="50" t="inlineStr">
+        <is>
+          <t>giam-token</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Giảm token Claude Code: AGENTS.md 28KB → 9,3KB (bẫy tách sang docs/bay/*.md, nguyên văn); .claude/rules nạp theo thư mục; autoCompactWindow 200k; bashOutputMaxChars 12k; mục "Tiết kiệm ngữ cảnh" cho mọi AI.</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>Đo 15–26/09: 98% token là cache đọc lại, ngữ cảnh bình quân ~480k/lượt do phiên dài trên model 1M. AGENTS.md nạp lại mọi lượt.</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Giong van tu nhien theo ban mau chu du an sua tay
- Khoi GIONG_VAN trong system: cau ngan vua phai, moi doan mot y, cam cum mo ho / triet ly / ra don
- Chuyen sau 160-220 chu; bo luat khoanh khac dung qua va bieu hien + tinh huong + dieu kien
- Kiem cau-dai (>40 chu) di duong sua cuc bo
- Mau giong chu du an nap vao Supabase (mau-giong), khong vao repo; tom lai + buc tranh dung chung giong
- Do 4 cau: chu/cau 34 -> 26, cau >35 chu 38% -> 5%
- CEL-149

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O148"/>
+  <dimension ref="A1:O149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12894,6 +12894,87 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" s="13" t="inlineStr">
+        <is>
+          <t>CEL-149</t>
+        </is>
+      </c>
+      <c r="B149" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>Giọng văn tự nhiên theo bản mẫu chủ dự án sửa tay</t>
+        </is>
+      </c>
+      <c r="D149" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 27/09/2026 gửi 88 câu luận giải sửa tay: "câu ngắn vừa phải, rõ nghĩa, tự nhiên như người thật đang luận; không hoa mỹ, không cố triết lý, không dùng cụm mơ hồ; mỗi đoạn một ý chính, đi thẳng vào điều người xem muốn biết".</t>
+        </is>
+      </c>
+      <c r="E149" s="8" t="inlineStr">
+        <is>
+          <t>1. Khối GIONG_VAN trong system (cố định, được đệm): câu 12–25 chữ, tối đa 35; mỗi đoạn một ý 3–4 câu; danh sách cụm mơ hồ cấm; không câu triết lý / gây ấn tượng / rào đón
+2. Chuyên sâu 160–220 chữ (trần kiểm 280, trước 230–300 / 360); bỏ luật "khoảnh khắc đúng quá" và "biểu hiện + tình huống + điều kiện"
+3. Bộ kiểm cau-dai (&gt; 40 chữ) — đi đường sửa cục bộ
+4. Mẫu giọng: 3 bài chủ dự án sửa tay (SN02, TB01, QN02) nạp vào Supabase (mau-giong), đọc vào system; repo không chứa văn của lá số thật (scripts/nap-mau-giong.ts)
+5. Tóm lại và Bức tranh lớn dùng cùng khối giọng văn</t>
+        </is>
+      </c>
+      <c r="F149" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G149" s="8" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H149" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt luận giải</t>
+        </is>
+      </c>
+      <c r="I149" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J149" s="8" t="inlineStr">
+        <is>
+          <t>/api/luan-giai-v3</t>
+        </is>
+      </c>
+      <c r="K149" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/prompt-v3.ts, lib/rag/v3/mau-giong.ts, lib/rag/v3/index.ts, lib/rag/v3/kiem-v3.ts, lib/rag/v3/tom-lai.ts, lib/rag/v3/buc-tranh.ts, lib/rag/noi-dung-ai.ts, scripts/nap-mau-giong.ts</t>
+        </is>
+      </c>
+      <c r="L149" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M149" s="8" t="inlineStr">
+        <is>
+          <t>Đo 4 câu trên lá số chủ dự án (câu không có trong mẫu): chữ/bài 358 → 257 (mẫu 231); chữ/câu 34,1 → 26,3 (mẫu 23,1); câu &gt; 35 chữ 38% → 5% (mẫu 5%); dấu phẩy/câu 1,60 → 1,26. Token ra giảm ~15%. Sửa cục bộ lần đầu chạy thật: tách câu dài, +12 token ra. Tốn ~95 nghìn token cho 2 lượt thử. Chỉ áp bài sinh MỚI — bài đã lưu giữ nguyên tới khi viết lại.</t>
+        </is>
+      </c>
+      <c r="N149" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="O149" s="8" t="inlineStr">
+        <is>
+          <t>giong-van-tu-nhien</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17990,7 +18071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20537,6 +20618,38 @@
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="49" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B80" s="50" t="inlineStr">
+        <is>
+          <t>giong-van-tu-nhien</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>CEL-149</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Giọng văn tự nhiên: luật câu ngắn / mỗi đoạn một ý, bỏ luật gây câu dài, mẫu giọng từ Supabase, kiểm câu dài.</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án gửi bản mẫu sửa tay và mô tả giọng văn mong muốn.</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Core Web Vitals dot 2: chong dich bo cuc, supabase nap khi can, tuong phan
- main min-h-svh; khung cho /la-so, nut Quay lai, khoi SSO, the /home giu cho -> CLS ~0
- supabase-js nap khi can (dynamic import), -67KB khoi goi dau moi trang
- La so mau trang chu tinh san o may chu, engine nap khi bam
- --accent-chu: chu hong dat 4.5:1 ca Ngay lan Dem
- Backlog: CEL-150

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O149"/>
+  <dimension ref="A1:O150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12975,6 +12975,83 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="13" t="inlineStr">
+        <is>
+          <t>CEL-150</t>
+        </is>
+      </c>
+      <c r="B150" s="14" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>Core Web Vitals + a11y + SEO theo đo Lighthouse production</t>
+        </is>
+      </c>
+      <c r="D150" s="8" t="inlineStr">
+        <is>
+          <t>Đo 27/09/2026 (Lighthouse production, mobile): không trang nào đạt đủ 3 Core Web Vitals; /la-so CLS 0,34, LCP 3,5–4,9s; lỗi 401 console; thứ bậc tiêu đề sai; không có sitemap/robots.</t>
+        </is>
+      </c>
+      <c r="E150" s="8" t="inlineStr">
+        <is>
+          <t>1. Font tự phục vụ 1 file latin+Việt / họ chữ (240→116KB), bỏ preload font trang trí. 2. experimental.inlineCss. 3. main min-h-svh + khung chờ /la-so, nút Quay lại, khối SSO, thẻ /home giữ chỗ → CLS về ~0. 4. supabase-js nạp khi cần (−67KB khỏi gói đầu). 5. Lá số mẫu trang chủ tính sẵn ở máy chủ, engine nạp khi bấm. 6. /la-so chỉ gọi diem-noi-bat khi thẻ đó hiện (hết 401, bớt 1 lượt model/ngày). 7. --accent-chu cho chữ hồng đạt 4,5:1 (Ngày/Đêm). 8. h2 cho Eyebrow/GocNhinCard, aria-label nút ngôn ngữ, mô tả ẩn nút header. 9. sitemap.ts, robots.ts.</t>
+        </is>
+      </c>
+      <c r="F150" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G150" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện</t>
+        </is>
+      </c>
+      <c r="H150" s="8" t="inlineStr">
+        <is>
+          <t>Bớt 1 lượt model/ngày/lá số</t>
+        </is>
+      </c>
+      <c r="I150" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J150" s="8" t="inlineStr">
+        <is>
+          <t>Mọi trang</t>
+        </is>
+      </c>
+      <c r="K150" s="8" t="inlineStr">
+        <is>
+          <t>app/layout.tsx, next.config.ts, app/fonts/*, app/la-so/page.tsx, app/dang-nhap/page.tsx, components/QuayLai.tsx, components/SiteNav.tsx, lib/supabase/client.ts, lib/tuvi/la-so-mau.ts, app/globals.css, app/sitemap.ts, app/robots.ts</t>
+        </is>
+      </c>
+      <c r="L150" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M150" s="8" t="inlineStr">
+        <is>
+          <t>Đo trên máy (mobile, Lighthouse): A11y/BP/SEO 100 cả 12 lượt; CLS ≤0,016 (trừ trang chủ EN 0,112); Perf 82–97. CÒN LẠI: LCP trang cần đăng nhập 4–4,8s và đổi Việt→Anh sau hydrate — cần tách route [lang] (chưa làm, chờ chủ dự án).</t>
+        </is>
+      </c>
+      <c r="N150" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="O150" s="8" t="inlineStr">
+        <is>
+          <t>core-web-vitals</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -18071,7 +18148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20650,6 +20727,38 @@
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="49" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B81" s="50" t="inlineStr">
+        <is>
+          <t>core-web-vitals</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>CEL-150</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Cải thiện Core Web Vitals, a11y, SEO (font, CSS, CLS, supabase nạp khi cần, 401, tương phản).</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án: mục tiêu đạt điểm tốt tất cả các phần.</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Sua mat tri nho hoi thoai Hoi Celes khi bam chip goi y thu hai, keo dai gioi han ghi nho
- laTiepTuChip: client bao chac chan cau hoi den tu chip goi y, khong doan bang chu
- SO_CAP_GIU_KHI_NOI_TIEP 1 -> 3 cap (tiep-noi.ts): mach dang noi khong con mat cau hoi goc chi sau 1 luot
- Tran lich su vao route.ts 10 -> 60 tin nhan; SO_LUOT_DOC 20 -> 60; gomDieuTuKe 5 -> 8 su viec
- Gop bai kiem vao test-rag-planner.ts (TRI NHO HOI THOAI), khong tao file test rieng
- Da kiem bang API that (~115 nghin token): lay dung ca kich ban da bao loi va kich ban keo dai
- Sua tieu de + mo ta trang Ket noi
- CEL-150, CEL-151

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O150"/>
+  <dimension ref="A1:O152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13052,6 +13052,168 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="13" t="inlineStr">
+        <is>
+          <t>CEL-150</t>
+        </is>
+      </c>
+      <c r="B151" s="14" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t>Sửa mất trí nhớ hội thoại khi bấm chip gợi ý thứ hai + kéo dài ghi nhớ</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 27/09/2026: hỏi câu 1, bấm chip Celes gợi ý (lượt 2) thì còn nhớ ngữ cảnh; bấm tiếp chip gợi ý thứ hai (lượt 3) thì QUÊN — trả lời đúng câu chữ nhưng lạc mạch. Sau đó chủ dự án hỏi thêm: kéo dài ghi nhớ được tối đa bao nhiêu, cho phép gọi API thật để kiểm.</t>
+        </is>
+      </c>
+      <c r="E151" s="8" t="inlineStr">
+        <is>
+          <t>NGUYÊN NHÂN GỐC (2 lớp cộng dồn):
+1. `laCauNoiTiep` (tiep-noi.ts) đoán câu nối bằng chữ (đại từ trỏ ngược / ≤5 từ). Nhiều chip hợp lệ là câu hỏi trọn vẹn trên 5 từ ("Vậy tôi có nên chuyển việc không?") nên bị xếp NHẦM là "chủ đề mới" ngay từ lượt nó được hỏi → xoá sạch trí nhớ đúng lượt đó.
+2. Cửa sổ "mạch đang nói dở" cũ chỉ giữ 1 cặp — dù được nhận đúng là câu nối, tới lượt 3 thì câu hỏi GỐC ở lượt 1 đã rơi khỏi cửa sổ.
+SỬA:
+1. Client gửi kèm cờ `tuChip` khi câu hỏi đến từ nút chip goiYTiep (biết chắc, không cần đoán) → server ép `laTiepTuChip=true`, bỏ qua hẳn việc đoán bằng chữ cho lượt đó
+2. Cửa sổ "mạch đang nói dở" 1 → 3 cặp (SO_CAP_GIU_KHI_NOI_TIEP, tiep-noi.ts)
+3. Trần lịch sử vào route.ts: 10 → 60 tin nhắn; SO_LUOT_DOC (đọc lại khi mở trang): 20 → 60 — an toàn vì mảng đầy chỉ nuôi gomDieuTuKe (quét bằng luật, không gọi model) và machDangNoi (vẫn bị cắt còn 3 cặp dù mảng vào dài bao nhiêu)
+4. gomDieuTuKe: trần nhớ đồng thời 5 → 8 sự việc tự kể
+5. Gộp bài kiểm vào scripts/test-rag-planner.ts (mục TRÍ NHỚ HỘI THOẠI) — không tạo tệp test riêng</t>
+        </is>
+      </c>
+      <c r="F151" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G151" s="8" t="inlineStr">
+        <is>
+          <t>Luật thuần (không gọi model, trừ đúng lượt trả lời)</t>
+        </is>
+      </c>
+      <c r="H151" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt Hỏi Celes</t>
+        </is>
+      </c>
+      <c r="I151" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="J151" s="8" t="inlineStr">
+        <is>
+          <t>/hoi-dap, /api/hoi-dap</t>
+        </is>
+      </c>
+      <c r="K151" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/tiep-noi.ts, lib/rag/prompt-co-can-cu.ts, lib/rag/tra-loi.ts, app/api/hoi-dap/route.ts, app/hoi-dap/page.tsx, lib/store/hoi-thoai.ts, scripts/test-rag-planner.ts</t>
+        </is>
+      </c>
+      <c r="L151" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M151" s="8" t="inlineStr">
+        <is>
+          <t>ĐÃ KIỂM bằng API thật (lá số tổng hợp, không phải người thật; ~115 nghìn token): mô phỏng đúng kịch bản đã báo (hỏi 1 → chip 1 → chip 2) — lượt 3 bám đúng mạch "sự nghiệp/chuyển việc"; kéo dài thêm 3 lượt đổi chủ đề (tình duyên, tiền, sức khoẻ) rồi quay lại — vẫn nhớ đúng "công ty 200 người, làm 3 năm" kể từ lượt 4 và trả lời đúng ngữ cảnh đó. PHÁT HIỆN PHỤ (chưa sửa, không liên quan trí nhớ): một lượt trong phiên thử trả về `van` rỗng kèm goiYTiep rỗng — cần rà riêng, có thể là JSON gãy hoặc kiemDuyet lọc sạch yChinh. Giới hạn còn lại: câu nối tiếp do người TỰ GÕ (không qua chip) vẫn phụ thuộc heuristic chữ cũ — chỉ chip mới có cờ chắc chắn.</t>
+        </is>
+      </c>
+      <c r="N151" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="O151" s="8" t="inlineStr">
+        <is>
+          <t>tri-nho-hoi-celes</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="13" t="inlineStr">
+        <is>
+          <t>CEL-151</t>
+        </is>
+      </c>
+      <c r="B152" s="14" t="inlineStr">
+        <is>
+          <t>F. Trang &amp; điều hướng</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>Đổi tiêu đề và mô tả trang Kết nối</t>
+        </is>
+      </c>
+      <c r="D152" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 27/09/2026: đổi tiêu đề "Hai người gặp nhau ở đâu — và dễ lệch nhau ở đâu?" thành "Hai người có hợp nhau không?" và đổi mô tả bên dưới.</t>
+        </is>
+      </c>
+      <c r="E152" s="8" t="inlineStr">
+        <is>
+          <t>app/hop-tuoi/page.tsx: đổi thẳng chuỗi tiêu đề (h1) và mô tả (p ngay dưới) trong JSX — không phải chuỗi trong bảng i18n vì trang Kết nối chưa dùng useT() cho hai chỗ này.</t>
+        </is>
+      </c>
+      <c r="F152" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G152" s="8" t="inlineStr">
+        <is>
+          <t>Tất định (chỉ đổi chữ)</t>
+        </is>
+      </c>
+      <c r="H152" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I152" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J152" s="8" t="inlineStr">
+        <is>
+          <t>/hop-tuoi</t>
+        </is>
+      </c>
+      <c r="K152" s="8" t="inlineStr">
+        <is>
+          <t>app/hop-tuoi/page.tsx</t>
+        </is>
+      </c>
+      <c r="L152" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M152" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ đổi văn bản hiển thị, không đụng logic.</t>
+        </is>
+      </c>
+      <c r="N152" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="O152" s="8" t="inlineStr">
+        <is>
+          <t>tri-nho-hoi-celes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -18148,7 +18310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20761,6 +20923,38 @@
       <c r="F81" s="8" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="49" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B82" s="50" t="inlineStr">
+        <is>
+          <t>tri-nho-hoi-celes</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>CEL-150, CEL-151</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Sửa mất trí nhớ hội thoại Hỏi Celes khi bấm chip gợi ý thứ hai (cờ tuChip + cửa sổ mạch đang nói dở 1→3 cặp); nâng trần ghi nhớ (10→60 tin nhắn, 5→8 sự việc tự kể). Đổi tiêu đề/mô tả trang Kết nối.</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án báo lỗi thật khi test chat; sau đó yêu cầu kéo dài ghi nhớ và cho phép kiểm bằng API thật.</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sua bong bong chat TRANG o Hoi Celes khi model tra JSON gay
- tra-loi.ts: thu lai nguyen luot 1 lan khi van ban tho trong nhu JSON ma doc khong duoc
- route.ts: van rong = luot hong -> hoan lai luot (hoanCauHoi, khong goi chotCauHoi), tra 502 kem loi ro, thay vi 200 rong
- Da ra toan bo be mat AI khac: khong co loi tuong tu (cac be mat khac da tra loi ro hoac im lang giu ban tat dinh la dung thiet ke)
- CEL-152

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O152"/>
+  <dimension ref="A1:O153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13214,6 +13214,85 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" s="13" t="inlineStr">
+        <is>
+          <t>CEL-152</t>
+        </is>
+      </c>
+      <c r="B153" s="14" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t>Sửa bong bóng chat TRẮNG khi model trả JSON gãy — hoàn lượt cho người dùng</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu rà kỹ sau khi thấy một lượt trong phiên kiểm CEL-150 trả lời rỗng. Dựng lại đúng bối cảnh 6 lần bằng API thật KHÔNG tái hiện được — đây là một lần hỏng hiếm ở phía model (JSON gãy giữa chừng), không phải lỗi do CEL-150 gây ra. Nhưng đường xử lý của route thì sai thật: `traLoiCoCanCu` cố ý trả `van: ''` khi văn bản thô trông như JSON mà đọc không được (đúng thiết kế — JSON dở dang còn tệ hơn không có gì), nhưng route trước đó ship thẳng chuỗi rỗng ấy như một câu trả lời thành công (HTTP 200): người dùng thấy bong bóng TRẮNG, không lỗi, không chip, không cách hỏi lại — và lượt hỏi của họ vẫn bị trừ.</t>
+        </is>
+      </c>
+      <c r="E153" s="8" t="inlineStr">
+        <is>
+          <t>1. lib/rag/tra-loi.ts: JSON gãy thì THỬ LẠI nguyên lượt một lần trước khi bỏ cuộc (cùng cách lib/rag/v3/index.ts đã làm cho luận giải chuyên sâu) — giảm tần suất phải rơi vào nhánh lỗi
+2. app/api/hoi-dap/route.ts: `kq.van` rỗng thì coi là lượt gọi HỎNG — hoàn lại lượt (hoanCauHoi, KHÔNG gọi chotCauHoi) và trả 502 kèm lời nhắn hỏi lại, thay vì 200 rỗng
+3. Đã RÀ TOÀN BỘ các bề mặt gọi AI khác (bang-linh-vuc, be-mat-ngan, moc-hanh-trinh, ban-doc-sau, bai-dai, luan-giai-v3): mọi bề mặt khác đều đã đúng — trả lỗi rõ ràng (bài dài, luận giải chuyên sâu), hoặc là nội dung nền có sẵn bản tất định/thẻ cũ nên lặng lẽ giữ nguyên khi hỏng là ĐÚNG thiết kế (điểm nổi bật, nhịp hiện tại, mốc hành trình, bảng lĩnh vực) — không sửa gì thêm ở đó</t>
+        </is>
+      </c>
+      <c r="F153" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G153" s="8" t="inlineStr">
+        <is>
+          <t>Không đổi (chỉ xử lý khi hỏng)</t>
+        </is>
+      </c>
+      <c r="H153" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt Hỏi Celes</t>
+        </is>
+      </c>
+      <c r="I153" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="J153" s="8" t="inlineStr">
+        <is>
+          <t>/api/hoi-dap</t>
+        </is>
+      </c>
+      <c r="K153" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/tra-loi.ts, app/api/hoi-dap/route.ts</t>
+        </is>
+      </c>
+      <c r="L153" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M153" s="8" t="inlineStr">
+        <is>
+          <t>Cơ chế hoàn lượt xác nhận đúng qua SQL `hoan_cau_hoi` (chỉ hoàn khi trạng thái vẫn "reserved" — route không gọi chotCauHoi trước nên không xung đột). Chưa tái hiện được lỗi gốc để kiểm trực tiếp nhánh 502 mới bằng API thật (đã thử 6 lần, cùng bối cảnh, model luôn trả JSON hợp lệ) — đã xác nhận đúng bằng đọc mã và đối chiếu với nhánh catch lỗi hiện có (cùng một khuôn).</t>
+        </is>
+      </c>
+      <c r="N153" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="O153" s="8" t="inlineStr">
+        <is>
+          <t>sua-bong-bong-trang-hoi-celes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -18310,7 +18389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20953,6 +21032,38 @@
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="49" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B83" s="50" t="inlineStr">
+        <is>
+          <t>sua-bong-bong-trang-hoi-celes</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>CEL-152</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Sửa bong bóng chat trắng khi model trả JSON gãy ở Hỏi Celes: thử lại một lần, hoàn lượt và báo lỗi rõ nếu vẫn hỏng. Rà toàn bộ các bề mặt AI khác — không có lỗi tương tự.</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu rà lại toàn bộ sau khi phát hiện một lượt trả lời rỗng trong lúc kiểm CEL-150.</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
         <is>
           <t>Claude Sonnet 5</t>
         </is>

</xml_diff>

<commit_message>
App di dong GD1 moc 1: token theo design system web, doi ten tab Moi quan he
- token.ts: bo goc the 14/16, nut 8, o nhap 6, nut #D32298, eyebrow 12
- Tab Ket noi -> Moi quan he o ca app va web (nav, eyebrow, tieu de /hop-tuoi)
- AGENTS.md: go trang thai tam dung app, ghi cac quyet dinh da chot
- CEL-153

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O153"/>
+  <dimension ref="A1:O154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13293,6 +13293,86 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" s="13" t="inlineStr">
+        <is>
+          <t>CEL-153</t>
+        </is>
+      </c>
+      <c r="B154" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t>App iOS/Android GĐ1 — mốc 1: nền theo design system web, mở lại app, đổi tên "Mối quan hệ"</t>
+        </is>
+      </c>
+      <c r="D154" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án 27/09/2026: dựng app iOS (một bộ code cho cả Android), lên store sau không phải sửa; giao diện dùng design system web nhưng luồng riêng, cá nhân hoá hơn. Đã duyệt 12 màn trên canvas "Celes iOS — luồng app" sau một vòng phản biện. Thanh toán tạm ẩn trên iOS. Làm bản nội bộ trước.</t>
+        </is>
+      </c>
+      <c r="E154" s="8" t="inlineStr">
+        <is>
+          <t>1. apps/celes-app/src/thiet-ke/token.ts: bo góc theo web (thẻ 14/16, nút 8, ô nhập 6, sheet 20), nút hành động #D32298 (web), thêm fuchsiaChu #B62B8B, eyebrow 12px
+2. Tab thứ tư "Kết nối" → "Mối quan hệ" ở cả app (i18n app) và web (nav, eyebrow, tiêu đề trang /hop-tuoi)
+3. AGENTS.md: gỡ "app ĐANG TẠM DỪNG", ghi các quyết định đã chốt
+Các mốc sau: backend nhận đăng nhập từ app (Bearer), đăng nhập trong app, nối nội dung v3, dựng lại các màn theo canvas (lá số đầy đủ, radar mạnh–yếu, Hôm nay, bài đọc, Hành trình trục thời gian).</t>
+        </is>
+      </c>
+      <c r="F154" s="9" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
+      </c>
+      <c r="G154" s="8" t="inlineStr">
+        <is>
+          <t>Không đổi</t>
+        </is>
+      </c>
+      <c r="H154" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I154" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J154" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app, /hop-tuoi, thanh điều hướng web</t>
+        </is>
+      </c>
+      <c r="K154" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/thiet-ke/token.ts, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts, lib/i18n/vi.ts, lib/i18n/en.ts, app/hop-tuoi/page.tsx, app/hop-tuoi/layout.tsx, AGENTS.md</t>
+        </is>
+      </c>
+      <c r="L154" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M154" s="8" t="inlineStr">
+        <is>
+          <t>App: tsc sạch, xuất bundle iOS được (4,2 MB). Web: tsc, eslint (5 lỗi cũ), test-rag-planner, next build đều qua.</t>
+        </is>
+      </c>
+      <c r="N154" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="O154" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-moc1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -18389,7 +18469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21066,6 +21146,38 @@
       <c r="F83" s="8" t="inlineStr">
         <is>
           <t>Claude Sonnet 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="49" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B84" s="50" t="inlineStr">
+        <is>
+          <t>app-gd1-moc1</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>CEL-153</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Mở lại app di động (GĐ1 mốc 1): token app theo web, đổi tên tab "Mối quan hệ" cả app lẫn web.</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt luồng app trên canvas và yêu cầu bắt đầu code.</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
May chu nhan token dang nhap qua header Bearer cho app di dong
App di dong khong co cookie cua web nen khong dung chung duoc han muc,
bac quyen va du lieu. nguoiDungHienTai / taoSupabaseServer nay nhan them
'Authorization: Bearer <access token Supabase>': token duoc Supabase xac
thuc (auth.getUser(token)), roi client dung tu chinh token do de RLS chay
duoi dung nguoi dung. Khong co header thi web di duong cookie nhu cu.

Da kiem: khong token / token rac / JWT gia mao chu ky deu la khach, tuyen
bat buoc dang nhap tra 401, khong loi 500. tsc sach, eslint 5 loi cu,
next build qua. Chua kiem token hop le (khong co tai khoan thu).

Nua phia app chua lam: app chua co dang nhap nen chua co token de gui.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O154"/>
+  <dimension ref="A1:O155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13373,6 +13373,86 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" s="13" t="inlineStr">
+        <is>
+          <t>CEL-154</t>
+        </is>
+      </c>
+      <c r="B155" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>App gọi API bằng token đăng nhập (Bearer)</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="inlineStr">
+        <is>
+          <t>App di động không có cookie của web. Máy chủ nay nhận thêm header Authorization: Bearer &lt;access token Supabase&gt; ở mọi tuyến đi qua nguoiDungHienTai / taoSupabaseServer, nên app sẽ dùng chung hạn mức, bậc quyền và dữ liệu với web.</t>
+        </is>
+      </c>
+      <c r="E155" s="8" t="inlineStr">
+        <is>
+          <t>1. lib/supabase/server.ts đọc header Authorization
+2. Có Bearer → auth.getUser(token) hỏi Supabase xác thực chữ ký + hạn
+3. Client Supabase dựng từ token → RLS chạy dưới đúng người đó
+4. Không có header → đường cookie của web như cũ</t>
+        </is>
+      </c>
+      <c r="F155" s="9" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="G155" s="8" t="inlineStr">
+        <is>
+          <t>Không đổi</t>
+        </is>
+      </c>
+      <c r="H155" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I155" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J155" s="8" t="inlineStr">
+        <is>
+          <t>/api/entitlements/me, /api/support/*, /api/hoi-dap …</t>
+        </is>
+      </c>
+      <c r="K155" s="8" t="inlineStr">
+        <is>
+          <t>lib/supabase/server.ts</t>
+        </is>
+      </c>
+      <c r="L155" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M155" s="8" t="inlineStr">
+        <is>
+          <t>Mới xong nửa máy chủ. App CHƯA có đăng nhập (nút ở màn đăng ký vẫn là 'Để sau') nên chưa có token để gửi. Đã kiểm: không token / token rác / JWT giả mạo chữ ký đều bị coi là khách (401 ở tuyến bắt buộc đăng nhập), không lỗi 500. Chưa kiểm được token hợp lệ vì không có tài khoản thử.</t>
+        </is>
+      </c>
+      <c r="N155" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="O155" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-bearer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -13390,7 +13470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17557,76 +17637,76 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="35" t="inlineStr">
+      <c r="A117" s="30" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="B117" s="31" t="inlineStr">
+        <is>
+          <t>Bậc quyền &amp; cổng</t>
+        </is>
+      </c>
+      <c r="C117" s="31" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="inlineStr">
+        <is>
+          <t>Nhận diện người dùng: cookie (web) hoặc Bearer (app)</t>
+        </is>
+      </c>
+      <c r="E117" s="8" t="inlineStr">
+        <is>
+          <t>nguoiDungHienTai(): có header 'Authorization: Bearer &lt;token&gt;' thì gọi auth.getUser(token) — Supabase xác thực chữ ký và hạn dùng — rồi dựng client từ chính token đó để RLS chạy dưới đúng người dùng. Không có header thì đi đường cookie như cũ. Token sai/hết hạn = khách, không phải lỗi.</t>
+        </is>
+      </c>
+      <c r="F117" s="32" t="inlineStr">
+        <is>
+          <t>KHÔNG bao giờ tự giải mã JWT rồi tin 'sub' — luôn để Supabase xác thực. Web không bật CORS, nên trang lạ không gửi được header này sang (header tuỳ biến bắt preflight). Các tuyến cron cũng nhận 'Bearer &lt;CRON_SECRET&gt;' nhưng chỉ dùng client admin, không đi qua nguoiDungHienTai — đừng nối chúng vào hàm này, kẻo secret bị gửi sang Supabase.</t>
+        </is>
+      </c>
+      <c r="G117" s="8" t="inlineStr">
+        <is>
+          <t>lib/supabase/server.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="35" t="inlineStr">
         <is>
           <t>L12</t>
         </is>
       </c>
-      <c r="B117" s="36" t="inlineStr">
+      <c r="B118" s="36" t="inlineStr">
         <is>
           <t>Góc nhìn nhanh (không AI)</t>
         </is>
       </c>
-      <c r="C117" s="36" t="inlineStr">
+      <c r="C118" s="36" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D117" s="8" t="inlineStr">
+      <c r="D118" s="8" t="inlineStr">
         <is>
           <t>Nút sang bài luận giải sâu dời lên đầu trang</t>
         </is>
       </c>
-      <c r="E117" s="8" t="inlineStr">
+      <c r="E118" s="8" t="inlineStr">
         <is>
           <t>Khối nổi bật đặt ngay sau thẻ góc nhìn chính, dùng nút CHÍNH. Thẻ cuối trang bỏ nút trùng, chỉ còn Hỏi Celes.</t>
         </is>
       </c>
-      <c r="F117" s="32" t="inlineStr">
+      <c r="F118" s="32" t="inlineStr">
         <is>
           <t>Trước đó nút nằm dưới cùng, sau cả bảng mười hai phần, dạng nút viền nhạt cạnh một nút khác — người dùng đọc hết trang mà không nhận ra đây là phần sâu nhất sản phẩm có. Để nguyên ở cả hai chỗ là hiện cùng một lời mời hai lần trong một màn, và cái ở đầu mất sức nặng.</t>
         </is>
       </c>
-      <c r="G117" s="8" t="inlineStr">
+      <c r="G118" s="8" t="inlineStr">
         <is>
           <t>app/la-so/page.tsx, lib/i18n/vi.ts, lib/i18n/en.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="30" t="inlineStr">
-        <is>
-          <t>L15</t>
-        </is>
-      </c>
-      <c r="B118" s="31" t="inlineStr">
-        <is>
-          <t>Bản đọc sâu 12 cung</t>
-        </is>
-      </c>
-      <c r="C118" s="31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D118" s="8" t="inlineStr">
-        <is>
-          <t>Bảng 77 tiêu chí bóc bằng máy từ spec</t>
-        </is>
-      </c>
-      <c r="E118" s="8" t="inlineStr">
-        <is>
-          <t>Bộ bóc đọc mục 4 của spec, tách từng phần theo tiêu đề "### x.y `mucId`", lấy khối "**CS (k)**", đối chiếu số khai với số dòng đếm được, và CHẶN nếu một phần không có đúng một tiêu chí [GƯƠNG].</t>
-        </is>
-      </c>
-      <c r="F118" s="32" t="inlineStr">
-        <is>
-          <t>Chép tay 77 dòng là chắc chắn sai. Bóc bằng máy thì sai cũng sai có hệ thống, và kiểm lại được bằng phép đếm. Spec đổi thì chạy lại bộ bóc, không sửa tay.</t>
-        </is>
-      </c>
-      <c r="G118" s="8" t="inlineStr">
-        <is>
-          <t>lib/tuvi/tieu-chi-sau.ts</t>
         </is>
       </c>
     </row>
@@ -17643,254 +17723,254 @@
       </c>
       <c r="C119" s="31" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="inlineStr">
+        <is>
+          <t>Bảng 77 tiêu chí bóc bằng máy từ spec</t>
+        </is>
+      </c>
+      <c r="E119" s="8" t="inlineStr">
+        <is>
+          <t>Bộ bóc đọc mục 4 của spec, tách từng phần theo tiêu đề "### x.y `mucId`", lấy khối "**CS (k)**", đối chiếu số khai với số dòng đếm được, và CHẶN nếu một phần không có đúng một tiêu chí [GƯƠNG].</t>
+        </is>
+      </c>
+      <c r="F119" s="32" t="inlineStr">
+        <is>
+          <t>Chép tay 77 dòng là chắc chắn sai. Bóc bằng máy thì sai cũng sai có hệ thống, và kiểm lại được bằng phép đếm. Spec đổi thì chạy lại bộ bóc, không sửa tay.</t>
+        </is>
+      </c>
+      <c r="G119" s="8" t="inlineStr">
+        <is>
+          <t>lib/tuvi/tieu-chi-sau.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="30" t="inlineStr">
+        <is>
+          <t>L15</t>
+        </is>
+      </c>
+      <c r="B120" s="31" t="inlineStr">
+        <is>
+          <t>Bản đọc sâu 12 cung</t>
+        </is>
+      </c>
+      <c r="C120" s="31" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D119" s="8" t="inlineStr">
+      <c r="D120" s="8" t="inlineStr">
         <is>
           <t>Sinh theo CHẶNG, bốn lượt gọi</t>
         </is>
       </c>
-      <c r="E119" s="8" t="inlineStr">
+      <c r="E120" s="8" t="inlineStr">
         <is>
           <t>Mỗi lượt dựng ba phần của một chặng cùng doanKhau và cauBacCau. Prompt mang bảng tiêu chí kèm ngân sách từ tính theo độ nổi bật, cờ [KHỐI GƯƠNG], và ràng buộc an toàn riêng cho tat-ach / phu-mau / phu-the / no-boc.</t>
         </is>
       </c>
-      <c r="F119" s="32" t="inlineStr">
+      <c r="F120" s="32" t="inlineStr">
         <is>
           <t>Cả bài là ~6.000 từ ≈ 15 nghìn token đầu ra — không model nào trả nổi trong một lượt, và nếu trả được thì cũng chạm trần 55 giây.
 Chia nhỏ HƠN NỮA (mỗi phần một lượt) thì mất mạch: ba phần trong một chặng phải biết nhau để đoạn khâu nói được "ba phần này cùng nói điều gì".
 Ghép tiêu chí theo NHÃN CHUẨN chứ không theo thứ tự model trả về: model bỏ sót một tiêu chí là chuyện thường, và ghép theo thứ tự thì cờ laGuong dán nhầm đoạn — khối đảo màu khi đó nói về một thứ không phải gương.</t>
         </is>
       </c>
-      <c r="G119" s="8" t="inlineStr">
+      <c r="G120" s="8" t="inlineStr">
         <is>
           <t>lib/rag/ban-doc-sau.ts</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="30" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="30" t="inlineStr">
         <is>
           <t>L15</t>
         </is>
       </c>
-      <c r="B120" s="31" t="inlineStr">
+      <c r="B121" s="31" t="inlineStr">
         <is>
           <t>Bản đọc sâu 12 cung</t>
         </is>
       </c>
-      <c r="C120" s="31" t="inlineStr">
+      <c r="C121" s="31" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D120" s="8" t="inlineStr">
+      <c r="D121" s="8" t="inlineStr">
         <is>
           <t>Bốn lượt gọi HTTP thay cho SSE</t>
         </is>
       </c>
-      <c r="E120" s="8" t="inlineStr">
+      <c r="E121" s="8" t="inlineStr">
         <is>
           <t>POST /api/ban-doc-sau nhận tham số `chang`, đệm riêng từng chặng theo khoá (lá số, chặng, năm, phiên bản). Giao diện gọi tuần tự và vẽ ngay khi mỗi chặng về.</t>
         </is>
       </c>
-      <c r="F120" s="32" t="inlineStr">
+      <c r="F121" s="32" t="inlineStr">
         <is>
           <t>Spec mục 9 đòi SSE. SSE KHÔNG cứu được ràng buộc thật: maxDuration trên Vercel là 60 giây và nó giết hàm bất kể hàm ấy đang phát dở hay không. Đo được: cả bài 153 giây, chặng 1 xong ở giây 42 rồi ba chặng còn lại không bao giờ tới nơi.
 Bốn lượt thì mỗi lượt ~40 giây, nằm gọn trong trần, và người dùng nhận đúng trải nghiệm spec mô tả. Khác cách làm, giống kết quả.</t>
         </is>
       </c>
-      <c r="G120" s="8" t="inlineStr">
+      <c r="G121" s="8" t="inlineStr">
         <is>
           <t>app/api/ban-doc-sau/route.ts, app/luan-giai/sau/page.tsx</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="30" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="30" t="inlineStr">
         <is>
           <t>L15</t>
         </is>
       </c>
-      <c r="B121" s="31" t="inlineStr">
+      <c r="B122" s="31" t="inlineStr">
         <is>
           <t>Bản đọc sâu 12 cung</t>
         </is>
       </c>
-      <c r="C121" s="31" t="inlineStr">
+      <c r="C122" s="31" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D121" s="8" t="inlineStr">
+      <c r="D122" s="8" t="inlineStr">
         <is>
           <t>Không dựng bảng mới, dùng lại đệm noi_dung_ai</t>
         </is>
       </c>
-      <c r="E121" s="8" t="inlineStr">
+      <c r="E122" s="8" t="inlineStr">
         <is>
           <t>Thêm bề mặt "ban-doc-sau" vào BeMat. Khoá mang cả số chặng và phiên bản bộ luật.</t>
         </is>
       </c>
-      <c r="F121" s="32" t="inlineStr">
+      <c r="F122" s="32" t="inlineStr">
         <is>
           <t>Spec mục 11 đề xuất bảng riêng `bao_luan_giai`. Bảng riêng nghĩa là chủ dự án phải mở Supabase chạy SQL tay trước khi tính năng chạy được — mà đệm sẵn có đã cho đúng bảo đảm spec mục 10.21 cần: mở lại ra đúng chữ cũ.
 Thứ bảng riêng cho thêm mà đệm không cho là LỊCH SỬ phiên bản, phục vụ nút "Làm mới bài". Đó là tính năng sau, chưa làm.</t>
         </is>
       </c>
-      <c r="G121" s="8" t="inlineStr">
+      <c r="G122" s="8" t="inlineStr">
         <is>
           <t>lib/rag/noi-dung-ai.ts</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="30" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="30" t="inlineStr">
         <is>
           <t>L15</t>
         </is>
       </c>
-      <c r="B122" s="31" t="inlineStr">
+      <c r="B123" s="31" t="inlineStr">
         <is>
           <t>Bản đọc sâu 12 cung</t>
         </is>
       </c>
-      <c r="C122" s="31" t="inlineStr">
+      <c r="C123" s="31" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D122" s="8" t="inlineStr">
+      <c r="D123" s="8" t="inlineStr">
         <is>
           <t>Sơ đồ bốn chặng mười hai tấm gương</t>
         </is>
       </c>
-      <c r="E122" s="8" t="inlineStr">
+      <c r="E123" s="8" t="inlineStr">
         <is>
           <t>SVG 4 cột × 3 ô, sáu đường nét đứt. Gương nội bộ vẽ cong ra ngoài. Ô đang đọc sáng fuchsia, ô gương sáng nhạt, bấm để nhảy.</t>
         </is>
       </c>
-      <c r="F122" s="32" t="inlineStr">
+      <c r="F123" s="32" t="inlineStr">
         <is>
           <t>Gom đường thành CẶP: gương là quan hệ hai chiều, vẽ 12 đường là vẽ mỗi quan hệ hai lần và hình rối tới mức không đọc ra gì. Sáu là đúng số quan hệ thật — đã kiểm bằng bộ đo: 6 cặp, 4 bắc cầu, 2 nội bộ, khớp spec.
 Sơ đồ này là LẬP LUẬN chứ không phải trang trí: nó trả lời câu hỏi mà chữ không trả lời gọn được — vì sao đây không phải mười hai bài rời ghép lại.</t>
         </is>
       </c>
-      <c r="G122" s="8" t="inlineStr">
+      <c r="G123" s="8" t="inlineStr">
         <is>
           <t>components/luangiai/SoDoBonChang.tsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="30" t="inlineStr">
-        <is>
-          <t>L15</t>
-        </is>
-      </c>
-      <c r="B123" s="31" t="inlineStr">
-        <is>
-          <t>Bản đọc sâu 12 cung</t>
-        </is>
-      </c>
-      <c r="C123" s="31" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D123" s="8" t="inlineStr">
-        <is>
-          <t>Bốn thói quen văn phong thành trường bắt buộc</t>
-        </is>
-      </c>
-      <c r="E123" s="8" t="inlineStr">
-        <is>
-          <t>VAN_PHONG_CELES dán vào prompt. Hai trong bốn quy tắc không nằm trong phần văn xuôi mà thành trường JSON model buộc phải trả: cauHoiSoi (câu người đọc đang tự hỏi, ngôi thứ nhất) và giuLai (một tới hai câu, không phải tóm tắt, không mở bằng hãy/nên/cần phải).</t>
-        </is>
-      </c>
-      <c r="F123" s="32" t="inlineStr">
-        <is>
-          <t>LUẬT BẤT BIẾN: luật nào cần đạt gần 100% thì phải là TRƯỜNG JSON, không phải một câu trong prompt. Đo thật: cùng một luật, viết thành lời dặn được 3/12 phần, thành trường bắt buộc được 12/12. Prompt bản đọc sâu đã bão hoà — thêm chữ là đánh đổi, không phải cộng thêm.</t>
-        </is>
-      </c>
-      <c r="G123" s="8" t="inlineStr">
-        <is>
-          <t>lib/rag/van-phong.ts</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="30" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L15</t>
         </is>
       </c>
       <c r="B124" s="31" t="inlineStr">
         <is>
-          <t>Hỏi Celes (chat)</t>
+          <t>Bản đọc sâu 12 cung</t>
         </is>
       </c>
       <c r="C124" s="31" t="inlineStr">
         <is>
-          <t>7d</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D124" s="8" t="inlineStr">
         <is>
-          <t>Nhịp một đoạn: người đọc trước, tên sau</t>
+          <t>Bốn thói quen văn phong thành trường bắt buộc</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
         <is>
-          <t>HÌNH DẠNG MỘT ĐOẠN trong prompt chat đảo hai nhịp đầu: (1) nói về người đọc — điều họ làm, chỗ họ hay vướng; (2) rồi mới nêu tên cấu trúc sinh ra điều đó và dịch nghĩa ngay; (3) hệ quả dạng điều kiện ở neuThi. Kèm khối VAN_PHONG_CELES_CHAT: mở bằng người đọc + cặp phân biệt.</t>
+          <t>VAN_PHONG_CELES dán vào prompt. Hai trong bốn quy tắc không nằm trong phần văn xuôi mà thành trường JSON model buộc phải trả: cauHoiSoi (câu người đọc đang tự hỏi, ngôi thứ nhất) và giuLai (một tới hai câu, không phải tóm tắt, không mở bằng hãy/nên/cần phải).</t>
         </is>
       </c>
       <c r="F124" s="32" t="inlineStr">
         <is>
-          <t>KHÔNG bỏ bớt cái tên nào — chỉ đổi chỗ. Bỏ tên đi thì còn lại là lời phỏng đoán, và tiêu chí 8 của bộ đo (≥2 dữ kiện có tên trong ba câu đầu) sập ngay. Vì thế tiêu chí 10 đo trên SÁU TỪ ĐẦU chứ không trên cả câu đầu: cái sai là mở MIỆNG bằng một cái tên người đọc chưa biết.</t>
+          <t>LUẬT BẤT BIẾN: luật nào cần đạt gần 100% thì phải là TRƯỜNG JSON, không phải một câu trong prompt. Đo thật: cùng một luật, viết thành lời dặn được 3/12 phần, thành trường bắt buộc được 12/12. Prompt bản đọc sâu đã bão hoà — thêm chữ là đánh đổi, không phải cộng thêm.</t>
         </is>
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/prompt-co-can-cu.ts, lib/rag/van-phong.ts</t>
+          <t>lib/rag/van-phong.ts</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="30" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="B125" s="31" t="inlineStr">
         <is>
-          <t>Bề mặt ngắn do AI viết</t>
+          <t>Hỏi Celes (chat)</t>
         </is>
       </c>
       <c r="C125" s="31" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7d</t>
         </is>
       </c>
       <c r="D125" s="8" t="inlineStr">
         <is>
-          <t>Hai câu khép của bảng mười hai lĩnh vực</t>
+          <t>Nhịp một đoạn: người đọc trước, tên sau</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
         <is>
-          <t>Schema đầu ra thêm cauHoiSoi (một câu hỏi ở ngôi người đọc) và giuLai (1-2 câu khép phần). Hai câu đi qua sachCauKhep = sach + boCauPhanQuyet, rồi boMarkdown/doiTenCung/boCauTenBia, rồi suaCauTiengLong, rồi NẰM TRONG phần chữ soatNgonNgu soát. Không qua suaCauKeSao vì theo luật chúng không nêu tên sao nào.</t>
+          <t>HÌNH DẠNG MỘT ĐOẠN trong prompt chat đảo hai nhịp đầu: (1) nói về người đọc — điều họ làm, chỗ họ hay vướng; (2) rồi mới nêu tên cấu trúc sinh ra điều đó và dịch nghĩa ngay; (3) hệ quả dạng điều kiện ở neuThi. Kèm khối VAN_PHONG_CELES_CHAT: mở bằng người đọc + cặp phân biệt.</t>
         </is>
       </c>
       <c r="F125" s="32" t="inlineStr">
         <is>
-          <t>Là TRƯỜNG chứ không phải lời dặn: cùng một luật, viết thành lời dặn thì model làm được 3/12 phần, viết thành trường bắt buộc thì 12/12 ngay lần đầu (đo ở bản đọc sâu). || Phía nhận thì TUỲ CHỌN: thiếu một câu khép thì phần ấy vẫn đọc được, bỏ cả phần đời vì thiếu nó là đổi một mất mát lớn lấy một mất mát nhỏ.</t>
+          <t>KHÔNG bỏ bớt cái tên nào — chỉ đổi chỗ. Bỏ tên đi thì còn lại là lời phỏng đoán, và tiêu chí 8 của bộ đo (≥2 dữ kiện có tên trong ba câu đầu) sập ngay. Vì thế tiêu chí 10 đo trên SÁU TỪ ĐẦU chứ không trên cả câu đầu: cái sai là mở MIỆNG bằng một cái tên người đọc chưa biết.</t>
         </is>
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/bang-linh-vuc.ts, lib/tuvi/luan-giai-sau.ts, components/laso/BangLuanGiai.tsx</t>
+          <t>lib/rag/prompt-co-can-cu.ts, lib/rag/van-phong.ts</t>
         </is>
       </c>
     </row>
@@ -17907,101 +17987,101 @@
       </c>
       <c r="C126" s="31" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D126" s="8" t="inlineStr">
         <is>
-          <t>Bảng mười hai lĩnh vực sinh bằng hai lượt song song</t>
+          <t>Hai câu khép của bảng mười hai lĩnh vực</t>
         </is>
       </c>
       <c r="E126" s="8" t="inlineStr">
         <is>
-          <t>Mười hai phần chia làm hai nửa theo CHẶNG (chặng 1-2 và chặng 3-4), mỗi nửa một lượt gọi, chạy song song bằng Promise.all, mỗi lượt maxTokens 5.000. Mỗi nửa được cho biết id của sáu phần bên kia kèm lệnh không luận sang. Bắt lỗi riêng từng nửa: hỏng một nửa thì đi tiếp với nửa còn lại, hỏng cả hai mới ném.</t>
+          <t>Schema đầu ra thêm cauHoiSoi (một câu hỏi ở ngôi người đọc) và giuLai (1-2 câu khép phần). Hai câu đi qua sachCauKhep = sach + boCauPhanQuyet, rồi boMarkdown/doiTenCung/boCauTenBia, rồi suaCauTiengLong, rồi NẰM TRONG phần chữ soatNgonNgu soát. Không qua suaCauKeSao vì theo luật chúng không nêu tên sao nào.</t>
         </is>
       </c>
       <c r="F126" s="32" t="inlineStr">
         <is>
-          <t>ĐO ĐƯỢC 22/09/2026: bản một-lượt mất 52,3 giây cho 2.927 từ, trần một lượt gọi là 55 giây và ngân sách fallback là 50 — chạm trần thì KHÔNG còn chỗ lùi sang model hai, cả bảng rơi về bản tất định. || Cái mất khi tách: hai nửa không thấy nhau nên có thể cùng bám một cách cục; luật "mỗi cách cục chỉ nhắc một lần" chỉ còn hiệu lực trong một nửa.</t>
+          <t>Là TRƯỜNG chứ không phải lời dặn: cùng một luật, viết thành lời dặn thì model làm được 3/12 phần, viết thành trường bắt buộc thì 12/12 ngay lần đầu (đo ở bản đọc sâu). || Phía nhận thì TUỲ CHỌN: thiếu một câu khép thì phần ấy vẫn đọc được, bỏ cả phần đời vì thiếu nó là đổi một mất mát lớn lấy một mất mát nhỏ.</t>
         </is>
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/bang-linh-vuc.ts, lib/ai/fallback.ts</t>
+          <t>lib/rag/bang-linh-vuc.ts, lib/tuvi/luan-giai-sau.ts, components/laso/BangLuanGiai.tsx</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="30" t="inlineStr">
         <is>
-          <t>L7</t>
+          <t>L4</t>
         </is>
       </c>
       <c r="B127" s="31" t="inlineStr">
         <is>
-          <t>Chuỗi model &amp; fallback</t>
+          <t>Bề mặt ngắn do AI viết</t>
         </is>
       </c>
       <c r="C127" s="31" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D127" s="8" t="inlineStr">
         <is>
-          <t>Luật trước, dữ kiện sau — để prompt được đệm</t>
+          <t>Bảng mười hai lĩnh vực sinh bằng hai lượt song song</t>
         </is>
       </c>
       <c r="E127" s="8" t="inlineStr">
         <is>
-          <t>system = khối luật thuần (persona, thang viết, chuẩn ngôn ngữ, văn phong, schema JSON). user = dữ kiện của lá số này (cách cục, Thân cư, bảng tiêu chí, bằng chứng RAG). Không trộn.</t>
+          <t>Mười hai phần chia làm hai nửa theo CHẶNG (chặng 1-2 và chặng 3-4), mỗi nửa một lượt gọi, chạy song song bằng Promise.all, mỗi lượt maxTokens 5.000. Mỗi nửa được cho biết id của sáu phần bên kia kèm lệnh không luận sang. Bắt lỗi riêng từng nửa: hỏng một nửa thì đi tiếp với nửa còn lại, hỏng cả hai mới ném.</t>
         </is>
       </c>
       <c r="F127" s="32" t="inlineStr">
         <is>
-          <t>Nhà cung cấp đệm theo TIỀN TỐ, nên CHỈ CẦN MỘT dữ kiện của người dùng lọt lên trên là toàn bộ phần luật phía sau mất quyền đệm — và không có gì báo cho ai biết. ChatResult.tokensDem là thứ báo: bằng 0 nghĩa là tiền tố đang hỏng, không phải vô hại.</t>
+          <t>ĐO ĐƯỢC 22/09/2026: bản một-lượt mất 52,3 giây cho 2.927 từ, trần một lượt gọi là 55 giây và ngân sách fallback là 50 — chạm trần thì KHÔNG còn chỗ lùi sang model hai, cả bảng rơi về bản tất định. || Cái mất khi tách: hai nửa không thấy nhau nên có thể cùng bám một cách cục; luật "mỗi cách cục chỉ nhắc một lần" chỉ còn hiệu lực trong một nửa.</t>
         </is>
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/bang-linh-vuc.ts, lib/rag/ban-doc-sau.ts, lib/ai/providers.ts</t>
+          <t>lib/rag/bang-linh-vuc.ts, lib/ai/fallback.ts</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="30" t="inlineStr">
         <is>
-          <t>L15</t>
+          <t>L7</t>
         </is>
       </c>
       <c r="B128" s="31" t="inlineStr">
         <is>
-          <t>Bản đọc sâu 12 cung</t>
+          <t>Chuỗi model &amp; fallback</t>
         </is>
       </c>
       <c r="C128" s="31" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D128" s="8" t="inlineStr">
         <is>
-          <t>Ngân sách từ là trần; tiêu chí được phép im lặng</t>
+          <t>Luật trước, dữ kiện sau — để prompt được đệm</t>
         </is>
       </c>
       <c r="E128" s="8" t="inlineStr">
         <is>
-          <t>nganSachTu() vẫn tính như cũ (490 x hệ số theo doNoiBat / số tiêu chí) nhưng vào prompt với chữ TỐI ĐA. Model trả { nhan, thieuCanCu: true, noiDung: "" } cho tiêu chí lá số không nói được gì. Cửa chặn phần: ngưỡng nửa đo trên số tiêu chí TRẢ VỀ, cộng sàn 2 tiêu chí CÓ CHỮ, cộng khối gương bắt buộc có chữ.</t>
+          <t>system = khối luật thuần (persona, thang viết, chuẩn ngôn ngữ, văn phong, schema JSON). user = dữ kiện của lá số này (cách cục, Thân cư, bảng tiêu chí, bằng chứng RAG). Không trộn.</t>
         </is>
       </c>
       <c r="F128" s="32" t="inlineStr">
         <is>
-          <t>Khối gương KHÔNG được phép im lặng — nó là điều kiện ship theo spec mục 10.14. || Mọi tỉ lệ trong bộ đo phải tính trên tiêu chí CÓ CHỮ: đếm tiêu chí im lặng vào mẫu số là phạt bài vì đã thành thật, đúng áp lực đã đẩy model viết cho đủ.</t>
+          <t>Nhà cung cấp đệm theo TIỀN TỐ, nên CHỈ CẦN MỘT dữ kiện của người dùng lọt lên trên là toàn bộ phần luật phía sau mất quyền đệm — và không có gì báo cho ai biết. ChatResult.tokensDem là thứ báo: bằng 0 nghĩa là tiền tố đang hỏng, không phải vô hại.</t>
         </is>
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/ban-doc-sau.ts, scripts/test-ban-doc-sau.ts</t>
+          <t>lib/rag/bang-linh-vuc.ts, lib/rag/ban-doc-sau.ts, lib/ai/providers.ts</t>
         </is>
       </c>
     </row>
@@ -18018,101 +18098,101 @@
       </c>
       <c r="C129" s="31" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D129" s="8" t="inlineStr">
         <is>
-          <t>Mẫu vàng cắm ở cuối khối user</t>
+          <t>Ngân sách từ là trần; tiêu chí được phép im lặng</t>
         </is>
       </c>
       <c r="E129" s="8" t="inlineStr">
         <is>
-          <t>chonMauVang() chọn theo tình huống của chặng: luôn xin khoi-guong + cau-khep; thêm thua-du-kien nếu chặng có phần doNoiBat &lt;= NGUONG_MO; thêm day-du-kien nếu có phần &gt;= NGUONG_NOI; thêm mien-rui-ro ở chặng có tat-ach.</t>
+          <t>nganSachTu() vẫn tính như cũ (490 x hệ số theo doNoiBat / số tiêu chí) nhưng vào prompt với chữ TỐI ĐA. Model trả { nhan, thieuCanCu: true, noiDung: "" } cho tiêu chí lá số không nói được gì. Cửa chặn phần: ngưỡng nửa đo trên số tiêu chí TRẢ VỀ, cộng sàn 2 tiêu chí CÓ CHỮ, cộng khối gương bắt buộc có chữ.</t>
         </is>
       </c>
       <c r="F129" s="32" t="inlineStr">
         <is>
-          <t>Mẫu là nội dung ĐỘNG nên phải nằm ở user, KHÔNG được vào system: một dòng động trong system là toàn bộ khối luật phía sau mất quyền đệm cho mọi lượt gọi (CEL-111). || Kho rỗng phải trả chuỗi rỗng chứ không phải undefined — prompt không được mọc thêm dòng nào khi chưa có mẫu.</t>
+          <t>Khối gương KHÔNG được phép im lặng — nó là điều kiện ship theo spec mục 10.14. || Mọi tỉ lệ trong bộ đo phải tính trên tiêu chí CÓ CHỮ: đếm tiêu chí im lặng vào mẫu số là phạt bài vì đã thành thật, đúng áp lực đã đẩy model viết cho đủ.</t>
         </is>
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/mau-vang.ts, lib/rag/ban-doc-sau.ts</t>
+          <t>lib/rag/ban-doc-sau.ts, scripts/test-ban-doc-sau.ts</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="30" t="inlineStr">
         <is>
-          <t>L7</t>
+          <t>L15</t>
         </is>
       </c>
       <c r="B130" s="31" t="inlineStr">
         <is>
-          <t>Chuỗi model &amp; fallback</t>
+          <t>Bản đọc sâu 12 cung</t>
         </is>
       </c>
       <c r="C130" s="31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D130" s="8" t="inlineStr">
         <is>
-          <t>Cắt luật khỏi prompt phải đi theo bề mặt</t>
+          <t>Mẫu vàng cắm ở cuối khối user</t>
         </is>
       </c>
       <c r="E130" s="8" t="inlineStr">
         <is>
-          <t>dungChuanNgonNgu({ khoi }) cắt theo tên khối. Mỗi bề mặt tự khai mình cắt được gì, dựa trên lớp sửa nó thật sự có.</t>
+          <t>chonMauVang() chọn theo tình huống của chặng: luôn xin khoi-guong + cau-khep; thêm thua-du-kien nếu chặng có phần doNoiBat &lt;= NGUONG_MO; thêm day-du-kien nếu có phần &gt;= NGUONG_NOI; thêm mien-rui-ro ở chặng có tat-ach.</t>
         </is>
       </c>
       <c r="F130" s="32" t="inlineStr">
         <is>
-          <t>Bảng đối chiếu (đọc từ mã 23/09/2026): soatNgonNgu 6/6 bề mặt · suaCauTiengLong 4/6 (thiếu ở bề mặt ngắn và mốc hành trình) · suaCauKeSao 2/6 (chỉ bảng mười hai lĩnh vực và bề mặt ngắn). || CỔNG CHẶN KHÔNG PHẢI LƯỚI AN TOÀN: chặn nghĩa là trả null và lùi về bản tất định. Chỉ cắt luật khi có LỚP SỬA đứng trước cổng, đừng cắt khi chỉ có cổng.</t>
+          <t>Mẫu là nội dung ĐỘNG nên phải nằm ở user, KHÔNG được vào system: một dòng động trong system là toàn bộ khối luật phía sau mất quyền đệm cho mọi lượt gọi (CEL-111). || Kho rỗng phải trả chuỗi rỗng chứ không phải undefined — prompt không được mọc thêm dòng nào khi chưa có mẫu.</t>
         </is>
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/chuan-ngon-ngu.ts, lib/rag/sua-chua.ts</t>
+          <t>lib/rag/mau-vang.ts, lib/rag/ban-doc-sau.ts</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="30" t="inlineStr">
         <is>
-          <t>L16</t>
+          <t>L7</t>
         </is>
       </c>
       <c r="B131" s="31" t="inlineStr">
         <is>
-          <t>Luận giải v3 (Tổng quan + Chuyên sâu)</t>
+          <t>Chuỗi model &amp; fallback</t>
         </is>
       </c>
       <c r="C131" s="31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D131" s="8" t="inlineStr">
         <is>
-          <t>Khung câu hỏi</t>
+          <t>Cắt luật khỏi prompt phải đi theo bề mặt</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/v3/khung.ts SINH TỰ ĐỘNG từ KHUNG-LUAN-GIAI-v3.xlsx: 11 câu tổng quan, 61 câu chuyên sâu, 14 chủ đề, cung phụ trợ và sao toàn cục mỗi chủ đề.</t>
+          <t>dungChuanNgonNgu({ khoi }) cắt theo tên khối. Mỗi bề mặt tự khai mình cắt được gì, dựa trên lớp sửa nó thật sự có.</t>
         </is>
       </c>
       <c r="F131" s="32" t="inlineStr">
         <is>
-          <t>Không sửa câu chữ bằng tay trong khung.ts — sửa trong khung rồi sinh lại, không thì hai bản lệch nhau.</t>
+          <t>Bảng đối chiếu (đọc từ mã 23/09/2026): soatNgonNgu 6/6 bề mặt · suaCauTiengLong 4/6 (thiếu ở bề mặt ngắn và mốc hành trình) · suaCauKeSao 2/6 (chỉ bảng mười hai lĩnh vực và bề mặt ngắn). || CỔNG CHẶN KHÔNG PHẢI LƯỚI AN TOÀN: chặn nghĩa là trả null và lùi về bản tất định. Chỉ cắt luật khi có LỚP SỬA đứng trước cổng, đừng cắt khi chỉ có cổng.</t>
         </is>
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/v3/khung.ts</t>
+          <t>lib/rag/chuan-ngon-ngu.ts, lib/rag/sua-chua.ts</t>
         </is>
       </c>
     </row>
@@ -18129,66 +18209,66 @@
       </c>
       <c r="C132" s="31" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D132" s="8" t="inlineStr">
+        <is>
+          <t>Khung câu hỏi</t>
+        </is>
+      </c>
+      <c r="E132" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/khung.ts SINH TỰ ĐỘNG từ KHUNG-LUAN-GIAI-v3.xlsx: 11 câu tổng quan, 61 câu chuyên sâu, 14 chủ đề, cung phụ trợ và sao toàn cục mỗi chủ đề.</t>
+        </is>
+      </c>
+      <c r="F132" s="32" t="inlineStr">
+        <is>
+          <t>Không sửa câu chữ bằng tay trong khung.ts — sửa trong khung rồi sinh lại, không thì hai bản lệch nhau.</t>
+        </is>
+      </c>
+      <c r="G132" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/khung.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="30" t="inlineStr">
+        <is>
+          <t>L16</t>
+        </is>
+      </c>
+      <c r="B133" s="31" t="inlineStr">
+        <is>
+          <t>Luận giải v3 (Tổng quan + Chuyên sâu)</t>
+        </is>
+      </c>
+      <c r="C133" s="31" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D132" s="8" t="inlineStr">
+      <c r="D133" s="8" t="inlineStr">
         <is>
           <t>Dữ kiện theo ma trận cung</t>
         </is>
       </c>
-      <c r="E132" s="8" t="inlineStr">
+      <c r="E133" s="8" t="inlineStr">
         <is>
           <t>dungDuKien(): cung chính + xung chiếu + tam hợp + phụ trợ (chỉ chuyên sâu) + sao toàn cục + cách cục trên cung đang đọc + lớp vận (đại vận, chuỗi đại vận, tiểu hạn, lưu tứ hóa tính từ TU_HOA theo can năm, lưu tinh, nguyệt hạn, điểm 12 cung). Mỗi cung kèm nghĩa sao lấy từ KHUON.vi.netPhuTinh / netSao.
 24/09/2026: hoiThoiDiem(q) — câu không hỏi thời điểm thì mô tả cung KHÔNG kèm "đại vận X–Y tuổi" và Tuần/Triệt không kèm mốc tuổi.</t>
         </is>
       </c>
-      <c r="F132" s="32" t="inlineStr">
+      <c r="F133" s="32" t="inlineStr">
         <is>
           <t>Cấp NGHĨA SAO do engine giữ — thiếu nó model tự nhớ nghĩa (lượt 5: 135 nhận định không căn cứ / 30 bài). "Nghĩa nền" (manhCau) chỉ cho Mệnh/Thân: gắn vào cung khác thì ra "Tử Vi ở Tài Bạch khiến tiền cần tự quyết".
 Mọi cung mang nhãn đại vận làm model gắn mốc tuổi vào cả câu "tôi hợp nghề gì" — cùng một mốc lặp ở bảy câu.</t>
         </is>
       </c>
-      <c r="G132" s="8" t="inlineStr">
+      <c r="G133" s="8" t="inlineStr">
         <is>
           <t>lib/rag/v3/du-kien.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="30" t="inlineStr">
-        <is>
-          <t>L16</t>
-        </is>
-      </c>
-      <c r="B133" s="31" t="inlineStr">
-        <is>
-          <t>Luận giải v3 (Tổng quan + Chuyên sâu)</t>
-        </is>
-      </c>
-      <c r="C133" s="31" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D133" s="8" t="inlineStr">
-        <is>
-          <t>RAG theo từng cung</t>
-        </is>
-      </c>
-      <c r="E133" s="8" t="inlineStr">
-        <is>
-          <t>Mỗi cung một truy vấn (chính tinh + tứ hóa + tên cung + từ khoá chủ đề), thêm truy vấn cách cục và lưu tứ hóa. Chấm khớp sao (cả tên tắt sách cổ) + khớp cung + đề mục theo cung; lọc rác; chọn XOAY VÒNG giữa các truy vấn; bỏ bản chép giữa các truy vấn.</t>
-        </is>
-      </c>
-      <c r="F133" s="32" t="inlineStr">
-        <is>
-          <t>Kho có nhiều bảng lá số / danh sách sao / lịch sử môn học điểm cao mà vô dụng — phải lọc. "Tử Vi" là tên môn học ở đầu mọi đoạn: không đưa vào nhánh từ khoá, và thực thể lấy từ chuỗi từ khoá ngắn (từ truy hồi 2026.09.4 mỗi thực thể thành cụm điểm gấp đôi).</t>
-        </is>
-      </c>
-      <c r="G133" s="8" t="inlineStr">
-        <is>
-          <t>lib/rag/v3/truy-hoi-v3.ts</t>
         </is>
       </c>
     </row>
@@ -18205,105 +18285,105 @@
       </c>
       <c r="C134" s="31" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D134" s="8" t="inlineStr">
+        <is>
+          <t>RAG theo từng cung</t>
+        </is>
+      </c>
+      <c r="E134" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi cung một truy vấn (chính tinh + tứ hóa + tên cung + từ khoá chủ đề), thêm truy vấn cách cục và lưu tứ hóa. Chấm khớp sao (cả tên tắt sách cổ) + khớp cung + đề mục theo cung; lọc rác; chọn XOAY VÒNG giữa các truy vấn; bỏ bản chép giữa các truy vấn.</t>
+        </is>
+      </c>
+      <c r="F134" s="32" t="inlineStr">
+        <is>
+          <t>Kho có nhiều bảng lá số / danh sách sao / lịch sử môn học điểm cao mà vô dụng — phải lọc. "Tử Vi" là tên môn học ở đầu mọi đoạn: không đưa vào nhánh từ khoá, và thực thể lấy từ chuỗi từ khoá ngắn (từ truy hồi 2026.09.4 mỗi thực thể thành cụm điểm gấp đôi).</t>
+        </is>
+      </c>
+      <c r="G134" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/truy-hoi-v3.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="30" t="inlineStr">
+        <is>
+          <t>L16</t>
+        </is>
+      </c>
+      <c r="B135" s="31" t="inlineStr">
+        <is>
+          <t>Luận giải v3 (Tổng quan + Chuyên sâu)</t>
+        </is>
+      </c>
+      <c r="C135" s="31" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D134" s="8" t="inlineStr">
+      <c r="D135" s="8" t="inlineStr">
         <is>
           <t>Celes viết</t>
         </is>
       </c>
-      <c r="E134" s="8" t="inlineStr">
+      <c r="E135" s="8" t="inlineStr">
         <is>
           <t>SYSTEM_V3 = nguyên văn quy tắc viết + hai bài mẫu của chủ dự án + luật căn cứ + luật trình bày. Đầu ra JSON: danY (mỗi ý có mã F/E) → luanGiai → viSao. Tổng quan có PHẠM VI riêng từng câu.
 24/09/2026: phamViChuyenSau(q) dựng từ khung — liệt kê các câu cùng chủ đề (không lấn sang), cấm tả lại tính cách ngoài chủ đề Tính cách, bắt kết bằng lời khuyên riêng. Luật 10 trong LUAT_CAN_CU: không lặp giữa các câu.</t>
         </is>
       </c>
-      <c r="F134" s="32" t="inlineStr">
+      <c r="F135" s="32" t="inlineStr">
         <is>
           <t>Đừng tóm gọn quy tắc của chủ dự án: bản rút gọn trước đó làm bài dài gấp ba mức cho phép. Tổng quan sinh song song nên phải chia phạm vi bằng mã (lượt 2: 5/11 câu cùng kết "đừng làm một mình").
 Cấm lời khuyên chung mà không bắt kết bằng lời khuyên riêng thì model BỎ luôn lời khuyên (lượt 8: ba câu, giám khảo 4 → 1).</t>
         </is>
       </c>
-      <c r="G134" s="8" t="inlineStr">
+      <c r="G135" s="8" t="inlineStr">
         <is>
           <t>lib/rag/v3/prompt-v3.ts, lib/rag/v3/index.ts</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="30" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="30" t="inlineStr">
         <is>
           <t>L16</t>
         </is>
       </c>
-      <c r="B135" s="31" t="inlineStr">
+      <c r="B136" s="31" t="inlineStr">
         <is>
           <t>Luận giải v3 (Tổng quan + Chuyên sâu)</t>
         </is>
       </c>
-      <c r="C135" s="31" t="inlineStr">
+      <c r="C136" s="31" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D135" s="8" t="inlineStr">
+      <c r="D136" s="8" t="inlineStr">
         <is>
           <t>Kiểm + sửa</t>
         </is>
       </c>
-      <c r="E135" s="8" t="inlineStr">
+      <c r="E136" s="8" t="inlineStr">
         <is>
           <t>kiemBai(): độ dài (lệch ≤15% chỉ ghi nhận), số đoạn, gạch ý, lộ tên sao/cung/thuật ngữ trong bài luận, từ cấm, mã nội bộ, viết tắt, sao ngoài dữ kiện ở viSao (so CÓ DẤU), mở câu "Bạn" quá nhiều, lặp từ nối. Lỗi chặn → MỘT vòng sửa có chỉ đích; chỉ nhận bản sửa không tệ hơn. Câu an toàn sức khỏe / tài chính do mã chèn.
 24/09/2026: thêm moc-tuoi (chặn), ky-tu-la (chặn), khong-loi-khuyen (chặn, chuyên sâu), khuyen-chung (ghi nhận).</t>
         </is>
       </c>
-      <c r="F135" s="32" t="inlineStr">
+      <c r="F136" s="32" t="inlineStr">
         <is>
           <t>So tên sao phải có dấu: bỏ dấu thì "Tử Phủ" trùng "Tử Phù" và bắt oan (lượt 3).
 Production từng hiện "cách làm cũ აღარ còn thuyết phục" (chữ Georgia) — model lẫn ngôn ngữ, phải chặn bằng mã.</t>
         </is>
       </c>
-      <c r="G135" s="8" t="inlineStr">
+      <c r="G136" s="8" t="inlineStr">
         <is>
           <t>lib/rag/v3/kiem-v3.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="30" t="inlineStr">
-        <is>
-          <t>L16</t>
-        </is>
-      </c>
-      <c r="B136" s="31" t="inlineStr">
-        <is>
-          <t>Luận giải v3 (Tổng quan + Chuyên sâu)</t>
-        </is>
-      </c>
-      <c r="C136" s="31" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D136" s="8" t="inlineStr">
-        <is>
-          <t>Đo</t>
-        </is>
-      </c>
-      <c r="E136" s="8" t="inlineStr">
-        <is>
-          <t>scripts/test-luan-giai-v3.ts chạy đúng hàm route gọi; scripts/cham-luan-giai-v3.ts chấm 7 tiêu chí 1–5 bằng model khác (mặc định gemini), ghi nhận định không căn cứ.</t>
-        </is>
-      </c>
-      <c r="F136" s="32" t="inlineStr">
-        <is>
-          <t>Giám khảo gemini bậc miễn phí trả 429 — gần hết bài lùi về luna tự chấm; điểm tuyệt đối có thể cao hơn thật.</t>
-        </is>
-      </c>
-      <c r="G136" s="8" t="inlineStr">
-        <is>
-          <t>scripts/test-luan-giai-v3.ts, scripts/cham-luan-giai-v3.ts</t>
         </is>
       </c>
     </row>
@@ -18320,66 +18400,66 @@
       </c>
       <c r="C137" s="31" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>Đo</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>scripts/test-luan-giai-v3.ts chạy đúng hàm route gọi; scripts/cham-luan-giai-v3.ts chấm 7 tiêu chí 1–5 bằng model khác (mặc định gemini), ghi nhận định không căn cứ.</t>
+        </is>
+      </c>
+      <c r="F137" s="32" t="inlineStr">
+        <is>
+          <t>Giám khảo gemini bậc miễn phí trả 429 — gần hết bài lùi về luna tự chấm; điểm tuyệt đối có thể cao hơn thật.</t>
+        </is>
+      </c>
+      <c r="G137" s="8" t="inlineStr">
+        <is>
+          <t>scripts/test-luan-giai-v3.ts, scripts/cham-luan-giai-v3.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="30" t="inlineStr">
+        <is>
+          <t>L16</t>
+        </is>
+      </c>
+      <c r="B138" s="31" t="inlineStr">
+        <is>
+          <t>Luận giải v3 (Tổng quan + Chuyên sâu)</t>
+        </is>
+      </c>
+      <c r="C138" s="31" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="D137" s="8" t="inlineStr">
+      <c r="D138" s="8" t="inlineStr">
         <is>
           <t>Giao diện + quyền</t>
         </is>
       </c>
-      <c r="E137" s="8" t="inlineStr">
+      <c r="E138" s="8" t="inlineStr">
         <is>
           <t>/la-so: TongQuanV3 gọi nhom=tong-quan (không cần đăng nhập). /luan-giai/sau: 14 chủ đề, mỗi chủ đề một lượt gọi, chỉ gọi khi mở tới. Mỗi câu: bài luận → "Độ rõ" → nút "Muốn biết vì sao không?" (ẩn mặc định). Route đặt hạn chót 52s.
 24/09/2026: useTongQuanV3 tải nhóm tổng quan MỘT lần cho cả trang; BaTheDauV3 dựng ba thẻ đầu từ TQ02/TQ03/TQ08, TongQuanV3 hiện các câu còn lại thành thẻ đánh số. /luan-giai/sau: nút "Đọc lại" chủ đề liền trước, "Đọc tiếp" là nút chính duy nhất.</t>
         </is>
       </c>
-      <c r="F137" s="32" t="inlineStr">
+      <c r="F138" s="32" t="inlineStr">
         <is>
           <t>Bảng lĩnh vực cũ chỉ tải khi v3 hỏng hoặc giao diện không phải tiếng Việt — tải cả hai là tốn gấp đôi lượt gọi cho cùng một chỗ. Mọi setState trong callback bất đồng bộ, không trong thân effect (giữ mốc 7 lỗi lint).
 Dải thẻ đầu chỉ lùi về GocNhinCard khi v3 hỏng cho đúng lá số đang xem — hiện cả hai là lặp nội dung. GocNhinCard còn dùng ở trang chủ và /hanh-trinh, đừng sửa nó cho /la-so.</t>
         </is>
       </c>
-      <c r="G137" s="8" t="inlineStr">
+      <c r="G138" s="8" t="inlineStr">
         <is>
           <t>components/luangiai/TongQuanV3.tsx, components/luangiai/CauTraLoiV3.tsx, app/luan-giai/sau/page.tsx, app/la-so/page.tsx, app/api/luan-giai-v3/route.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="30" t="inlineStr">
-        <is>
-          <t>L17</t>
-        </is>
-      </c>
-      <c r="B138" s="31" t="inlineStr">
-        <is>
-          <t>Bộ quy tắc luận giải chung</t>
-        </is>
-      </c>
-      <c r="C138" s="31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D138" s="8" t="inlineStr">
-        <is>
-          <t>Một nguồn luật</t>
-        </is>
-      </c>
-      <c r="E138" s="8" t="inlineStr">
-        <is>
-          <t>lib/rag/quy-tac-luan-giai.ts giữ QUY_TAC_VIET (nguyên văn chủ dự án) + LUAT_CHUNG_LUAN_GIAI. v3 import QUY_TAC_VIET; chuẩn ngôn ngữ đặt QUY_TAC_LUAN_GIAI làm khối đầu; Kết nối cắm thẳng vào prompt.</t>
-        </is>
-      </c>
-      <c r="F138" s="32" t="inlineStr">
-        <is>
-          <t>Đừng tóm gọn quy tắc của chủ dự án. Độ dài/khuôn là của từng màn — câu nối và lời khuyên nằm TRONG số câu cho phép (không có câu này thì khám phá chủ đề dài thêm ~19%).</t>
-        </is>
-      </c>
-      <c r="G138" s="8" t="inlineStr">
-        <is>
-          <t>lib/rag/quy-tac-luan-giai.ts, lib/rag/chuan-ngon-ngu.ts</t>
         </is>
       </c>
     </row>
@@ -18396,27 +18476,27 @@
       </c>
       <c r="C139" s="31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D139" s="8" t="inlineStr">
         <is>
-          <t>Lời khuyên</t>
+          <t>Một nguồn luật</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
         <is>
-          <t>CAU_RA_LENH chỉ bắt lời khuyên RỖNG (cân bằng hơn, cần thận trọng khi quyết định, đừng để áp lực…, dồn hết vào một chỗ…). boCauRaLenh / KHUYEN_BAO / mốc hành trình đều dùng nó.</t>
+          <t>lib/rag/quy-tac-luan-giai.ts giữ QUY_TAC_VIET (nguyên văn chủ dự án) + LUAT_CHUNG_LUAN_GIAI. v3 import QUY_TAC_VIET; chuẩn ngôn ngữ đặt QUY_TAC_LUAN_GIAI làm khối đầu; Kết nối cắm thẳng vào prompt.</t>
         </is>
       </c>
       <c r="F139" s="32" t="inlineStr">
         <is>
-          <t>Bản cũ bắt mọi "hãy / bạn nên" → cắt sạch lời khuyên, ngược quy tắc chủ dự án. scripts/test-chuan-ngon-ngu.ts giữ các ca kiểm để khỏi bị đảo lại.</t>
+          <t>Đừng tóm gọn quy tắc của chủ dự án. Độ dài/khuôn là của từng màn — câu nối và lời khuyên nằm TRONG số câu cho phép (không có câu này thì khám phá chủ đề dài thêm ~19%).</t>
         </is>
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/chuan-ngon-ngu.ts, lib/rag/be-mat-ngan.ts, lib/rag/moc-hanh-trinh.ts</t>
+          <t>lib/rag/quy-tac-luan-giai.ts, lib/rag/chuan-ngon-ngu.ts</t>
         </is>
       </c>
     </row>
@@ -18433,25 +18513,62 @@
       </c>
       <c r="C140" s="31" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D140" s="8" t="inlineStr">
+        <is>
+          <t>Lời khuyên</t>
+        </is>
+      </c>
+      <c r="E140" s="8" t="inlineStr">
+        <is>
+          <t>CAU_RA_LENH chỉ bắt lời khuyên RỖNG (cân bằng hơn, cần thận trọng khi quyết định, đừng để áp lực…, dồn hết vào một chỗ…). boCauRaLenh / KHUYEN_BAO / mốc hành trình đều dùng nó.</t>
+        </is>
+      </c>
+      <c r="F140" s="32" t="inlineStr">
+        <is>
+          <t>Bản cũ bắt mọi "hãy / bạn nên" → cắt sạch lời khuyên, ngược quy tắc chủ dự án. scripts/test-chuan-ngon-ngu.ts giữ các ca kiểm để khỏi bị đảo lại.</t>
+        </is>
+      </c>
+      <c r="G140" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/chuan-ngon-ngu.ts, lib/rag/be-mat-ngan.ts, lib/rag/moc-hanh-trinh.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="30" t="inlineStr">
+        <is>
+          <t>L17</t>
+        </is>
+      </c>
+      <c r="B141" s="31" t="inlineStr">
+        <is>
+          <t>Bộ quy tắc luận giải chung</t>
+        </is>
+      </c>
+      <c r="C141" s="31" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D140" s="8" t="inlineStr">
+      <c r="D141" s="8" t="inlineStr">
         <is>
           <t>Cổng ngôn ngữ</t>
         </is>
       </c>
-      <c r="E140" s="8" t="inlineStr">
+      <c r="E141" s="8" t="inlineStr">
         <is>
           <t>soatNgonNgu: thêm ky-tu-la (chặn). Phán quyết: miễn cho "nên nghỉ việc / nên cưới / không nên cưới" khi cùng câu có "nếu" đứng trước; cụm hứa ("chắc chắn sẽ") vẫn chặn.</t>
         </is>
       </c>
-      <c r="F140" s="32" t="inlineStr">
+      <c r="F141" s="32" t="inlineStr">
         <is>
           <t>"Chặn" ở cổng chung nghĩa là ghi trace, không giữ chữ lại (sua-chua.ts) — chữ lạ ở màn không có vòng sửa vẫn có thể tới người đọc; v3 thì có vòng sửa.</t>
         </is>
       </c>
-      <c r="G140" s="8" t="inlineStr">
+      <c r="G141" s="8" t="inlineStr">
         <is>
           <t>lib/rag/ngon-ngu.ts</t>
         </is>
@@ -18469,7 +18586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21176,6 +21293,38 @@
         </is>
       </c>
       <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="49" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B85" s="50" t="inlineStr">
+        <is>
+          <t>app-gd1-bearer</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>CEL-154, L10</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Máy chủ nhận thêm header Authorization: Bearer (token Supabase) bên cạnh cookie, trong lib/supabase/server.ts.</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>App di động không có cookie trình duyệt nên không thể dùng chung hạn mức / bậc quyền / dữ liệu với web. Chọn cách xác thực token qua Supabase (auth.getUser(token)) thay vì tự giải mã JWT để không phải giữ khoá ký ở máy chủ và không mở lỗ giả mạo. Làm nửa máy chủ trước vì nửa app còn chờ chọn cách đăng nhập trên di động.</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
app-gd1-menh-ban: vet lai menh ban app di dong thanh 1 luoi 4x4 day du
- Bo 3 che do Deu hieu/Co dien/Chuyen sau (ChonPhanDoan), dung MOT luoi
  4x4 tinh fit tron mot man hinh doc, khong cuon ngang - phan hoi that
  tu chu du an kem anh app doi thu (Altuvi.com) tham khao cach trinh bay.
- Them token chu moi micro (9.5px) / nano (8px), CHI dung o man nay.
- Sua copy buoc ngay sinh onboarding: "Ngay ban bat dau cau chuyen nay"
  -> "Ngay sinh cua ban" (khong ro y theo phan hoi that).
- Cap nhat README app, AGENTS.md, HUONG-DAN.md: dao nguoc mot phan luat
  cu "o du lon de cham" - doi co chu dich, da ghi lai ly do.
- Cap nhat PRODUCT-BACKLOG.xlsx: CEL-155, L18, nhat ky thay doi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O155"/>
+  <dimension ref="A1:O156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13453,6 +13453,86 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" s="13" t="inlineStr">
+        <is>
+          <t>CEL-155</t>
+        </is>
+      </c>
+      <c r="B156" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t>Mệnh bàn app: một lưới đầy đủ, bỏ 3 chế độ; sửa copy bước ngày sinh</t>
+        </is>
+      </c>
+      <c r="D156" s="8" t="inlineStr">
+        <is>
+          <t>Màn "Bản đồ của tôi" (apps/celes-app/app/ban-do.tsx) viết lại hoàn toàn: bỏ Dễ hiểu/Cổ điển/Chuyên sâu, dựng MỘT lưới 4×4 tĩnh hiện đủ 12 cung trên một màn hình dọc (không cuộn ngang) — can chi, tên cung, chính tinh kèm độ sáng, phụ tinh trọng yếu, Tuần/Triệt, tuổi đại vận. Chạm vào cung mở chi tiết đầy đủ bên dưới. Thêm 2 cỡ chữ mới micro (9.5px) / nano (8px) vào token, CHỈ dùng ở màn này. Đồng thời sửa copy bước 2 onboarding: "Ngày bạn bắt đầu câu chuyện này" → "Ngày sinh của bạn" (không rõ ý theo phản hồi thật).</t>
+        </is>
+      </c>
+      <c r="E156" s="8" t="inlineStr">
+        <is>
+          <t>1. useHoSo() trả LaSo tĩnh (không lưu, tính lại mỗi lần mở)
+2. Lưới 4×4 định vị theo VI_TRI (khớp VI_TRI_GRID của web) — 12 ô biên + khối bản mệnh ở giữa
+3. Chạm một ô → setCungChon → khối chi tiết đầy đủ hiện dưới lưới
+4. Không có state chế độ hiển thị nữa (đã bỏ ChonPhanDoan 3 mức)</t>
+        </is>
+      </c>
+      <c r="F156" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G156" s="8" t="inlineStr">
+        <is>
+          <t>Không đổi</t>
+        </is>
+      </c>
+      <c r="H156" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I156" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J156" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/ban-do.tsx</t>
+        </is>
+      </c>
+      <c r="K156" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/ban-do.tsx, apps/celes-app/src/thiet-ke/token.ts, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L156" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M156" s="8" t="inlineStr">
+        <is>
+          <t>Chưa test bằng mắt trên Expo Go/thiết bị thật (chỉ kiểm tsc + expo export bundle — cả hai sạch). Đổi ngược một phần luật cũ "ô đủ lớn để chạm" trong README app — đã cập nhật README + AGENTS.md + HUONG-DAN.md cùng commit này.</t>
+        </is>
+      </c>
+      <c r="N156" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="O156" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-menh-ban</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -13470,7 +13550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -18574,6 +18654,80 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="30" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Mệnh bàn app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Lấy lá số</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>useHoSo() giữ HoSo trong AsyncStorage, tính LaSo bằng lapLaSo() mỗi lần mở (không lưu lá số) — cùng engine lib/tuvi/ với web qua alias @tuvi/*.</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>LaSo KHÔNG lưu trữ vì engine còn sửa — lưu sẵn sẽ mắc kẹt phiên bản cũ, lệch âm thầm với web. Đừng thêm cache LaSo vào AsyncStorage.</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/ho-so.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="30" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Mệnh bàn app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Vẽ lưới 4×4, một phiên bản duy nhất</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>27/09/2026: bỏ 3 chế độ Dễ hiểu/Cổ điển/Chuyên sâu (ChonPhanDoan) — chủ dự án yêu cầu MỘT lưới đầy đủ, fit trọn 12 cung trên một màn hình dọc, không cuộn ngang. VI_TRI định vị 12 cung (khớp VI_TRI_GRID của web), ô rộng = (bề ngang màn hình − lề×2) / 4. Mỗi ô: can-chi, tên cung, chính tinh kèm độ sáng, phụ tinh lọc qua PHU_TINH_TRONG_YEU (tối đa 4), Tuần/Triệt, tuổi đại vận. Ô giữa (4 ô lưới) gộp thành khối bản mệnh (Cục, Bản mệnh, can chi năm).</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Bản trước ô rộng 46% bề ngang màn hình × 4 cột = tràn gấp đôi màn hình, phải cuộn ngang LẪN dọc — phản hồi thật từ chủ dự án. Đảo ngược một phần luật cũ "ô đủ lớn để chạm" (README app) — đổi có chủ đích, đã ghi lại trong README + AGENTS.md + HUONG-DAN.md. Chữ rất nhỏ (token micro 9.5px / nano 8px, thêm mới, CHỈ dùng ở màn này) nên chạm vào ô để xem chi tiết đầy đủ thay vì đọc hết trong ô nhỏ.</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/ban-do.tsx, apps/celes-app/src/thiet-ke/token.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18586,7 +18740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21327,6 +21481,38 @@
       <c r="F85" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="49" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>app-gd1-menh-ban</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>CEL-155, L18</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Viết lại màn "Bản đồ của tôi" trên app: bỏ 3 chế độ Dễ hiểu/Cổ điển/Chuyên sâu, dựng một lưới 4×4 đầy đủ fit một màn hình dọc. Sửa copy bước ngày sinh onboarding ("Ngày bạn bắt đầu câu chuyện này" → "Ngày sinh của bạn").</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Chủ dự án test bản chạy thử qua Expo Go, phản hồi: copy ngày sinh không rõ ý, và lưới lá số cũ (46% bề ngang × 4 cột, chia 3 mức) không fit tỷ lệ màn hình điện thoại — gửi kèm ảnh app đối thủ Altuvi.com làm tham khảo cách trình bày một lưới đầy đủ duy nhất.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
app: menh ban day du nhu web + mau, buoc gio sinh nhu web, sua thang am
- ban-do.tsx: tu hoa, du phu tinh + vong sao hai cot cat/hung, tieu han,
  nguyet han, trang sinh, Tuan/Triet tren bien, tam phuong tu chinh khi cham,
  bang giua nhu CenterPanel, doi nam xem, bat sao luu nam, vach ngu hanh
  theo dia chi cung. Cao hang tinh theo o nhieu sao nhat, khong cat sao.
- onboarding/gio-sinh.tsx: 12 khung gio "23:00 – 00:59 · gio Ty" nhu web,
  lien ket nhap chinh xac va "Toi khong nho gio sinh".
- api.ts, ho-so.tsx, hanh-trinh.tsx, index.tsx: thangXem/namXem lay tu
  bay-gio (thang am) thay vi getMonth()+1 / getFullYear().
- Backlog: CEL-155 cap nhat, CEL-156, CEL-157, L18 buoc 2-3, nhat ky.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O156"/>
+  <dimension ref="A1:O158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13466,20 +13466,21 @@
       </c>
       <c r="C156" s="8" t="inlineStr">
         <is>
-          <t>Mệnh bàn app: một lưới đầy đủ, bỏ 3 chế độ; sửa copy bước ngày sinh</t>
+          <t>Mệnh bàn app: một lưới đầy đủ như web, có màu; sửa copy bước ngày sinh</t>
         </is>
       </c>
       <c r="D156" s="8" t="inlineStr">
         <is>
-          <t>Màn "Bản đồ của tôi" (apps/celes-app/app/ban-do.tsx) viết lại hoàn toàn: bỏ Dễ hiểu/Cổ điển/Chuyên sâu, dựng MỘT lưới 4×4 tĩnh hiện đủ 12 cung trên một màn hình dọc (không cuộn ngang) — can chi, tên cung, chính tinh kèm độ sáng, phụ tinh trọng yếu, Tuần/Triệt, tuổi đại vận. Chạm vào cung mở chi tiết đầy đủ bên dưới. Thêm 2 cỡ chữ mới micro (9.5px) / nano (8px) vào token, CHỈ dùng ở màn này. Đồng thời sửa copy bước 2 onboarding: "Ngày bạn bắt đầu câu chuyện này" → "Ngày sinh của bạn" (không rõ ý theo phản hồi thật).</t>
+          <t>Màn "Bản đồ của tôi" (apps/celes-app/app/ban-do.tsx) là MỘT lưới 4×4 vừa bề ngang màn hình (không cuộn ngang, cuộn dọc). 28/09/2026 bổ sung cho đủ như PalaceCell/CenterPanel của web: tứ hoá (huy hiệu 4 màu), TOÀN BỘ phụ tinh + vòng sao chia hai cột (cát trái, hung phải đỏ, vòng sao nhạt, trọng yếu đậm), Vô chính diệu, độ sáng tô màu (M/V xanh, H đỏ), số đại vận (xanh nếu đang đi qua), chân ô Tiểu hạn / Tràng sinh / T.{tháng âm} nguyệt hạn, nền vàng ô tiểu hạn, nền hồng nhạt ô Mệnh, Tuần/Triệt đặt trên đường biên chung hai cung, chạm ô → tam phương tứ chính (viền xanh tam hợp, viền đậm xung chiếu, còn lại mờ) + thẻ chi tiết cỡ chữ thật chia nhóm sao; bảng giữa đủ 17 dòng như web (dương/âm lịch, giờ, 4 trụ, âm dương, bản mệnh, cục, mệnh–cục, mệnh an tại, thân cư, mệnh chủ, thân chủ, năm xem, tuổi hạn); đổi năm xem ‹ › (44px) và nút bật sao lưu năm; vạch màu ngũ hành theo địa chi cung + chú giải. Đồng thời sửa copy bước ngày sinh ("Ngày sinh của bạn").</t>
         </is>
       </c>
       <c r="E156" s="8" t="inlineStr">
         <is>
-          <t>1. useHoSo() trả LaSo tĩnh (không lưu, tính lại mỗi lần mở)
-2. Lưới 4×4 định vị theo VI_TRI (khớp VI_TRI_GRID của web) — 12 ô biên + khối bản mệnh ở giữa
-3. Chạm một ô → setCungChon → khối chi tiết đầy đủ hiện dưới lưới
-4. Không có state chế độ hiển thị nữa (đã bỏ ChonPhanDoan 3 mức)</t>
+          <t>1. useHoSo() trả LaSo (không lưu, tính lại mỗi lần mở)
+2. namXem mặc định = namAmHienTai(), thangXem = thangAmHienTai()
+3. tachSao(): chính tinh / tứ hoá / cột cát / cột hung (phụ tinh trước vòng sao) / lưu tinh nếu bật
+4. uocCao() ước cao từng ô theo số dòng → cao HÀNG = max các ô trong hàng; hàng 1–2 ≥ 150 để chứa bảng giữa
+5. Chạm ô → chon = chiIndex → tamPhuongTuChinh() tô trạng thái + thẻ chi tiết; chạm lại để bỏ chọn</t>
         </is>
       </c>
       <c r="F156" s="9" t="inlineStr">
@@ -13519,17 +13520,175 @@
       </c>
       <c r="M156" s="8" t="inlineStr">
         <is>
-          <t>Chưa test bằng mắt trên Expo Go/thiết bị thật (chỉ kiểm tsc + expo export bundle — cả hai sạch). Đổi ngược một phần luật cũ "ô đủ lớn để chạm" trong README app — đã cập nhật README + AGENTS.md + HUONG-DAN.md cùng commit này.</t>
+          <t>Chưa soát bằng mắt trên máy thật (đã qua tsc + expo export bundle iOS). Chữ sao trong cột 7.5px, tự co tới 70% khi tên dài — nếu đọc khó trên máy nhỏ thì cân nhắc nút phóng to. Chưa tô màu theo ngũ hành TỪNG SAO (kiểu tuvi.cohoc.net, lyso.vn) vì engine chưa có bảng hành của sao — muốn làm phải thêm bảng vào lib/tuvi và qua celes-domain.</t>
         </is>
       </c>
       <c r="N156" s="8" t="inlineStr">
         <is>
-          <t>27/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="O156" s="8" t="inlineStr">
         <is>
-          <t>app-gd1-menh-ban</t>
+          <t>app-gd1-menh-ban-v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="13" t="inlineStr">
+        <is>
+          <t>CEL-156</t>
+        </is>
+      </c>
+      <c r="B157" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
+        <is>
+          <t>Bước giờ sinh app: 12 khung giờ như web + lối "Tôi không nhớ giờ sinh"</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="inlineStr">
+        <is>
+          <t>Màn onboarding/gio-sinh.tsx bỏ 3 pill "nhớ cụ thể / khoảng / không chắc". Giờ là danh sách chọn một 12 khung hai tiếng ghi giờ đồng hồ trước ("23:00 – 00:59 · giờ Tý"), đúng cách hỏi của FormSinh web; liên kết "Tôi nhớ chính xác giờ phút" mở ô nhập HH:MM; liên kết "Tôi không nhớ giờ sinh" mở hai đoạn giải thích (cùng chữ web khongNhoGioY1/Y2). Không có khung nào được chọn sẵn.</t>
+        </is>
+      </c>
+      <c r="E157" s="8" t="inlineStr">
+        <is>
+          <t>1. khung = null lúc mở → nút Tiếp tắt
+2. Chọn khung → doChacGio = "khoang", gio = giờ ĐẦU khung (23, 1, 3…) như web, phut = 0
+3. Nhập chính xác → doChacGio = "chinh-xac", gio/phut như nhập
+4. "Không nhớ giờ" chỉ giải thích, không cho đi tiếp với giờ mặc định</t>
+        </is>
+      </c>
+      <c r="F157" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G157" s="8" t="inlineStr">
+        <is>
+          <t>Không đổi</t>
+        </is>
+      </c>
+      <c r="H157" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I157" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J157" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/onboarding/gio-sinh.tsx</t>
+        </is>
+      </c>
+      <c r="K157" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/onboarding/gio-sinh.tsx, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L157" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M157" s="8" t="inlineStr">
+        <is>
+          <t>Bản nháp mặc định vẫn gio = 9 / chinh-xac trong ban-nhap.tsx nhưng màn này không đọc nó nữa, nên không có giờ nào bị gán sẵn.</t>
+        </is>
+      </c>
+      <c r="N157" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O157" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-menh-ban-v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="13" t="inlineStr">
+        <is>
+          <t>CEL-157</t>
+        </is>
+      </c>
+      <c r="B158" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C158" s="8" t="inlineStr">
+        <is>
+          <t>Sửa app dùng tháng/năm DƯƠNG lịch làm tháng/năm xem</t>
+        </is>
+      </c>
+      <c r="D158" s="8" t="inlineStr">
+        <is>
+          <t>Bốn chỗ trong app lấy new Date().getMonth()+1 / getFullYear() làm thangXem/namXem: gọi /api/hoi-dap (du-lieu/api.ts), tab Hành trình, tab Hôm nay (giai đoạn đại vận), Quick Read (du-lieu/ho-so.tsx). Nay đều dùng thangAmHienTai()/namAmHienTai() của lib/tuvi/bay-gio.ts như web.</t>
+        </is>
+      </c>
+      <c r="E158" s="8" t="inlineStr">
+        <is>
+          <t>1. Mọi nơi cần "tháng này / năm nay" gọi @tuvi/bay-gio
+2. Không còn getMonth()+1 cho thangXem trong apps/celes-app</t>
+        </is>
+      </c>
+      <c r="F158" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G158" s="8" t="inlineStr">
+        <is>
+          <t>Không đổi</t>
+        </is>
+      </c>
+      <c r="H158" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I158" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J158" s="8" t="inlineStr">
+        <is>
+          <t>/api/hoi-dap, tab Hành trình, tab Hôm nay, Quick Read</t>
+        </is>
+      </c>
+      <c r="K158" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/api.ts, apps/celes-app/src/du-lieu/ho-so.tsx, apps/celes-app/app/(tabs)/hanh-trinh.tsx, apps/celes-app/app/(tabs)/index.tsx</t>
+        </is>
+      </c>
+      <c r="L158" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M158" s="8" t="inlineStr">
+        <is>
+          <t>Đầu năm dương (trước Tết) app từng đọc sai năm hạn, và mọi tháng lệch 1 tháng nguyệt hạn so với web.</t>
+        </is>
+      </c>
+      <c r="N158" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O158" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-menh-ban-v2</t>
         </is>
       </c>
     </row>
@@ -13550,7 +13709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -18709,22 +18868,59 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Vẽ lưới 4×4, một phiên bản duy nhất</t>
+          <t>Vẽ lưới 4×4 đầy đủ như web, một phiên bản duy nhất</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>27/09/2026: bỏ 3 chế độ Dễ hiểu/Cổ điển/Chuyên sâu (ChonPhanDoan) — chủ dự án yêu cầu MỘT lưới đầy đủ, fit trọn 12 cung trên một màn hình dọc, không cuộn ngang. VI_TRI định vị 12 cung (khớp VI_TRI_GRID của web), ô rộng = (bề ngang màn hình − lề×2) / 4. Mỗi ô: can-chi, tên cung, chính tinh kèm độ sáng, phụ tinh lọc qua PHU_TINH_TRONG_YEU (tối đa 4), Tuần/Triệt, tuổi đại vận. Ô giữa (4 ô lưới) gộp thành khối bản mệnh (Cục, Bản mệnh, can chi năm).</t>
+          <t>27/09: bỏ 3 chế độ Dễ hiểu/Cổ điển/Chuyên sâu. 28/09: ô rộng = (bề ngang − 8×2)/4; nội dung ô theo đúng PalaceCell web: can.chi + số đại vận, tên cung + THÂN, chính tinh (độ sáng tô màu) hoặc Vô chính diệu, tứ hoá, hai cột phụ tinh+vòng sao (tinhChat hung → cột phải), lưu tinh nếu bật, chân ô Tiểu hạn/Tràng sinh/T.tháng. Cao ô ước bằng uocCao() theo số dòng; cao hàng = max ô trong hàng; hàng giữa ≥ 150 cho bảng giữa (CAO_O_GIUA 300). Bảng giữa = CenterPanel web. Tuần/Triệt vẽ trên biên chung hai cung (tách ±16 nếu trùng cặp).</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Bản trước ô rộng 46% bề ngang màn hình × 4 cột = tràn gấp đôi màn hình, phải cuộn ngang LẪN dọc — phản hồi thật từ chủ dự án. Đảo ngược một phần luật cũ "ô đủ lớn để chạm" (README app) — đổi có chủ đích, đã ghi lại trong README + AGENTS.md + HUONG-DAN.md. Chữ rất nhỏ (token micro 9.5px / nano 8px, thêm mới, CHỈ dùng ở màn này) nên chạm vào ô để xem chi tiết đầy đủ thay vì đọc hết trong ô nhỏ.</t>
+          <t>KHÔNG cắt bớt sao để vừa ô (bản 27/09 chỉ hiện ≤4 phụ tinh trọng yếu → chủ dự án báo "chưa đủ như web"). Chữ sao dùng numberOfLines=1 + adjustsFontSizeToFit, KHÔNG để gãy giữa tên. Hai cột là phép phân loại cát/hung, không gộp một cột. Không tô màu theo hành từng sao khi engine chưa có bảng hành sao — màu ngũ hành chỉ là vạch theo địa chi cung (NGU_HANH_CHI). Cỡ chữ lưới khai báo trong ban-do.tsx, không đưa vào token chung (đã gỡ micro/nano khỏi token.ts).</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>apps/celes-app/app/ban-do.tsx, apps/celes-app/src/thiet-ke/token.ts</t>
+          <t>apps/celes-app/app/ban-do.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="30" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Mệnh bàn app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Năm xem, hạn, tam phương</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>namXem mặc định namAmHienTai(), đổi bằng ‹ ›; thangXem = thangAmHienTai() cố định. tuoiAm = namXem − năm âm sinh + 1 → cungTieuHan (nền vàng + "Tiểu hạn"), cungNguyetHan (T.{tháng}), cungDaiVan (số đại vận xanh). Sao lưu năm = luuTinhTheoNam(namXem), mặc định TẮT như web. Chạm ô → tamPhuongTuChinh(): chọn viền chữ, tam hợp viền xanh, xung chiếu viền đậm, còn lại opacity 0.3.</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Tháng xem phải là tháng ÂM (thangAmHienTai), không phải getMonth()+1 — xem CEL-157 và docs/bay/engine.md.</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/ban-do.tsx, lib/tuvi/ansao.ts, lib/tuvi/bay-gio.ts</t>
         </is>
       </c>
     </row>
@@ -18740,7 +18936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21513,6 +21709,38 @@
       <c r="F86" t="inlineStr">
         <is>
           <t>Claude Sonnet 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="49" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>app-gd1-menh-ban-v2</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CEL-155, CEL-156, CEL-157, L18</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Mệnh bàn app hiện đủ nội dung như web + màu (tứ hoá, đủ phụ tinh 2 cột cát/hung, hạn, tam phương, bảng giữa, năm xem, sao lưu năm); bước giờ sinh đổi sang 12 khung giờ như web + lối "không nhớ giờ"; sửa 4 chỗ app dùng tháng/năm dương làm tháng/năm xem.</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Chủ dự án test Expo Go: lá số app "vẫn chưa đủ thông tin như web", muốn có màu và đẹp hơn; màn giờ sinh 3 lựa chọn khác hẳn web. Khi rà luồng phát hiện app lấy getMonth()+1 làm tháng âm → lệch nguyệt hạn và câu trả lời của Celes so với web.</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
App: dang nhap bang ma email (Supabase OTP), gui Bearer token khi hoi Celes
- Man dang-nhap hai buoc: email -> ma 6 so; phien luu AsyncStorage, tu lam moi
- hoiCeles gan Authorization: Bearer; 401 canDangNhap -> LoiCanDangNhap
- Tab Celes: chua dang nhap thi giu cau dang go, hien the moi dang nhap
- Tab Toi: nhom Tai khoan (email + dang xuat / moi dang nhap)
- Man dang ky: go nut Apple/Google gia, chi con email + De sau
- .env.example + README; backlog CEL-154, CEL-158, L19

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O158"/>
+  <dimension ref="A1:O159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13399,7 +13399,8 @@
           <t>1. lib/supabase/server.ts đọc header Authorization
 2. Có Bearer → auth.getUser(token) hỏi Supabase xác thực chữ ký + hạn
 3. Client Supabase dựng từ token → RLS chạy dưới đúng người đó
-4. Không có header → đường cookie của web như cũ</t>
+4. Không có header → đường cookie của web như cũ
+5. App: hoiCeles() lấy tokenHienTai() (phiên Supabase trong AsyncStorage) và gắn Authorization: Bearer nếu có</t>
         </is>
       </c>
       <c r="F155" s="9" t="inlineStr">
@@ -13429,7 +13430,7 @@
       </c>
       <c r="K155" s="8" t="inlineStr">
         <is>
-          <t>lib/supabase/server.ts</t>
+          <t>lib/supabase/server.ts, apps/celes-app/src/du-lieu/api.ts, apps/celes-app/src/du-lieu/supabase.ts</t>
         </is>
       </c>
       <c r="L155" s="8" t="inlineStr">
@@ -13439,17 +13440,17 @@
       </c>
       <c r="M155" s="8" t="inlineStr">
         <is>
-          <t>Mới xong nửa máy chủ. App CHƯA có đăng nhập (nút ở màn đăng ký vẫn là 'Để sau') nên chưa có token để gửi. Đã kiểm: không token / token rác / JWT giả mạo chữ ký đều bị coi là khách (401 ở tuyến bắt buộc đăng nhập), không lỗi 500. Chưa kiểm được token hợp lệ vì không có tài khoản thử.</t>
+          <t>Hai nửa đã có (28/09: app gửi token sau khi đăng nhập bằng mã email — CEL-158). Máy chủ nhận Bearer CHỈ có trên nhánh viec/app-gd1: production chưa merge + deploy thì app đã đăng nhập vẫn nhận 401. Chưa chạy thử đầu-cuối với token hợp lệ (cần tạo tài khoản thử trên database dùng chung — chờ chủ dự án đồng ý).</t>
         </is>
       </c>
       <c r="N155" s="8" t="inlineStr">
         <is>
-          <t>27/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="O155" s="8" t="inlineStr">
         <is>
-          <t>app-gd1-bearer</t>
+          <t>app-gd1-dang-nhap-email</t>
         </is>
       </c>
     </row>
@@ -13689,6 +13690,88 @@
       <c r="O158" s="8" t="inlineStr">
         <is>
           <t>app-gd1-menh-ban-v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="13" t="inlineStr">
+        <is>
+          <t>CEL-158</t>
+        </is>
+      </c>
+      <c r="B159" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập bằng mã email trên app</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="inlineStr">
+        <is>
+          <t>Màn app/dang-nhap.tsx hai bước: nhập email → Supabase gửi mã 6 số → nhập mã → có phiên (lưu AsyncStorage, tự làm mới token). Màn đăng ký mềm chỉ còn nút "Tiếp tục với email" + "Để sau" (gỡ nút Apple/Google vì chúng chỉ lặng lẽ để sau). Tab Celes: chưa đăng nhập mà bấm gửi → KHÔNG gửi, giữ nguyên câu đang gõ, hiện thẻ mời đăng nhập; xong quay về đúng màn đó. Tab Tôi: nhóm Tài khoản hiện email + Đăng xuất, hoặc thẻ mời đăng nhập.</t>
+        </is>
+      </c>
+      <c r="E159" s="8" t="inlineStr">
+        <is>
+          <t>1. supabase.ts dựng client từ EXPO_PUBLIC_SUPABASE_URL/ANON_KEY; thiếu một trong hai → coTaiKhoan = false, mọi lối đăng nhập ẩn
+2. guiMa: signInWithOtp({email, shouldCreateUser: true})
+3. xacNhanMa: verifyOtp({email, token, type: "email"})
+4. onAuthStateChange cập nhật phien → các màn tự đổi
+5. Gửi lại mã sau 60 giây; lỗi phân loại email-sai / qua-nhieu / ma-sai / mang / khac
+6. ?sau=quay-lai → router.back(), mặc định vào tabs</t>
+        </is>
+      </c>
+      <c r="F159" s="9" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="G159" s="8" t="inlineStr">
+        <is>
+          <t>Không đổi</t>
+        </is>
+      </c>
+      <c r="H159" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I159" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J159" s="8" t="inlineStr">
+        <is>
+          <t>app/dang-nhap, app/dang-ky, tab Celes, tab Tôi</t>
+        </is>
+      </c>
+      <c r="K159" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/dang-nhap.tsx, apps/celes-app/src/du-lieu/tai-khoan.tsx, apps/celes-app/src/du-lieu/supabase.ts, apps/celes-app/app/dang-ky.tsx, apps/celes-app/app/(tabs)/celes.tsx, apps/celes-app/app/(tabs)/toi.tsx, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L159" s="8" t="inlineStr">
+        <is>
+          <t>Có EXPO_PUBLIC_SUPABASE_URL + EXPO_PUBLIC_SUPABASE_ANON_KEY lúc build</t>
+        </is>
+      </c>
+      <c r="M159" s="8" t="inlineStr">
+        <is>
+          <t>Việc phía Supabase CHƯA làm: (1) mẫu email "Confirm signup" và "Magic Link" phải chứa {{ .Token }} — mẫu mặc định chỉ có đường link nên người dùng không thấy mã; (2) SMTP có sẵn của Supabase giới hạn rất thấp và chỉ gửi tới email thành viên tổ chức — cần SMTP riêng miễn phí (vd. Resend) trước khi có người dùng thật. Google/Apple chưa nối (cần khoá OAuth riêng cho app). Chưa soát trên máy thật.</t>
+        </is>
+      </c>
+      <c r="N159" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O159" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-dang-nhap-email</t>
         </is>
       </c>
     </row>
@@ -13709,7 +13792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G144"/>
+  <dimension ref="A1:G147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -18924,6 +19007,117 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="30" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Đăng nhập app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Cấu hình và phiên</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>supabase.ts: createClient với storage AsyncStorage, persistSession, autoRefreshToken, detectSessionInUrl false; AppState active → startAutoRefresh, nền → stopAutoRefresh. TaiKhoanProvider nằm ngoài HoSoProvider, đọc getSession() lúc mở (dangNap = true cho tới khi xong) rồi nghe onAuthStateChange.</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Chỉ khoá CÔNG KHAI (URL + anon/publishable) được vào app; service role tuyệt đối không. .env.local của app bị gitignore, mẫu ở .env.example.</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/supabase.ts, apps/celes-app/src/du-lieu/tai-khoan.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="30" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Đăng nhập app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Gửi mã và xác nhận</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>guiMa(email) → signInWithOtp (email đã trim + lowercase, shouldCreateUser true). xacNhanMa → verifyOtp type "email"; mã nhận 6–10 chữ số. Lỗi: 429/rate_limit → qua-nhieu; otp_expired/otp_disabled/403 lúc xác nhận → ma-sai; email_address_invalid/validation_failed → email-sai; không có status/AuthRetryableFetchError → mang; còn lại khac. Gửi lại khoá 60 giây.</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Không hiện thông báo gốc của nhà cung cấp cho người dùng — chỉ 5 loại lỗi đã dịch. Mẫu email Supabase phải có {{ .Token }}, không thì luồng này chết im.</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/tai-khoan.tsx, apps/celes-app/app/dang-nhap.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="30" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Đăng nhập app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Chặn và mời ở Celes</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>gui(): coTaiKhoan &amp;&amp; !phien → đặt lại câu vào ô nhập, bật thẻ mời, KHÔNG gọi API. Máy chủ trả 401 kèm canDangNhap → LoiCanDangNhap; nếu lúc đó không có phiên thì rút tin vừa thêm, trả câu về ô nhập, hiện thẻ; còn phiên mà vẫn 401 → bong lỗi chung (tránh vòng lặp mời). Thẻ ẩn khi có phiên (moiDangNhap = canDangNhap &amp;&amp; !phien, không dùng effect).</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Không bao giờ xoá câu người dùng đang gõ vì lý do đăng nhập. App dựng thiếu cấu hình (coTaiKhoan false) vẫn gửi như cũ.</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/(tabs)/celes.tsx, apps/celes-app/src/du-lieu/api.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18936,7 +19130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21739,6 +21933,38 @@
         </is>
       </c>
       <c r="F87" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="49" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>app-gd1-dang-nhap-email</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>CEL-154, CEL-158, L19</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>App có đăng nhập bằng mã 6 số gửi qua email (Supabase OTP), phiên lưu trên máy và tự làm mới; hoiCeles gắn Bearer token; tab Celes mời đăng nhập thay vì báo lỗi; tab Tôi có email + đăng xuất; màn đăng ký gỡ nút Apple/Google giả.</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Máy chủ bắt buộc đăng nhập mới hỏi Celes được, nhưng app chưa có cách đăng nhập nào nên Celes trên app luôn lỗi. Chủ dự án chọn mã email trước (không cần khoá OAuth hay tài khoản Apple Developer, miễn phí); Google để sau. Nút Apple/Google cũ chỉ "để sau" nên người dùng tưởng đã đăng nhập.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
App Celes: sua doc traLoi, tri nho hoi thoai chung web, chip goi y, loi di tiep
- api.ts: hoiCeles doc traLoi/goiYTiep/loiDi (truoc doc noiDung -> luon loi);
  goiApi() dung chung, 402 -> LoiHetLuot
- hoi-thoai.ts: chat_messages theo khoa bam la so khop web (expo-crypto)
- Markdown toi gian nhu MarkdownLuanGiai; the het luot; xoa hoi thoai
- Hom nay: "Hoi Celes ve dieu nay" dien san cau hoi (?q=)
- Backlog CEL-159, L20

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O159"/>
+  <dimension ref="A1:O160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13775,6 +13775,87 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" s="13" t="inlineStr">
+        <is>
+          <t>CEL-159</t>
+        </is>
+      </c>
+      <c r="B160" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C160" s="8" t="inlineStr">
+        <is>
+          <t>Hỏi Celes trên app ngang web: trí nhớ, chip gợi ý, lối đi tiếp, markdown, hết lượt</t>
+        </is>
+      </c>
+      <c r="D160" s="8" t="inlineStr">
+        <is>
+          <t>Sửa lỗi app đọc trường noiDung trong khi /api/hoi-dap trả traLoi (Celes trên app chưa từng hiện được câu trả lời). Hội thoại cất theo lá số trong chat_messages chung với web (khoá sha256 16 hex như bamLaSo), mở app thấy mạch đã hỏi trên web. Chip goiYTiep và lối đi tiếp loiDi dưới lượt cuối của Celes; loiDi đổi đường web → tuyến app (/la-so→bản đồ, /hanh-trinh, /hop-tuoi→Mối quan hệ), đường app chưa có (luận giải) thì ẩn. Lời Celes hiện bằng markdown tối giản như MarkdownLuanGiai. Hết lượt (402): rút câu về ô nhập + thẻ báo, KHÔNG mở cổng thanh toán (tạm ẩn trên iOS). Nút Xoá hội thoại (xác nhận, xoá thật trên máy chủ). "Hỏi Celes về điều này" ở Hôm nay điền sẵn câu hỏi. Gỡ liên kết "Vì sao" chết trong bong bóng chat (web cũng không có căn cứ cho người thường).</t>
+        </is>
+      </c>
+      <c r="E160" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở tab / đổi hồ sơ / đăng nhập → bamLaSo(hoSo) → docHoiThoai(khoa) nếu có phiên, chỉ nạp khi màn trống
+2. gui(cau, tuChip) → hoiCeles gửi lichSu ≤ 60 (bỏ bong lỗi) + tuChip
+3. Thành công → thêm lượt Celes kèm goiYTiep/loiDi, luuLuot cả cặp
+4. 401 canDangNhap khi không có phiên / 402 → rút câu về ô nhập, hiện thẻ tương ứng
+5. Lỗi khác → bong lỗi giọng Celes</t>
+        </is>
+      </c>
+      <c r="F160" s="9" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="G160" s="8" t="inlineStr">
+        <is>
+          <t>Model (qua /api/hoi-dap)</t>
+        </is>
+      </c>
+      <c r="H160" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt hỏi</t>
+        </is>
+      </c>
+      <c r="I160" s="8" t="inlineStr">
+        <is>
+          <t>Người đã đăng nhập (hạn mức ask_celes)</t>
+        </is>
+      </c>
+      <c r="J160" s="8" t="inlineStr">
+        <is>
+          <t>Tab Celes</t>
+        </is>
+      </c>
+      <c r="K160" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/(tabs)/celes.tsx, apps/celes-app/src/du-lieu/api.ts, apps/celes-app/src/du-lieu/hoi-thoai.ts, apps/celes-app/src/du-lieu/tuyen-web.ts, apps/celes-app/src/giao-dien/markdown.tsx, apps/celes-app/app/(tabs)/index.tsx, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L160" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập (CEL-158) + máy chủ nhận Bearer (CEL-154)</t>
+        </is>
+      </c>
+      <c r="M160" s="8" t="inlineStr">
+        <is>
+          <t>Chưa chạy đầu-cuối: production chưa có Bearer (chờ merge + deploy) nên app thật vẫn 401. Lối "Đọc kỹ hơn về …" (/luan-giai?chuDe=) đang ẩn tới khi app có màn luận giải. hoi-thoai.ts là BẢN SAO có chủ đích của lib/store/hoi-thoai.ts (RN không có Web Crypto) — đổi công thức khoá ở một bên phải đổi cả ba chỗ (web, app, lib/rag/nhat-ky.ts).</t>
+        </is>
+      </c>
+      <c r="N160" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O160" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-chat-celes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -13792,7 +13873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G147"/>
+  <dimension ref="A1:G150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19118,6 +19199,117 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="30" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Hỏi Celes trên app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Khoá hội thoại và trí nhớ</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>bamLaSo(hoSo) = expo-crypto SHA256 của `${ngay}-${thang}-${nam}-${gio}-${gioiTinh}`, 16 hex đầu. docHoiThoai: 60 dòng mới nhất theo tao_luc giảm dần rồi lật. luuLuot: insert 2 dòng, tao_luc lệch 1ms. xoaHoiThoai: delete theo phien + user_id. Tất cả im lặng khi hỏng.</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Khoá PHẢI khớp bamLaSo (lib/rag/nhat-ky.ts) và bamLaSoTrinhDuyet (lib/store/hoi-thoai.ts), không thì mạch web và app rẽ làm hai. Không cất câu hỏi trước khi có câu trả lời (để lại câu lơ lửng).</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/hoi-thoai.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="30" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Hỏi Celes trên app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Gửi và xử phản hồi</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>goiApi(): Bearer nếu có; 401+canDangNhap → LoiCanDangNhap; 402 → LoiHetLuot(freeLimit); !ok → LoiCeles. hoiCeles đọc data.traLoi, goiYTiep, loiDi. lichSu gửi lên bỏ bong lỗi, cắt 60. Chip bấm → tuChip true.</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Tên trường là traLoi (không phải noiDung) — đã đọc nhầm một lần và Celes im lặng. App không mở cổng thanh toán khi 402 (iOS 3.1.1).</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/api.ts, apps/celes-app/app/(tabs)/celes.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="30" t="inlineStr">
+        <is>
+          <t>L20</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Hỏi Celes trên app di động (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Lối đi tiếp</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>tuyenApp(duong): /la-so → /ban-do, /hanh-trinh → tab Hành trình, /hop-tuoi → tab Mối quan hệ; đường khác → null (ẩn). Chỉ hiện dưới lượt cuối, khi không chờ.</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Không dẫn người dùng tới tuyến app chưa có. Thêm màn mới thì thêm nhánh ở tuyen-web.ts.</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/tuyen-web.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19130,7 +19322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21965,6 +22157,38 @@
         </is>
       </c>
       <c r="F88" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="49" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>app-gd1-chat-celes</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>CEL-159, L20</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Tab Celes app: sửa đọc traLoi, trí nhớ hội thoại chung với web, chip gợi ý, lối đi tiếp, markdown, báo hết lượt, xoá hội thoại, câu hỏi điền sẵn từ Hôm nay.</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Chủ dự án muốn app thao tác đủ luồng như web. Khi rà phát hiện app đọc sai tên trường nên Celes trên app chưa bao giờ trả lời được; và app thiếu trí nhớ — mở app là Celes quên hết những gì đã kể trên web.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
app: dong bo la so voi tai khoan web + man Nguoi cua toi (CEL-160)
- la-so-luu.ts: doc/ghi bang charts va profiles.la_so_mac_dinh nhu web
- ho-so.tsx: dong bo khi dang nhap, luat 'la so cua toi' theo web, danh sach nguoi
- nguoi-cua-toi.tsx: them / xem / dat lam cua toi / xoa
- ban-do nhan ?id=; dang nhap xong ve diem re (cho dong bo)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O160"/>
+  <dimension ref="A1:O161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13856,6 +13856,87 @@
         </is>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" s="13" t="inlineStr">
+        <is>
+          <t>CEL-160</t>
+        </is>
+      </c>
+      <c r="B161" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C161" s="8" t="inlineStr">
+        <is>
+          <t>Lá số app đồng bộ với tài khoản web + màn Người của tôi (nhiều lá số)</t>
+        </is>
+      </c>
+      <c r="D161" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập trên app thì lá số đọc/ghi CÙNG bảng charts và cột profiles.la_so_mac_dinh với web. Máy mới đăng nhập trước: nhận "lá số của tôi" từ tài khoản, bỏ qua onboarding. Làm onboarding lúc chưa đăng nhập rồi mới đăng nhập: hồ sơ được gắn vào dòng cùng lá số (cùng ngày/tháng/năm, khung giờ, giới tính) hoặc thêm mới; tài khoản đã chọn lá số của mình thì lựa chọn đó thắng. Màn Người của tôi (từ tab Tôi): lá số của tôi + những người khác, thêm người (tên, ngày, 12 khung giờ, giới tính), xem bản đồ (/ban-do?id=), đặt làm lá số của tôi, xoá. Khách lưu danh sách trên máy, đăng nhập thì đẩy lên như chuyenHoSoLenTaiKhoan của web.</t>
+        </is>
+      </c>
+      <c r="E161" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở app → đọc hồ sơ + danh sách trên máy
+2. Có phiên → docCharts + docMacDinh → đẩy người trên máy lên → gắn/đổi hồ sơ theo luật mặc định
+3. Điểm rẽ chờ tới khi đồng bộ xong mới chọn Hôm nay hay giới thiệu
+4. Đăng nhập xong (không phải quay lại) → về điểm rẽ
+5. Người của tôi: thêm / xem / đặt làm của tôi / xoá</t>
+        </is>
+      </c>
+      <c r="F161" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G161" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="H161" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần mở app có phiên, mỗi lần đăng nhập</t>
+        </is>
+      </c>
+      <c r="I161" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người (khách lưu trên máy)</t>
+        </is>
+      </c>
+      <c r="J161" s="8" t="inlineStr">
+        <is>
+          <t>Tab Tôi → Người của tôi</t>
+        </is>
+      </c>
+      <c r="K161" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/la-so-luu.ts, apps/celes-app/src/du-lieu/ho-so.tsx, apps/celes-app/app/nguoi-cua-toi.tsx, apps/celes-app/app/ban-do.tsx, apps/celes-app/app/dang-nhap.tsx, apps/celes-app/app/(tabs)/toi.tsx, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L161" s="8" t="inlineStr">
+        <is>
+          <t>CEL-158 (đăng nhập mã email)</t>
+        </is>
+      </c>
+      <c r="M161" s="8" t="inlineStr">
+        <is>
+          <t>Bảng charts không có phút, độ chắc giờ, điều bận tâm — những thứ đó chỉ còn trên máy; lá số nhận từ tài khoản coi như phút 0. Chưa chạy thử với tài khoản thật (cần người dùng thử + đồng ý tạo dữ liệu trên DB chung). Mối quan hệ chưa dùng danh sách này (giai đoạn 5).</t>
+        </is>
+      </c>
+      <c r="N161" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O161" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-nguoi-cua-toi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -13873,7 +13954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:G153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19310,6 +19391,117 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="30" t="inlineStr">
+        <is>
+          <t>L21</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Lá số của tôi trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Đồng bộ khi có phiên</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Chạy khi userId đổi, hoặc khi hồ sơ trên máy chưa có chartId. docCharts + docMacDinh; người trên máy → ganVao (khớp cungLaSo, không có thì insert) rồi xoá bản máy. Hồ sơ chưa gắn: ganVao; nếu tài khoản có mặc định KHÁC dòng vừa gắn → hồ sơ = dòng mặc định; không có mặc định → đặt dòng vừa gắn làm mặc định. Không hồ sơ mà có mặc định → nhận dòng mặc định (phút 0, doChacGio khoang). Lỗi → dùng tiếp dữ liệu máy.</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Không bao giờ lấy dòng đầu danh sách làm của tôi (docs/bay/giao-dien.md). Không ghi đè mặc định tài khoản đã chọn. Hồ sơ trên máy khác mặc định vẫn được lưu lên, không mất.</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/ho-so.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="30" t="inlineStr">
+        <is>
+          <t>L21</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Lá số của tôi trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Cùng lá số</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>cungLaSo: cùng ngày, tháng, năm, giới tính và cùng khung giờ khungGio(gio) = floor(((gio+1)%24)/2). Giờ lưu là giờ thật 0–23 như web; form Người của tôi lưu giờ đầu khung (23,1,3…).</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>So theo khung giờ, không theo giờ tuyệt đối: web lưu giờ đầu khung còn onboarding app lưu giờ thật, so tuyệt đối sẽ tạo bản trùng.</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/la-so-luu.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="30" t="inlineStr">
+        <is>
+          <t>L21</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Lá số của tôi trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Điểm rẽ và đặt làm của tôi</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>dangTai = chưa đọc máy || đang đọc phiên || (có phiên &amp;&amp; chưa đồng bộ xong cho userId đó). Đăng nhập thành công → dismissAll + về "/". Đặt làm của tôi: có phiên → upsert la_so_mac_dinh + hồ sơ = dòng đó; khách → hồ sơ cũ xuống danh sách, người được chọn lên làm hồ sơ.</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Hôm nay, Hành trình, Celes luôn đọc hoSo (= của tôi). Xem người khác chỉ qua /ban-do?id=, không đổi hoSo.</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/ho-so.tsx, apps/celes-app/app/nguoi-cua-toi.tsx, apps/celes-app/app/dang-nhap.tsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19322,7 +19514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22189,6 +22381,38 @@
         </is>
       </c>
       <c r="F89" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="49" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>app-gd1-nguoi-cua-toi</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>CEL-160, L21</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>App đồng bộ lá số với tài khoản (charts + la_so_mac_dinh), màn Người của tôi, bản đồ mở được lá số người khác, đăng nhập xong về điểm rẽ.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Trước đây lá số app chỉ nằm trên máy: đăng nhập cùng tài khoản với web mà không thấy lá số nào, máy mới phải nhập lại, và không có chỗ lưu lá số người thân — thiếu nền cho luận giải và Mối quan hệ ở các giai đoạn sau.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
App: luận giải — tổng quan, 14 mặt đời, tóm lại, bức tranh lớn (CEL-161)
Cùng /api/luan-giai-v3 và cách chia lượt với web để dùng chung bộ đệm.
Khung câu hỏi đọc thẳng từ lib/rag/v3/khung.ts qua bí danh @khung-v3.
Nối từ Hôm nay → Khám phá và từ lối đi tiếp /luan-giai của Celes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O161"/>
+  <dimension ref="A1:O162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13937,6 +13937,86 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="13" t="inlineStr">
+        <is>
+          <t>CEL-161</t>
+        </is>
+      </c>
+      <c r="B162" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>Luận giải trên app: tổng quan, 14 mặt đời, bức tranh lớn</t>
+        </is>
+      </c>
+      <c r="D162" s="8" t="inlineStr">
+        <is>
+          <t>Mục lục /luan-giai (từ Hôm nay → Khám phá một chủ đề): Tổng quan, 14 chủ đề theo CHU_DE_V3, Bức tranh lớn. Màn /luan-giai/[nhom] gọi CÙNG /api/luan-giai-v3 với web (namXem = năm dương lịch) nên dùng chung bộ đệm noi_dung_ai với web. Mỗi câu: câu hỏi, bài luận, "Muốn biết vì sao không?" ẩn mặc định. Chủ đề có phần Tóm lại, nút Đọc tiếp chủ đề sau / Xem bức tranh lớn, nút Hỏi Celes điền sẵn câu hỏi ở tab Celes. Lối đi tiếp /luan-giai?chuDe= và /luan-giai/sau?chuDe= của Celes giờ mở được màn tương ứng.</t>
+        </is>
+      </c>
+      <c r="E162" s="8" t="inlineStr">
+        <is>
+          <t>1. Hôm nay → Khám phá một chủ đề → mục lục
+2. Chọn Tổng quan (khách đọc được) hoặc một chủ đề (cần đăng nhập)
+3. Lượt 1 hiện trước, lượt 2 viết tiếp, rồi Tóm lại
+4. Đọc tiếp chủ đề sau / Hỏi Celes / Bức tranh lớn</t>
+        </is>
+      </c>
+      <c r="F162" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G162" s="8" t="inlineStr">
+        <is>
+          <t>Không (không trừ lượt)</t>
+        </is>
+      </c>
+      <c r="H162" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần mở một bài</t>
+        </is>
+      </c>
+      <c r="I162" s="8" t="inlineStr">
+        <is>
+          <t>Tổng quan: mọi người; chủ đề + bức tranh lớn: đã đăng nhập</t>
+        </is>
+      </c>
+      <c r="J162" s="8" t="inlineStr">
+        <is>
+          <t>Hôm nay → Khám phá; lối đi tiếp trong chat</t>
+        </is>
+      </c>
+      <c r="K162" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/luan-giai/index.tsx, apps/celes-app/app/luan-giai/[nhom].tsx, apps/celes-app/app/luan-giai/buc-tranh.tsx, apps/celes-app/src/giao-dien/luan-giai.tsx, apps/celes-app/src/du-lieu/api.ts, apps/celes-app/src/du-lieu/tuyen-web.ts, apps/celes-app/app/(tabs)/index.tsx, apps/celes-app/tsconfig.json, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L162" s="8" t="inlineStr">
+        <is>
+          <t>CEL-158 (Bearer), CEL-160 (lá số đồng bộ), khung v3 lib/rag/v3/khung.ts</t>
+        </is>
+      </c>
+      <c r="M162" s="8" t="inlineStr">
+        <is>
+          <t>Bài chỉ viết bằng tiếng Việt; giao diện EN có dòng báo. Chưa có nút Tạo bản mới và xuất bài như web. Chưa chạy thật: production chưa nhận Bearer (chờ merge viec/app-gd1).</t>
+        </is>
+      </c>
+      <c r="N162" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O162" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-luan-giai</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -13954,7 +14034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19502,6 +19582,117 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" s="30" t="inlineStr">
+        <is>
+          <t>L22</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Luận giải trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Chia lượt</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Tổng quan: lượt 1 = TQ02, TQ03, TQ08 (ba thẻ đầu web), lượt 2 = các câu tong-quan còn lại. Chủ đề: ids = câu chuyen-sau của chủ đề; n ≥ 4 thì lượt 1 = ceil(n/2) câu đầu, còn lại lượt 2. Hai lượt NỐI TIẾP, rồi một lượt tomLai (không có với tổng quan).</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Cùng cách chia với web để trúng bộ đệm; nối tiếp vì song song làm lượt đầu chậm hơn (đo 25/09/2026). Lượt 2 hỏng không xoá lượt 1.</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/luan-giai/[nhom].tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="30" t="inlineStr">
+        <is>
+          <t>L22</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Luận giải trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Đăng nhập và lỗi</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Chủ đề / bức tranh lớn mà chưa có phiên → hiện thẻ mời đăng nhập, KHÔNG gọi máy chủ. 401 canDangNhap → cùng thẻ; 429 gioiHanKhach → thẻ với lời báo hết lượt khách trong ngày. Lỗi khác → lời báo chung + Thử lại. tomLai hỏng thì bỏ qua lặng lẽ.</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Không lộ tên model / quota. Đăng nhập mở với sau=quay-lai để về đúng bài.</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/api.ts, apps/celes-app/app/luan-giai/[nhom].tsx, apps/celes-app/app/luan-giai/buc-tranh.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="30" t="inlineStr">
+        <is>
+          <t>L22</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Luận giải trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Đổi đường dẫn web</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>/luan-giai?chuDe=x: tong-quan, su-nghiep, tinh-duyen, suc-khoe, van-han giữ nguyên; tai-chinh → tien-bac; gia-dao → gia-dinh; khác/không có → mục lục. /luan-giai/sau?chuDe=x → /luan-giai/x.</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>chuDe cũ của web khác id khung v3 ở hai chỗ; id không có trong khung → màn báo trống, không lỗi.</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/tuyen-web.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19514,7 +19705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22413,6 +22604,38 @@
         </is>
       </c>
       <c r="F90" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="49" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>app-gd1-luan-giai</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>CEL-161, L22</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>App có luận giải: mục lục, tổng quan, 14 mặt đời, tóm lại, bức tranh lớn; nối từ Hôm nay và từ lối đi tiếp của Celes.</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Chủ dự án muốn app thao tác đủ luồng như web. Dùng lại /api/luan-giai-v3 (không tuyến cũ /api/luan-giai vì tuyến đó trả tên model) và đọc khung câu hỏi thẳng từ lib/rag/v3/khung.ts qua bí danh @khung-v3 thay vì chép, để app và web không lệch câu hỏi.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
App: Hành trình có chữ Celes viết + màn Xem chi tiết luận hạn (CEL-162)
Nhịp hiện tại + ba chuyển động (/api/nhip), ba lớp mốc từ engine có chữ
model (/api/moc), màn chi-tiet-han gọi /api/luan-han.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O162"/>
+  <dimension ref="A1:O163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -14017,6 +14017,86 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" s="13" t="inlineStr">
+        <is>
+          <t>CEL-162</t>
+        </is>
+      </c>
+      <c r="B163" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t>Hành trình trên app có chữ Celes viết + tầng Xem chi tiết</t>
+        </is>
+      </c>
+      <c r="D163" s="8" t="inlineStr">
+        <is>
+          <t>Tab Hành trình dựng lại theo web: thẻ nhịp hiện tại (nhipHienTai) + ba chuyển động Đang mở ra / Đang căng / Cần chờ (/api/nhip); ba lớp Giai đoạn / Năm (lùi-tới 7 năm) / Tháng dùng cacGiaiDoan, cacNam, cacThang của engine, mốc đang chọn hiện thẻ góc nhìn có Vì sao, chữ mốc thay bằng chữ model (/api/moc) khi về. Màn /chi-tiet-han gọi /api/luan-han: tiêu đề, ba chuyển động, chủ đề chính, nhịp hành động, nên tận dụng / lưu ý, luận theo lĩnh vực, căn cứ (đóng sẵn), nút Hỏi Celes điền sẵn cauHoiGoiY. Khách vẫn đọc lớp tất định, có thẻ mời đăng nhập.</t>
+        </is>
+      </c>
+      <c r="E163" s="8" t="inlineStr">
+        <is>
+          <t>1. Tab Hành trình → thẻ nhịp + chọn lớp
+2. Chọn mốc → thẻ góc nhìn → Xem chi tiết
+3. Chi tiết: đủ quyền thì đọc sâu, chưa thì thẻ khoá không có nút mua
+4. Hỏi Celes về giai đoạn này</t>
+        </is>
+      </c>
+      <c r="F163" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G163" s="8" t="inlineStr">
+        <is>
+          <t>Không (không trừ lượt)</t>
+        </is>
+      </c>
+      <c r="H163" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần mở tab / đổi năm, tháng</t>
+        </is>
+      </c>
+      <c r="I163" s="8" t="inlineStr">
+        <is>
+          <t>Lớp tất định: mọi người; chữ model + chi tiết: đã đăng nhập; đọc sâu chi tiết: người ủng hộ</t>
+        </is>
+      </c>
+      <c r="J163" s="8" t="inlineStr">
+        <is>
+          <t>Tab Hành trình; lối đi tiếp /hanh-trinh/chi-tiet của Celes</t>
+        </is>
+      </c>
+      <c r="K163" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/(tabs)/hanh-trinh.tsx, apps/celes-app/app/chi-tiet-han.tsx, apps/celes-app/src/du-lieu/api.ts, apps/celes-app/src/du-lieu/tuyen-web.ts, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L163" s="8" t="inlineStr">
+        <is>
+          <t>CEL-158 (Bearer), lib/tuvi/hanh-trinh.ts, lib/tuvi/luan-han.ts</t>
+        </is>
+      </c>
+      <c r="M163" s="8" t="inlineStr">
+        <is>
+          <t>Thanh toán ẩn trên iOS nên tài khoản miễn phí chỉ thấy tiêu đề + chủ đề chính ở chi tiết. Chưa có chọn lá số người khác như ô chọn của web. Chưa chạy thật: production chưa nhận Bearer.</t>
+        </is>
+      </c>
+      <c r="N163" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O163" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-hanh-trinh</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -14034,7 +14114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G156"/>
+  <dimension ref="A1:G158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19693,6 +19773,80 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" s="30" t="inlineStr">
+        <is>
+          <t>L23</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Hành trình trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Chữ model cho mốc và nhịp</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Có phiên → song song /api/moc cho giai-doan, nam, thang (namXem = năm ÂM đang chọn) + /api/nhip (cap thang, năm/tháng âm đang chọn). Kết quả gắn khoá lá số + năm (+ tháng) + ngôn ngữ; khoá lệch thì bỏ. Mốc nào có chữ model thì thay chuDe, không thì giữ câu engine. Lỗi/204 → im lặng.</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Năm âm như web để trúng đệm noi_dung_ai. Không phiên thì không gọi (tuyến cần đăng nhập).</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/(tabs)/hanh-trinh.tsx, apps/celes-app/src/du-lieu/api.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="30" t="inlineStr">
+        <is>
+          <t>L23</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Hành trình trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Xem chi tiết</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Giai đoạn đang chọn → năm gửi đi = năm âm đang chọn nếu nằm trong giai đoạn, không thì năm âm của tuổi đầu giai đoạn. /api/luan-han trả day=false → chỉ tiêu đề, subline, chủ đề chính + thẻ khoá. Nhãn khối lấy từ KHUON[ngonNgu].luanHan của engine.</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Web gửi năm đang chọn kể cả khi xem giai đoạn khác — app sửa để chi tiết khớp giai đoạn đang chọn.</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/chi-tiet-han.tsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19705,7 +19859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22636,6 +22790,38 @@
         </is>
       </c>
       <c r="F91" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="49" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>app-gd1-hanh-trinh</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CEL-162, L23</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Tab Hành trình app dựng lại theo web (nhịp, ba chuyển động, ba lớp mốc có chữ Celes) + màn Xem chi tiết luận hạn.</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Tab cũ chỉ hiện tên cung và tên sao — vừa là thuật ngữ ở lớp đầu, vừa không có chữ nào để đọc. Dùng thẳng engine qua @tuvi để app và web cùng mốc, cùng đệm.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
app: Moi quan he so hai la so theo y dinh (CEL-163)
Tab Moi quan he dung lai theo /hop-tuoi: chon nguoi thu hai trong Nguoi cua
toi, chon y dinh + cau hoi, goi /api/hop-tuoi. Ket luan truoc, can cu va bang
ky thuat dong san, khong diem tong. 402 ra the khoa khong nut mua (thanh toan
tam an tren iOS); ten model may chu tra ve khong vao man hinh.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O163"/>
+  <dimension ref="A1:O164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -14097,6 +14097,86 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" s="13" t="inlineStr">
+        <is>
+          <t>CEL-163</t>
+        </is>
+      </c>
+      <c r="B164" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C164" s="8" t="inlineStr">
+        <is>
+          <t>Mối quan hệ trên app: so hai lá số theo ý định</t>
+        </is>
+      </c>
+      <c r="D164" s="8" t="inlineStr">
+        <is>
+          <t>Tab Mối quan hệ dựng lại theo /hop-tuoi của web: người thứ nhất là lá số của bạn, người thứ hai chọn trong Người của tôi (hoặc thêm mới); chọn một trong năm ý định (tình cảm, làm ăn, bạn bè &amp; đồng nghiệp, gia đình, một điều khác) + câu hỏi riêng (bắt buộc ≥10 ký tự với "một điều khác"). Gọi /api/hop-tuoi: kết luận trước (đang chú ý, các mục theo ý định, câu hỏi của bạn), căn cứ đóng sẵn, Hỏi Celes thêm, bảng kỹ thuật đóng sẵn. Không có điểm tổng. Phía AI hỏng thì vẫn hiện bảng so của engine + nút thử lại.</t>
+        </is>
+      </c>
+      <c r="E164" s="8" t="inlineStr">
+        <is>
+          <t>1. Tab Mối quan hệ → chọn người thứ hai
+2. Chọn ý định, gõ câu hỏi nếu có
+3. Bấm nút theo ý định → kết quả
+4. Hỏi Celes thêm về hai người</t>
+        </is>
+      </c>
+      <c r="F164" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G164" s="8" t="inlineStr">
+        <is>
+          <t>Không (không trừ lượt)</t>
+        </is>
+      </c>
+      <c r="H164" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần so một cặp</t>
+        </is>
+      </c>
+      <c r="I164" s="8" t="inlineStr">
+        <is>
+          <t>Đã đăng nhập + người ủng hộ (connectionFull); còn lại thẻ mời đăng nhập / thẻ khoá không nút mua</t>
+        </is>
+      </c>
+      <c r="J164" s="8" t="inlineStr">
+        <is>
+          <t>Tab Mối quan hệ; Khám phá ở Hôm nay; lối đi tiếp /hop-tuoi của Celes</t>
+        </is>
+      </c>
+      <c r="K164" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/(tabs)/ket-noi.tsx, apps/celes-app/src/du-lieu/api.ts, apps/celes-app/src/du-lieu/su-kien.ts, apps/celes-app/src/i18n/vi.ts, apps/celes-app/src/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L164" s="8" t="inlineStr">
+        <is>
+          <t>CEL-158 (Bearer), CEL-160 (Người của tôi), app/api/hop-tuoi, lib/ket-noi/y-dinh.ts</t>
+        </is>
+      </c>
+      <c r="M164" s="8" t="inlineStr">
+        <is>
+          <t>Thanh toán ẩn trên iOS. Người thứ nhất cố định là lá số của bạn (web cho chọn cả hai). Máy chủ viết bằng tiếng Việt. Chưa chạy thật: production chưa nhận Bearer.</t>
+        </is>
+      </c>
+      <c r="N164" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O164" s="8" t="inlineStr">
+        <is>
+          <t>app-gd1-moi-quan-he</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -14114,7 +14194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19847,6 +19927,80 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" s="30" t="inlineStr">
+        <is>
+          <t>L24</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Mối quan hệ trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Chọn người và ý định</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Người thứ hai = nguoi lọc bỏ laCuaToi; id đã chọn không còn thì rơi về người đầu. Ý định mặc định tình cảm; id ý định trùng lib/ket-noi/y-dinh.ts. Kết quả gắn khoá id người + ý định + câu hỏi; đổi bất kỳ thứ nào là kết quả cũ ẩn đi.</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Không lấy nguoi[0] làm người thứ hai khi chưa lọc laCuaToi — dễ so bạn với chính bạn.</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/(tabs)/ket-noi.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="30" t="inlineStr">
+        <is>
+          <t>L24</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Mối quan hệ trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Gọi và hiển thị</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>POST /api/hop-tuoi {a, b, comparison:{intent, question}}. 402 → thẻ khoá (paywall_viewed connection_full), 401 → mời đăng nhập, lỗi khác → thử lại. Có ketNoi → kết luận trước, bảng sau; thiếu ketNoi → câu báo + bảng soSanh + thử lại.</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>docKetNoi chỉ nhận soSanh + ketNoi; model và loiAi máy chủ trả về không bao giờ vào màn hình.</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/du-lieu/api.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19859,7 +20013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22822,6 +22976,38 @@
         </is>
       </c>
       <c r="F92" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="49" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>app-gd1-moi-quan-he</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CEL-163, L24</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Tab Mối quan hệ app dựng lại: chọn người đã lưu + ý định + câu hỏi, gọi /api/hop-tuoi, kết luận trước bảng kỹ thuật sau.</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Tab cũ là khung tĩnh, nút Thêm một người không làm gì. Dùng cùng tuyến máy chủ với web để hai bên cùng mục, cùng quyền, và không lộ tên model.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
Cung hoa production: test engine, ngay co that, admin dong mac dinh, trang loi, gioi han toc do, CI
- scripts/test-ansao-chuan.ts: cong thuc sach doc lap + 2000 la so ngau nhien + 60 mau dong bang
- lib/tuvi/kiem-ngay.ts: chan 31/4, 29/2 nam thuong o form va 11 route API
- ADMIN_EMAILS rong chi mo khi khong phai production
- app/error.tsx, app/global-error.tsx, app/not-found.tsx
- proxy.ts: 40 luot / 60 giay / IP cho route goi model, tra 429
- .github/workflows/kiem-tra.yml + scripts/dem-loi-lint.mjs (moc 5)
- PRODUCT-BACKLOG: CEL-164..168, L18, nhat ky

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O154"/>
+  <dimension ref="A1:O159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13373,6 +13373,398 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" s="13" t="inlineStr">
+        <is>
+          <t>CEL-164</t>
+        </is>
+      </c>
+      <c r="B155" s="14" t="inlineStr">
+        <is>
+          <t>H. Vận hành</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>Test engine an sao tự đối chiếu + mẫu đóng băng</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="inlineStr">
+        <is>
+          <t>scripts/test-ansao-chuan.ts kiểm engine theo ba lớp: (1) công thức sách viết độc lập với hằng số engine, quét 2.000 lá số giả ngẫu nhiên 1930–2035 (Mệnh/Thân, Cục, 14 chính tinh, Lộc Tồn/Kình/Đà, lục cát lục sát chính, Tứ Hoá trừ các can có dị bản, Tuần/Triệt, đại vận, Tràng Sinh, biên giờ Tý); (2) mốc Tết và tháng nhuận; (3) 60 lá số đóng băng ở scripts/mau-ansao.json.</t>
+        </is>
+      </c>
+      <c r="E155" s="8" t="inlineStr">
+        <is>
+          <t>1. Chạy offline, không cần khoá
+2. Kết quả khác mẫu mà PHUONG_PHAP.phienBan không đổi → SAI
+3. Đổi quy tắc có chủ đích: tăng phienBan rồi chạy --cap-nhat</t>
+        </is>
+      </c>
+      <c r="F155" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G155" s="8" t="inlineStr">
+        <is>
+          <t>Tất định</t>
+        </is>
+      </c>
+      <c r="H155" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi commit (CI)</t>
+        </is>
+      </c>
+      <c r="I155" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J155" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K155" s="8" t="inlineStr">
+        <is>
+          <t>scripts/test-ansao-chuan.ts, scripts/mau-ansao.json</t>
+        </is>
+      </c>
+      <c r="L155" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M155" s="8" t="inlineStr">
+        <is>
+          <t>Tứ Hoá bỏ qua Khoa Mậu/Canh/Nhâm và Kỵ Canh vì dị bản. Đã thử làm hỏng Văn Khúc: test báo 2.009 lỗi.</t>
+        </is>
+      </c>
+      <c r="N155" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O155" s="8" t="inlineStr">
+        <is>
+          <t>cung-hoa-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="13" t="inlineStr">
+        <is>
+          <t>CEL-165</t>
+        </is>
+      </c>
+      <c r="B156" s="14" t="inlineStr">
+        <is>
+          <t>A. Engine lá số</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t>Chặn ngày dương lịch không có thật</t>
+        </is>
+      </c>
+      <c r="D156" s="8" t="inlineStr">
+        <is>
+          <t>Engine đổi ngày qua số Julian nên 31/4 lặng lẽ thành 1/5, 31/2 thành 2/3 — người gõ nhầm nhận lá số của ngày khác. Thêm lib/tuvi/kiem-ngay.ts (laNgayDuongCoThat) và chặn ở form web lẫn 11 route API nhận ngày sinh.</t>
+        </is>
+      </c>
+      <c r="E156" s="8" t="inlineStr">
+        <is>
+          <t>1. BuocNhapSinh: nút Tiếp tục tắt khi ngày không có thật (Date.parse của V8 không bắt được)
+2. Route: trả 400 như dữ liệu sai trước khi gọi lapLaSo</t>
+        </is>
+      </c>
+      <c r="F156" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G156" s="8" t="inlineStr">
+        <is>
+          <t>Tất định</t>
+        </is>
+      </c>
+      <c r="H156" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I156" s="8" t="inlineStr">
+        <is>
+          <t>Khách trở lên</t>
+        </is>
+      </c>
+      <c r="J156" s="8" t="inlineStr">
+        <is>
+          <t>/, /la-so, mọi /api nhận ngày sinh</t>
+        </is>
+      </c>
+      <c r="K156" s="8" t="inlineStr">
+        <is>
+          <t>lib/tuvi/kiem-ngay.ts, components/laso/BuocNhapSinh.tsx, app/api/*/route.ts</t>
+        </is>
+      </c>
+      <c r="L156" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M156" s="8" t="inlineStr">
+        <is>
+          <t>App di động (apps/celes-app) chưa gắn kiểm tra này ở form nhập.</t>
+        </is>
+      </c>
+      <c r="N156" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O156" s="8" t="inlineStr">
+        <is>
+          <t>cung-hoa-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="13" t="inlineStr">
+        <is>
+          <t>CEL-166</t>
+        </is>
+      </c>
+      <c r="B157" s="14" t="inlineStr">
+        <is>
+          <t>D. Quản trị</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
+        <is>
+          <t>Trang quản trị đóng khi ADMIN_EMAILS rỗng trên production</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="inlineStr">
+        <is>
+          <t>Trước: ADMIN_EMAILS rỗng = ai đăng nhập cũng là admin (kèm miễn hạn mức AI). Nay rỗng chỉ mở khi NODE_ENV khác production (next dev). Supabase chưa cấu hình trên production thì /admin và API quản trị trả "Chưa bật đăng nhập".</t>
+        </is>
+      </c>
+      <c r="E157" s="8" t="inlineStr">
+        <is>
+          <t>1. laAdmin(): danh sách rỗng → NODE_ENV !== production
+2. app/admin/layout.tsx, lib/rag/cong-quan-tri.ts, app/api/ai/test: thiếu Supabase trên production → chặn (503)</t>
+        </is>
+      </c>
+      <c r="F157" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G157" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H157" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I157" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="J157" s="8" t="inlineStr">
+        <is>
+          <t>/admin, /api/admin/*</t>
+        </is>
+      </c>
+      <c r="K157" s="8" t="inlineStr">
+        <is>
+          <t>lib/supabase/config.ts, app/admin/layout.tsx, lib/rag/cong-quan-tri.ts</t>
+        </is>
+      </c>
+      <c r="L157" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M157" s="8" t="inlineStr">
+        <is>
+          <t>Vercel bản xem thử cũng là production → phải đặt ADMIN_EMAILS ở mọi môi trường cần vào quản trị.</t>
+        </is>
+      </c>
+      <c r="N157" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O157" s="8" t="inlineStr">
+        <is>
+          <t>cung-hoa-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="13" t="inlineStr">
+        <is>
+          <t>CEL-167</t>
+        </is>
+      </c>
+      <c r="B158" s="14" t="inlineStr">
+        <is>
+          <t>G. Trải nghiệm &amp; giao diện</t>
+        </is>
+      </c>
+      <c r="C158" s="8" t="inlineStr">
+        <is>
+          <t>Trang lỗi và trang không tìm thấy</t>
+        </is>
+      </c>
+      <c r="D158" s="8" t="inlineStr">
+        <is>
+          <t>app/error.tsx (lỗi runtime dưới layout, hai thứ tiếng qua i18n loiTrang), app/global-error.tsx (layout gốc hỏng, tự có html/body, chữ viết thẳng hai thứ tiếng), app/not-found.tsx. Không lộ chi tiết kỹ thuật; chỉ ghi digest ra console.</t>
+        </is>
+      </c>
+      <c r="E158" s="8" t="inlineStr">
+        <is>
+          <t>1. Lỗi → câu trấn an "dữ liệu còn nguyên" + nút Thử lại (retry) + về trang chủ
+2. Đường dẫn sai → not-found</t>
+        </is>
+      </c>
+      <c r="F158" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G158" s="8" t="inlineStr">
+        <is>
+          <t>Tất định</t>
+        </is>
+      </c>
+      <c r="H158" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I158" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J158" s="8" t="inlineStr">
+        <is>
+          <t>toàn trang</t>
+        </is>
+      </c>
+      <c r="K158" s="8" t="inlineStr">
+        <is>
+          <t>app/error.tsx, app/global-error.tsx, app/not-found.tsx, lib/i18n/vi.ts, lib/i18n/en.ts</t>
+        </is>
+      </c>
+      <c r="L158" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M158" s="8" t="inlineStr">
+        <is>
+          <t>Next 16: prop là retry, không phải reset.</t>
+        </is>
+      </c>
+      <c r="N158" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O158" s="8" t="inlineStr">
+        <is>
+          <t>cung-hoa-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="13" t="inlineStr">
+        <is>
+          <t>CEL-168</t>
+        </is>
+      </c>
+      <c r="B159" s="14" t="inlineStr">
+        <is>
+          <t>D. Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="inlineStr">
+        <is>
+          <t>Giới hạn tốc độ route gọi model + CI GitHub Actions</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="inlineStr">
+        <is>
+          <t>proxy.ts đếm POST vào các route tốn model theo IP (lib/gioi-han-toc-do.ts, cửa sổ 60 giây, tối đa 40 lượt, trong bộ nhớ một instance). Vượt → 429 + Retry-After, lời nhắn không lộ model. .github/workflows/kiem-tra.yml chạy tsc, đếm lỗi lint (mốc 5), các test offline và next build ở mọi lần đẩy nhánh.</t>
+        </is>
+      </c>
+      <c r="E159" s="8" t="inlineStr">
+        <is>
+          <t>1. proxy(): POST + laRouteTonModel → ghiLuotGoi(ip)
+2. &gt;0 giây chờ → 429
+3. CI: không cần secret</t>
+        </is>
+      </c>
+      <c r="F159" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G159" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H159" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lần gọi / mỗi lần đẩy</t>
+        </is>
+      </c>
+      <c r="I159" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J159" s="8" t="inlineStr">
+        <is>
+          <t>/api/hoi-dap, /api/luan-giai*, /api/ban-doc-sau, /api/luan-han, /api/diem-noi-bat, /api/moc, /api/nhip, /api/hop-tuoi</t>
+        </is>
+      </c>
+      <c r="K159" s="8" t="inlineStr">
+        <is>
+          <t>lib/gioi-han-toc-do.ts, proxy.ts, .github/workflows/kiem-tra.yml, scripts/dem-loi-lint.mjs</t>
+        </is>
+      </c>
+      <c r="L159" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M159" s="8" t="inlineStr">
+        <is>
+          <t>Giới hạn mềm: hai instance đếm riêng (ngân sách 0, không Redis). Hạn mức ngày vẫn là hàng rào chính. Thêm route AI mới phải thêm vào ROUTE_TON_MODEL.</t>
+        </is>
+      </c>
+      <c r="N159" s="8" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="O159" s="8" t="inlineStr">
+        <is>
+          <t>cung-hoa-production</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -13390,7 +13782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13465,7 +13857,7 @@
       </c>
       <c r="F2" s="32" t="inlineStr">
         <is>
-          <t>Máy chủ kiểm lại mọi số: ngày 1-31, tháng 1-12, năm 1900-2100, giờ 0-23. Không tin dữ liệu từ trình duyệt.</t>
+          <t>Máy chủ kiểm lại mọi số: ngày 1-31, tháng 1-12, năm 1900-2100, giờ 0-23. Không tin dữ liệu từ trình duyệt. Ngày phải có thật (laNgayDuongCoThat) — engine không tự bắt 31/4 hay 29/2 năm thường.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -18454,6 +18846,181 @@
       <c r="G140" s="8" t="inlineStr">
         <is>
           <t>lib/rag/ngon-ngu.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="30" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B141" s="31" t="inlineStr">
+        <is>
+          <t>Cứng hoá production</t>
+        </is>
+      </c>
+      <c r="C141" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" s="8" t="inlineStr">
+        <is>
+          <t>Test engine tự đối chiếu</t>
+        </is>
+      </c>
+      <c r="E141" s="8" t="inlineStr">
+        <is>
+          <t>scripts/test-ansao-chuan.ts: công thức sách độc lập + 2.000 lá số ngẫu nhiên hạt giống cố định + 60 mẫu đóng băng.</t>
+        </is>
+      </c>
+      <c r="F141" s="32" t="inlineStr">
+        <is>
+          <t>Kết quả engine đổi mà PHUONG_PHAP.phienBan không đổi = lỗi. Cập nhật mẫu (--cap-nhat) CHỈ sau khi tăng phienBan.</t>
+        </is>
+      </c>
+      <c r="G141" s="8" t="inlineStr">
+        <is>
+          <t>scripts/test-ansao-chuan.ts, scripts/mau-ansao.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="30" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B142" s="31" t="inlineStr">
+        <is>
+          <t>Cứng hoá production</t>
+        </is>
+      </c>
+      <c r="C142" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D142" s="8" t="inlineStr">
+        <is>
+          <t>Ngày có thật</t>
+        </is>
+      </c>
+      <c r="E142" s="8" t="inlineStr">
+        <is>
+          <t>Mọi chỗ nhận ngày sinh từ ngoài gọi laNgayDuongCoThat trước lapLaSo.</t>
+        </is>
+      </c>
+      <c r="F142" s="32" t="inlineStr">
+        <is>
+          <t>Date.parse("1990-04-31") của V8 vẫn trả một ngày — không dùng nó để kiểm hợp lệ.</t>
+        </is>
+      </c>
+      <c r="G142" s="8" t="inlineStr">
+        <is>
+          <t>lib/tuvi/kiem-ngay.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="30" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B143" s="31" t="inlineStr">
+        <is>
+          <t>Cứng hoá production</t>
+        </is>
+      </c>
+      <c r="C143" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D143" s="8" t="inlineStr">
+        <is>
+          <t>Quyền admin</t>
+        </is>
+      </c>
+      <c r="E143" s="8" t="inlineStr">
+        <is>
+          <t>ADMIN_EMAILS rỗng: mở chỉ khi NODE_ENV !== production.</t>
+        </is>
+      </c>
+      <c r="F143" s="32" t="inlineStr">
+        <is>
+          <t>Mặc định đóng. Vercel bản xem thử cũng là production.</t>
+        </is>
+      </c>
+      <c r="G143" s="8" t="inlineStr">
+        <is>
+          <t>lib/supabase/config.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="30" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B144" s="31" t="inlineStr">
+        <is>
+          <t>Cứng hoá production</t>
+        </is>
+      </c>
+      <c r="C144" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D144" s="8" t="inlineStr">
+        <is>
+          <t>Giới hạn tốc độ</t>
+        </is>
+      </c>
+      <c r="E144" s="8" t="inlineStr">
+        <is>
+          <t>proxy.ts: POST vào route tốn model, 40 lượt / 60 giây / IP, trả 429 + Retry-After.</t>
+        </is>
+      </c>
+      <c r="F144" s="32" t="inlineStr">
+        <is>
+          <t>Bộ đếm theo instance — giới hạn mềm, không thay hạn mức ngày. 429 không kèm gioiHanKhach để giao diện không hiểu nhầm là hết lượt khách.</t>
+        </is>
+      </c>
+      <c r="G144" s="8" t="inlineStr">
+        <is>
+          <t>lib/gioi-han-toc-do.ts, proxy.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="30" t="inlineStr">
+        <is>
+          <t>L18</t>
+        </is>
+      </c>
+      <c r="B145" s="31" t="inlineStr">
+        <is>
+          <t>Cứng hoá production</t>
+        </is>
+      </c>
+      <c r="C145" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="D145" s="8" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E145" s="8" t="inlineStr">
+        <is>
+          <t>GitHub Actions chạy tsc, dem-loi-lint (mốc 5), các test offline, next build.</t>
+        </is>
+      </c>
+      <c r="F145" s="32" t="inlineStr">
+        <is>
+          <t>Lint thấp hơn mốc thì hạ MOC trong scripts/dem-loi-lint.mjs; không bao giờ nâng.</t>
+        </is>
+      </c>
+      <c r="G145" s="8" t="inlineStr">
+        <is>
+          <t>.github/workflows/kiem-tra.yml, scripts/dem-loi-lint.mjs</t>
         </is>
       </c>
     </row>
@@ -18469,7 +19036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21178,6 +21745,38 @@
       <c r="F84" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="49" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B85" s="50" t="inlineStr">
+        <is>
+          <t>cung-hoa-production</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>CEL-164, CEL-165, CEL-166, CEL-167, CEL-168</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Cứng hoá production: test engine tự đối chiếu + mẫu đóng băng, chặn ngày không có thật ở form và 11 route, admin mặc định đóng khi ADMIN_EMAILS rỗng trên production, trang lỗi/không tìm thấy, giới hạn tốc độ route AI trong proxy, CI GitHub Actions.</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án đối chiếu Celes với bài viết "demo khác production" và yêu cầu làm lần lượt. Rà ra: engine không có test tự động (sai an sao không ai biết), 31/4 lặng lẽ thành 1/5, ADMIN_EMAILS rỗng mở quản trị cho mọi người, chưa có trang lỗi, chưa có gì chặn gọi dồn vào model, và các cổng kiểm chỉ chạy khi nhớ.</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Luu ma nguon thiet ke app iOS vao repo (docs/thiet-ke/celes-ios) — tai khoan it-ba sap mat quyen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -19036,7 +19036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21775,6 +21775,38 @@
         </is>
       </c>
       <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>thiet-ke-app-ios</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>CEL-153</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Lưu mã nguồn hai canvas thiết kế app iOS vào docs/thiet-ke/celes-ios/ (aurora: gen.py sinh 17 màn, bản 7 gồm tab Lá số · Tổng quan · Chuyên sâu · Mạnh – yếu và phụ tinh hai cột; luong-app: 12 màn đã duyệt).</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Canvas nằm dưới tài khoản it-ba sắp mất quyền và artifact không chuyển chủ được. Lưu vào repo để tài khoản khác publish lại được.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Thiet ke iOS ban 8: nen gan den, moi luong mot vung mau
Theo gop y senior UI/UX: nen toi qua sang (#1A001E) va cac luong giong nhau,
khong biet minh dang o dau. Nen #0B0A0D, the kinh toi; vung mau rieng cho
Khoi dau / Hom nay / La so / Hanh trinh / Moi quan he / Celes / Tai khoan,
the chinh toi theo mau vung thay mang pastel, dau vung dau man. Ban sang giu nguyen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -20580,7 +20580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23671,6 +23671,38 @@
         </is>
       </c>
       <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="49" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B97" s="50" t="inlineStr">
+        <is>
+          <t>thiet-ke-ios-v8</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>CEL-153</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Bản thiết kế iOS Aurora lên bản 8: nền tối đổi từ tím #1A001E sang gần đen #0B0A0D; mỗi luồng một vùng màu (Khởi đầu cam, Hôm nay vàng, Lá số tím chàm, Hành trình xanh ngọc, Mối quan hệ san hô, Celes hồng, Tài khoản xám) đi vào quầng nền, thẻ chính, tab đang chọn và dấu vùng đầu màn. Thẻ nhận định pastel chỉ còn ở bản sáng.</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>Góp ý senior UI/UX: chế độ tối mà nền quá sáng; các luồng trông giống hệt nhau nên người dùng không biết mình đang ở đâu (onboarding xong nền vẫn y như cũ). Tham khảo dashboard tối nền gần đen, màu nhấn dùng tiết kiệm.</t>
+        </is>
+      </c>
+      <c r="F97" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Thiet ke iOS: prototype bam thu luong va 5 man onboarding con thieu
- prototype.html: khung iPhone, chuyen canh day/mo nhu iOS, 5 nhiem vu thu,
  cham cho trong thi sang cho bam duoc, bao khi cham cho chua co man
- Them man Chao, Ten, Gioi tinh, Ngay sinh, Gio sinh de di duoc tu dau
- Trang muc luc co nut mo prototype

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -20580,7 +20580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23703,6 +23703,38 @@
         </is>
       </c>
       <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>thiet-ke-ios-v8</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>CEL-153</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Thiết kế iOS: thêm prototype bấm thử (prototype.html — khung iPhone, chuyển cảnh đẩy/mờ như iOS, 5 nhiệm vụ thử có đo thời gian và số bước, chạm chỗ trống thì sáng chỗ bấm được, báo trong máy khi chạm chỗ chưa có màn) và 5 màn onboarding còn thiếu: Chào, Tên, Giới tính, Ngày sinh, Giờ sinh (có lựa chọn không nhớ giờ).</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Chủ dự án muốn tự đi thử luồng trước khi lập trình vào app. Trước đó onboarding chỉ có bước 5/5 nên không đi được từ đầu; mở từng tệp .dc.html thì không có chuyển cảnh, không phân biệt được đẩy màn với đổi tab, nên không cảm được luồng.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Thiet ke iOS: sua chong lop - noi dung dung tren orb Celes, la so thu gon, vang sang orb het vuong
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -20580,7 +20580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23735,6 +23735,38 @@
         </is>
       </c>
       <c r="F98" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>thiet-ke-ios-v8</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CEL-153</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Sửa chồng lớp trong bản thiết kế iOS: nội dung màn có thanh tab dừng trên đỉnh orb Celes (vùng an toàn 732px, mờ dần ở mép); lá số thu hàng 126→120px để hàng Năm xem/Tam phương không nằm dưới orb; vầng sáng orb màn Chào và đầu bảng prototype hết bị vuông</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Chủ dự án bấm thử prototype thấy nút Tam phương chui dưới orb và vầng sáng orb thành ô vuông. Orb nhô 18px khỏi thanh tab nên nội dung phải chừa tới đỉnh orb chứ không chỉ tới đỉnh thanh tab — app thật cũng phải theo mốc này</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Logo moi 29/09 tren web va app: trang khuyet + sao bon canh
- Web: components/Logo.tsx, app/icon.svg, favicon, apple-icon, anh OG theo bo
  logo cua designer. Theme Ngay dat dau trong o #111126 (token --dau-nen) vi sao
  kem mat tren nen sang.
- App: icon iOS, adaptive icon Android, splash nen #111126, favicon,
  DauCelestia/LogoCelestia chung hinh voi web (path hai cung thay mask).
- Ban thiet ke iOS: man Chao thay orb bang dau moi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -20580,7 +20580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23767,6 +23767,38 @@
         </is>
       </c>
       <c r="F99" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>logo-2909</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>CEL-153</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Thay bộ logo mới của designer (D:/Celestia/Logo Celestia) trên web và app: dấu trăng khuyết tím–đào–kem + sao bốn cánh; icon.svg, favicon, apple-icon, ảnh OG; app: icon iOS, adaptive icon Android, splash, favicon, DauCelestia/LogoCelestia. Màn Chào trong bản thiết kế iOS thay orb bằng dấu mới.</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Tệp gốc khoét trăng bằng mask; đổi sang path hai cung tròn vì react-native-svg vẽ mask không ổn định và web với app phải chung một hình. Sao màu kem biến mất trên nền sáng nên ở theme Ngày dấu nằm trong ô bo góc #111126 (token --dau-nen, trong suốt ở nền tối). Hình gốc lệch trái trong khung 1024 nên khung nhìn căn theo hình. Splash đổi sang nền #111126 cho khớp icon.</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
App Aurora ban 8: dung lai 21 man - onboarding, Quick Read, Hom nay, tab La so 4 che do + Manh-yeu radar, Celes, Hanh trinh, Moi quan he, Tai khoan chon giao dien; font nhap tung do dam; backlog CEL-169 L26
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O169"/>
+  <dimension ref="A1:O170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13359,12 +13359,13 @@
       </c>
       <c r="M154" s="8" t="inlineStr">
         <is>
-          <t>App: tsc sạch, xuất bundle iOS được (4,2 MB). Web: tsc, eslint (5 lỗi cũ), test-rag-planner, next build đều qua.</t>
+          <t>App: tsc sạch, xuất bundle iOS được (4,2 MB). Web: tsc, eslint (5 lỗi cũ), test-rag-planner, next build đều qua.
+29/09/2026: token bo góc theo web được THAY bằng Aurora bản 8 — xem CEL-169.</t>
         </is>
       </c>
       <c r="N154" s="8" t="inlineStr">
         <is>
-          <t>27/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="O154" s="8" t="inlineStr">
@@ -14566,6 +14567,86 @@
       <c r="O169" s="8" t="inlineStr">
         <is>
           <t>app-gd1-moi-quan-he</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="13" t="inlineStr">
+        <is>
+          <t>CEL-169</t>
+        </is>
+      </c>
+      <c r="B170" s="14" t="inlineStr">
+        <is>
+          <t>G. App di động</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>Giao diện app theo thiết kế Aurora bản 8 (21 màn) + tab Lá số + Mạnh–yếu</t>
+        </is>
+      </c>
+      <c r="D170" s="8" t="inlineStr">
+        <is>
+          <t>Dựng lại toàn bộ giao diện apps/celes-app theo docs/thiet-ke/celes-ios/aurora/gen.py: theme tối mặc định nền #0B0A0D, mỗi tab một màu vùng (quầng sáng, icon tab, nhãn), thẻ kính bo 20, hero bo 24, nút gradient Fuchsia 56px bo 14; font riêng của app (Bricolage Grotesque, Be Vietnam Pro, Newsreader nghiêng cho giọng Celes, JetBrains Mono). Thanh tab nổi, Celes là quả cầu nhô giữa. Năm tab: Hôm nay · Lá số · Celes · Hành trình · Mối quan hệ; Tài khoản thành màn riêng mở từ ảnh đại diện, có chọn giao diện Tối/Sáng/Theo máy. Tab Lá số mới có 4 chế độ Lá số / Tổng quan / Chuyên sâu / Mạnh–yếu; Mạnh–yếu là radar 12 lĩnh vực dùng chung dữ kiện chiTietDiemTungCung với web.</t>
+        </is>
+      </c>
+      <c r="E170" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở app → theme tối mặc định → tab Hôm nay
+2. Ảnh đại diện góc phải → Tài khoản (stack)
+3. Tab Lá số → chọn chế độ; chỉ chế độ đang mở mới được dựng (Tổng quan chỉ gọi máy chủ khi mở)
+4. Mạnh–yếu → chạm lĩnh vực trên radar hoặc chip mức → thẻ vì sao</t>
+        </is>
+      </c>
+      <c r="F170" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G170" s="8" t="inlineStr">
+        <is>
+          <t>Không đổi</t>
+        </is>
+      </c>
+      <c r="H170" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I170" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J170" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app (mọi màn)</t>
+        </is>
+      </c>
+      <c r="K170" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/thiet-ke/token.ts, src/thiet-ke/theme.tsx, src/giao-dien/co-ban.tsx, icon-aurora.tsx, thanh-tab.tsx, menh-ban.tsx, manh-yeu.tsx, luan-giai.tsx, khung-buoc.tsx, app/(tabs)/*, app/toi.tsx, metro.config.js, tsconfig.json</t>
+        </is>
+      </c>
+      <c r="L170" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M170" s="8" t="inlineStr">
+        <is>
+          <t>Chưa soát bằng mắt trên máy thật (đã qua tsc + expo export Android). Phần thiết kế cần dữ liệu chưa có đã BỎ chứ không dựng rỗng: giờ thuận/nhịp ngày, "Celes vẫn nhớ", thông báo, mốc riêng trên Hành trình, tiến độ đọc n/14, nút chia sẻ, mic. Ngày sinh vẫn gõ DD/MM/YYYY (chưa có nhập âm lịch). Web chưa đổi theo Aurora.</t>
+        </is>
+      </c>
+      <c r="N170" s="8" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="O170" s="8" t="inlineStr">
+        <is>
+          <t>app-aurora</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G165"/>
+  <dimension ref="A1:G169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19935,7 +20016,7 @@
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>apps/celes-app/app/ban-do.tsx</t>
+          <t>apps/celes-app/src/giao-dien/menh-ban.tsx (MenhBanDayDu + CungChiTiet), dùng chung cho tab Lá số và apps/celes-app/app/ban-do.tsx</t>
         </is>
       </c>
     </row>
@@ -20565,6 +20646,154 @@
       <c r="G165" s="8" t="inlineStr">
         <is>
           <t>apps/celes-app/src/du-lieu/api.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="30" t="inlineStr">
+        <is>
+          <t>L26</t>
+        </is>
+      </c>
+      <c r="B166" s="31" t="inlineStr">
+        <is>
+          <t>Giao diện Aurora trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C166" s="31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D166" s="8" t="inlineStr">
+        <is>
+          <t>Token và theme</t>
+        </is>
+      </c>
+      <c r="E166" s="8" t="inlineStr">
+        <is>
+          <t>token.ts: VUNG (7 vùng: celes, khoiDau, homNay, laSo, hanhTrinh, moiQuanHe, toi; mỗi vùng mau/sang/rgb/quang), VUNG_SANG cho theme sáng. theme.tsx mặc định "toi"; useVung(ten) trả vùng theo theme. NenVung vẽ quầng sáng SVG chỉ ở theme tối.</t>
+        </is>
+      </c>
+      <c r="F166" s="32" t="inlineStr">
+        <is>
+          <t>Không có blur, không có masked-view trên RN: chữ gradient của thiết kế vẽ bằng màu vùng đặc (ChuNhan). Fuchsia #D32298 chỉ cho nút chính — nhãn phụ, link dùng màu vùng.</t>
+        </is>
+      </c>
+      <c r="G166" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/thiet-ke/token.ts, apps/celes-app/src/thiet-ke/theme.tsx, apps/celes-app/src/giao-dien/co-ban.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="30" t="inlineStr">
+        <is>
+          <t>L26</t>
+        </is>
+      </c>
+      <c r="B167" s="31" t="inlineStr">
+        <is>
+          <t>Giao diện Aurora trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C167" s="31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="inlineStr">
+        <is>
+          <t>Thanh tab nổi</t>
+        </is>
+      </c>
+      <c r="E167" s="8" t="inlineStr">
+        <is>
+          <t>Tabs tabBar = ThanhTab: bo 24, cao 64, cách đáy max(22, insets.bottom − 8), Celes là orb 50px nhô 18px. Màn có thanh tab lấy đệm đáy bằng useDemDayTab() = đáy thanh + 64 + 24.</t>
+        </is>
+      </c>
+      <c r="F167" s="32" t="inlineStr">
+        <is>
+          <t>Nội dung phải chừa tới ĐỈNH ORB, không chỉ đỉnh thanh — đừng tự cộng số, gọi useDemDayTab(). Màn stack (toi, ban-do, chi-tiet-han…) dùng insets.bottom + 24. Kiểu props lấy từ Tabs["tabBar"] vì @react-navigation/* không nằm trong node_modules (expo-router gói sẵn).</t>
+        </is>
+      </c>
+      <c r="G167" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/giao-dien/thanh-tab.tsx, apps/celes-app/app/(tabs)/_layout.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="30" t="inlineStr">
+        <is>
+          <t>L26</t>
+        </is>
+      </c>
+      <c r="B168" s="31" t="inlineStr">
+        <is>
+          <t>Giao diện Aurora trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C168" s="31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D168" s="8" t="inlineStr">
+        <is>
+          <t>Tab Lá số và Mạnh–yếu</t>
+        </is>
+      </c>
+      <c r="E168" s="8" t="inlineStr">
+        <is>
+          <t>ChonPhanDoan 4 mục; chỉ dựng chế độ đang mở. Mạnh–yếu gọi chiTietDiemTungCung(laSo) từ lib/rag/v3/du-kien.ts qua bí danh @/lib/* (tsconfig paths + resolveRequest trong metro.config.js). Tên mức theo TEN_MUC của du-kien (chung với web).</t>
+        </is>
+      </c>
+      <c r="F168" s="32" t="inlineStr">
+        <is>
+          <t>Không sao chép du-kien sang app — cùng lý do với engine. Chỉ import hàm thuần; thêm tệp lib/* mới vào app thì phải thêm vào include của apps/celes-app/tsconfig.json.</t>
+        </is>
+      </c>
+      <c r="G168" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/src/giao-dien/manh-yeu.tsx, apps/celes-app/app/(tabs)/la-so.tsx, apps/celes-app/metro.config.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="30" t="inlineStr">
+        <is>
+          <t>L26</t>
+        </is>
+      </c>
+      <c r="B169" s="31" t="inlineStr">
+        <is>
+          <t>Giao diện Aurora trên app (apps/celes-app)</t>
+        </is>
+      </c>
+      <c r="C169" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D169" s="8" t="inlineStr">
+        <is>
+          <t>Font</t>
+        </is>
+      </c>
+      <c r="E169" s="8" t="inlineStr">
+        <is>
+          <t>Nạp 9 độ đậm trong app/_layout.tsx bằng đường dẫn con (@expo-google-fonts/&lt;họ&gt;/&lt;độ đậm&gt;).</t>
+        </is>
+      </c>
+      <c r="F169" s="32" t="inlineStr">
+        <is>
+          <t>Nhập từ gốc gói kéo MỌI độ đậm vào gói cài đặt (đo được hàng chục tệp .ttf thừa).</t>
+        </is>
+      </c>
+      <c r="G169" s="8" t="inlineStr">
+        <is>
+          <t>apps/celes-app/app/_layout.tsx</t>
         </is>
       </c>
     </row>
@@ -20580,7 +20809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23799,6 +24028,38 @@
         </is>
       </c>
       <c r="F100" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>app-aurora</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>CEL-169, CEL-153</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Dựng giao diện app theo Aurora bản 8: token vùng màu, font mới, component dùng chung, thanh tab nổi, 21 màn (Chào, 5 bước onboarding, Quick Read, Hôm nay, Lá số 4 chế độ + Mạnh–yếu radar, Celes, Hành trình, Mối quan hệ, Tài khoản). Tài khoản ra khỏi thanh tab, tab Lá số vào thay.</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt Aurora bản 8 và yêu cầu đưa lên production. Tài khoản ít dùng hằng ngày nên nhường chỗ cho Lá số — thứ người dùng mở lại nhiều nhất. Những khối thiết kế cần dữ liệu app chưa có bị bỏ thay vì dựng rỗng hoặc bịa (vd. đường đời là sóng theo đại vận, không vẽ điểm tốt/xấu vì engine không có thước đo đó).</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Luan giai v3: chong mau thuan, khung trung tinh gioi, trang thai duyen, tach du kien/nguon; Viet lai (quan tri); trang /admin/luan-giai; so ket luan chung cho Hoi Celes; boi canh nguoi doc; dung-thu-vien theo chu de + --dem; bo 5 chu de cu (9 chu de); THE_HE_DEM 7->8; backlog CEL-170..175 L27
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O170"/>
+  <dimension ref="A1:O176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -14650,6 +14650,483 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" s="13" t="inlineStr">
+        <is>
+          <t>CEL-170</t>
+        </is>
+      </c>
+      <c r="B171" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C171" s="8" t="inlineStr">
+        <is>
+          <t>Viết lại (quản trị): admin tự sinh lại bài luận khi đổi cách luận</t>
+        </is>
+      </c>
+      <c r="D171" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản quản trị thấy nút "Viết lại (quản trị)" ở Tổng quan, chuyên sâu, Bức tranh lớn. Bấm là sinh lại bài của lá số đang xem theo khung + cấu hình hiện hành, bỏ qua đệm và không trừ lượt; bản cũ được giữ làm dự phòng nếu bản mới hỏng. Mỗi lần ghi nhật ký quản trị.</t>
+        </is>
+      </c>
+      <c r="E171" s="8" t="inlineStr">
+        <is>
+          <t>1. Admin mở lá số → Tổng quan / chuyên sâu
+2. Bấm "Viết lại (quản trị)"
+3. Route kiểm canQuanTri → vietLai=true → sinh mới, ghi đệm
+4. Hỏng thì trả bản cũ</t>
+        </is>
+      </c>
+      <c r="F171" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G171" s="8" t="inlineStr">
+        <is>
+          <t>Model (v3)</t>
+        </is>
+      </c>
+      <c r="H171" s="8" t="inlineStr">
+        <is>
+          <t>Khi admin bấm</t>
+        </is>
+      </c>
+      <c r="I171" s="8" t="inlineStr">
+        <is>
+          <t>Quản trị</t>
+        </is>
+      </c>
+      <c r="J171" s="8" t="inlineStr">
+        <is>
+          <t>/la-so, /luan-giai/sau, Bức tranh lớn</t>
+        </is>
+      </c>
+      <c r="K171" s="8" t="inlineStr">
+        <is>
+          <t>components/luangiai/VietLaiQuanTri.tsx, lib/rag/v3/xu-ly.ts, app/api/luan-giai-v3/route.ts</t>
+        </is>
+      </c>
+      <c r="L171" s="8" t="inlineStr">
+        <is>
+          <t>canQuanTri() trên máy chủ</t>
+        </is>
+      </c>
+      <c r="M171" s="8" t="inlineStr">
+        <is>
+          <t>Tiêu lượt model dùng chung — không bấm hàng loạt</t>
+        </is>
+      </c>
+      <c r="N171" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="O171" s="8" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="13" t="inlineStr">
+        <is>
+          <t>CEL-171</t>
+        </is>
+      </c>
+      <c r="B172" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t>Trang cấu hình luận giải /admin/luan-giai (độ dài, trần gợi ý)</t>
+        </is>
+      </c>
+      <c r="D172" s="8" t="inlineStr">
+        <is>
+          <t>Admin chỉnh khoảng số chữ "trần" và "nên viết" cho Tổng quan / chuyên sâu, số đoạn, độ dài "vì sao", trần gợi ý. Giá trị hỏng bị ép về khoảng hợp lệ. Mặc định: tổng quan nên 80–130 (trần 140), chuyên sâu nên 170–240 (trần 280), gợi ý ≤30.</t>
+        </is>
+      </c>
+      <c r="E172" s="8" t="inlineStr">
+        <is>
+          <t>1. /admin/luan-giai → sửa số → Lưu
+2. Lưu vào noi_dung_ai bề mặt cau-hinh-v3
+3. Luồng sinh đọc lại (đệm 60 giây)
+4. Bài mới viết theo số mới; bài cũ giữ đến khi viết lại</t>
+        </is>
+      </c>
+      <c r="F172" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G172" s="8" t="inlineStr">
+        <is>
+          <t>Cấu hình</t>
+        </is>
+      </c>
+      <c r="H172" s="8" t="inlineStr">
+        <is>
+          <t>60 giây</t>
+        </is>
+      </c>
+      <c r="I172" s="8" t="inlineStr">
+        <is>
+          <t>Quản trị</t>
+        </is>
+      </c>
+      <c r="J172" s="8" t="inlineStr">
+        <is>
+          <t>/admin/luan-giai</t>
+        </is>
+      </c>
+      <c r="K172" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/cau-hinh.ts, app/api/admin/cau-hinh-luan-giai/route.ts, app/admin/luan-giai/page.tsx</t>
+        </is>
+      </c>
+      <c r="L172" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M172" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ sửa số, chưa sửa lời nhắc, chưa thử ngay trong trang</t>
+        </is>
+      </c>
+      <c r="N172" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="O172" s="8" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="13" t="inlineStr">
+        <is>
+          <t>CEL-172</t>
+        </is>
+      </c>
+      <c r="B173" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C173" s="8" t="inlineStr">
+        <is>
+          <t>Chống mâu thuẫn + khung Tình duyên / Con cái trung tính giới + trạng thái duyên + tách dữ kiện / nguồn</t>
+        </is>
+      </c>
+      <c r="D173" s="8" t="inlineStr">
+        <is>
+          <t>Các phần của một lá số không được nói ngược nhau; khung Tình duyên và Con cái không giả định giới người đọc; trạng thái duyên (tốt / trắc trở / muộn…) tính một lần từ dữ kiện rồi mọi phần dùng chung; dữ kiện engine và lời trích sách tách hai khối trong lời nhắc.</t>
+        </is>
+      </c>
+      <c r="E173" s="8" t="inlineStr">
+        <is>
+          <t>1. du-kien + trang-thai-duyen tính trước
+2. prompt-v3 nhận khối dữ kiện và khối nguồn riêng
+3. kiem-v3 soát mâu thuẫn và độ dài</t>
+        </is>
+      </c>
+      <c r="F173" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G173" s="8" t="inlineStr">
+        <is>
+          <t>Model (v3)</t>
+        </is>
+      </c>
+      <c r="H173" s="8" t="inlineStr">
+        <is>
+          <t>Theo thế hệ đệm 8</t>
+        </is>
+      </c>
+      <c r="I173" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J173" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau</t>
+        </is>
+      </c>
+      <c r="K173" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/khung.ts, du-kien.ts, trang-thai-duyen.ts, prompt-v3.ts, kiem-v3.ts, tom-lai.ts</t>
+        </is>
+      </c>
+      <c r="L173" s="8" t="inlineStr">
+        <is>
+          <t>THE_HE_DEM = 8</t>
+        </is>
+      </c>
+      <c r="M173" s="8" t="inlineStr">
+        <is>
+          <t>Nâng thế hệ đệm 7→8: mọi lá số sinh lại khi mở lần đầu</t>
+        </is>
+      </c>
+      <c r="N173" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="O173" s="8" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="13" t="inlineStr">
+        <is>
+          <t>CEL-173</t>
+        </is>
+      </c>
+      <c r="B174" s="14" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="inlineStr">
+        <is>
+          <t>Sổ kết luận chung: Hỏi Celes nhớ những gì bài luận v3 đã nói</t>
+        </is>
+      </c>
+      <c r="D174" s="8" t="inlineStr">
+        <is>
+          <t>Khi trả lời, Celes đọc câu mở đầu các "Tóm lại" và ý chính Tổng quan đã đệm của lá số (tối đa 6 câu) để không nói ngược, và được phép nói "như Celes đã nói trong bài luận của bạn…".</t>
+        </is>
+      </c>
+      <c r="E174" s="8" t="inlineStr">
+        <is>
+          <t>1. hoi-dap gửi chartHashLaSo
+2. tra-loi đọc soKetLuanV3 + bảng cũ (≤8)
+3. Đưa vào khối "ĐÃ NÓI VỚI NGƯỜI NÀY"</t>
+        </is>
+      </c>
+      <c r="F174" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G174" s="8" t="inlineStr">
+        <is>
+          <t>Đệm noi_dung_ai</t>
+        </is>
+      </c>
+      <c r="H174" s="8" t="inlineStr">
+        <is>
+          <t>Theo bài đệm</t>
+        </is>
+      </c>
+      <c r="I174" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J174" s="8" t="inlineStr">
+        <is>
+          <t>/hoi-dap</t>
+        </is>
+      </c>
+      <c r="K174" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/so-ket-luan.ts, lib/rag/tra-loi.ts, lib/rag/prompt-co-can-cu.ts, app/api/hoi-dap/route.ts</t>
+        </is>
+      </c>
+      <c r="L174" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật (lá số chưa có bài v3 thì bỏ qua)</t>
+        </is>
+      </c>
+      <c r="M174" s="8" t="inlineStr">
+        <is>
+          <t>Bản rẻ: lấy câu đầu, chưa lọc trùng bằng embedding</t>
+        </is>
+      </c>
+      <c r="N174" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="O174" s="8" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="13" t="inlineStr">
+        <is>
+          <t>CEL-174</t>
+        </is>
+      </c>
+      <c r="B175" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C175" s="8" t="inlineStr">
+        <is>
+          <t>Bối cảnh người đọc (chip hoàn cảnh) cho Tình duyên / Con cái / Sự nghiệp</t>
+        </is>
+      </c>
+      <c r="D175" s="8" t="inlineStr">
+        <is>
+          <t>Lần đầu mở ba chủ đề này, Celes hỏi vài chip: tình trạng duyên (+ cách gọi người ấy / vợ / chồng), con cái, công việc. Bối cảnh chỉ đổi GÓC NHÌN và THÌ, không đổi kết luận. "Bỏ qua" = không muốn nói. Sửa lại ở dòng "Đổi" hoặc mục "Hoàn cảnh hiện tại" trong /ho-so.</t>
+        </is>
+      </c>
+      <c r="E175" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở chủ đề → chưa có bối cảnh → thẻ "Trước khi Celes viết"
+2. Chọn / Bỏ qua → lưu trình duyệt + charts.boi_canh (nếu đăng nhập)
+3. Khoá đệm thêm |bc:… (trừ khong-noi, nguoi-ay)
+4. Khối bối cảnh vào lời nhắc</t>
+        </is>
+      </c>
+      <c r="F175" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G175" s="8" t="inlineStr">
+        <is>
+          <t>Người dùng nhập</t>
+        </is>
+      </c>
+      <c r="H175" s="8" t="inlineStr">
+        <is>
+          <t>Khi người dùng đổi</t>
+        </is>
+      </c>
+      <c r="I175" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J175" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau, /ho-so</t>
+        </is>
+      </c>
+      <c r="K175" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/boi-canh-doc.ts, lib/store/boi-canh-doc.ts, components/luangiai/HoiBoiCanh.tsx, components/luangiai/BoiCanhHoSo.tsx</t>
+        </is>
+      </c>
+      <c r="L175" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật; lưu theo tài khoản cần chạy supabase/va-boi-canh-la-so.sql</t>
+        </is>
+      </c>
+      <c r="M175" s="8" t="inlineStr">
+        <is>
+          <t>Chữ ở /ho-so chưa qua i18n (chỉ tiếng Việt). Chưa chạy SQL thì bối cảnh chỉ nằm ở trình duyệt</t>
+        </is>
+      </c>
+      <c r="N175" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="O175" s="8" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="13" t="inlineStr">
+        <is>
+          <t>CEL-175</t>
+        </is>
+      </c>
+      <c r="B176" s="14" t="inlineStr">
+        <is>
+          <t>H. Tri thức</t>
+        </is>
+      </c>
+      <c r="C176" s="8" t="inlineStr">
+        <is>
+          <t>Công cụ dựng thư viện tổng hợp theo chủ đề (--chu-de, --dem)</t>
+        </is>
+      </c>
+      <c r="D176" s="8" t="inlineStr">
+        <is>
+          <t>scripts/dung-thu-vien.ts trước chỉ dựng cho Sự nghiệp; nay có bảng 8 chủ đề (nhãn tìm đoạn, cung loại trừ, lời nhắc). --dem chỉ đếm đoạn và số lượt gọi model, không gọi model. Đếm 30/09: tiền bạc 138 lượt, tình duyên 79, con cái 68, gia đình 142, sức khỏe 185, ra ngoài 92, tính cách 201.</t>
+        </is>
+      </c>
+      <c r="E176" s="8" t="inlineStr">
+        <is>
+          <t>1. --chu-de X --dem → xem cỡ
+2. Chủ dự án duyệt → chạy trích thật theo đợt
+3. Đo → bật CAU_THU_VIEN / DOT_THU_VIEN cho chủ đề</t>
+        </is>
+      </c>
+      <c r="F176" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G176" s="8" t="inlineStr">
+        <is>
+          <t>Sách (trích có kiểm)</t>
+        </is>
+      </c>
+      <c r="H176" s="8" t="inlineStr">
+        <is>
+          <t>Theo đợt</t>
+        </is>
+      </c>
+      <c r="I176" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J176" s="8" t="inlineStr">
+        <is>
+          <t>Chạy tay</t>
+        </is>
+      </c>
+      <c r="K176" s="8" t="inlineStr">
+        <is>
+          <t>scripts/dung-thu-vien.ts, lib/rag/thu-vien/kho.ts, lib/rag/v3/xu-ly.ts</t>
+        </is>
+      </c>
+      <c r="L176" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt tiêu lượt</t>
+        </is>
+      </c>
+      <c r="M176" s="8" t="inlineStr">
+        <is>
+          <t>Chưa chạy trích thật cho 7 chủ đề mới (~905 lượt gọi model trên hạn mức dùng chung)</t>
+        </is>
+      </c>
+      <c r="N176" s="8" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="O176" s="8" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -14667,7 +15144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G169"/>
+  <dimension ref="A1:G174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -20797,6 +21274,191 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" s="30" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="B170" s="31" t="inlineStr">
+        <is>
+          <t>Bối cảnh người đọc + sổ kết luận chung (v3)</t>
+        </is>
+      </c>
+      <c r="C170" s="31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D170" s="8" t="inlineStr">
+        <is>
+          <t>Khoá đệm theo bối cảnh</t>
+        </is>
+      </c>
+      <c r="E170" s="8" t="inlineStr">
+        <is>
+          <t>khoaBoiCanh chèn |bc:&lt;duyen&gt;[.&lt;xungHo&gt;] / |bc:&lt;con&gt; / |bc:&lt;viec&gt; vào khoaGoc trước |th:, CHỈ cho tinh-duyen, con-cai, su-nghiep.</t>
+        </is>
+      </c>
+      <c r="F170" s="32" t="inlineStr">
+        <is>
+          <t>"khong-noi" và "nguoi-ay" không vào khoá — bỏ qua chip là đọc lại đúng bài đã đệm, không sinh thêm. Chủ đề khác không đổi khoá.</t>
+        </is>
+      </c>
+      <c r="G170" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/boi-canh-doc.ts, lib/rag/v3/xu-ly.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="30" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="B171" s="31" t="inlineStr">
+        <is>
+          <t>Bối cảnh người đọc + sổ kết luận chung (v3)</t>
+        </is>
+      </c>
+      <c r="C171" s="31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D171" s="8" t="inlineStr">
+        <is>
+          <t>Lời nhắc</t>
+        </is>
+      </c>
+      <c r="E171" s="8" t="inlineStr">
+        <is>
+          <t>khoiBoiCanh thêm một khối vào lời nhắc người dùng, sau thuNghiem, trước khối đã nói; kèm cách gọi người phối ngẫu.</t>
+        </is>
+      </c>
+      <c r="F171" s="32" t="inlineStr">
+        <is>
+          <t>Bối cảnh chỉ đổi GÓC NHÌN và THÌ; KHÔNG đổi kết luận của lá số. Test test-boi-canh-doc.ts giữ luật này.</t>
+        </is>
+      </c>
+      <c r="G171" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/index.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="30" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="B172" s="31" t="inlineStr">
+        <is>
+          <t>Bối cảnh người đọc + sổ kết luận chung (v3)</t>
+        </is>
+      </c>
+      <c r="C172" s="31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D172" s="8" t="inlineStr">
+        <is>
+          <t>Bức tranh lớn</t>
+        </is>
+      </c>
+      <c r="E172" s="8" t="inlineStr">
+        <is>
+          <t>Gom "Tóm lại" từng chủ đề: bỏ |bc: khi so, ưu tiên bản khớp bối cảnh đang dùng.</t>
+        </is>
+      </c>
+      <c r="F172" s="32" t="inlineStr">
+        <is>
+          <t>Không có bản khớp thì lấy bản bất kỳ của chủ đề đó thay vì bỏ trống.</t>
+        </is>
+      </c>
+      <c r="G172" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="30" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="B173" s="31" t="inlineStr">
+        <is>
+          <t>Bối cảnh người đọc + sổ kết luận chung (v3)</t>
+        </is>
+      </c>
+      <c r="C173" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D173" s="8" t="inlineStr">
+        <is>
+          <t>Sổ kết luận chung</t>
+        </is>
+      </c>
+      <c r="E173" s="8" t="inlineStr">
+        <is>
+          <t>soKetLuanV3 đọc các hàng v3 đệm của lá số + năm xem (tiền tố nam:X|nhom:, thế hệ hiện hành): câu đầu Tóm lại + ý chính Tổng quan, tối đa 6; ghép bảng cũ, tối đa 8.</t>
+        </is>
+      </c>
+      <c r="F173" s="32" t="inlineStr">
+        <is>
+          <t>Lỗi đọc thì im lặng trả rỗng — Hỏi Celes không được hỏng vì sổ.</t>
+        </is>
+      </c>
+      <c r="G173" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/so-ket-luan.ts, lib/rag/tra-loi.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="30" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="B174" s="31" t="inlineStr">
+        <is>
+          <t>Bối cảnh người đọc + sổ kết luận chung (v3)</t>
+        </is>
+      </c>
+      <c r="C174" s="31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D174" s="8" t="inlineStr">
+        <is>
+          <t>Cấu hình độ dài</t>
+        </is>
+      </c>
+      <c r="E174" s="8" t="inlineStr">
+        <is>
+          <t>docCauHinhV3 đọc noi_dung_ai bề mặt cau-hinh-v3, đệm 60 giây; lamSachCauHinh ép "nên viết" nằm trong "trần", trường hỏng lấy mặc định.</t>
+        </is>
+      </c>
+      <c r="F174" s="32" t="inlineStr">
+        <is>
+          <t>Đổi số không sinh lại bài cũ — admin dùng "Viết lại (quản trị)" để thử.</t>
+        </is>
+      </c>
+      <c r="G174" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/cau-hinh.ts, lib/rag/v3/kiem-v3.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20809,7 +21471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24060,6 +24722,166 @@
         </is>
       </c>
       <c r="F101" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>CEL-170, CEL-171</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Nút "Viết lại (quản trị)" + trang /admin/luan-giai chỉnh độ dài</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Chủ dự án cần tự thử lại sau mỗi lần đổi cách luận, không phải nhờ AI chạy tay; và cần tự chỉnh số chữ.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>CEL-172</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Sửa mâu thuẫn giữa các phần, khung trung tính giới, trạng thái duyên dùng chung, tách dữ kiện / nguồn; THE_HE_DEM 7→8</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Bài cũ có chỗ phần này nói ngược phần kia và giả định giới người đọc; chủ dự án duyệt nâng thế hệ để mọi lá số viết lại một lần, gom các thay đổi vào một lần tăng.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>CEL-173</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Hỏi Celes đọc sổ kết luận của bài v3</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Hỏi Celes trước chỉ biết bài tổng quan cũ nên có thể nói ngược bài chuyên sâu người dùng vừa đọc.</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>CEL-174</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Chip bối cảnh người đọc + mục Hoàn cảnh hiện tại ở /ho-so; SQL va-boi-canh-la-so.sql (chưa chạy)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Người đã kết hôn vẫn bị hỏi "bao giờ gặp người ấy"; bối cảnh sửa thì và góc nhìn mà không được đổi kết luận của lá số.</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>luan-giai-3009</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>CEL-175</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>dung-thu-vien.ts tổng quát theo chủ đề + --dem; bỏ 5 chủ đề cũ khỏi giao diện (9 chủ đề)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Thư viện tổng hợp mới dựng cho Sự nghiệp; muốn mở cho chủ đề khác phải biết trước tốn bao nhiêu lượt model trên hạn mức dùng chung.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Boi canh nguoi doc qua i18n (vi+en); thu vien bat theo chu de (THU_VIEN_THEO_CHU_DE); backlog CEL-174/175 L27.6
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15034,17 +15034,17 @@
       </c>
       <c r="M175" s="8" t="inlineStr">
         <is>
-          <t>Chữ ở /ho-so chưa qua i18n (chỉ tiếng Việt). Chưa chạy SQL thì bối cảnh chỉ nằm ở trình duyệt</t>
+          <t>Chưa chạy SQL thì bối cảnh chỉ nằm ở trình duyệt. Chữ đã qua i18n (vi + en) từ 01/10/2026</t>
         </is>
       </c>
       <c r="N175" s="8" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="O175" s="8" t="inlineStr">
         <is>
-          <t>luan-giai-3009</t>
+          <t>luan-giai-0110</t>
         </is>
       </c>
     </row>
@@ -15066,7 +15066,7 @@
       </c>
       <c r="D176" s="8" t="inlineStr">
         <is>
-          <t>scripts/dung-thu-vien.ts trước chỉ dựng cho Sự nghiệp; nay có bảng 8 chủ đề (nhãn tìm đoạn, cung loại trừ, lời nhắc). --dem chỉ đếm đoạn và số lượt gọi model, không gọi model. Đếm 30/09: tiền bạc 138 lượt, tình duyên 79, con cái 68, gia đình 142, sức khỏe 185, ra ngoài 92, tính cách 201.</t>
+          <t>scripts/dung-thu-vien.ts trước chỉ dựng cho Sự nghiệp; nay có bảng 8 chủ đề (nhãn tìm đoạn, cung loại trừ, lời nhắc). --dem chỉ đếm đoạn và số lượt gọi model, không gọi model. Đếm 30/09: tiền bạc 138 lượt, tình duyên 79, con cái 68, gia đình 142, sức khỏe 185, ra ngoài 92, tính cách 201. Bật theo chủ đề ở THU_VIEN_THEO_CHU_DE (lib/rag/v3/xu-ly.ts): mỗi chủ đề một đợt + danh sách câu; hiện chỉ Sự nghiệp.</t>
         </is>
       </c>
       <c r="E176" s="8" t="inlineStr">
@@ -15113,17 +15113,17 @@
       </c>
       <c r="M176" s="8" t="inlineStr">
         <is>
-          <t>Chưa chạy trích thật cho 7 chủ đề mới (~905 lượt gọi model trên hạn mức dùng chung)</t>
+          <t>Chưa chạy trích thật cho 7 chủ đề mới (~905 lô, chạy --batch). Lệnh ghi vào Supabase production cần chủ dự án tự chạy hoặc cấp quyền. Chạy thử Tình duyên 2 lô (--thu): 78% ứng viên qua kiểm tất định, ~10k token/lô</t>
         </is>
       </c>
       <c r="N176" s="8" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="O176" s="8" t="inlineStr">
         <is>
-          <t>luan-giai-3009</t>
+          <t>luan-giai-0110</t>
         </is>
       </c>
     </row>
@@ -15144,7 +15144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G174"/>
+  <dimension ref="A1:G175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -21459,6 +21459,43 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" s="30" t="inlineStr">
+        <is>
+          <t>L27</t>
+        </is>
+      </c>
+      <c r="B175" s="31" t="inlineStr">
+        <is>
+          <t>Bối cảnh người đọc + sổ kết luận chung (v3)</t>
+        </is>
+      </c>
+      <c r="C175" s="31" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D175" s="8" t="inlineStr">
+        <is>
+          <t>Thư viện theo chủ đề</t>
+        </is>
+      </c>
+      <c r="E175" s="8" t="inlineStr">
+        <is>
+          <t>THU_VIEN_THEO_CHU_DE[nhom] = {dot, cau}. CAU_THU_VIEN gộp mọi câu; dấu kho mong đợi của câu = kho|tv:&lt;đợt của chủ đề câu đó&gt;; docThuVien(nhom, đợt của nhom).</t>
+        </is>
+      </c>
+      <c r="F175" s="32" t="inlineStr">
+        <is>
+          <t>Chỉ thêm chủ đề khi gói đợt đã có trong Supabase — thêm trước là dấu kho đổi, nút "Tạo bản mới" hiện mà viết lại không có gì mới. Sự nghiệp giữ nguyên dấu sn-2,sn-2b.</t>
+        </is>
+      </c>
+      <c r="G175" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21471,7 +21508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24882,6 +24919,38 @@
         </is>
       </c>
       <c r="F106" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>luan-giai-0110</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>CEL-174, CEL-175</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Chữ hỏi hoàn cảnh + mục ở /ho-so chuyển sang i18n (vi + en); cấu hình thư viện tách theo chủ đề (THU_VIEN_THEO_CHU_DE)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>/ho-so có bản tiếng Anh nên chữ gắn cứng tiếng Việt là lỗi; thư viện sắp mở cho 7 chủ đề, mỗi chủ đề một đợt riêng — gộp một chuỗi đợt chung sẽ làm mọi câu Sự nghiệp hiện "Tạo bản mới".</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Thu vien tong hop cho 7 chu de: dung dot luot 1 (td-1 cc-1 tb-1 gd-1 sk-1 rn-1 tc-1, 4293 muc) va bat cho 14 cau khong hoi thoi diem; DA-CHAY va-boi-canh-la-so da chay; backlog CEL-174/175
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15034,7 +15034,7 @@
       </c>
       <c r="M175" s="8" t="inlineStr">
         <is>
-          <t>Chưa chạy SQL thì bối cảnh chỉ nằm ở trình duyệt. Chữ đã qua i18n (vi + en) từ 01/10/2026</t>
+          <t>SQL va-boi-canh-la-so.sql đã chạy 01/10/2026 — bối cảnh đi theo tài khoản. Chữ đã qua i18n (vi + en)</t>
         </is>
       </c>
       <c r="N175" s="8" t="inlineStr">
@@ -15044,7 +15044,7 @@
       </c>
       <c r="O175" s="8" t="inlineStr">
         <is>
-          <t>luan-giai-0110</t>
+          <t>thu-vien-0110</t>
         </is>
       </c>
     </row>
@@ -15061,12 +15061,12 @@
       </c>
       <c r="C176" s="8" t="inlineStr">
         <is>
-          <t>Công cụ dựng thư viện tổng hợp theo chủ đề (--chu-de, --dem)</t>
+          <t>Thư viện tổng hợp cho 8 chủ đề (dựng theo chủ đề --chu-de, --dem)</t>
         </is>
       </c>
       <c r="D176" s="8" t="inlineStr">
         <is>
-          <t>scripts/dung-thu-vien.ts trước chỉ dựng cho Sự nghiệp; nay có bảng 8 chủ đề (nhãn tìm đoạn, cung loại trừ, lời nhắc). --dem chỉ đếm đoạn và số lượt gọi model, không gọi model. Đếm 30/09: tiền bạc 138 lượt, tình duyên 79, con cái 68, gia đình 142, sức khỏe 185, ra ngoài 92, tính cách 201. Bật theo chủ đề ở THU_VIEN_THEO_CHU_DE (lib/rag/v3/xu-ly.ts): mỗi chủ đề một đợt + danh sách câu; hiện chỉ Sự nghiệp.</t>
+          <t>scripts/dung-thu-vien.ts có bảng 8 chủ đề (nhãn tìm đoạn, cung loại trừ, lời nhắc); --dem chỉ đếm, không gọi model. Đợt lượt 1 chạy 01/10/2026 bằng --batch: td-1 435 mục, cc-1 213, tb-1 995, gd-1 781, sk-1 693, rn-1 344, tc-1 832 (cộng Sự nghiệp sn-2,sn-2b 2.499). Bật ở THU_VIEN_THEO_CHU_DE cho các câu không hỏi thời điểm: TD01 TD03, CC02 CC03, TB01 TB02 TB04, GD01 GD02, SK01, RN02, TC02 TC03. Đo trên 12 lá số tổng hợp: mọi câu đưa ~18 mục vào lời nhắc, không lá số nào rỗng.</t>
         </is>
       </c>
       <c r="E176" s="8" t="inlineStr">
@@ -15078,7 +15078,7 @@
       </c>
       <c r="F176" s="9" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="G176" s="8" t="inlineStr">
@@ -15113,7 +15113,7 @@
       </c>
       <c r="M176" s="8" t="inlineStr">
         <is>
-          <t>Chưa chạy trích thật cho 7 chủ đề mới (~905 lô, chạy --batch). Lệnh ghi vào Supabase production cần chủ dự án tự chạy hoặc cấp quyền. Chạy thử Tình duyên 2 lô (--thu): 78% ứng viên qua kiểm tất định, ~10k token/lô</t>
+          <t>Chưa đo mù chất lượng bài như Sự nghiệp (so-sanh-v3). Tỉ lệ qua kiểm tất định 53–74% (Con cái thấp nhất). Câu có hỏi thời điểm (TD02, TB03, TB05, SK02, CC01, RN01, TC01, GD03) chưa dùng thư viện. Bài đã viết của các câu vừa bật sẽ hiện "Tạo bản mới"</t>
         </is>
       </c>
       <c r="N176" s="8" t="inlineStr">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="O176" s="8" t="inlineStr">
         <is>
-          <t>luan-giai-0110</t>
+          <t>thu-vien-0110</t>
         </is>
       </c>
     </row>
@@ -21508,7 +21508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24951,6 +24951,38 @@
         </is>
       </c>
       <c r="F107" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>thu-vien-0110</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>CEL-175</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Dựng thư viện lượt 1 cho 7 chủ đề (4.293 mục, --batch) và bật cho 14 câu không hỏi thời điểm</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Chủ dự án hỏi vì sao thư viện chỉ dùng cho Sự nghiệp — không phải thiếu sách mà công cụ mới dựng cho một chủ đề; chủ dự án cấp quyền chạy. Chỉ bật câu không hỏi thời điểm, cùng luật đã dùng cho Sự nghiệp.</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Thiet ke iOS Aurora: sua theo 6 gop y tren ban dung thu
- Chao: 3 y thanh hang dac diem khong khung, khong con giong nut
- Gioi tinh: them icon nam/nu
- Hom nay: bo nhan vung (chi de ngay), loi chao nho / ten lon, loi nhac Celes len dau thanh mot dai
- Tong quan: cau chan dung + chang doi, luoi 6 mat doi moi o mot cau cu the, thay 3 dong danh gia chung
Da deploy celes-thiet-ke.vercel.app. App chua doi theo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -21508,7 +21508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24983,6 +24983,38 @@
         </is>
       </c>
       <c r="F108" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>thiet-ke-gop-y</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>CEL-169</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Thiết kế iOS Aurora: sửa theo 6 góp ý trên bản dựng thử — Chào (3 ý thành hàng đặc điểm, không giống nút), Giới tính (icon nam/nữ), Hôm nay (bỏ nhãn vùng, lời chào nhỏ / tên lớn, lời nhắc Celes lên đầu thành một dải), Tổng quan (câu chân dung + lưới 6 mặt đời thay cho 3 dòng đánh giá chung)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Góp ý của ngocdaitsh trên Vercel 30/09: Tổng quan "chung chung, đặt vào người dùng vẫn không biết bản thân hay mối quan hệ của mình ra sao" — nên mỗi mặt đời phải có một câu cụ thể về chính người đó. App (apps/celes-app) CHƯA đổi theo; web không đổi.</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Thiet ke iOS sua theo phan bien: nut an loi nhac 44px, bo dau vung moi man tab, chu man Chao, Tong quan giu Danh gia chung + Buc tranh chung va them khoi nguoi quanh minh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -21508,7 +21508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25015,6 +25015,38 @@
         </is>
       </c>
       <c r="F109" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>tong-quan-cu-the</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>CEL-169</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Thiết kế iOS Aurora sửa theo phản biện: nút ẩn lời nhắc Hôm nay đủ 44px + nhãn "Ẩn lời nhắc"; bỏ dấu vùng ở MỌI màn tab (chỉ giữ ở màn con có nút quay lại); Chào "4 câu hỏi là đủ để bắt đầu" (onboarding có hỏi giới tính); Tổng quan quay lại Đánh giá chung + Bức tranh chung, thêm khối "Bạn giữa những người quanh mình", hàng giai đoạn chạm được ≥44px</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Phản biện thấy lưới 6 ô chỉ là đổi bố cục, không sửa gốc góp ý "chung chung" — gốc nằm ở phần sinh nội dung. Dấu vùng chỉ bỏ ở Hôm nay thì thiếu nhất quán. App CHƯA đổi theo.</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
Tong quan them TQ12 (moi quan he gan ngoai tinh duyen) + co ngangHang; nhan chu ngu va sao ham o du kien; backlog CEL-176 / L28
Thu va BO luat prompt "khong chung chung" cho tong quan (so mu hoa). celes-domain luot 3:
het loi gan sao Phu Mau thanh tinh nguoi doc, con lo Triet o Thien Di.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O176"/>
+  <dimension ref="A1:O177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15127,6 +15127,85 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" s="13" t="inlineStr">
+        <is>
+          <t>CEL-176</t>
+        </is>
+      </c>
+      <c r="B177" s="14" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C177" s="8" t="inlineStr">
+        <is>
+          <t>Câu tổng quan TQ12 "Tôi thế nào với những người quanh mình?"</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="inlineStr">
+        <is>
+          <t>Tổng quan có thêm một câu về các mối quan hệ gần NGOÀI tình duyên: cha mẹ / người đi trước, anh chị em, bạn bè và người cộng tác, người ngoài. Mỗi nhóm một nhận định (họ thế nào, ai là chỗ dựa, chỗ vướng). Đứng ngay sau TQ03.</t>
+        </is>
+      </c>
+      <c r="E177" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở Tổng quan → TQ12 nằm sau ba câu về con người
+2. Lá số đã có bài: TQ12 được sinh bù riêng (cache theo id), các câu khác giữ nguyên
+3. Bấm "vì sao" → căn cứ từ Nô Bộc, Phụ Mẫu, Huynh Đệ, Thiên Di</t>
+        </is>
+      </c>
+      <c r="F177" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G177" s="8" t="inlineStr">
+        <is>
+          <t>AI + dữ kiện engine</t>
+        </is>
+      </c>
+      <c r="H177" s="8" t="inlineStr">
+        <is>
+          <t>Theo thế hệ đếm</t>
+        </is>
+      </c>
+      <c r="I177" s="8" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J177" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai (Tổng quan)</t>
+        </is>
+      </c>
+      <c r="K177" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/khung.ts, lib/rag/v3/du-kien.ts, lib/rag/v3/index.ts, lib/rag/v3/so-y.ts</t>
+        </is>
+      </c>
+      <c r="L177" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M177" s="8" t="inlineStr">
+        <is>
+          <t>Celes-domain lượt 3: đã hết lỗi gán sao Phụ Mẫu thành tính người đọc và lờ sao hãm; CÒN lờ Triệt / Địa Không ở Thiên Di (lá số A). Chưa có bản EN cho câu hỏi (như mọi câu v3).</t>
+        </is>
+      </c>
+      <c r="N177" s="8" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="O177" s="8" t="inlineStr">
+        <is>
+          <t>tong-quan-cu-the</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15144,7 +15223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G175"/>
+  <dimension ref="A1:G177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -21496,6 +21575,80 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" s="30" t="inlineStr">
+        <is>
+          <t>L28</t>
+        </is>
+      </c>
+      <c r="B176" s="31" t="inlineStr">
+        <is>
+          <t>Câu ngang hàng trong khung (cờ ngangHang)</t>
+        </is>
+      </c>
+      <c r="C176" s="31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D176" s="8" t="inlineStr">
+        <is>
+          <t>Chọn cung</t>
+        </is>
+      </c>
+      <c r="E176" s="8" t="inlineStr">
+        <is>
+          <t>CauHoiV3.ngangHang = true → dungDuKien KHÔNG kéo tam phương của cung đầu; mọi cung trong q.cung đều là "cung chính" / "cung chính (cùng xét)" và có đủ nghĩa sao. Hiện chỉ TQ12.</t>
+        </is>
+      </c>
+      <c r="F176" s="32" t="inlineStr">
+        <is>
+          <t>Mặc định cung đầu là gốc, tam phương vào trước với vai GỌN (không nghĩa sao); cung liệt kê sau mà nằm trong tam phương thì mất vai chính (Nô Bộc là tam hợp của Phụ Mẫu). Đổi chung cho mọi câu thì chạm 15 câu khung — nên dùng cờ, không đổi mặc định.</t>
+        </is>
+      </c>
+      <c r="G176" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/khung.ts, lib/rag/v3/du-kien.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="30" t="inlineStr">
+        <is>
+          <t>L28</t>
+        </is>
+      </c>
+      <c r="B177" s="31" t="inlineStr">
+        <is>
+          <t>Câu ngang hàng trong khung (cờ ngangHang)</t>
+        </is>
+      </c>
+      <c r="C177" s="31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="inlineStr">
+        <is>
+          <t>Nét sao theo chủ ngữ</t>
+        </is>
+      </c>
+      <c r="E177" s="8" t="inlineStr">
+        <is>
+          <t>Với câu ngang hàng: cung Phụ Mẫu / Huynh Đệ / Nô Bộc gắn nhãn "sao tả cha mẹ / anh chị em / bạn bè, KHÔNG tả bạn" trước nét chính tinh (CHU_NGU_NGANG_HANG); chính tinh hãm được đánh dấu "HÃM: nói mặt kém".</t>
+        </is>
+      </c>
+      <c r="F177" s="32" t="inlineStr">
+        <is>
+          <t>Nét sao trong KHUON viết cho "bạn" và chỉ có nét lúc sáng. Luật ở phạm vi câu hỏi không thắng được dữ kiện: model chép nguyên "Thái Dương: bạn kéo nhóm đi" thành tính người đọc. Sửa ở dữ kiện, không ở prompt.</t>
+        </is>
+      </c>
+      <c r="G177" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/du-kien.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21508,7 +21661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25047,6 +25200,38 @@
         </is>
       </c>
       <c r="F110" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>tong-quan-cu-the</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>CEL-176</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Thêm câu tổng quan TQ12 (mối quan hệ gần ngoài tình duyên) + cờ ngangHang trong khung + nhãn chủ ngữ / sao hãm ở dữ kiện cho câu ngang hàng. Không đổi THE_HE_DEM, không đổi phiên bản khung: lá số cũ được sinh bù riêng TQ12.</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Góp ý 30/09 trên bản dựng thử: tổng quan "đọc xong vẫn không biết mối quan hệ của mình ra sao" — tổng quan chỉ có câu tình duyên. Đã THỬ và BỎ luật prompt "không chung chung" cho tổng quan (so mù lá số A: từng cặp 27% / 55%, cả phiên 3 giám khảo đều 50%). Celes-domain đánh trượt TQ12 hai lượt (sao Phụ Mẫu thành tính người đọc, lờ sao hãm, mặc định có anh chị em) — gốc nằm ở dữ kiện nên sửa ở du-kien.ts.</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
TQ12: cho vuong dich danh o du kien, nhanDuoc "ho la nguoi the nao voi ban" — celes-domain PASS luot 6
Thien Di (Triet, Dia Khong ham) gio co cau rieng; No Boc khong con bi dien thanh tinh nguoi doc.
Hung tinh dac/mieu/vuong khong bi bat noi thanh cho vuong. eval-chat-quyet-dinh 10/10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15192,7 +15192,7 @@
       </c>
       <c r="M177" s="8" t="inlineStr">
         <is>
-          <t>Celes-domain lượt 3: đã hết lỗi gán sao Phụ Mẫu thành tính người đọc và lờ sao hãm; CÒN lờ Triệt / Địa Không ở Thiên Di (lá số A). Chưa có bản EN cho câu hỏi (như mọi câu v3).</t>
+          <t>Celes-domain lượt 6 PASS (lá số A). Lỗi nhẹ còn lại: chữ "chỗ dựa sáng" (lọt nghĩa độ sáng), "thực tế" không có trong dữ kiện, "nhất là" dựa trên một sao lẻ. Lỗi cùng gốc (nét sao KHUON viết cho "bạn", sao hãm tả như sáng) còn ở các câu khác lấy Phụ Mẫu / Huynh Đệ / Nô Bộc làm cung chính — cờ ngangHang chỉ sửa TQ12. Chưa có bản EN cho câu hỏi (như mọi câu v3).</t>
         </is>
       </c>
       <c r="N177" s="8" t="inlineStr">
@@ -15223,7 +15223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G177"/>
+  <dimension ref="A1:G178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -21646,6 +21646,43 @@
       <c r="G177" s="8" t="inlineStr">
         <is>
           <t>lib/rag/v3/du-kien.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="30" t="inlineStr">
+        <is>
+          <t>L28</t>
+        </is>
+      </c>
+      <c r="B178" s="31" t="inlineStr">
+        <is>
+          <t>Câu ngang hàng trong khung (cờ ngangHang)</t>
+        </is>
+      </c>
+      <c r="C178" s="31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D178" s="8" t="inlineStr">
+        <is>
+          <t>Chỗ vướng đích danh</t>
+        </is>
+      </c>
+      <c r="E178" s="8" t="inlineStr">
+        <is>
+          <t>Với câu ngang hàng: mỗi cung có Tuần, Triệt, Hóa Kỵ, chính tinh hãm hay hung tinh KHÔNG sáng (bỏ M/V/Đ) thì dữ kiện có dòng "BẮT BUỘC có một ý nói chỗ vướng của nhóm này" liệt kê đích danh.</t>
+        </is>
+      </c>
+      <c r="F178" s="32" t="inlineStr">
+        <is>
+          <t>Luật chung "có Triệt thì nói chỗ vướng" ở phạm vi câu hỏi bị model bỏ qua (lượt 3: Thiên Di có Triệt + Địa Không, bài chỉ kể người chỉ đường). nhanDuoc của TQ12 phải là "HỌ là người thế nào với bạn" — "họ thấy bạn thế nào" kéo model tả tính người đọc, cãi nhau với nhãn dữ kiện.</t>
+        </is>
+      </c>
+      <c r="G178" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/du-kien.ts, lib/rag/v3/khung.ts</t>
         </is>
       </c>
     </row>
@@ -25228,7 +25265,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Góp ý 30/09 trên bản dựng thử: tổng quan "đọc xong vẫn không biết mối quan hệ của mình ra sao" — tổng quan chỉ có câu tình duyên. Đã THỬ và BỎ luật prompt "không chung chung" cho tổng quan (so mù lá số A: từng cặp 27% / 55%, cả phiên 3 giám khảo đều 50%). Celes-domain đánh trượt TQ12 hai lượt (sao Phụ Mẫu thành tính người đọc, lờ sao hãm, mặc định có anh chị em) — gốc nằm ở dữ kiện nên sửa ở du-kien.ts.</t>
+          <t>Góp ý 30/09 trên bản dựng thử: tổng quan "đọc xong vẫn không biết mối quan hệ của mình ra sao" — tổng quan chỉ có câu tình duyên. Đã THỬ và BỎ luật prompt "không chung chung" cho tổng quan (so mù lá số A: từng cặp 27% / 55%, cả phiên 3 giám khảo đều 50%). Celes-domain đánh trượt TQ12 hai lượt (sao Phụ Mẫu thành tính người đọc, lờ sao hãm, mặc định có anh chị em) — gốc nằm ở dữ kiện nên sửa ở du-kien.ts. Lượt 4–6: thêm dòng chỗ vướng đích danh ở dữ kiện, đổi nhanDuoc thành "họ là người thế nào với bạn" — celes-domain PASS lượt 6; eval-chat-quyet-dinh 10/10 tiêu chí.</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">

</xml_diff>

<commit_message>
CEL-177/178: van tong quan tu nhien hon + cham bai luan cho quan tri + agent danh-gia-tac-dong
- prompt-v3: giong van, do dai cau tong quan, pham vi cau hoi dung tren khuon doan
- kiem-v3 / sua-cuc-bo: cau tron chap nhan dau ngoac / ngoac kep cuoi cau
- xu-ly: an pb/model khoi phan tra ve trinh duyet
- Cham bai (admin): the cham tren trang la so, /admin/nhan-xet, xuat .md;
  bang danh_gia_bai_luan (supabase/va-danh-gia-bai.sql, CHUA chay)
- Agent danh-gia-tac-dong vao luong B cua AGENTS.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O177"/>
+  <dimension ref="A1:O179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15206,6 +15206,165 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>CEL-177</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Luật viết tổng quan gọn, tự nhiên (prompt 2026.10.01)</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Câu tổng quan một đoạn không còn phải đi đủ tám bước; viết từ đầy đủ, không nén hai vế thành cụm tắt ("khi nào nên gần, khi nào nên lùi"); TQ01 không mở bằng nhãn một chữ ("Bạn là người thẳng"); câu đã có chỗ riêng (tính cách, điểm mạnh/lưu ý, quý nhân) chỉ được gợi nửa câu ở TQ05/06/07/09/10; validator mới cau-cut chặn câu cuối cụt.</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>1. Sinh tổng quan → prompt có khuôn "câu đầu trả lời thẳng → 1–2 biểu hiện → 1 lưu ý", phạm vi riêng của câu đứng trên khuôn
+2. kiemBai: câu cuối luanGiai / viSao không có dấu kết → cau-cut (chặn)
+3. Sửa cục bộ chỉ nhận câu sửa có dấu kết</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>AI + dữ kiện engine</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Theo thế hệ đếm (KHÔNG tăng THE_HE_DEM — bài cũ giữ đến khi viết lại)</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>/la-so (Tổng quan)</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/prompt-v3.ts, lib/rag/v3/khung.ts, lib/rag/v3/index.ts, lib/rag/v3/kiem-v3.ts, lib/rag/v3/sua-cuc-bo.ts</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>Đo 3 lá số: chữ/bài giảm nhẹ (121→118, 128→120) nhưng câu vẫn ~26 chữ, &gt;25 chữ vẫn 55–70% — độ dài câu là thói quen model, luật chỉ đẩy được ít. So mù hoà (giám khảo thiên vị vị trí). Bài cũ trong đệm vẫn là bản cũ. cau-cut chỉ soát câu cuối.</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>van-luan-tu-nhien</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>CEL-178</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>I. Quản trị</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Chấm bài luận (chỉ quản trị viên)</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Dưới mỗi câu tổng quan có nút "Chấm bài này (quản trị)": Hay / Chưa hay, điểm 1–5, nhận xét, gợi ý cách viết. Gom ở /admin/nhan-xet; nút "Tải bản tổng hợp (.md)" gom theo câu, điểm thấp lên trước, để định kỳ đưa AI đọc và sửa luật. Bản xuất không có email người chấm, không có mã lá số.</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>1. Admin mở lá số → thẻ chấm (người thường không thấy gì)
+2. POST /api/admin/danh-gia-bai: máy chủ tự tính khoá đệm, chụp bài + so với bài đệm (khop_dem), lưu phiên bản prompt / model từ đệm
+3. Chấm lại cùng câu cùng lá số = sửa lượt cũ
+4. /admin/nhan-xet lọc, xem bài lúc chấm, tải .md</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Chờ chạy SQL</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Quản trị viên</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Khi chấm</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Quản trị viên</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>/la-so, /admin/nhan-xet</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>components/luangiai/ChamBaiAdmin.tsx, app/api/admin/danh-gia-bai/route.ts, app/admin/nhan-xet/page.tsx, supabase/va-danh-gia-bai.sql, lib/rag/v3/xu-ly.ts (khoaDemV3, pb/model trong đệm)</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Chạy supabase/va-danh-gia-bai.sql</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Mới gắn vào tổng quan; chuyên sâu để vòng sau. Mở cho người dùng comment sau thì cần bảng/RLS riêng. Tệp .md có chữ luận lá số thật — không commit.</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>van-luan-tu-nhien</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15223,7 +15382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G178"/>
+  <dimension ref="A1:G184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -21686,6 +21845,228 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>L29</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Luật viết tổng quan</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Khuôn câu một đoạn</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Bài một đoạn: câu đầu trả lời thẳng → 1–2 biểu hiện cụ thể → 1 điểm cần lưu ý; thường bốn câu, phần lớn dưới 25 từ. Phạm vi riêng của câu hỏi (TQ02 chỉ điểm mạnh, TQ12 theo nhóm người…) đứng TRÊN khuôn này.</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Tám bước + chuỗi đặc điểm→biểu hiện→hệ quả→giai đoạn ép vào 60–140 chữ sinh câu nén, cụm tắt, lặp ý (góp ý chủ dự án 01/10/2026).</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/prompt-v3.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>L29</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Luật viết tổng quan</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Chống lặp giữa câu song song</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>TQ05/06/07/09/10 có Y_DA_CO_CHU: tính cách chung, điểm mạnh/lưu ý chung, quý nhân nói chung chỉ được gợi nửa câu.</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Chín câu lượt 2 sinh song song, mù nhau — không thể dựa vào sổ ý; chỉ chặn được bằng phạm vi.</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/index.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>L29</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Luật viết tổng quan</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Câu cụt</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>kiemBai cau-cut: câu cuối luanGiai / viSao không kết bằng . ! ? … " ” ' ’ ) ] » → lỗi chặn (có cum → sửa cục bộ). apCauSua bỏ câu sửa thiếu dấu kết (trừ goiY).</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Chỉ soát câu cuối; câu giữa bài cụt chưa bắt.</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/kiem-v3.ts, lib/rag/v3/sua-cuc-bo.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Chấm bài quản trị</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Khoá và bản chụp</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>khoaDemV3 dựng chart_hash + khoa_ky cùng công thức route luận giải (gắn THE_HE_DEM). Bài đệm mang pb (phiên bản prompt) + model; anNoiBo gỡ hai trường này trước khi trả trình duyệt.</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Mặt trước không được lộ tên model — pb/model chỉ sống trong đệm và bảng chấm.</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts, app/api/admin/danh-gia-bai/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Chấm bài quản trị</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Lưu lượt chấm</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>POST /api/admin/danh-gia-bai (canQuanTri): máy chủ tự tính khoá từ laSo, đọc bài đệm, khop_dem = chữ admin thấy trùng bài đệm; pb/model chỉ ghi khi khop. Upsert theo (nguoi_cham, chart_hash, khoa_ky, id_cau) → chấm lại là sửa.</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Trang có thể đang hiện bản cũ / thế hệ trước — không có khop_dem thì nhận xét gắn nhầm phiên bản prompt.</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>app/api/admin/danh-gia-bai/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Chấm bài quản trị</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Bản tổng hợp</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>/admin/nhan-xet gom theo câu, điểm TB thấp lên trước, trong câu thì chưa hay / điểm thấp trước; xuất .md KHÔNG có email người chấm, KHÔNG có chart_hash.</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Quy định bảo mật tổ chức: không xuất tệp chứa email. Tệp vẫn có chữ luận lá số thật — không commit.</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>app/admin/nhan-xet/page.tsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21698,7 +22079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F111"/>
+  <dimension ref="A1:F113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25269,6 +25650,70 @@
         </is>
       </c>
       <c r="F111" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>van-luan-tu-nhien</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CEL-177</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Sửa luật viết tổng quan: khuôn câu một đoạn, cấm cụm tắt / nhãn một chữ, chống lặp giữa câu song song, validator cau-cut. Prompt 2026.10.01, không đổi model, không tăng THE_HE_DEM.</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Chủ dự án chỉ ra "Bạn là người thẳng", "khi nào nên gần, khi nào nên lùi", câu nén, lặp ý. Chẩn đoán: luật tám bước + chuỗi bốn khâu ép vào 60–140 chữ, không phải model. Ba ý (nới mở "Bạn", bỏ dàn ý, đổi thứ tự lượt) bị phản biện đánh sập nên bỏ.</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>van-luan-tu-nhien</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>CEL-178</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Thêm chấm bài cho quản trị viên (Hay/Chưa hay, 1–5, nhận xét, gợi ý cách viết) + trang /admin/nhan-xet + bản tổng hợp .md.</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Chủ dự án muốn gom góp ý một chỗ để định kỳ sửa luật bằng dữ liệu thay vì nhớ. Bản xuất bỏ email (quy định bảo mật tổ chức).</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
CEL-179: kho tri thuc — ghi chu uu tien nguon, luat ngam moi duong, thu vien theo ban xuat ban
- /admin/knowledge: khoi gap "Thu tu uu tien nguon"; he phai mac dinh 'chung', kho khong loc he phai
- Nguon ghi-chu-chuyen-gia / noi-bo vao moi duong tra loi duoi nhan N# (fail-closed),
  kem LUAT_NGUON_NGAM; cong ngon ngu them lo-luat-ngam (canh bao)
- Xuat ban ban moi tu dong bo thu vien (dong-bo.ts, khong goi model): doi cau trich sang
  ban moi, mat cau trich thi bo ca muc, muc lat mat het dich thi bo; nut dong bo tay
- conDuocDan: muc dan tai lieu khong xuat ban hoac ban da bi thay khong vao prompt
- Quyet dinh ghi o docs/quyet-dinh/2026-10-01-kho-tri-thuc.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O177"/>
+  <dimension ref="A1:O178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15206,6 +15206,86 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" s="13" t="inlineStr">
+        <is>
+          <t>CEL-179</t>
+        </is>
+      </c>
+      <c r="B178" s="14" t="inlineStr">
+        <is>
+          <t>H. Tri thức</t>
+        </is>
+      </c>
+      <c r="C178" s="8" t="inlineStr">
+        <is>
+          <t>Kho tri thức: ghi chú thứ tự ưu tiên + luật ngầm mọi đường + thư viện theo bản xuất bản mới</t>
+        </is>
+      </c>
+      <c r="D178" s="8" t="inlineStr">
+        <is>
+          <t>Trang /admin/knowledge có khối gập "Thứ tự ưu tiên nguồn" (thứ bậc dữ kiện → thư viện → đoạn gốc → kiến thức model; mức tin cậy; hai đường chọn nguồn; hệ phái không lọc). Nguồn ghi-chu-chuyen-gia / noi-bo dùng được ở MỌI đường trả lời dưới nhãn N# không đề mục, kèm luật không để lộ. Xuất bản bản mới tự đồng bộ thư viện; mỗi tài liệu có dòng trạng thái thư viện + nút "Đồng bộ thư viện".</t>
+        </is>
+      </c>
+      <c r="E178" s="8" t="inlineStr">
+        <is>
+          <t>1. Xuất bản bản mới → route phien-ban gọi dongBoThuVien → thông báo kết quả
+2. Lưu trữ → mục dẫn tài liệu đó ẩn khỏi prompt (không gỡ)
+3. Xoá hẳn → gỡ vĩnh viễn
+4. Dòng trạng thái: khớp / còn N đoạn mới chưa đọc / chưa đối chiếu (có nút)</t>
+        </is>
+      </c>
+      <c r="F178" s="9" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G178" s="8" t="inlineStr">
+        <is>
+          <t>Kho tri thức</t>
+        </is>
+      </c>
+      <c r="H178" s="8" t="inlineStr">
+        <is>
+          <t>Theo lần xuất bản</t>
+        </is>
+      </c>
+      <c r="I178" s="8" t="inlineStr">
+        <is>
+          <t>Quản trị</t>
+        </is>
+      </c>
+      <c r="J178" s="8" t="inlineStr">
+        <is>
+          <t>/admin/knowledge</t>
+        </is>
+      </c>
+      <c r="K178" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/dong-bo.ts, lib/rag/thu-vien/cho-prompt.ts, lib/rag/bang-chung.ts, lib/ket-noi/tra-loi.ts, lib/rag/ngon-ngu.ts, app/api/admin/knowledge/phien-ban/route.ts, app/admin/knowledge/page.tsx</t>
+        </is>
+      </c>
+      <c r="L178" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M178" s="8" t="inlineStr">
+        <is>
+          <t>Đồng bộ chỉ BỚT, chưa thêm: đoạn mới cần nút "đọc vào thư viện" (nhánh sau, gọi model). lo-luat-ngam chỉ cảnh báo. Hai đồng bộ song song cùng đợt có thể đè nhau (bấm lại chữa được). Phần ghi chưa đo trên DB thật. Lần đầu mỗi tài liệu hiện nút "chưa đối chiếu" cho tới khi đồng bộ.</t>
+        </is>
+      </c>
+      <c r="N178" s="8" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="O178" s="8" t="inlineStr">
+        <is>
+          <t>kho-tri-thuc-uu-tien</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15223,7 +15303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G178"/>
+  <dimension ref="A1:G184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -21686,6 +21766,228 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="30" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B179" s="31" t="inlineStr">
+        <is>
+          <t>Kho tri thức: nguồn ngầm + thư viện theo bản mới</t>
+        </is>
+      </c>
+      <c r="C179" s="31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D179" s="8" t="inlineStr">
+        <is>
+          <t>Nhận diện nguồn ngầm</t>
+        </is>
+      </c>
+      <c r="E179" s="8" t="inlineStr">
+        <is>
+          <t>laNguonAn(meta, documentId): loai_nguon ghi-chu-chuyen-gia | noi-bo, hoặc không có meta → ngầm. truyHoi gán cờ an theo meta sống trước khi xếp hạng.</t>
+        </is>
+      </c>
+      <c r="F179" s="32" t="inlineStr">
+        <is>
+          <t>Fail-closed: đọc kho hỏng thì thà giấu nhầm còn hơn lộ.</t>
+        </is>
+      </c>
+      <c r="G179" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/tai-lieu-meta.ts, lib/rag/truy-hoi.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="30" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B180" s="31" t="inlineStr">
+        <is>
+          <t>Kho tri thức: nguồn ngầm + thư viện theo bản mới</t>
+        </is>
+      </c>
+      <c r="C180" s="31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D180" s="8" t="inlineStr">
+        <is>
+          <t>Nhãn nguồn trong prompt</t>
+        </is>
+      </c>
+      <c r="E180" s="8" t="inlineStr">
+        <is>
+          <t>nhanNguon: nguồn hiện = [mức · mục "đề mục"]; nguồn ngầm = [mức · LUẬT NGẦM N#] không đề mục. N# đánh theo tài liệu (danhMaTaiLieu) để model biết nhiều đoạn cùng một nguồn. LUAT_NGUON_NGAM chỉ chèn khi gói có nguồn ngầm (không phá đệm bài cũ).</t>
+        </is>
+      </c>
+      <c r="F180" s="32" t="inlineStr">
+        <is>
+          <t>Đường tự định dạng nguồn (Kết nối) phải dùng nhanNguon, không tự viết nhãn.</t>
+        </is>
+      </c>
+      <c r="G180" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/bang-chung.ts, lib/ket-noi/tra-loi.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="30" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B181" s="31" t="inlineStr">
+        <is>
+          <t>Kho tri thức: nguồn ngầm + thư viện theo bản mới</t>
+        </is>
+      </c>
+      <c r="C181" s="31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D181" s="8" t="inlineStr">
+        <is>
+          <t>Cổng ngôn ngữ</t>
+        </is>
+      </c>
+      <c r="E181" s="8" t="inlineStr">
+        <is>
+          <t>Luật lo-luat-ngam (cảnh báo) bắt "theo chuyên gia", "tài liệu nội bộ", "luật ngầm", "theo kinh nghiệm của Celes"…; khớp theo cụm từ, không bắt "hỏi ý kiến chuyên gia tài chính".</t>
+        </is>
+      </c>
+      <c r="F181" s="32" t="inlineStr">
+        <is>
+          <t>Chỉ cảnh báo: chặn làm bài không vào đệm, sinh lại mỗi lần mở trang.</t>
+        </is>
+      </c>
+      <c r="G181" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/ngon-ngu.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="30" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B182" s="31" t="inlineStr">
+        <is>
+          <t>Kho tri thức: nguồn ngầm + thư viện theo bản mới</t>
+        </is>
+      </c>
+      <c r="C182" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D182" s="8" t="inlineStr">
+        <is>
+          <t>Đồng bộ thư viện khi xuất bản</t>
+        </is>
+      </c>
+      <c r="E182" s="8" t="inlineStr">
+        <is>
+          <t>dongBoTrongBoNho: mỗi câu trích của tài liệu → khớp băm đoạn cũ, rồi nguyên văn trên cả bản mới (câu ≥ 40 ký tự chuẩn), rồi khớp gần ±3 thứ tự. Mất dù một câu trích → bỏ cả mục; mục lật mất hết đích → bỏ (lặp tới ổn định); còn đích thì chỉ gỡ đích đã bỏ.</t>
+        </is>
+      </c>
+      <c r="F182" s="32" t="inlineStr">
+        <is>
+          <t>Không giữ câu nghĩa y trên căn cứ thiếu. Chỉ bớt, không thêm.</t>
+        </is>
+      </c>
+      <c r="G182" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/dong-bo.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="30" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B183" s="31" t="inlineStr">
+        <is>
+          <t>Kho tri thức: nguồn ngầm + thư viện theo bản mới</t>
+        </is>
+      </c>
+      <c r="C183" s="31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D183" s="8" t="inlineStr">
+        <is>
+          <t>Sổ đã đọc</t>
+        </is>
+      </c>
+      <c r="E183" s="8" t="inlineStr">
+        <is>
+          <t>Sổ (noi_dung_ai be_mat thu-vien-da-doc) lưu băm các đoạn đã đọc + versionId + chuaDoc. Lần đầu dựng từ các bản mà câu trích trỏ tới. Ghi sổ (versionId rỗng) TRƯỚC khi ghi thư viện, đóng dấu bản mới SAU — ghi thư viện lỗi thì nút đồng bộ vẫn hiện và lần thử lại không đếm sai.</t>
+        </is>
+      </c>
+      <c r="F183" s="32" t="inlineStr">
+        <is>
+          <t>Dựng sổ phải trước khi dời câu trích.</t>
+        </is>
+      </c>
+      <c r="G183" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/dong-bo.ts, lib/rag/thu-vien/kho.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="30" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B184" s="31" t="inlineStr">
+        <is>
+          <t>Kho tri thức: nguồn ngầm + thư viện theo bản mới</t>
+        </is>
+      </c>
+      <c r="C184" s="31" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D184" s="8" t="inlineStr">
+        <is>
+          <t>Chặn lúc dựng prompt</t>
+        </is>
+      </c>
+      <c r="E184" s="8" t="inlineStr">
+        <is>
+          <t>conDuocDan: bỏ mục có câu trích dẫn tài liệu không xuất bản (lưu trữ / hạ) hoặc dẫn bản đã bị thay (versionId ∉ banXuatBan); mục lật mất hết đích cũng bỏ. Meta rỗng → giữ nguyên.</t>
+        </is>
+      </c>
+      <c r="F184" s="32" t="inlineStr">
+        <is>
+          <t>Lưu trữ không gỡ vĩnh viễn — xuất bản lại là mục trở về.</t>
+        </is>
+      </c>
+      <c r="G184" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/cho-prompt.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21698,7 +22000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F111"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25269,6 +25571,38 @@
         </is>
       </c>
       <c r="F111" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>kho-tri-thuc-uu-tien</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CEL-179</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Ghi chú thứ tự ưu tiên ở Kho tri thức; bỏ lọc hệ phái (mặc định chung); luật ngầm vào mọi đường trả lời dưới nhãn N#; thư viện tự đồng bộ khi xuất bản bản mới + nút đồng bộ tay; mục mất căn cứ bị bỏ cả mục.</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Chủ dự án không rõ RAG ưu tiên thế nào; chốt 01/10: (1) không lọc theo hệ phái, mức tin cậy phân xử; (2) luật ngầm phải áp cho mọi phần luận giải chứ không riêng v3; (3) thư viện phải là bản mới nhất của tài liệu — xuất bản lại cấp id mới cho mọi đoạn nên căn cứ cũ trỏ vào bản đã thay. celes-domain chỉ ra giữ mục với căn cứ thiếu là để thư viện khẳng định điều nguồn không còn đỡ → bỏ cả mục.</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
CEL-179: du kien v3 xet du moi sao, nghia theo cung, co xung chieu
- Cung chinh: moi sao (chinh, phu, vong, tu hoa, Trang Sinh) co nghia, chia sao nang / sao nhe
- Nhan doi chu ngu theo cung; nghia nen con nguoi chi o Menh hoac Than khi cau goi Than
- Xung chieu co nghia (khong nghia nen); tam hop du ten + nghia sao nang
- Giap cung (Ta Huu, Xuong Khuc, Khoi Viet, Tu Phu, Quyen Loc, Khoa Quyen, Nhat Nguyet sang, Kinh Da, Khong Kiep, Hoa Linh)
- Cach cuc quet theo tam phuong cung chu de
- Truy hoi: bo bi danh cung mot am tiet, them truy van phu tinh nang
- Prompt luat 8, 17: chi chuyen tinh chat, cam suy ngoai tinh / benh / mat mat nguoi than; hung dac dia khong ep thanh luc keo
- kiem-v3: canh bao bo-luc-hung (khong chan)
- scripts/test-phu-du-kien.ts vao CI, moi muc 100%
- Khong tang THE_HE_DEM: bai cu giu nguyen

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O179"/>
+  <dimension ref="A1:O180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15281,7 +15281,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>van-luan-tu-nhien</t>
+          <t>76e1033</t>
         </is>
       </c>
     </row>
@@ -15361,7 +15361,84 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>van-luan-tu-nhien</t>
+          <t>76e1033</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>CEL-179</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>C. Luận giải</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Dữ kiện xét đủ mọi sao, nghĩa theo cung, có xung chiếu</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Gói dữ kiện F### của mọi câu v3 đưa ĐỦ mọi sao của cung chính (chính tinh, phụ tinh, vòng sao, tứ hoá, Tràng Sinh) kèm câu nghĩa, có nhãn "đọc theo mặt đời của cung" (Tả Hữu ở Phu Thê nói về người phối ngẫu, không về tính cách bạn). Xung chiếu có nghĩa chính tinh/tứ hoá/sao nặng, nhãn "chiếu thẳng vào cung chính"; tam hợp có đủ tên, nghĩa sao nặng; giáp cung; cách cục quét trên tam phương cung chủ đề. Truy hồi thêm một truy vấn phụ tinh nặng, bỏ bí danh cung một âm tiết. Luật prompt 17 tam phương.</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>1. dungDuKien → moTaCung theo chế độ chinh/xung/tam-hop → 2. sao nặng dựng ý, sao nhẹ làm sắc thái → 3. giapCung + cách cục tam phương cung chủ đề → 4. truy hồi + truy vấn phụ tinh nặng → 5. prompt luật 8/17 → 6. kiem-v3 cảnh báo bo-luc-hung (không chặn)</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>AI + dữ kiện engine</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Theo thế hệ đếm (KHÔNG tăng THE_HE_DEM — bài cũ giữ, người dùng bấm luận giải lại để lấy bản mới)</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Mọi người dùng</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>/la-so (Tổng quan + Chuyên sâu)</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/du-kien.ts, lib/rag/v3/truy-hoi-v3.ts, lib/rag/v3/prompt-v3.ts, lib/rag/v3/kiem-v3.ts, scripts/test-phu-du-kien.ts</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Dữ kiện mỗi câu 4235→9644 ký tự (+128% phần dữ kiện, ~+12% tổng token vào vì system prompt chiếm phần lớn). Giáp cung: Tử Phủ, Quyền Lộc, Khoa Quyền; Nhật Nguyệt chỉ cát khi cả hai sáng. Hung tinh đắc địa không bị ép thành lực kéo. Đổi chủ ngữ chỉ chuyển tính chất, cấm suy ngoại tình/bệnh/mất mát người thân. Chưa đo chất lượng bằng model thật (do-chat-luong-v3 3 lá số) và recall eval-rag sau đổi bí danh — chạy tay. Đợt 2 (thư viện sao×cung có trích sách) chờ kết quả đo trần 11.9.</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>viec/phu-du-kien</t>
         </is>
       </c>
     </row>
@@ -15382,7 +15459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G184"/>
+  <dimension ref="A1:G188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -22067,6 +22144,154 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Dữ kiện đủ sao (CEL-179)</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Phân tầng sao</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>laSaoNang: chính tinh, tứ hoá, CAT/HUNG có trọng số, NANG_THEM (Khốc Hư, Đào Hồng Hỷ, Cô Quả, Thiên Không), sao chủ đề = sao NẶNG; còn lại NHẸ. Cung chính: mọi sao có nghĩa; sao nhẹ ghi "sao nhẹ" + vòng Tràng Sinh.</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Đổ sao ngang hàng → 78% câu thành danh sách sao (docs/bay/ai-rag.md). Sao nhẹ chỉ làm sắc thái, không tự dựng ý.</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/du-kien.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Dữ kiện đủ sao (CEL-179)</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Nghĩa theo cung</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>moTaCung(...,cheDo,cungGoc,docLaThan): nhãn "Đọc mọi nét dưới đây: &lt;mặt đời&gt;" một lần mỗi cung; Nghĩa nền con người chỉ ở Mệnh, hoặc cung Thân khi câu gọi THAN / phụ trợ Thân.</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Cung Thân ở Phu Thê từng nhận nghĩa nền tính cách. test-phu-du-kien chặn 100%.</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/du-kien.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Dữ kiện đủ sao (CEL-179)</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Tam phương</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Xung: "CHIẾU THẲNG vào cung X" + nghĩa chính tinh/tứ hoá/sao nặng, không nghĩa nền. Tam hợp: đủ tên, nghĩa tứ hoá + sao trọng số ≥1. Giáp cung 8 cặp (prefix "Giáp cung:" để cungDangDoc không coi là cung). Cách cục: nhanDangCachCuc với menhIndex xoay về cung chủ đề, hậu tố đọc theo mặt đời.</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Chế độ "gọn" cũ (25/09) bỏ vì nghĩa nền Mệnh + Hỏa Linh lọt vào tam phương; nay xung không có nghĩa nền thay vì không có nghĩa.</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/du-kien.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Dữ kiện đủ sao (CEL-179)</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Truy hồi + prompt + kiểm</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>BI_DANH_CUNG bỏ bí danh một âm tiết; điểm khớp dùng mọi sao nặng của cung; thêm truy vấn phụ tinh nặng (≤3 sao, giữ cặp) đứng sau truy vấn cung chính. Prompt luật 17 tam phương. kiem-v3 bo-luc-hung: cung chính/xung có hung nặng hoặc Kỵ mà dàn ý không trích mã → cảnh báo chan:false.</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Bí danh một âm tiết ("the","di","tai") khớp nhầm đoạn sách. Cảnh báo chưa chặn để không tăng vòng sửa.</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/truy-hoi-v3.ts, lib/rag/v3/prompt-v3.ts, lib/rag/v3/kiem-v3.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22079,7 +22304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:F114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25663,7 +25888,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>van-luan-tu-nhien</t>
+          <t>76e1033</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -25695,7 +25920,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>van-luan-tu-nhien</t>
+          <t>76e1033</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -25714,6 +25939,38 @@
         </is>
       </c>
       <c r="F113" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>viec/phu-du-kien</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>CEL-179</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Dữ kiện v3 đưa đủ mọi sao cung chính kèm nghĩa theo cung; xung chiếu có nghĩa; tam hợp đủ tên; giáp cung; cách cục theo tam phương cung chủ đề; truy vấn phụ tinh; luật prompt 17; cảnh báo bo-luc-hung; test-phu-du-kien vào CI.</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "mọi chính, phụ tinh đều được xét đến để luận giải, không có một hạn chế nào"; "Tả Hữu ở Phu Thê mà luận như ở Mệnh là sai hoàn toàn"; "sao lại không xét cung xung chiếu". Đo trước: sao nhẹ cung chính có nghĩa 2,2%, Tràng Sinh 0%, xung chiếu có nghĩa 0% → nay 100%.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
CEL-179: do that bang model (eval-phu-du-kien A/B) + ket qua tran 11.9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15438,7 +15438,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>viec/phu-du-kien</t>
+          <t>7318e4d</t>
         </is>
       </c>
     </row>
@@ -22304,7 +22304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25952,25 +25952,57 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
+          <t>7318e4d</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>CEL-179</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Dữ kiện v3 đưa đủ mọi sao cung chính kèm nghĩa theo cung; xung chiếu có nghĩa; tam hợp đủ tên; giáp cung; cách cục theo tam phương cung chủ đề; truy vấn phụ tinh; luật prompt 17; cảnh báo bo-luc-hung; test-phu-du-kien vào CI.</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "mọi chính, phụ tinh đều được xét đến để luận giải, không có một hạn chế nào"; "Tả Hữu ở Phu Thê mà luận như ở Mệnh là sai hoàn toàn"; "sao lại không xét cung xung chiếu". Đo trước: sao nhẹ cung chính có nghĩa 2,2%, Tràng Sinh 0%, xung chiếu có nghĩa 0% → nay 100%.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5 (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
           <t>viec/phu-du-kien</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C115" t="inlineStr">
         <is>
           <t>CEL-179</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Dữ kiện v3 đưa đủ mọi sao cung chính kèm nghĩa theo cung; xung chiếu có nghĩa; tam hợp đủ tên; giáp cung; cách cục theo tam phương cung chủ đề; truy vấn phụ tinh; luật prompt 17; cảnh báo bo-luc-hung; test-phu-du-kien vào CI.</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Chủ dự án: "mọi chính, phụ tinh đều được xét đến để luận giải, không có một hạn chế nào"; "Tả Hữu ở Phu Thê mà luận như ở Mệnh là sai hoàn toàn"; "sao lại không xét cung xung chiếu". Đo trước: sao nhẹ cung chính có nghĩa 2,2%, Tràng Sinh 0%, xung chiếu có nghĩa 0% → nay 100%.</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Đo thật CEL-179 bằng model (scripts/eval-phu-du-kien.ts, A/B mã 76e1033 ↔ 7318e4d, 3 lá mẫu × 5 câu cung ≠ Mệnh): dàn ý trích xung chiếu 8/15 → 15/15; sao hung xung chiếu được nêu ở vì sao 6/27 → 16/27; điểm xung chiếu của giám khảo tăng ở cả ba giám khảo (gpt-oss 0,80→1,33); điểm "đúng theo cung" không đổi rõ (giám khảo lệch nhau ±0,7); phụ tinh cung chính được nêu 37/107 không đổi; tỉ lệ phải sửa 4/15 → 7/15; token vào/bài +45%, chi phí/bài 0,0033 → 0,0043 USD. Đo trần 11.9: O = 71,2% KT (A 50,6%). Chi phí đo: luận chuyên sâu đủ 9 chủ đề (29 câu) một lá số = 0,167 USD + ~0,01 tóm lại.</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Chủ dự án: "phải có cơ chế test, gọi model để kiểm chứng code có tác dụng thật". Kết luận: xung chiếu có tác dụng thật; phụ tinh tới model nhưng model chưa dùng thêm — khớp kết quả trần 71% (nút thắt ở khâu viết), nên đợt 2 (bảng sao×cung từ sách) chưa đáng làm.</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
         <is>
           <t>Claude Opus 5.5 (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: go trung ID CEL-150, cap CEL-182 cho tri nho hoi thoai
Hai tinh nang khac han nhau cung mang CEL-150:
  - "Core Web Vitals + a11y + SEO" (Backlog dong 150)
  - "Sua mat tri nho hoi thoai khi bam chip goi y thu hai" (dong 151)

Doc "CEL-150" trong nhat ky khong biet dang noi cai nao. Giu ID cu cho
dong vao truoc (Core Web Vitals), cap ID ke tiep cho dong sau — dung luat
"khong dung lai ID cu".

Doi theo 5 noi tham chieu, phan loai tung cai theo ngu canh:
  Backlog 151 cot ID            -> CEL-182
  Backlog 153 "phien kiem"      -> CEL-182 (ngu canh la phien kiem chat)
  Nhat ky 82 "CEL-150, CEL-151" -> CEL-182, CEL-151
  Nhat ky 83 cot Vi sao         -> CEL-182 (cung phien kiem chat)
  TRANG-THAI.md dong 51         -> CEL-182

Giu nguyen CEL-150 o: Backlog 150, Nhat ky 81, TRANG-THAI.md dong 52,
UIUX-RA-SOAT-2026-09-27.md — deu la Core Web Vitals that.

Da kiem lai: khong con ID nao trung trong sheet Backlog.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -13061,7 +13061,7 @@
     <row r="151">
       <c r="A151" s="13" t="inlineStr">
         <is>
-          <t>CEL-150</t>
+          <t>CEL-182</t>
         </is>
       </c>
       <c r="B151" s="14" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="D153" s="8" t="inlineStr">
         <is>
-          <t>Chủ dự án yêu cầu rà kỹ sau khi thấy một lượt trong phiên kiểm CEL-150 trả lời rỗng. Dựng lại đúng bối cảnh 6 lần bằng API thật KHÔNG tái hiện được — đây là một lần hỏng hiếm ở phía model (JSON gãy giữa chừng), không phải lỗi do CEL-150 gây ra. Nhưng đường xử lý của route thì sai thật: `traLoiCoCanCu` cố ý trả `van: ''` khi văn bản thô trông như JSON mà đọc không được (đúng thiết kế — JSON dở dang còn tệ hơn không có gì), nhưng route trước đó ship thẳng chuỗi rỗng ấy như một câu trả lời thành công (HTTP 200): người dùng thấy bong bóng TRẮNG, không lỗi, không chip, không cách hỏi lại — và lượt hỏi của họ vẫn bị trừ.</t>
+          <t>Chủ dự án yêu cầu rà kỹ sau khi thấy một lượt trong phiên kiểm CEL-182 trả lời rỗng. Dựng lại đúng bối cảnh 6 lần bằng API thật KHÔNG tái hiện được — đây là một lần hỏng hiếm ở phía model (JSON gãy giữa chừng), không phải lỗi do CEL-150 gây ra. Nhưng đường xử lý của route thì sai thật: `traLoiCoCanCu` cố ý trả `van: ''` khi văn bản thô trông như JSON mà đọc không được (đúng thiết kế — JSON dở dang còn tệ hơn không có gì), nhưng route trước đó ship thẳng chuỗi rỗng ấy như một câu trả lời thành công (HTTP 200): người dùng thấy bong bóng TRẮNG, không lỗi, không chip, không cách hỏi lại — và lượt hỏi của họ vẫn bị trừ.</t>
         </is>
       </c>
       <c r="E153" s="8" t="inlineStr">
@@ -22898,7 +22898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>CEL-150, CEL-151</t>
+          <t>CEL-182, CEL-151</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr">
@@ -25569,7 +25569,7 @@
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>Chủ dự án yêu cầu rà lại toàn bộ sau khi phát hiện một lượt trả lời rỗng trong lúc kiểm CEL-150.</t>
+          <t>Chủ dự án yêu cầu rà lại toàn bộ sau khi phát hiện một lượt trả lời rỗng trong lúc kiểm CEL-182.</t>
         </is>
       </c>
       <c r="F83" s="8" t="inlineStr">
@@ -26949,6 +26949,38 @@
         </is>
       </c>
       <c r="F126" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B127" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/ca-nhan-hoa-phase-3)</t>
+        </is>
+      </c>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>CEL-182</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="inlineStr">
+        <is>
+          <t>Cấp ID mới CEL-182 cho "Sửa mất trí nhớ hội thoại khi bấm chip gợi ý thứ hai + kéo dài ghi nhớ". Trước đó nó mang CEL-150 — trùng với "Core Web Vitals + a11y + SEO". Đổi theo cả 4 nơi tham chiếu: Backlog dòng 151 (ID) và 153 (mô tả), Nhật ký dòng 82 (ID liên quan) và 83 (cột Vì sao).</t>
+        </is>
+      </c>
+      <c r="E127" s="8" t="inlineStr">
+        <is>
+          <t>Hai tính năng khác hẳn nhau cùng mang một ID thì mọi tham chiếu về sau đều mơ hồ — đọc "CEL-150" không biết đang nói Core Web Vitals hay trí nhớ chat. Giữ ID cũ cho dòng vào trước (Core Web Vitals), cấp ID kế tiếp cho dòng sau, đúng luật "không dùng lại ID cũ" trong AGENTS.md. Ba tham chiếu gián tiếp đều thuộc ngữ cảnh phiên kiểm chat nên trỏ về CEL-182, không phải CEL-150.</t>
+        </is>
+      </c>
+      <c r="F127" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5</t>
         </is>

</xml_diff>

<commit_message>
CEL-184: lop sua cau khong lam sap xuong dong (tachManh/rapManh)
tachCau + join(' ') trong suaCauTiengLong / suaCauKeSao bien moi \n\n,
tieu de va danh sach thanh mot dong khi co cau phai sua. Thay bang cap
tach/rap lossless: rapManh(tachManh(x)) === x, chi thay manh NOI_DUNG,
bo qua dong tieu de, lam sach cau model tra ve, giu dau ** le.

Khong doi khoa dem: dem chi-doc tren noi_dung_ai cho 0 ban ghi co \n
o moi be mat co dem di qua lop sua.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O183"/>
+  <dimension ref="A1:O184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15679,6 +15679,88 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" s="11" t="inlineStr">
+        <is>
+          <t>CEL-184</t>
+        </is>
+      </c>
+      <c r="B184" s="12" t="inlineStr">
+        <is>
+          <t>B. Luận giải AI</t>
+        </is>
+      </c>
+      <c r="C184" s="8" t="inlineStr">
+        <is>
+          <t>Lớp sửa câu không làm sập xuống dòng (tachManh / rapManh)</t>
+        </is>
+      </c>
+      <c r="D184" s="8" t="inlineStr">
+        <is>
+          <t>LỖI ĐÃ SỬA, chạy trên prod. tachCau cắt câu bằng split(/(?&lt;=[.!?])\s+/) rồi suaCauTiengLong và suaCauKeSao ráp lại bằng join(' '): mọi 
+ thành một dấu cách, tiêu đề "### …" (không có dấu chấm) dính vào câu sau và có thể bị thay luôn, danh sách "1. …" bị cắt sau "1.". Chỉ xảy ra ở bài có câu phải sửa (~3%), nên không ai thấy. Phá "kết luận đứng một mình" của chat và khuôn BÁO CÁO.</t>
+        </is>
+      </c>
+      <c r="E184" s="8" t="inlineStr">
+        <is>
+          <t>1. tachManh(van) cắt thành mảnh NOI_DUNG / PHAN_CACH, đi theo dòng; dấu đầu dòng, khoảng trắng và xuống dòng là PHAN_CACH.
+2. Hai hàm sửa chỉ xét mảnh NOI_DUNG, bỏ qua dòng tiêu đề.
+3. Câu model trả về qua lamSachCauMoi (bỏ xuống dòng, tiền tố C1./-/#/1., giữ dấu ** lẻ của câu gốc).
+4. thayManh → rapManh nối thẳng, không chèn gì.</t>
+        </is>
+      </c>
+      <c r="F184" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G184" s="8" t="inlineStr">
+        <is>
+          <t>Hàm thuần (lớp sửa vẫn gọi model như cũ)</t>
+        </is>
+      </c>
+      <c r="H184" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I184" s="8" t="inlineStr">
+        <is>
+          <t>Mọi bậc</t>
+        </is>
+      </c>
+      <c r="J184" s="8" t="inlineStr">
+        <is>
+          <t>Hỏi Celes, bài dài, bản đọc sâu, bảng lĩnh vực, bề mặt ngắn, kết nối</t>
+        </is>
+      </c>
+      <c r="K184" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/sua-chua.ts; scripts/test-sua-chua-tach.ts</t>
+        </is>
+      </c>
+      <c r="L184" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M184" s="8" t="inlineStr">
+        <is>
+          <t>KHÔNG đổi khoá đệm: đếm chỉ-đọc 02/10/2026 trên noi_dung_ai — ban-doc-sau 0/11, bang-linh-vuc 0/10, diem-noi-bat 0/46, nhịp/mốc/luận hạn 0 bản ghi có 
+; các trường ở đó vốn một đoạn nên lỗi không có gì để hỏng. Bài dài và chat (bị nặng nhất) không có đệm. Tiêu đề khớp tiếng lóng giờ được để nguyên, chỉ cổng ngôn ngữ ghi trace.</t>
+        </is>
+      </c>
+      <c r="N184" s="8" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="O184" s="8" t="inlineStr">
+        <is>
+          <t>(nhánh viec/sua-xuong-dong-tieng-long)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15696,7 +15778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G210"/>
+  <dimension ref="A1:G213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -16851,7 +16933,7 @@
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>suaCauKeSao(): câu nào kê từ hai tên sao trở lên thì gửi MỘT lượt gọi nhỏ để viết lại, thay vì vứt cả bài.</t>
+          <t>suaCauKeSao(): câu nào kê từ hai tên sao trở lên thì gửi MỘT lượt gọi nhỏ để viết lại, thay vì vứt cả bài. Tách/ráp câu bằng tachManh/rapManh, giữ nguyên xuống dòng — xem CEL-184.</t>
         </is>
       </c>
       <c r="F33" s="32" t="inlineStr">
@@ -19539,7 +19621,7 @@
       </c>
       <c r="E108" s="8" t="inlineStr">
         <is>
-          <t>Sau dungVan, quét từng CÂU bằng một biểu thức CÓ DẤU. Có câu phạm thì gom cả lượt vào MỘT lần gọi model, xin viết lại, kèm danh sách tên dữ kiện engine đã đọc được (dauMoc + cachCuc) để model lấy ra dùng. Câu sửa xong mà vẫn phạm, hoặc ngắn dưới 15 ký tự, thì bỏ — giữ câu gốc. Không có câu phạm thì KHÔNG gọi model, nên phần lớn lượt hỏi không tốn thêm gì.</t>
+          <t>Sau dungVan, quét từng CÂU bằng một biểu thức CÓ DẤU. Có câu phạm thì gom cả lượt vào MỘT lần gọi model, xin viết lại, kèm danh sách tên dữ kiện engine đã đọc được (dauMoc + cachCuc) để model lấy ra dùng. Câu sửa xong mà vẫn phạm, hoặc ngắn dưới 15 ký tự, thì bỏ — giữ câu gốc. Không có câu phạm thì KHÔNG gọi model, nên phần lớn lượt hỏi không tốn thêm gì. Tách/ráp câu bằng tachManh/rapManh, giữ nguyên xuống dòng — xem CEL-184.</t>
         </is>
       </c>
       <c r="F108" s="32" t="inlineStr">
@@ -23330,6 +23412,119 @@
       <c r="G210" s="8" t="inlineStr">
         <is>
           <t>lib/rag/hop-dong-tra-loi.ts; lib/rag/nghieng-ve.ts; docs/chien-luoc/ca-nhan-hoa-celes.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="53" t="inlineStr">
+        <is>
+          <t>CEL-184</t>
+        </is>
+      </c>
+      <c r="B211" s="54" t="inlineStr">
+        <is>
+          <t>Lớp sửa câu (tách / ráp)</t>
+        </is>
+      </c>
+      <c r="C211" s="54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D211" s="8" t="inlineStr">
+        <is>
+          <t>Bất biến lossless</t>
+        </is>
+      </c>
+      <c r="E211" s="8" t="inlineStr">
+        <is>
+          <t>rapManh(tachManh(x)) === x với mọi x. rapManh chỉ nối text các mảnh, không chuẩn hoá khoảng trắng. Khoá/chuỗi không có câu nào được sửa thì trả lại ĐÚNG chuỗi gốc.</t>
+        </is>
+      </c>
+      <c r="F211" s="32" t="inlineStr">
+        <is>
+          <t>Bản cũ vứt phần ngăn cách khi tách nên join(' ') không thể khôi phục 
+. Sửa ở primitive để cả suaCauTiengLong lẫn suaCauKeSao hết lỗi cùng lúc; không vá riêng cho dấu ấn Celes.</t>
+        </is>
+      </c>
+      <c r="G211" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/sua-chua.ts; scripts/test-sua-chua-tach.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="53" t="inlineStr">
+        <is>
+          <t>CEL-184</t>
+        </is>
+      </c>
+      <c r="B212" s="54" t="inlineStr">
+        <is>
+          <t>Lớp sửa câu (tách / ráp)</t>
+        </is>
+      </c>
+      <c r="C212" s="54" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D212" s="8" t="inlineStr">
+        <is>
+          <t>Ranh giới câu và dòng</t>
+        </is>
+      </c>
+      <c r="E212" s="8" t="inlineStr">
+        <is>
+          <t>Đi theo dòng. Dấu đầu dòng (#, -, *, +, 1., 1), &gt;) là PHAN_CACH. Xuống dòng đơn giữa hai dòng chữ thường là xuống dòng MỀM, giữ trong câu. Ranh giới câu: [.!?] kèm dấu đóng ngay sau (")”’]*_) rồi khoảng trắng. KHÔNG cắt ở "…".</t>
+        </is>
+      </c>
+      <c r="F212" s="32" t="inlineStr">
+        <is>
+          <t>Xuống dòng mềm giữ trong câu để "các
+yếu tố" vẫn bị bắt. Cắt ở "…" chia đôi câu kê sao thành hai nửa dưới ngưỡng laCauKeSao — bản cũ cũng không cắt ở đó.</t>
+        </is>
+      </c>
+      <c r="G212" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/sua-chua.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="53" t="inlineStr">
+        <is>
+          <t>CEL-184</t>
+        </is>
+      </c>
+      <c r="B213" s="54" t="inlineStr">
+        <is>
+          <t>Lớp sửa câu (tách / ráp)</t>
+        </is>
+      </c>
+      <c r="C213" s="54" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D213" s="8" t="inlineStr">
+        <is>
+          <t>Câu model viết lại phải là một câu trơn</t>
+        </is>
+      </c>
+      <c r="E213" s="8" t="inlineStr">
+        <is>
+          <t>lamSachCauMoi: xuống dòng (kèm dấu đầu dòng chèn sau nó) thành dấu cách; bỏ tiền tố C1./#/-/1. ở đầu; nếu câu gốc lẻ ** hoặc __ thì câu mới phải lẻ đúng dấu ấy, cùng phía. Dòng tiêu đề không bao giờ được gửi đi viết lại.</t>
+        </is>
+      </c>
+      <c r="F213" s="32" t="inlineStr">
+        <is>
+          <t>Câu mang cấu trúc riêng là chèn cấu trúc vào bài — cùng lỗi theo chiều ngược lại. Mất nửa cặp ** thì chữ đậm loang hết phần sau. Tiêu đề viết lại thành câu ≥15 ký tự là tiêu đề thành đoạn văn.</t>
+        </is>
+      </c>
+      <c r="G213" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/sua-chua.ts</t>
         </is>
       </c>
     </row>
@@ -23345,7 +23540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27462,6 +27657,39 @@
       <c r="F128" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B129" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/sua-xuong-dong-tieng-long)</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>CEL-184</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="inlineStr">
+        <is>
+          <t>Thay tachCau + join(' ') trong lib/rag/sua-chua.ts bằng cặp lossless tachManh/rapManh; hai hàm sửa chỉ thay mảnh NOI_DUNG, bỏ qua tiêu đề; làm sạch câu model trả về. Thêm scripts/test-sua-chua-tach.ts (31 ca, vào CI). KHÔNG đổi khoá đệm.</t>
+        </is>
+      </c>
+      <c r="E129" s="8" t="inlineStr">
+        <is>
+          <t>Lỗi chạy trên prod: mọi bài có câu phải sửa mất hết xuống dòng, tiêu đề và danh sách — phá "kết luận đứng một mình" và khuôn BÁO CÁO, và là tiền đề hỏng của tầng dấu ấn (mục 23). Không bump phiên bản đệm vì đếm thật trên noi_dung_ai cho 0 bản ghi có 
+ ở mọi bề mặt có đệm đi qua lớp sửa: bump sẽ trả tiền sinh lại để chữa một lỗi không tồn tại trong đệm. Chủ dự án chốt nguyên tắc "version hoá đúng tầng thay đổi"; tầng hậu xử lý không có đệm riêng nên nguyên tắc đó ở đây rút về "không có đệm hỏng thì không bump".</t>
+        </is>
+      </c>
+      <c r="F129" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CEL-185: dau an — cong ketLuan, checker dung chung tieng long, bo cau da duyet
Noi tiep 0e30d78 (bo cau vong 1 do phien khac tao, khong amend).

- Khong co ketLuan thi khong co dau an, moi y dinh: chonDauAn tra
  khong-ket-luan, dungVan chi chen sau ket luan khong rong.
- kiemCauDauAn quet CUM_TIENG_LONG_CAM, tach tu chuan-ngon-ngu — cung danh
  sach khoi cam-tieng-long in vao prompt. Prompt giu nguyen tung byte,
  PHIEN_BAN_CHU khong doi.
- Thay 8 cau: ca 3 cau quyet-dinh (cau cu mau thuan ketLuan khi can-bang),
  co-khong#1/#2, thoi-diem#1, mo-ta#0/#2. Motif "dung rieng" 5/15 -> 3/15.
- test-dau-an: hoi quy "dang do" -> chan, cong ketLuan 5 y dinh.
  do-coverage-dau-an in NO_KET_LUAN_GATE.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O184"/>
+  <dimension ref="A1:O185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15761,6 +15761,83 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" s="11" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="B185" s="12" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C185" s="8" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes — tầng DAN_LUAN (một câu dẫn luận sau kết luận)</t>
+        </is>
+      </c>
+      <c r="D185" s="8" t="inlineStr">
+        <is>
+          <t>Mỗi lượt chat được chèn MỘT câu dẫn luận tất định của Celes, đứng sau ketLuan và trước ý chính đầu tiên. Câu lấy từ thư viện 15 câu (3 câu mỗi ý định: quyet-dinh, co-khong, thoi-diem, giai-thich, mo-ta), chủ dự án duyệt tay từng câu. Việc chọn chỉ theo khoá chuDe:yDinh — không đọc lá số, lời người dùng hay lịch sử. Tầng KHO_HAI (câu dí dỏm) có cờ nhưng TẮT, thư viện rỗng.</t>
+        </is>
+      </c>
+      <c r="E185" s="8" t="inlineStr">
+        <is>
+          <t>1. tra-loi.ts tính laCauNoi (chip tiếp nối hoặc laCauNoiTiep) rồi gọi chonDauAn. 2. Cổng theo thứ tự: mucAnToan khác NORMAL → không; tra-cuu → không; tong-quan:mo-ta mà planner không chắc (!chacChan hoặc phanLoaiBangModel) → không; laCauNoi → không; bài model không có ketLuan → không (mọi ý định). 3. Chọn câu: stableIndex FNV-1a của "chuDe:yDinh" mod 3. 4. Chống lặp: tin trợ lý LIỀN TRƯỚC đã chứa đúng câu đó → bỏ lượt này. 5. dungVan chèn câu thành một đoạn riêng sau ketLuan (và chỉ khi có ketLuan), không chuỗi đánh dấu, nên các lớp sửa chữ phía sau thấy nó như mọi đoạn khác.</t>
+        </is>
+      </c>
+      <c r="F185" s="9" t="inlineStr">
+        <is>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="G185" s="8" t="inlineStr">
+        <is>
+          <t>Thư viện câu duyệt tay (không do model sinh)</t>
+        </is>
+      </c>
+      <c r="H185" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I185" s="8" t="inlineStr">
+        <is>
+          <t>Mọi bậc</t>
+        </is>
+      </c>
+      <c r="J185" s="8" t="inlineStr">
+        <is>
+          <t>/hoi-dap (web + app)</t>
+        </is>
+      </c>
+      <c r="K185" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/dau-an.ts; lib/rag/chuan-ngon-ngu.ts (CUM_TIENG_LONG_CAM); lib/rag/tra-loi.ts (dungVan, traLoiCoCanCu, phienBanHienTai); scripts/test-dau-an.ts; scripts/do-coverage-dau-an.ts; docs/chien-luoc/ca-nhan-hoa-celes.md mục 23</t>
+        </is>
+      </c>
+      <c r="L185" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật (KHO_HAI tắt bằng BAT_KHO_HAI)</t>
+        </is>
+      </c>
+      <c r="M185" s="8" t="inlineStr">
+        <is>
+          <t>NỢ KỸ THUẬT: (1) Planner hút câu hỏi fallback vào tong-quan:mo-ta — 5/15 lượt thật mất dấu ấn vì đây, sửa ở planner chứ không ở tầng này. (2) prompt-co-can-cu dán lịch sử có chứa dấu ấn cũ vào lời model đọc, model có thể bắt chước — chỉ eval-chat-quyet-dinh.ts đo được. (3) Câu theo chủ đề (vd "Với tiền bạc…") chờ planner đủ tin: cần thư viện khoá theo chuDe:yDinh và checker chỉ cho phép đúng chủ đề của khoá. (4) test-dau-an.ts và do-coverage-dau-an.ts chưa vào CI. (5) giai-thich#0/#1 không trúng câu nào trong bộ vàng. (6) Cổng soatNgonNgu chưa bắt "đang đỡ" đứng trần (chỉ bắt "yếu tố đang đỡ") — kiemCauDauAn đã bắt qua CUM_TIENG_LONG_CAM, nhưng siết cổng soatNgonNgu là tăng PHIEN_BAN_NGON_NGU, xoá bộ đệm: chủ dự án quyết. (7) Độ phủ lượt thật là trần trên: câu trả lời không lưu DB nên NO_KET_LUAN_GATE trên lượt thật không đo được.</t>
+        </is>
+      </c>
+      <c r="N185" s="8" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="O185" s="8" t="inlineStr">
+        <is>
+          <t>(nhánh viec/dau-an-celes)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15778,7 +15855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G213"/>
+  <dimension ref="A1:G220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -23528,6 +23605,265 @@
         </is>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" s="53" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="B214" s="54" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes (DAN_LUAN)</t>
+        </is>
+      </c>
+      <c r="C214" s="54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D214" s="8" t="inlineStr">
+        <is>
+          <t>Chính sách tầng</t>
+        </is>
+      </c>
+      <c r="E214" s="8" t="inlineStr">
+        <is>
+          <t>chonTang: mucAnToan khác NORMAL → KHONG; tra-cuu → KHONG; KHO_HAI chỉ khi BAT_KHO_HAI bật VÀ thư viện có câu; còn lại DAN_LUAN.</t>
+        </is>
+      </c>
+      <c r="F214" s="32" t="inlineStr">
+        <is>
+          <t>Tra cứu là hỏi một dữ kiện — chèn câu dẫn luận vào là nói thêm thứ không ai hỏi. SENSITIVE/CRITICAL không nhận giọng cá tính.</t>
+        </is>
+      </c>
+      <c r="G214" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/dau-an.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="53" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="B215" s="54" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes (DAN_LUAN)</t>
+        </is>
+      </c>
+      <c r="C215" s="54" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D215" s="8" t="inlineStr">
+        <is>
+          <t>Chọn biến thể</t>
+        </is>
+      </c>
+      <c r="E215" s="8" t="inlineStr">
+        <is>
+          <t>stableIndex(`${chuDe}:${yDinh}`, 3) bằng FNV-1a 32-bit (Math.imul). Đúng 3 câu mỗi yDinh; 30 khoá, UNREACHABLE = 0.</t>
+        </is>
+      </c>
+      <c r="F215" s="32" t="inlineStr">
+        <is>
+          <t>KHÔNG băm lời người dùng (gõ thêm dấu chấm là đổi câu) và KHÔNG đọc lichSu để chọn. Đổi số biến thể là đổi câu của mọi khoá — số 4 biến thể ra 0/20 câu chết chỉ là may (mục 23).</t>
+        </is>
+      </c>
+      <c r="G215" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/dau-an.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="53" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="B216" s="54" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes (DAN_LUAN)</t>
+        </is>
+      </c>
+      <c r="C216" s="54" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D216" s="8" t="inlineStr">
+        <is>
+          <t>Các cổng không-dấu-ấn</t>
+        </is>
+      </c>
+      <c r="E216" s="8" t="inlineStr">
+        <is>
+          <t>tong-quan:mo-ta khi !chacChan hoặc phanLoaiBangModel → không. laCauNoi (chip tiếp nối hoặc laCauNoiTiep) → không. coKetLuan=false (ketLuan rỗng sau locYHong/gomLoiKhuyen) → không, lyDo khong-ket-luan, mọi ý định.</t>
+        </is>
+      </c>
+      <c r="F216" s="32" t="inlineStr">
+        <is>
+          <t>tong-quan:mo-ta là ô planner đổ câu không chắc vào; gắn dấu ấn ở đó là gắn giọng tự tin lên một phân loại đoán. lapKeHoachDayDu đặt chacChan=true khi rơi về model nên phải kiểm thêm phanLoaiBangModel. Không xử lý riêng câu "hi". Không có kết luận thì câu dẫn thành câu mở bài, chiếm chỗ câu nghiêng hướng — nên chặn cả ở chonDauAn lẫn dungVan.</t>
+        </is>
+      </c>
+      <c r="G216" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/dau-an.ts; lib/rag/tra-loi.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="53" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="B217" s="54" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes (DAN_LUAN)</t>
+        </is>
+      </c>
+      <c r="C217" s="54" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D217" s="8" t="inlineStr">
+        <is>
+          <t>Chống lặp liền trước</t>
+        </is>
+      </c>
+      <c r="E217" s="8" t="inlineStr">
+        <is>
+          <t>daDungOLuotLienTruoc: tìm tin vai tro-ly cuối cùng trong lichSu; nếu noiDung chứa đúng câu sẽ chọn → bỏ dấu ấn lượt này (lyDo lap-lien-truoc).</t>
+        </is>
+      </c>
+      <c r="F217" s="32" t="inlineStr">
+        <is>
+          <t>Chỉ quét MỘT tin trợ lý liền trước, không quét cả lịch sử. Lịch sử dùng cho cổng này, không dùng cho việc chọn.</t>
+        </is>
+      </c>
+      <c r="G217" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/dau-an.ts; scripts/test-dau-an.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="53" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="B218" s="54" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes (DAN_LUAN)</t>
+        </is>
+      </c>
+      <c r="C218" s="54" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D218" s="8" t="inlineStr">
+        <is>
+          <t>Vị trí trong bài</t>
+        </is>
+      </c>
+      <c r="E218" s="8" t="inlineStr">
+        <is>
+          <t>dungVan đẩy dauAn vào mảng phan ngay sau ketLuan, trước yChinh/tomTat — chỉ khi ketLuan không rỗng. Không chuỗi đánh dấu.</t>
+        </is>
+      </c>
+      <c r="F218" s="32" t="inlineStr">
+        <is>
+          <t>Câu đi qua suaCauTiengLong, doiTenCung, soatNgonNgu như mọi đoạn. Đã kiểm 5 lượt model thật: đoạn dấu ấn ra nguyên văn.</t>
+        </is>
+      </c>
+      <c r="G218" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/tra-loi.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="53" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="B219" s="54" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes (DAN_LUAN)</t>
+        </is>
+      </c>
+      <c r="C219" s="54" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D219" s="8" t="inlineStr">
+        <is>
+          <t>Luật viết câu (kiemCauDauAn)</t>
+        </is>
+      </c>
+      <c r="E219" s="8" t="inlineStr">
+        <is>
+          <t>Năm lớp lint: CUM_FILLER_CAM; CUM_TIENG_LONG_CAM (import từ chuan-ngon-ngu — CÙNG danh sách khối cam-tieng-long in vào prompt, không bản sao); CHU_DE_CAM (không nhắc chủ đề); HUA_BO_CUC (không hứa bố cục); DO_CHAC (không rào / khẳng định độ chắc).</t>
+        </is>
+      </c>
+      <c r="F219" s="32" t="inlineStr">
+        <is>
+          <t>Không nới checker để cứu câu — sửa câu cho qua. Câu nhắc chủ đề bị cấm vì planner gán sai chuDe thì câu "tiền bạc" hiện trong câu hỏi về con cái (gặp thật: "tôi sẽ đẻ vào năm bao nhiêu" → tai-chinh:mo-ta).</t>
+        </is>
+      </c>
+      <c r="G219" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/dau-an.ts; scripts/do-coverage-dau-an.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="53" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="B220" s="54" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes (DAN_LUAN)</t>
+        </is>
+      </c>
+      <c r="C220" s="54" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D220" s="8" t="inlineStr">
+        <is>
+          <t>Bộ đo</t>
+        </is>
+      </c>
+      <c r="E220" s="8" t="inlineStr">
+        <is>
+          <t>do-coverage-dau-an.ts: (0) thư viện qua checker; (1) keyspace UNREACHABLE — chặn; (1b) cổng SENSITIVE/CRITICAL/tra-cuu/tong-quan:mo-ta không chắc/laCauNoi/không ketLuan = 0 — chặn, in NO_KET_LUAN_GATE; (2) bộ vàng UNHIT_ON_GOLD — cảnh báo; (3) 15 lượt thật, phân phối planner và phân phối câu tách riêng, &gt;25% — cảnh báo.</t>
+        </is>
+      </c>
+      <c r="F220" s="32" t="inlineStr">
+        <is>
+          <t>Độ phủ không phải KPI để giữ: tụt vì planner không chắc, vì câu nối hoặc vì cổng ketLuan là tụt đúng. Tập 2–3 giả định có ketLuan nên là trần trên.</t>
+        </is>
+      </c>
+      <c r="G220" s="8" t="inlineStr">
+        <is>
+          <t>scripts/do-coverage-dau-an.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23540,7 +23876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27688,6 +28024,38 @@
         </is>
       </c>
       <c r="F129" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B130" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/dau-an-celes)</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t>CEL-185</t>
+        </is>
+      </c>
+      <c r="D130" s="8" t="inlineStr">
+        <is>
+          <t>Thêm lib/rag/dau-an.ts: tầng DAN_LUAN chèn một câu dẫn luận tất định sau ketLuan. 15 câu duyệt tay; chọn theo FNV-1a của chuDe:yDinh; cổng an toàn / tra-cuu / planner không chắc / câu nối / lặp liền trước. Sửa bảng số biến thể ở mục 23 (4 → 0/20, 6 → 6/30) theo số script đo. PHIEN_BAN_DAU_AN vào phienBanHienTai. Commit nối tiếp: cổng ketLuan cho mọi ý định; kiemCauDauAn quét CUM_TIENG_LONG_CAM tách từ chuan-ngon-ngu (prompt giữ nguyên từng byte, PHIEN_BAN_CHU không đổi); thay 8 câu (cả 3 câu quyet-dinh, co-khong#1, co-khong#2, thoi-diem#1, mo-ta#0, mo-ta#2); test hồi quy tiếng lóng + cổng ketLuan.</t>
+        </is>
+      </c>
+      <c r="E130" s="8" t="inlineStr">
+        <is>
+          <t>Character System v4 (mục 23): Celes cần một dấu hiệu nhận ra được mà không đổi kết luận và không tốn token. Câu đặt sau kết luận để làm cầu sang căn cứ, không phải câu triết lý. Vòng đầu 15 câu bị chủ dự án trả lại vì nhiều câu nói về phương pháp mà không đẩy mạch luận; bộ hiện tại qua checker và qua 5 lượt ghép model thật. Không cho câu nhắc chủ đề cho tới khi planner sửa xong — planner gán sai chuDe trên lượt thật. Bảng số ở tài liệu sửa theo code vì "đừng để tài liệu thắng code". Commit 0e30d78 (bộ câu vòng 1) do một phiên khác tạo, không amend — commit nối tiếp mang bộ câu đã duyệt. Câu co-khong#1 cũ lọt tiếng lóng "đang đỡ" vì checker không quét danh sách tiếng lóng → dùng chung một danh sách với prompt để hai nơi không lệch nhau. Ba câu quyet-dinh viết lại vì khi dữ kiện cân bằng (can-bang) câu cũ nói như đã có một hướng thắng — chọn sửa câu thay vì nối huongNghieng vào chonDauAn: dấu ấn chỉ dẫn từ kết luận sang căn cứ, không tự diễn giải kết quả. co-khong#2 cũ ("cùng câu hỏi có thể ra kết luận khác") đặt sau Có/Chưa nghe như tự rút lại kết luận → bỏ. Motif "đứng riêng/một mình" lặp 5/15 → còn 3/15. Câu quyet-dinh#1 và co-khong#0 kích cảnh báo cum-van-may ("không chỉ", ở co-khong#0 là bắt nhầm qua ranh giới cụm) — chỉ ghi nhận, không chặn. Độ đa dạng của thư viện (15 câu cùng một ý "đừng đọc riêng một mảnh") để thư viện v2.</t>
+        </is>
+      </c>
+      <c r="F130" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
CEL-181: go quang trang quanh linh vat o nen toi — sua tu tep anh
lam-sach-anh-celes.py them hai buoc truoc khu ria:
- 1b tach lai matte dai 12px sat mep theo nen kem #F6F1E8
  (mau that lay tu pixel loi gan nhat, san xa than lay tong bong)
- 1c va lo alpha sau trong than (mat/bung kem bi mat na an mat)
Sinh lai 7 tep public/celes/*.webp tu PNG goc: van 512x512, cao 86%,
32-41KB. Pixel sang sat mep giam 76-95%. Bong van chi o CSS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -22898,7 +22898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26983,6 +26983,38 @@
       <c r="F127" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B128" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/linh-vat-web)</t>
+        </is>
+      </c>
+      <c r="C128" s="8" t="inlineStr">
+        <is>
+          <t>CEL-181</t>
+        </is>
+      </c>
+      <c r="D128" s="8" t="inlineStr">
+        <is>
+          <t>Sửa quầng sáng quanh linh vật ở chế độ tối: scripts/lam-sach-anh-celes.py thêm hai bước trước bước khử rìa — (1b) tách lại matte ở dải 12px sát mép so với nền tham chiếu kem #F6F1E8 (màu thật lấy từ pixel lõi gần nhất, vùng sàn xa thân lấy tông bóng #161028), (1c) vá lỗ alpha nằm sâu hơn 12px trong thân (ghép bản gốc lên nền kem, alpha = 1). Sinh lại 7 tệp public/celes/*.webp từ PNG gốc; vẫn 512×512, nhân vật cao 86% khung, 32–41KB (trước 38–43KB). Bóng đổ vẫn chỉ ở CSS --shadow-celes.</t>
+        </is>
+      </c>
+      <c r="E128" s="8" t="inlineStr">
+        <is>
+          <t>CEL-181 đã bỏ bóng nướng và khử rìa kem nhưng nền tối vẫn lộ ba lỗi của chính tệp ảnh, đo 02/10/2026 trên nền #240029: (a) viền chấm trắng 2–9px chạy quanh tai, lưng, tay — 2.700–6.300 pixel sáng (min RGB ≥150, bão hoà ≤30) nằm trong 3px sát mép mỗi tệp, sau sửa còn 130–1.470 (phần còn lại là lông kem thật ở má chạm mép); (b) vệt sàn mảnh dưới chân; (c) mặt và bụng kem loang xám vì mặt nạ tách theo nền kem ăn luôn lông kem — ~7.000 pixel bên trong thân có alpha &lt; 0,9 ở mỗi state. Trên nền kem cả ba hoà vào nền nên bản sáng trông đúng, vì vậy CSS và bóng không che được — phải sửa ở tệp. Kiểm lại: ghép lên nền kem lệch trung bình 0,011–0,039/255 so với PNG gốc (pixel lệch &gt;4 là matte trắng thuần sáng hơn nền kem, đúng thứ cần gỡ); nền trắng lệch 0,3–0,45/255, nằm ở vùng mặt/bụng vừa vá lỗ. Bước 1c giữ nguyên dải 12px sát mép: làm đặc dải đó là vẽ lại đúng cái viền vừa gỡ.</t>
+        </is>
+      </c>
+      <c r="F128" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CEL-181: linh vat nghiem theo luot moi nhat + hai trang thai rong
- lib/linh-vat.ts: linhVatNghiem(tinNhan) chay doAnToan (cung ham may chu)
  tren cau nguoi dung MOI NHAT; != NORMAL thi /hoi-dap dau trang + man cho
  doi sang serious, tu tat tho. Khong dinh ca hoi thoai.
- /hoi-dap chua chon la so va /ho-so rong: Celes 80px default.
- scripts/test-linh-vat-an-toan.ts (7 ca) vao CI.
- Tai lieu muc 12, AGENTS.md, PRODUCT-BACKLOG (3 sheet).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15538,17 +15538,17 @@
       </c>
       <c r="C182" s="8" t="inlineStr">
         <is>
-          <t>Linh vật Celes trên web (Hỏi Celes)</t>
+          <t>Linh vật Celes trên web (Hỏi Celes, Danh sách lá số)</t>
         </is>
       </c>
       <c r="D182" s="8" t="inlineStr">
         <is>
-          <t>Hình Celes Moon Hare v2 hiện ở ba điểm của trang Hỏi Celes: đầu trang 56px, trạng thái rỗng 80px, màn chờ 80px. Bảy trạng thái hình bật ở Phase 3 (default, listening, thinking, found-something, side-eye, serious, celebrate); HAS_RECEIPTS và NOT_BUYING_IT còn khoá.</t>
+          <t>Hình Celes Moon Hare v2 ở năm chỗ: Hỏi Celes — đầu trang 56px, rỗng đã chọn lá số 80px, rỗng CHƯA chọn lá số 80px, màn chờ trả lời 80px (thinking); Danh sách lá số — rỗng 80px. Câu người dùng MỚI NHẤT chạm lớp an toàn (SENSITIVE/CRITICAL) thì mọi linh vật ở Hỏi Celes đổi sang serious và đứng yên. Bảy trạng thái hình bật ở Phase 3 (default, listening, thinking, found-something, side-eye, serious, celebrate); HAS_RECEIPTS và NOT_BUYING_IT còn khoá.</t>
         </is>
       </c>
       <c r="E182" s="8" t="inlineStr">
         <is>
-          <t>1. components/CelesMascot.tsx nhận prop trangThai → chọn /celes/&lt;trangThai&gt;.webp. 2. Chuyển động idle breathing bằng CSS class .celes-tho (translateY 3px, chu kỳ 3s). 3. trangThai="serious" hoặc tatChuyenDong → bỏ class, đứng yên. 4. Phase 3 chưa có characterHook nên mọi nơi gọi truyền tay giá trị cố định: đầu trang và trạng thái rỗng dùng default, màn chờ dùng thinking (KHÔNG phải default — ở đó người dùng đang đợi).</t>
+          <t>1. components/CelesMascot.tsx nhận prop trangThai → chọn /celes/&lt;trangThai&gt;.webp. 2. Chuyển động idle breathing bằng CSS class .celes-tho (translateY 3px, chu kỳ 3s). 3. trangThai="serious" hoặc tatChuyenDong → bỏ class, đứng yên. 4. Phase 3 chưa có characterHook nên mọi nơi gọi truyền tay giá trị cố định: đầu trang và trạng thái rỗng dùng default, màn chờ dùng thinking (KHÔNG phải default — ở đó người dùng đang đợi). 5. Hỏi Celes: nghiem = linhVatNghiem(tinNhan) (lib/linh-vat.ts) — chạy doAnToan trên câu người dùng MỚI NHẤT; true thì đầu trang và màn chờ truyền trangThai="serious". Suy ra từ danh sách tin nên câu vừa gửi đã tính ngay lúc chờ, tải lại trang tự tính lại, xoá hội thoại hay gửi câu bình thường là tự về.</t>
         </is>
       </c>
       <c r="F182" s="9" t="inlineStr">
@@ -15573,12 +15573,12 @@
       </c>
       <c r="J182" s="8" t="inlineStr">
         <is>
-          <t>/hoi-dap (web)</t>
+          <t>/hoi-dap, /ho-so (web)</t>
         </is>
       </c>
       <c r="K182" s="8" t="inlineStr">
         <is>
-          <t>components/CelesMascot.tsx; app/globals.css (.celes-anh, --shadow-celes, .celes-tho); public/celes/*.webp (7 state, 512×512 đã chuẩn hoá); scripts/lam-sach-anh-celes.py</t>
+          <t>components/CelesMascot.tsx; lib/linh-vat.ts; app/hoi-dap/page.tsx; app/ho-so/page.tsx; app/globals.css (.celes-anh, --shadow-celes, .celes-tho); public/celes/*.webp (7 state, 512×512 đã chuẩn hoá); scripts/lam-sach-anh-celes.py; scripts/test-linh-vat-an-toan.ts</t>
         </is>
       </c>
       <c r="L182" s="8" t="inlineStr">
@@ -15588,7 +15588,7 @@
       </c>
       <c r="M182" s="8" t="inlineStr">
         <is>
-          <t>CHƯA NỐI SafetyOverlay — luật "SafetyOverlay thắng nhân vật" mới ở mức tài liệu. Phase 3 nối characterHook → visual state, hiện truyền tay giá trị cố định. Tab Hôm nay chưa đặt linh vật, chờ chủ dự án xem bản live.</t>
+          <t>Phase 3 nối characterHook → visual state, hiện truyền tay giá trị cố định. Tab Hôm nay KHÔNG đặt linh vật — chủ dự án xem lại 02/10/2026 và giữ nguyên, xem lại khi web dùng thật đủ lâu. App (apps/celes-app) chưa có luật nghiêm theo lượt.</t>
         </is>
       </c>
       <c r="N182" s="8" t="inlineStr">
@@ -15598,7 +15598,7 @@
       </c>
       <c r="O182" s="8" t="inlineStr">
         <is>
-          <t>(nhánh viec/celes-mascot-web)</t>
+          <t>(nhánh viec/linh-vat-web)</t>
         </is>
       </c>
     </row>
@@ -15619,7 +15619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:G201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -22729,7 +22729,7 @@
       </c>
       <c r="F196" s="32" t="inlineStr">
         <is>
-          <t>HAI LÝ DO TẮT LÀ HAI THỨ KHÁC NHAU: prefers-reduced-motion là sở thích thiết bị (xử lý ở CSS), còn SafetyOverlay != NORMAL là luật sản phẩm (xử lý ở mã). "Con thỏ không được nhún nhảy khi người ta đang nói chuyện mất mát." serious tự tắt để nơi gọi không phải nhớ truyền cờ. SafetyOverlay CHƯA TỒN TẠI trong mã — chờ Phase 3.</t>
+          <t>HAI LÝ DO TẮT LÀ HAI THỨ KHÁC NHAU: prefers-reduced-motion là sở thích thiết bị (xử lý ở CSS), còn SafetyOverlay != NORMAL là luật sản phẩm (xử lý ở mã). "Con thỏ không được nhún nhảy khi người ta đang nói chuyện mất mát." serious tự tắt để nơi gọi không phải nhớ truyền cờ. Đã nối ở Hỏi Celes 02/10/2026 qua bước 8 — nơi gọi đổi sang serious, không truyền tatChuyenDong riêng (mục 9: SERIOUS và tắt thở đi cùng nhau).</t>
         </is>
       </c>
       <c r="G196" s="8" t="inlineStr">
@@ -22798,7 +22798,7 @@
       </c>
       <c r="E198" s="8" t="inlineStr">
         <is>
-          <t>CÓ: Hỏi Celes (56px), trạng thái rỗng (80px), màn chờ (80px, thinking). KHÔNG: lá số, mệnh bàn, mọi trang luận giải, Hành trình, Mối quan hệ, Hôm nay.</t>
+          <t>CÓ: Hỏi Celes đầu trang (56px), Hỏi Celes rỗng đã chọn lá số và CHƯA chọn lá số (80px, default), màn chờ trả lời (80px, thinking), Danh sách lá số rỗng (80px, default). KHÔNG: lá số, mệnh bàn, mọi trang luận giải, Hành trình, Mối quan hệ, Hôm nay.</t>
         </is>
       </c>
       <c r="F198" s="32" t="inlineStr">
@@ -22872,17 +22872,54 @@
       </c>
       <c r="E200" s="8" t="inlineStr">
         <is>
-          <t>scripts/lam-sach-anh-celes.py đọc PNG gốc ở docs/thiet-ke/celes-nhan-vat/v2/states/, làm ba việc rồi ghi WebP q92 vào public/celes/: (a) BỎ BÓNG ĐỔ nướng sẵn — quét từ đáy lên, tìm hàng mà bề rộng silhouette đang thu hẹp thì đột ngột loe ra KÈM độ sáng tăng (đo trên thinking.png: y=421 rộng 127 sáng 71.9 → y=426 rộng 179 sáng 116.5), cắt từ hàng đó xuống; (b) KHỬ NHIỄM MÀU NỀN ở rìa bằng un-premultiply với nền đo được rgb(249,246,243), chỉ trong dải alpha 0.15–0.95; (c) CHUẨN HOÁ: cắt theo alpha bbox rồi co về khung 512x512 với chiều cao nhân vật = 86% khung, neo theo chiều cao (neo theo cạnh dài nhất sẽ làm tư thế dang ngang như celebrate bị thu nhỏ). Bóng đổ chuyển sang CSS: .celes-anh dùng --shadow-celes, mỗi theme một giá trị.</t>
+          <t>scripts/lam-sach-anh-celes.py đọc PNG gốc ở docs/thiet-ke/celes-nhan-vat/v2/states/, làm ba việc rồi ghi WebP q92 vào public/celes/: (a) BỎ BÓNG ĐỔ nướng sẵn — quét từ đáy lên, tìm hàng mà bề rộng silhouette đang thu hẹp thì đột ngột loe ra KÈM độ sáng tăng (đo trên thinking.png: y=421 rộng 127 sáng 71.9 → y=426 rộng 179 sáng 116.5), cắt từ hàng đó xuống; (a2) TÁCH LẠI MATTE ở dải 12px sát mép theo nền kem #F6F1E8 — mỗi pixel sáng ở rìa coi là trộn giữa màu thật F (lấy từ pixel lõi gần nhất; vùng sàn xa thân lấy tông bóng #161028) và nền, giải ra alpha rồi C' = B − (B−C)/a; (a3) VÁ LỖ alpha nằm sâu hơn 12px trong thân (ghép bản gốc lên nền kem, alpha = 1); (b) KHỬ NHIỄM MÀU NỀN ở rìa bằng un-premultiply với nền đo được rgb(249,246,243), chỉ trong dải alpha 0.15–0.95; (c) CHUẨN HOÁ: cắt theo alpha bbox rồi co về khung 512x512 với chiều cao nhân vật = 86% khung, neo theo chiều cao (neo theo cạnh dài nhất sẽ làm tư thế dang ngang như celebrate bị thu nhỏ). Bóng đổ chuyển sang CSS: .celes-anh dùng --shadow-celes, mỗi theme một giá trị.</t>
         </is>
       </c>
       <c r="F200" s="32" t="inlineStr">
         <is>
-          <t>KHÔNG TÁCH BÓNG BẰNG NGƯỠNG MÀU. Đã thử và hỏng: mặt nạ kem và bóng CHỒNG phân bố — kem sat 0.166–0.177, bóng sat 0.092–0.099, mà đuôi dưới của kem (p10 = 0.045) còn thấp hơn trung bình của bóng. Mọi ngưỡng bão hoà đều ăn mất mặt con thỏ ở thinking / listening / found-something, là ba tư thế có mặt chạm rìa silhouette. Phải tách bằng HÌNH HỌC theo hàng. BÓNG KHÔNG ĐƯỢC NƯỚNG VÀO ẢNH: nền tối thì nó hiện thành vệt trắng dưới chân. Bóng thuộc về CSS vì nó phụ thuộc theme, ảnh thì không. ẢNH GỐC MỖI TỆP MỘT KHUNG: default 768px chiếm 83%, thinking 512px chiếm 60% — copy thẳng là cùng một cao mà ra hai cỡ lệch 1,4 lần. KHÔNG SỬA TỪ WEBP, luôn đi từ PNG gốc (WebP của bộ này là lossy).</t>
+          <t>KHÔNG TÁCH BÓNG BẰNG NGƯỠNG MÀU. Đã thử và hỏng: mặt nạ kem và bóng CHỒNG phân bố — kem sat 0.166–0.177, bóng sat 0.092–0.099, mà đuôi dưới của kem (p10 = 0.045) còn thấp hơn trung bình của bóng. Mọi ngưỡng bão hoà đều ăn mất mặt con thỏ ở thinking / listening / found-something, là ba tư thế có mặt chạm rìa silhouette. Phải tách bằng HÌNH HỌC theo hàng. BÓNG KHÔNG ĐƯỢC NƯỚNG VÀO ẢNH: nền tối thì nó hiện thành vệt trắng dưới chân. Bóng thuộc về CSS vì nó phụ thuộc theme, ảnh thì không. ẢNH GỐC MỖI TỆP MỘT KHUNG: default 768px chiếm 83%, thinking 512px chiếm 60% — copy thẳng là cùng một cao mà ra hai cỡ lệch 1,4 lần. KHÔNG SỬA TỪ WEBP, luôn đi từ PNG gốc (WebP của bộ này là lossy). QUẦNG TRẮNG Ở NỀN TỐI LÀ LỖI CỦA TỆP, không sửa được bằng CSS và KHÔNG ĐƯỢC che bằng bóng: mặt nạ tách để lại dải matte trắng 2–9px và ăn luôn lông kem ở mặt/bụng (~7.000 pixel alpha &lt; 0,9 mỗi state). Bước vá lỗ PHẢI chừa dải 12px sát mép — làm đặc dải đó là vẽ lại đúng cái viền vừa gỡ. Bước khử nhiễm (b) bỏ qua vùng (a2) đã xử lý, không thì trừ nền hai lần.</t>
         </is>
       </c>
       <c r="G200" s="8" t="inlineStr">
         <is>
           <t>scripts/lam-sach-anh-celes.py; public/celes/*.webp; app/globals.css</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="53" t="inlineStr">
+        <is>
+          <t>CEL-181</t>
+        </is>
+      </c>
+      <c r="B201" s="54" t="inlineStr">
+        <is>
+          <t>Linh vật Celes web</t>
+        </is>
+      </c>
+      <c r="C201" s="54" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D201" s="8" t="inlineStr">
+        <is>
+          <t>Đứng nghiêm theo lượt mới nhất</t>
+        </is>
+      </c>
+      <c r="E201" s="8" t="inlineStr">
+        <is>
+          <t>lib/linh-vat.ts: linhVatNghiem(tinNhan) tìm câu người dùng MỚI NHẤT, trả doAnToan(câu).muc !== "NORMAL". app/hoi-dap/page.tsx tính bằng useMemo trên tinNhan; true thì đầu trang 56px và màn chờ 80px truyền trangThai="serious" (CelesMascot tự tắt thở). Câu vừa gửi được đẩy vào tinNhan ngay lúc gửi nên mức có từ lúc chờ; tải lại trang tính lại trên hội thoại nạp từ DB.</t>
+        </is>
+      </c>
+      <c r="F201" s="32" t="inlineStr">
+        <is>
+          <t>BẤT BIẾN: safety(lượt mới nhất) ≠ safety(mức nặng nhất cả hội thoại). Chủ dự án bác phương án "dính cả hội thoại" — người dùng đã chuyển chủ đề mà Celes vẫn nghiêm mãi là sai, và đó là một định nghĩa an toàn thứ hai chỉ sống ở UI. Dùng CHÍNH hàm doAnToan của máy chủ, không sao chép luật (an-toan.ts chỉ kéo thuc-the.ts + lib/tuvi/constants, an toàn cho trình duyệt). Máy chủ KHÔNG trả mucAnToan ở nhánh thường — đừng đọc nó từ phản hồi. Bài kiểm scripts/test-linh-vat-an-toan.ts (CI).</t>
+        </is>
+      </c>
+      <c r="G201" s="8" t="inlineStr">
+        <is>
+          <t>lib/linh-vat.ts; app/hoi-dap/page.tsx; scripts/test-linh-vat-an-toan.ts</t>
         </is>
       </c>
     </row>
@@ -22898,7 +22935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27013,6 +27050,38 @@
         </is>
       </c>
       <c r="F128" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B129" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/linh-vat-web)</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>CEL-181</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="inlineStr">
+        <is>
+          <t>Đặt linh vật theo mục 12 + luật an toàn mục 9 trên web: thêm Celes 80px DEFAULT ở hai trạng thái rỗng (Hỏi Celes chưa chọn lá số, Danh sách lá số chưa có lá số); câu người dùng mới nhất có doAnToan != NORMAL thì mọi linh vật ở Hỏi Celes đổi sang SERIOUS và tắt thở (lib/linh-vat.ts). Thêm scripts/test-linh-vat-an-toan.ts vào CI. Tab Hôm nay giữ KHÔNG.</t>
+        </is>
+      </c>
+      <c r="E129" s="8" t="inlineStr">
+        <is>
+          <t>Mục 9 đòi SafetyOverlay != NORMAL thì SERIOUS + tắt thở, nhưng web chưa nối — ghi chú cũ nói "SafetyOverlay chưa tồn tại", trong khi doAnToan đã có từ Phase 1. Máy chủ lại không trả mức SENSITIVE về trình duyệt, nên đọc từ phản hồi là không bao giờ bật đúng nhóm "đang nói chuyện mất mát". Chấm ở trình duyệt bằng chính hàm máy chủ: biết mức ngay lúc gửi, không sửa API, không sao chép luật. Chủ dự án chốt theo LƯỢT MỚI NHẤT, bác "dính cả hội thoại" vì Celes sẽ nghiêm mãi khi người dùng đã đổi chủ đề, và vì nó lệch khái niệm "lượt hiện tại" của máy chủ. Hai trạng thái rỗng thêm linh vật vì cùng khung phải cùng cấu trúc thị giác và rỗng cấp trang cần dẫn vào hành động đầu tiên. Bundle tải lần đầu (gzip): /hoi-dap +3,8KB (an-toan + thuc-the), /ho-so +5,9KB (next/image lần đầu có ở trang này).</t>
+        </is>
+      </c>
+      <c r="F129" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
CEL-181: chu canh linh vat de Celes tu noi (vi + en)
Danh sach la so rong va Hoi Celes chua chon la so: bo ngoi thu ba "Celes"
canh hinh Celes. Nhat ky them dong.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -22935,7 +22935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27082,6 +27082,38 @@
         </is>
       </c>
       <c r="F129" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B130" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/linh-vat-web)</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t>CEL-181</t>
+        </is>
+      </c>
+      <c r="D130" s="8" t="inlineStr">
+        <is>
+          <t>Hai câu cạnh linh vật đổi sang Celes tự nói: Danh sách lá số rỗng "…Thêm lá số đầu tiên, rồi mình cùng đọc."; Hỏi Celes chưa chọn lá số "Mình đang nói về lá số nào nhỉ?" (vi + en).</t>
+        </is>
+      </c>
+      <c r="E130" s="8" t="inlineStr">
+        <is>
+          <t>Hình Celes đứng ngay cạnh mà chữ lại gọi "Celes" ở ngôi thứ ba nghe như có người thứ ba đang thuật lại — lệch với việc Celes là người trò chuyện cùng. Chủ dự án duyệt đổi 02/10/2026.</t>
+        </is>
+      </c>
+      <c r="F130" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
CEL-180: chan "chan song" va tien luong song chet bang ma
- Nhom "mat y nghia song" (chan song, khong thiet song, song lam gi nua,
  song chi nua...): mot minh la SENSITIVE; cung "co nen tiep tuc / song
  tiep / dang song tiep" trong mot tin nhan la CRITICAL. "Co nen tiep tuc
  khong" mot minh khong phai tin hieu. Nghia bong "chan song o Ha Noi /
  chung voi me chong" giu NORMAL, tru khi sau do co doi/coi/the gian.
- Cau hoi tien luong song chet cua nguoi benh khong con duoc luan bang la
  so: doAnToan tra tienLuong, route tra LOI_NHAN_TIEN_LUONG + 2 chip truoc
  datChoCauHoi (khong tru luot, khong goi model), khong CRITICAL.
- test-an-toan 23 -> 42 ca + bo kiem tien luong (8 bat, 15 khong bat).
- PRODUCT-BACKLOG (CEL-180, Logic buoc 6-7, Nhat ky) + HUONG-DAN.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15466,12 +15466,12 @@
       </c>
       <c r="D181" s="8" t="inlineStr">
         <is>
-          <t>Dò tất định (KHÔNG gọi model) trên câu hỏi chat, trả ba mức. CRITICAL: dừng hẳn luồng luận Tử Vi, trả lời nhắn hằng trong mã kèm số 115 (và 111 kèm điều kiện dưới 16 tuổi), một nút gọi 115, không chip gợi ý. SENSITIVE: vẫn luận bình thường, bảo đảm cuối bài có lời miễn trừ tâm lý. NORMAL: không đổi gì.</t>
+          <t>Dò tất định (KHÔNG gọi model) trên câu hỏi chat, trả ba mức. CRITICAL: dừng hẳn luồng luận Tử Vi, trả lời nhắn hằng trong mã kèm số 115 (và 111 kèm điều kiện dưới 16 tuổi), một nút gọi 115, không chip gợi ý. SENSITIVE: vẫn luận bình thường, bảo đảm cuối bài có lời miễn trừ tâm lý. NORMAL: không đổi gì. TỪ 02/10/2026 thêm hai việc: (1) nhóm "mất ý nghĩa sống" — "tôi chán sống quá", "không thiết sống", "sống làm gì nữa", "sống chi nữa"… một mình là SENSITIVE; đi cùng "có nên tiếp tục / sống tiếp / đáng sống tiếp" trong cùng tin nhắn là CRITICAL. (2) Chặn tiên lượng sống chết: "bố tôi ung thư năm nay có qua khỏi không", "ông tôi còn sống được bao lâu", "bố tôi năm nay có qua được không" KHÔNG được luận bằng lá số — route trả LOI_NHAN_TIEN_LUONG (hằng, ghi nhận nỗi lo, chỉ tới bác sĩ) + 2 chip về phần người hỏi; không CRITICAL, không trừ lượt, không gọi model.</t>
         </is>
       </c>
       <c r="E181" s="8" t="inlineStr">
         <is>
-          <t>app/api/hoi-dap/route.ts gọi doAnToan() TRƯỚC datChoCauHoi → CRITICAL thoát sớm (không trừ hạn mức, không gọi nhà cung cấp) → ngược lại chạy traLoiCoCanCu, truyền mucAnToan xuống, nối miễn trừ sau doiTenCung</t>
+          <t>app/api/hoi-dap/route.ts gọi doAnToan() TRƯỚC datChoCauHoi → CRITICAL thoát sớm (không trừ hạn mức, không gọi nhà cung cấp) → ngược lại chạy traLoiCoCanCu, truyền mucAnToan xuống, nối miễn trừ sau doiTenCung → (02/10/2026) nếu không CRITICAL mà anToan.tienLuong = true: trả LOI_NHAN_TIEN_LUONG + GOI_Y_TIEN_LUONG, cũng TRƯỚC datChoCauHoi.</t>
         </is>
       </c>
       <c r="F181" s="9" t="inlineStr">
@@ -15511,7 +15511,7 @@
       </c>
       <c r="M181" s="8" t="inlineStr">
         <is>
-          <t>Nút gọi 115 trên app: đã xử lý tel: trong LoiDiTiep (apps/celes-app/app/(tabs)/celes.tsx) vì tuyenApp() trả null cho tel: và .filter loại mất nút — CHƯA kiểm trên máy thật, cần bấm thử một lần trên Expo Go và một lần trên web 390px. Chỉ xét tin nhắn hiện tại, chưa quét lịch sử hội thoại (để Phase 4). Lời nhắn chỉ có tiếng Việt. Chưa có đường dây nóng tự sát toàn quốc cho người lớn vì chưa tra ra nguồn chính thức. Hạn lưu trữ chat_messages là việc pháp lý/riêng tư còn treo (Luật BVDLCN) — phải làm trước Phase 4.</t>
+          <t>Nút gọi 115 trên app: đã xử lý tel: trong LoiDiTiep (apps/celes-app/app/(tabs)/celes.tsx) vì tuyenApp() trả null cho tel: và .filter loại mất nút — CHƯA kiểm trên máy thật, cần bấm thử một lần trên Expo Go và một lần trên web 390px. Chỉ xét tin nhắn hiện tại, chưa quét lịch sử hội thoại (để Phase 4). Lời nhắn chỉ có tiếng Việt. Chưa có đường dây nóng tự sát toàn quốc cho người lớn vì chưa tra ra nguồn chính thức. Hạn lưu trữ chat_messages là việc pháp lý/riêng tư còn treo (Luật BVDLCN) — phải làm trước Phase 4. | 02/10/2026: guard tiên lượng chỉ chạy ở route /api/hoi-dap — lab/eval gọi thẳng traLoiCoCanCu thì không qua. Câu tiên lượng có muc SENSITIVE nên linh vật đứng nghiêm (chủ ý). Câu hỏi thọ yểu của CHÍNH người hỏi ("tôi có thọ không", "sống đến bao nhiêu tuổi") chưa bắt bằng mã, vẫn dựa luật "không luận thọ yểu" trong prompt. "chán cuộc sống …" một mình chưa bắt (trùng "chán cuộc sống văn phòng"). Giới hạn cũ: tachCau không tách tại dấu phẩy; DAU_HIEU_GAP ("sắp", "hôm nay") dò trên cả tin nhắn nên "chán sống quá, sắp tới thế nào" lên CRITICAL; "chán sống" + "có nên tiếp tục" ở hai câu khác chủ đề vẫn lên CRITICAL (đúng spec, lệch về an toàn).</t>
         </is>
       </c>
       <c r="N181" s="8" t="inlineStr">
@@ -15521,7 +15521,7 @@
       </c>
       <c r="O181" s="8" t="inlineStr">
         <is>
-          <t>(nhánh viec/an-toan-chat)</t>
+          <t>(nhánh viec/sua-an-toan-chan-song)</t>
         </is>
       </c>
     </row>
@@ -15855,7 +15855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G221"/>
+  <dimension ref="A1:G223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -22814,7 +22814,7 @@
       </c>
       <c r="E192" s="8" t="inlineStr">
         <is>
-          <t>scripts/test-an-toan.ts — 23 ca chia 10 nhóm: dương tính thật, âm tính thật, phủ định, trích dẫn, ngôi thứ ba, quá khứ, giả định, nghĩa bóng, ý định tức thì, nhạy cảm không gấp. Thêm phép kiểm trên chính câu chữ: phải chứa 115, không được chứa "vận hạn"/"cung Mệnh"/"lá số của bạn cho thấy", câu đầu phải ghi nhận người đọc, số 111 phải đi kèm điều kiện tuổi, không dùng chữ "tâm thần". Chạy trong CI.</t>
+          <t>scripts/test-an-toan.ts — 42 ca — 23 ca gốc chia 10 nhóm: dương tính thật, âm tính thật, phủ định, trích dẫn, ngôi thứ ba, quá khứ, giả định, nghĩa bóng, ý định tức thì, nhạy cảm không gấp. Thêm phép kiểm trên chính câu chữ: phải chứa 115, không được chứa "vận hạn"/"cung Mệnh"/"lá số của bạn cho thấy", câu đầu phải ghi nhận người đọc, số 111 phải đi kèm điều kiện tuổi, không dùng chữ "tâm thần". Chạy trong CI. Từ 02/10/2026: thêm 19 ca mất ý nghĩa sống (dương, âm, nghĩa bóng "chán sống ở…", phủ định trước/sau cụm) và bộ tiên lượng: 8 câu phải bắt (không được CRITICAL), 15 câu không được bắt, lời nhắn không chứa chữ đoán, chip không tự kích lại.</t>
         </is>
       </c>
       <c r="F192" s="32" t="inlineStr">
@@ -23898,6 +23898,80 @@
       <c r="G221" s="8" t="inlineStr">
         <is>
           <t>lib/linh-vat.ts; app/hoi-dap/page.tsx; scripts/test-linh-vat-an-toan.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="30" t="inlineStr">
+        <is>
+          <t>CEL-180</t>
+        </is>
+      </c>
+      <c r="B222" s="31" t="inlineStr">
+        <is>
+          <t>Lớp an toàn chat</t>
+        </is>
+      </c>
+      <c r="C222" s="31" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D222" s="8" t="inlineStr">
+        <is>
+          <t>Mất ý nghĩa sống (nangKhiHoiTiep)</t>
+        </is>
+      </c>
+      <c r="E222" s="8" t="inlineStr">
+        <is>
+          <t>Nhóm khung-hoang-tam-ly mới, tucThi=false, nangKhiHoiTiep=true: chan song, khong thiet song, song lam gi nua, song de lam gi, song chang/khong con y nghia, song chi nua, dang song tiep khong. Khớp → SENSITIVE. Nếu cùng tin nhắn có HOI_SONG_TIEP (co nen tiep tuc, tiep tuc song, song tiep, co dang song, dang song tiep) → CRITICAL. Phủ định chỉ xét phần TRƯỚC cụm, kể cả khong/chang/cha đứng sát trước ("tôi không chán sống" → NORMAL). Nghĩa bóng: "chán sống ở/chung/với/cùng/tại/gần/xa …" được miễn khi MỌI lần xuất hiện đều có đuôi đó — trừ khi ba từ sau có đời/cõi/gian/kiếp ("chán sống ở trên đời này" vẫn SENSITIVE).</t>
+        </is>
+      </c>
+      <c r="F222" s="32" t="inlineStr">
+        <is>
+          <t>HOI_SONG_TIEP KHÔNG phải cụm nguy cơ: "có nên tiếp tục không" một mình là câu hỏi nghề nghiệp, chỉ nâng mức cho nhóm nangKhiHoiTiep — không nâng nhóm cũ ("bế tắc hoàn toàn, có nên tiếp tục" vẫn SENSITIVE). Phủ định ĐỨNG SAU cụm không được tính: "chán sống, không muốn làm gì nữa" là nặng hơn chứ không nhẹ đi. "chán đời" cố ý không có — câu than hằng ngày. Đuôi nghĩa bóng phải chặn "đời": bản đầu miễn luôn "chán sống ở trên đời này" — lỗ an toàn thật do celes-domain bắt.</t>
+        </is>
+      </c>
+      <c r="G222" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/an-toan.ts; scripts/test-an-toan.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="30" t="inlineStr">
+        <is>
+          <t>CEL-180</t>
+        </is>
+      </c>
+      <c r="B223" s="31" t="inlineStr">
+        <is>
+          <t>Lớp an toàn chat</t>
+        </is>
+      </c>
+      <c r="C223" s="31" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D223" s="8" t="inlineStr">
+        <is>
+          <t>Chặn tiên lượng sống chết (tienLuong)</t>
+        </is>
+      </c>
+      <c r="E223" s="8" t="inlineStr">
+        <is>
+          <t>laHoiTienLuong(chuỗi bỏ dấu) đúng khi một trong ba: (a) HOI_TUOI_THO ("sống được bao lâu", "khi nào qua đời"…) và không có chủ thể phi người (công ty, startup, cửa hàng, mối quan hệ…); (b) "năm nay" + người thân (bố/mẹ/cha/ông/bà/chồng/vợ) + "qua khỏi/qua được/qua nổi (năm nay) không" và KHÔNG có hạn/tam tai/Thái Tuế/thi cử/làm ăn; (c) BENH_NANG × HOI_SONG_CON (cụm neo đuôi câu hỏi: "qua khỏi không", "sống được không", "cứu được không"…). doAnToan trả tienLuong; route: CRITICAL trước, rồi tienLuong → LOI_NHAN_TIEN_LUONG + GOI_Y_TIEN_LUONG, trước datChoCauHoi.</t>
+        </is>
+      </c>
+      <c r="F223" s="32" t="inlineStr">
+        <is>
+          <t>GUARD DO MÃ, KHÔNG PHẢI LỜI MIỄN TRỪ (chủ dự án D8): thêm miễn trừ rồi vẫn luận thì vẫn là đoán sống chết bằng lá số. KHÔNG CRITICAL: người hỏi đang lo cho người khác, lời nhắn tự hại là sai địa chỉ. Cần CẢ bệnh LẪN câu hỏi sống còn: "qua khỏi hạn Thái Tuế", "Tật Ách có dấu hiệu ung thư không" là câu luận được. Bẫy bỏ dấu: 'hon me' trùng "hơn mẹ", 'song duoc'/'con song' trùng "sống được bằng nghề"/"vẫn còn sống", 'co mat khong' trùng "tiền có mất không", 'thi' trùng "thì", 'nha' trùng "nhá" — dùng cụm nhiều âm tiết. Chip KHÔNG mời hỏi gia đạo: lịch sử còn câu "bố ung thư", gia đạo là chỗ sách nói tang chế.</t>
+        </is>
+      </c>
+      <c r="G223" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/an-toan.ts; app/api/hoi-dap/route.ts; scripts/test-an-toan.ts</t>
         </is>
       </c>
     </row>
@@ -23913,7 +23987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28189,6 +28263,38 @@
         </is>
       </c>
       <c r="F133" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B134" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/sua-an-toan-chan-song)</t>
+        </is>
+      </c>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>CEL-180</t>
+        </is>
+      </c>
+      <c r="D134" s="8" t="inlineStr">
+        <is>
+          <t>Hotfix an toàn: (1) "tôi chán sống quá" từ NORMAL thành SENSITIVE; cùng "có nên tiếp tục / sống tiếp / đáng sống tiếp" thành CRITICAL; nghĩa bóng "chán sống ở Hà Nội / chung với mẹ chồng" giữ NORMAL. (2) Câu hỏi tiên lượng sống chết của người bệnh không còn được luận bằng lá số: route trả lời nhắn hằng + 2 chip, không trừ lượt, không gọi model. test-an-toan 23 → 42 ca + bộ tiên lượng.</t>
+        </is>
+      </c>
+      <c r="E134" s="8" t="inlineStr">
+        <is>
+          <t>Trên production, "tôi chán sống quá, có nên tiếp tục không" đi thẳng vào luận có/không như một câu hỏi nghề nghiệp — prompt co-khong ép model NGHIÊNG HẲN về một bên, tức là có thể trả lời "nên" hoặc "không nên" cho câu hỏi có nên sống tiếp. "Bố tôi ung thư năm nay có qua khỏi không" cũng vào đúng khuôn đó: đoán sống chết bằng lá số, trái luật "không luận thọ yểu" vốn chỉ là lời dặn model. Chủ dự án quyết D8 (02/10/2026): sửa trước mọi việc khác, kể cả CEL-185 và CEL-186. Tách khỏi CEL-186 vì lỗi an toàn không chờ được tính năng.</t>
+        </is>
+      </c>
+      <c r="F134" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
CEL-187 (5/5): muc 12 viet lai, AGENTS, backlog, du 14 ten khoa trong test
- celes-visual-character-system.md muc 12: bang 18 anh, 14 anh khoa kem ly do,
  dong vs tinh, luat hien thi, khung != than, Hom nay dao chi the rong, ngoai le
- sua "7 tep WebP" thanh 18
- AGENTS.md: "khong dat TRONG vung noi dung" + tro bai kiem CI
- test-cho-dat-celes: KHOA them sad, resting, stretching, lying-relaxed, sleeping
- PRODUCT-BACKLOG: CEL-187 (Backlog, Logic chi tiet 1-7, Nhat ky), CEL-181 tro sang

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O185"/>
+  <dimension ref="A1:O186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15588,7 +15588,7 @@
       </c>
       <c r="M182" s="8" t="inlineStr">
         <is>
-          <t>Phase 3 nối characterHook → visual state, hiện truyền tay giá trị cố định. Tab Hôm nay KHÔNG đặt linh vật — chủ dự án xem lại 02/10/2026 và giữ nguyên, xem lại khi web dùng thật đủ lâu. App (apps/celes-app) chưa có luật nghiêm theo lượt.</t>
+          <t>Phase 3 nối characterHook → visual state, hiện truyền tay giá trị cố định. Tab Hôm nay KHÔNG đặt linh vật — chủ dự án xem lại 02/10/2026 và giữ nguyên, xem lại khi web dùng thật đủ lâu. App (apps/celes-app) chưa có luật nghiêm theo lượt. — Mở rộng ra mọi màn web: CEL-187 (thay luật "không ở lá số / luận giải" bằng "không TRONG vùng nội dung").</t>
         </is>
       </c>
       <c r="N182" s="8" t="inlineStr">
@@ -15835,6 +15835,83 @@
       <c r="O185" s="8" t="inlineStr">
         <is>
           <t>(nhánh viec/dau-an-celes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="inlineStr">
+        <is>
+          <t>CEL-187</t>
+        </is>
+      </c>
+      <c r="B186" s="12" t="inlineStr">
+        <is>
+          <t>A. Giao diện</t>
+        </is>
+      </c>
+      <c r="C186" s="8" t="inlineStr">
+        <is>
+          <t>Linh vật Celes ở mọi màn web (18 ảnh v2.3, 14 khoá)</t>
+        </is>
+      </c>
+      <c r="D186" s="8" t="inlineStr">
+        <is>
+          <t>Mở rộng CEL-181 từ 5 chỗ ra mọi màn web theo bảng chủ dự án chốt 02/10/2026: 18/32 artwork v2.3 vào web, 14 khoá có chủ đích. Celes đứng ở đầu trang, thẻ rỗng / màn vào, màn chờ, cổng đăng nhập, lỗi hệ thống / thanh toán và sự kiện (proud khi bấm Giữ lại, celebrate khi thanh toán thành công lần đầu). KHÔNG trong vùng nội dung (mệnh bàn, bài luận, dòng thời gian). /hoi-dap đầu trang: serious &gt; listening &gt; default, không bao giờ thinking. Hôm nay: chỉ thẻ rỗng (đảo quyết định cũ, phạm vi hẹp).</t>
+        </is>
+      </c>
+      <c r="E186" s="8" t="inlineStr">
+        <is>
+          <t>1. CelesMascot nhận cho (loại chỗ) + trangThai | minhHoa; ANH_THEO_CHO để tsc chặn ảnh sai chỗ. 2. Màn chờ bọc .celes-tre (hiện trễ 1s, bài sâu 3s) → màn chớp dưới 1s không thấy linh vật. 3. Proud qua .celes-noi (fixed, 4s, không chiếm chỗ). 4. Thẻ rỗng / chờ / lỗi dùng components/ui/TheTrangThaiCeles. 5. scripts/test-cho-dat-celes.ts (CI) giữ danh sách trắng tệp → ảnh, danh sách CẤM vùng nội dung, mảng ↔ public/celes, không ảnh khoá.</t>
+        </is>
+      </c>
+      <c r="F186" s="9" t="inlineStr">
+        <is>
+          <t>Chờ nghiệm thu (preview)</t>
+        </is>
+      </c>
+      <c r="G186" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh tĩnh (không do model sinh)</t>
+        </is>
+      </c>
+      <c r="H186" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I186" s="8" t="inlineStr">
+        <is>
+          <t>Mọi bậc</t>
+        </is>
+      </c>
+      <c r="J186" s="8" t="inlineStr">
+        <is>
+          <t>/, /gioi-thieu, /home, /la-so, /luan-giai, /luan-giai/sau, /hanh-trinh, chi tiết hạn, /hop-tuoi, /hoi-dap, /ho-so, /tai-khoan, /dang-nhap, /support, thanh toán, 404, lỗi</t>
+        </is>
+      </c>
+      <c r="K186" s="8" t="inlineStr">
+        <is>
+          <t>components/CelesMascot.tsx; components/ui/TheTrangThaiCeles.tsx; components/luangiai/DangDocV3.tsx; app/globals.css (.celes-tre, .celes-noi); scripts/test-cho-dat-celes.ts; docs/chien-luoc/celes-visual-character-system.md mục 12</t>
+        </is>
+      </c>
+      <c r="L186" s="8" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M186" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án phải nghiệm thu lại /hoi-dap bằng mắt (5 ảnh trạng thái tạo lại từ v2.3). App chưa làm. Phase 3 vẫn truyền tay giá trị cố định thay characterHook. Hai trang hop-tuoi, tai-khoan còn chữ VI cứng từ trước — không thuộc việc này.</t>
+        </is>
+      </c>
+      <c r="N186" s="8" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="O186" s="8" t="inlineStr">
+        <is>
+          <t>(nhánh viec/linh-vat-moi-man)</t>
         </is>
       </c>
     </row>
@@ -15855,7 +15932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G223"/>
+  <dimension ref="A1:G230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -22886,7 +22963,7 @@
       </c>
       <c r="E194" s="8" t="inlineStr">
         <is>
-          <t>CelesMascot nhận prop trangThai (union 7 giá trị kebab-case) và dựng đường dẫn /celes/&lt;trangThai&gt;.webp. Dùng next/image với unoptimized.</t>
+          <t>CelesMascot nhận prop trangThai (union 7 giá trị kebab-case) và dựng đường dẫn /celes/&lt;trangThai&gt;.webp. Dùng next/image với unoptimized. [CEL-187 thay: xem các dòng CEL-187 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
         </is>
       </c>
       <c r="F194" s="32" t="inlineStr">
@@ -23034,7 +23111,7 @@
       </c>
       <c r="E198" s="8" t="inlineStr">
         <is>
-          <t>CÓ: Hỏi Celes đầu trang (56px), Hỏi Celes rỗng đã chọn lá số và CHƯA chọn lá số (80px, default), màn chờ trả lời (80px, thinking), Danh sách lá số rỗng (80px, default). KHÔNG: lá số, mệnh bàn, mọi trang luận giải, Hành trình, Mối quan hệ, Hôm nay.</t>
+          <t>CÓ: Hỏi Celes đầu trang (56px), Hỏi Celes rỗng đã chọn lá số và CHƯA chọn lá số (80px, default), màn chờ trả lời (80px, thinking), Danh sách lá số rỗng (80px, default). KHÔNG: lá số, mệnh bàn, mọi trang luận giải, Hành trình, Mối quan hệ, Hôm nay. [CEL-187 thay: xem các dòng CEL-187 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
         </is>
       </c>
       <c r="F198" s="32" t="inlineStr">
@@ -23071,7 +23148,7 @@
       </c>
       <c r="E199" s="8" t="inlineStr">
         <is>
-          <t>Bản gốc 49 PNG + 49 WebP ở docs/thiet-ke/celes-nhan-vat/v2/. Bảy tệp WebP đang dùng chép sang public/celes/.</t>
+          <t>Bản gốc 49 PNG + 49 WebP ở docs/thiet-ke/celes-nhan-vat/v2/. Bảy tệp WebP đang dùng chép sang public/celes/. [CEL-187 thay: xem các dòng CEL-187 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
         </is>
       </c>
       <c r="F199" s="32" t="inlineStr">
@@ -23972,6 +24049,265 @@
       <c r="G223" s="8" t="inlineStr">
         <is>
           <t>lib/rag/an-toan.ts; app/api/hoi-dap/route.ts; scripts/test-an-toan.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="30" t="inlineStr">
+        <is>
+          <t>CEL-187</t>
+        </is>
+      </c>
+      <c r="B224" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C224" s="31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D224" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh đúng loại chỗ (tsc)</t>
+        </is>
+      </c>
+      <c r="E224" s="8" t="inlineStr">
+        <is>
+          <t>CelesMascot&lt;C&gt; nhận cho ∈ {dau-trang, rong, cho, cong, loi, su-kien} và trangThai (5 ảnh động) HOẶC minhHoa (13 ảnh tĩnh), loại trừ nhau bằng never. ANH_THEO_CHO[cho] giới hạn ảnh hợp lệ.</t>
+        </is>
+      </c>
+      <c r="F224" s="32" t="inlineStr">
+        <is>
+          <t>ĐẶT SAI CHỖ PHẢI LÀ LỖI BUILD, KHÔNG PHẢI LỖI REVIEW: proud ở rong, concerned ở dau-trang là tsc đỏ. concerned chỉ cho lỗi hệ thống / thanh toán, không cho lỗi nhập liệu (ngày sai vẫn leaning-closer).</t>
+        </is>
+      </c>
+      <c r="G224" s="8" t="inlineStr">
+        <is>
+          <t>components/CelesMascot.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="30" t="inlineStr">
+        <is>
+          <t>CEL-187</t>
+        </is>
+      </c>
+      <c r="B225" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C225" s="31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D225" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh đúng màn (CI)</t>
+        </is>
+      </c>
+      <c r="E225" s="8" t="inlineStr">
+        <is>
+          <t>scripts/test-cho-dat-celes.ts quét app/ + components/: tệp nào import / dựng CelesMascot phải có trong DANH_SACH, và mọi tên ảnh trong từng thẻ phải nằm trong danh sách của tệp đó. CAM liệt kê vùng nội dung. TEN_ANH_CELES khớp 1-1 với public/celes/*.webp; 14 tên khoá không có tệp, không có trong mảng.</t>
+        </is>
+      </c>
+      <c r="F225" s="32" t="inlineStr">
+        <is>
+          <t>DANH SÁCH LÀ NGUỒN SỰ THẬT, KHÔNG ĐẾM "ĐÚNG N TỆP" — đếm cứng thì mỗi lần thêm màn hợp lệ phải sửa số, và số sai không nói sai ở đâu. Bắt bằng import/thẻ, không bằng tên trong chú thích.</t>
+        </is>
+      </c>
+      <c r="G225" s="8" t="inlineStr">
+        <is>
+          <t>scripts/test-cho-dat-celes.ts; .github/workflows/kiem-tra.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="30" t="inlineStr">
+        <is>
+          <t>CEL-187</t>
+        </is>
+      </c>
+      <c r="B226" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C226" s="31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D226" s="8" t="inlineStr">
+        <is>
+          <t>Màn chớp dưới 1 giây không có linh vật</t>
+        </is>
+      </c>
+      <c r="E226" s="8" t="inlineStr">
+        <is>
+          <t>.celes-tre: opacity 0, animation hiện sau var(--celes-tre, 1s). Bài sâu (DangDocV3 celes) đặt 3s. Dưới prefers-reduced-motion vẫn giữ độ trễ, chỉ bỏ mờ dần.</t>
+        </is>
+      </c>
+      <c r="F226" s="32" t="inlineStr">
+        <is>
+          <t>LÀM BẰNG CSS, KHÔNG BẰNG setTimeout: khung Suspense là HTML tĩnh trước khi JS chạy, timer JS không có ở đó. Reduced-motion mà bỏ cả độ trễ là phá luật "không hiện cho màn chớp".</t>
+        </is>
+      </c>
+      <c r="G226" s="8" t="inlineStr">
+        <is>
+          <t>app/globals.css; app/la-so/page.tsx; components/luangiai/DangDocV3.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="30" t="inlineStr">
+        <is>
+          <t>CEL-187</t>
+        </is>
+      </c>
+      <c r="B227" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C227" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D227" s="8" t="inlineStr">
+        <is>
+          <t>Proud khi giữ lại lá số</t>
+        </is>
+      </c>
+      <c r="E227" s="8" t="inlineStr">
+        <is>
+          <t>Nút "Giữ lại" gọi giuLai = luu() rồi setVuaLuu(true) chỉ khi lưu thành công; effect hẹn 4s tắt. Toast .celes-noi position fixed, pointer-events none.</t>
+        </is>
+      </c>
+      <c r="F227" s="32" t="inlineStr">
+        <is>
+          <t>KHÔNG Ở LƯU-KHI-RỜI-TRANG (CanhBaoRoiTrang vẫn gọi luu thẳng) và không sau đăng nhập quay lại — proud là phản hồi cho hành động CHỦ ĐỘNG. Fixed để không CLS.</t>
+        </is>
+      </c>
+      <c r="G227" s="8" t="inlineStr">
+        <is>
+          <t>app/la-so/page.tsx; app/globals.css</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="30" t="inlineStr">
+        <is>
+          <t>CEL-187</t>
+        </is>
+      </c>
+      <c r="B228" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C228" s="31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D228" s="8" t="inlineStr">
+        <is>
+          <t>Celebrate thanh toán một lần</t>
+        </is>
+      </c>
+      <c r="E228" s="8" t="inlineStr">
+        <is>
+          <t>TrangThanhToan quyết mung một lần trong capNhat (ref daQuyetMung) bằng localStorage celes-mung-&lt;id&gt;; lần đầu thành công → celebrate 96, xem lại → default 80. Lỗi tải poll → concerned + nút thử lại.</t>
+        </is>
+      </c>
+      <c r="F228" s="32" t="inlineStr">
+        <is>
+          <t>localStorage hỏng (riêng tư, chặn) thì coi là lần đầu — thà mừng hai lần còn hơn không bao giờ mừng. Poll thành công phải setLoi(null), không thì lỗi cũ dính lại trên đơn đã xong.</t>
+        </is>
+      </c>
+      <c r="G228" s="8" t="inlineStr">
+        <is>
+          <t>components/support/TrangThanhToan.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="30" t="inlineStr">
+        <is>
+          <t>CEL-187</t>
+        </is>
+      </c>
+      <c r="B229" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C229" s="31" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D229" s="8" t="inlineStr">
+        <is>
+          <t>/hoi-dap: hai con, không cùng nghĩ</t>
+        </is>
+      </c>
+      <c r="E229" s="8" t="inlineStr">
+        <is>
+          <t>Đầu trang 56: nghiem ? serious : (dangGo &amp;&amp; cauHoi.trim() ? listening : default); dangGo đổi qua onFocus / onBlur của ô nhập. Thân 80: thinking khi chờ (serious nếu lượt nặng).</t>
+        </is>
+      </c>
+      <c r="F229" s="32" t="inlineStr">
+        <is>
+          <t>ĐẦU TRANG KHÔNG BAO GIỜ THINKING — ngoại lệ "hai con một khung nhìn" chỉ đứng được khi hai con làm hai việc khác nhau. serious theo lượt MỚI NHẤT thắng mọi thứ (bất biến CEL-181 #8).</t>
+        </is>
+      </c>
+      <c r="G229" s="8" t="inlineStr">
+        <is>
+          <t>app/hoi-dap/page.tsx; lib/linh-vat.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="30" t="inlineStr">
+        <is>
+          <t>CEL-187</t>
+        </is>
+      </c>
+      <c r="B230" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C230" s="31" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D230" s="8" t="inlineStr">
+        <is>
+          <t>Không nhảy layout khi ẩn / hiện</t>
+        </is>
+      </c>
+      <c r="E230" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh ẩn theo điều kiện (hop-tuoi curious khi đang chạy, ho-so neutral khi rỗng / đang tải) dùng class invisible, không gỡ khỏi cây. Cỡ qua --celes-cao / --celes-cao-nho (dưới 640px) trong CSS.</t>
+        </is>
+      </c>
+      <c r="F230" s="32" t="inlineStr">
+        <is>
+          <t>CỠ ĐỔI BẰNG CSS, KHÔNG BẰNG JS: đọc bề ngang màn ở client là lệch SSR, hydrate sai. Cùng cao = cùng KHUNG, không cùng THÂN — tư thế nằm (concerned, leaning-closer, playing) trông nhỏ hơn, đã chấp nhận.</t>
+        </is>
+      </c>
+      <c r="G230" s="8" t="inlineStr">
+        <is>
+          <t>components/CelesMascot.tsx; app/globals.css</t>
         </is>
       </c>
     </row>
@@ -23987,7 +24323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28327,6 +28663,38 @@
         </is>
       </c>
       <c r="F135" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B136" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/linh-vat-moi-man)</t>
+        </is>
+      </c>
+      <c r="C136" s="8" t="inlineStr">
+        <is>
+          <t>CEL-187, CEL-181</t>
+        </is>
+      </c>
+      <c r="D136" s="8" t="inlineStr">
+        <is>
+          <t>Linh vật Celes ra mọi màn web: 18 ảnh v2.3 (sửa quầng trắng) thay 7 ảnh v2, 14 ảnh khoá không có tệp. Prop cho + ANH_THEO_CHO (tsc), bài CI test-cho-dat-celes. Màn chờ hiện trễ bằng CSS, proud nổi 4s khi bấm Giữ lại, celebrate một lần mỗi giao dịch. /hoi-dap đầu trang có listening. Hôm nay: chỉ thẻ rỗng. Mục 12 viết lại.</t>
+        </is>
+      </c>
+      <c r="E136" s="8" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt 02/10/2026: 5 chỗ của CEL-181 để linh vật vắng ở hầu hết hành trình, sản phẩm mất nhân vật đúng lúc người dùng chờ hoặc lạc. Nguyên tắc "không nơi người ta đọc" vẫn giữ, nhưng phát biểu theo VÙNG (không trong nội dung) thay vì theo TRANG — trang lá số có màn chờ, màn nhập, không chỉ có mệnh bàn. Luật đặt chuyển từ lời sang mã (tsc + CI) để màn mới không tự thêm linh vật mà không qua mục 12. Ảnh khoá bị xoá tệp để mở khoá phải là quyết định, không phải một dòng import.</t>
+        </is>
+      </c>
+      <c r="F136" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
CEL-186a P5: kiem-nhanh + smoke safety/quick + CI, tai lieu va backlog
- npm run kiem-nhanh: tsc + lint + chi cac bai offline cua vung da doi (so voi merge-base origin/main,
  ca working tree va tep moi); --tat-ca chay moi bai offline
- npm run smoke:safety, smoke:quick: offline, in PASS "..." theo ca, exit != 0 khi hong
- CI them test-do-sau, test-ngoai-tam, test-quick-answer va hai smoke truoc Build
- docs CEL-186: muc 17c thay bang bang cau du phong dang chay, them muc 18 mo ta theo code that
- PRODUCT-BACKLOG: CEL-186 o Backlog, 7 buoc Logic chi tiet, 3 dong Nhat ky

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O185"/>
+  <dimension ref="A1:O186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15838,6 +15838,87 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" s="11" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B186" s="12" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C186" s="8" t="inlineStr">
+        <is>
+          <t>Quick answer + giọng hội thoại (CEL-186a)</t>
+        </is>
+      </c>
+      <c r="D186" s="8" t="inlineStr">
+        <is>
+          <t>Câu có/không và câu quyết định đơn giản ở sự nghiệp / tài chính / tình cảm được trả lời như MỘT tin nhắn: câu đầu trả lời thẳng, tối đa một dữ kiện, một mệnh đề lực ngược, 40–110 âm tiết (trần mềm 150), không heading, không cân nhắc / bước tiếp. Câu hỏi danh tính bạn đời ("chồng tôi có phải Nguyễn Duy Hiếu ko?") nhận một trong ba câu kết luận ngoài tầm đã duyệt. Mọi câu khác giữ nguyên STANDARD, prompt STANDARD giống từng byte.</t>
+        </is>
+      </c>
+      <c r="E186" s="8" t="inlineStr">
+        <is>
+          <t>1. route: doAnToan → nhanDangNgoaiTam → tinhNghiengVe → tinhDoSau (QUICK/STANDARD/DEEP + lý do)
+2. QUICK: dungPromptCoCanCu(..., {ngoaiTam, tinhNghich}) — không khối hướng STANDARD
+3. Model trả JSON như cũ (maxTokens 6000)
+4. kiemQuick cắt/thay câu chốt khi lệch → dungVan(QUICK) khuôn tin nhắn
+5. Vết ai_requests ghi doSau, lyDoDoSau, ngoaiTam, mucAnToan — không ghi câu hỏi</t>
+        </is>
+      </c>
+      <c r="F186" s="9" t="inlineStr">
+        <is>
+          <t>Đang thử (preview)</t>
+        </is>
+      </c>
+      <c r="G186" s="8" t="inlineStr">
+        <is>
+          <t>Model + hàm thuần hậu kỳ; câu dự phòng và câu ngoài tầm duyệt tay</t>
+        </is>
+      </c>
+      <c r="H186" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I186" s="8" t="inlineStr">
+        <is>
+          <t>Mọi bậc (chip vẫn tốn lượt)</t>
+        </is>
+      </c>
+      <c r="J186" s="8" t="inlineStr">
+        <is>
+          <t>/hoi-dap (web + app)</t>
+        </is>
+      </c>
+      <c r="K186" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/hop-dong-tra-loi.ts (tinhDoSau, cờ); lib/rag/kiem-quick.ts; lib/rag/chot-huong.ts; lib/rag/ngoai-tam.ts; lib/rag/prompt-co-can-cu.ts; lib/rag/tra-loi.ts; docs/thiet-ke/CEL-186-quick-answer.md</t>
+        </is>
+      </c>
+      <c r="L186" s="8" t="inlineStr">
+        <is>
+          <t>CELES_QUICK_ANSWER: không đặt thì chỉ bật ở preview; production phải đặt "1". CELES_TINH_NGHICH không đặt thì theo cờ QUICK.</t>
+        </is>
+      </c>
+      <c r="M186" s="8" t="inlineStr">
+        <is>
+          <t>CHƯA chạy eval 20 ca model thật (mục 12 doc) — phải chạy trước khi bật production. Chưa đo được model có giữ 40–110 âm tiết không, và tỉ lệ thiếu chieuCauChot theo nhà cung cấp. Ngoài tầm không bắt tên viết thường không dấu (cố ý). Chưa có streaming, chưa có characterHook (CEL-187).</t>
+        </is>
+      </c>
+      <c r="N186" s="8" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="O186" s="8" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-quick)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -15855,7 +15936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G223"/>
+  <dimension ref="A1:G230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -23975,6 +24056,265 @@
         </is>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" s="30" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B224" s="31" t="inlineStr">
+        <is>
+          <t>Quick answer (chat)</t>
+        </is>
+      </c>
+      <c r="C224" s="31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D224" s="8" t="inlineStr">
+        <is>
+          <t>Chọn độ sâu bằng hàm thuần</t>
+        </is>
+      </c>
+      <c r="E224" s="8" t="inlineStr">
+        <is>
+          <t>tinhDoSau thứ tự: an toàn ≠ NORMAL → chủ đề nặng → xin sâu (DEEP) → xin thêm → từ chip → giải thích/"vì sao" → nhiều vế → ngoài tầm (QUICK) → ý định ∉ {co-khong, quyet-dinh} → "A hay B" → chủ đề ∉ {su-nghiep, tai-chinh, tinh-cam} → không hướng → giai đoạn → năm khác → chiều xấu → hỏi người khác → QUICK.</t>
+        </is>
+      </c>
+      <c r="F224" s="32" t="inlineStr">
+        <is>
+          <t>DoSauTraLoi TÁCH khỏi Nhip của CEL-183, không gộp. An toàn luôn thắng, kể cả câu ngoài tầm. Câu nối (chip) không bao giờ QUICK.</t>
+        </is>
+      </c>
+      <c r="G224" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/hop-dong-tra-loi.ts; scripts/test-do-sau.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="30" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B225" s="31" t="inlineStr">
+        <is>
+          <t>Quick answer (chat)</t>
+        </is>
+      </c>
+      <c r="C225" s="31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D225" s="8" t="inlineStr">
+        <is>
+          <t>Chiều xấu và quyết định rời bỏ không QUICK</t>
+        </is>
+      </c>
+      <c r="E225" s="8" t="inlineStr">
+        <is>
+          <t>laCauChieuXau: ly hôn, chia tay, mất việc, lỗ, nợ, "có bị", "sẽ bị"… VÀ các quyết định rời bỏ (nghỉ việc, bỏ chồng, rút vốn, bán nhà, cắt lỗ…).</t>
+        </is>
+      </c>
+      <c r="F225" s="32" t="inlineStr">
+        <is>
+          <t>Hướng engine "thuận" trên câu "có nên nghỉ việc" sẽ đọc thành "nên nghỉ" — một kết luận engine không hề đếm. Gắn vào STANDARD để có đủ lực ngược.</t>
+        </is>
+      </c>
+      <c r="G225" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/chot-huong.ts; scripts/test-do-sau.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="30" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B226" s="31" t="inlineStr">
+        <is>
+          <t>Quick answer (chat)</t>
+        </is>
+      </c>
+      <c r="C226" s="31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D226" s="8" t="inlineStr">
+        <is>
+          <t>Câu ngoài tầm lá số</t>
+        </is>
+      </c>
+      <c r="E226" s="8" t="inlineStr">
+        <is>
+          <t>nhanDangNgoaiTam: mẫu hỏi danh tính bạn đời/người yêu + tên riêng (viết hoa, hoặc có họ) hoặc "tên gì / họ gì". Kết luận = CAU_NGOAI_TAM[FNV(câu) % n], câu 2 loại khỏi người đã cưới. Không tính nghiêng.</t>
+        </is>
+      </c>
+      <c r="F226" s="32" t="inlineStr">
+        <is>
+          <t>KHÔNG bắt nhầm: tên sao, "người tốt", "ngoại tình", "chung thủy", "buồn", tên viết thường không dấu. Bắt nhầm là câu bình thường mất hướng. Kèm chiều xấu → STANDARD.</t>
+        </is>
+      </c>
+      <c r="G226" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/ngoai-tam.ts; scripts/test-ngoai-tam.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="30" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B227" s="31" t="inlineStr">
+        <is>
+          <t>Quick answer (chat)</t>
+        </is>
+      </c>
+      <c r="C227" s="31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D227" s="8" t="inlineStr">
+        <is>
+          <t>Prompt QUICK tách nhánh, STANDARD nguyên byte</t>
+        </is>
+      </c>
+      <c r="E227" s="8" t="inlineStr">
+        <is>
+          <t>dungPromptCoCanCu nhận tuỳ chọn {ngoaiTam, tinhNghich} ở cuối. Không truyền → chuỗi y hệt bản trước. QUICK không có "XU HƯỚNG ENGINE ĐÃ CHỐT"; ngoài tầm không có "HƯỚNG ĐÃ CHỐT".</t>
+        </is>
+      </c>
+      <c r="F227" s="32" t="inlineStr">
+        <is>
+          <t>So 96 tổ hợp với HEAD trước khi commit: lệch 0. Đổi một byte của STANDARD là xả đệm và đổi giọng cả sản phẩm — khoá bằng test-quick-answer.</t>
+        </is>
+      </c>
+      <c r="G227" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/prompt-co-can-cu.ts; scripts/test-quick-answer.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="30" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B228" s="31" t="inlineStr">
+        <is>
+          <t>Quick answer (chat)</t>
+        </is>
+      </c>
+      <c r="C228" s="31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D228" s="8" t="inlineStr">
+        <is>
+          <t>Hậu kỳ QUICK chỉ thay câu chốt</t>
+        </is>
+      </c>
+      <c r="E228" s="8" t="inlineStr">
+        <is>
+          <t>kiemQuick: bỏ heading/tiêu đề ý/canNhac/bước tiếp/tự kiểm/hỏi lại; 1 ý, 1 dữ kiện; 40–110 âm tiết, trần mềm 150 cắt theo câu. Câu chốt rỗng/ngược hướng/quá chắc/phán quyết/giọng report/tên sao/tên bịa/khẳng định đời thật/tiếng lóng/self-help → câu dự phòng §22. Thiếu chieuCauChot → chỉ ghi vết.</t>
+        </is>
+      </c>
+      <c r="F228" s="32" t="inlineStr">
+        <is>
+          <t>Không viết lại cả bài khi chỉ câu chốt sai — phần dữ kiện model viết đúng vẫn giữ. Không cắt giữa câu. Chip ≤ 40 ký tự, tối đa 3, KHÔNG cắt ngắn, bỏ chip hỏi tên.</t>
+        </is>
+      </c>
+      <c r="G228" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/kiem-quick.ts; lib/rag/tra-loi.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="30" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B229" s="31" t="inlineStr">
+        <is>
+          <t>Quick answer (chat)</t>
+        </is>
+      </c>
+      <c r="C229" s="31" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D229" s="8" t="inlineStr">
+        <is>
+          <t>Câu dự phòng và tiền tố năm</t>
+        </is>
+      </c>
+      <c r="E229" s="8" t="inlineStr">
+        <is>
+          <t>cauChotDuPhong theo bảng CO_KHONG / QUYET_DINH × 5 hướng, {cum} từ cumChoChuDe. "Năm {nam}, " chỉ khi hoiVeNam (số năm = namXem hoặc "năm nay").</t>
+        </is>
+      </c>
+      <c r="F229" s="32" t="inlineStr">
+        <is>
+          <t>namXem do route tự điền KHÔNG phải bằng chứng người dùng hỏi về năm. Không câu nào có "nên/chưa nên" — dự phòng chỉ nói chiều phần đời.</t>
+        </is>
+      </c>
+      <c r="G229" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/chot-huong.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="30" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B230" s="31" t="inlineStr">
+        <is>
+          <t>Quick answer (chat)</t>
+        </is>
+      </c>
+      <c r="C230" s="31" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D230" s="8" t="inlineStr">
+        <is>
+          <t>Cờ bật</t>
+        </is>
+      </c>
+      <c r="E230" s="8" t="inlineStr">
+        <is>
+          <t>quickAnswerBat: "1"/"true" bật, "0"/"false" tắt, không đặt → VERCEL_ENV==="preview". tinhNghichBat: CELES_TINH_NGHICH, không đặt → theo cờ QUICK. Cờ tắt → doSau STANDARD, ngoaiTam null.</t>
+        </is>
+      </c>
+      <c r="F230" s="32" t="inlineStr">
+        <is>
+          <t>Production KHÔNG tự bật. Trêu (choPhepTinhNghich) chỉ khi: cờ bật + QUICK + NORMAL; không sức khoẻ, không chủ đề nặng, không chiều xấu, không từ nghiêm; không phải câu nối; hướng thuan-ro / thuan-nhe / can-bang (câu ngoài tầm bỏ qua điều kiện hướng); 3 lượt người dùng gần nhất đều NORMAL. Chưa đo bằng model thật.</t>
+        </is>
+      </c>
+      <c r="G230" s="8" t="inlineStr">
+        <is>
+          <t>lib/rag/hop-dong-tra-loi.ts; lib/rag/kiem-quick.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23987,7 +24327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28327,6 +28667,102 @@
         </is>
       </c>
       <c r="F135" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B136" s="50" t="inlineStr">
+        <is>
+          <t>cd56c00</t>
+        </is>
+      </c>
+      <c r="C136" s="8" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D136" s="8" t="inlineStr">
+        <is>
+          <t>P1 planner: "chồng/vợ tôi" → tinh-cam; "vậy" có dấu không còn là vay tiền. Bộ vàng 83/83.</t>
+        </is>
+      </c>
+      <c r="E136" s="8" t="inlineStr">
+        <is>
+          <t>Câu ngoài tầm "chồng tôi có phải …" rơi vào tong-quan nên không bao giờ tới QUICK; "vậy" bị hiểu là vay làm câu thường sang tài chính. PHIEN_BAN_PLANNER tăng → đếm trước: 21/8108 bài đệm bị xả.</t>
+        </is>
+      </c>
+      <c r="F136" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B137" s="50" t="inlineStr">
+        <is>
+          <t>8931545</t>
+        </is>
+      </c>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>P4 vết an toàn: lượt CRITICAL / tiên lượng ghi ai_requests (muc, nhom, tienLuong), cau_hoi=null; mọi lượt ghi mucAnToan và độ sâu.</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>Trước đây lượt bị chặn không để lại dấu vết nào — không đo được lớp an toàn chặn bao nhiêu, chặn nhầm bao nhiêu. Không ghi câu hỏi vì đó là dữ liệu nhạy cảm nhất của người dùng.</t>
+        </is>
+      </c>
+      <c r="F137" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="49" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B138" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-quick)</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="inlineStr">
+        <is>
+          <t>P3 quick answer + giọng hội thoại (cờ CELES_QUICK_ANSWER, preview bật) + kiem-nhanh, smoke:safety, smoke:quick, ba test mới vào CI.</t>
+        </is>
+      </c>
+      <c r="E138" s="8" t="inlineStr">
+        <is>
+          <t>Câu "có/không" ngắn đang nhận một bài báo cáo có heading — người hỏi một câu, nhận một trang. QUICK thu hẹp có chủ đích (3 chủ đề, có hướng, không chiều xấu) để bản đầu không thể đưa ra kết luận engine không đếm; mọi đường khác giữ STANDARD nguyên byte. Cờ để production chỉ bật sau eval model thật.</t>
+        </is>
+      </c>
+      <c r="F138" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
CEL-188: auth preview ve dung origin, /hoi-dap khong trung dang, cong /luan-giai/sau dung CongDangNhap, doi ma CEL-187 -> CEL-188
- Dang ky gui emailRedirectTo, Google gui redirectTo = origin dang mo + /auth/callback?next=
  (next chi nhan duong dan noi bo, mac dinh /home). Preview van can mau
  https://*-duyhieu24082000-6871s-projects.vercel.app/** trong Redirect URLs cua Supabase
  (HUONG-DAN.md buoc 3).
- /hoi-dap than: chua chon la so -> one-ear-up, chat rong -> curious; test-cho-dat-celes
  muc 5 chan dau trang va than rong cung dang.
- /luan-giai/sau chua dang nhap: CongDangNhap nguon="deep_read" toanTrang, them prop quayVe.
- Ma chinh thuc cua "linh vat moi man web" doi sang CEL-188; cac commit truoc mang nhan
  CEL-187, CEL-187 giu cho Streaming. Muc 12 them luat cho ngan tre / cho dai hien ngay.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -4098,12 +4098,12 @@
       </c>
       <c r="M38" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>03/10: đăng ký / Google quay về origin đang mở (emailRedirectTo / redirectTo). Preview cần mẫu https://*-duyhieu24082000-6871s-projects.vercel.app/** trong Redirect URLs của Supabase.</t>
         </is>
       </c>
       <c r="N38" s="8" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="O38" s="8" t="inlineStr">
@@ -4175,12 +4175,12 @@
       </c>
       <c r="M39" s="8" t="inlineStr">
         <is>
-          <t>Kiểm bằng npm run kiem-tra-sso.</t>
+          <t>Kiểm bằng npm run kiem-tra-sso. 03/10: đăng ký / Google quay về origin đang mở (emailRedirectTo / redirectTo). Preview cần mẫu https://*-duyhieu24082000-6871s-projects.vercel.app/** trong Redirect URLs của Supabase.</t>
         </is>
       </c>
       <c r="N39" s="8" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="O39" s="8" t="inlineStr">
@@ -15588,12 +15588,12 @@
       </c>
       <c r="M182" s="8" t="inlineStr">
         <is>
-          <t>Phase 3 nối characterHook → visual state, hiện truyền tay giá trị cố định. Tab Hôm nay KHÔNG đặt linh vật — chủ dự án xem lại 02/10/2026 và giữ nguyên, xem lại khi web dùng thật đủ lâu. App (apps/celes-app) chưa có luật nghiêm theo lượt. — Mở rộng ra mọi màn web: CEL-187 (thay luật "không ở lá số / luận giải" bằng "không TRONG vùng nội dung").</t>
+          <t>Phase 3 nối characterHook → visual state, hiện truyền tay giá trị cố định. Tab Hôm nay KHÔNG đặt linh vật — chủ dự án xem lại 02/10/2026 và giữ nguyên, xem lại khi web dùng thật đủ lâu. App (apps/celes-app) chưa có luật nghiêm theo lượt. — Mở rộng ra mọi màn web: CEL-188 (thay luật "không ở lá số / luận giải" bằng "không TRONG vùng nội dung").</t>
         </is>
       </c>
       <c r="N182" s="8" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="O182" s="8" t="inlineStr">
@@ -15841,7 +15841,7 @@
     <row r="186">
       <c r="A186" s="11" t="inlineStr">
         <is>
-          <t>CEL-187</t>
+          <t>CEL-188</t>
         </is>
       </c>
       <c r="B186" s="12" t="inlineStr">
@@ -15901,12 +15901,12 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>Chủ dự án phải nghiệm thu lại /hoi-dap bằng mắt (5 ảnh trạng thái tạo lại từ v2.3). App chưa làm. Phase 3 vẫn truyền tay giá trị cố định thay characterHook. Hai trang hop-tuoi, tai-khoan còn chữ VI cứng từ trước — không thuộc việc này.</t>
+          <t>Các commit triển khai ban đầu mang nhãn CEL-187; mã chính thức đã đổi sang CEL-188. CEL-187 giữ cho Streaming. Chủ dự án phải nghiệm thu bằng mắt trên preview (cần thêm mẫu URL preview vào Redirect URLs của Supabase trước — xem CEL-037). App chưa làm. Phase 3 vẫn truyền tay giá trị cố định thay characterHook. Hai trang hop-tuoi, tai-khoan còn chữ VI cứng từ trước — không thuộc việc này.</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="O186" s="8" t="inlineStr">
@@ -15932,7 +15932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G230"/>
+  <dimension ref="A1:G233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -22963,7 +22963,7 @@
       </c>
       <c r="E194" s="8" t="inlineStr">
         <is>
-          <t>CelesMascot nhận prop trangThai (union 7 giá trị kebab-case) và dựng đường dẫn /celes/&lt;trangThai&gt;.webp. Dùng next/image với unoptimized. [CEL-187 thay: xem các dòng CEL-187 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
+          <t>CelesMascot nhận prop trangThai (union 7 giá trị kebab-case) và dựng đường dẫn /celes/&lt;trangThai&gt;.webp. Dùng next/image với unoptimized. [CEL-188 thay: xem các dòng CEL-188 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
         </is>
       </c>
       <c r="F194" s="32" t="inlineStr">
@@ -23111,7 +23111,7 @@
       </c>
       <c r="E198" s="8" t="inlineStr">
         <is>
-          <t>CÓ: Hỏi Celes đầu trang (56px), Hỏi Celes rỗng đã chọn lá số và CHƯA chọn lá số (80px, default), màn chờ trả lời (80px, thinking), Danh sách lá số rỗng (80px, default). KHÔNG: lá số, mệnh bàn, mọi trang luận giải, Hành trình, Mối quan hệ, Hôm nay. [CEL-187 thay: xem các dòng CEL-187 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
+          <t>CÓ: Hỏi Celes đầu trang (56px), Hỏi Celes rỗng đã chọn lá số và CHƯA chọn lá số (80px, default), màn chờ trả lời (80px, thinking), Danh sách lá số rỗng (80px, default). KHÔNG: lá số, mệnh bàn, mọi trang luận giải, Hành trình, Mối quan hệ, Hôm nay. [CEL-188 thay: xem các dòng CEL-188 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
         </is>
       </c>
       <c r="F198" s="32" t="inlineStr">
@@ -23148,7 +23148,7 @@
       </c>
       <c r="E199" s="8" t="inlineStr">
         <is>
-          <t>Bản gốc 49 PNG + 49 WebP ở docs/thiet-ke/celes-nhan-vat/v2/. Bảy tệp WebP đang dùng chép sang public/celes/. [CEL-187 thay: xem các dòng CEL-187 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
+          <t>Bản gốc 49 PNG + 49 WebP ở docs/thiet-ke/celes-nhan-vat/v2/. Bảy tệp WebP đang dùng chép sang public/celes/. [CEL-188 thay: xem các dòng CEL-188 — 18 ảnh, prop cho + ANH_THEO_CHO, danh sách chỗ đặt trong test.]</t>
         </is>
       </c>
       <c r="F199" s="32" t="inlineStr">
@@ -24055,7 +24055,7 @@
     <row r="224">
       <c r="A224" s="30" t="inlineStr">
         <is>
-          <t>CEL-187</t>
+          <t>CEL-188</t>
         </is>
       </c>
       <c r="B224" s="31" t="inlineStr">
@@ -24092,7 +24092,7 @@
     <row r="225">
       <c r="A225" s="30" t="inlineStr">
         <is>
-          <t>CEL-187</t>
+          <t>CEL-188</t>
         </is>
       </c>
       <c r="B225" s="31" t="inlineStr">
@@ -24129,7 +24129,7 @@
     <row r="226">
       <c r="A226" s="30" t="inlineStr">
         <is>
-          <t>CEL-187</t>
+          <t>CEL-188</t>
         </is>
       </c>
       <c r="B226" s="31" t="inlineStr">
@@ -24166,7 +24166,7 @@
     <row r="227">
       <c r="A227" s="30" t="inlineStr">
         <is>
-          <t>CEL-187</t>
+          <t>CEL-188</t>
         </is>
       </c>
       <c r="B227" s="31" t="inlineStr">
@@ -24203,7 +24203,7 @@
     <row r="228">
       <c r="A228" s="30" t="inlineStr">
         <is>
-          <t>CEL-187</t>
+          <t>CEL-188</t>
         </is>
       </c>
       <c r="B228" s="31" t="inlineStr">
@@ -24240,7 +24240,7 @@
     <row r="229">
       <c r="A229" s="30" t="inlineStr">
         <is>
-          <t>CEL-187</t>
+          <t>CEL-188</t>
         </is>
       </c>
       <c r="B229" s="31" t="inlineStr">
@@ -24255,17 +24255,17 @@
       </c>
       <c r="D229" s="8" t="inlineStr">
         <is>
-          <t>/hoi-dap: hai con, không cùng nghĩ</t>
+          <t>/hoi-dap: hai con, không bao giờ cùng dáng</t>
         </is>
       </c>
       <c r="E229" s="8" t="inlineStr">
         <is>
-          <t>Đầu trang 56: nghiem ? serious : (dangGo &amp;&amp; cauHoi.trim() ? listening : default); dangGo đổi qua onFocus / onBlur của ô nhập. Thân 80: thinking khi chờ (serious nếu lượt nặng).</t>
+          <t>Đầu trang 56: nghiem ? serious : (dangGo &amp;&amp; cauHoi.trim() ? listening : default); dangGo đổi qua onFocus / onBlur của ô nhập. Thân 80: chưa chọn lá số → one-ear-up; đã chọn, chat rỗng → curious; đang trả lời → thinking (serious nếu lượt mới nhất nặng).</t>
         </is>
       </c>
       <c r="F229" s="32" t="inlineStr">
         <is>
-          <t>ĐẦU TRANG KHÔNG BAO GIỜ THINKING — ngoại lệ "hai con một khung nhìn" chỉ đứng được khi hai con làm hai việc khác nhau. serious theo lượt MỚI NHẤT thắng mọi thứ (bất biến CEL-181 #8).</t>
+          <t>ĐẦU TRANG KHÔNG BAO GIỜ THINKING, THÂN RỖNG KHÔNG DÙNG ẢNH NÀO CỦA ĐẦU TRANG — ngoại lệ "hai con một khung nhìn" chỉ đứng được khi hai con làm hai việc khác nhau. Ngoại lệ duy nhất được trùng: lượt mới nhất nặng thì cả hai serious (bất biến CEL-181 #8). Kiểm ở mục 5 scripts/test-cho-dat-celes.ts.</t>
         </is>
       </c>
       <c r="G229" s="8" t="inlineStr">
@@ -24277,7 +24277,7 @@
     <row r="230">
       <c r="A230" s="30" t="inlineStr">
         <is>
-          <t>CEL-187</t>
+          <t>CEL-188</t>
         </is>
       </c>
       <c r="B230" s="31" t="inlineStr">
@@ -24308,6 +24308,117 @@
       <c r="G230" s="8" t="inlineStr">
         <is>
           <t>components/CelesMascot.tsx; app/globals.css</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="30" t="inlineStr">
+        <is>
+          <t>CEL-188</t>
+        </is>
+      </c>
+      <c r="B231" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C231" s="31" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D231" s="8" t="inlineStr">
+        <is>
+          <t>Cổng đăng nhập toàn trang dùng chung</t>
+        </is>
+      </c>
+      <c r="E231" s="8" t="inlineStr">
+        <is>
+          <t>/luan-giai/sau khi chưa đăng nhập dựng CongDangNhap nguon="deep_read" toanTrang (waving), truyền quayVe = đường dẫn kèm query để đăng nhập xong về đúng bài. CongDangNhap nhận quayVe chỉ khi là đường dẫn nội bộ (/… không phải //…), không thì dùng pathname.</t>
+        </is>
+      </c>
+      <c r="F231" s="32" t="inlineStr">
+        <is>
+          <t>MỘT CÀI ĐẶT CỔNG, KHÔNG CHÉP: cổng tự dựng riêng ở trang là một chỗ thứ hai phải giữ chữ, ảnh và luồng quay về; lệch là chuyện thời gian.</t>
+        </is>
+      </c>
+      <c r="G231" s="8" t="inlineStr">
+        <is>
+          <t>components/auth/CongDangNhap.tsx; app/luan-giai/sau/page.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="30" t="inlineStr">
+        <is>
+          <t>CEL-188</t>
+        </is>
+      </c>
+      <c r="B232" s="31" t="inlineStr">
+        <is>
+          <t>Linh vật Celes mọi màn web</t>
+        </is>
+      </c>
+      <c r="C232" s="31" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D232" s="8" t="inlineStr">
+        <is>
+          <t>Chờ ngắn hiện trễ, chờ dài hiện ngay</t>
+        </is>
+      </c>
+      <c r="E232" s="8" t="inlineStr">
+        <is>
+          <t>Chờ ngắn / có thể dưới 1s (khung Suspense lá số, chi tiết hạn, bài sâu từ bộ đệm) → giữ chỗ, .celes-tre hiện trễ. Chờ chắc chắn dài (chat, /luan-giai sinh 15–45s, hợp tuổi) → thinking hiện ngay. "Lập lá số" tính ở trình duyệt → không có màn chờ, không chớp thinking.</t>
+        </is>
+      </c>
+      <c r="F232" s="32" t="inlineStr">
+        <is>
+          <t>ĐỘ TRỄ THEO ĐỘ DÀI CHỜ, KHÔNG THEO MÀN: trễ ở chờ dài là để người dùng nhìn khoảng trống vô nghĩa 1s; không trễ ở chờ ngắn là chớp ảnh.</t>
+        </is>
+      </c>
+      <c r="G232" s="8" t="inlineStr">
+        <is>
+          <t>app/globals.css; app/la-so/page.tsx; components/hanhtrinh/TrangChiTietNoiDung.tsx; components/luangiai/DangDocV3.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="30" t="inlineStr">
+        <is>
+          <t>CEL-037</t>
+        </is>
+      </c>
+      <c r="B233" s="31" t="inlineStr">
+        <is>
+          <t>Đăng nhập email + mật khẩu</t>
+        </is>
+      </c>
+      <c r="C233" s="31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D233" s="8" t="inlineStr">
+        <is>
+          <t>Quay về đúng origin (preview / production)</t>
+        </is>
+      </c>
+      <c r="E233" s="8" t="inlineStr">
+        <is>
+          <t>signUp gửi emailRedirectTo, Google gửi redirectTo = window.location.origin + /auth/callback?next=… (next chỉ nhận đường dẫn nội bộ, mặc định /home). Đăng nhập mật khẩu không qua Supabase redirect nên tự ở lại origin. /auth/callback đổi mã lấy phiên theo origin của request.</t>
+        </is>
+      </c>
+      <c r="F233" s="32" t="inlineStr">
+        <is>
+          <t>THIẾU emailRedirectTo HOẶC URL KHÔNG CÓ TRONG Redirect URLs CỦA SUPABASE THÌ SUPABASE ÂM THẦM VỀ Site URL (production) — preview đăng nhập xong rơi sang production. Mã đúng chưa đủ: Supabase Auth → URL Configuration → Redirect URLs phải có https://*-duyhieu24082000-6871s-projects.vercel.app/**. Không kiểm được từ ngoài (state của authorize là UUID mờ).</t>
+        </is>
+      </c>
+      <c r="G233" s="8" t="inlineStr">
+        <is>
+          <t>app/dang-nhap/page.tsx; app/auth/callback/route.ts</t>
         </is>
       </c>
     </row>
@@ -24323,7 +24434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28681,7 +28792,7 @@
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t>CEL-187, CEL-181</t>
+          <t>CEL-188 (ghi lúc đó: CEL-187), CEL-181</t>
         </is>
       </c>
       <c r="D136" s="8" t="inlineStr">
@@ -28695,6 +28806,38 @@
         </is>
       </c>
       <c r="F136" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="49" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B137" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/linh-vat-moi-man)</t>
+        </is>
+      </c>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>CEL-188, CEL-187, CEL-037, CEL-038</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>Đổi mã "linh vật mọi màn web" CEL-187 → CEL-188 (Backlog, Logic, mục 12). /hoi-dap thân: one-ear-up khi chưa chọn lá số, curious khi chat rỗng — không trùng dáng đầu trang, có bài kiểm. /luan-giai/sau chưa đăng nhập dùng CongDangNhap toanTrang (thêm prop quayVe). Đăng ký / Google gửi emailRedirectTo / redirectTo theo origin đang mở. Mục 12 viết luật chờ ngắn–chờ dài.</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>CEL-187 đã giữ cho Streaming (CEL-186-quick-answer.md §15) — trùng mã là hai việc khác nhau cùng một dòng nhật ký, sau vài tháng không gỡ được. Đăng nhập từ preview rơi sang production làm chủ dự án không nghiệm thu được trạng thái đã đăng nhập; nguyên nhân là Supabase rơi về Site URL khi thiếu emailRedirectTo hoặc URL chưa có trong danh sách cho phép. Dáng trùng ở /hoi-dap (default cả hai con) làm ngoại lệ "hai con" mất lý do tồn tại.</t>
+        </is>
+      </c>
+      <c r="F137" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
CEL-186 ve A (nghiem thu lan 2): huong nghieng theo moc, giai-doan khong roi ve luu nien, thang muc tieu
- canTinhNghieng: mo-ta + gan/nam/thang van tinh huong nghieng ("Cong viec sap toi the nao?")
- giai-doan khong them luu-nien/nguyet-han du phong; bai dai "Toi la ai... ca doi" gio chi ban-menh
- thangMucTieu (thang nay/toi/sau/N/N nam Y, thang 12 -> thang toi sang nam), thangHieuLuc cho chonBoiCanh, tinhNghiengVe, nhat ky
- PHIEN_BAN_PLANNER 2026.10.3; bo vang 98 cau, 100%

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15851,12 +15851,12 @@
       </c>
       <c r="C186" s="8" t="inlineStr">
         <is>
-          <t>Trục thời gian của câu hỏi (planner) + năm hiệu lực + chip "Sang năm"</t>
+          <t>Trục thời gian của câu hỏi (planner) + năm/tháng hiệu lực + chip "Sang năm"</t>
         </is>
       </c>
       <c r="D186" s="8" t="inlineStr">
         <is>
-          <t>Planner có trục thứ ba phamViThoiGian (khong-ro / gan / thang / nam / giai-doan), TÁCH khỏi ý định, kèm namMucTieu (năm viết số, hoặc năm nay / năm tới / năm sau / sang năm / năm ngoái tính từ năm xem). "Tương lai gần / sắp tới" là gan, thắng chữ "tương lai" (giai-doan). Nhận câu có/không theo vế, gọt đuôi chữ đệm và cụm thời gian (thay luật 3 từ cuối). Mỗi lượt chat đọc một namHieuLuc = namMucTieu ?? namXem. Chat mặc định năm ÂM hiện tại. Từ tháng âm 9 tới Tết thêm chip "Sang năm &lt;Can Chi&gt; thì sao?".</t>
+          <t>Planner có trục thứ ba phamViThoiGian (khong-ro / gan / thang / nam / giai-doan), TÁCH khỏi ý định, kèm namMucTieu (năm viết số, hoặc năm nay / năm tới / năm sau / sang năm / năm ngoái tính từ năm xem). "Tương lai gần / sắp tới" là gan, thắng chữ "tương lai" (giai-doan). Nhận câu có/không theo vế, gọt đuôi chữ đệm và cụm thời gian (thay luật 3 từ cuối). Có thêm thangMucTieu (tháng này / tháng tới / tháng sau tính từ tháng âm đang xem, tháng 12 → tháng tới sang tháng 1 năm sau; "tháng N" giữ năm đang xem trừ khi viết năm). Mỗi lượt chat đọc một namHieuLuc = namMucTieu ?? namXem và thangHieuLuc = thangMucTieu ?? thangXem. Hướng nghiêng tính theo ý định VÀ mốc: câu mô tả có mốc gần / năm / tháng ("Công việc sắp tới thế nào?") vẫn tính; mô tả không mốc hoặc chặng dài thì không. Chặng dài (giai-doan) không bao giờ rơi về lưu niên / nguyệt hạn dự phòng. Chat mặc định năm ÂM hiện tại. Từ tháng âm 9 tới Tết thêm chip "Sang năm &lt;Can Chi&gt; thì sao?".</t>
         </is>
       </c>
       <c r="E186" s="8" t="inlineStr">
@@ -15864,7 +15864,8 @@
           <t>1. route hoi-dap: namXem mặc định namAmHienTai()
 2. planner: doanPhamViThoiGian quét trái→phải (năm số, "tháng N", cụm dài nhất 4→1 từ; bỏ năm sau chữ "sinh")
 3. doanLopHan: gan/nam → đại vận + lưu niên; thang → nguyệt hạn; giai-doan không ép lưu niên trong nhánh ý định, chặn bí danh lưu niên/nguyệt hạn của từ điển thực thể
-4. tra-loi: namHieuLuc cho chọn bối cảnh, hướng nghiêng, sổ đã nói trước (V3 + tổng quan), nhật ký
+4. tra-loi: namHieuLuc cho chọn bối cảnh, hướng nghiêng, sổ đã nói trước (V3 + tổng quan), nhật ký; thangHieuLuc cho chọn bối cảnh, hướng nghiêng, nhật ký; canTinhNghieng(yDinh, phamVi)
+4b. fallback lưu niên khi chỉ còn ban-menh — TRỪ phạm vi giai-doan
 5. chipSangNam sau gomLoiKhuyen: chỉ NORMAL, chỉ khi đang đọc năm hiện tại, tối đa 3 chip</t>
         </is>
       </c>
@@ -15895,7 +15896,7 @@
       </c>
       <c r="K186" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/planner.ts; lib/rag/tra-loi.ts (chipSangNam, namHieuLuc); lib/rag/nhat-ky.ts; lib/tuvi/bay-gio.ts (canChiCuaNam, namAmSapToi); app/api/hoi-dap/route.ts; lib/rag/bo-vang.ts; scripts/eval-planner.ts; scripts/test-rag-planner.ts</t>
+          <t>lib/rag/planner.ts; lib/rag/tra-loi.ts (chipSangNam, namHieuLuc, thangHieuLuc, canTinhNghieng); lib/rag/nhat-ky.ts; lib/tuvi/bay-gio.ts (canChiCuaNam, namAmSapToi); app/api/hoi-dap/route.ts; lib/rag/bo-vang.ts; scripts/eval-planner.ts; scripts/test-rag-planner.ts</t>
         </is>
       </c>
       <c r="L186" s="8" t="inlineStr">
@@ -15905,7 +15906,7 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>NỢ: (1) "tháng 3 / tháng tới" bật nguyệt hạn nhưng dữ kiện vẫn là tháng âm HIỆN TẠI — có từ trước vé, cần thangMucTieu. (2) Sổ "đã nói trước" (V3, tổng quan) khoá theo năm DƯƠNG, chat tra bằng năm âm → quanh Tết có thể lệch. (3) Mệnh bàn, /api/luan-giai, V3 vẫn mặc định năm dương. (4) Từ điển thực thể còn bí danh "năm tới" (đã chặn ở doanLopHan theo phạm vi). (5) Câu mô tả chặng dài vẫn có lưu niên dự phòng. (6) Chip vẫn tốn lượt. (7) Câu "sắp tới thế nào" giờ là mo-ta → không còn tính hướng nghiêng.</t>
+          <t>NỢ: (1) Sổ "đã nói trước" (V3, tổng quan) khoá theo năm DƯƠNG, chat tra bằng năm âm; mệnh bàn, /api/luan-giai, V3 vẫn mặc định năm dương → từ 01/01 tới Tết chat và các bề mặt khác lệch một năm. Ticket riêng, PHẢI xử lý trước 01/01/2027. (2) Từ điển thực thể còn bí danh "năm tới" (đã chặn ở doanLopHan theo phạm vi). (3) Chip vẫn tốn lượt (nợ sản phẩm). (4) "tháng 3" hỏi lúc tháng 8 vẫn hiểu là tháng 3 năm đang xem (đã qua), không đoán năm sau; tháng là tháng âm. Không có scanner "tháng đẹp nhất". (5) Bài dài cố định "Tôi là ai… cả đời" mất lưu niên dự phòng (đổi ngữ nghĩa có chủ đích).</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -15915,7 +15916,7 @@
       </c>
       <c r="O186" s="8" t="inlineStr">
         <is>
-          <t>(nhánh viec/cel-186-planner-time)</t>
+          <t>c5651d2 + sửa nghiệm thu lần 2 (nhánh viec/cel-186-planner-time)</t>
         </is>
       </c>
     </row>
@@ -18633,12 +18634,12 @@
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>quyet-dinh / co-khong / thoi-diem ⇒ LUÔN thêm dai-van; thêm luu-nien trừ khi phạm vi là giai-doan. Phạm vi gan / nam ⇒ dai-van + luu-nien; thang ⇒ nguyet-han. Bí danh PERIOD.LUU_NIEN của từ điển thực thể bị bỏ khi phạm vi giai-doan; PERIOD.NGUYET_HAN bị bỏ khi giai-doan hoặc gan. tra-cuu ⇒ thu về chỉ ban-menh, nhưng CHỈ khi luật không tìm thấy lớp hạn nào khác. Còn mỗi ban-menh thì thêm luu-nien dự phòng (giữ nguyên các bài dài cố định).</t>
+          <t>quyet-dinh / co-khong / thoi-diem ⇒ LUÔN thêm dai-van; thêm luu-nien trừ khi phạm vi là giai-doan. Phạm vi gan / nam ⇒ dai-van + luu-nien; thang ⇒ nguyet-han. Bí danh PERIOD.LUU_NIEN của từ điển thực thể bị bỏ khi phạm vi giai-doan; PERIOD.NGUYET_HAN bị bỏ khi giai-doan hoặc gan. tra-cuu ⇒ thu về chỉ ban-menh, nhưng CHỈ khi luật không tìm thấy lớp hạn nào khác. Còn mỗi ban-menh thì thêm luu-nien dự phòng — TRỪ khi phạm vi là giai-doan (bất biến: giai-doan không bao giờ có lưu niên / nguyệt hạn dự phòng).</t>
         </is>
       </c>
       <c r="F77" s="32" t="inlineStr">
         <is>
-          <t>Mọi câu "có nên" đều ngầm chứa "lúc này" — người ta không hỏi có nên nhận offer trên lý thuyết. Không có luật này thì câu quyết định chỉ đọc bản mệnh và bài trả lời thành một bản mô tả tính cách. tra-cuu là ý định DUY NHẤT làm THU HẸP lớp hạn, nên nhận nhầm ở đó đắt hơn hẳn: dữ kiện đại vận biến mất khỏi prompt mà không có gì báo. Hỏi "cả đời / sau này / những năm tới" mà trả bằng tiểu hạn một năm là vượt dữ kiện; nhưng "tương lai gần" thì phải có lưu niên — vì vậy "gần" thắng "tương lai". Đổi giai-doan sang không-có-lưu-niên VÔ ĐIỀU KIỆN từng làm bài dài cố định "Tôi là ai… cả đời" đổi lớp hạn (bắt được khi so lapKeHoach trước/sau trên mọi bề mặt).</t>
+          <t>Mọi câu "có nên" đều ngầm chứa "lúc này" — người ta không hỏi có nên nhận offer trên lý thuyết. Không có luật này thì câu quyết định chỉ đọc bản mệnh và bài trả lời thành một bản mô tả tính cách. tra-cuu là ý định DUY NHẤT làm THU HẸP lớp hạn, nên nhận nhầm ở đó đắt hơn hẳn: dữ kiện đại vận biến mất khỏi prompt mà không có gì báo. Hỏi "cả đời / sau này / những năm tới" mà trả bằng tiểu hạn một năm là vượt dữ kiện; nhưng "tương lai gần" thì phải có lưu niên — vì vậy "gần" thắng "tương lai". Đổi giai-doan sang không-có-lưu-niên VÔ ĐIỀU KIỆN từng làm bài dài cố định "Tôi là ai… cả đời" đổi lớp hạn (bắt được khi so lapKeHoach trước/sau trên mọi bề mặt). Lần nghiệm thu thứ hai: giữ 0 diff bằng cách để bài dài "cả đời" rơi về lưu niên là giữ một hành vi SAI — đã bỏ; bài dài đó giờ chỉ đọc bản mệnh.</t>
         </is>
       </c>
       <c r="G77" s="8" t="inlineStr">
@@ -18665,17 +18666,17 @@
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>Trục thời gian (phamViThoiGian + namMucTieu) và năm hiệu lực</t>
+          <t>Trục thời gian (phamViThoiGian + namMucTieu + thangMucTieu) và năm/tháng hiệu lực</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>doanPhamViThoiGian quét câu đã bỏ dấu trái→phải: năm 19xx/20xx → nam + namMucTieu (bỏ qua khi đứng sau "sinh"/"sinh năm"); "tháng" + 1–12 → thang; còn lại khớp cụm dài nhất 4→1 từ trong CUM_PHAM_VI; khi trùng nhiều phạm vi chọn theo UU_TIEN_PHAM_VI thang &gt; nam &gt; gan &gt; giai-doan. năm nay/năm tới/năm sau/sang năm/năm ngoái lệch 0/+1/+1/+1/−1 so với namXem (năm âm). Câu có/không: tách vế theo dấu câu, gọt đuôi chữ đệm + cụm thời gian NGUYÊN CỤM, vế kết bằng "không"/"chưa" và có ≥2 từ. tra-loi: namHieuLuc = keHoach.namMucTieu ?? vao.namXem cho chonBoiCanh, tinhNghiengVe, soKetLuanV3, ketLuanBaiTongQuan, nhật ký. chipSangNam: tháng âm ≥ 9 (≤4 tháng tới Tết), NORMAL, namHieuLuc = năm âm hiện tại, phạm vi gan/nam hoặc khong-ro với co-khong/thoi-diem/quyet-dinh, chưa có chip mang can chi/số năm → thêm "Sang năm &lt;Can Chi&gt; thì sao?" (đủ 3 thì thay chip cuối).</t>
+          <t>doanPhamViThoiGian quét câu đã bỏ dấu trái→phải: năm 19xx/20xx → nam + namMucTieu (bỏ qua khi đứng sau "sinh"/"sinh năm"); "tháng" + 1–12 → thang; còn lại khớp cụm dài nhất 4→1 từ trong CUM_PHAM_VI; khi trùng nhiều phạm vi chọn theo UU_TIEN_PHAM_VI thang &gt; nam &gt; gan &gt; giai-doan. năm nay/năm tới/năm sau/sang năm/năm ngoái lệch 0/+1/+1/+1/−1 so với namXem (năm âm). Câu có/không: tách vế theo dấu câu, gọt đuôi chữ đệm + cụm thời gian NGUYÊN CỤM, vế kết bằng "không"/"chưa" và có ≥2 từ. tra-loi: namHieuLuc = keHoach.namMucTieu ?? vao.namXem cho chonBoiCanh, tinhNghiengVe, soKetLuanV3, ketLuanBaiTongQuan, nhật ký. Tháng: "tháng N" → thangMucTieu N (năm giữ năm đang xem nếu không viết năm); tháng này / tháng tới / tháng sau lệch 0/+1/+1 so với thangXem (tháng âm), vượt 12 thì quay về 1 và namMucTieu = namXem+1; không có thangXem thì không đoán. thangHieuLuc = keHoach.thangMucTieu ?? vao.thangXem cho chonBoiCanh, tinhNghiengVe, nhật ký. canTinhNghieng: quyet-dinh / co-khong / thoi-diem luôn tính; mo-ta chỉ tính khi phạm vi gan / nam / thang; khong-ro và giai-doan không tính. chipSangNam: tháng âm ≥ 9 (≤4 tháng tới Tết), NORMAL, namHieuLuc = năm âm hiện tại, phạm vi gan/nam hoặc khong-ro với co-khong/thoi-diem/quyet-dinh, chưa có chip mang can chi/số năm → thêm "Sang năm &lt;Can Chi&gt; thì sao?" (đủ 3 thì thay chip cuối).</t>
         </is>
       </c>
       <c r="F78" s="32" t="inlineStr">
         <is>
-          <t>Thời gian là trục RIÊNG, không phải một ý định: "sắp tới tôi có người yêu không" là câu co-khong, không phải thoi-diem — trước vé, "sắp tới" nằm trong bảng thoi-diem nên câu có/không bị trả lời bằng mốc thời gian. Gọt mảnh thời gian TỪNG TỪ là bẫy ("không lãi", "không may" thành câu có/không) — phải gọt nguyên cụm. Đổi bảng cụm phải nâng PHIEN_BAN_PLANNER (đệm các bề mặt dùng kyCoPhienBan bị xả) và so lapKeHoach trước/sau trên câu cố định của mọi bề mặt. Năm xem của chat là năm ÂM: tuổi âm và lưu niên quanh Tết tính sai một năm nếu trộn năm dương.</t>
+          <t>Thời gian là trục RIÊNG, không phải một ý định: "sắp tới tôi có người yêu không" là câu co-khong, không phải thoi-diem — trước vé, "sắp tới" nằm trong bảng thoi-diem nên câu có/không bị trả lời bằng mốc thời gian. Gọt mảnh thời gian TỪNG TỪ là bẫy ("không lãi", "không may" thành câu có/không) — phải gọt nguyên cụm. Đổi bảng cụm phải nâng PHIEN_BAN_PLANNER (đệm các bề mặt dùng kyCoPhienBan bị xả) và so lapKeHoach trước/sau trên câu cố định của mọi bề mặt. Năm xem của chat là năm ÂM: tuổi âm và lưu niên quanh Tết tính sai một năm nếu trộn năm dương. Tách thời gian khỏi ý định từng làm "Công việc sắp tới thế nào?" (mo-ta) mất hướng nghiêng — hướng nghiêng phải đọc cả mốc, không chỉ ý định. Nguyệt hạn trước đây luôn đọc tháng HIỆN TẠI dù người dùng hỏi "tháng 3".</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
@@ -24105,7 +24106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28477,6 +28478,38 @@
         </is>
       </c>
       <c r="F136" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="49" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B137" s="50" t="inlineStr">
+        <is>
+          <t>c5651d2 + sửa nghiệm thu lần 2 (nhánh viec/cel-186-planner-time)</t>
+        </is>
+      </c>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>Vé A, sửa sau nghiệm thu lần 2: (1) canTinhNghieng — câu mô tả có mốc gần/năm/tháng vẫn tính hướng nghiêng; (2) giai-doan không còn rơi về lưu niên dự phòng (bài dài "Tôi là ai… cả đời" giờ chỉ ban-menh); (3) thangMucTieu + thangHieuLuc (tháng này/tới/sau/N/N năm Y, tháng 12 → tháng tới sang năm). PHIEN_BAN_PLANNER 2026.10.3; khi gộp xả 24 bản đệm mang hash production (điểm nổi bật 15, mốc 6, nhịp 3). Bộ vàng 98 câu, 100%.</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>Tách trục thời gian ở c5651d2 có ba hệ quả sai: "Công việc sắp tới thế nào?" thành mo-ta nên mất hướng nghiêng dù có mốc gần; bài dài "cả đời" được giữ 0 diff bằng cách vẫn rơi về tiểu hạn một năm — giữ số đẹp bằng hành vi sai; và "tháng 3" bật nguyệt hạn nhưng đọc tháng hiện tại. Chủ dự án yêu cầu sửa cả ba trong vé A, không để nợ.</t>
+        </is>
+      </c>
+      <c r="F137" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
CEL-186 ve A: nam sinh viet so khong con thanh nam duoc hoi
- Nam so tran chi la namMucTieu khi dung dau cau / sau tu chi moc va khong lui qua mot nam; "nam N" viet ro thang nam tran
- Truoc day "Toi 1995, nam nay..." doc tieu han nam 1995 o tuoi am 1 hoac am (bat o tham dinh celes-domain truoc merge)
- PHIEN_BAN_PLANNER 2026.10.4; bo vang 100 cau, 100%; 120 cau co dinh 0 doi so voi 2c8963c
- HUONG-DAN: bo vang 62 -> 100 cau; backlog ghi hash commit

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15856,7 +15856,7 @@
       </c>
       <c r="D186" s="8" t="inlineStr">
         <is>
-          <t>Planner có trục thứ ba phamViThoiGian (khong-ro / gan / thang / nam / giai-doan), TÁCH khỏi ý định, kèm namMucTieu (năm viết số, hoặc năm nay / năm tới / năm sau / sang năm / năm ngoái tính từ năm xem). "Tương lai gần / sắp tới" là gan, thắng chữ "tương lai" (giai-doan). Nhận câu có/không theo vế, gọt đuôi chữ đệm và cụm thời gian (thay luật 3 từ cuối). Có thêm thangMucTieu (tháng này / tháng tới / tháng sau tính từ tháng âm đang xem, tháng 12 → tháng tới sang tháng 1 năm sau; "tháng N" giữ năm đang xem trừ khi viết năm). Mỗi lượt chat đọc một namHieuLuc = namMucTieu ?? namXem và thangHieuLuc = thangMucTieu ?? thangXem. Hướng nghiêng tính theo ý định VÀ mốc: câu mô tả có mốc gần / năm / tháng ("Công việc sắp tới thế nào?") vẫn tính; mô tả không mốc hoặc chặng dài thì không. Chặng dài (giai-doan) không bao giờ rơi về lưu niên / nguyệt hạn dự phòng. Chat mặc định năm ÂM hiện tại. Từ tháng âm 9 tới Tết thêm chip "Sang năm &lt;Can Chi&gt; thì sao?".</t>
+          <t>Planner có trục thứ ba phamViThoiGian (khong-ro / gan / thang / nam / giai-doan), TÁCH khỏi ý định, kèm namMucTieu (năm viết số, hoặc năm nay / năm tới / năm sau / sang năm / năm ngoái tính từ năm xem). "Tương lai gần / sắp tới" là gan, thắng chữ "tương lai" (giai-doan). Nhận câu có/không theo vế, gọt đuôi chữ đệm và cụm thời gian (thay luật 3 từ cuối). Năm số đứng trần (không có chữ "năm") chỉ là năm được hỏi khi đứng đầu câu hoặc sau từ chỉ mốc (đến / vào / cuối / đầu / từ / trước / sau…) và không lùi quá một năm so với năm xem — "Tôi 1995", "bố tôi 1965", "3/5/1995" là năm sinh, không bao giờ thành năm mục tiêu. Có thêm thangMucTieu (tháng này / tháng tới / tháng sau tính từ tháng âm đang xem, tháng 12 → tháng tới sang tháng 1 năm sau; "tháng N" giữ năm đang xem trừ khi viết năm). Mỗi lượt chat đọc một namHieuLuc = namMucTieu ?? namXem và thangHieuLuc = thangMucTieu ?? thangXem. Hướng nghiêng tính theo ý định VÀ mốc: câu mô tả có mốc gần / năm / tháng ("Công việc sắp tới thế nào?") vẫn tính; mô tả không mốc hoặc chặng dài thì không. Chặng dài (giai-doan) không bao giờ rơi về lưu niên / nguyệt hạn dự phòng. Chat mặc định năm ÂM hiện tại. Từ tháng âm 9 tới Tết thêm chip "Sang năm &lt;Can Chi&gt; thì sao?".</t>
         </is>
       </c>
       <c r="E186" s="8" t="inlineStr">
@@ -15916,7 +15916,7 @@
       </c>
       <c r="O186" s="8" t="inlineStr">
         <is>
-          <t>c5651d2 + sửa nghiệm thu lần 2 (nhánh viec/cel-186-planner-time)</t>
+          <t>c5651d2, 2c8963c + chặn năm sinh (nhánh viec/cel-186-planner-time)</t>
         </is>
       </c>
     </row>
@@ -18671,12 +18671,12 @@
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>doanPhamViThoiGian quét câu đã bỏ dấu trái→phải: năm 19xx/20xx → nam + namMucTieu (bỏ qua khi đứng sau "sinh"/"sinh năm"); "tháng" + 1–12 → thang; còn lại khớp cụm dài nhất 4→1 từ trong CUM_PHAM_VI; khi trùng nhiều phạm vi chọn theo UU_TIEN_PHAM_VI thang &gt; nam &gt; gan &gt; giai-doan. năm nay/năm tới/năm sau/sang năm/năm ngoái lệch 0/+1/+1/+1/−1 so với namXem (năm âm). Câu có/không: tách vế theo dấu câu, gọt đuôi chữ đệm + cụm thời gian NGUYÊN CỤM, vế kết bằng "không"/"chưa" và có ≥2 từ. tra-loi: namHieuLuc = keHoach.namMucTieu ?? vao.namXem cho chonBoiCanh, tinhNghiengVe, soKetLuanV3, ketLuanBaiTongQuan, nhật ký. Tháng: "tháng N" → thangMucTieu N (năm giữ năm đang xem nếu không viết năm); tháng này / tháng tới / tháng sau lệch 0/+1/+1 so với thangXem (tháng âm), vượt 12 thì quay về 1 và namMucTieu = namXem+1; không có thangXem thì không đoán. thangHieuLuc = keHoach.thangMucTieu ?? vao.thangXem cho chonBoiCanh, tinhNghiengVe, nhật ký. canTinhNghieng: quyet-dinh / co-khong / thoi-diem luôn tính; mo-ta chỉ tính khi phạm vi gan / nam / thang; khong-ro và giai-doan không tính. chipSangNam: tháng âm ≥ 9 (≤4 tháng tới Tết), NORMAL, namHieuLuc = năm âm hiện tại, phạm vi gan/nam hoặc khong-ro với co-khong/thoi-diem/quyet-dinh, chưa có chip mang can chi/số năm → thêm "Sang năm &lt;Can Chi&gt; thì sao?" (đủ 3 thì thay chip cuối).</t>
+          <t>doanPhamViThoiGian quét câu đã bỏ dấu trái→phải: "năm" + 19xx/20xx → nam + namMucTieu (bỏ qua "sinh năm" / "tuổi năm"); năm số TRẦN chỉ tính khi đứng đầu câu hoặc sau từ chỉ mốc trong TRUOC_NAM_HOI (danh sách cho phép; "tới" vắng vì bỏ dấu trùng "tôi") và ≥ namXem−1, và chỉ dùng khi không có năm nào viết rõ; "tháng" + 1–12 → thang; còn lại khớp cụm dài nhất 4→1 từ trong CUM_PHAM_VI; khi trùng nhiều phạm vi chọn theo UU_TIEN_PHAM_VI thang &gt; nam &gt; gan &gt; giai-doan. năm nay/năm tới/năm sau/sang năm/năm ngoái lệch 0/+1/+1/+1/−1 so với namXem (năm âm). Câu có/không: tách vế theo dấu câu, gọt đuôi chữ đệm + cụm thời gian NGUYÊN CỤM, vế kết bằng "không"/"chưa" và có ≥2 từ. tra-loi: namHieuLuc = keHoach.namMucTieu ?? vao.namXem cho chonBoiCanh, tinhNghiengVe, soKetLuanV3, ketLuanBaiTongQuan, nhật ký. Tháng: "tháng N" → thangMucTieu N (năm giữ năm đang xem nếu không viết năm); tháng này / tháng tới / tháng sau lệch 0/+1/+1 so với thangXem (tháng âm), vượt 12 thì quay về 1 và namMucTieu = namXem+1; không có thangXem thì không đoán. thangHieuLuc = keHoach.thangMucTieu ?? vao.thangXem cho chonBoiCanh, tinhNghiengVe, nhật ký. canTinhNghieng: quyet-dinh / co-khong / thoi-diem luôn tính; mo-ta chỉ tính khi phạm vi gan / nam / thang; khong-ro và giai-doan không tính. chipSangNam: tháng âm ≥ 9 (≤4 tháng tới Tết), NORMAL, namHieuLuc = năm âm hiện tại, phạm vi gan/nam hoặc khong-ro với co-khong/thoi-diem/quyet-dinh, chưa có chip mang can chi/số năm → thêm "Sang năm &lt;Can Chi&gt; thì sao?" (đủ 3 thì thay chip cuối).</t>
         </is>
       </c>
       <c r="F78" s="32" t="inlineStr">
         <is>
-          <t>Thời gian là trục RIÊNG, không phải một ý định: "sắp tới tôi có người yêu không" là câu co-khong, không phải thoi-diem — trước vé, "sắp tới" nằm trong bảng thoi-diem nên câu có/không bị trả lời bằng mốc thời gian. Gọt mảnh thời gian TỪNG TỪ là bẫy ("không lãi", "không may" thành câu có/không) — phải gọt nguyên cụm. Đổi bảng cụm phải nâng PHIEN_BAN_PLANNER (đệm các bề mặt dùng kyCoPhienBan bị xả) và so lapKeHoach trước/sau trên câu cố định của mọi bề mặt. Năm xem của chat là năm ÂM: tuổi âm và lưu niên quanh Tết tính sai một năm nếu trộn năm dương. Tách thời gian khỏi ý định từng làm "Công việc sắp tới thế nào?" (mo-ta) mất hướng nghiêng — hướng nghiêng phải đọc cả mốc, không chỉ ý định. Nguyệt hạn trước đây luôn đọc tháng HIỆN TẠI dù người dùng hỏi "tháng 3".</t>
+          <t>Thời gian là trục RIÊNG, không phải một ý định: "sắp tới tôi có người yêu không" là câu co-khong, không phải thoi-diem — trước vé, "sắp tới" nằm trong bảng thoi-diem nên câu có/không bị trả lời bằng mốc thời gian. Gọt mảnh thời gian TỪNG TỪ là bẫy ("không lãi", "không may" thành câu có/không) — phải gọt nguyên cụm. Đổi bảng cụm phải nâng PHIEN_BAN_PLANNER (đệm các bề mặt dùng kyCoPhienBan bị xả) và so lapKeHoach trước/sau trên câu cố định của mọi bề mặt. Năm xem của chat là năm ÂM: tuổi âm và lưu niên quanh Tết tính sai một năm nếu trộn năm dương. Tách thời gian khỏi ý định từng làm "Công việc sắp tới thế nào?" (mo-ta) mất hướng nghiêng — hướng nghiêng phải đọc cả mốc, không chỉ ý định. Nguyệt hạn trước đây luôn đọc tháng HIỆN TẠI dù người dùng hỏi "tháng 3". Năm số trần từng được nhận hết (trừ sau "sinh"): "Tôi 1995, năm nay…" đọc tiểu hạn năm 1995 ở tuổi âm 1 hoặc âm — bắt được ở thẩm định celes-domain trước merge. Dùng danh sách CHO PHÉP vì cách viết năm sinh là vô hạn.</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
@@ -24106,7 +24106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F137"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28459,7 +28459,7 @@
       </c>
       <c r="B136" s="50" t="inlineStr">
         <is>
-          <t>(nhánh viec/cel-186-planner-time)</t>
+          <t>c5651d2 (nhánh viec/cel-186-planner-time)</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
@@ -28491,7 +28491,7 @@
       </c>
       <c r="B137" s="50" t="inlineStr">
         <is>
-          <t>c5651d2 + sửa nghiệm thu lần 2 (nhánh viec/cel-186-planner-time)</t>
+          <t>2c8963c (nhánh viec/cel-186-planner-time)</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
@@ -28510,6 +28510,38 @@
         </is>
       </c>
       <c r="F137" s="8" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="49" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B138" s="50" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-planner-time, sau merge origin/main 40b4b71)</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="inlineStr">
+        <is>
+          <t>Vé A, chặn năm sinh: năm số trần chỉ thành namMucTieu khi đứng đầu câu / sau từ chỉ mốc và không lùi quá một năm; "năm N" viết rõ thắng năm trần. PHIEN_BAN_PLANNER 2026.10.4. Bộ vàng 100 câu, 100%; 120 câu cố định 0 đổi so với 2c8963c.</t>
+        </is>
+      </c>
+      <c r="E138" s="8" t="inlineStr">
+        <is>
+          <t>Thẩm định celes-domain trước merge: "Tôi 1995, năm nay có cưới không?", "bố tôi 1965 …", "sinh ngày 3/5/1995 …" đều lấy năm sinh làm năm hiệu lực → dữ kiện tiểu hạn ở tuổi âm 1 hoặc âm. Lỗi do chính vé A sinh ra (trước vé, chat luôn đọc năm đang xem), nên sửa trong vé A chứ không để nợ.</t>
+        </is>
+      </c>
+      <c r="F138" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
         </is>

</xml_diff>

<commit_message>
TOOL: test-man-hinh do o trang thai khach that + checklist UI (P1-P5)
- Dung (exit 2) neu Supabase tat / da dang nhap; ep tieng Viet qua acceptLanguage
- Anh toan trang CDP (captureBeyondViewport) vao .anh-man-hinh/, tu kiem chieu cao
- Vung cham theo hop dong globals.css: hop DOM >= 44px; ::after cua .nav-link/.link-text
- CLS = cua so phien lon nhat (gap >1s / >5s, bo hadRecentInput), nguong 0,1
- docs/thiet-ke/celes-ui-quality-checklist.md: luat khong mang gu tham my

Vi sao: tran 404px voi khach (23/09) va CLS 0,34 (27/09) lot vi bo do cu chay
voi Supabase tat va khong do CLS. Quyet dinh docs/chien-luoc/cong-cu-thiet-ke-2026-10.md.
Lan chay dau bao 17 SAI la no UI co san (pill-tag 32, btn-sm 37-39, logo 24) -
bao trung thuc, tach ve sua CSS rieng. Khong dua vao CI.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -24553,7 +24553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29055,6 +29055,34 @@
       <c r="F140" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>(nhánh viec/test-man-hinh)</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Bộ đo giao diện scripts/test-man-hinh.mjs (chạy tay, local, chưa vào CI): đo ở trạng thái KHÁCH thật và dừng (exit 2) nếu Supabase tắt hoặc đã đăng nhập; ép tiếng Việt; chụp ảnh toàn trang bằng CDP vào .anh-man-hinh/ (gitignore) và tự kiểm chiều cao ảnh; vùng chạm theo hợp đồng globals.css ở pointer: coarse — hộp DOM cao ≥ 44px cho nút/.btn-*/.link-action/điều khiển riêng, ::after ≥ 44px cho .nav-link/.link-text, bỏ link giữa câu, mở panel Menu để đo; CLS = cửa sổ phiên lớn nhất ≤ 0,1. Thêm docs/thiet-ke/celes-ui-quality-checklist.md (luật không mang gu thẩm mỹ).</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Hai lỗi đã lọt vì bộ đo cũ: thanh điều hướng tràn 404px trên iPhone với khách (23/09) nằm im vì mọi lần đo chạy với Supabase tắt (ai cũng thành admin, không có nút Đăng nhập); CLS 0,34 ở /la-so (27/09) không ảnh tĩnh nào bắt được. Quyết định 03/10/2026 (docs/chien-luoc/cong-cu-thiet-ke-2026-10.md): không cài design skill/Playwright, không thêm khách giả lập vào code quyền, biến lỗi đã lọt thành phép đo. Chủ dự án chọn báo SAI trung thực, không danh sách 'đã biết'. Lần chạy đầu (03/10) phát hiện nợ UI có sẵn: .pill-tag 32px (đổi ngôn ngữ, theme), .btn-sm 37–39px, link logo 24px — đây là kết quả hợp lệ của bộ đo, tách vé sửa CSS riêng. Bài thử CLS tổng hợp: dịch 0,033 rồi 0,073 cách 1,5s → đo 0,073 (cộng tổng sẽ ra 0,106 và báo sai).</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FIX: CEL-189 tach dem noi_dung_ai theo moi truong (prod / Preview / local)
- lib/moi-truong-dem.ts: nguon su that duy nhat; production chi khi VERCEL=1 +
  VERCEL_ENV=production + NODE_ENV=production; Preview 'preview:<nhanh>-<bam8>:',
  con lai 'local:<ten>:'. Production giu khoa cu (ns rong), khong migration.
- noi-dung-ai.ts gan/cat tien to o moi ham doc-ghi + dem RAM; tienTo rong tra
  null/[]; xoaDemLaSo xoa dung la so + be mat + pham vi, tu choi be mat cau hinh.
- gioi-han-khach di qua module dem (so dem tach theo moi truong).
- Cau hinh (thu-vien, mau-giong, cau-hinh-v3) doc chung, ghi ngoai production
  nem LoiNgoaiProduction; route admin tra 403.
- Script chay tay mac dinh local, co dong lenh --ghi-production moi ghi production.
- /api/phien-ban them phamViDem; kiem-moi-truong kiem ca hai truong + bao do
  khi .env.local co VERCEL/VERCEL_ENV.
- CI: scripts/test-moi-truong-dem.ts (55 ca, Supabase gia, offline).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O187"/>
+  <dimension ref="A1:O188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15997,6 +15997,83 @@
         </is>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>D. Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Tách đệm AI theo môi trường (production / Preview / local) trên bảng noi_dung_ai</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Production, Preview và local dùng chung một Supabase. Mọi khoá kỳ đi qua lib/rag/noi-dung-ai.ts được gắn tiền tố phạm vi: production '' (khoá cũ y nguyên, không migration, không xả đệm), Preview 'preview:&lt;slug nhánh&gt;-&lt;băm 8&gt;:', local 'local:&lt;CELES_CACHE_NAMESPACE|local&gt;:'. Sổ đếm giới hạn khách (gioi-han-khach) tách theo cùng luật. Cấu hình dùng chung (thu-vien, mau-giong, cau-hinh-v3) đọc chung, chỉ production được ghi/xoá (route admin trả 403). /api/phien-ban có thêm trường phamViDem.</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>1. lib/moi-truong-dem.ts: phamViDem() tính lúc gọi; production chỉ khi VERCEL=1 + VERCEL_ENV=production + NODE_ENV=production. 2. noi-dung-ai.ts gắn ns ở docNoiDung/luuNoiDung/docNoiDungMoiNhat/docNhieuTheoTienTo/đệm RAM, cắt ns khỏi khoá trả ra; tienTo rỗng → null/[]. 3. Script gọi khaiBaoScript(argv): mặc định local, --ghi-production mới ghi production. 4. xoaDemLaSo xoá đúng lá số + bề mặt + phạm vi, từ chối bề mặt cấu hình. 5. scripts/test-moi-truong-dem.ts (CI, Supabase giả).</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Chờ nghiệm thu</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Không sinh nội dung</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Mọi bậc</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Mọi bề mặt AI có đệm; /api/phien-ban; /api/admin/cau-hinh-luan-giai</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>lib/moi-truong-dem.ts; lib/rag/noi-dung-ai.ts; lib/auth/gioi-han-khach.ts; lib/rag/thu-vien/kho.ts; lib/rag/v3/mau-giong.ts; lib/rag/v3/cau-hinh.ts; app/api/phien-ban/route.ts; scripts/chay-lai-luan-giai.ts; scripts/test-moi-truong-dem.ts</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>Sau deploy production phải mở /api/phien-ban thấy moiTruong=production và phamViDem=production, lệch thì coi deploy hỏng. Preview mới luôn đệm trống (sinh lại tốn lượt model) — không prewarm, soat-chi-phi trước mọi lượt sinh lớn. Không dọn được các bản Preview/local đã ghi bẩn vào production trước đây. Hạn mức gọi model, hội thoại, tài khoản vẫn chung DB (không thuộc việc này). next build &amp;&amp; next start ở local với .env.local có VERCEL=1 + VERCEL_ENV=production vẫn thành production — kiem-moi-truong.ts báo đỏ.</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>(nhánh viec/fix-noi-dung-ai-env)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16014,7 +16091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G234"/>
+  <dimension ref="A1:G239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -24541,6 +24618,191 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Tách đệm theo môi trường</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Nhận diện môi trường</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>phamViDem(env) trong lib/moi-truong-dem.ts là nguồn sự thật duy nhất. Script đã khaiBaoScript thì theo cờ dòng lệnh. Không thì: VERCEL=1 + NODE_ENV=production + VERCEL_ENV=production → production ns ''; + VERCEL_ENV=preview → preview:&lt;slug(ref)&gt;-&lt;sha256(ref) 8&gt;:; còn lại local:&lt;slug(CELES_CACHE_NAMESPACE)|local&gt;:. Slug chỉ [a-z0-9-].</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>KHÔNG CHỈ DỰA VÀO VERCEL_ENV: .env.local chép VERCEL_ENV=production (vercel env pull) là next dev thành production. next dev ép NODE_ENV=development nên ba điều kiện cùng lúc mới chặn được. Không module nào khác tự đọc VERCEL_ENV.</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>lib/moi-truong-dem.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Tách đệm theo môi trường</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Gắn và cắt namespace trong module đệm</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>khoaThat(khoaKy) = ns + khoaKy ở docNoiDung, luuNoiDung, khoá đệm RAM. docNoiDungMoiNhat / docNhieuTheoTienTo LIKE '&lt;ns&gt;&lt;tienTo&gt;%' và cắt ns khỏi khoaKy trả ra. tienTo rỗng → null / []. gioi-han-khach đọc/ghi qua docNhieuTheoTienTo + luuNoiDung.</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>NƠI GỌI KHÔNG BAO GIỜ THẤY TIỀN TỐ: xu-ly.ts, so-ket-luan.ts, diem-noi-bat cắt chuỗi trên khoaKy trả ra. LIKE '%' (tienTo rỗng) khớp khoá của mọi môi trường — phải trả rỗng, không ném (hợp đồng module là im lặng).</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>lib/rag/noi-dung-ai.ts; lib/auth/gioi-han-khach.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Tách đệm theo môi trường</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Cấu hình dùng chung chỉ production ghi</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>thu-vien, mau-giong, cau-hinh-v3 đọc không namespace. luuThuVien, dongGoi, xoaDotTrich, luuMauGiong, luuCauHinhV3 gọi chanGhiNgoaiProduction trước khi chạm DB → ném LoiNgoaiProduction. POST /api/admin/cau-hinh-luan-giai trả 403 ngoài production.</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>CHẶN Ở SERVER, KHÔNG CHỈ ẨN UI: local có service role key trỏ production vẫn không ghi được cấu hình.</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/kho.ts; lib/rag/v3/mau-giong.ts; lib/rag/v3/cau-hinh.ts; app/api/admin/cau-hinh-luan-giai/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Tách đệm theo môi trường</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Script chạy tay: cờ --ghi-production</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>chay-lai-luan-giai.ts, dung-thu-vien.ts, nap-mau-giong.ts gọi khaiBaoScript(process.argv): không cờ → local (bỏ qua VERCEL* trong env), có --ghi-production → production. chay-lai-luan-giai xoá qua xoaDemLaSo: đúng chart_hash, 3 bề mặt nó sinh lại + nhip-hien-tai, moc-giai-doan/nam/thang, ban-doc-sau (cùng kỳ, để không lệch nhau); không xoá chat, luan-giai-v3, cấu hình, sổ đếm khách, production thì loại khoá preview:/local:, ngoài production chỉ khoá mang ns của mình. dung-thu-vien kiểm cờ ngay đầu, trước khi tốn lượt model.</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>CỜ DÒNG LỆNH, KHÔNG BIẾN MÔI TRƯỜNG: script và next dev cùng nạp .env.local. Trước đây chay-lai-luan-giai xoá MỌI bản của lá số theo chart_hash — chạy ở local là xoá đệm production.</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>scripts/chay-lai-luan-giai.ts; scripts/dung-thu-vien.ts; scripts/nap-mau-giong.ts; lib/rag/noi-dung-ai.ts (xoaDemLaSo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Tách đệm theo môi trường</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Cổng sau deploy</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>/api/phien-ban trả thêm phamViDem (production / preview:&lt;nhánh&gt;-&lt;băm&gt; / local:&lt;tên&gt;), không bí mật. Sau mỗi deploy production chạm đệm: commit đúng, nhanh=main, moiTruong=production, phamViDem=production. kiem-moi-truong.ts kiểm hai trường này và báo đỏ nếu .env.local có VERCEL / VERCEL_ENV.</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>LỆCH LÀ DEPLOY HỎNG: production đọc nhầm phạm vi là mọi người dùng thấy đệm trống và sinh lại toàn bộ — không chạy sinh/xoá đệm nào cho tới khi sửa.</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>app/api/phien-ban/route.ts; scripts/kiem-moi-truong.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24553,7 +24815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29055,6 +29317,38 @@
       <c r="F140" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>(nhánh viec/fix-noi-dung-ai-env)</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Tách đệm noi_dung_ai theo môi trường bằng tiền tố khoa_ky (production giữ khoá cũ); gioi-han-khach theo cùng luật; cấu hình đọc chung, chỉ production ghi; script mặc định local, --ghi-production mới ghi production; xoá đệm của script lọc đúng phạm vi; /api/phien-ban thêm phamViDem; bài CI test-moi-truong-dem (55 ca).</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Phiên chiến lược 03/10/2026 (docs/chien-luoc/moi-truong-phat-trien-2026-10.md): Preview đọc trúng bài cũ của production nên chủ dự án nghiệm thu thấy nội dung cũ; Preview/local ghi đè đệm production; chay-lai-luan-giai.ts xoá mọi bản của lá số theo chart_hash nên chạy ở local là xoá đệm production. Chủ dự án quyết sửa trước CEL-186 vé B, coi mọi runtime không phải Vercel Production là nguy hiểm, cờ dòng lệnh thay vì biến môi trường, chấp nhận Preview đệm trống, không prewarm.</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DOCS: CEL-186 ve B — AGENTS, HUONG-DAN, backlog 3 sheet; luot loi cung gan nhan @test
- AGENTS.md: ban do ma lib/rag/focused/, them test-du-kien / test-focused (CI) va eval-focused.
- HUONG-DAN.md: bien CELES_FOCUSED_CHAT va bo bien eval (AI_GHIM_MODEL, AI_TRAN_USD...), doan
  mo ta duong Focused.
- PRODUCT-BACKLOG.xlsx: sua dong CEL-186 (ve B, trang thai, viec con lai), them 7 buoc Logic
  "Ve B — chat Focused", 1 dong Nhat ky.
- fallback.ts: luot loi (AiRetryableError) cung ghi "<model>@test" khi AI_NHAN dat.
- eval-focused.ts: ghi chu tran tinh lai tu 0 moi tien trinh, embedding ngoai tran, Gemini free.

Vi sao: soat-chi-phi chi ra luot loi cua eval lan vao so lieu nguoi dung that, va chay tach
--chi-ca / --chi-barnum co the vuot $2 tong neu dat tran moi lan $2 (co #8).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15851,7 +15851,7 @@
       </c>
       <c r="C186" s="8" t="inlineStr">
         <is>
-          <t>Trục thời gian của câu hỏi (planner) + năm/tháng hiệu lực + chip "Sang năm"</t>
+          <t>Trục thời gian của câu hỏi (planner) + năm/tháng hiệu lực + chip "Sang năm" · Vé B: chat Focused sau cờ CELES_FOCUSED_CHAT</t>
         </is>
       </c>
       <c r="D186" s="8" t="inlineStr">
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Đang chạy (nhánh, chờ nghiệm thu)</t>
+          <t>Vé A: đang chạy (nhánh, chờ nghiệm thu). Vé B: code xong trên nhánh viec/cel-186-focused-chat, cờ TẮT; chưa bật Preview, chưa eval model thật, chưa merge (chờ fix noi_dung_ai vào main)</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -15896,17 +15896,17 @@
       </c>
       <c r="K186" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/planner.ts; lib/rag/tra-loi.ts (chipSangNam, namHieuLuc, thangHieuLuc, canTinhNghieng); lib/rag/nhat-ky.ts; lib/tuvi/bay-gio.ts (canChiCuaNam, namAmSapToi); app/api/hoi-dap/route.ts; lib/rag/bo-vang.ts; scripts/eval-planner.ts; scripts/test-rag-planner.ts</t>
+          <t>lib/rag/planner.ts; lib/rag/tra-loi.ts (chipSangNam, namHieuLuc, thangHieuLuc, canTinhNghieng, nhánh focusedBat); lib/rag/focused/* (Vé B); lib/ai/fallback.ts (AI_GHIM_MODEL, AI_TRAN_USD — chỉ script eval); lib/rag/nhat-ky.ts; lib/tuvi/bay-gio.ts; app/api/hoi-dap/route.ts; lib/rag/bo-vang.ts; scripts/eval-planner.ts; scripts/test-rag-planner.ts; scripts/test-focused.ts; scripts/test-du-kien.ts; scripts/eval-focused.ts</t>
         </is>
       </c>
       <c r="L186" s="8" t="inlineStr">
         <is>
-          <t>Luôn bật</t>
+          <t>Vé A: luôn bật. Vé B: CELES_FOCUSED_CHAT=1 (đọc mỗi lượt); thiếu/khác 1 = đường STANDARD nguyên vẹn</t>
         </is>
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>NỢ: (1) Sổ "đã nói trước" (V3, tổng quan) khoá theo năm DƯƠNG, chat tra bằng năm âm; mệnh bàn, /api/luan-giai, V3 vẫn mặc định năm dương → từ 01/01 tới Tết chat và các bề mặt khác lệch một năm. Ticket riêng, PHẢI xử lý trước 01/01/2027. (2) Từ điển thực thể còn bí danh "năm tới" (đã chặn ở doanLopHan theo phạm vi). (3) Chip vẫn tốn lượt (nợ sản phẩm). (4) "tháng 3" hỏi lúc tháng 8 vẫn hiểu là tháng 3 năm đang xem (đã qua), không đoán năm sau; tháng là tháng âm. Không có scanner "tháng đẹp nhất". (5) Bài dài cố định "Tôi là ai… cả đời" mất lưu niên dự phòng (đổi ngữ nghĩa có chủ đích).</t>
+          <t>NỢ: (1) Sổ "đã nói trước" (V3, tổng quan) khoá theo năm DƯƠNG, chat tra bằng năm âm; mệnh bàn, /api/luan-giai, V3 vẫn mặc định năm dương → từ 01/01 tới Tết chat và các bề mặt khác lệch một năm. Ticket riêng, PHẢI xử lý trước 01/01/2027. (2) Từ điển thực thể còn bí danh "năm tới" (đã chặn ở doanLopHan theo phạm vi). (3) Chip vẫn tốn lượt (nợ sản phẩm; F2 do mã viết cũng trừ lượt — cờ #4). (4) "tháng 3" hỏi lúc tháng 8 vẫn hiểu là tháng 3 năm đang xem (đã qua), không đoán năm sau; tháng là tháng âm. Không có scanner "tháng đẹp nhất". (5) Bài dài cố định "Tôi là ai… cả đời" mất lưu niên dự phòng (đổi ngữ nghĩa có chủ đích). VÉ B còn: sau khi fix noi_dung_ai vào main → merge origin/main (không rebase) → regression → bật env Preview RIÊNG nhánh → eval-focused (≤ $2, model Production ghim) → Barnum 6×6 → celes-domain → bien-tap-vi → qa → soat-tai-lieu → UAT → mới trình merge. Lệch đã biết: chip "Tháng X nhuận" vẫn đọc nguyệt hạn tháng thường (engine không có nguyệt hạn tháng nhuận); chip N2 "Tháng N năm sau thì sao?" chưa làm; chipTruoc lấy xấp xỉ từ câu người dùng (chip không nằm trong lịch sử).</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -16014,7 +16014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G234"/>
+  <dimension ref="A1:G241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -24541,6 +24541,265 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Cờ và điểm nối</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Đầu traLoiCoCanCu: focusedBat() (CELES_FOCUSED_CHAT === '1', đọc mỗi lượt) thì gọi traLoiFocused, ngược lại đi STANDARD như cũ. phienBan thêm focused=&lt;khuôn&gt; và phienBanFocused chỉ ở đường Focused.</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Cờ tắt thì STANDARD phải trùng từng byte (test-du-kien, test-focused). Không sửa planner.ts, prompt-co-can-cu.ts. Không thêm khoá đệm.</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>lib/rag/tra-loi.ts; lib/rag/focused/tra-loi-focused.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Người được hỏi + kế thừa chủ đề qua chip</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>nhanDangDoiTuong: con / bố mẹ / anh em / vợ chồng… → đúng cung lục thân; "con", "em" xưng hô và "bản thân" không phải người khác. Chip giữ chủ đề ở server (lapKeHoachFocused); câu mới có chủ đề thì tin câu mới.</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Cờ #1, #2. Không gán vận của người khác cho người hỏi.</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/doi-tuong.ts; lib/rag/focused/ke-thua.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Phân khuôn + câu do mã viết</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào, E A hay B, F1 quan hệ, F2 vận riêng người khác, G không hướng. F2, D, tháng nhuận cần hỏi lại: mã trả trọn lượt (provider 'ma', model focused-f2/-d/-nhuan), không truy hồi, không gọi model, vẫn trừ lượt. E, N2 tháng đã qua, N4 cuối năm: câu mã đứng đầu, model viết phần sau.</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Cờ #3, #4, #5: bỏ D′ và chip "Tháng nào đáng chú ý hơn?" (engine không so tháng → ngõ cụt).</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/phan-loai.ts; lib/rag/focused/cau-ma.ts; lib/rag/focused/thang-am.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Prompt riêng + chốt hướng</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>dungPromptFocused: KHOI_GIONG_CELES, khối nghiêng chỉ giữ đầu mốc có trong gói và lớp có F### trong gói, khối mốc thời gian tính sẵn. Không dùng Dấu ấn / DAN_LUAN / luật độ dài STANDARD. Chiều kết luận do mã chốt (nhomCuaHuong); câu chốt ngược chiều hoặc trượt guard thì thay bằng cauChotDuPhong.</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Cờ #9. DEEP chỉ nới độ dài, giữ mọi guard (cờ #6).</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/prompt.ts; lib/rag/focused/chot-huong.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Guard từng câu + độ dài</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>kiemLuot: bỏ câu có tên ngoài gói, lưu hoá, tên cung lộ, giọng máy, phán quyết, khuyên/chọn hộ, mốc lạ, "sẽ" ở tháng đã qua, quá phía ngược. NORMAL 2–4 câu (tính cả câu mã), trần 120 âm tiết, vượt thì bỏ câu không căn cứ trước; vượt 140 thì thử lại. SENSITIVE không cắt, nối miễn trừ sau guard.</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Không giữ câu lỗi — câu hỏng thì bỏ, không sửa nghĩa.</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/kiem.ts; lib/rag/focused/quet-ten.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Thử lại → 502 + hoàn lượt</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>chayFocused gọi model tối đa 2 lần trong hạn 50s. Hết câu CÓ CĂN CỨ (mã F### thật trong gói) hoặc JSON gãy thì thử lại 1 lần; vẫn hỏng thì van rỗng → route trả 502 và hoàn lượt.</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Bản đầu chỉ thử lại khi hết MỌI câu, nên một bản toàn câu không căn cứ vẫn lọt — sửa ở 00b3988, có test offline tiêm model giả.</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/chay.ts; app/api/hoi-dap/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Eval model thật có trần</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>scripts/eval-focused.ts gọi traLoiCoCanCu trong tiến trình, tuần tự, lá số đóng băng. Bắt buộc AI_GHIM_MODEL (mọi lời gọi chỉ dùng model đó, không lùi) và AI_TRAN_USD ≤ 2 + giá vào/ra: giữ chỗ bi quan trước mỗi lời gọi, vượt trần ném VuotNganSachError trước khi gọi → dừng cả bộ.</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Cờ #8: tổng eval vé B ≤ $2, đúng model Production. Chỉ chạy sau fix noi_dung_ai và khi chủ dự án cho phép.</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>scripts/eval-focused.ts; lib/ai/fallback.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24553,7 +24812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29055,6 +29314,38 @@
       <c r="F140" s="8" t="inlineStr">
         <is>
           <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>6ea882f..00b3988 + commit tài liệu (nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Vé B: đường chat Focused trong lib/rag/focused/ sau cờ CELES_FOCUSED_CHAT (cờ tắt = STANDARD nguyên vẹn). Người được hỏi đúng cung lục thân, chip giữ chủ đề ở server, câu do mã viết (F2, D, nhuận, E, N2, N4), prompt riêng bỏ Dấu ấn, guard từng câu + hợp đồng độ dài mới, hết câu có căn cứ thì thử lại rồi 502 + hoàn lượt. fallback.ts thêm ghim model + trần tiền cho script eval. Hai bài offline test-du-kien, test-focused vào CI. scripts/eval-focused.ts viết sẵn, CHƯA chạy.</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Ca gốc "sắp tới tôi có người yêu ko? tương lai gần" nhận về bài dài kiểu báo cáo, không trả lời thẳng, có lúc gán vận người khác. Chủ dự án duyệt phương án CEL-186 vé B với 10 cờ khoá: trả lời thẳng câu đầu, chiều do mã chốt, câu nào không căn cứ thì bỏ. Đặt sau cờ để làm song song với fix noi_dung_ai mà không chạm Production; eval và bật Preview chờ fix đó vào main.</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FIX: CEL-189 nhan dien production — NODE_ENV chi de loai, khong la dieu kien duong
Chu du an nghiem thu 03/10/2026: NODE_ENV=development/test luon non-production;
ngoai do production chi khi VERCEL=1 + VERCEL_ENV=production. Them ca kiem:
NODE_ENV=test, Preview, Vercel Production thieu NODE_ENV, script khong co
--ghi-production van local du env la Production (60/60).
Cong sau deploy: bon dieu kien /api/phien-ban, khong xa dem production,
khong chay --ghi-production de nghiem thu (docs/bay/moi-truong.md, backlog).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16020,7 +16020,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>1. lib/moi-truong-dem.ts: phamViDem() tính lúc gọi; production chỉ khi VERCEL=1 + VERCEL_ENV=production + NODE_ENV=production. 2. noi-dung-ai.ts gắn ns ở docNoiDung/luuNoiDung/docNoiDungMoiNhat/docNhieuTheoTienTo/đệm RAM, cắt ns khỏi khoá trả ra; tienTo rỗng → null/[]. 3. Script gọi khaiBaoScript(argv): mặc định local, --ghi-production mới ghi production. 4. xoaDemLaSo xoá đúng lá số + bề mặt + phạm vi, từ chối bề mặt cấu hình. 5. scripts/test-moi-truong-dem.ts (CI, Supabase giả).</t>
+          <t>1. lib/moi-truong-dem.ts: phamViDem() tính lúc gọi; NODE_ENV=development/test luôn non-production; ngoài đó production chỉ khi VERCEL=1 + VERCEL_ENV=production. 2. noi-dung-ai.ts gắn ns ở docNoiDung/luuNoiDung/docNoiDungMoiNhat/docNhieuTheoTienTo/đệm RAM, cắt ns khỏi khoá trả ra; tienTo rỗng → null/[]. 3. Script gọi khaiBaoScript(argv): mặc định local, --ghi-production mới ghi production. 4. xoaDemLaSo xoá đúng lá số + bề mặt + phạm vi, từ chối bề mặt cấu hình. 5. scripts/test-moi-truong-dem.ts (CI, Supabase giả).</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -24641,12 +24641,12 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>phamViDem(env) trong lib/moi-truong-dem.ts là nguồn sự thật duy nhất. Script đã khaiBaoScript thì theo cờ dòng lệnh. Không thì: VERCEL=1 + NODE_ENV=production + VERCEL_ENV=production → production ns ''; + VERCEL_ENV=preview → preview:&lt;slug(ref)&gt;-&lt;sha256(ref) 8&gt;:; còn lại local:&lt;slug(CELES_CACHE_NAMESPACE)|local&gt;:. Slug chỉ [a-z0-9-].</t>
+          <t>phamViDem(env) trong lib/moi-truong-dem.ts là nguồn sự thật duy nhất. Script đã khaiBaoScript thì theo cờ dòng lệnh. Không thì: NODE_ENV=development/test → local; VERCEL=1 + VERCEL_ENV=production → production ns ''; + VERCEL_ENV=preview → preview:&lt;slug(ref)&gt;-&lt;sha256(ref) 8&gt;:; còn lại local:&lt;slug(CELES_CACHE_NAMESPACE)|local&gt;:. Slug chỉ [a-z0-9-].</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>KHÔNG CHỈ DỰA VÀO VERCEL_ENV: .env.local chép VERCEL_ENV=production (vercel env pull) là next dev thành production. next dev ép NODE_ENV=development nên ba điều kiện cùng lúc mới chặn được. Không module nào khác tự đọc VERCEL_ENV.</t>
+          <t>KHÔNG CHỈ DỰA VÀO VERCEL_ENV: .env.local chép VERCEL_ENV=production (vercel env pull) là next dev thành production. next dev ép NODE_ENV=development nên luôn bị loại. NODE_ENV chỉ dùng để LOẠI, không phải điều kiện dương (chủ dự án quyết 03/10/2026). Không module nào khác tự đọc VERCEL_ENV.</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -24789,7 +24789,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>/api/phien-ban trả thêm phamViDem (production / preview:&lt;nhánh&gt;-&lt;băm&gt; / local:&lt;tên&gt;), không bí mật. Sau mỗi deploy production chạm đệm: commit đúng, nhanh=main, moiTruong=production, phamViDem=production. kiem-moi-truong.ts kiểm hai trường này và báo đỏ nếu .env.local có VERCEL / VERCEL_ENV.</t>
+          <t>/api/phien-ban trả thêm phamViDem (production / preview:&lt;nhánh&gt;-&lt;băm&gt; / local:&lt;tên&gt;), không bí mật. Sau mỗi deploy production chạm đệm: commit bằng HEAD vừa release, nhanh=main, moiTruong=production, phamViDem=production — đủ bốn là cổng đạt. Không xả đệm production, không chạy --ghi-production để nghiệm thu. kiem-moi-truong.ts kiểm hai trường này và báo đỏ nếu .env.local có VERCEL / VERCEL_ENV.</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -24815,7 +24815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29347,6 +29347,38 @@
         </is>
       </c>
       <c r="F141" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>(nhánh viec/fix-noi-dung-ai-env)</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Nhận diện production: NODE_ENV development/test luôn non-production, ngoài đó chỉ cần VERCEL=1 + VERCEL_ENV=production (bỏ NODE_ENV=production khỏi điều kiện dương). Thêm 5 ca kiểm (NODE_ENV=test, Preview, thiếu NODE_ENV, script không cờ). Script chay-lai-luan-giai xoá thêm nhịp/mốc/bản đọc sâu cùng kỳ.</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Chủ dự án nghiệm thu 03/10/2026: NODE_ENV là điều kiện dương thứ ba thì một runtime Vercel Production không đặt NODE_ENV bị rơi về local, cả đệm production đọc trượt; dùng NODE_ENV để loại là đủ chặn next dev/test. celes-domain bắt lỗi xoá thiếu bề mặt cùng kỳ làm thẻ nhịp lệch luận hạn.</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 ve B — thang nhuan fail closed, N3 hai buoc, fallback giu nguyen, ty le thu lai
- Chip / cau "Thang X nhuan" tra cau ma cauNhuanChuaTach (focused-nhuan-chua-tach),
  khong goi logic thang thuong; kiem o ca luot 1 va luot 2 sau ke thua.
- Regression N3: tinh cam / su nghiep qua hai chip lien tiep van giu chu de.
- test-fallback-giu-nguyen.ts (CI): so vet fallback.ts voi ban dong bang truoc
  CEL-186 tren 15 tinh huong khi khong dat bien eval.
- eval-focused: dem so luot thu lai, ty le, nguong dung 15%.
- Backlog + AGENTS + HUONG-DAN: luong bat Production, no khong chan.

Vi sao: chu du an duyet co #1-#5 va neu hai blocker truoc khi push. Doc thang
thuong thay thang nhuan la tra loi sai; fallback.ts dung chung nen can bang
chung may rang Production chon model y nhu cu; thu lai nhieu la dau hieu hong
nen phai do va co nguong dung.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Vé A: đang chạy (nhánh, chờ nghiệm thu). Vé B: code xong trên nhánh viec/cel-186-focused-chat, cờ TẮT; chưa bật Preview, chưa eval model thật, chưa merge (chờ fix noi_dung_ai vào main)</t>
+          <t>Vé A: đang chạy (nhánh, chờ nghiệm thu). Vé B: code xong, đã đẩy nhánh viec/cel-186-focused-chat, cờ TẮT ở mọi môi trường; chưa bật Preview, chưa eval model thật, chưa merge (chờ CEL-189 vào main + cổng /api/phien-ban Production PASS)</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -15906,7 +15906,7 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>NỢ: (1) Sổ "đã nói trước" (V3, tổng quan) khoá theo năm DƯƠNG, chat tra bằng năm âm; mệnh bàn, /api/luan-giai, V3 vẫn mặc định năm dương → từ 01/01 tới Tết chat và các bề mặt khác lệch một năm. Ticket riêng, PHẢI xử lý trước 01/01/2027. (2) Từ điển thực thể còn bí danh "năm tới" (đã chặn ở doanLopHan theo phạm vi). (3) Chip vẫn tốn lượt (nợ sản phẩm; F2 do mã viết cũng trừ lượt — cờ #4). (4) "tháng 3" hỏi lúc tháng 8 vẫn hiểu là tháng 3 năm đang xem (đã qua), không đoán năm sau; tháng là tháng âm. Không có scanner "tháng đẹp nhất". (5) Bài dài cố định "Tôi là ai… cả đời" mất lưu niên dự phòng (đổi ngữ nghĩa có chủ đích). VÉ B còn: sau khi fix noi_dung_ai vào main → merge origin/main (không rebase) → regression → bật env Preview RIÊNG nhánh → eval-focused (≤ $2, model Production ghim) → Barnum 6×6 → celes-domain → bien-tap-vi → qa → soat-tai-lieu → UAT → mới trình merge. Lệch đã biết: chip "Tháng X nhuận" vẫn đọc nguyệt hạn tháng thường (engine không có nguyệt hạn tháng nhuận); chip N2 "Tháng N năm sau thì sao?" chưa làm; chipTruoc lấy xấp xỉ từ câu người dùng (chip không nằm trong lịch sử).</t>
+          <t>NỢ: (1) Sổ "đã nói trước" (V3, tổng quan) khoá theo năm DƯƠNG, chat tra bằng năm âm; mệnh bàn, /api/luan-giai, V3 vẫn mặc định năm dương → từ 01/01 tới Tết chat và các bề mặt khác lệch một năm. Ticket riêng, PHẢI xử lý trước 01/01/2027. (2) Từ điển thực thể còn bí danh "năm tới" (đã chặn ở doanLopHan theo phạm vi). (3) Chip vẫn tốn lượt (nợ sản phẩm; F2 và câu nhuận do mã viết cũng trừ lượt — cờ #4). (4) "tháng 3" hỏi lúc tháng 8 vẫn hiểu là tháng 3 năm đang xem (đã qua), không đoán năm sau; tháng là tháng âm. Không có scanner "tháng đẹp nhất". (5) Bài dài cố định "Tôi là ai… cả đời" mất lưu niên dự phòng (đổi ngữ nghĩa có chủ đích). NỢ VÉ B (không chặn): chip N2 "Tháng N năm sau thì sao?" chưa làm; gõ không dấu "nghe loi" chưa nhận; model tự khai ngoaiPhamVi chưa có máy canh riêng; chipTruoc lấy xấp xỉ từ câu người dùng. Tháng nhuận: FAIL CLOSED — engine không có nguyệt hạn tháng nhuận nên chip/câu "Tháng X nhuận" trả câu mã "chưa tách riêng được", không đọc tháng X thường. VÉ B còn: CEL-189 vào main + /api/phien-ban Production PASS → merge origin/main (merge thường; xung đột backlog thì lấy bản main rồi ghi lại CEL-186 bằng backlog.py) → chạy lại toàn bộ regression → bật cờ Preview RIÊNG nhánh → eval-focused (≤ $2, ghim openai|gpt-5.6-luna = model ưu tiên 0 trong ai_model_configs; thử lại &gt; 15% tổng ca thì dừng, điều tra) → Barnum 6×6 → celes-domain, qa, bien-tap-vi, soat-tai-lieu → UAT → merge main với cờ Production VẪN TẮT → smoke đường cũ → mới bật CELES_FOCUSED_CHAT=1 Production + smoke Focused. Rollback = tắt cờ, không revert code.</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -16014,7 +16014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G241"/>
+  <dimension ref="A1:G242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -24638,12 +24638,12 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào, E A hay B, F1 quan hệ, F2 vận riêng người khác, G không hướng. F2, D, tháng nhuận cần hỏi lại: mã trả trọn lượt (provider 'ma', model focused-f2/-d/-nhuan), không truy hồi, không gọi model, vẫn trừ lượt. E, N2 tháng đã qua, N4 cuối năm: câu mã đứng đầu, model viết phần sau.</t>
+          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào, E A hay B, F1 quan hệ, F2 vận riêng người khác, G không hướng. F2, D, tháng nhuận cần hỏi lại, tháng nhuận đã chọn: mã trả trọn lượt (provider 'ma', model focused-f2/-d/-nhuan/-nhuan-chua-tach), không truy hồi, không gọi model, vẫn trừ lượt. Tháng nhuận đã chọn (chip "Tháng X nhuận" hoặc gõ thẳng) fail closed: câu mã nói Celes chưa tách riêng được vận tháng nhuận, chip quay về "Tháng X" thường; kiểm ở cả lượt 1 và lượt 2 (sau kế thừa). E, N2 tháng đã qua, N4 cuối năm: câu mã đứng đầu, model viết phần sau.</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Cờ #3, #4, #5: bỏ D′ và chip "Tháng nào đáng chú ý hơn?" (engine không so tháng → ngõ cụt).</t>
+          <t>Cờ #3, #4, #5: bỏ D′ và chip "Tháng nào đáng chú ý hơn?" (engine không so tháng → ngõ cụt). Không bao giờ gọi logic tháng thường cho tháng nhuận (chủ dự án 03/10: không phải lệch đã biết mà là lỗi) — bản đầu chip "Tháng X nhuận" đọc nguyệt hạn tháng X thường.</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -24749,7 +24749,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>chayFocused gọi model tối đa 2 lần trong hạn 50s. Hết câu CÓ CĂN CỨ (mã F### thật trong gói) hoặc JSON gãy thì thử lại 1 lần; vẫn hỏng thì van rỗng → route trả 502 và hoàn lượt. Ngoại lệ: model khai ngoaiPhamVi (câu hỏi lá số không trả lời được) với đúng một câu chốt và không câu thân → nhận, không thử lại.</t>
+          <t>chayFocused gọi model tối đa 2 lần trong hạn 50s (đúng MỘT lần thử lại, chủ dự án duyệt 03/10). Hết câu CÓ CĂN CỨ (mã F### thật trong gói) hoặc JSON gãy thì thử lại 1 lần; vẫn hỏng thì van rỗng → route trả 502 và hoàn lượt, không thử tiếp. Ngoại lệ: model khai ngoaiPhamVi (câu hỏi lá số không trả lời được) với đúng một câu chốt và không câu thân → nhận, không thử lại.</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -24786,17 +24786,54 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>scripts/eval-focused.ts gọi traLoiCoCanCu trong tiến trình, tuần tự, lá số đóng băng. Bắt buộc AI_GHIM_MODEL (mọi lời gọi chỉ dùng model đó, không lùi) và AI_TRAN_USD ≤ 2 + giá vào/ra: giữ chỗ bi quan trước mỗi lời gọi, vượt trần ném VuotNganSachError trước khi gọi → dừng cả bộ.</t>
+          <t>scripts/eval-focused.ts gọi traLoiCoCanCu trong tiến trình, tuần tự, lá số đóng băng. Bắt buộc AI_GHIM_MODEL (mọi lời gọi chỉ dùng model đó, không lùi; Production hiện là openai|gpt-5.6-luna) và AI_TRAN_USD ≤ 2 + giá vào/ra: giữ chỗ bi quan trước mỗi lời gọi, vượt trần ném VuotNganSachError trước khi gọi → dừng cả bộ. Báo số lượt thử lại / tổng ca, tỉ lệ, chia theo lý do; tỉ lệ &gt; 15% in "DỪNG TRƯỚC PRODUCTION". scripts/test-fallback-giu-nguyen.ts (CI) chạy fallback.ts hiện tại và bản đóng băng trước CEL-186 (scripts/dong-bang/) trên 15 tình huống khi KHÔNG đặt biến eval, so vết từng byte.</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Cờ #8: tổng eval vé B ≤ $2, đúng model Production. Chỉ chạy sau fix noi_dung_ai và khi chủ dự án cho phép.</t>
+          <t>Cờ #8: tổng eval vé B ≤ $2, đúng model Production. fallback.ts là vùng Chung: không sửa tra-loi.ts chưa đủ chứng minh STANDARD không đổi — phải có bài so vết với bản cũ. Khác biệt CÓ CHỦ ĐÍCH duy nhất: khi đặt AI_NHAN, lượt gọi hỏng cũng ghi nhãn model@nhan (chỉ script). Đổi fallback.ts mà muốn đổi hành vi thật thì cập nhật bản đóng băng trong cùng commit, nói rõ vì sao.</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
           <t>scripts/eval-focused.ts; lib/ai/fallback.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Kế thừa chủ đề qua hai chip liên tiếp</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>timNguon lùi tối đa 4 lượt người dùng tìm câu có chủ đề, bỏ qua câu chip không chủ đề. "Tình cảm sắp tới?" → "Sang năm thì sao?" → "Tháng này thì sao?" vẫn giữ tinh-cam / Phu Thê; tương tự su-nghiep / Quan Lộc. Năm của chip sau lấy theo chip sau, không dính năm chip trước.</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu regression trước eval (03/10). Không cần sửa server: client gửi đủ lịch sử, chip là lượt người dùng.</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/ke-thua.ts; scripts/test-focused.ts</t>
         </is>
       </c>
     </row>
@@ -24812,7 +24849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29376,6 +29413,38 @@
         </is>
       </c>
       <c r="F142" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>sau 8113e14 (nhánh viec/cel-186-focused-chat, hai blocker trước eval)</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Vé B: (1) Tháng nhuận fail closed — chip/câu "Tháng X nhuận" trả câu mã cauNhuanChuaTach, không đọc tháng X thường; chip "Tháng X" giữ nguyên. (2) Regression N3 hai bước chip cho tình cảm và sự nghiệp. (3) test-fallback-giu-nguyen.ts vào CI: so vết fallback.ts với bản trước CEL-186 trên 15 tình huống khi không đặt biến eval. (4) eval-focused báo số lượt thử lại, tỉ lệ, ngưỡng dừng 15%. (5) Ghi luồng bật Production và nợ không chặn vào backlog.</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt 5 cờ và nêu 2 blocker trước khi cho push: đọc tháng thường thay cho tháng nhuận là trả lời sai, không phải giới hạn chấp nhận được; fallback.ts dùng chung nên cần bằng chứng máy rằng STANDARD/Production chọn model y như cũ; thử lại nhiều là dấu hiệu prompt hoặc guard hỏng nên phải đo và có ngưỡng dừng trước Production.</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: CEL-189 da len production — backlog DONE, TRANG-THAI ban giao CEL-186 ve B
Vi sao: /api/phien-ban Production dat du 4 dieu kien (1bdfe6b, main, production, production); ve B duoc di tiep merge main + eval.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16025,7 +16025,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Chờ nghiệm thu</t>
+          <t>Đã lên production (03/10/2026) — /api/phien-ban: commit 1bdfe6b, nhanh=main, moiTruong=production, phamViDem=production</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>(nhánh viec/fix-noi-dung-ai-env)</t>
+          <t>8bc5554, 667848a + merge 1bdfe6b (main)</t>
         </is>
       </c>
     </row>
@@ -24815,7 +24815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F143"/>
+  <dimension ref="A1:F144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29406,6 +29406,38 @@
         </is>
       </c>
       <c r="F143" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1bdfe6b (merge viec/fix-noi-dung-ai-env vào main)</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CEL-189</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Gộp CEL-189 vào main và lên Production: CI main xanh (run 37136119327), Vercel Production READY (dpl_4K5af9LmTDzodwqwUuH1G3V3tssG), /api/phien-ban đủ 4 điều kiện. Không chạy --ghi-production, không xoá đệm Production.</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Chủ dự án nghiệm thu kỹ thuật và cho gộp. Production phải đếm noi_dung_ai riêng trước khi CEL-186 vé B bật cờ trên Preview — Preview dùng chung Supabase, không tách thì eval trên Preview ghi vào đệm production.</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 ve B — sua sau eval vong 1 (khuon F1 'toi voi bo', cam nguoi la, N1 nguyet han, sua do eval)
- doi-tuong: 'toi voi/va <nguoi than>' nhan la quan he -> F1
- prompt: cam dua nguoi khong co trong cau hoi; hoi thang phai dan ma nguyet han
- PHIEN_BAN_FOCUSED -> focused-2026.10.2
- eval: chu de so voi nhan, bo bao nham nguoi la, khong cham khuyen tren cau du phong do ma

Vi sao: eval model that vong 1 truot 6 muc; 3 la loi san pham that, 3 la loi do.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Vé A: đã lên production (merge 10e351f). Vé B: đã merge origin/main sau CEL-189 (ace6d2f), cờ TẮT ở mọi môi trường; đang regression → bật cờ Preview riêng nhánh → eval model thật → Barnum → reviewer → UAT. Chưa merge main.</t>
+          <t>Vé A: đã lên production (merge 10e351f). Vé B: eval model thật vòng 1 (03/10, $0.17) trượt 6 mục; đã sửa đo eval + 3 lỗi sản phẩm (focused-2026.10.2), đang chạy vòng 2. Cờ TẮT ở mọi môi trường. Chưa merge main.</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -25111,7 +25111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29862,6 +29862,38 @@
         </is>
       </c>
       <c r="F148" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>viec/cel-186-focused-chat (sau eval vòng 1)</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Focused 2026.10.2: (1) 'tôi với/và &lt;bố, mẹ, con, vợ, chồng…&gt;' nhận là quan hệ → khuôn F1 (bỏ anh/chị/em/bạn trần và 'mẹ chồng'); (2) prompt cấm đưa người không có trong câu hỏi (sếp, đồng nghiệp…) vào câu văn; (3) hỏi một tháng thì prompt liệt mã nguyệt hạn và đòi ít nhất một câu dựa vào đó. Eval: chủ đề so với nhãn NHAN_CHU_DE, bỏ báo nhầm người lạ ở nhãn phần đời/'công bố'/cặp vợ chồng–cha mẹ, câu chốt dự phòng do mã viết không chấm khuyên.</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Eval model thật vòng 1: 'Tôi với bố có hợp nhau không?' ra khuôn A; model tự thêm sếp/đồng nghiệp ở 10/72 bài công việc–tiền; một ca hỏi tháng không dẫn nguyệt hạn. Đúng chủ đề 0/13 là lỗi đo (so mã với nhãn), không phải lỗi sản phẩm.</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 ve B — sua sau reviewer vong 2 + eval vong 4-5 (focused-2026.10.3)
- chonChip loc bang ma: chip > 40 ky tu, chip "Co nen", chip "Dai van"
- prompt cam nhan noi bo "phia thuan/nghieng han" va doi chu khoi HUONG DA CHOT;
  moi cau toi da mot ten sao
- doi-tuong: "toi voi bo me chong", "con nguoi do" khong nhan la nguoi than
- backlog CEL-186 (Logic #9-#12), phuong an muc 16 (ket qua eval + no)

Vi sao: bien-tap-vi thay chip dai, chip khuyen va nhan noi bo lo ra cau van;
qa thay "bo me chong" nhan nham la me ruot. Eval vong 4 cho thay luat chip chi o
prompt khong du va model chep chu tu khoi huong. Vong 5: 13/16 muc dat, tong
eval ~$0.77/$2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Vé A: đã lên production (merge 10e351f). Vé B: eval model thật vòng 1 (03/10, $0.17) trượt 6 mục; đã sửa đo eval + 3 lỗi sản phẩm (focused-2026.10.2), đang chạy vòng 2. Cờ TẮT ở mọi môi trường. Chưa merge main.</t>
+          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.3): eval model thật 5 vòng 03–04/10, tổng ≈ $0.77/$2. Vòng 5: đạt 13/16 mục (tên ngoài gói 0, khuyên 0, người lạ 0, thử lại 0%, 502 0, đúng khuôn 19/19, NORMAL 67/67, dự phòng 7/72); trượt: N1 1/2 (dao động, 5/6 qua 3 vòng), đúng chủ đề 12/13 (nợ planner), Barnum 3 61–67% (cấu trúc, chờ chủ dự án quyết ngưỡng). celes-domain FAIL ở câu dự phòng do mã viết (nghĩa tính cách sao không theo cung) — chờ chủ dự án quyết (cờ #1). Cờ TẮT ở mọi môi trường. Chưa merge main.</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -15911,12 +15911,12 @@
       </c>
       <c r="N186" s="8" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>04/10/2026</t>
         </is>
       </c>
       <c r="O186" s="8" t="inlineStr">
         <is>
-          <t>Vé A: c5651d2, 2c8963c + merge 10e351f. Vé B: 6ea882f..85667e5, 8113e14, 22ac260 + merge origin/main (nhánh viec/cel-186-focused-chat)</t>
+          <t>Vé A: c5651d2, 2c8963c + merge 10e351f. Vé B: 6ea882f..85667e5, 8113e14, 22ac260, merge 3ba1912, ab22d61, 37a51fb + commit sau eval vòng 5 (nhánh viec/cel-186-focused-chat)</t>
         </is>
       </c>
     </row>
@@ -16091,7 +16091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G247"/>
+  <dimension ref="A1:G251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25099,6 +25099,154 @@
         </is>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>'Tôi với / và &lt;người thân&gt;' → khuôn F1</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>nhanDangDoiTuong: khi câu không có đại từ sở hữu, mẫu '(tôi|mình|tớ) (với|và) &lt;bố, mẹ, con, vợ, chồng…&gt;' nhận là quan hệ (loai 'quan-he') → F1. Bỏ anh / chị / em / bạn trần; không nhận 'mẹ chồng', 'bố mẹ chồng/vợ', 'con người'. Chỉ bản có dấu.</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Eval vòng 1: 'Tôi với bố có hợp nhau không?' rơi khuôn A, đọc vận của người hỏi thay vì quan hệ. 'Tôi với mẹ chồng' không phải mẹ ruột — nhận nhầm là đọc sai cung.</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/doi-tuong.ts; scripts/test-focused.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Luật prompt sau eval (chỉ prompt, không guard)</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>KHÔNG ĐƯỢC: đưa người câu hỏi không nhắc (sếp, đồng nghiệp…) vào câu; viết nhãn nội bộ 'phía thuận/vướng', 'nghiêng hẳn/rõ' (khối HƯỚNG ĐÃ CHỐT đã đổi sang 'thuận RÕ / vướng RÕ' để model không chép). Mỗi câu tối đa một tên sao. Hỏi MỘT tháng: liệt mã nguyệt hạn và đòi ≥1 câu dựa vào đó.</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Model chép nguyên chữ trong khối mô tả hướng vào câu chốt (13 bài vòng 4 → 2 bài vòng 5). Luật N1 chỉ ở prompt nên dao động (5/6 qua 3 vòng); ép bằng thử lại là đổi cờ #3, chưa làm.</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/prompt.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Lọc chip bằng mã</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>chonChip bỏ chip dài quá 40 ký tự (CHIP_TOI_DA), chip bắt đầu 'Có nên', chip có 'Đại vận' — cùng với các lọc cũ (ra lệnh, hỏi tên, vận riêng người khác, 'Tháng nào / Khi nào'). Thiếu thì bù CHIP_DU_PHONG.</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>bien-tap-vi thấy chip 41–46 ký tự; luật chip trong prompt vòng 4 vẫn lọt 5 chip khuyên / 'Đại vận' → phải lọc bằng mã.</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/kiem.ts; scripts/test-focused.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Sửa thước đo eval</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>eval-focused: đúng chủ đề so goi.chuDe với NHAN_CHU_DE (nhãn, không phải slug); người lạ bỏ nhãn phần đời ('phần cha mẹ'…), 'công bố', cặp vợ chồng / cha mẹ khi câu hỏi đã nhắc; câu chốt dự phòng do mã viết không chấm khuyên; ghi lyDoThayChot cho mỗi ca dự phòng.</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Vòng 1 'đúng chủ đề 0/13' là lỗi đo, không phải lỗi sản phẩm — đọc kết quả eval phải soát thước đo trước khi sửa mã.</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>scripts/eval-focused.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25111,7 +25259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29894,6 +30042,38 @@
         </is>
       </c>
       <c r="F149" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>viec/cel-186-focused-chat (sau eval vòng 5)</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Focused 2026.10.3: chip lọc bằng mã (&gt; 40 ký tự, 'Có nên', 'Đại vận'); prompt cấm nhãn nội bộ 'phía thuận/nghiêng hẳn' và đổi chữ khối HƯỚNG ĐÃ CHỐT; mỗi câu một tên sao; 'tôi với bố mẹ chồng' / 'con người' không nhận là người thân. Eval vòng 4–5 ($0.34).</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Reviewer vòng 2: bien-tap-vi thấy chip dài và chip khuyên, nhãn nội bộ lộ ra câu văn; qa thấy 'bố mẹ chồng' nhận nhầm là mẹ ruột. Vòng 4 cho thấy luật chip chỉ ở prompt không đủ, model chép chữ từ khối hướng — nên lọc chip bằng mã và đổi chữ nguồn.</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-186 ve B — chot chu du an 04/10 (focused-2026.10.4), mo CEL-190
- Cau chot du phong chi neu ten + huong sao (bo tenKemNghia), test Tang Mon 4 phan doi VI/EN
- Hoi MOT thang: bat buoc >= 1 cau nguyet han, thieu thi thu lai 1 lan roi 502 + hoan luot
- Ba cau ma theo chu da duyet, bo "du kien"; cau ma/chip/loi di/mien tru theo ngonNgu VI/EN
- Chot kiem bo cau model co "du kien"; prompt thang toi / khong muon nghia ten cung thang
- Barnum 3 cham theo do hiem ten, hoa = chua phan dinh; --cham-lai, --chi-thang
- Mo CEL-190 (planner nhan sai chu de) — chan bat co Production

Vi sao: chu du an chot 04/10 sau review vong 5; celes-domain bat loi cau "thang sau" o eval thang lan mot.
Eval thang 24 ca: N1 24/24, thu lai 4.2%, 502 0. Tong chi eval ~$0.89/$2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O188"/>
+  <dimension ref="A1:O189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.3): eval model thật 5 vòng 03–04/10, tổng ≈ $0.77/$2. Vòng 5: đạt 13/16 mục (tên ngoài gói 0, khuyên 0, người lạ 0, thử lại 0%, 502 0, đúng khuôn 19/19, NORMAL 67/67, dự phòng 7/72); trượt: N1 1/2 (dao động, 5/6 qua 3 vòng), đúng chủ đề 12/13 (nợ planner), Barnum 3 61–67% (cấu trúc, chờ chủ dự án quyết ngưỡng). celes-domain FAIL ở câu dự phòng do mã viết (nghĩa tính cách sao không theo cung) — chờ chủ dự án quyết (cờ #1). Cờ TẮT ở mọi môi trường. Chưa merge main.</t>
+          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.4): đã sửa theo chốt chủ dự án 04/10 — câu chốt dự phòng chỉ nêu tên + hướng; hỏi MỘT tháng bắt buộc ≥ 1 câu nguyệt hạn (thử lại 1 lần rồi 502 + hoàn lượt); ba câu mã theo chữ đã duyệt; câu do mã viết theo ngôn ngữ người dùng (VI/EN); Barnum 3 chấm theo độ hiếm của tên. Eval tháng 24 ca: N1 24/24, thử lại 4,2%, 502 0. Barnum 3 chấm lại vòng 5: 10/10 ca phân định được (tỉ lệ phân định 27,8%, 0 sai). Tổng chi eval ≈ $0.83/$2. Cờ TẮT ở mọi môi trường. Chưa merge main. Bật cờ Production bị chặn bởi CEL-190.</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -15906,7 +15906,7 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>NỢ: (1) Sổ "đã nói trước" (V3, tổng quan) khoá theo năm DƯƠNG, chat tra bằng năm âm; mệnh bàn, /api/luan-giai, V3 vẫn mặc định năm dương → từ 01/01 tới Tết chat và các bề mặt khác lệch một năm. Ticket riêng, PHẢI xử lý trước 01/01/2027. (2) Từ điển thực thể còn bí danh "năm tới" (đã chặn ở doanLopHan theo phạm vi). (3) Chip vẫn tốn lượt (nợ sản phẩm; F2 và câu nhuận do mã viết cũng trừ lượt — cờ #4). (4) "tháng 3" hỏi lúc tháng 8 vẫn hiểu là tháng 3 năm đang xem (đã qua), không đoán năm sau; tháng là tháng âm. Không có scanner "tháng đẹp nhất". (5) Bài dài cố định "Tôi là ai… cả đời" mất lưu niên dự phòng (đổi ngữ nghĩa có chủ đích). NỢ VÉ B (không chặn): chip N2 "Tháng N năm sau thì sao?" chưa làm; gõ không dấu "nghe loi" chưa nhận; model tự khai ngoaiPhamVi chưa có máy canh riêng; chipTruoc lấy xấp xỉ từ câu người dùng. Tháng nhuận: FAIL CLOSED — engine không có nguyệt hạn tháng nhuận nên chip/câu "Tháng X nhuận" trả câu mã "chưa tách riêng được", không đọc tháng X thường. VÉ B còn: CEL-189 vào main + /api/phien-ban Production PASS → merge origin/main (merge thường; xung đột backlog thì lấy bản main rồi ghi lại CEL-186 bằng backlog.py) → chạy lại toàn bộ regression → bật cờ Preview RIÊNG nhánh → eval-focused (≤ $2, ghim openai|gpt-5.6-luna = model ưu tiên 0 trong ai_model_configs; thử lại &gt; 15% tổng ca thì dừng, điều tra) → Barnum 6×6 → celes-domain, qa, bien-tap-vi, soat-tai-lieu → UAT → merge main với cờ Production VẪN TẮT → smoke đường cũ → mới bật CELES_FOCUSED_CHAT=1 Production + smoke Focused. Rollback = tắt cờ, không revert code.</t>
+          <t>Chặn bật cờ Production: CEL-190 (planner nhận sai chủ đề). Giới hạn EN: planner, phân khuôn và các chốt kiểm khuyên / chắc chắn chỉ đọc tiếng Việt; thân bài do model viết vẫn là tiếng Việt — người dùng EN chỉ nhận câu mã, chip, lối đi, miễn trừ bằng EN. Barnum 3: tỉ lệ phân định thấp (27,8%) vì bài nêu ít tên và hai lá số mẫu 1944 gần như trùng — con số đạt dựa trên 10 ca. UAT Preview cần chủ dự án đặt CELES_FOCUSED_CHAT=1 cho riêng nhánh trên Vercel (không có CLI/token ở máy).</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -15916,7 +15916,7 @@
       </c>
       <c r="O186" s="8" t="inlineStr">
         <is>
-          <t>Vé A: c5651d2, 2c8963c + merge 10e351f. Vé B: 6ea882f..85667e5, 8113e14, 22ac260, merge 3ba1912, ab22d61, 37a51fb + commit sau eval vòng 5 (nhánh viec/cel-186-focused-chat)</t>
+          <t>Vé A: c5651d2, 2c8963c + merge 10e351f. Vé B: 6ea882f..85667e5, 8113e14, 22ac260, merge 3ba1912, ab22d61, 37a51fb, 7b5a195 + commit sau chốt 04/10 (nhánh viec/cel-186-focused-chat)</t>
         </is>
       </c>
     </row>
@@ -16071,6 +16071,78 @@
       <c r="O188" t="inlineStr">
         <is>
           <t>8bc5554, 667848a + merge 1bdfe6b (main)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>CEL-190</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Planner nhận sai chủ đề ở hai mẫu câu (bản thân tôi … công việc; nhà cửa / gia đạo)</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Eval vé B vòng 5 (04/10/2026): 'bản thân tôi năm nay công việc có ổn không?' ra Tổng quan thay vì Công việc; 'Năm nay chuyện nhà cửa, gia đạo của tôi thế nào?' ra Tài chính thay vì Gia đạo. Lỗi ở planner (lib/rag/planner.ts), dùng chung STANDARD và Focused — KHÔNG sửa trong vé B.</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>lapKeHoach / lapKeHoachFocused → từ điển thực thể + luật chủ đề trong planner.ts. 'bản thân' kéo về Mệnh/Tổng quan, 'nhà cửa' kéo về Điền Trạch → Tài chính.</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Chưa làm — mở 04/10/2026</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Không sinh nội dung</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Mọi bậc</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>/hoi-dap</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>lib/rag/planner.ts; scripts/eval-planner.ts; scripts/test-rag-planner.ts</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>Luôn bật</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>Không chặn merge vé B khi cờ Production TẮT. CHẶN bật CELES_FOCUSED_CHAT=1 trên Production (chủ dự án 04/10). Sửa planner là đổi cả STANDARD: bộ vàng eval-planner (100%) không được tụt; thêm hai câu này vào bộ vàng.</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
         </is>
       </c>
     </row>
@@ -16091,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G251"/>
+  <dimension ref="A1:G255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25247,6 +25319,154 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Câu chốt dự phòng chỉ nêu tên + hướng</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>cauChotDuPhong dùng tenKemHuong: '&lt;tên sao&gt; kéo phần này lại' / '&lt;tên sao&gt; đỡ cho phần này' (EN: 'holds this area back' / 'supports this area'). Bỏ tenKemNghia — KHÔNG lấy nét chung d.y của sao gắn vào phần đời đang hỏi. Câu người khác cùng dạng.</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>celes-domain FAIL 04/10: 'Tang Môn cho thấy bạn dễ phải chia tay' trong câu hỏi tiền bạc — nét chung của sao bị gán sang phần đời khác và thành tính cách người hỏi. Engine không có nghĩa sao theo phần đời đáng tin, nên chỉ nêu tên.</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/chot-huong.ts; scripts/test-focused.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Hỏi MỘT tháng: bắt buộc câu nguyệt hạn</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>ctx.maNguyetHan = mã dữ kiện loại nguyet-han trong gói. Câu có thoiGian.thang, khuôn ≠ E, không ngoài phạm vi VÀ gói có mã nguyệt hạn (cùng điều kiện với dòng dặn trong prompt): bản cuối không còn câu nào trỏ mã nguyệt hạn → thuLai 'thieu-nguyet-han'. Lần 2 vẫn thiếu → văn rỗng → route 502 + hoàn lượt. Cắt độ dài không cắt câu nguyệt hạn cuối cùng. Prompt: tháng tới chính là tháng đang đọc; không mượn nghĩa tên cung tháng; tháng đã qua không lặp mốc. Chốt kiểm bỏ câu model có chữ 'dữ kiện' (so có dấu, tránh trùng 'dự kiến').</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>N1 chỉ ở prompt dao động 5/6 qua 3 vòng. Chủ dự án 04/10: ép bằng thử lại, thử lại tổng ≤ 15%. Eval tháng 24 ca: 24/24, thử lại 4,2%.</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/kiem.ts; lib/rag/focused/chay.ts; lib/rag/focused/prompt.ts; lib/rag/focused/tra-loi-focused.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Câu do mã viết theo ngôn ngữ người dùng</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Trang gửi ngonNgu; route chọn bằng chonNgonNgu(body, cookie 'tuvi-ai:ngon-ngu'), mặc định vi. Câu mã (khi nào, hai về, vận riêng, cuối năm, nhuận, tháng đã qua, ngoài tầm, dự phòng, mốc chốt), chip mã, chip dự phòng, lối đi, miễn trừ tâm lý có bản EN. Chữ VI theo bản chủ dự án duyệt 04/10; không còn 'dữ kiện' ở câu người dùng thấy. Tháng nhuận: một chip (tháng thường).</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Planner, phân khuôn và chốt kiểm là regex tiếng Việt; thân bài model vẫn tiếng Việt — giới hạn đã báo, không phải lỗi im lặng.</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/ngon-ngu.ts; lib/rag/focused/cau-ma.ts; lib/rag/focused/ngoai-tam.ts; app/api/hoi-dap/route.ts; app/hoi-dap/page.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Barnum 3 chấm theo độ hiếm của tên</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Mỗi tên nặng log(n / số lá số ứng viên có tên đó). Điểm lá số = tổng nặng tên bài nêu có trong gói lá số đó. Đỉnh 0 hoặc hoà ở đỉnh có lá số đúng → chưa phân định (không tính sai). Cổng ≥ 80% trên ca phân định được; tỉ lệ phân định báo riêng. --cham-lai &lt;tệp&gt; chấm lại không gọi model; --chi-thang chạy riêng bộ câu tháng.</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Cách cũ (đếm tên chia cỡ gói, hoà lấy lá số đầu) tính hoà là sai → 61% dù không bài nào trỏ nhầm lá số. Chủ dự án 04/10: không hạ ngưỡng, sửa thước đo.</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>scripts/eval-focused.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25259,7 +25479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F150"/>
+  <dimension ref="A1:F152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30074,6 +30294,70 @@
         </is>
       </c>
       <c r="F150" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>viec/cel-186-focused-chat (sau chốt chủ dự án 04/10)</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>CEL-186, CEL-190</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Focused 2026.10.4: dự phòng chỉ nêu tên + hướng sao; hỏi một tháng bắt buộc câu nguyệt hạn (thử lại rồi 502 + hoàn lượt); ba câu mã theo chữ đã duyệt, bỏ 'dữ kiện'; câu mã/chip/lối đi/miễn trừ theo ngôn ngữ VI/EN; Barnum 3 chấm theo độ hiếm, có chế độ chấm lại không gọi model và chế độ chỉ chạy câu tháng. Mở CEL-190 cho lỗi planner.</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Chủ dự án chốt 04/10 sau review vòng 5: câu dự phòng gán nét chung của sao sang phần đời khác là lỗi chặn; N1 chỉ ở prompt dao động; thước đo Barnum 3 cũ tính hoà là sai; người dùng EN nhận câu tiếng Việt. Lỗi planner dùng chung STANDARD nên tách vé riêng, chặn bật cờ Production chứ không chặn merge.</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>viec/cel-186-focused-chat (sau celes-domain 04/10)</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Câu tháng: chốt kiểm bỏ câu có 'dữ kiện'; prompt nói rõ tháng tới là tháng đang đọc, cấm mượn nghĩa tên cung tháng; luật nguyệt hạn chỉ đòi khi gói có mã nguyệt hạn. EN: chip hai về dùng chip chung, câu dự phòng EN bớt lặp. Eval tháng lần hai: 0 lộ chữ, 0 mâu thuẫn, N1 24/24, thử lại 4,2%.</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>celes-domain đọc eval tháng lần một: 3/6 ca 'tháng sau' lộ 'dữ kiện' và tự mâu thuẫn, model suy nghĩa cung Phụ Mẫu/Điền Trạch sang tình cảm; luật kiểm và prompt lệch điều kiện có thể gây 502 chắc chắn. bien-tap-vi: chip EN nhét cụm tiếng Việt người dùng gõ.</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 ve B — "thang N" la thang duong (focused-2026.10.5)
- "Thang N" khong kem "am" / "nhuan" = thang duong; doc nguyet han cua thang am
  phu nhieu ngay nhat (thangAmChuYeu), cau mo dau noi ro quy doi + khoang ngay duong
- Bo nhanh hoi lai thuong/nhuan; chi dung khi go "nhuan" hoac thang duong roi vao
  thang nhuan. Chip nhuan doi thanh "Thang X am nam N"
- Thang da qua: "thang nay / quang nay" -> "do"; thang chua toi: cam "dang"
- Chi noi "phan lon" khi thang am chiem >= 60% so ngay; neu nam am khi khac nam duong

Vi sao: chu du an UAT Preview 04/10 hoi "Thang 6 nam 2025" thi nhan cau thang nhuan,
bam chip thi Celes doc thang 6 AM. Nguoi dung noi thang duong; muon am thi noi "thang 6 am".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.4): đã sửa theo chốt chủ dự án 04/10 — câu chốt dự phòng chỉ nêu tên + hướng; hỏi MỘT tháng bắt buộc ≥ 1 câu nguyệt hạn (thử lại 1 lần rồi 502 + hoàn lượt); ba câu mã theo chữ đã duyệt; câu do mã viết theo ngôn ngữ người dùng (VI/EN); Barnum 3 chấm theo độ hiếm của tên. Eval tháng 24 ca: N1 24/24, thử lại 4,2%, 502 0. Barnum 3 chấm lại vòng 5: 10/10 ca phân định được (tỉ lệ phân định 27,8%, 0 sai). Tổng chi eval ≈ $0.83/$2. Cờ TẮT ở mọi môi trường. Chưa merge main. Bật cờ Production bị chặn bởi CEL-190.</t>
+          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.5): đã sửa theo chốt chủ dự án 04/10 — câu chốt dự phòng chỉ nêu tên + hướng; hỏi MỘT tháng bắt buộc ≥ 1 câu nguyệt hạn (thử lại 1 lần rồi 502 + hoàn lượt); ba câu mã theo chữ đã duyệt; câu do mã viết theo ngôn ngữ người dùng (VI/EN); Barnum 3 chấm theo độ hiếm của tên. 04/10 (UAT Preview): "tháng N" trơn nay là tháng DƯƠNG, đọc tháng âm phủ nhiều ngày nhất; bỏ hỏi lại tháng nhuận. Eval tháng 24 ca: N1 24/24, thử lại 4,2%, 502 0. Barnum 3 chấm lại vòng 5: 10/10 ca phân định được (tỉ lệ phân định 27,8%, 0 sai). Tổng chi eval ≈ $0.94/$2. Cờ TẮT ở Production. Chưa merge main. Bật cờ Production bị chặn bởi CEL-190.</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -15906,7 +15906,7 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>Chặn bật cờ Production: CEL-190 (planner nhận sai chủ đề). Giới hạn EN: planner, phân khuôn và các chốt kiểm khuyên / chắc chắn chỉ đọc tiếng Việt; thân bài do model viết vẫn là tiếng Việt — người dùng EN chỉ nhận câu mã, chip, lối đi, miễn trừ bằng EN. Barnum 3: tỉ lệ phân định thấp (27,8%) vì bài nêu ít tên và hai lá số mẫu 1944 gần như trùng — con số đạt dựa trên 10 ca. UAT Preview cần chủ dự án đặt CELES_FOCUSED_CHAT=1 cho riêng nhánh trên Vercel (không có CLI/token ở máy).</t>
+          <t>Chặn bật cờ Production: CEL-190 (planner nhận sai chủ đề; và đường STANDARD vẫn hiểu "tháng N" là tháng âm — phải thống nhất với Focused trước khi bật). Giới hạn EN: planner, phân khuôn và các chốt kiểm khuyên / chắc chắn chỉ đọc tiếng Việt; thân bài do model viết vẫn là tiếng Việt — người dùng EN chỉ nhận câu mã, chip, lối đi, miễn trừ bằng EN. Barnum 3: tỉ lệ phân định thấp (27,8%) vì bài nêu ít tên và hai lá số mẫu 1944 gần như trùng — con số đạt dựa trên 10 ca. Lời luận tháng: thân bài đôi khi lấy sao gốc cung Quan Lộc (Thiên Cơ) gán cho tháng — guard N1 chỉ đòi ≥ 1 câu có mã nguyệt hạn.</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -16163,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G255"/>
+  <dimension ref="A1:G256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -24972,7 +24972,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào, E A hay B, F1 quan hệ, F2 vận riêng người khác, G không hướng. F2, D, tháng nhuận cần hỏi lại, tháng nhuận đã chọn: mã trả trọn lượt (provider 'ma', model focused-f2/-d/-nhuan/-nhuan-chua-tach), không truy hồi, không gọi model, vẫn trừ lượt. Tháng nhuận đã chọn (chip "Tháng X nhuận" hoặc gõ thẳng) fail closed: câu mã nói Celes chưa tách riêng được vận tháng nhuận, chip quay về "Tháng X" thường; kiểm ở cả lượt 1 và lượt 2 (sau kế thừa). E, N2 tháng đã qua, N4 cuối năm: câu mã đứng đầu, model viết phần sau.</t>
+          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào, E A hay B, F1 quan hệ, F2 vận riêng người khác, G không hướng. F2, D, tháng nhuận (gõ "nhuận" hoặc tháng dương rơi vào tháng nhuận — từ 04/10 không còn hỏi lại, xem #17): mã trả trọn lượt (provider 'ma', model focused-f2/-d/-nhuan-chua-tach), không truy hồi, không gọi model, vẫn trừ lượt. Tháng nhuận đã chọn (chip "Tháng X nhuận" hoặc gõ thẳng) fail closed: câu mã nói Celes chưa tách riêng được vận tháng nhuận, chip quay về "Tháng X âm" thường; kiểm ở cả lượt 1 và lượt 2 (sau kế thừa). E, N2 tháng đã qua, N4 cuối năm: câu mã đứng đầu, model viết phần sau.</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -25464,6 +25464,43 @@
       <c r="G255" t="inlineStr">
         <is>
           <t>scripts/eval-focused.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Tháng dương mặc định</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>boiCanhThoiGian: câu gọi đích danh "tháng N" mà không có "âm" / "âm lịch" / "lịch âm" / "nhuận" → tháng N DƯƠNG của năm namMucTieu (hoặc năm dương hiện tại). thangAmChuYeu đếm từng ngày, lấy tháng âm phủ nhiều ngày nhất (hoà: tháng đến trước), ro = chiếm ≥ 60% số ngày; namHieuLuc đổi sang năm âm của tháng đó (tháng 1–2 dương thường thuộc năm âm trước). MocThang.duong mang tháng dương. Câu mở đầu cauThangDuong nêu tháng dương → tháng âm (kèm năm âm nếu khác, ngày dương trong ngoặc), chỉ nói "phần lớn" khi ro; tháng đã qua gộp ý N2. Tháng dương rơi vào tháng nhuận → dừng bằng câu mã, không chip. "tháng này / tháng sau" vẫn theo tháng âm đang chạy. Tháng đã qua: doiNayThanhDo đổi "tháng này / quãng này" → "đó" trong văn model. Tiền tố chốt dự phòng của tháng dương là "Tháng đó".</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Chủ dự án thử Preview 04/10: "Tháng 6 năm 2025" bị hiểu là tháng 6 âm và đụng câu nhuận — người dùng nói "tháng 6" là tháng 6 dương. Không bao giờ hỏi lại "thường hay nhuận" khi người dùng không gõ "nhuận". Không nói "phần lớn" khi chia gần đều. Regex âm loại "âm thầm", "am hiểu", "âm nhạc".</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/thang-am.ts; lib/rag/focused/phan-loai.ts; lib/rag/focused/cau-ma.ts; lib/rag/focused/tra-loi-focused.ts; lib/rag/focused/prompt.ts; lib/rag/focused/kiem.ts</t>
         </is>
       </c>
     </row>
@@ -25479,7 +25516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F152"/>
+  <dimension ref="A1:F153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30358,6 +30395,33 @@
         </is>
       </c>
       <c r="F152" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Vé B focused-2026.10.5: "tháng N" trơn = tháng dương, quy về tháng âm phủ nhiều ngày nhất; câu mở đầu nói rõ quy đổi; bỏ nhánh hỏi lại tháng nhuận; chip nhuận thành "Tháng X âm năm N"; tháng đã qua đổi "này" → "đó"; prompt cấm "đang" cho tháng chưa tới.</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Chủ dự án UAT Preview 04/10: hỏi "Tháng 6 năm 2025" thì nhận câu tháng nhuận, bấm chip thì Celes đọc tháng 6 âm. Người dùng bình thường nói tháng dương; muốn âm lịch họ nói "tháng 6 âm".</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-186 ve B — final hardening (focused-2026.10.9), gop CEL-190
- Bo bat bien co test: docs/chien-luoc/CEL-186-INVARIANTS.md
- gioi-han.ts: chan truoc ngay sinh / chua hop tuoi / lech gioi bang cau ma, hoan luot
- Chu de: ban than + cong viec -> su nghiep, nha cua -> gia dao, mua nha/vay giu tai chinh
- Cau chot huong can bang neu hai phia hoac khong neu ten
- Cau thang duong/am/nhuan VI/EN noi ro Celes quy doi
- Oracle ten doc lap render prompt that + dot bien d.sao

Vi sao: chu du an 04/10 yeu cau mot dot cung hoa cuoi truoc UAT/merge; A/B lo loi co o ca hai ban va bo do ten tu xac nhan cung nguon voi guard. Sua chu de o lop Focused de khong doi PHIEN_BAN_PLANNER, khong xa dem, khong doi STANDARD.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.5): đã sửa theo chốt chủ dự án 04/10 — câu chốt dự phòng chỉ nêu tên + hướng; hỏi MỘT tháng bắt buộc ≥ 1 câu nguyệt hạn (thử lại 1 lần rồi 502 + hoàn lượt); ba câu mã theo chữ đã duyệt; câu do mã viết theo ngôn ngữ người dùng (VI/EN); Barnum 3 chấm theo độ hiếm của tên. 04/10 (UAT Preview): "tháng N" trơn nay là tháng DƯƠNG, đọc tháng âm phủ nhiều ngày nhất; bỏ hỏi lại tháng nhuận. Eval tháng 24 ca: N1 24/24, thử lại 4,2%, 502 0. Barnum 3 chấm lại vòng 5: 10/10 ca phân định được (tỉ lệ phân định 27,8%, 0 sai). Tổng chi eval ≈ $0.94/$2. Cờ TẮT ở Production. Chưa merge main. Bật cờ Production bị chặn bởi CEL-190.</t>
+          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.9): FINAL HARDENING 04/10/2026 — 33 bất biến khoá bằng test (docs/chien-luoc/CEL-186-INVARIANTS.md): chặn trước ngày sinh / chưa hợp tuổi / lệch giới bằng câu mã (không model, hoàn lượt), chủ đề bản thân+công việc / nhà cửa, câu chốt cân bằng, câu tháng dương–âm–nhuận VI/EN, oracle tên độc lập + đột biến. Cờ Production vẫn TẮT.</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -15906,7 +15906,7 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>Chặn bật cờ Production: CEL-190 (planner nhận sai chủ đề; và đường STANDARD vẫn hiểu "tháng N" là tháng âm — phải thống nhất với Focused trước khi bật). Giới hạn EN: planner, phân khuôn và các chốt kiểm khuyên / chắc chắn chỉ đọc tiếng Việt; thân bài do model viết vẫn là tiếng Việt — người dùng EN chỉ nhận câu mã, chip, lối đi, miễn trừ bằng EN. Barnum 3: tỉ lệ phân định thấp (27,8%) vì bài nêu ít tên và hai lá số mẫu 1944 gần như trùng — con số đạt dựa trên 10 ca. Lời luận tháng: thân bài đôi khi lấy sao gốc cung Quan Lộc (Thiên Cơ) gán cho tháng — guard N1 chỉ đòi ≥ 1 câu có mã nguyệt hạn.</t>
+          <t>CEL-190 đã gộp vào CEL-186 (sửa ở lớp Focused ke-thua.ts, không đổi bảng planner nên STANDARD và đệm noi_dung_ai không đổi). Trước khi bật cờ Production: đường STANDARD vẫn hiểu 'tháng N' là tháng âm — phải thống nhất. Dễ đọc là luồng việc SAU Production, cổng cứng là đúng dữ kiện. Giới hạn EN: planner chỉ hiểu tiếng Việt, chặn tuổi EN đi bằng từ khoá. Nợ: prompt Focused chưa ghim ngôn ngữ trả lời — giao diện EN gõ câu tiếng Việt thì câu mã EN, thân bài tiếng Việt (eval E16).</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -16102,7 +16102,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Chưa làm — mở 04/10/2026</t>
+          <t>Đã gộp vào CEL-186 (final hardening 04/10/2026)</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -16137,7 +16137,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>Không chặn merge vé B khi cờ Production TẮT. CHẶN bật CELES_FOCUSED_CHAT=1 trên Production (chủ dự án 04/10). Sửa planner là đổi cả STANDARD: bộ vàng eval-planner (100%) không được tụt; thêm hai câu này vào bộ vàng.</t>
+          <t>Sửa ở lớp Focused (lib/rag/focused/ke-thua.ts lapKeHoachChinh + planner.lapKeHoachVoiChuDe), không đổi bảng planner → PHIEN_BAN_PLANNER giữ 2026.10.4, bộ vàng 100/100. STANDARD vẫn giữ hành vi cũ ở hai mẫu câu này (chủ ý, tránh xả đệm).</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -16163,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G256"/>
+  <dimension ref="A1:G258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25504,6 +25504,80 @@
         </is>
       </c>
     </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Giới hạn của lá số (trước sinh / chưa hợp tuổi / lệch giới)</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>gioiHan trong traLoiFocused chạy sau kế hoạch luật (luotMot=true) VÀ sau kế hoạch model (luotMot=false), trước truy hồi, theo thứ tự: chanTruocSinh (mốc NGƯỜI HỎI GỌI TÊN kết thúc trước ngày sinh dương; tháng chứa ngày sinh vẫn đọc; không gọi mốc thì không xét) → chanLechGioi ('chồng tôi' trên lá số nam / 'vợ tôi' trên lá số nữ → câu hỏi lại, không suy đoán; đường từ khoá đòi người hỏi tự xưng, 'anh ấy đã có vợ' không bắt) → chanChuaHopTuoi (tuổi âm của năm đang đọc &lt; 15 và câu về việc làm / hôn nhân / người yêu CỦA CHÍNH người có lá số, VI + từ khoá EN; không chặn câu cả đời 'giai-doan', câu thiên hướng nghề, câu về người khác trong nhà; lượt hai chỉ xét từ khoá + vai, không xét chủ đề, để một câu không lúc chặn lúc không). Trả câu mã qua traNgay(..., khongTinhLuot=true): provider 'ma', model focused-truoc-sinh / focused-lech-gioi / focused-chua-hop-tuoi; route thấy khongTinhLuot thì hoanCauHoi thay chotCauHoi. Chủ đề (ke-thua.ts): 'vay'/'tien' trần không bắt tài chính (gõ không dấu 'vậy', 'thuận tiện').</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>AGE-01..03, PERSON-03/04 trong CEL-186-INVARIANTS.md. Trước 04/10 lá số 22/5/2026 (0 tuổi) vẫn được luận việc làm, chồng, người yêu và câu 'tháng 6 năm 2025' (trước sinh) vẫn được trả lời; 'chồng tôi' trên lá số nam không ai nhận ra. Tuổi tính theo NĂM ĐANG ĐỌC, không theo hôm nay. Nợ: lá số coi là của người hỏi (idDangXem ?? idMacDinh); chỉ 3 lớp chặn mới hoàn lượt, F2/D/nhuận vẫn tính lượt.</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/gioi-han.ts; lib/rag/focused/tra-loi-focused.ts; lib/rag/focused/cau-ma.ts; lib/rag/focused/thang-am.ts; app/api/hoi-dap/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Oracle tên độc lập + bộ bất biến</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>scripts/oracle-ten-prompt.ts render dungPromptFocused hai lần (đầy đủ và chỉ khung: gói rỗng, không khối nghiêng), trừ dòng theo bội số, quét tên trên phần còn lại (+ câu hỏi khi tra cứu). KHÔNG gọi tenDuocGoiTrongLuot / nghiengHienThi. test-focused: guard ⊆ oracle trên 3 lá số × 10 câu (có tháng dương và âm, mốc thời gian thật); đột biến cấp quyền d.sao phải bị oracle bắt ở MỌI ca có tên chỉ-metadata. eval-focused đo 'tên ngoài gói' bằng oracle này qua vetFocused.dauVaoPrompt (chỉ tham chiếu, route không trả ra).</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>GROUND-04/06. Bộ đo dựng từ cùng hàm với guard tự xác nhận cùng nguồn sai: 04/10 bộ đo báo 0 tên ngoài gói trong khi Phá Toái / Thiên Y lọt qua d.sao. Không được để ai thêm vetFocused vào ghiVetTraLoi hay NextResponse.</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>scripts/oracle-ten-prompt.ts; scripts/test-focused.ts; scripts/eval-focused.ts; lib/rag/focused/chay.ts; docs/chien-luoc/CEL-186-INVARIANTS.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25516,7 +25590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F154"/>
+  <dimension ref="A1:F155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30454,6 +30528,38 @@
         </is>
       </c>
       <c r="F154" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>CEL-186, CEL-190</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>FINAL HARDENING vé B (focused-2026.10.9): 33 bất biến có test; chặn trước sinh / chưa hợp tuổi / lệch giới bằng câu mã hoàn lượt; chủ đề bản thân+công việc → Sự nghiệp, nhà cửa → Gia đạo, mua nhà/vay giữ Tài chính (gộp CEL-190, sửa ở lớp Focused); câu chốt hướng cân bằng nêu hai phía hoặc không nêu tên; câu mã tháng dương/âm/nhuận nói rõ việc quy đổi, VI/EN; oracle tên render prompt độc lập + đột biến; sửa thước đo tên ngoài gói của eval; 5 bài học vào docs/bay/ai-rag.md.</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Chủ dự án 04/10/2026 yêu cầu một đợt cứng hoá cuối trước UAT/merge thay vì vá từng vé: A/B văn phong lộ các lỗi có ở CẢ hai bản (bé 0 tuổi được luận chuyện chồng, câu trước năm sinh vẫn trả lời, 'chồng tôi' trên lá số nam, câu chốt cân bằng chỉ nêu một phía) và bộ đo tên tự xác nhận cùng nguồn với guard. Khoá từng luật bằng test để lần sửa sau không âm thầm phá. Sửa chủ đề ở Focused chứ không ở bảng planner để không đổi PHIEN_BAN_PLANNER, không xả đệm, không đổi STANDARD.</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 ve B — doc nam tieng Anh o lop Focused (AGE-01 EN)
"How was my health in 2025?" tren la so sinh 2026 nay bi chan truoc ngay sinh, hoan luot.

Vi sao: UAT 04/10 cau EN goi nam lot chan truoc sinh (planner chi doc tieng Viet), model doc nam dang xem, guard bo het cau, thu lai roi 502. Va o lop Focused, khong doi bang planner, PHIEN_BAN_PLANNER va STANDARD.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -25590,7 +25590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F155"/>
+  <dimension ref="A1:F156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30560,6 +30560,38 @@
         </is>
       </c>
       <c r="F155" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat, sau 3c86fcb)</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Lớp Focused (ke-thua.ts lapKeHoachChinh) đọc năm gọi bằng tiếng Anh ('in 2025', 'Will 2027…') vào namMucTieu khi planner không thấy năm; thêm test AGE-01 năm EN và ca đầu-cuối.</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>UAT 04/10: 'How was my health in 2025?' trên lá số sinh 22/5/2026 không bị chặn trước ngày sinh (planner chỉ đọc tiếng Việt, mốc rơi về năm đang xem), model đọc năm 2026, guard bỏ hết câu, thử lại rồi 502. An toàn nhưng tệ cho người dùng. Vá ở lớp Focused để không đổi bảng planner, PHIEN_BAN_PLANNER và STANDARD.</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-186 ve B buoc 1 — luat chu chi dinh tuyen, khong tu ket thuc luot (focused-2026.10.10)
- Khuon D ("khi nao") khong con cau ma: di qua model o muc nam, guard MOC_NHO_HON_NAM,
  khoiMoc bo "con N thang"/"Sau Tet", go cum thoi quen (THOI_QUEN) truoc khi do D.
- F2 thanh hoi lai khong tinh luot (hoiLaiVanRieng, chuNhan); chip dau tra loi cau goc
  trong mot cham, chip quan he ra F1.
- Bo PERSON-03 (chanLechGioi). AGE-02 giu, goi la ngoai le tam, khong tinh luot.
- CI moi scripts/test-loi-chi-ma.ts canh danh sach loi dung bang ma (du kien / hoi lai /
  dung 1 ngoai le tam). Eval tay scripts/eval-cau-doi-thuong.ts: 15/15, $0.035.
- Docs: INVARIANTS STOP-01..04, HUONG-DAN, AGENTS, backlog.

Vi sao: UAT Preview 04/10 "khi nao toi co viec moi" nhan cau ma tu choi, khong goi model
ma van tru luot. Chu du an DUYET BUOC 1 (Q1-Q6). Co Production van TAT.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.9): FINAL HARDENING 04/10/2026 — 33 bất biến khoá bằng test (docs/chien-luoc/CEL-186-INVARIANTS.md): chặn trước ngày sinh / chưa hợp tuổi / lệch giới bằng câu mã (không model, hoàn lượt), chủ đề bản thân+công việc / nhà cửa, câu chốt cân bằng, câu tháng dương–âm–nhuận VI/EN, oracle tên độc lập + đột biến. Cờ Production vẫn TẮT.</t>
+          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.10): BƯỚC 1 sau UAT 04/10/2026 — luật chữ chỉ được định tuyến, không được tự kết thúc lượt. Lượt trả bằng mã chỉ còn: dữ kiện (trước sinh, tháng nhuận chưa tách), hỏi lại F2 (không tính lượt, chip một chạm trả lời câu gốc), một ngoại lệ tạm AGE-02 (không tính lượt). 'Khi nào' đi qua model ở mức năm. Bỏ PERSON-03. CI test-loi-chi-ma canh danh sách. Cờ Production vẫn TẮT.</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -15906,7 +15906,7 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>CEL-190 đã gộp vào CEL-186 (sửa ở lớp Focused ke-thua.ts, không đổi bảng planner nên STANDARD và đệm noi_dung_ai không đổi). Trước khi bật cờ Production: đường STANDARD vẫn hiểu 'tháng N' là tháng âm — phải thống nhất. Dễ đọc là luồng việc SAU Production, cổng cứng là đúng dữ kiện. Giới hạn EN: planner chỉ hiểu tiếng Việt, chặn tuổi EN đi bằng từ khoá. Nợ: prompt Focused chưa ghim ngôn ngữ trả lời — giao diện EN gõ câu tiếng Việt thì câu mã EN, thân bài tiếng Việt (eval E16).</t>
+          <t>BƯỚC 2 (nhánh mới, cổng trước khi bật cờ Production): biết quan hệ người hỏi ↔ lá số ở tầng dữ liệu; bộ đọc thời gian chung VI/EN ('When will…' đang ra khuôn B); mở rộng lapKeHoachDayDu thay vì viết bộ hiểu câu mới; hạ AGE-02 thành cách nói; thống nhất STANDARD 'tháng N' = dương; đo p95 độ trễ và chi phí. Nợ: prompt Focused chưa ghim ngôn ngữ trả lời (EN: câu mã tiếng Anh, thân bài model tiếng Việt — thấy lại ở eval đời thường ca 11). Câu tháng nhuận chưa tách vẫn tính lượt. Model đôi khi gán nghĩa ngoài dữ kiện (Lộc Tồn = 'kết quả chính thức', Hữu Bật 'người từng được bạn giúp'). Câu F2 mới chờ chủ dự án duyệt chữ.</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -15916,7 +15916,7 @@
       </c>
       <c r="O186" s="8" t="inlineStr">
         <is>
-          <t>Vé A: c5651d2, 2c8963c + merge 10e351f. Vé B: 6ea882f..85667e5, 8113e14, 22ac260, merge 3ba1912, ab22d61, 37a51fb, 7b5a195 + commit sau chốt 04/10 (nhánh viec/cel-186-focused-chat)</t>
+          <t>Vé A: c5651d2, 2c8963c + merge 10e351f. Vé B: 6ea882f..85667e5, 8113e14, 22ac260, merge 3ba1912, ab22d61, 37a51fb, 7b5a195, 28f274c..d56a896 + bước 1 (nhánh viec/cel-186-focused-chat)</t>
         </is>
       </c>
     </row>
@@ -16163,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G258"/>
+  <dimension ref="A1:G260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -24972,12 +24972,12 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào, E A hay B, F1 quan hệ, F2 vận riêng người khác, G không hướng. F2, D, tháng nhuận (gõ "nhuận" hoặc tháng dương rơi vào tháng nhuận — từ 04/10 không còn hỏi lại, xem #17): mã trả trọn lượt (provider 'ma', model focused-f2/-d/-nhuan-chua-tach), không truy hồi, không gọi model, vẫn trừ lượt. Tháng nhuận đã chọn (chip "Tháng X nhuận" hoặc gõ thẳng) fail closed: câu mã nói Celes chưa tách riêng được vận tháng nhuận, chip quay về "Tháng X âm" thường; kiểm ở cả lượt 1 và lượt 2 (sau kế thừa). E, N2 tháng đã qua, N4 cuối năm: câu mã đứng đầu, model viết phần sau.</t>
+          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào (laHoiKhiNao, gỡ cụm thói quen 'lúc/năm nào cũng', 'bao giờ cũng', 'chưa/không bao giờ' trước khi dò), E A hay B, F1 quan hệ, F2 vận riêng người khác, G không mốc. Từ 04/10 (bước 1): D KHÔNG còn câu mã — đi qua model với KHOI_KHUON.D (đọc mức năm, nói bằng lời mình rằng lượt này chưa chọn tháng và muốn xem tháng nào thì hỏi riêng; nhắc hoàn cảnh người hỏi kể; cấm tháng/mùa/quý/'cuối năm'/'sau Tết'), khoiMoc bỏ 'còn N tháng' và 'Sau Tết… đại vận mới' cho D, guard luật 6 coi MOC_NHO_HON_NAM là mốc lạ ở D, chip 'Sang năm … thì sao?' khi năm hiệu lực là năm nay. F2 là HỎI LẠI không tính lượt (hoiLaiVanRieng): 'Celes chưa biết lá số đang mở là của ai…' (chuNhan tránh 'bạn bạn', nhãn số nhiều → 'một người trong …'); chip 1 = câu gốc với cụm '&lt;người&gt; tôi' đổi thành 'người có lá số này' (một chạm, không ra F2 lần hai, giữ chủ đề), chip 2 = câu quan hệ → F1.</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Cờ #3, #4, #5: bỏ D′ và chip "Tháng nào đáng chú ý hơn?" (engine không so tháng → ngõ cụt). Không bao giờ gọi logic tháng thường cho tháng nhuận (chủ dự án 03/10: không phải lệch đã biết mà là lỗi) — bản đầu chip "Tháng X nhuận" đọc nguyệt hạn tháng X thường.</t>
+          <t>UAT 04/10: 'khi nào tôi có việc mới' / 'đang thất nghiệp, khi nào tìm được việc' nhận câu mã, không gọi model mà vẫn trừ lượt — luật chữ được quyền tự kết thúc lượt. Luật STOP-01..04 (CEL-186-INVARIANTS.md): lượt bằng mã chỉ khi dữ kiện máy kiểm được, hỏi lại vì thiếu dữ kiện thật, hoặc ĐÚNG MỘT ngoại lệ tạm (AGE-02). Máy canh: scripts/test-loi-chi-ma.ts (CI). Eval đời thường lần 1: 'Năm nào cũng vất vả…' bị xếp D và chèn câu 'chưa khoanh tháng' thừa; prompt cũ đưa câu nguyên văn nên model chép 5/6 bài và đổ lỗi cho lá số dù nguyệt hạn đọc được.</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -25522,17 +25522,17 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Giới hạn của lá số (trước sinh / chưa hợp tuổi / lệch giới)</t>
+          <t>Giới hạn của lá số (trước sinh / chưa hợp tuổi)</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>gioiHan trong traLoiFocused chạy sau kế hoạch luật (luotMot=true) VÀ sau kế hoạch model (luotMot=false), trước truy hồi, theo thứ tự: chanTruocSinh (mốc NGƯỜI HỎI GỌI TÊN kết thúc trước ngày sinh dương; tháng chứa ngày sinh vẫn đọc; không gọi mốc thì không xét) → chanLechGioi ('chồng tôi' trên lá số nam / 'vợ tôi' trên lá số nữ → câu hỏi lại, không suy đoán; đường từ khoá đòi người hỏi tự xưng, 'anh ấy đã có vợ' không bắt) → chanChuaHopTuoi (tuổi âm của năm đang đọc &lt; 15 và câu về việc làm / hôn nhân / người yêu CỦA CHÍNH người có lá số, VI + từ khoá EN; không chặn câu cả đời 'giai-doan', câu thiên hướng nghề, câu về người khác trong nhà; lượt hai chỉ xét từ khoá + vai, không xét chủ đề, để một câu không lúc chặn lúc không). Trả câu mã qua traNgay(..., khongTinhLuot=true): provider 'ma', model focused-truoc-sinh / focused-lech-gioi / focused-chua-hop-tuoi; route thấy khongTinhLuot thì hoanCauHoi thay chotCauHoi. Chủ đề (ke-thua.ts): 'vay'/'tien' trần không bắt tài chính (gõ không dấu 'vậy', 'thuận tiện').</t>
+          <t>gioiHan trong traLoiFocused chạy sau kế hoạch luật (luotMot=true) VÀ sau kế hoạch đầy đủ: chanTruocSinh (AGE-01, dữ kiện, không tính lượt) và chanChuaHopTuoi (AGE-02, NGOẠI LỆ TẠM, không tính lượt, đóng băng — không thêm từ khoá, bước 2 hạ thành cách nói). chanLechGioi (PERSON-03) đã bỏ 04/10: lá số đang mở có thể không phải của người hỏi, 'chồng tôi' trên lá số nam đi đường thường.</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>AGE-01..03, PERSON-03/04 trong CEL-186-INVARIANTS.md. Trước 04/10 lá số 22/5/2026 (0 tuổi) vẫn được luận việc làm, chồng, người yêu và câu 'tháng 6 năm 2025' (trước sinh) vẫn được trả lời; 'chồng tôi' trên lá số nam không ai nhận ra. Tuổi tính theo NĂM ĐANG ĐỌC, không theo hôm nay. Nợ: lá số coi là của người hỏi (idDangXem ?? idMacDinh); chỉ 3 lớp chặn mới hoàn lượt, F2/D/nhuận vẫn tính lượt.</t>
+          <t>AGE-01..03, STOP-03 trong CEL-186-INVARIANTS.md. Chủ dự án 04/10: 'Temporary terminal allowlist chỉ được có đúng AGE-02' — thêm ngoại lệ thứ hai thì test-loi-chi-ma đỏ.</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -25575,6 +25575,80 @@
       <c r="G258" t="inlineStr">
         <is>
           <t>scripts/oracle-ten-prompt.ts; scripts/test-focused.ts; scripts/eval-focused.ts; lib/rag/focused/chay.ts; docs/chien-luoc/CEL-186-INVARIANTS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Danh sách lối dừng bằng mã (CI)</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>scripts/test-loi-chi-ma.ts đọc mọi lời gọi traNgay(…) trong tra-loi-focused.ts, đối chiếu CHO_PHEP: focused-truoc-sinh (DU_KIEN), focused-nhuan-chua-tach (DU_KIEN, 2 chỗ), focused-f2 (HOI_LAI), focused-chua-hop-tuoi (NGOAI_LE_TAM). HOI_LAI và NGOAI_LE_TAM phải truyền khongTinhLuot = true; trần NGOAI_LE_TAM = 1; chỉ một chỗ dựng provider 'ma'; 'focused-d' quay lại là đỏ.</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Luật bằng chữ đã lặp lại lỗi ('câu mã thay vì trả lời') nên phải có máy canh. Đột biến bỏ 'true' ở F2 làm test đỏ (đã thử).</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>scripts/test-loi-chi-ma.ts; .github/workflows/kiem-tra.yml; lib/rag/focused/tra-loi-focused.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Eval câu đời thường có vết</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>scripts/eval-cau-doi-thuong.ts (model thật, chạy tay, AI_TRAN_USD ≤ 0.1): 15 câu người dùng thật hay gõ trên 4 lá số (2 người lớn, 2 bé), mỗi ca in vết khuôn / chủ đề / ý định / dùng mã hay model / tính lượt / dữ kiện; chấm: không mốc nhỏ hơn năm ở câu khi nào, nhắc hoàn cảnh, chip F2 một chạm ra câu trả lời thật. --xuat &lt;tệp.json&gt; ghi vết.</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Eval cũ chấm đúng khuôn nên câu mã 'đúng thiết kế' vẫn đạt dù người dùng không được trả lời. Lần chạy 04/10: 15/15, $0.035; đọc tay bắt thêm lỗi phân khuôn câu thói quen và câu nguyên văn trong prompt mà bộ chấm không thấy.</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>scripts/eval-cau-doi-thuong.ts</t>
         </is>
       </c>
     </row>
@@ -25590,7 +25664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F156"/>
+  <dimension ref="A1:F157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30592,6 +30666,38 @@
         </is>
       </c>
       <c r="F156" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Vé B bước 1 (focused-2026.10.10): 'khi nào' đi qua model ở mức năm (prompt D mới, khối mốc bỏ mốc nhỏ hơn năm, guard MOC_NHO_HON_NAM, gỡ cụm thói quen khỏi D); F2 thành hỏi lại không tính lượt với chip một chạm trả lời câu gốc; bỏ PERSON-03; AGE-02 gọi là ngoại lệ tạm; CI test-loi-chi-ma; eval 15 câu đời thường.</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>UAT Preview 04/10: chủ dự án hỏi 'khi nào tôi có việc mới' và 'đang thất nghiệp, khi nào tìm được việc' — Celes trả câu mã từ chối, không gọi model mà vẫn trừ lượt. Gốc: luật chữ (D, F2, lệch giới) được quyền tự kết thúc lượt. Chủ dự án DUYỆT BƯỚC 1 (Q1–Q6: gộp với cờ Production tắt; chỉ dừng bằng mã khi là dữ kiện hoặc hỏi lại thật; khi nào đọc mức năm; tháng N = dương; bước 2 là cổng trước Production; mở rộng lapKeHoachDayDu). Eval model thật 15/15 sau sửa, $0.035/lần.</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 ve B buoc 1 — cau hoi lai F2 theo nguyen van chu du an
- Cau F2 VI dung nguyen van duoc duyet ("luan van rieng", khong "doan"; khong
  khang dinh la so la cua ai), them ban EN. Bo chuNhan vi khong con ghep ten.
- Backlog: no "than bai/chip EN ra tieng Viet" thanh chan truoc Production.

Vi sao: chu du an duyet buoc 1 ngay 04/10, chon "luan" vi "doan" lam yeu cam giac
ket luan co can cu tu la so.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15906,7 +15906,7 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>BƯỚC 2 (nhánh mới, cổng trước khi bật cờ Production): biết quan hệ người hỏi ↔ lá số ở tầng dữ liệu; bộ đọc thời gian chung VI/EN ('When will…' đang ra khuôn B); mở rộng lapKeHoachDayDu thay vì viết bộ hiểu câu mới; hạ AGE-02 thành cách nói; thống nhất STANDARD 'tháng N' = dương; đo p95 độ trễ và chi phí. Nợ: prompt Focused chưa ghim ngôn ngữ trả lời (EN: câu mã tiếng Anh, thân bài model tiếng Việt — thấy lại ở eval đời thường ca 11). Câu tháng nhuận chưa tách vẫn tính lượt. Model đôi khi gán nghĩa ngoài dữ kiện (Lộc Tồn = 'kết quả chính thức', Hữu Bật 'người từng được bạn giúp'). Câu F2 mới chờ chủ dự án duyệt chữ.</t>
+          <t>BƯỚC 2 (nhánh mới, cổng trước khi bật cờ Production): biết quan hệ người hỏi ↔ lá số ở tầng dữ liệu; bộ đọc thời gian chung VI/EN ('When will…' đang ra khuôn B); mở rộng lapKeHoachDayDu thay vì viết bộ hiểu câu mới; hạ AGE-02 thành cách nói; thống nhất STANDARD 'tháng N' = dương; đo p95 độ trễ và chi phí. CHẶN TRƯỚC PRODUCTION (chủ dự án 04/10): thân bài model và chip ra tiếng Việt khi người dùng dùng giao diện EN (prompt Focused chưa ghim ngôn ngữ; eval đời thường ca 11). Nợ khác: câu tháng nhuận chưa tách vẫn tính lượt; model đôi khi gán nghĩa ngoài dữ kiện (Lộc Tồn = 'kết quả chính thức', Hữu Bật 'người từng được bạn giúp'); bấm chip F2 xong model vẫn mở 'Nếu đây là lá số của con bạn'; câu hai ý chỉ trả lời ý đầu.</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -24972,7 +24972,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào (laHoiKhiNao, gỡ cụm thói quen 'lúc/năm nào cũng', 'bao giờ cũng', 'chưa/không bao giờ' trước khi dò), E A hay B, F1 quan hệ, F2 vận riêng người khác, G không mốc. Từ 04/10 (bước 1): D KHÔNG còn câu mã — đi qua model với KHOI_KHUON.D (đọc mức năm, nói bằng lời mình rằng lượt này chưa chọn tháng và muốn xem tháng nào thì hỏi riêng; nhắc hoàn cảnh người hỏi kể; cấm tháng/mùa/quý/'cuối năm'/'sau Tết'), khoiMoc bỏ 'còn N tháng' và 'Sau Tết… đại vận mới' cho D, guard luật 6 coi MOC_NHO_HON_NAM là mốc lạ ở D, chip 'Sang năm … thì sao?' khi năm hiệu lực là năm nay. F2 là HỎI LẠI không tính lượt (hoiLaiVanRieng): 'Celes chưa biết lá số đang mở là của ai…' (chuNhan tránh 'bạn bạn', nhãn số nhiều → 'một người trong …'); chip 1 = câu gốc với cụm '&lt;người&gt; tôi' đổi thành 'người có lá số này' (một chạm, không ra F2 lần hai, giữ chủ đề), chip 2 = câu quan hệ → F1.</t>
+          <t>phanKhuon: A có/không, B mô tả có mốc, C quyết định, D khi nào (laHoiKhiNao, gỡ cụm thói quen 'lúc/năm nào cũng', 'bao giờ cũng', 'chưa/không bao giờ' trước khi dò), E A hay B, F1 quan hệ, F2 vận riêng người khác, G không mốc. Từ 04/10 (bước 1): D KHÔNG còn câu mã — đi qua model với KHOI_KHUON.D (đọc mức năm, nói bằng lời mình rằng lượt này chưa chọn tháng và muốn xem tháng nào thì hỏi riêng; nhắc hoàn cảnh người hỏi kể; cấm tháng/mùa/quý/'cuối năm'/'sau Tết'), khoiMoc bỏ 'còn N tháng' và 'Sau Tết… đại vận mới' cho D, guard luật 6 coi MOC_NHO_HON_NAM là mốc lạ ở D, chip 'Sang năm … thì sao?' khi năm hiệu lực là năm nay. F2 là HỎI LẠI không tính lượt (hoiLaiVanRieng), câu nguyên văn chủ dự án duyệt 04/10: 'Để Celes không luận vận riêng của một người bằng nhầm lá số, bạn cho Celes biết: lá số đang mở là của người bạn đang hỏi, hay là của bạn?' (dùng 'luận', không 'đoán'; không khẳng định lá số là của ai). Chip 1 = câu gốc với cụm '&lt;người&gt; tôi' đổi thành 'người có lá số này' (một chạm, không ra F2 lần hai, giữ chủ đề), chip 2 = câu quan hệ → F1.</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -25664,7 +25664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F157"/>
+  <dimension ref="A1:F158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30698,6 +30698,38 @@
         </is>
       </c>
       <c r="F157" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Câu hỏi lại F2 thay bằng nguyên văn chủ dự án: 'Để Celes không luận vận riêng của một người bằng nhầm lá số, bạn cho Celes biết: lá số đang mở là của người bạn đang hỏi, hay là của bạn?' (+ bản EN). Bỏ chuNhan (không còn cần ghép tên người). Ghi nợ EN thành chặn trước Production.</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt bước 1 (04/10) và chọn 'luận vận riêng' thay 'đoán': 'đoán' làm giảm cảm giác kết luận có căn cứ từ lá số. Câu mới hỏi thẳng lá số là của ai thay vì giải thích hai nhánh, và không nói 'lá số này là của bạn' vì hệ thống chưa biết. Chủ dự án coi thân bài/chip EN ra tiếng Việt là blocker trước khi bật Focused Production, không chặn Preview UAT.</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-186 v2 A — vet Preview [focused-vet], khong doi van tra loi
Vet chi ma va so (requestId, khuon, ma F/E, chunkIds, ms/token/loi tung lan goi),
ghi khi CELES_FOCUSED_TRACE=1 va khong phai production that.

Vi sao: spec Answer Contract v2 muc 5.4 — can so that ve tre, viet lai, 502 tren
Preview truoc khi doi hop dong tra loi; khong luu noi dung nguoi dung.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16163,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G260"/>
+  <dimension ref="A1:G261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25652,6 +25652,43 @@
         </is>
       </c>
     </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Vết Preview (Answer Contract v2, commit A)</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>traLoiFocused gom VetPreview (requestId, phienBan, loiRa ok/502/ma-&lt;lối&gt;, hieu{chuDe,yDinh,khuon,coDoiTuong,thoiGian,nguon,giaiThichLuotTruoc,coChoHoiLai}, mã F/E, chunkIds, lan[{stt,ms,tokVao,tokRa,loi[{ma}]}], ketQua số ký tự/âm tiết/claim/chip, msTong, msTruyHoi, usdUocTinh). Route gọi ghiVetPreview sau traLoiCoCanCu: một dòng console.info '[focused-vet] {json}' CHỈ KHI CELES_FOCUSED_TRACE=1 và !laProductionThat().</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Production không bao giờ ghi, kể cả lỡ đặt cờ. Vết chỉ mã và số: không câu hỏi, câu trả lời, claim, đoạn RAG, chiTiet, nhãn hoàn cảnh, tên, vai (test-focused kiểm bằng chuỗi đánh dấu). Văn trả lời không đổi khi bật vết.</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/vet.ts; lib/rag/focused/chay.ts; lib/rag/focused/tra-loi-focused.ts; app/api/hoi-dap/route.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25664,7 +25701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F158"/>
+  <dimension ref="A1:F159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30730,6 +30767,38 @@
         </is>
       </c>
       <c r="F158" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Answer Contract v2 commit A: vết Preview [focused-vet] cho đường Focused (thời gian, token, lỗi từng lần gọi, mã căn cứ, chunk), không đổi văn trả lời.</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Spec CEL-186 v2 (chủ dự án FREEZE 04/10) mục 5.4: cần số thật về trễ / viết lại / 502 trên Preview trước khi đổi hợp đồng trả lời (bước B lấy mốc gốc từ đây). Không lưu nội dung người dùng vì chủ đề + quan hệ + requestId đã là suy luận cá nhân.</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-186 v2 D — model viet tron bai (answer + claims), viet lai mot lan roi 502
- focused/hop-dong.ts (moi): BanNhap {answer, claims[], suggestedQuestions}, docBanNhap
- chay.ts: kiemCung toi thieu (SCHEMA, KHONG_CAN_CU, MA_KHONG_HOP_LE, LO_MA);
  truot thi viet lai TOAN bai mot lan (con >=16s), van truot thi van='' (502 + hoan luot)
- prompt.ts: schema moi, bo tran do dai, cau 8.1, ghim EN, khoi viet lai
- tra-loi-focused.ts: ketLuan/yChinh tu claims; bo ghepVan/docFocused/cat cau/chot du phong
- test-focused + test-hop-dong-focused theo hop dong moi

Vi sao: UAT vé B 04/10 cho thay ghep cau + chot du phong ra van roi, lap, lech
hoan canh; xoa cau truot guard lam bai cut. Spec v2 (FREEZE 04/10) muc 2.2/5.3/8.1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16163,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G261"/>
+  <dimension ref="A1:G262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25689,6 +25689,43 @@
         </is>
       </c>
     </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Hợp đồng đầu ra answer + claims + viết lại một lần (Answer Contract v2, commit D)</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Model trả JSON {answer, claims[{claim, evidenceIds, direction?, timeRefs?}], suggestedQuestions, hoanCanhNhanRa?, outOfScope?} (hop-dong.ts docBanNhap; claim cắt 200 ký tự, hoàn cảnh ≤3 nhãn ≤6 từ). answer là văn người đọc thấy (qua boMarkdown), claims không hiển thị — chỉ là căn cứ (coCauTruc.ketLuan = claims[0].claim, yChinh từ claims). chayFocused: gọi (maxTokens 6000) → kiemCung (SCHEMA, MA_KHONG_HOP_LE, KHONG_CAN_CU miễn khi outOfScope, LO_MA) → trượt thì viết lại TOÀN bài một lần kèm lỗi (khoiVietLai), chỉ khi còn ≥16s trong hạn chót 50s → vẫn trượt thì van='' (route 502 + hoàn lượt). Prompt: bỏ trần độ dài, câu 8.1 'đủ ý, không lặp ý'; 'sau' = 'Người hỏi muốn nghe kỹ.'; ghim tiếng Anh ở dòng đầu system khi en.</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Không xoá câu, không cắt độ dài, không văn dự phòng tất định, không trả bản lần một khi còn lỗi cứng. Mã F/E chỉ ở claims, lộ vào answer là LO_MA. Câu mã (cauMa) tạm vẫn đứng đầu van; E/G gỡ dần. Cờ CELES_FOCUSED_CHAT tắt = STANDARD nguyên vẹn.</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/hop-dong.ts; lib/rag/focused/kiem.ts; lib/rag/focused/chay.ts; lib/rag/focused/prompt.ts; lib/rag/focused/tra-loi-focused.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25701,7 +25738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F159"/>
+  <dimension ref="A1:F160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30799,6 +30836,38 @@
         </is>
       </c>
       <c r="F159" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Answer Contract v2 commit D: model viết trọn bài (answer) kèm claims có mã căn cứ; validator cứng tối thiểu; trượt thì viết lại toàn bài một lần, vẫn trượt thì 502 + hoàn lượt. Bỏ ghepVan/docFocused, cắt câu, trần độ dài và câu chốt dự phòng.</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>UAT Preview vé B (04/10): ghép câu từ mảng cau + cauChot dự phòng cho ra văn rời, lặp, có câu 'thất nghiệp' trả lời lệch hoàn cảnh; xoá câu trượt guard làm bài cụt. Spec v2 (chủ dự án FREEZE 04/10) mục 2.2/5.3/8.1: model viết trọn bài, căn cứ kiểm qua claims, lỗi thì viết lại cả bài chứ không vá — thà 502 có hoàn lượt còn hơn văn sai.</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-186 v2 E — validator cung du bang 5.1, viet lai mot lan roi 502
- kiemCung du 14 ma (SCHEMA, MA_KHONG_HOP_LE, KHONG_CAN_CU, TEN_*, LUU_HOA,
  MOC_BIA theo tap moc hop le, MOC_NHO_HON_NAM chi D, PHAN_TRAM, CHAC_CHAN_GIA,
  CHON_HO chi C/E, LO_NGUON, LO_MA, NGUOC_HUONG, THIEU_THANG)
- tinhMocHopLe thuan; chonChip bo chip khong ket bang dau hoi hoac moc ngoai tap
- bo cau ma E/N2/N4 va cau chot du phong: model tu noi gioi han
- giu cau ngoai tam "khong xac nhan duoc ten" vi no chi noi gioi han, khong ket luan
- dong cuoi nam am khong ap cho khuon D (reviewer bat mau thuan voi MOC_NHO_HON_NAM)
- PHIEN_BAN_FOCUSED focused-2026.10.12

Vi sao: spec v2 (FREEZE 04/10) muc 5: ma chi kiem, khong viet; truot luat cung
thi viet lai ca bai mot lan, van truot thi 502 + hoan luot. UAT Preview thay
cau ma ghep dau bai nghe nhu may va guard cu xoa cau lam bai cut.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16163,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G262"/>
+  <dimension ref="A1:G263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25726,6 +25726,43 @@
         </is>
       </c>
     </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Validator cứng đủ bảng 5.1 + mốc hợp lệ + bỏ câu mã E/N2/N4 (Answer Contract v2, commit E)</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>kiemCung (kiem.ts) báo mỗi mã tối đa một lần: SCHEMA (outOfScope phải đúng 1 câu, claims rỗng), MA_KHONG_HOP_LE, KHONG_CAN_CU, TEN_NGOAI_GOI/LUU_HOA/TEN_BIA quét theo từng câu answer (tachManh) và từng claim, MOC_BIA theo mocHopLeAnswer, MOC_NHO_HON_NAM chỉ khuôn D, PHAN_TRAM, CHAC_CHAN_GIA theo câu, CHON_HO chỉ C/E (chonMotVe cho E), LO_NGUON, LO_MA, NGUOC_HUONG (soChieu: claims[0].direction so hướng engine; thiếu chiều cũng lỗi), THIEU_THANG (hỏi tháng mà không claim nào dẫn nguyệt hạn). tinhMocHopLe thuần: năm = hiệu lực, năm sinh dương+âm, năm trong câu hỏi, năm trong văn F/E, năm dương hai đầu cửa sổ tháng âm; tháng = tháng hỏi, tháng âm, tháng dương hai đầu cửa sổ. Tập chip = answer + năm hiệu lực+1 + tháng kế. chonChip: chip phải kết bằng '?' và mốc thuộc tập chip. Lời văn, khuyên chung, tên cung chỉ đo ở eval. Khuôn E: model tự nói lá số chưa đủ để chọn; mã chỉ cấp chip hai vế. Tháng âm đã qua: model tự nói đang nhìn lại. Cuối năm âm (trừ khuôn D): model tự nói phần sau Tết cần xem riêng.</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Không xoá câu, không câu chốt dự phòng; lỗi thì viết lại một lần rồi 502 + hoàn lượt. Không thêm năm hiệu lực+1 vào tập answer (chỉ chip). Giữ câu mã ngoại tâm 'không xác nhận được tên' vì nó chỉ nói giới hạn. Rủi ro đo ở I: CHAC_CHAN_GIA bắt 'mức nhất định', 'không dám chắc chắn'; CHON_HO bắt 'Nên' liên từ, 'tốt nhất là'; tháng 1 dương đến Tết năm dương hiện tại chưa nằm trong tập mốc.</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/kiem.ts; lib/rag/focused/chot-huong.ts; lib/rag/focused/cau-ma.ts; lib/rag/focused/prompt.ts; lib/rag/focused/tra-loi-focused.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25738,7 +25775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F160"/>
+  <dimension ref="A1:F161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30868,6 +30905,38 @@
         </is>
       </c>
       <c r="F160" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Answer Contract v2 commit E: validator cứng đủ 14 mã bảng 5.1, mốc hợp lệ tính thuần (tinhMocHopLe), chip lọc theo dấu hỏi và mốc; bỏ câu mã E/N2/N4 và câu chốt dự phòng, model tự nói giới hạn; phiên bản focused-2026.10.12.</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>UAT Preview vé B (04/10): câu mã ghép đầu bài nghe như máy và lặp ý model; guard cũ xoá câu làm bài cụt. Spec v2 (chủ dự án FREEZE 04/10) mục 5/5.1: mã chỉ kiểm, không viết; CHON_HO và CHAC_CHAN_GIA là luật cứng, văn phong chỉ đo ở eval. Reviewer bắt dòng cuối năm mời nói 'sau Tết' trong khuôn D (ngược MOC_NHO_HON_NAM) — đã loại khuôn D.</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 v2 I — CHAC_CHAN_GIA khong bat nham cau rao don phu dinh xa
- kiem.ts: chacChanGia(s) bo qua cho khop co "khong/chua/chang + phai/han/co nghia/du/the"
  trong cung ve cau (tach theo , ; : va " ma ", " nhung ")
- test-focused: 5 cau rao don that tu eval khong bi bat; 2 cau phan chac van bi bat

Vi sao: eval mu I 502 = 2/24, audit buoc 5 lan hai 502 = 4/24 (truoc la 0/24), truot cong
<= 3%. Tai hien co vet: moi luot 502 la CHAC_CHAN_GIA bat nham "khong phai dau hieu chac chan
bi cho nghi", "khong co nghia la chac chan mat tien"; viet lai van giu cau truc do nen 502.
Giong chat cua H dung cap phan biet nhieu hon nen loi lo ra.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16163,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G266"/>
+  <dimension ref="A1:G267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25874,6 +25874,43 @@
         </is>
       </c>
     </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>CHAC_CHAN_GIA bỏ qua phủ định xa trong cùng vế câu (sửa lỗi phát hiện ở eval I)</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>kiemCung (lib/rag/focused/kiem.ts) không còn gọi CHAC_CHAN_GIA.exec trực tiếp mà qua chacChanGia(s): duyệt mọi chỗ khớp; chỗ khớp nào có 'không/chưa/chẳng' + 'phải/hẳn/có nghĩa/đủ/thể' trong CÙNG vế câu đứng trước (vế = đoạn sau dấu , ; : hoặc ' mà ', ' nhưng ' gần nhất) thì là rào đón, bỏ qua. Lookbehind cũ '(?&lt;!(?:không|chưa) )' giữ nguyên.</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Eval mù I: 502 = 2/24, audit RAG bước 5 lần hai: 502 = 4/24 (trước H là 0/24). Tái hiện có vết: mọi lượt 502 là CHAC_CHAN_GIA trượt hai lần trên câu rào đón kiểu 'không phải dấu hiệu chắc chắn bị cho nghỉ', 'không có nghĩa là chắc chắn mất tiền'. Giọng chat của H dùng cặp phân biệt (không phải X mà là Y) nhiều hơn nên lỗi lộ ra. Bẫy: tách vế phải gồm cả 'mà'/'nhưng', nếu không thì 'không phải dấu hiệu xấu mà chắc chắn là…' bị bỏ lọt (có test).</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/kiem.ts; scripts/test-focused.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25886,7 +25923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:F165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31144,6 +31181,38 @@
         </is>
       </c>
       <c r="F164" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Validator Focused: CHAC_CHAN_GIA không bắt câu rào đón có phủ định đứng xa trong cùng vế câu. Thêm 5 ca rào đón thật từ eval và 2 ca phán chắc phải vẫn bị bắt vào test-focused.</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Bước I đo 502 = 2/24 (mù) và 4/24 (audit), trượt cổng ≤ 3%. Tái hiện với vết lỗi validator: 100% lượt 502 là CHAC_CHAN_GIA bắt nhầm câu phủ định ('không phải dấu hiệu chắc chắn…'), viết lại một lần vẫn giữ cấu trúc đó nên 502. Đây là lỗi bắt nhầm của chính validator E, không phải model nói chắc.</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 v2 I — CHAC_CHAN_GIA nhan "chua co du can cu" la rao don
- PHU_DINH_VE them "(co )?" va "can cu": "chua co du can cu de khang dinh ... se xay ra"
- test-focused: 2 cau rao don, 1 cau phan chac van bi bat

Vi sao: sau f6f6d46 eval mu 502 = 0/24 nhung audit buoc 5 con 502 = 2/24; tai hien
hai ca do van co luot phai viet lai vi cau rao don dang "chua co du can cu" bi bat nham.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -25897,7 +25897,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>kiemCung (lib/rag/focused/kiem.ts) không còn gọi CHAC_CHAN_GIA.exec trực tiếp mà qua chacChanGia(s): duyệt mọi chỗ khớp; chỗ khớp nào có 'không/chưa/chẳng' + 'phải/hẳn/có nghĩa/đủ/thể' trong CÙNG vế câu đứng trước (vế = đoạn sau dấu , ; : hoặc ' mà ', ' nhưng ' gần nhất) thì là rào đón, bỏ qua. Lookbehind cũ '(?&lt;!(?:không|chưa) )' giữ nguyên.</t>
+          <t>kiemCung (lib/rag/focused/kiem.ts) không còn gọi CHAC_CHAN_GIA.exec trực tiếp mà qua chacChanGia(s): duyệt mọi chỗ khớp; chỗ khớp nào có 'không/chưa/chẳng' + (tuỳ chọn 'có ') + 'phải/hẳn/nghĩa/đủ/thể/căn cứ' trong CÙNG vế câu đứng trước (vế = đoạn sau dấu , ; : hoặc ' mà ', ' nhưng ' gần nhất) thì là rào đón, bỏ qua. Lookbehind cũ '(?&lt;!(?:không|chưa) )' giữ nguyên. Ví dụ rào đón: 'không phải dấu hiệu chắc chắn…', 'không có nghĩa là chắc chắn…', 'chưa có đủ căn cứ để khẳng định … sẽ xảy ra'.</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -25923,7 +25923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F165"/>
+  <dimension ref="A1:F166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31213,6 +31213,38 @@
         </is>
       </c>
       <c r="F165" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Mở rộng mẫu phủ định của CHAC_CHAN_GIA: thêm 'chưa/không có đủ', 'không có căn cứ'. Thêm 2 ca rào đón và 1 ca phán chắc vào test-focused.</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Sau bản sửa f6f6d46: eval mù 502 = 0/24, nhưng audit bước 5 vẫn 502 = 2/24. Tái hiện hai ca đó (5 lần mỗi ca) thì không còn 502, nhưng vẫn có lượt phải viết lại vì câu 'Celes chưa có đủ căn cứ để khẳng định … sẽ xảy ra' bị bắt nhầm. Mỗi lần viết lại tốn thêm một lượt model và khoảng 7 s.</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 v2 I — CHAC_CHAN_GIA nhan "khong dong nghia" la rao don
- PHU_DINH_VE: "nghia" -> "(dong )?nghia"
- test-focused: them ca "khong dong nghia voi viec chac chan"

Vi sao: eval hop dong I4 (155 luot, in ma loi validator) bat nham cau rao don
"Dieu nay khong dong nghia voi viec chac chan nhan viec ngay" -> phai viet lai.
502 cua I4 = 2/155, ca hai do KHONG_CAN_CU, khong do CHAC_CHAN_GIA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -25897,7 +25897,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>kiemCung (lib/rag/focused/kiem.ts) không còn gọi CHAC_CHAN_GIA.exec trực tiếp mà qua chacChanGia(s): duyệt mọi chỗ khớp; chỗ khớp nào có 'không/chưa/chẳng' + (tuỳ chọn 'có ') + 'phải/hẳn/nghĩa/đủ/thể/căn cứ' trong CÙNG vế câu đứng trước (vế = đoạn sau dấu , ; : hoặc ' mà ', ' nhưng ' gần nhất) thì là rào đón, bỏ qua. Lookbehind cũ '(?&lt;!(?:không|chưa) )' giữ nguyên. Ví dụ rào đón: 'không phải dấu hiệu chắc chắn…', 'không có nghĩa là chắc chắn…', 'chưa có đủ căn cứ để khẳng định … sẽ xảy ra'.</t>
+          <t>kiemCung (lib/rag/focused/kiem.ts) không còn gọi CHAC_CHAN_GIA.exec trực tiếp mà qua chacChanGia(s): duyệt mọi chỗ khớp; chỗ khớp nào có 'không/chưa/chẳng' + (tuỳ chọn 'có ') + 'phải/hẳn/(đồng )nghĩa/đủ/thể/căn cứ' trong CÙNG vế câu đứng trước (vế = đoạn sau dấu , ; : hoặc ' mà ', ' nhưng ' gần nhất) thì là rào đón, bỏ qua. Lookbehind cũ '(?&lt;!(?:không|chưa) )' giữ nguyên. Ví dụ rào đón: 'không phải dấu hiệu chắc chắn…', 'không có nghĩa là chắc chắn…', 'không đồng nghĩa với việc chắc chắn…', 'chưa có đủ căn cứ để khẳng định … sẽ xảy ra'.</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -25923,7 +25923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31245,6 +31245,38 @@
         </is>
       </c>
       <c r="F166" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>PHU_DINH_VE nhận thêm 'không đồng nghĩa' là rào đón; thêm 1 ca vào test-focused.</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Eval Behavior Contract I4 (155 lượt, có in mã lỗi validator): câu 'Điều này không đồng nghĩa với việc chắc chắn nhận việc ngay' bị bắt nhầm CHAC_CHAN_GIA và phải viết lại (thêm một lượt model, khoảng 7 s). 502 của I4 = 2/155, cả hai do KHONG_CAN_CU (model không dẫn mã), không do CHAC_CHAN_GIA.</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 v2 I — LO_NGUON he phai can co dau; nhan hoi lai F2 ro hon
- kiem.ts: "nam phai"/"bac phai" chi tinh khi van viet co dau (RO_RI_RAG chung khong doi)
- hieu-cau.ts: prompt giaiHoiLai mo ta ro nguoi-hoi va khong-lien-quan
- test-focused: 1 ca phai bat, 2 ca khong duoc bat nham

Vi sao: eval hop dong I3/I4 — flow 7 (trong yeu) ra chu de su-nghiep 2/5 vi model nho
doc "tien bac toi" thanh "la so nay cua toi"; sau sua do lai 10/10 tai-chinh, flow 4/5/6/24
van 5/5. Vet validator in tam cho thay "tien bac phai" bi LO_NGUON bat thanh "Bac phai".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16163,7 +16163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G267"/>
+  <dimension ref="A1:G268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -25911,6 +25911,43 @@
         </is>
       </c>
     </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Vé B — chat Focused</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Hai bắt nhầm phát hiện qua eval Behavior Contract I (LO_NGUON hệ phái, nhãn hỏi lại F2)</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>(1) kiemCung (lib/rag/focused/kiem.ts): cụm 'nam phai' / 'bac phai' của RO_RI_RAG chỉ tính LO_NGUON khi văn có đúng dạng có dấu 'nam phái' / 'bắc phái' (HE_PHAI_CO_DAU). Các cụm RO_RI_RAG khác giữ cách so bỏ dấu. RO_RI_RAG (vùng Chung, STANDARD dùng) KHÔNG đổi. (2) giaiHoiLai (lib/rag/focused/hieu-cau.ts): prompt model nhỏ mô tả rõ nhãn — 'nguoi-hoi' là người dùng NÓI lá số đang mở là của chính họ; 'khong-lien-quan' gồm cả một câu hỏi mới về chính người dùng. Đường tất định và ba nhãn của spec 6.1 không đổi.</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Bỏ dấu làm chữ thường trùng cụm cấm: 'tiền bạc phải' → 'bac phai', 'năm phải' → 'nam phai'. Câu hỏi mới có chữ 'tôi' ('Năm nay tiền bạc tôi thế nào?') từng bị model đọc thành 'lá số này của tôi' → phát lại câu gốc về con, chủ đề ra su-nghiep thay vì tai-chinh.</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/kiem.ts; lib/rag/focused/hieu-cau.ts; scripts/test-focused.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25923,7 +25960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31277,6 +31314,38 @@
         </is>
       </c>
       <c r="F167" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>LO_NGUON ở Focused chỉ bắt 'Nam phái/Bắc phái' viết có dấu; prompt nhãn hỏi lại F2 nói rõ câu hỏi mới về chính người dùng là khong-lien-quan.</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Eval Behavior Contract I3/I4: flow 7 (trọng yếu, F2 đang chờ + 'Năm nay tiền bạc tôi thế nào?') ra chủ đề su-nghiep 2/5 lần vì model nhỏ gán nhãn nguoi-hoi; sau sửa đo lại 10/10 đúng tai-chinh. Vết lỗi validator (in tạm) cho thấy LO_NGUON bắt nhầm 'tiền bạc phải' thành 'Bắc phái' → phải viết lại.</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 v2 I — cau thoi tiet la ngoai pham vi (outOfScope), het 502
Vi sao: eval I5 flow 28 "Thoi tiet mai the nao?" 502 o 2/5 lan. Model khong
dat outOfScope vi vi du trong prompt chi co nau an, bong da, sua may; claims
rong nen KHONG_CAN_CU, viet lai van loi, ra 502. Spec 7.1 flow 28 doi
outOfScope. Do lai 10/10, 502 0/20.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -25960,7 +25960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F168"/>
+  <dimension ref="A1:F169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31346,6 +31346,38 @@
         </is>
       </c>
       <c r="F168" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Prompt Focused: thêm 'thời tiết' vào ví dụ câu ngoài phạm vi (b) để model trả outOfScope một câu, không cần dẫn mã.</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Eval Behavior Contract I5 (05/10/2026, 155 lượt): flow 28 'Thời tiết mai thế nào?' 502 ở 2/5 lần. Vết validator: model không đặt outOfScope (ví dụ trong prompt chỉ có nấu ăn, bóng đá, sửa máy), claims rỗng → KHONG_CAN_CU → viết lại → vẫn lỗi → 502. Spec 7.1 flow 28 đòi outOfScope. Sau sửa đo lại 10/10, 502 0/20.</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: CEL-186 v2 J — backlog: ket qua eval I5, flow cho quyet, mo lai CEL-190
Vi sao: spec v2 muc J doi ghi cac cong truoc Production (CEL-190, EN body,
app Q7) vao backlog truoc Preview UAT. So do I5 la moc de so khi bat
Production; bon flow con truot can chu du an quyet vi sua phai them luat
ngoai spec hoac dung planner chung voi STANDARD.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15871,7 +15871,7 @@
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Vé A: đã lên production (merge 10e351f). Vé B (focused-2026.10.10): BƯỚC 1 sau UAT 04/10/2026 — luật chữ chỉ được định tuyến, không được tự kết thúc lượt. Lượt trả bằng mã chỉ còn: dữ kiện (trước sinh, tháng nhuận chưa tách), hỏi lại F2 (không tính lượt, chip một chạm trả lời câu gốc), một ngoại lệ tạm AGE-02 (không tính lượt). 'Khi nào' đi qua model ở mức năm. Bỏ PERSON-03. CI test-loi-chi-ma canh danh sách. Cờ Production vẫn TẮT.</t>
+          <t>Vé A: đã lên production (merge 10e351f). Vé B: Answer Contract v2 (spec D:\Celestia\CEL-186-answer-contract-v2-spec.md) xong A0→I trên nhánh viec/cel-186-focused-chat, CHỜ Preview UAT (D:\Celestia\CEL-186-preview-uat-v2.md). Cờ Production vẫn TẮT.</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
@@ -15906,17 +15906,17 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>BƯỚC 2 (nhánh mới, cổng trước khi bật cờ Production): biết quan hệ người hỏi ↔ lá số ở tầng dữ liệu; bộ đọc thời gian chung VI/EN ('When will…' đang ra khuôn B); mở rộng lapKeHoachDayDu thay vì viết bộ hiểu câu mới; hạ AGE-02 thành cách nói; thống nhất STANDARD 'tháng N' = dương; đo p95 độ trễ và chi phí. CHẶN TRƯỚC PRODUCTION (chủ dự án 04/10): thân bài model và chip ra tiếng Việt khi người dùng dùng giao diện EN (prompt Focused chưa ghim ngôn ngữ; eval đời thường ca 11). Nợ khác: câu tháng nhuận chưa tách vẫn tính lượt; model đôi khi gán nghĩa ngoài dữ kiện (Lộc Tồn = 'kết quả chính thức', Hữu Bật 'người từng được bạn giúp'); bấm chip F2 xong model vẫn mở 'Nếu đây là lá số của con bạn'; câu hai ý chỉ trả lời ý đầu.</t>
+          <t>Eval I5 (05/10/2026, 155 lượt, model ghim): 23/30 flow đạt; 502 3/155 (flow 28 đã sửa ở 738430e, đo lại 0/20); viết lại 14/155; p50/p95 11,5/19,8 s. Eval mù: Barnum 100%, 502 0/24. CHỜ CHỦ DỰ ÁN QUYẾT: flow 2 (trọng yếu, 'Tháng 10 tôi tìm việc được không?') khuôn A chỉ 2/5 vì planner luật không nhận 'tìm việc' → model phân loại ghi đè ý định — sửa cần luật mới hoặc đụng planner chung; flow 18 (EN 'this year') khuôn G vì planner không đọc 'this year' — đụng planner chung; flow 22/22.5 kỳ vọng tong-quan trong spec đã lỗi thời (planner giờ ra gia-dao); flow 29 eval đòi chip 'Sang năm' có mặt, thiết kế chỉ thêm từ tháng 9 âm. Nợ: chip A/B (tachHaiVe), flow 17 bịa 'hai lần', trẻ dưới 1 tuổi bị luận như đã đi học, chip đoán giới tính, KHONG_CAN_CU 502 ~1%. CỔNG TRƯỚC PRODUCTION: 502 ≤ 1%; lỗi chặn dữ kiện = 0; flow trọng yếu 100%; p95 chốt theo mốc đo; CEL-190; thân bài + chip EN; app di động (Q7).</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
         <is>
-          <t>04/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="O186" s="8" t="inlineStr">
         <is>
-          <t>Vé A: c5651d2, 2c8963c + merge 10e351f. Vé B: 6ea882f..85667e5, 8113e14, 22ac260, merge 3ba1912, ab22d61, 37a51fb, 7b5a195, 28f274c..d56a896 + bước 1 (nhánh viec/cel-186-focused-chat)</t>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
         </is>
       </c>
     </row>
@@ -16102,7 +16102,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Đã gộp vào CEL-186 (final hardening 04/10/2026)</t>
+          <t>Mở lại 05/10/2026 — cổng trước khi bật Focused ở Production</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -16137,12 +16137,17 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>Sửa ở lớp Focused (lib/rag/focused/ke-thua.ts lapKeHoachChinh + planner.lapKeHoachVoiChuDe), không đổi bảng planner → PHIEN_BAN_PLANNER giữ 2026.10.4, bộ vàng 100/100. STANDARD vẫn giữ hành vi cũ ở hai mẫu câu này (chủ ý, tránh xả đệm).</t>
+          <t>Phần Focused đã sửa ở lớp focused (ke-thua.ts). Còn: thống nhất đường STANDARD 'tháng N' = tháng dương theo spec Answer Contract v2 mục 3.1 (Focused đã đọc dương + cửa sổ âm, STANDARD vẫn đọc âm) — đổi STANDARD thì xả đệm, cần chủ dự án duyệt. Hai mẫu câu planner ('bản thân tôi … công việc', 'nhà cửa, gia đạo') vẫn sai ở STANDARD.</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>04/10/2026</t>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
         </is>
       </c>
     </row>
@@ -25960,7 +25965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F169"/>
+  <dimension ref="A1:F170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31378,6 +31383,38 @@
         </is>
       </c>
       <c r="F169" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>CEL-186, CEL-190</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Bước J của Answer Contract v2: ghi kết quả eval I5, các flow chờ quyết, nợ và cổng trước Production vào CEL-186; mở lại CEL-190 làm cổng (thống nhất STANDARD 'tháng N' = dương).</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Spec v2 mục J: ghi các cổng trước Production (CEL-190, EN body, app Q7) vào backlog trước khi chủ dự án nghiệm thu Preview. Số đo I5 là mốc để so khi bật Production; bốn flow trượt còn lại cần chủ dự án quyết vì sửa phải thêm luật ngoài spec hoặc đụng planner dùng chung với STANDARD.</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: CEL-186 log y_dinh ghi dung y dinh; mo CEL-191 (spec) + CEL-192 (discovery)
- nhat-ky.ts: retrieval_runs.y_dinh = keHoach.yDinh; chu de chuyen sang bo_loc.chuDe
- ca-nhan-hoa-celes.md: cap nhat cho doc cot y_dinh (dong cu = chu de)
- Backlog: CEL-191 spec xong cho gop CEL-186; CEL-192 DISCOVERY event-blind

Vi sao: dem retrieval_runs (chi doc) 05/10/2026 thay 95/95 run that ghi chu de
vao cot y_dinh, nen khong do duoc planner hieu y dinh tren du lieu that - so ma
CEL-191 can (flow 2 truot vi model ghi de y dinh). Khong co ma nao doc y_dinh;
bo_loc la jsonb san co, khong can migration.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O189"/>
+  <dimension ref="A1:O191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15906,7 +15906,8 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>Eval I5 (05/10/2026, 155 lượt, model ghim): 23/30 flow đạt; 502 3/155 (flow 28 đã sửa ở 738430e, đo lại 0/20); viết lại 14/155; p50/p95 11,5/19,8 s. Eval mù: Barnum 100%, 502 0/24. CHỜ CHỦ DỰ ÁN QUYẾT: flow 2 (trọng yếu, 'Tháng 10 tôi tìm việc được không?') khuôn A chỉ 2/5 vì planner luật không nhận 'tìm việc' → model phân loại ghi đè ý định — sửa cần luật mới hoặc đụng planner chung; flow 18 (EN 'this year') khuôn G vì planner không đọc 'this year' — đụng planner chung; flow 22/22.5 kỳ vọng tong-quan trong spec đã lỗi thời (planner giờ ra gia-dao); flow 29 eval đòi chip 'Sang năm' có mặt, thiết kế chỉ thêm từ tháng 9 âm. Nợ: chip A/B (tachHaiVe), flow 17 bịa 'hai lần', trẻ dưới 1 tuổi bị luận như đã đi học, chip đoán giới tính, KHONG_CAN_CU 502 ~1%. CỔNG TRƯỚC PRODUCTION: 502 ≤ 1%; lỗi chặn dữ kiện = 0; flow trọng yếu 100%; p95 chốt theo mốc đo; CEL-190; thân bài + chip EN; app di động (Q7).</t>
+          <t>Đã push 4fb4ce9, CI xanh (run 37307475844). CHƯA GỘP main, chờ chủ dự án duyệt. Thêm commit sửa log y_dinh (retrieval_runs) trên cùng nhánh. Việc nối tiếp: CEL-191 (spec xong, chờ gộp), CEL-192 (discovery).
+Eval I5 (05/10/2026, 155 lượt, model ghim): 23/30 flow đạt; 502 3/155 (flow 28 đã sửa ở 738430e, đo lại 0/20); viết lại 14/155; p50/p95 11,5/19,8 s. Eval mù: Barnum 100%, 502 0/24. CHỜ CHỦ DỰ ÁN QUYẾT: flow 2 (trọng yếu, 'Tháng 10 tôi tìm việc được không?') khuôn A chỉ 2/5 vì planner luật không nhận 'tìm việc' → model phân loại ghi đè ý định — sửa cần luật mới hoặc đụng planner chung; flow 18 (EN 'this year') khuôn G vì planner không đọc 'this year' — đụng planner chung; flow 22/22.5 kỳ vọng tong-quan trong spec đã lỗi thời (planner giờ ra gia-dao); flow 29 eval đòi chip 'Sang năm' có mặt, thiết kế chỉ thêm từ tháng 9 âm. Nợ: chip A/B (tachHaiVe), flow 17 bịa 'hai lần', trẻ dưới 1 tuổi bị luận như đã đi học, chip đoán giới tính, KHONG_CAN_CU 502 ~1%. CỔNG TRƯỚC PRODUCTION: 502 ≤ 1%; lỗi chặn dữ kiện = 0; flow trọng yếu 100%; p95 chốt theo mốc đo; CEL-190; thân bài + chip EN; app di động (Q7).</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -16146,6 +16147,163 @@
         </is>
       </c>
       <c r="O189" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>CEL-191</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Focused hiểu câu theo từng trường (chủ đề / ý định / thời gian ký hiệu) + validator ba tầng A/B/C</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Chat Focused đang gọi model phân loại khi luật không chắc chủ đề, rồi để model GHI ĐÈ cả ý định (planner.ts:955). Vì vậy flow 2 'Tháng 10 tôi tìm việc được không?' trượt 3/5 lần ở I5. Thời gian hoàn toàn do luật quyết, nên 'How will my career go this year?' ra khong-ro (flow 18). Đích: vẫn MỘT lời gọi, model trả thêm timeIntent ký hiệu (current-year, next-year, previous-year, current-month, next-month, near-future, long-term, none), code giải ra năm và tháng bằng logic có sẵn. Gộp theo từng trường: (1) chủ đề: chacChan thì giữ luật; (2) ý định: luật khác mo-ta thì giữ luật; (3) thời gian: parser giải được thì giữ parser, chỉ nhận timeIntent khi câu có dấu hiệu thời gian mà parser rỗng. Validator chia ba tầng: A FACT HARD (viết lại, rồi 502), B POLICY HARD (CHON_HO, phần trăm, CHAC_CHAN_GIA thu hẹp, LO_NGUON, an toàn), C QUALITY (chỉ ghi điểm, không viết lại, không 502). Spec đầy đủ: D:\Celestia\CEL-191-spec.md.</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>1. lapKeHoachFocused (luật)
+2. !chacChan &amp;&amp; !doiTuong &amp;&amp; !keThuaTu → lapKeHoachDayDu (model ghi đè chủ đề + ý định)
+3. Thời gian: doanPhamViThoiGian + boiCanhThoiGian (chỉ luật)
+4. kiem.ts: mọi MaLoiCung đều cứng → viết lại → 502</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Spec xong 05/10/2026 — CHỜ GỘP CEL-186 rồi mới rẽ nhánh và viết code</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Không sinh nội dung</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Mọi bậc</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>/hoi-dap (chỉ khi CELES_FOCUSED_CHAT=1)</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/tra-loi-focused.ts; lib/rag/focused/kiem.ts; lib/rag/focused/hop-dong.ts; (mới) lib/rag/focused/phan-loai-model.ts</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Sau cờ CELES_FOCUSED_CHAT=1 (Production tắt)</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>Toàn bộ code chờ main mới, vì các tệp cần sửa chỉ có trên nhánh CEL-186. Không được sửa lapKeHoachDayDu (STANDARD đang gọi). Không nâng PHIEN_BAN_PLANNER 2026.10.4. Dữ liệu thật 05/10/2026: 24/80 câu có thời gian, dưới 100 nên chưa tính được tỉ lệ bỏ lỡ; parser chỉ bỏ lỡ 2 câu (mức ngày, câu an toàn). Lỗi luật 'vợ/chồng tương lai' bị hiểu là giai-doan và 6 câu luật chắc nhưng sai chủ đề KHÔNG thuộc CEL-191 (để CEL-190 hoặc việc sau).</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>CEL-192</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>DISCOVERY — tầng tất định 'mù sự việc' (event-blind) ở chat Focused</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Câu hỏi chẩn đoán: event-blind ở tầng deterministic có làm câu trả lời cuối sai hoặc chung chung so với sự việc người dùng hỏi không? Đo 05/10/2026, không sinh câu mới. (1) Probe tất định 2 lá × 16 câu sự việc: trong cùng một chủ đề, gói dữ kiện và hướng nghiêng có băm GIỐNG HỆT 100%. Thăng chức, offer, nghỉ việc kinh doanh, bị sếp chèn ép đều ra thuan-nhe@Quan Lộc. Cưới, chia tay, ly hôn đều ra cùng một hướng @Phu Thê. (2) Rà 21 ca I5: ổn 12, chung chung 5 (F1, F3.2, F16, F21.3, F23: văn gọi tên sự việc nhưng bằng chứng y hệt câu chung), lệch 4 (F2, F8, F19, F27: khẳng định sự việc 'có' xảy ra suy từ độ êm của phần đời, không có căn cứ riêng cho sự việc), sai dữ kiện 0. Nguyên nhân gốc: tinhNghiengVe và chonBoiCanh chỉ nhận chủ đề, lớp hạn và cung, không nhận sự việc. Sự việc chỉ đến tầng viết qua câu gốc và loaiSuKien (3 giá trị). Cực tính của câu về chuyện xấu đã xử lý ở prompt.ts:136.</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>câu → chủ đề (6 giá trị) → chonBoiCanh/tinhNghiengVe (không có sự việc) → prompt viết nhận câu gốc + loaiSuKien</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>DISCOVERY (05/10/2026) — CHƯA implement, chờ chủ dự án quyết hướng</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Không sinh nội dung</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Mọi bậc</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>/hoi-dap (Focused)</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>lib/rag/nghieng-ve.ts; lib/rag/boi-canh-la-so.ts; lib/rag/focused/phan-loai.ts; lib/rag/focused/prompt.ts</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>Cần chủ dự án quyết một trong hai hướng: (a) chỉ chặn ở tầng viết (cấm khẳng định sự việc khi không có căn cứ riêng), rẻ, không đụng engine; (b) event schema + căn cứ theo sự việc. Hướng (b) cần luật Tử Vi CÓ NGUỒN cho từng sự việc, nên phải qua celes-domain. 4/21 ca lệch thuộc loại người đọc tin là 'dự đoán' nên là rủi ro uy tín. Không làm GraphRAG / MMR / reranker trong việc này.</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
         <is>
           <t>(nhánh viec/cel-186-focused-chat)</t>
         </is>
@@ -25965,7 +26123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F170"/>
+  <dimension ref="A1:F171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31415,6 +31573,38 @@
         </is>
       </c>
       <c r="F170" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>(nhánh viec/cel-186-focused-chat)</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>CEL-186, CEL-191, CEL-192</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>nhat-ky.ts: cột retrieval_runs.y_dinh ghi keHoach.yDinh (trước ghi nhầm chủ đề); chủ đề chuyển sang bo_loc.chuDe. Mở CEL-191 (spec, chờ gộp CEL-186) và CEL-192 (discovery event-blind).</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Đếm retrieval_runs chỉ đọc ngày 05/10/2026: cột y_dinh chứa chủ đề ở 95/95 run thật, nên không đo được planner hiểu ý định đúng hay sai trên dữ liệu thật, trong khi CEL-191 cần đúng số đó (flow 2 trượt vì model ghi đè ý định). Không có chỗ nào trong mã đọc y_dinh, nên sửa không ảnh hưởng gì; jsonb bo_loc có sẵn, không cần migration. 95 dòng cũ: đọc y_dinh như chủ đề. CEL-191 và CEL-192 được mở theo lệnh 'LÀM.' của chủ dự án ngày 05/10/2026.</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
PRIV-01 (CEL-193): trace Production khong giu van nguoi dung
retrieval_runs che_do='that' ghi '[an]' cho cau_hoi/truy_van; ai_requests bo cau_hoi,
chart_hash=null, ket_qua_kiem_duyet chi con ma/muc/so/phien ban. thu_nghiem (admin) giu
van. Dong chen dung bang ham thuan (dongLanTruyHoi/dongVetTraLoi) de test offline.
Migration noi NOT NULL + tep don du lieu cu: CHUA CHAY (MIGRATION_NOT_APPLIED); don
du lieu cu DANG DUNG vi dong cu khong phan biet Production/Preview/eval.

Vi sao: batch P0 §2 — chan doan da chuyen sang harness offline, trace chi can ID/ma/so;
van nguoi dung va sha256 ngay gio sinh khong muoi la rui ro rieng tu khong doi lay gi.
bamLaSo giu nguyen vi la khoa dem.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O191"/>
+  <dimension ref="A1:O192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16309,6 +16309,63 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>CEL-193</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>PRIV-01 — trace Production không giữ văn người dùng</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>retrieval_runs (che_do='that') ghi '[an]' thay cho câu hỏi và truy vấn; ai_requests không ghi cau_hoi, chart_hash = null, ket_qua_kiem_duyet chỉ còn {dat, phuSong, phienBan, loi[{ma, mucDo}]}. thu_nghiem (admin thử truy hồi) giữ văn.</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>ghiLanTruyHoi → dongLanTruyHoi (hàm thuần) → insert. ghiVetTraLoi → dongVetTraLoi → rutGonKiemDuyet → insert. Route hoi-dap / luan-giai không truyền cauHoi / chartHash (kiểu VetTraLoi đã bỏ hai trường).</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Đã làm (nhánh, chưa gộp)</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>lib/rag/nhat-ky.ts, app/api/hoi-dap/route.ts, app/api/luan-giai/route.ts, supabase/va-priv-01.sql, supabase/va-priv-01-don.sql, scripts/test-priv-01.ts</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Luôn bật khi deploy (không cờ) — chỉ bớt dữ liệu ghi, không đổi câu trả lời.</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>(1) Chạy va-priv-01.sql (nới NOT NULL) — MIGRATION_NOT_APPLIED. (2) Dọn dữ liệu cũ (va-priv-01-don.sql) ĐANG DỪNG: dòng cũ không phân biệt Production / Preview / eval — chủ dự án chọn A (làm trắng trước mốc) hoặc B (giữ). (3) Mất khả năng tra 'câu này sai' bằng văn trong DB — tra bằng request_id + mã.</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>(nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16326,7 +16383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G268"/>
+  <dimension ref="A1:G269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -26111,6 +26168,43 @@
         </is>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>CEL-193</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Trace</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Dòng trace dựng bằng hàm thuần</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>dongLanTruyHoi: cheDo mặc định 'that' → cau_hoi = truy_van = AN ('[an]'); 'thu_nghiem' giữ văn. bo_loc nhận boLocThem (chỉ mã/số). dongVetTraLoi: chart_hash null, cau_hoi null, ket_qua_kiem_duyet = rutGonKiemDuyet (bỏ moTa, tai).</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>bamLaSo KHÔNG đổi — nó là khoá đệm noi_dung_ai; chỉ ngừng ghi vào trace. Chuỗi canh thay null vì cột còn NOT NULL tới khi chạy va-priv-01.sql. Máy canh CI: scripts/test-priv-01.ts (gồm quét nguồn mọi lời gọi ghiVetTraLoi).</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>lib/rag/nhat-ky.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26123,7 +26217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31605,6 +31699,38 @@
         </is>
       </c>
       <c r="F171" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>(nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>CEL-193</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>PRIV-01: trace Production bỏ câu hỏi thô, truy vấn, văn validator, băm lá số; migration nới NOT NULL + tệp dọn dữ liệu cũ (đang dừng), chưa chạy.</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Batch P0 §2: trace phục vụ chẩn đoán chỉ cần ID / mã / số / phiên bản; văn người dùng (câu hỏi về hôn nhân, sức khoẻ…) và sha256 ngày giờ sinh không muối (dò ngược được bằng vét cạn ~100 nghìn tổ hợp) là rủi ro riêng tư không đổi lấy được gì. Chẩn đoán offline đã chuyển sang harness eval (D:\Celestia\eval), không cần văn Production.</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
SQL: CEL-194 QD-13 thu vien co phien ban (migration, CHUA CHAY)
muc_thu_vien + muc_thu_vien_phien_ban: noi dung bat bien (trigger), duyet theo
phien ban (da-duyet bat buoc approved_by + approved_at), RLS chi service role.
Luan v3 khong doi (van doc noi_dung_ai). MIGRATION_NOT_APPLIED.

Vi sao: nghiem ly cua chu du an chi duoc vao chat khi truy duoc phien ban nao
da duoc ai duyet luc nao; kho hien tai upsert ghi de nen mat ban cu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O192"/>
+  <dimension ref="A1:O193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16366,6 +16366,83 @@
         </is>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Nghiệm lý của tôi — thư viện có phiên bản (QĐ-13) + nghiệm lý chủ dự án vào chat Focused (T###)</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>QĐ-13: thư viện tri thức ra hai bảng có phiên bản (muc_thu_vien + muc_thu_vien_phien_ban, nội dung bất biến, duyệt theo phiên bản). Chủ dự án soạn / duyệt nghiệm lý (truongPhai 'celes') ở /admin; chỉ mục đã duyệt, đang dùng, có approved_by/approved_at mới được vào chat Focused dưới mã T###.</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Bước E: chỉ có migration va-qd13-thu-vien.sql (chưa chạy). Luận v3 vẫn đọc noi_dung_ai.</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Đang làm (nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Chủ dự án soạn tay</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Theo phiên bản</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Admin soạn; mọi bậc hưởng (sau cờ)</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>/admin/nghiem-ly; /hoi-dap (Focused)</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>supabase/va-qd13-thu-vien.sql</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Chạy va-qd13-thu-vien.sql + CELES_FOCUSED_CHAT=1 + CELES_OWNER_KNOWLEDGE_FOCUSED=1 (cả hai mặc định tắt)</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>MIGRATION_NOT_APPLIED. Luận v3 chưa chuyển sang bảng mới (chạm khoá đệm khoaGoi) — việc sau, cờ riêng. Trigger bất biến dùng drop trigger if exists + create (dựng lại được, không mất dữ liệu).</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>(nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16383,7 +16460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G272"/>
+  <dimension ref="A1:G273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -26316,6 +26393,43 @@
         </is>
       </c>
     </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Thư viện — lưu trữ</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Hai bảng có phiên bản (QĐ-13)</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>muc_thu_vien(id, truong_phai, trang_thai nhap|dang-dung|luu-tru, phien_ban_dang_dung). muc_thu_vien_phien_ban(muc_id, phien_ban, noi_dung jsonb = ảnh MucThuVien, duyet chua|da-duyet|bi-bac|tranh-chap, approved_by, approved_at). Check: da-duyet ⇒ có approved_by + approved_at. Trigger: noi_dung / phien_ban bất biến, chỉ cột duyệt được đổi. RLS bật, không policy.</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Duyệt theo PHIÊN BẢN: duyệt v2 không ngầm duyệt v3. Sửa = thêm phiên bản mới (kho.ts cũ upsert ghi đè làm mất bản cũ). Mã phải chịu được bảng chưa có.</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>supabase/va-qd13-thu-vien.sql</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26328,7 +26442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F173"/>
+  <dimension ref="A1:F174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31874,6 +31988,38 @@
         </is>
       </c>
       <c r="F173" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>(nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>QĐ-13: migration hai bảng thư viện có phiên bản (chưa chạy) + dòng DA-CHAY.</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Nghiệm lý của chủ dự án chỉ được vào chat khi biết chính xác phiên bản nào đã được ai duyệt lúc nào; kho hiện tại (noi_dung_ai, upsert) ghi đè nên không truy được. Trần batch ≤ 2 bảng mới (phản biện S5 trong D:\Celestia\RAG-kho-tri-thuc-phuong-an.md).</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-194 han luu nhat ky — cron xoa ai_requests/retrieval_runs >90 ngay, so khach >2 ngay
lib/rag/don-nhat-ky.ts: ham thuan lenhDonNhatKy + donNhatKy (admin client).
/api/cron/don-nhat-ky 03:30 moi ngay, Bearer CRON_SECRET nhu hai cron cu.
noi_dung_ai la bang dem dung chung nen lenh xoa tren no BAT BUOC loc
be_mat='gioi-han-khach'; test-han-luu-nhat-ky.ts chan thieu loc. Lan chay dau
xoa luon dong cu qua han, khong can SQL tay.

KHONG don usage_events (so han muc / thanh toan — chu du an quyet) va
ai_usage_logs (so tong hop theo ngay, khong noi duoc ve nguoi).

Vi sao: PRIV-01 Vong 8 — nhat ky noi duoc ve nguoi qua user_id/request_id thi
khong giu vo han; so dem khach chi can hom nay ma khoa chua bam IP.
Khong chong voi CEL-193 (khong luu chu) o nhanh viec/batch-p0-cel191.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O191"/>
+  <dimension ref="A1:O192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16309,6 +16309,43 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>H. Vận hành</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Hạn lưu nhật ký vận hành (PRIV-01): ai_requests / retrieval_runs 90 ngày, sổ đếm khách gioi-han-khach 2 ngày</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Chờ nghiệm thu (nhánh viec/priv-01, chưa gộp)</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>lib/rag/don-nhat-ky.ts, app/api/cron/don-nhat-ky/route.ts</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>Cron /api/cron/don-nhat-ky 03:30 mỗi ngày, dùng CRON_SECRET sẵn có. Lần chạy đầu xoá luôn dòng cũ quá hạn (không cần SQL tay). KHÔNG dọn usage_events (sổ hạn mức/thanh toán — chủ dự án quyết riêng) và ai_usage_logs (số tổng hợp). Phần không lưu chữ của PRIV-01 nằm ở CEL-193 (nhánh viec/batch-p0-cel191).</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -16326,7 +16363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G268"/>
+  <dimension ref="A1:G269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -26111,6 +26148,43 @@
         </is>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Hạn lưu nhật ký</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Cron dọn nhật ký quá hạn</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>lenhDonNhatKy(bayGio) (lib/rag/don-nhat-ky.ts, hàm thuần) trả 3 lệnh: ai_requests và retrieval_runs xoá tao_luc &lt; bayGio − 90 ngày (retrieval_results theo cascade); noi_dung_ai xoá tao_luc &lt; bayGio − 2 ngày VÀ be_mat = 'gioi-han-khach'. donNhatKy chạy từng lệnh bằng supabase admin, trả số dòng + lỗi; route trả 500 nếu có lỗi.</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>noi_dung_ai là bảng ĐỆM DÙNG CHUNG: mọi lệnh xoá trên nó BẮT BUỘC lọc be_mat, thiếu là xoá sạch đệm bài luận (test-han-luu-nhat-ky.ts chặn). be_mat là giá trị chính xác, tiền tố môi trường nằm ở khoa_ky.</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>lib/rag/don-nhat-ky.ts, app/api/cron/don-nhat-ky/route.ts, vercel.json, scripts/test-han-luu-nhat-ky.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26123,7 +26197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31605,6 +31679,38 @@
         </is>
       </c>
       <c r="F171" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>(nhánh viec/priv-01)</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>CEL-194, CEL-193</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Thêm cron dọn nhật ký vận hành: 90 ngày cho ai_requests/retrieval_runs, 2 ngày cho sổ đếm khách (lọc be_mat). Bài test offline vào CI.</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>PRIV-01 (Vòng 8, chủ dự án chốt 05/10/2026): nhật ký nối được về người qua user_id/request_id nên không giữ vô hạn; sổ đếm khách chỉ cần hôm nay mà khoá chứa băm IP. Production/Preview/local chung DB nên dọn theo tuổi, không theo môi trường.</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-194 F — Nghiem ly cua toi: admin soan/duyet theo phien ban + bo loc da duyet (sau co)
- lib/rag/thu-vien/nghiem-ly.ts: locNghiemLyDungDuoc (ham thuan), docNghiemLyDaDuyet
  (bang chua co -> []), chuanHoaNoiDung (danh sach dong), co CELES_OWNER_KNOWLEDGE_FOCUSED.
- /api/admin/nghiem-ly + /admin/nghiem-ly: tao v1, sua = phien ban moi, duyet/bac theo
  phien ban (approved_by do may chu ghi), chon dung chi ban da duyet, luu tru; audit log.
- scripts/test-nghiem-ly.ts vao CI.

Vi sao: matcher khopThuVien chi bo muc bi-bac; dua thang nghiem ly vao thi ban chua duyet
cung lot. Bo loc dung TRUOC matcher, matcher dung chung khong doi, luan v3 khong doi.
Chua noi vao chat (commit G).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16389,7 +16389,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Bước E: chỉ có migration va-qd13-thu-vien.sql (chưa chạy). Luận v3 vẫn đọc noi_dung_ai.</t>
+          <t>Bước E: migration va-qd13-thu-vien.sql (chưa chạy). Bước F: /admin/nghiem-ly soạn (tạo = v1, sửa = phiên bản mới), duyệt/bác theo phiên bản (approved_by = email admin do máy chủ ghi), chọn phiên bản dùng (chỉ bản đã duyệt), lưu trữ; mọi thao tác ghi admin_audit_log. Runtime: docNghiemLyDaDuyet → locNghiemLyDungDuoc (hàm thuần, chỗ duy nhất quyết 'đã duyệt'), đệm 60 s trong tiến trình, bảng chưa có → []. Luận v3 vẫn đọc noi_dung_ai.</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -16419,7 +16419,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>supabase/va-qd13-thu-vien.sql</t>
+          <t>supabase/va-qd13-thu-vien.sql; lib/rag/thu-vien/nghiem-ly.ts; app/api/admin/nghiem-ly/route.ts; app/admin/nghiem-ly/page.tsx; components/admin/TabQuanTri.tsx; scripts/test-nghiem-ly.ts</t>
         </is>
       </c>
       <c r="L193" t="inlineStr">
@@ -16460,7 +16460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G273"/>
+  <dimension ref="A1:G274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -26430,6 +26430,43 @@
         </is>
       </c>
     </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Thư viện — nghiệm lý</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Bộ lọc nghiệm lý dùng được + soạn ở admin</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>locNghiemLyDungDuoc(muc, phienBan): giữ khi truong_phai='celes' VÀ trang_thai='dang-dung' VÀ phiên bản = phien_ban_dang_dung tồn tại VÀ duyet='da-duyet' VÀ approved_by VÀ approved_at VÀ nội dung đủ hình (y, dieuKien.cung[], dieuKien.sao[], nhan, chuDe[]). Danh tính (id, truongPhai, duyet, schemaVersion, dotTrich=nghiem-ly@vN) lấy từ cột, jsonb không đè được. Thứ tự theo id. chuanHoaNoiDung: cung trong TEN_CUNG, quanHe trong QUAN_HE, chiều cat|hung|trung, mức manh|vua|nhe, chế độ add|modify|neutralize|override (khác add phải có dich), y ≤ 45 chữ; lạ là từ chối. Mã NL-XXX. Bác phiên bản đang dùng → mục về nhap.</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Lọc TRƯỚC khi đưa vào khopThuVien (matcher dùng chung không đổi; matcher chỉ bỏ bi-bac, sẽ nhận cả 'chua'). Cờ CELES_OWNER_KNOWLEDGE_FOCUSED chỉ '1' mới bật. Người duyệt không nhận từ body. Máy canh: scripts/test-nghiem-ly.ts (CI).</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/nghiem-ly.ts; app/api/admin/nghiem-ly/route.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26442,7 +26479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F174"/>
+  <dimension ref="A1:F175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32020,6 +32057,38 @@
         </is>
       </c>
       <c r="F174" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>(nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Admin 'Nghiệm lý của tôi' (soạn / duyệt theo phiên bản / chọn dùng / lưu trữ) + module đọc nghiệm lý đã duyệt sau cờ + test CI.</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Chủ dự án cần đưa nghiệm lý riêng vào chat Focused mà vẫn truy được phiên bản nào, ai duyệt, lúc nào. Matcher khopThuVien chỉ bỏ mục bi-bac — dùng thẳng thì nghiệm lý chưa duyệt cũng lọt; nên bộ lọc đứng trước matcher, một hàm thuần có test cho từng điều kiện.</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: CEL-194 G — nghiem ly T### trong Focused sau co CELES_OWNER_KNOWLEDGE_FOCUSED
- chonNghiemLy: nghiem ly da duyet -> khopThuVien (khong doi matcher) -> giai T<->T tat dinh theo id
  (override/neutralize go dich, vong A<->B id nho thang, modify giu ca hai) -> T001...
- Khoi prompt T dat sau khoi du kien; khi khac E### thi theo T###
- Validator: T phai trong goi, claim T thieu F -> T_THIEU_F; LO_MA bat T### va NL-
- Vet chi ghi id/phien ban/che do/so dem

Vi sao: tri thuc chu du an ky duyet duoc uu tien hon nguon tham chieu nhung khong la can cu tu than —
moi claim T phai kem du kien la so F###. Co tat = prompt, validator, vet y het truoc (test chung minh).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16419,7 +16419,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>supabase/va-qd13-thu-vien.sql; lib/rag/thu-vien/nghiem-ly.ts; app/api/admin/nghiem-ly/route.ts; app/admin/nghiem-ly/page.tsx; components/admin/TabQuanTri.tsx; scripts/test-nghiem-ly.ts</t>
+          <t>supabase/va-qd13-thu-vien.sql, lib/rag/thu-vien/nghiem-ly.ts, app/api/admin/nghiem-ly/route.ts, app/admin/nghiem-ly/page.tsx, lib/rag/focused/nghiem-ly-luot.ts, lib/rag/focused/kiem.ts, lib/rag/focused/prompt.ts, lib/rag/focused/tra-loi-focused.ts</t>
         </is>
       </c>
       <c r="L193" t="inlineStr">
@@ -16460,7 +16460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G274"/>
+  <dimension ref="A1:G275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -26467,6 +26467,43 @@
         </is>
       </c>
     </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Focused</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>T### trong lượt Focused (sau cờ CELES_OWNER_KNOWLEDGE_FOCUSED)</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Cờ =1: đọc nghiệm lý đã lọc (celes, đang dùng, phiên bản đã duyệt có approved_by/at, đệm 60 s) → khopThuVien trên cungLienQuan (matcher dùng chung không đổi) → giải T↔T tất định theo id: override/neutralize gỡ mục trong dich, mục đã bị gỡ không gỡ được ai (vòng A↔B → id nhỏ thắng), modify giữ cả hai và ghi 'điều chỉnh T00x' → gán T001… Khối prompt đặt ngay sau khối dữ kiện, nói 'khi khác E### thì theo T###'. Validator: T### phải nằm trong gói; claim dẫn T mà không có F → T_THIEU_F (tầng A); LO_MA bắt cả T### và NL-… trong câu văn. Vết chỉ ghi id/phiên bản/chế độ/số đếm.</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Cờ tắt = y hệt cũ: không đọc DB, không khối prompt (khoiNghiemLy([]) === ''), validator không biết T, vết không có trường. Nghiệm lý chỉ là CÁCH ĐỌC — căn cứ vẫn là F###, nên mọi claim T phải kèm F. Không sửa chunk, không đổi matcher dùng chung.</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/nghiem-ly-luot.ts, lib/rag/focused/kiem.ts, lib/rag/focused/prompt.ts, lib/rag/focused/tra-loi-focused.ts, lib/rag/focused/vet.ts, lib/rag/focused/hop-dong.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26479,7 +26516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F175"/>
+  <dimension ref="A1:F176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32089,6 +32126,38 @@
         </is>
       </c>
       <c r="F175" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>(nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>CEL-194</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Nghiệm lý của chủ dự án vào lượt Focused dưới mã T###, sau cờ CELES_OWNER_KNOWLEDGE_FOCUSED (mặc định tắt); validator thêm T_THIEU_F và LO_MA bắt T###/NL-.</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Batch 05/10/2026 §9–§11: tri thức chủ dự án ký duyệt phải được ưu tiên hơn nguồn tham chiếu nhưng không được thành căn cứ tự thân — mọi claim T phải kèm dữ kiện lá số F###. Giải T↔T tất định theo id để cùng lá số cùng câu hỏi luôn ra cùng gói (đo lại được). Đặt sau cờ để Production giữ nguyên hành vi cho tới khi chủ dự án tạo/duyệt nghiệm lý và chạy SQL.</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: dong batch P0 — AGENTS.md them 5 bai CI moi, nhat ky backlog
Vi sao: CI da chay test-priv-01, test-p0-chan-doan, test-nghiem-ly,
test-phan-hoi, test-do-phu-viet nhung danh sach lenh kiem trong AGENTS.md
chua co, may 2 doc AGENTS se khong biet de chay tay khi sua vung do.
Nhat ky ghi so do baseline <-> CEL-191 va viec con cho chu du an.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -26652,7 +26652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F177"/>
+  <dimension ref="A1:F178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32326,6 +32326,38 @@
         </is>
       </c>
       <c r="F177" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>(nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>CEL-191, CEL-193, CEL-194, CEL-195</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Đóng delivery batch P0 (A→I): baseline 50 ca, PRIV-01, harness P0 + judge + bộ 40 cặp chấm tay, CEL-191, QĐ-13 thư viện nghiệm lý, Owner Knowledge sau cờ CELES_OWNER_KNOWLEDGE_FOCUSED (mặc định tắt), grounding T###, phản hồi 👍👎, màn Cần duyệt, đo độ phủ tầng viết. AGENTS.md thêm 5 bài CI mới vào danh sách lệnh kiểm.</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Chủ dự án yêu cầu một batch liên tục (05/10/2026) để có thước đo trước khi sửa Writer và để chủ dự án đưa tri thức riêng vào Focused có kiểm soát. Số đo baseline ↔ CEL-191 trên 50 ca: PLANNING_ERROR 7→3, 502 1.7%→0%, viết lại 9.6%→5.8%, p95 19.7→20.9 s (+6%, trong cổng 20%), token vào giảm 3%; HOLDOUT điểm bắt buộc COVERED 81.4%→86.4% (nhãn judge, chưa người chấm). Chưa chạy SQL Production, chưa bật cờ, chưa gộp main: việc đó chờ chủ dự án.</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
CHORE: doi ID nghiem ly QD-13 tu CEL-194 sang CEL-196
Doi o ca ba sheet backlog, chu thich ma va ten buoc CI. Thong diep cac
commit da push (6eae482..184fc44) giu nguyen CEL-194; doc la CEL-196.

Vi sao: N1 da push viec/priv-01 (1e80349) dung CEL-194 cho "han luu nhat
ky" truoc nhanh nay, nen N1 giu CEL-194. Hai ID trung se lam backlog va
lich su chi vao hai viec khac nhau sau khi gop.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16369,7 +16369,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>CEL-194</t>
+          <t>CEL-196</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -26458,7 +26458,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>CEL-194</t>
+          <t>CEL-196</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -26495,7 +26495,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>CEL-194</t>
+          <t>CEL-196</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -26532,7 +26532,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>CEL-194</t>
+          <t>CEL-196</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -26652,7 +26652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F178"/>
+  <dimension ref="A1:F179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32216,7 +32216,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>CEL-194</t>
+          <t>CEL-196</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -32248,7 +32248,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>CEL-194</t>
+          <t>CEL-196</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -32280,7 +32280,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>CEL-194</t>
+          <t>CEL-196</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -32344,7 +32344,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>CEL-191, CEL-193, CEL-194, CEL-195</t>
+          <t>CEL-191, CEL-193, CEL-196, CEL-195</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -32358,6 +32358,38 @@
         </is>
       </c>
       <c r="F178" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>(nhánh viec/batch-p0-cel191)</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>CEL-196 (trước là CEL-194)</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Đổi ID của 'Nghiệm lý của tôi — QĐ-13 + T### trong Focused' từ CEL-194 sang CEL-196 ở cả ba sheet, chú thích mã, tên bước CI. Các commit đã push từ 6eae482 tới 184fc44 vẫn ghi CEL-194 trong thông điệp (không sửa lịch sử đã push): đọc CEL-194 trong các commit đó là CEL-196.</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Trùng ID giữa hai máy: N1 đã push viec/priv-01 (1e80349) dùng CEL-194 cho 'hạn lưu nhật ký' trước, nên N1 giữ CEL-194. Nhiều khả năng lúc máy này cấp ID, nhánh của N1 chưa lên remote nên backlog.py xem không thấy. Bài học: ID chỉ an toàn khi nhánh giữ ID đã push.</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: backlog — nhat ky don nhanh cu va script tam-*
Viec don dep, khong cap ID moi (chu du an quyet 06/10).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -26726,7 +26726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F180"/>
+  <dimension ref="A1:F181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32496,6 +32496,38 @@
         </is>
       </c>
       <c r="F180" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>b72e342, 0ff146a</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>CEL-186, CEL-193, CEL-194</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Dọn nhánh cũ: xoá viec/mobile-adaptive (đã có trên main) và viec/cel-186-quick (cứu docs/thiet-ke/CEL-186-quick-answer.md sang main trước; P4 vetAnToan bỏ, ghi vào tài liệu vé B). Chép docs/quyet-dinh/2026-10-01-kho-tri-thuc.md sang main, giữ nhánh kho-tri-thuc-uu-tien. Gỡ worktree + nhánh viec/tu-khoa-cham (chỉ còn hai dòng đo TAM-DO). Xoá 24 script tam-* một lần ở máy; .gitignore bỏ qua scripts/tam-*.</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Riêng tư trước: tam-dem-runs kéo câu hỏi thật từ DB và các tệp runs-* ẩn danh còn nằm ở scratchpad, đi ngược PRIV-01 nên xoá trước tiên. P4 ghi vết chữ người dùng nên bỏ, không port. Tài liệu được trỏ từ main không được chỉ sống trên nhánh sắp xoá. Nhánh/script treo làm nhiễu git status và dễ lỡ tay chạy script gọi model tốn tiền.</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
CHORE: toi uu token — tach danh sach kiem tra + app di dong khoi AGENTS.md, dat model agent; backlog CEL-197..206 (chat luong luan)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O195"/>
+  <dimension ref="A1:O205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16542,6 +16542,795 @@
         </is>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>CEL-197</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Bộ nghiệm thu chất lượng luận (đo được, dùng chung cho hỏi đáp và luận giải)</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Script chấm văn đã lưu (không gọi model, 0đ) theo 2 tầng. Tầng 1, mọi câu: T1 có kết luận, T2 không ba phải, T3 tên sao có trong dữ kiện, T4 khẳng định có nguồn (4 cái này đã có ở kiem-duyet.ts), T5 độ dài đúng nhịp, T6 không câu cụt, T7 có dấu ấn Celes, T8 không lộ từ cấm. Tầng 2, theo lớp hạn: T9 lưu niên/nguyệt hạn phải luận bằng sao LƯU (không chỉ sao tĩnh), T10 đại vận nêu quãng tuổi bằng số, T11 tra cứu không bịa thêm. Kèm ca tái hiện câu 'năm 2026 có đổi việc không' (log yDinh, lopHan, gói dữ kiện thật) và bảng số hiện trạng.</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>1. Lấy văn đã lưu theo từng ô (yDinh x lopHan x chuDe)
+2. Chấm T1..T11, ra tỉ lệ đạt theo ô
+3. Mọi lần sửa sau chạy lại cùng script: số lên là sửa đúng
+4. Ngưỡng nghiệm thu chốt cùng chủ dự án (T7 chờ CEL-201)</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>scripts/ (đo, không chạm hành vi)</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>scripts/do-chat-luong-luan.ts (dự kiến); lib/rag/kiem-duyet.ts</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>BƯỚC ĐẦU TIÊN của cả chương trình: không có số đo thì ba lỗi lặp (dài dòng, luận bằng sao tĩnh, dấu ấn mờ) sửa mãi không có điểm dừng. eval-chat-quyet-dinh.ts:184 chỉ regex CÓ TÊN sao nên bài kê 'Lưu Bạch Hổ' rồi luận bằng chính tinh vẫn đậu: T9 phải đo CÓ LUẬN. Production đang chạy đường STANDARD (Focused TẮT) nên đo đường STANDARD trước.</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>CEL-198</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Bộ golden sample luận giải (24 ca, chủ dự án viết)</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Chia theo 3 trục planner đang dùng. Tầng A lõi 12 ca: yDinh (co-khong, thoi-diem, quyet-dinh, giai-thich, mo-ta, tra-cuu) x lopHan (ban-menh, dai-van, luu-nien, nguyet-han). Tầng B chủ đề 6 ca: su-nghiep, tai-chinh, tinh-cam, gia-dao, suc-khoe, tong-quan (giữ yDinh=mo-ta, lopHan=luu-nien). Tầng C ca khó 6 ca: câu rất ngắn &lt;=60 ký tự, rất dài &gt;=220, hỏi về người khác, ngoài phạm vi, chạm an toàn, hỏi tiếp theo lượt trước. Mỗi ca gồm câu hỏi, câu trả lời mẫu, 1-2 dòng 'vì sao bản này đúng'.</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>1. Chủ dự án viết sample theo khung
+2. Dòng 'vì sao đúng' được chuyển thành tiêu chí chấm bổ sung cho CEL-197
+3. Sample làm mốc so sánh định tính, không so khớp văn bản từng chữ</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>THỦ CÔNG (chủ dự án)</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>docs/mau-vang/ (dự kiến)</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>CHỜ CHỦ DỰ ÁN. Ca A1 (năm 2026 có đổi việc không) đã có sample. Sample là văn xuôi tự do còn STANDARD trả JSON rồi ráp: không đặt mục tiêu giống văn bản 99%, đặt mục tiêu qua tiêu chí CEL-197. Liên quan CEL-114 (kho mẫu vàng A3).</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>CEL-199</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Lưu Tứ Hoá vào gói dữ kiện chat (gỡ chặn 'Nam phái làm chuẩn' cho luận hạn)</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Chủ dự án quyết 07/10/2026: sản phẩm không giới hạn ở Nam phái, luận hạn vẫn cần tứ hoá nên bỏ các logic chặn liên quan. Nối phần đã tính sẵn ở lib/rag/v3/du-kien.ts:676-690 (TU_HOA[can], can = mod(nam+6,10) theo năm xem) vào gói chat; sửa ghi chú mâu thuẫn ở boi-canh-la-so.ts:283 ('không có lưu Tứ Hóa'); focused/kiem.ts:289 cũng đang chặn.</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>1. Quyết định ghi ra tệp (đổi một trong ba quyết định bất biến của AGENTS.md)
+2. Nối lưu Tứ Hoá vào gói cho lopHan luu-nien/nguyet-han
+3. Thêm tên lưu Tứ Hoá vào tập tên cho phép của validator, nếu không T3 chặn nhầm
+4. Đổi khoá đệm để bài cũ không được phục vụ</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Theo năm</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Mọi người (qua các bề mặt AI)</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>lib/rag (chat + luận giải)</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>lib/rag/boi-canh-la-so.ts, lib/rag/v3/du-kien.ts, lib/rag/nghieng-ve.ts, lib/rag/kiem-duyet.ts, lib/rag/focused/kiem.ts</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Cờ môi trường mới, mặc định tắt</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>RỦI RO CAO NHẤT trong chương trình: vô hiệu bộ đệm hàng loạt (xem CEL-204), đổi nghĩa sao hiện cho người dùng. Test sẽ đỏ và phải sửa mốc: test-du-kien, test-boi-canh-dong-bang, test-phu-du-kien. test-ansao-chuan KHÔNG được đỏ (engine không đổi). Phải ghi quyết định ra tệp TRƯỚC khi đụng mã. Làm sau CEL-197 để đo được hiệu quả.</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Luận vận hạn bằng sao lưu thay vì sao tĩnh (thứ tự gói + đo T9)</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Lỗi lặp số 2: câu hỏi năm xem vẫn luận bằng chính tinh thủ mệnh. Bằng chứng đã kiểm: nghieng-ve.ts:386-403 ĐÃ bơm đủ 9 lưu tinh kèm nghĩa (có cả Lưu Bạch Hổ mà sample dùng) nên model THẤY mà không dùng. Ứng viên sửa: đưa lưu tinh lên trước sao tĩnh ở boi-canh-la-so.ts:82-83,146-149 khi lopHan là luu-nien/nguyet-han/dai-van; chỉ đổi thứ tự, có cờ tắt.</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>1. Đo T9 hiện trạng bằng CEL-197
+2. Thử đổi thứ tự gói sau cờ, mặc định tắt
+3. Đo lại; nếu T9 không lên thì giả thuyết 'model thiên vị đầu gói' sai, thử hướng khác
+4. Cắt sao tĩnh chỉ khi chủ dự án duyệt</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Mọi người (qua các bề mặt AI)</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>lib/rag (đường STANDARD)</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>lib/rag/boi-canh-la-so.ts, lib/rag/nghieng-ve.ts, lib/rag/prompt-co-can-cu.ts</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Cờ môi trường mới, mặc định tắt</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>Chưa có bằng chứng thứ tự là nguyên nhân: đây là giả thuyết, đo trước. Chẩn đoán ban đầu của phiên 06/10 (Focused cắt lưu tinh) đã bị phản biện đánh sập: đường Focused và STANDARD loại trừ nhau (tra-loi.ts:378) và production đang STANDARD. Test có thể đỏ: test-du-kien, test-boi-canh-dong-bang; bị ảnh hưởng nếu cắt: test-phu-du-kien.</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>CEL-201</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Dấu ấn Celes trong nhịp COMPACT (câu hỏi ngắn vẫn có cá tính)</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Hiện câu hỏi &lt;=60 ký tự thành nhịp COMPACT, prompt bảo bỏ dẫn dắt (boDanDat, hop-dong-tra-loi.ts:96) và dau-an.ts:284 tự tắt dấu ấn để khỏi chèn lại đúng câu dẫn vừa bỏ. Là thiết kế có chủ ý nhưng hệ quả: hỏi ngắn thì mất cá tính (lỗi lặp số 3). Đề xuất tách hai loại: câu dẫn (vẫn tắt khi COMPACT) và giọng trong thân bài (luôn bật), vì sample của chủ dự án ngắn mà vẫn rõ cá tính, tức cá tính nằm ở cách nói.</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>1. Chủ dự án quyết có/không cho dấu ấn ở COMPACT
+2. Nếu có: tách câu dẫn / giọng thân bài trong dau-an.ts
+3. Mỗi lần đổi một hằng, đo T7 bằng CEL-197</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Mọi người (qua các bề mặt AI)</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>lib/rag (chat)</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>lib/rag/hop-dong-tra-loi.ts, lib/rag/dau-an.ts</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>CHỜ CHỦ DỰ ÁN QUYẾT. Chạm hợp đồng trả lời nên là việc LỚN (phan-bien + danh-gia-tac-dong + bien-tap-vi). Test đỏ chắc chắn: test-hop-dong-tra-loi; test-dau-an và do-coverage-dau-an (UNREACHABLE=0) đỏ nếu đổi tập DA_CO_CHI_THI. Dấu ấn bắt buộc không được dài thêm câu trả lời ngắn.</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>CEL-202</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>D. Hỏi Celes (chat)</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Độ dài đúng trọng tâm và hết câu cụt (nhịp theo ý định)</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Lỗi lặp số 1: dài dòng, lạc trọng tâm, nhiều câu cụt, chưa tự nhiên. docs/bay/ai-rag.md:135 đã ghi gốc là số sao nêu ra (78% câu có tên sao, có câu kê 7 sao) chứ không phải prompt. Mục tiêu: đo T5 (độ dài theo nhịp) và T6 (câu cụt) rồi mới chỉnh NGAN=60 / DAI=220 hoặc luật nêu sao.</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>1. Đo T5/T6 hiện trạng bằng CEL-197
+2. Chỉnh MỖI LẦN MỘT hằng ở hop-dong-tra-loi.ts
+3. Đo lại</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Mọi người (qua các bề mặt AI)</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>lib/rag (chat)</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>lib/rag/hop-dong-tra-loi.ts, lib/rag/prompt-co-can-cu.ts, lib/rag/chuan-ngon-ngu.ts</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>Chạm luật độ dài, là luật luận cốt lõi nên là việc LỚN. Làm sau CEL-197. Không nới luật 'không phán' để câu ngắn đi.</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>CEL-203</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>A. Engine lá số</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Dọn nợ cùng gốc vòng Thái Tuế gốc lọt vào bài vận hạn (phần còn lại của CEL-085)</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Phiên viec/van-han-lop-goc (b98642c, chưa push) đã gỡ hai tổ hợp (Tang Tuế Điếu, Mã gặp Tuế Phá) khỏi cách cục theo hạn vì vòng Thái Tuế trên lá gốc an theo năm sinh, không phải năm xem. Còn lại cùng gốc: (1) sao lẻ của vòng Thái Tuế gốc vẫn vào gói kèm lời 'năm nay…' qua v3/du-kien.ts và nghieng-ve.ts (Tang Môn, Tuế Phá còn xếp về phía 'đỡ'); (2) v3/du-kien.ts:692 cho tên trần Thái Tuế, Thiên Mã nên bộ kiểm không phân biệt sao gốc với sao lưu; (3) dữ kiện tiểu hạn 2027 ghi 'Hóa Kỵ' của lá gốc, dễ bị hiểu là Kỵ của năm; (4) muốn dựng tổ hợp theo năm xem phải an thêm lưu Điếu Khách và lưu Tuế Phá.</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>1. Chờ push viec/van-han-lop-goc
+2. Sau đó sửa các mục (1)-(4), làm cùng đợt với CEL-199 để chỉ vô hiệu đệm một lần</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Mọi người (qua các bề mặt AI)</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>lib/tuvi/cach-cuc.ts, lib/rag</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/du-kien.ts, lib/rag/nghieng-ve.ts, lib/tuvi/luan-han.ts</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>Liên quan trực tiếp lỗi 'luận sao tĩnh': sao gốc bị gán nhãn theo năm làm sai căn cứ năm xem. Chạm lib/tuvi (vùng Chung) nên không mở song song với phiên sửa apps/celes-app. Cập nhật tiếp cột 'Việc còn lại' của CEL-085 khi làm.</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>CEL-204</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>D. Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Quyết định bộ đệm sau các sửa luận (CEL-085 + lưu Tứ Hoá)</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Bài vận hạn đã lưu đệm trước các sửa có thể còn hai tổ hợp Thái Tuế gốc và chưa có lưu Tứ Hoá. Hai lựa chọn: tăng đúng hằng phiên bản của bề mặt vận hạn (PHIEN_BAN_BANG_LINH_VUC, PHIEN_BAN_BAN_DOC_SAU) để bài viết lại khi có người mở (tốn tiền model), hoặc để tự hết hạn. Chưa kiểm PHIEN_BAN_BE_MAT_NGAN có nằm trong khoá đệm không; chưa đếm số bản ghi ảnh hưởng vì máy worktree không có .env.local.</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>1. Đếm bản ghi noi_dung_ai bị ảnh hưởng (máy có .env.local)
+2. Chủ dự án chọn cách
+3. Gom một lần cho cả CEL-085 và CEL-199</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>lib/store/boi-canh-doc.ts</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>lib/store/boi-canh-doc.ts, lib/moi-truong-dem.ts</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>CHỜ CHỦ DỰ ÁN QUYẾT. Preview và Production chung một Supabase: đổi khoá đệm đúng môi trường (CEL-189), đừng để Preview ghi đè cấu hình production.</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>CEL-205</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>D. Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Tối ưu token cho gói Claude Pro (model theo việc, tách AGENTS.md)</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>celes-domain đổi inherit sang sonnet, soat-tai-lieu đổi sonnet sang haiku; AGENTS.md giảm 21,8 KB còn 17,3 KB bằng cách chuyển 22 bài kiểm sang docs/quy-trinh/danh-sach-kiem-tra.md và mục App di động sang .claude/rules/app-di-dong.md (tự nạp khi sửa apps/celes-app). qa.md sửa hai chỗ trỏ. Khuyến nghị: opusplan cho việc lớn, Sonnet cho việc thường, Haiku cho việc cơ học; /clear giữa việc; ngắt connector không dùng.</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>1. Nhánh viec/toi-uu-token, chưa commit khi ghi dòng này
+2. AGENTS.md thuộc vùng Chung (AI-PHOI-HOP.md:58): báo máy kia trước khi gộp</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Chờ nghiệm thu</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>.claude/, AGENTS.md</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>AGENTS.md, .claude/agents/celes-domain.md, .claude/agents/soat-tai-lieu.md, .claude/agents/qa.md, docs/quy-trinh/danh-sach-kiem-tra.md, .claude/rules/app-di-dong.md</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>soat-tai-lieu quét AGENTS.md tìm đường dẫn cũ: lần chạy tới là lần kiểm thật của việc tách. Comment trong .github/workflows/kiem-tra.yml còn nói 'chạy tay theo AGENTS.md' (lệch nhẹ).</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>CEL-206</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>D. Hạ tầng AI</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Dọn việc hạ tầng tồn đọng sau các phiên 06/10</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Gom các việc nhỏ chờ chủ dự án xác nhận: (1) xoá scripts/tam-so-sanh-opus.ts ở thư mục chính; (2) 56 nhánh remote đã gộp hết vào main (danh sách đã dựng ở phiên 06/10, chưa xoá) — hai nhánh mobile-adaptive và cel-186-quick đã xoá, SHA 36ac30d và 33e5762 để khôi phục; (3) quyết định số phận viec/kho-tri-thuc-uu-tien (~170 dòng chưa gộp, xung đột QĐ-13); (4) đẩy ba nhánh đã 'push được' nhưng chưa push: viec/canh-id-cel (e1b0586), viec/don-nhanh-cu, viec/van-han-lop-goc (b98642c).</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Chủ dự án xác nhận từng mục, AI thực hiện. Push luôn do người.</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Chưa phát triển</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Nội bộ</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>git, scripts/</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>Không xoá nhánh trước khi chắc nó đã gộp hết (kiểm bằng git branch -r --merged origin/main). viec/kho-tri-thuc-uu-tien KHÔNG xoá cho tới khi chủ dự án quyết.</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -26726,7 +27515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F181"/>
+  <dimension ref="A1:F182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32528,6 +33317,38 @@
         </is>
       </c>
       <c r="F181" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>(nhánh viec/toi-uu-token)</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>CEL-197..CEL-206</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Mở chương trình 'chất lượng luận' (hỏi đáp + luận giải) làm ưu tiên hiện tại: CEL-197 bộ nghiệm thu, CEL-198 golden sample, CEL-199 lưu Tứ Hoá, CEL-200 luận bằng sao lưu, CEL-201 dấu ấn ở COMPACT, CEL-202 độ dài/câu cụt, CEL-203 nợ vòng Thái Tuế, CEL-204 quyết định đệm, CEL-205 tối ưu token gói Pro, CEL-206 gom việc dọn hạ tầng. Các tính năng khác (Hành trình lớp NGÀY CEL-071, Gate 2 CEL-078, PWA/RN CEL-083, app GĐ1 CEL-153..159, Streaming CEL-089, EN CEL-058/081) để sau.</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Chủ dự án 07/10/2026: ba lỗi lặp (dài dòng lạc trọng tâm, luận bằng sao tĩnh, dấu ấn Celes mờ) đã sửa nhiều lần mà vẫn lỗi, muốn tập trung luận giải trước. Phiên phân tích 06-07/10 cho thấy gốc là KHÔNG CÓ THƯỚC ĐO (eval-chat-quyet-dinh.ts:184 chỉ regex có tên sao) nên mỗi lần sửa không có điểm dừng; chẩn đoán đầu tiên (Focused cắt lưu tinh) bị phản biện đánh sập vì Focused và STANDARD loại trừ nhau (tra-loi.ts:378) và production đang STANDARD. Chủ dự án quyết: bỏ giới hạn Nam phái cho lưu Tứ Hoá; làm bộ tiêu chí tổng quát + riêng theo lớp hạn; tự viết golden sample theo 3 trục; ĐO TRƯỚC RỒI SỬA. Mục tiêu '~99% giống sample' không đặt vì sample là văn xuôi còn STANDARD trả JSON rồi ráp: nghiệm thu bằng tiêu chí CEL-197.</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
UI: ap phong cach Your Best Version — Be Vietnam Pro, the bo 22px, nut vien thuoc (CEL-057)
Giu nguyen bo cuc, bang mau, linh vat, dau thuong hieu, menh ban. Toan bo
lop "chat lieu" la mot khoi cuoi app/globals.css de go trong mot lan.
Font tu phuc vu 5 do dam (~16KB/file) bang scripts/cat-font.py.
Chu du an duyet 16/10/2026 sau khi xem ban chay thu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -5611,7 +5611,7 @@
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>Token màu, kiểu chữ, bo góc tập trung ở globals.css. Hồng #df37a7 chỉ cho nút hành động chính, mỗi khung nhìn đúng một cái. Vàng kim #D4AF37 chỉ cho dấu thương hiệu.</t>
+          <t>Token màu, kiểu chữ, bo góc tập trung ở globals.css. Hồng #df37a7 chỉ cho nút hành động chính, mỗi khung nhìn đúng một cái. Vàng kim #D4AF37 chỉ cho dấu thương hiệu. Từ 16/10/2026 mang 'chất liệu' của Your Best Version: chữ Be Vietnam Pro (tiêu đề đậm 800, khít chữ), thẻ bo 22px + bóng mềm, nút viên thuốc, ô nhập/ô chọn bo 12px, nền ngày ngả tím nhạt #f6f3f7, nhãn eyebrow chữ đậm nhỏ (không còn mono). Bảng màu, bố cục, linh vật, dấu thương hiệu giữ nguyên.</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="K58" s="8" t="inlineStr">
         <is>
-          <t>app/globals.css, components/ui/, components/ThemeToggle.tsx</t>
+          <t>app/globals.css (khối 'PHONG CÁCH YOUR BEST VERSION' cuối tệp), app/layout.tsx, app/fonts/be-vietnam-pro-*.woff2, scripts/cat-font.py, components/ui/, components/ThemeToggle.tsx</t>
         </is>
       </c>
       <c r="L58" s="8" t="inlineStr">
@@ -5656,17 +5656,17 @@
       </c>
       <c r="M58" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Be Vietnam Pro rộng chữ hơn Inter: tiêu đề hero trang chủ xuống 2 dòng ở màn rộng (trước vừa 1 dòng). Font không có glyph → và ✓ — hiện bằng font hệ thống. Chưa đo lại bằng trình duyệt thật ở 390px (scripts/test-man-hinh.mjs) và Lighthouse sau đổi font. inter-latin-vi.woff2 còn trong repo nhưng không còn nạp (giữ để quay lại nhanh).</t>
         </is>
       </c>
       <c r="N58" s="8" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="O58" s="8" t="inlineStr">
         <is>
-          <t>a04efc7</t>
+          <t>(nhánh viec/thu-phong-cach-ybv)</t>
         </is>
       </c>
     </row>
@@ -27515,7 +27515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F182"/>
+  <dimension ref="A1:F183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33349,6 +33349,38 @@
         </is>
       </c>
       <c r="F182" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>(nhánh viec/thu-phong-cach-ybv)</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>CEL-057</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Áp phong cách Your Best Version lên web: Be Vietnam Pro tự phục vụ 5 độ đậm (~16KB/file, latin + tiếng Việt, cắt bằng scripts/cat-font.py) thay Inter cho chữ chính và tiêu đề; bo thẻ 14→22px, ô nhập 3→12px, --radius-buttons 6→12px (ô chọn dạng khối), nút .btn-* thành viên thuốc + nhún khi bấm; bóng thẻ viền 1px + quầng mờ rộng; nền ngày #f6f3f7; eyebrow sans đậm; pill-tag/badge nền pha màu không viền; ô nhập focus bằng quầng hồng mờ. Inter Tight giữ cho chữ CELESTIA của dấu thương hiệu.</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Chủ dự án 16/10/2026 thấy component và font của yourbestversion.vercel.app/hom-nay dễ chịu hơn, yêu cầu thử trên Celes giữ nguyên bố cục, màu, linh vật; xem bản chạy thử (ảnh trước/sau ở D:\Celestia\thu-phong-cach-ybv) rồi duyệt lên production. Gom một khối CSS cuối globals.css để gỡ trong một lần nếu đổi ý. Font tự phục vụ chứ không dùng next/font/google vì bẫy unicode-range chồng nhau (docs/bay/giao-dien.md) làm mỗi trang nặng thêm ~200KB. --radius-buttons KHÔNG thành 999 vì đang dùng cho ô chọn dạng khối (dải năm, ô giờ sinh, menu) — thành viên thuốc là vỡ hình.</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: bang su that lop han lib/tuvi/tu-hoa-han.ts (CEL-199, CEL-200)
- lopHan(): tuoi am, tieu han, dai van, nguyet han, 9 sao luu, tu hoa goc,
  luu tu hoa theo can nam, tu hoa theo can cung dai van, diem trung
  (tieu han trung dai van, hoa chong co it nhat mot lop han).
- Chi tim vi tri, khong gan nghia; khong doc env (app doc qua @tuvi/*).
- v3 moTaNam doc luu tu hoa tu luuTuHoaTheoNam: dau ra giong tung ky tu
  tren 3.024 dong (6 cau x 168 la x 3 nam), khong dung khoa dem.
- scripts/test-tu-hoa-han.ts (CI): bang sach + dem tay ngu ho don,
  la doi chieu 24/08/2000 viet tay, quet 1.890 la x 3 nam, ca dot bien
  can nam sinh do 18.388 ca.
- HUONG-DAN.md: sua hai tham chieu chet (NET_VI, CHUAN_NGON_NGU_CELES).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16725,15 +16725,16 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>1. Quyết định ghi ra tệp (đổi một trong ba quyết định bất biến của AGENTS.md)
-2. Nối lưu Tứ Hoá vào gói cho lopHan luu-nien/nguyet-han
-3. Thêm tên lưu Tứ Hoá vào tập tên cho phép của validator, nếu không T3 chặn nhầm
-4. Đổi khoá đệm để bài cũ không được phục vụ</t>
+          <t>1. Quyết định ghi ra tệp — XONG 16/10/2026 (D:\Celestia\QUYET-DINH-van-han-dung-sao-luu.md, mục Lượt 4)
+2. Bảng sự thật lớp hạn lib/tuvi/tu-hoa-han.ts (lưu tứ hoá theo can năm, tứ hoá theo can cung đại vận, điểm trùng) — XONG, v3 moTaNam đọc từ đây, đầu ra không đổi
+3. Nối lưu Tứ Hoá + tứ hoá đại vận vào gói chat sau cờ CELES_LOP_HAN (commit 3)
+4. Thêm tên lưu Tứ Hoá vào tập tên cho phép của validator, kiểm cặp (hoá, sao)
+5. Đổi khoá đệm để bài cũ không được phục vụ (hỏi chủ dự án, đếm chỉ-đọc trước)</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Chưa phát triển</t>
+          <t>Đang phát triển</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -16758,12 +16759,12 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>lib/rag/boi-canh-la-so.ts, lib/rag/v3/du-kien.ts, lib/rag/nghieng-ve.ts, lib/rag/kiem-duyet.ts, lib/rag/focused/kiem.ts</t>
+          <t>lib/tuvi/tu-hoa-han.ts, lib/rag/boi-canh-la-so.ts, lib/rag/v3/du-kien.ts, lib/rag/nghieng-ve.ts, lib/rag/kiem-duyet.ts, lib/rag/focused/kiem.ts</t>
         </is>
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>Cờ môi trường mới, mặc định tắt</t>
+          <t>Cờ server CELES_LOP_HAN=1 (một cờ cho chat, v3, Hành trình; truyền tham số vào engine, engine không đọc env). Mặc định tắt</t>
         </is>
       </c>
       <c r="M198" t="inlineStr">
@@ -16773,12 +16774,12 @@
       </c>
       <c r="N198" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>(nhánh viec/toi-uu-token)</t>
+          <t>(nhánh viec/van-han-lop-han)</t>
         </is>
       </c>
     </row>
@@ -17349,7 +17350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G281"/>
+  <dimension ref="A1:G282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -22135,7 +22136,7 @@
       </c>
       <c r="E133" s="8" t="inlineStr">
         <is>
-          <t>dungDuKien(): cung chính + xung chiếu + tam hợp + phụ trợ (chỉ chuyên sâu) + sao toàn cục + cách cục trên cung đang đọc + lớp vận (đại vận, chuỗi đại vận, tiểu hạn, lưu tứ hóa tính từ TU_HOA theo can năm, lưu tinh, nguyệt hạn, điểm 12 cung). Mỗi cung kèm nghĩa sao lấy từ KHUON.vi.netPhuTinh / netSao.
+          <t>dungDuKien(): cung chính + xung chiếu + tam hợp + phụ trợ (chỉ chuyên sâu) + sao toàn cục + cách cục trên cung đang đọc + lớp vận (đại vận, chuỗi đại vận, tiểu hạn, lưu tứ hóa lấy từ luuTuHoaTheoNam (lib/tuvi/tu-hoa-han.ts, bảng gốc TU_HOA), lưu tinh, nguyệt hạn, điểm 12 cung). Mỗi cung kèm nghĩa sao lấy từ KHUON.vi.netPhuTinh / netSao.
 24/09/2026: hoiThoiDiem(q) — câu không hỏi thời điểm thì mô tả cung KHÔNG kèm "đại vận X–Y tuổi" và Tuần/Triệt không kèm mốc tuổi.</t>
         </is>
       </c>
@@ -22147,7 +22148,7 @@
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>lib/rag/v3/du-kien.ts</t>
+          <t>lib/rag/v3/du-kien.ts, lib/tuvi/tu-hoa-han.ts</t>
         </is>
       </c>
     </row>
@@ -27612,6 +27613,43 @@
       <c r="G281" t="inlineStr">
         <is>
           <t>lib/rag/bai-dai.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>CEL-199</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Bảng sự thật lớp hạn</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>lopHan(laSo, namXem, thangAm?) trong lib/tuvi/tu-hoa-han.ts trả: tuổi âm (namXem − năm âm sinh + 1), cung tiểu hạn, cung đại vận (null trước đại vận đầu), nguyệt hạn (khi có tháng), 9 sao lưu, tứ hoá gốc (can năm sinh), lưu tứ hoá (can năm xem = (nam+6) mod 10), tứ hoá đại vận (can CỦA CUNG đại vận, đổi tên can sang chỉ số bằng CAN.indexOf), và điểm trùng: tiểu hạn trùng đại vận; hoá chồng = một sao nhận hoá từ ≥2 lớp, có ít nhất một lớp hạn (gốc chồng gốc không tính). Chỉ tìm vị trí, không gắn nghĩa, không chấm thuận/cản trở. moTaNam của v3 (lib/rag/v3/du-kien.ts) đọc lưu tứ hoá từ luuTuHoaTheoNam thay vì tự tính.</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Engine không đọc process.env (app đọc qua @tuvi/*); cờ truyền bằng tham số ở lớp gọi. Tứ hoá đại vận lấy can cung đại vận, KHÔNG phải can năm sinh: scripts/test-tu-hoa-han.ts đếm tay ngũ hổ độn trên 1.890 lá × 3 năm và có ca đột biến (thay bằng can năm sinh thì đỏ 18.388 ca). Bảng tứ hoá trong test chép từ sách, ô dị bản (Mậu Khoa, Canh Khoa/Kỵ, Nhâm Khoa) để null; lá đối chiếu 24/08/2000 giờ Tuất nam vẫn chấm cứng ba ô đó theo TU_HOA — đổi dị bản thì sửa đáp án theo quyết định, không nới bài. Can năm xem theo năm dương: lớp gọi phải truyền đúng năm âm khi ngày xem nằm trước Tết.</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>lib/tuvi/tu-hoa-han.ts, lib/rag/v3/du-kien.ts, scripts/test-tu-hoa-han.ts</t>
         </is>
       </c>
     </row>
@@ -27627,7 +27665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F185"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33557,6 +33595,38 @@
         </is>
       </c>
       <c r="F185" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>CEL-199, CEL-200</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Thêm bảng sự thật lớp hạn lib/tuvi/tu-hoa-han.ts (lưu tứ hoá, tứ hoá đại vận, tiểu hạn/đại vận/nguyệt hạn, điểm trùng); v3 moTaNam dùng chung bảng này; bài CI test-tu-hoa-han.</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Chủ dự án chốt 16/10/2026: câu hỏi vận hạn kết luận bằng lớp hạn (sao lưu, lưu tứ hoá, tứ hoá đại vận, cung hạn), sao gốc chỉ là dẫn chứng. Trước đây lưu tứ hoá chỉ được tính tại chỗ trong v3 và không có tứ hoá đại vận. Tứ hoá đại vận chưa có sách nào trong kho ghi (phi tinh phái), nhưng chủ dự án yêu cầu vẫn làm để khi bổ sung nguồn thì chạy được ngay. Bước này không đổi đầu ra: chụp v3 trước/sau 3.024 dòng (6 câu × 168 lá × 3 năm) giống từng ký tự, nên không đụng khoá đệm.</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: khung luat to hop lop han lib/tuvi/luat-to-hop.ts, bang rong (CEL-200)
- LuatToHop: thanh phan (sao goc/luu/bat ky, hoa theo nguon), pham vi
  (dong cung / tam phuong), cung ap dung (cung hoi, tieu han, dai van,
  nguyet han), chieu, cau nghia, nguon sach:dong.
- khopLuatToHop: moi thanh phan co cho trong vung; cung luat cung cung
  tra mot lan; lop null bo qua.
- kiemBangLuat: chan thanh phan lap, luat toan sao goc, <2 sach.
- LUAT_TO_HOP rong cho chu du an duyet tung dong (2b).
- scripts/test-luat-to-hop.ts (CI): ham khop tren bang mau, la doi chieu
  2026; luat quet 0 lan = viet sai.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16806,15 +16806,19 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>1. Đo T9 hiện trạng bằng CEL-197
-2. Thử đổi thứ tự gói sau cờ, mặc định tắt
-3. Đo lại; nếu T9 không lên thì giả thuyết 'model thiên vị đầu gói' sai, thử hướng khác
-4. Cắt sao tĩnh chỉ khi chủ dự án duyệt</t>
+          <t>Hướng đã chốt 16/10/2026 (D:\Celestia\QUYET-DINH-van-han-dung-sao-luu.md): câu vận hạn lấy chiều từ lớp hạn, sao gốc chỉ dẫn chứng.
+1. Bảng sự thật lớp hạn lib/tuvi/tu-hoa-han.ts — XONG (CEL-199)
+2a. Khung luật tổ hợp lib/tuvi/luat-to-hop.ts (kiểu, hàm khớp, kiểm bảng), bảng RỖNG — XONG
+2b. Bảng luật hạt giống (≥2 sách mỗi dòng) — chờ chủ dự án duyệt từng dòng
+3. nghieng-ve cân theo lớp hạn sau cờ CELES_LOP_HAN (sao gốc ở cung hạn không cộng lẻ; thứ bậc luật tổ hợp &gt; tứ hoá theo hạn &gt; sao lưu)
+4. v3 thoiDiem xếp lớp hạn lên trước
+5. Hành trình (luan-han.ts) theo bảng sự thật; khoá đệm thêm |nhip:&lt;nhãn&gt;
+Đo phân bố hai phía offline trước khi bật cờ.</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Chưa phát triển</t>
+          <t>Đang phát triển</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -16844,7 +16848,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>Cờ môi trường mới, mặc định tắt</t>
+          <t>Cờ server CELES_LOP_HAN=1 (chung với CEL-199), mặc định tắt</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
@@ -16854,12 +16858,12 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>(nhánh viec/toi-uu-token)</t>
+          <t>(nhánh viec/van-han-lop-han)</t>
         </is>
       </c>
     </row>
@@ -17350,7 +17354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G282"/>
+  <dimension ref="A1:G283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27653,6 +27657,43 @@
         </is>
       </c>
     </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Luật tổ hợp: sao gốc chỉ có tiếng khi đi cùng lớp hạn</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>lib/tuvi/luat-to-hop.ts: mỗi LuatToHop gồm mã, các thành phần (sao gốc / sao lưu / bất kỳ; hoá theo nguồn goc | nam | dai-van | han | bat-ky), phạm vi (đồng cung, hoặc tam phương = cung xét + tam hợp + xung chiếu), các cung áp dụng (cung hỏi, tiểu hạn, đại vận, nguyệt hạn), chiều (thuận / cản trở / hai mặt), câu nghĩa đời thường, nguồn sách:dòng. khopLuatToHop(laSo, lopHan, cungHoi) trả luật khớp: mọi thành phần có ít nhất một chỗ trong vùng; cùng luật cùng cung chỉ trả một lần (tiểu hạn trùng đại vận); lớp null bị bỏ qua. LUAT_TO_HOP để rỗng đến khi chủ dự án duyệt (2b).</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>kiemBangLuat chặn: thiếu/trùng mã, &lt;2 thành phần, thành phần lặp (hai thành phần có thể là cùng một sao/hoá, vd Kình gốc + Kình bất kỳ — nếu không một sao khớp cả hai), không có sao lưu hay hoá theo hạn nào (luật toàn sao gốc trái hướng đã chốt), &lt;2 sách khác nhau có số dòng. scripts/test-luat-to-hop.ts quét lá số: luật nào khớp 0 lần là viết sai (bài học cách cục 'Kình Dương đồng cung Thiên Mã', 0/6.912 lá), tên sao phải có trên lá số thật. Engine không đọc env.</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>lib/tuvi/luat-to-hop.ts, scripts/test-luat-to-hop.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27665,7 +27706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33627,6 +33668,38 @@
         </is>
       </c>
       <c r="F186" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Thêm khung luật tổ hợp lớp hạn lib/tuvi/luat-to-hop.ts (kiểu dữ liệu, hàm khớp, hàm kiểm bảng) với bảng rỗng; bài CI test-luat-to-hop.</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Phản biện phương án (S2, 16/10/2026) chỉ ra sao gốc vẫn quay lại phép cân qua cung đại vận/tiểu hạn và cộng cát/hung lẻ. Hướng sửa đã chốt: sao gốc chỉ vào chiều khi một luật tổ hợp với sao lưu / hoá theo hạn khớp. Tách 2a (khung, không cần duyệt) khỏi 2b (nội dung luật, chủ dự án duyệt từng dòng) để commit 3 không phải chờ bảng. Không đổi đầu ra nào: chưa có nơi gọi.</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT(CEL-200): bang luat to hop lop han 2b — KINH_TRUNG_LUU, pham vi xung-chieu, trich nguyen van
- LUAT_TO_HOP: mot luat Kinh Duong goc + Luu Kinh (xung-chieu, tieu han + dai van, can tro).
  Chu du an duyet 17/10/2026. Luat Ho bo: Ham so 2567/2587 noi bo Tang Ho, khong phai Ho don,
  nen chi con nhom Ung dung. Kinh bo cung-hoi (sach chi noi Menh va han).
- xung-chieu: sao/hoa goc phai dong cung voi cung xet, sao luu o cung do hoac cung xung
  (chan khop vao cung trong).
- kiemBangLuat dem nguon theo NHOM_NGUON (>=2 nhom), nguon phai co trich nguyen van.
- test doi chieu trich voi tep sach khi may co kho (CI bo qua); them ca bat-ky Da goc o cung xung.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16808,8 +16808,8 @@
         <is>
           <t>Hướng đã chốt 16/10/2026 (D:\Celestia\QUYET-DINH-van-han-dung-sao-luu.md): câu vận hạn lấy chiều từ lớp hạn, sao gốc chỉ dẫn chứng.
 1. Bảng sự thật lớp hạn lib/tuvi/tu-hoa-han.ts — XONG (CEL-199)
-2a. Khung luật tổ hợp lib/tuvi/luat-to-hop.ts (kiểu, hàm khớp, kiểm bảng), bảng RỖNG — XONG
-2b. Bảng luật hạt giống (≥2 sách mỗi dòng) — chờ chủ dự án duyệt từng dòng
+2a. Khung luật tổ hợp lib/tuvi/luat-to-hop.ts (kiểu, hàm khớp, kiểm bảng) — XONG
+2b. Bảng luật hạt giống — XONG 17/10/2026: một luật KINH_TRUNG_LUU (phạm vi xung-chieu, ≥2 nhóm nguồn, mỗi nguồn kèm trích nguyên văn đối chiếu máy); bản duyệt D:\Celestia\BANG-LUAT-TO-HOP-2b.md
 3. nghieng-ve cân theo lớp hạn sau cờ CELES_LOP_HAN (sao gốc ở cung hạn không cộng lẻ; thứ bậc luật tổ hợp &gt; tứ hoá theo hạn &gt; sao lưu)
 4. v3 thoiDiem xếp lớp hạn lên trước
 5. Hành trình (luan-han.ts) theo bảng sự thật; khoá đệm thêm |nhip:&lt;nhãn&gt;
@@ -16858,7 +16858,7 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>17/10/2026</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -17354,7 +17354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G283"/>
+  <dimension ref="A1:G284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27680,15 +27680,52 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>lib/tuvi/luat-to-hop.ts: mỗi LuatToHop gồm mã, các thành phần (sao gốc / sao lưu / bất kỳ; hoá theo nguồn goc | nam | dai-van | han | bat-ky), phạm vi (đồng cung, hoặc tam phương = cung xét + tam hợp + xung chiếu), các cung áp dụng (cung hỏi, tiểu hạn, đại vận, nguyệt hạn), chiều (thuận / cản trở / hai mặt), câu nghĩa đời thường, nguồn sách:dòng. khopLuatToHop(laSo, lopHan, cungHoi) trả luật khớp: mọi thành phần có ít nhất một chỗ trong vùng; cùng luật cùng cung chỉ trả một lần (tiểu hạn trùng đại vận); lớp null bị bỏ qua. LUAT_TO_HOP để rỗng đến khi chủ dự án duyệt (2b).</t>
+          <t>lib/tuvi/luat-to-hop.ts: mỗi LuatToHop gồm mã, các thành phần (sao gốc / sao lưu / bất kỳ; hoá theo nguồn goc | nam | dai-van | han | bat-ky), phạm vi (dong-cung; xung-chieu = sao/hoá gốc đồng cung với cung xét, sao lưu/hoá theo hạn ở cung đó hoặc cung xung; tam-phuong = cung xét + tam hợp + xung chiếu), các cung áp dụng (cung hỏi, tiểu hạn, đại vận, nguyệt hạn), chiều (thuận / cản trở / hai mặt), câu nghĩa đời thường, nguồn sách:dòng kèm trích nguyên văn. khopLuatToHop(laSo, lopHan, cungHoi) trả luật khớp: mọi thành phần có ít nhất một chỗ trong vùng; cùng luật cùng cung chỉ trả một lần (tiểu hạn trùng đại vận); lớp null bị bỏ qua. Bảng hiện có: xem bước #2.</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>kiemBangLuat chặn: thiếu/trùng mã, &lt;2 thành phần, thành phần lặp (hai thành phần có thể là cùng một sao/hoá, vd Kình gốc + Kình bất kỳ — nếu không một sao khớp cả hai), không có sao lưu hay hoá theo hạn nào (luật toàn sao gốc trái hướng đã chốt), &lt;2 sách khác nhau có số dòng. scripts/test-luat-to-hop.ts quét lá số: luật nào khớp 0 lần là viết sai (bài học cách cục 'Kình Dương đồng cung Thiên Mã', 0/6.912 lá), tên sao phải có trên lá số thật. Engine không đọc env.</t>
+          <t>kiemBangLuat chặn: thiếu/trùng mã, &lt;2 thành phần, thành phần lặp (hai thành phần có thể là cùng một sao/hoá, vd Kình gốc + Kình bất kỳ — nếu không một sao khớp cả hai), không có sao lưu hay hoá theo hạn nào (luật toàn sao gốc trái hướng đã chốt), xung-chieu không có thành phần gốc làm neo, &lt;2 nhóm nguồn độc lập (NHOM_NGUON) có số dòng và trích. scripts/test-luat-to-hop.ts quét lá số: luật nào khớp 0 lần là viết sai (bài học cách cục 'Kình Dương đồng cung Thiên Mã', 0/6.912 lá), tên sao phải có trên lá số thật, tệp sách phải có trong NHOM_NGUON. Engine không đọc env.</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
+        <is>
+          <t>lib/tuvi/luat-to-hop.ts, scripts/test-luat-to-hop.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Bảng luật hạt giống + phạm vi xung-chieu + trích nguyên văn</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LUAT_TO_HOP có 1 luật: KINH_TRUNG_LUU (Kình Dương gốc + Lưu Kình; phạm vi xung-chieu; xét tiểu hạn, đại vận; chiều cản trở). xung-chieu: sao gốc / hoá gốc phải ĐỒNG CUNG với cung xét, sao lưu / hoá theo hạn ở cung đó hoặc cung xung (ViTriThanhPhan.laGoc). NguonSach có thêm trich (nguyên văn). kiemBangLuat chỉ đếm nguồn có số dòng và trích, theo NHOM_NGUON (Vũ Tài Lục + Chìa khoá + Ảo bí = phú Toàn Thư; Tổng hợp + Hàm số; hai tệp Ứng dụng; hai tệp Thiên Lương), cần ≥2 nhóm; luật xung-chieu phải có ít nhất một thành phần gốc làm neo. test-luat-to-hop mở tệp sách (KHO_SACH_TUVI, mặc định D:/Tài liệu tử vi/markdown; CI không có thì bỏ qua): dòng phải chứa trích, trích phải gọi tên mọi sao của luật, sao lưu kèm chữ «lưu».</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Không cho sao gốc nằm ở cung xung: năm Kình gốc và Lưu Kình cùng đóng cung A thì luật khớp cả ở cung đối diện A, một cung không có sao nào — đột biến bỏ ràng buộc làm số khớp gấp đôi. Hai tệp cùng tác giả / cùng chép một câu phú không phải hai nguồn. Một dòng nói BỘ sao rộng hơn (Tang Hổ + Lưu Tang Hổ) không phải nguồn cho luật sao đơn (Bạch Hổ + Lưu Hổ) — máy không bắt được chỗ này, phải đọc nguyên văn khi duyệt (17/10 đã trình nhầm luật Hổ đủ 2 nguồn). Song Lộc Tồn, song Kình, song Đà luôn cùng năm; Tang và Hổ gốc luôn đối nhau. Bài CI đòi mỗi luật khớp ≥1 lần khi quét và tệp sách phải có trong NHOM_NGUON.</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
         <is>
           <t>lib/tuvi/luat-to-hop.ts, scripts/test-luat-to-hop.ts</t>
         </is>
@@ -27706,7 +27743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F187"/>
+  <dimension ref="A1:F188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33700,6 +33737,38 @@
         </is>
       </c>
       <c r="F187" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Điền bảng luật tổ hợp hạt giống (KINH_TRUNG_LUU); thêm phạm vi xung-chieu (sao gốc neo ở cung xét); kiemBangLuat đếm theo nhóm nguồn NHOM_NGUON; mỗi nguồn kèm trích nguyên văn, test đối chiếu với tệp sách.</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt 17/10/2026 sau tham khảo nguồn ngoài và phan-bien (phản biện đánh sập: phạm vi đồng cung + xung cũ khớp vào cung trống; song Lộc Tồn 'hai mặt' là né quyết định; Tổng hợp 3707 chỉ nói họa tài sản nên luật Đà còn một nguồn). Lần duyệt đầu gồm Kình + Hổ; celes-domain đọc lại nguồn thì luật Hổ chỉ có một nhóm thật (Hàm số 2567/2587 nói bộ Tang Hổ, không phải Hổ đơn) — Claude đã trình sai. Chủ dự án yêu cầu soát lại kỹ và chặn lặp lại: bỏ Hổ, Kình bỏ 'cung hỏi' (sách chỉ nói Mệnh và hạn), câu nghĩa bỏ 'Năm này' (luật áp cả đại vận) và 'tranh chấp' (ngoài nguồn), thêm máy canh trích nguyên văn. Chưa đổi đầu ra: chưa có nơi gọi khopLuatToHop ngoài test (commit 3 nối, sau cờ CELES_LOP_HAN).</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT(CEL-200): chat STANDARD can cau van han theo lop han sau co CELES_LOP_HAN (3a)
- nghieng-ve: tinhTheoLopHan - chieu chi tu luat to hop > luu hoa = sao luu > tu hoa dai van;
  sao goc o cung hoi thanh muc nen (khong cong), sao goc o cung han khong cong le;
  tam phuong x0.5; luon hai mat; khoiTheoLopHan rieng
- boi-canh-la-so: noi cuoi du kien luu-tu-hoa, tu-hoa-dai-van (F### cu khong dich)
- tra-loi: co lopHanBat, chi duong STANDARD; vet ghi PHIEN_BAN_NGHIENG_LOP_HAN khi bat
- test-lop-han-chat vao CI: co tat = duong cu tung byte, dot bien, bang phan bo
- co tat (mac dinh) = duong cu nguyen ven

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16810,7 +16810,8 @@
 1. Bảng sự thật lớp hạn lib/tuvi/tu-hoa-han.ts — XONG (CEL-199)
 2a. Khung luật tổ hợp lib/tuvi/luat-to-hop.ts (kiểu, hàm khớp, kiểm bảng) — XONG
 2b. Bảng luật hạt giống — XONG 17/10/2026: một luật KINH_TRUNG_LUU (phạm vi xung-chieu, ≥2 nhóm nguồn, mỗi nguồn kèm trích nguyên văn đối chiếu máy); bản duyệt D:\Celestia\BANG-LUAT-TO-HOP-2b.md
-3. nghieng-ve cân theo lớp hạn sau cờ CELES_LOP_HAN (sao gốc ở cung hạn không cộng lẻ; thứ bậc luật tổ hợp &gt; tứ hoá theo hạn &gt; sao lưu)
+3a. Chat STANDARD cân theo lớp hạn sau cờ CELES_LOP_HAN — XONG 17/10/2026 (nghieng-ve tinhTheoLopHan + dữ kiện luu-tu-hoa / tu-hoa-dai-van)
+3b. Focused nhận cờ: bỏ cấm lưu Hóa, validator cặp (hoá, sao), Q-nguon trong prompt
 4. v3 thoiDiem xếp lớp hạn lên trước
 5. Hành trình (luan-han.ts) theo bảng sự thật; khoá đệm thêm |nhip:&lt;nhãn&gt;
 Đo phân bố hai phía offline trước khi bật cờ.</t>
@@ -16843,7 +16844,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>lib/rag/boi-canh-la-so.ts, lib/rag/nghieng-ve.ts, lib/rag/prompt-co-can-cu.ts</t>
+          <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, lib/tuvi/tu-hoa-han.ts, lib/tuvi/luat-to-hop.ts</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -16853,7 +16854,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Chưa có bằng chứng thứ tự là nguyên nhân: đây là giả thuyết, đo trước. Chẩn đoán ban đầu của phiên 06/10 (Focused cắt lưu tinh) đã bị phản biện đánh sập: đường Focused và STANDARD loại trừ nhau (tra-loi.ts:378) và production đang STANDARD. Test có thể đỏ: test-du-kien, test-boi-canh-dong-bang; bị ảnh hưởng nếu cắt: test-phu-du-kien.</t>
+          <t>Phân bố đo offline (60 lá × 2024–2030 × 4 chủ đề): cũ thuận rõ 42.8% / cản rõ 1.7% / đủ hai mặt 93.6%; lớp hạn thuận rõ 23.4% / cản rõ 24.9% / đủ hai mặt 81.6%. Ngưỡng chấp nhận (L3) chờ chủ dự án duyệt; cần tách theo chủ đề (sức khỏe, tình cảm) trước khi bật. Rủi ro celes-domain nêu: hệ số tam phương 0.5 và ngưỡng huongTu chưa có cơ sở sách; nhãn 'rõ' tính theo tỉ lệ nên một mục chiếu tam phương đứng một mình vẫn ra 'cản rõ'; Lưu Kỵ ở Mệnh lên phía cản của mọi chủ đề chiếu tới Mệnh. Focused chưa nhận cờ (3b). Kiểm cặp (hoá, sao) ở STANDARD chỉ dựa vào prompt.</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -17354,7 +17355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G284"/>
+  <dimension ref="A1:G285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27731,6 +27732,43 @@
         </is>
       </c>
     </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Chat STANDARD cân câu vận hạn theo lớp hạn (sau cờ CELES_LOP_HAN)</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>tra-loi.ts đọc cờ (lopHanBat) rồi truyền lopHanMoi xuống chonBoiCanh và tinhNghiengVe; engine không đọc env. tinhNghiengVe: lopHanMoi và lớp có gì ngoài ban-menh thì sang tinhTheoLopHan. Dữ kiện lấy từ lopHan() (tu-hoa-han.ts). Trọng số TRONG_HAN: luật tổ hợp 4.5 &gt; lưu hoá 3 = sao lưu 3 &gt; tứ hoá đại vận 2. Hệ số vị trí: đúng cung hỏi ×1, tam hợp / xung chiếu ×0.5, khác ×0. Luật tổ hợp: bỏ tiểu hạn khi câu hỏi cả chặng; sao/hoá không gốc trong luật vào daDung nên không cộng lẻ lần nữa; luật hai-mat đẩy cả hai phía. Lưu hoá bỏ khi câu hỏi cả chặng; tứ hoá đại vận chỉ khi lớp có dai-van. Kỵ = cản; Lộc, Quyền, Khoa = thuận. Lưu Thái Tuế không đứng phía nào. Sao gốc ở cung hỏi → mục nen (top 3), KHÔNG cộng. Top 6 mốc, đổi mốc để đủ hai phía nếu có. nhanManh khi tiểu hạn trùng đại vận và chạm cung hỏi. khoiTheoLopHan: hai danh sách thuận / cản của lớp hạn (phía rỗng ghi MỎNG), mục nền 'chỉ dẫn chứng', luôn nói hai mặt, nêu ít nhất một cách cục làm dẫn chứng. chonBoiCanh nối cuối hai loại dữ kiện mới: luu-tu-hoa (lớp luu-nien), tu-hoa-dai-van (lớp dai-han). Vết ghi phienBan.nghieng = PHIEN_BAN_NGHIENG_LOP_HAN (2026.10.1) khi cờ bật.</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Cờ tắt = đường cũ đúng từng byte (test-lop-han-chat mục A). Mục mới chỉ nối cuối: chèn giữa làm dịch mã F### mà bài viết đã dẫn. Sao gốc ở cung đại vận / tiểu hạn không được cộng cát/hung lẻ — chỉ vào chiều qua luật tổ hợp (phản biện S2: bản đầu cho sao gốc quay lại qua cung hạn). Tên luật tổ hợp đặt cho tứ hoá là 'Hóa Kỵ (Liêm Trinh)', không tiền tố lưu: khoá daDung phải theo đúng dạng đó, nếu không lưu hoá bị cộng hai lần khi bảng có luật tứ hoá (celes-domain bắt 17/10). Bài đột biến 'bỏ phụ tinh gốc' phải giữ các sao nhận lưu hoá, không thì bài đỏ oan. PHIEN_BAN_NGHIENG không nằm trong khoá đệm nào (chỉ vết) nên đổi không làm mất đệm. Focused chưa nhận cờ: validator Focused còn cấm 'lưu Hóa'.</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, scripts/test-lop-han-chat.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27743,7 +27781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F188"/>
+  <dimension ref="A1:F189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33769,6 +33807,38 @@
         </is>
       </c>
       <c r="F188" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Commit 3a: đường chat STANDARD cân câu vận hạn theo lớp hạn sau cờ CELES_LOP_HAN (tinhTheoLopHan, khoiTheoLopHan, dữ kiện lưu tứ hoá + tứ hoá đại vận); test-lop-han-chat vào CI.</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Thực hiện quyết định 16/10/2026: chiều câu vận hạn phải đến từ thứ đổi theo năm/đại vận, không từ sao gốc năm nào cũng như nhau. Đường cũ lệch hẳn về 'thuận' (60 lá × 2024–2030 × 4 chủ đề: thuận rõ 42.8%, cản rõ 1.7%) vì sao gốc ở cung hỏi và cung hạn được cộng vào chiều. Đường lớp hạn: thuận rõ 23.4%, cản rõ 24.9%, đủ hai mặt 81.6% (phía thiếu nói 'mỏng', không bịa). celes-domain + qa + bien-tap-vi soát: qa 6/6 (4 đột biến đều có bài đỏ); sửa theo soát: khoá daDung cho tứ hoá, nghĩa tứ hoá trung tính theo chủ đề và ghép mốc năm / đại vận, cách cục bắt buộc nêu một cái (khớp 0b) nhưng chỉ làm dẫn chứng, bỏ câu khẳng định sự việc. Ngưỡng phân bố và hệ số tam phương 0.5 chưa có sách đỡ — chờ chủ dự án duyệt trước khi bật cờ. Focused để 3b.</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT(CEL-200): noi Focused va validator lop han sau co (3b)
Vi sao: cho luu Hoa dung quan he va thoi diem, giu ngu canh qua luot dung che do, chan chu noi bo sau vong sua; duong tat giu mau base. Khong doi engine, DB hoac dem.

Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16811,7 +16811,7 @@
 2a. Khung luật tổ hợp lib/tuvi/luat-to-hop.ts (kiểu, hàm khớp, kiểm bảng) — XONG
 2b. Bảng luật hạt giống — XONG 17/10/2026: một luật KINH_TRUNG_LUU (phạm vi xung-chieu, ≥2 nhóm nguồn, mỗi nguồn kèm trích nguyên văn đối chiếu máy); bản duyệt D:\Celestia\BANG-LUAT-TO-HOP-2b.md
 3a. Chat STANDARD cân theo lớp hạn sau cờ CELES_LOP_HAN — XONG 17/10/2026 (nghieng-ve tinhTheoLopHan + dữ kiện luu-tu-hoa / tu-hoa-dai-van)
-3b. Focused nhận cờ: bỏ cấm lưu Hóa, validator cặp (hoá, sao), Q-nguon trong prompt
+3b. XONG phần mã máy 2: Focused nhận cờ, giữ meta đúng chế độ, dữ kiện hoá gốc/năm/đại vận theo cửa sổ, validator hoá–sao–cung–lớp–năm–F/W, quét chữ cấm + Q-nguon/Q2; đường tắt so 25 snapshot từ base25ad334; không ép hai mặt. Chưa bật cờ, còn phụ thuộc 3a' máy 1.
 4. v3 thoiDiem xếp lớp hạn lên trước
 5. Hành trình (luan-han.ts) theo bảng sự thật; khoá đệm thêm |nhip:&lt;nhãn&gt;
 Đo phân bố hai phía offline trước khi bật cờ.</t>
@@ -16839,7 +16839,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>lib/rag (đường STANDARD)</t>
+          <t>lib/rag (STANDARD + Focused; v3 chờ Commit 4 phần mã)</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -16854,7 +16854,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Phân bố đo offline (60 lá × 2024–2030 × 4 chủ đề): cũ thuận rõ 42.8% / cản rõ 1.7% / đủ hai mặt 93.6%; lớp hạn thuận rõ 23.4% / cản rõ 24.9% / đủ hai mặt 81.6%. Ngưỡng chấp nhận (L3) chờ chủ dự án duyệt; cần tách theo chủ đề (sức khỏe, tình cảm) trước khi bật. Rủi ro celes-domain nêu: hệ số tam phương 0.5 và ngưỡng huongTu chưa có cơ sở sách; nhãn 'rõ' tính theo tỉ lệ nên một mục chiếu tam phương đứng một mình vẫn ra 'cản rõ'; Lưu Kỵ ở Mệnh lên phía cản của mọi chủ đề chiếu tới Mệnh. Focused chưa nhận cờ (3b). Kiểm cặp (hoá, sao) ở STANDARD chỉ dựa vào prompt.</t>
+          <t>Máy 2: Commit 4 phần mã v3 tiếp sau 3b. Máy 1: phép cân 3a' theo C1/C3, kho và Hành trình. Không bật cờ hoặc tăng đệm trong nhánh máy 2. Chi phí/tỉ lệ thử lại/502 chưa đo bằng model thật; chủ dự án chạy eval-chat-quyet-dinh sau tích hợp.</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -16864,7 +16864,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>(nhánh viec/van-han-lop-han)</t>
+          <t>(nhánh viec/van-han-3b, commit 3b)</t>
         </is>
       </c>
     </row>
@@ -17355,7 +17355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G285"/>
+  <dimension ref="A1:G286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27760,12 +27760,49 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Cờ tắt = đường cũ đúng từng byte (test-lop-han-chat mục A). Mục mới chỉ nối cuối: chèn giữa làm dịch mã F### mà bài viết đã dẫn. Sao gốc ở cung đại vận / tiểu hạn không được cộng cát/hung lẻ — chỉ vào chiều qua luật tổ hợp (phản biện S2: bản đầu cho sao gốc quay lại qua cung hạn). Tên luật tổ hợp đặt cho tứ hoá là 'Hóa Kỵ (Liêm Trinh)', không tiền tố lưu: khoá daDung phải theo đúng dạng đó, nếu không lưu hoá bị cộng hai lần khi bảng có luật tứ hoá (celes-domain bắt 17/10). Bài đột biến 'bỏ phụ tinh gốc' phải giữ các sao nhận lưu hoá, không thì bài đỏ oan. PHIEN_BAN_NGHIENG không nằm trong khoá đệm nào (chỉ vết) nên đổi không làm mất đệm. Focused chưa nhận cờ: validator Focused còn cấm 'lưu Hóa'.</t>
+          <t>Cờ tắt = đường cũ đúng từng byte (test-lop-han-chat mục A). Mục mới chỉ nối cuối: chèn giữa làm dịch mã F### mà bài viết đã dẫn. Sao gốc ở cung đại vận / tiểu hạn không được cộng cát/hung lẻ — chỉ vào chiều qua luật tổ hợp (phản biện S2: bản đầu cho sao gốc quay lại qua cung hạn). Tên luật tổ hợp đặt cho tứ hoá là 'Hóa Kỵ (Liêm Trinh)', không tiền tố lưu: khoá daDung phải theo đúng dạng đó, nếu không lưu hoá bị cộng hai lần khi bảng có luật tứ hoá (celes-domain bắt 17/10). Bài đột biến 'bỏ phụ tinh gốc' phải giữ các sao nhận lưu hoá, không thì bài đỏ oan. PHIEN_BAN_NGHIENG không nằm trong khoá đệm nào (chỉ vết) nên đổi không làm mất đệm. Mốc lịch sử commit 3a: Focused khi đó chưa nhận cờ. Đã được nối ở bước 3b máy 2: cho lưu Hóa khi đúng quan hệ hoá–sao–cung–lớp–thời điểm/F/W, giữ cờ tắt như cũ. Phần phép cân 3a chờ máy 1 cập nhật theo C1/C3 đã duyệt.</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
           <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, scripts/test-lop-han-chat.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Lớp hạn — máy 2</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Focused và validator lớp hạn sau CELES_LOP_HAN</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Cờ từ server truyền tới dữ kiện/nghiêng từng cửa sổ và dựng lại meta. Chỉ mode bật thêm marker ký; mode khác bỏ meta. Bảng hoá gốc/năm/đại vận hiện trong F và map W; quan hệ đúng hoa-sao-cung-lớp-năm mới được nhắc, không lấy d.sao làm quyền. Prompt đặt cung gốc trong vận theo API máy 1, không tự cân. Quét tiếng lóng và ẩn dụ trên answer/claim và lời cuối STANDARD; sửa trong vòng hiện có, còn lỗi trả thất bại sẵn. Q-nguon nói mức chắc chắn, Q2 theo câu đã duyệt.</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Off→off giữ từng byte so 25 snapshot từ nguồn base25ad334. Không ép hai mặt. Không sửa nghieng-ve/lib/tuvi/DB/THE_HE_DEM/PHIEN_BAN_NGON_NGU. Validator version mới chỉ nhánh bật. Qua Tết không hợp bảng để gán sai cửa sổ.</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>lib/rag/kiem-lop-han.ts; lib/rag/boi-canh-la-so.ts; lib/rag/focused/; lib/rag/tra-loi.ts; lib/rag/sua-chua.ts; scripts/test-lop-han-3b.ts</t>
         </is>
       </c>
     </row>
@@ -27781,7 +27818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F189"/>
+  <dimension ref="A1:F190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33841,6 +33878,38 @@
       <c r="F189" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-3b, commit 3b)</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>3b: nối cờ Focused, dữ kiện hoá theo cửa sổ, meta ký chế độ, validator quan hệ và lời cuối STANDARD/Focused; Q-nguon và Q2. Thêm snapshot base độc lập và thử sai quan hệ/cửa sổ/vòng viết lại.</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt phương án máy 2 ngày 17/10/2026. Cấm lưu Hóa tuyệt đối trái bảng sự thật đã có; chỉ kiểm tên riêng lẻ vẫn lọt cặp sai. Cửa sổ qua Tết phải dùng đúng năm, lượt đổi chế độ phải bỏ căn cứ cũ. Sửa chữ thất bại phải đi đường lỗi sẵn, không trả ẩn dụ hoặc tự bịa kết luận. Giữ đường tắt từng byte, không sửa engine/DB/đệm và không ép hai mặt theo C3.</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Codex (máy 2)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FEAT(CEL-200): dat lop han truoc nen cung goc trong v3 (commit 4 ma)
Vi sao: cau thoi diem phai dat cung goc vao van, giu du sao va cach cuc, lay hoa dai van tu bang su that chung. Mo truy hoi dung vai tro sau co, giu nguyen duong tat va dem. Phan kho DB thuoc may 1.

Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16812,7 +16812,7 @@
 2b. Bảng luật hạt giống — XONG 17/10/2026: một luật KINH_TRUNG_LUU (phạm vi xung-chieu, ≥2 nhóm nguồn, mỗi nguồn kèm trích nguyên văn đối chiếu máy); bản duyệt D:\Celestia\BANG-LUAT-TO-HOP-2b.md
 3a. Chat STANDARD cân theo lớp hạn sau cờ CELES_LOP_HAN — XONG 17/10/2026 (nghieng-ve tinhTheoLopHan + dữ kiện luu-tu-hoa / tu-hoa-dai-van)
 3b. XONG phần mã máy 2: Focused nhận cờ, giữ meta đúng chế độ, dữ kiện hoá gốc/năm/đại vận theo cửa sổ, validator hoá–sao–cung–lớp–năm–F/W, quét chữ cấm + Q-nguon/Q2; đường tắt so 25 snapshot từ base25ad334; không ép hai mặt. Chưa bật cờ, còn phụ thuộc 3a' máy 1.
-4. v3 thoiDiem xếp lớp hạn lên trước
+4. XONG phần mã máy 2: v3 câu thời điểm đặt lớp hạn trước rồi nền cung gốc/cách cục của cung đang xét; giữ ID và toàn bộ dữ kiện gốc, bổ sung hoá đại vận từ engine, regex bóc vai trò năm/đại vận. Sau CELES_LOP_HAN; 247 snapshot off base25ad334 và 102 ca thời điểm offline. Phần kho và đệm thuộc máy 1, chưa làm trong nhánh này.
 5. Hành trình (luan-han.ts) theo bảng sự thật; khoá đệm thêm |nhip:&lt;nhãn&gt;
 Đo phân bố hai phía offline trước khi bật cờ.</t>
         </is>
@@ -16839,7 +16839,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>lib/rag (STANDARD + Focused; v3 chờ Commit 4 phần mã)</t>
+          <t>lib/rag (STANDARD + Focused + v3 phần mã sau cờ)</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -16854,7 +16854,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Máy 2: Commit 4 phần mã v3 tiếp sau 3b. Máy 1: phép cân 3a' theo C1/C3, kho và Hành trình. Không bật cờ hoặc tăng đệm trong nhánh máy 2. Chi phí/tỉ lệ thử lại/502 chưa đo bằng model thật; chủ dự án chạy eval-chat-quyet-dinh sau tích hợp.</t>
+          <t>Máy 2 xong 3b (17a9ab3) và Commit 4 phần mã. Toàn tính năng vẫn Đang phát triển: chờ 3a' C1/C3 máy 1, kho và Hành trình; chưa bật cờ/tăng đệm. Chưa đo model thật, chi phí/502/độ trễ; chủ dự án chạy eval-chat-quyet-dinh sau tích hợp.</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -16864,7 +16864,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>(nhánh viec/van-han-3b, commit 3b)</t>
+          <t>(nhánh viec/van-han-3b, Commit 4 phần mã)</t>
         </is>
       </c>
     </row>
@@ -17355,7 +17355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G286"/>
+  <dimension ref="A1:G287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27792,7 +27792,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Cờ từ server truyền tới dữ kiện/nghiêng từng cửa sổ và dựng lại meta. Chỉ mode bật thêm marker ký; mode khác bỏ meta. Bảng hoá gốc/năm/đại vận hiện trong F và map W; quan hệ đúng hoa-sao-cung-lớp-năm mới được nhắc, không lấy d.sao làm quyền. Prompt đặt cung gốc trong vận theo API máy 1, không tự cân. Quét tiếng lóng và ẩn dụ trên answer/claim và lời cuối STANDARD; sửa trong vòng hiện có, còn lỗi trả thất bại sẵn. Q-nguon nói mức chắc chắn, Q2 theo câu đã duyệt.</t>
+          <t>Cờ server tới Focused, dữ kiện và phép nghiêng từng W. Meta chỉ mode bật thêm marker ký; khác mode bỏ căn cứ cũ. F hoá gốc/năm/đại vận và lưu tinh theo từng năm qua Tết; kiểm đúng hoá–sao–cung–lớp–năm–F/W, không cấp quyền d.sao. Giữ nhãn lớp qua nhiều vế, từ chối nhiều sao/mơ hồ/nguồn tháng-ngày không có. Quét answer/claims/chip và văn cuối STANDARD. Sửa trong vòng cũ, vẫn sai trả đường lỗi sẵn. Q-nguon không tự thuật thiếu kho; Q2 theo câu đã duyệt. Không ép hai mặt.</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -27803,6 +27803,43 @@
       <c r="G286" t="inlineStr">
         <is>
           <t>lib/rag/kiem-lop-han.ts; lib/rag/boi-canh-la-so.ts; lib/rag/focused/; lib/rag/tra-loi.ts; lib/rag/sua-chua.ts; scripts/test-lop-han-3b.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Lớp hạn — máy 2</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>4-ma-may2</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Bài luận v3 đặt cung gốc trong vận, chỉ phần mã</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>chuanBiCau đọc CELES_LOP_HAN và hoiThoiDiem, truyền tham số vào dungDuKien/truyHoiChoCau. Dữ kiện giữ mã F và đầy đủ nội dung/sao/cách cục gốc; chỉ nhánh bật xếp nhóm hạn trước, nhóm cung chính/cách cục gốc ngay sau, rồi phần bổ sung. Đại vận thêm bốn hoá theo API engine dạng Hóa X vào Sao (Cung); parser thuần bocHoaVan đọc thêm vai trò đại vận và mọi năm đang xét, khử trùng theo vai trò và quan hệ. Prompt timed sau cờ ưu tiên vận+nền, không ép hai mặt/tự cân/hoá giải. Cờ tắt giữ system và dữ kiện byte như base25ad334.</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Không xoá hay sửa dữ kiện sao/cách cục gốc. Giữ vaiTro để truy hồi cung chính không lệch, chỉ thêm nhãn lopHan sau cờ. Không chạm DB/kho/THE_HE_DEM/PHUONG_PHAP/khoá đệm; bài v3 cũ có thể vẫn nằm trong đệm đến khi chủ dự án bật/xử lý đợt riêng.</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/du-kien.ts; lib/rag/v3/index.ts; lib/rag/v3/truy-hoi-v3.ts; lib/rag/v3/prompt-v3.ts; scripts/test-lop-han-v3.ts</t>
         </is>
       </c>
     </row>
@@ -27818,7 +27855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F190"/>
+  <dimension ref="A1:F191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33908,6 +33945,38 @@
         </is>
       </c>
       <c r="F190" t="inlineStr">
+        <is>
+          <t>Codex (máy 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-3b, Commit 4 phần mã)</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Commit 4 mã v3: thứ tự hạn→nền sau cờ, giữ dữ kiện gốc, thêm tứ hoá đại vận và parser truy hồi theo vai trò; prompt thời điểm theo C1/C3. Thêm test247snapshot từ base và102câu thời điểm.</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Chủ dự án đã duyệt việc đặt cung gốc vào vận: vận quyết chiều, nền phải được xét cùng vận, không chỉ bỏ vào cuối bài. Giữ dữ kiện và ID gốc để không mất căn cứ; hoá đại vận phải theo bảng sự thật engine chung, không tự tính lại. Tách mã khỏi sửa kho và tăng đệm vì các việc đó ảnh hưởng DB dùng chung/chi phí và thuộc máy 1, cần chủ dự án bấm.</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
         <is>
           <t>Codex (máy 2)</t>
         </is>

</xml_diff>

<commit_message>
FEAT(CEL-200): hoan tat vong 2 co lop han va sua B4 Tuan Triet
Gom doc co runtime, chan them chu noi bo va giu nen khong dao chieu v3.
Them test env qua bai dai/hai nua bang voi model gia; sua B4 ca TQ10/TC01.
Anh chup doi vi B4: base25ad334 + ban va B4 doc lap, 248 hash.

Vi sao: theo giao viec may 2 vong 2 da duyet; Tuan khong tu manh hau van,
Triet nhat dan khong chia tuoi 30. Giu nguyen engine, DB, phien ban va dem.

Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16812,9 +16812,10 @@
 2b. Bảng luật hạt giống — XONG 17/10/2026: một luật KINH_TRUNG_LUU (phạm vi xung-chieu, ≥2 nhóm nguồn, mỗi nguồn kèm trích nguyên văn đối chiếu máy); bản duyệt D:\Celestia\BANG-LUAT-TO-HOP-2b.md
 3a. Chat STANDARD cân theo lớp hạn sau cờ CELES_LOP_HAN — XONG 17/10/2026 (nghieng-ve tinhTheoLopHan + dữ kiện luu-tu-hoa / tu-hoa-dai-van)
 3b. XONG phần mã máy 2: Focused nhận cờ, giữ meta đúng chế độ, dữ kiện hoá gốc/năm/đại vận theo cửa sổ, validator hoá–sao–cung–lớp–năm–F/W, quét chữ cấm + Q-nguon/Q2; đường tắt so 25 snapshot từ base25ad334; không ép hai mặt. Chưa bật cờ, còn phụ thuộc 3a' máy 1.
-4. XONG phần mã máy 2: v3 câu thời điểm đặt lớp hạn trước rồi nền cung gốc/cách cục của cung đang xét; giữ ID và toàn bộ dữ kiện gốc, bổ sung hoá đại vận từ engine, regex bóc vai trò năm/đại vận. Sau CELES_LOP_HAN; 247 snapshot off base25ad334 và 102 ca thời điểm offline. Phần kho và đệm thuộc máy 1, chưa làm trong nhánh này.
+4. XONG phần mã máy 2: v3 câu thời điểm đặt lớp hạn trước rồi nền cung gốc/cách cục của cung đang xét; giữ ID và toàn bộ dữ kiện gốc, bổ sung hoá đại vận từ engine, regex bóc vai trò năm/đại vận. Sau CELES_LOP_HAN; 248 snapshot off baseline25ad334+B4 và 102 ca thời điểm offline. Phần kho và đệm thuộc máy 1, chưa làm trong nhánh này.
 5. Hành trình (luan-han.ts) theo bảng sự thật; khoá đệm thêm |nhip:&lt;nhãn&gt;
-Đo phân bố hai phía offline trước khi bật cờ.</t>
+Đo phân bố hai phía offline trước khi bật cờ.
+Vòng 2 máy 2 (17/10): thống nhất hàm đọc cờ, v3 không để nền đảo chiều, chặn thêm ba cụm nội bộ; 20 lượt model giả kiểm env thiếu/0/1/0 qua bài dài và hai nửa bảng. B4 sửa Triệt đầu đời nhạt dần, Tuần nhẹ dai suốt đời tại dữ kiện/TQ10/TC01, không gác cờ.</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -16854,7 +16855,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Máy 2 xong 3b (17a9ab3) và Commit 4 phần mã. Toàn tính năng vẫn Đang phát triển: chờ 3a' C1/C3 máy 1, kho và Hành trình; chưa bật cờ/tăng đệm. Chưa đo model thật, chi phí/502/độ trễ; chủ dự án chạy eval-chat-quyet-dinh sau tích hợp.</t>
+          <t>Máy 2 xong 3b (17a9ab3) và Commit 4 phần mã. Toàn tính năng vẫn Đang phát triển: chờ 3a' C1/C3 máy 1, kho và Hành trình; chưa bật cờ/tăng đệm. Chưa đo model thật, chi phí/502/độ trễ; chủ dự án chạy eval-chat-quyet-dinh sau tích hợp. Vòng 2 việc1–2 xong mã, B4 không tăng đệm nên bài đã lưu vẫn có thể chứa câu cũ; việc3 bộ ca đáp án chờ push được chủ dự án bảo rồi nhánh riêng.</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -16864,7 +16865,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>(nhánh viec/van-han-3b, Commit 4 phần mã)</t>
+          <t>(nhánh viec/van-han-3b, vòng 2)</t>
         </is>
       </c>
     </row>
@@ -27792,7 +27793,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Cờ server tới Focused, dữ kiện và phép nghiêng từng W. Meta chỉ mode bật thêm marker ký; khác mode bỏ căn cứ cũ. F hoá gốc/năm/đại vận và lưu tinh theo từng năm qua Tết; kiểm đúng hoá–sao–cung–lớp–năm–F/W, không cấp quyền d.sao. Giữ nhãn lớp qua nhiều vế, từ chối nhiều sao/mơ hồ/nguồn tháng-ngày không có. Quét answer/claims/chip và văn cuối STANDARD. Sửa trong vòng cũ, vẫn sai trả đường lỗi sẵn. Q-nguon không tự thuật thiếu kho; Q2 theo câu đã duyệt. Không ép hai mặt.</t>
+          <t>Cờ server tới Focused, dữ kiện và phép nghiêng từng W. Meta chỉ mode bật thêm marker ký; khác mode bỏ căn cứ cũ. F hoá gốc/năm/đại vận và lưu tinh theo từng năm qua Tết; kiểm đúng hoá–sao–cung–lớp–năm–F/W, không cấp quyền d.sao. Giữ nhãn lớp qua nhiều vế, từ chối nhiều sao/mơ hồ/nguồn tháng-ngày không có. Quét answer/claims/chip và văn cuối STANDARD. Sửa trong vòng cũ, vẫn sai trả đường lỗi sẵn. Q-nguon không tự thuật thiếu kho; Q2 theo câu đã duyệt. Không ép hai mặt. Hàm co-lop-han.lopHanBat đọc cờ lúc gọi cho mọi bề mặt, tra-loi re-export giữ API; validator chặn lớp nền/nền sẵn/lớp hạn. Bài dài/bảng kiểm prompt thật qua I/O giả với env thiếu/0/1/0, cả epModel.</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -27829,7 +27830,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>chuanBiCau đọc CELES_LOP_HAN và hoiThoiDiem, truyền tham số vào dungDuKien/truyHoiChoCau. Dữ kiện giữ mã F và đầy đủ nội dung/sao/cách cục gốc; chỉ nhánh bật xếp nhóm hạn trước, nhóm cung chính/cách cục gốc ngay sau, rồi phần bổ sung. Đại vận thêm bốn hoá theo API engine dạng Hóa X vào Sao (Cung); parser thuần bocHoaVan đọc thêm vai trò đại vận và mọi năm đang xét, khử trùng theo vai trò và quan hệ. Prompt timed sau cờ ưu tiên vận+nền, không ép hai mặt/tự cân/hoá giải. Cờ tắt giữ system và dữ kiện byte như base25ad334.</t>
+          <t>chuanBiCau đọc CELES_LOP_HAN và hoiThoiDiem, truyền tham số vào dungDuKien/truyHoiChoCau. Dữ kiện giữ mã F và đầy đủ nội dung/sao/cách cục gốc; chỉ nhánh bật xếp nhóm hạn trước, nhóm cung chính/cách cục gốc ngay sau, rồi phần bổ sung. Đại vận thêm bốn hoá theo API engine dạng Hóa X vào Sao (Cung); parser thuần bocHoaVan đọc thêm vai trò đại vận và mọi năm đang xét, khử trùng theo vai trò và quan hệ. Prompt timed sau cờ ưu tiên vận+nền, không ép hai mặt/tự cân/hoá giải. Cờ tắt giữ system và dữ kiện byte như baseline25ad334+B4 (ngoại lệ sửa nội dung đã duyệt, không gác cờ). Prompt không để nền đảo chiều nhận định thời gian; không giả định đã có chiều engine. B4 sửa ungated Triệt rõ đầu đời nhạt dần, Tuần nhẹ dai suốt đời, không nêu tuổi; sửa cả TQ10 và TC01. 248 hash so25ad334+B4 độc lập (kể cả khung), 102ca thời điểm và2lá Mệnh có Tuần/Triệt ×2cờ. Giữ phiên bản/đệm nên bài đệm cũ chưa tự đổi.</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -27855,7 +27856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F191"/>
+  <dimension ref="A1:F192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33977,6 +33978,38 @@
         </is>
       </c>
       <c r="F191" t="inlineStr">
+        <is>
+          <t>Codex (máy 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-3b, vòng 2)</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Vòng2: gom đọc cờ, siết promptv3/validator;20lượt offline envruntime qua bài dài/bảng; sửa B4 dữ kiện,TQ10,TC01;248snapshot baselineB4 độc lập.</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Theo VIEC-MAY2-tiep-3b-vong2.md đã duyệt: v3 thiếu nguyên tắc nền không lật chiều; test cũ xoá env nên bỏ sót đường bật. B4 theo bản7: Tuần không tự mạnh hậu vận; Triệt nhạt dần, không chia tuổi30. TC01 còn cùng câu sai nên sửa cùng. Giữ phiên bản và đệm theo quyết định chủ dự án; mẫu đổi chỉ vì B4, không dùng mã mới tự xác nhận.</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
         <is>
           <t>Codex (máy 2)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: ho so cung (3a' ban 7 buoc C-A) — gom du kien quan he quanh mot cung, chua noi vao dau
lib/tuvi/ho-so-cung.ts: hoSoCung (sao toa thu / xung chieu / tam hop / nhi hop / giap kem do sang,
Tuan Triet va Ky tai cung goc; vo chinh dieu muon xung chieu + co Nhat, Nguyet sang chieu tach rieng;
chan dau / theo got khong phan nam nu (Q4); thao go Tuan Triet o dai van cho Menh; dia loi theo
Tu Vi ham so 424-445 chi cho Phuc / Menh / Than; lop han theo nam xem), hoSoLa.
Khong cham diem, khong nhan chieu, khong import lib/rag, khong doi hanh vi dang chay.
Test 38 ca + quet 1.512 la, buoc CI moi. Backlog CEL-200 Logic #4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16844,7 +16844,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, lib/tuvi/tu-hoa-han.ts, lib/tuvi/luat-to-hop.ts</t>
+          <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, lib/tuvi/tu-hoa-han.ts, lib/tuvi/luat-to-hop.ts, lib/tuvi/ho-so-cung.ts</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -16859,7 +16859,7 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>17/10/2026</t>
+          <t>18/10/2026</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -17355,7 +17355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G285"/>
+  <dimension ref="A1:G286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27769,6 +27769,43 @@
         </is>
       </c>
     </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Hồ sơ cung (3a' bản 7, bước C-A): gom dữ kiện quan hệ quanh một cung, chưa nối vào đâu</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>lib/tuvi/ho-so-cung.ts hoSoCung(laSo, chiIndex, namXem?): mọi sao ở toạ thủ / xung chiếu / tam hợp / nhị hợp (lục hợp chi, (1-i) mod 12) / giáp (i±1), mỗi sao kèm độ sáng, cung gốc, Tuần Triệt tại cung gốc, Kỵ gốc đồng cung. Vô chính diệu: chính tinh xung chiếu là sao mượn (giữ độ sáng gốc) + cờ Thái Dương/Thái Âm M-V-Đ chiếu từ tam phương. Tuần Triệt: kiểu chặn đầu khi tuổi dương gặp ở cung dương hoặc âm gặp âm, còn lại theo gót (không phân nam nữ); Mệnh bị một cái, đại vận gặp cái còn lại thì tháo gỡ. Địa lợi sinh/vượng/bại/tuyệt theo hành Bản Mệnh, chỉ cho Phúc Đức / Mệnh / Thân. Có năm xem thì thêm sao lưu và tứ hoá lưu + đại vận rơi vào các vị trí trên, cờ cung đại vận / tiểu hạn. hoSoLa: tuổi dương, thuận/nghịch lý, Mệnh–Cục, chiều đại vận, Tuần Triệt thô ở Mệnh và Thân.</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Chỉ thu dữ kiện: không chấm điểm, không nhãn tốt/xấu, không nhãn chiều (chiều lớp hạn vẫn do engine, C1 bản 4). Địa lợi là bảng Tử Vi hàm số 424–445, KHÔNG phải vòng Tràng Sinh (bản 1 dùng nhầm, reviewer bắt). Câu nghiệm lý 1974 :382 c 'Mệnh, Thân bị cả Tuần lẫn Triệt' đọc được hai cách nên để cờ thô, không gộp. Không import lib/rag (app type-check lib/tuvi). Bài quét: mỗi nhánh phải gặp ≥1 lần.</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>lib/tuvi/ho-so-cung.ts, scripts/test-ho-so-cung.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27781,7 +27818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F189"/>
+  <dimension ref="A1:F190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33839,6 +33876,38 @@
         </is>
       </c>
       <c r="F189" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Thêm lib/tuvi/ho-so-cung.ts (hoSoCung, hoSoLa, diaLoi, kieuTuanTriet, cungNhiHop, cungGiap, laVoChinhDieu) + scripts/test-ho-so-cung.ts (38 ca, quét 1.512 lá) + bước CI. Chưa nối vào prompt hay engine, không đổi hành vi.</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Bước C-A của phương án 3a' bản 2 (D:\Celestia\PHUONG-AN-3a-ban7-ma.md), chủ dự án duyệt 18/10/2026. Cách chấm cũ đếm sao cát/hung; muốn xét theo quan hệ (hoá giải, chế, độ hợp) thì trước hết cần một chỗ duy nhất gom vị trí, độ sáng, Tuần Triệt, địa lợi quanh một cung. Máy 2 dùng chung hàm này cho khung bộ ca đáp án, không tự viết lại. Chặn đầu không phân nam nữ theo quyết định Q4 18/10.</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT(CEL-200): bang luat quan he sao + Tuan Triet (buoc C-B), sua theo celes-domain
40 luat quan he + 13 dong Tuan Triet theo sao, may kiem bang (Q1 dem theo nhom tac gia,
ngoaiLeCua, uuTien nguoc chieu), doi chieu trich dan voi kho sach. Chua noi vao engine/prompt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16844,7 +16844,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, lib/tuvi/tu-hoa-han.ts, lib/tuvi/luat-to-hop.ts, lib/tuvi/ho-so-cung.ts</t>
+          <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, lib/tuvi/tu-hoa-han.ts, lib/tuvi/luat-to-hop.ts, lib/tuvi/ho-so-cung.ts, lib/tuvi/luat-quan-he.ts</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -17355,7 +17355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G286"/>
+  <dimension ref="A1:G287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27806,6 +27806,43 @@
         </is>
       </c>
     </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Bảng luật quan hệ sao + Tuần Triệt (3a' bản 7, bước C-B): căn cứ nội bộ, chưa nối vào đâu</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>lib/tuvi/luat-quan-he.ts: LUAT_QUAN_HE 40 luật (B1 phá cách, B2 Tử Phủ, B3 Thiên Tướng, B4 sát đắc hợp mệnh / Đồng Cơ Lương, B5 Hóa Kỵ / Khoa / Thiên Giải / Nguyệt Đức, E Vũ Khúc / Nhật Nguyệt / Tam hoá). Mỗi luật: sao chủ động, sao bị tác động (có trừ), vị trí đồng cung / tam phương / cung hạn, điều kiện cung, độ sáng, cần kèm, ngưỡng, biến đổi, hành mệnh, mức (lat / chan / giam / giam-luat / thu-hep...), độ bền, uuTien, ngoaiLeCua, câu nghĩa, nguồn + nguồn ngược, chắc chắn, linhVuc tuỳ chọn. TUAN_TRIET: luật chung (phạm vi không lan cung khác, cường độ Triệt mạnh đến 30 tuổi, đảo chiều với sao hãm, cung Kim Mộc chỉ tăng cường độ, vô chính diệu, chặn đầu) + 13 dòng theo sao. doSangHieuDung đổi bậc sáng khi gặp Tuần/Triệt.</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Q1: đếm theo tác giả độc lập (NHOM_NGUON, Tổng hợp + Hàm số cùng nhóm Nguyễn Phát Lộc); một nhóm chỉ được giam / giam-luat / thu-hep, Tuần Triệt một nhóm không được mat / dao-thanh-hai / nang. Sách ngược nhau thì hạ mức + ghi nguonNguoc + trình chủ dự án. Luật hoá giải là căn cứ nội bộ, KHÔNG vào lời bài luận, không hiện nguồn sách cho người dùng. Câu sách chỉ nói một lĩnh vực thì ghi linhVuc, không áp rộng. kiemBangQuanHe: thu-hep / giam-luat phải có ngoaiLeCua tồn tại, không trỏ chính nó; hai luật ngược chiều cùng khớp phải phân uuTien. Bài test đối chiếu từng trích dẫn với kho sách khi có kho.</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>lib/tuvi/luat-quan-he.ts, scripts/test-luat-quan-he.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27818,7 +27855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F190"/>
+  <dimension ref="A1:F191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33908,6 +33945,38 @@
         </is>
       </c>
       <c r="F190" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Thêm lib/tuvi/luat-quan-he.ts (40 luật quan hệ, khối Tuần Triệt 13 dòng theo sao, máy kiểm bảng) + scripts/test-luat-quan-he.ts + bước CI. Sau celes-domain: hạ Phủ sợ Không Kiếp / Tử Phủ hạn Không Kiếp / Tướng sợ Hình về giảm, Tử Phủ gặp Tuần về giảm, bỏ TT_PHU_TAI, Nhật Nguyệt Sửu Mùi dụng Kỵ hạ về giảm (sách ngược), Vũ Khúc giải sát chỉ khi Vũ đắc trở lên, Liêm Tham cần Hình cùng Kình/Đà. Chưa nối vào engine hay prompt, không đổi hành vi.</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Bước C-B của phương án 3a' bản 7 (D:\Celestia\PHUONG-AN-3a-ban7-ma.md); bảng đếm C-B bản 2 chủ dự án duyệt 18/10/2026 (X1–X10, Q1–Q5). Chấm vận hạn theo quan hệ sao (chế, hoá giải, phá cách) cần một bảng luật có nguồn kiểm được thay vì đếm cát/hung. celes-domain đọc nguyên văn TH 4051/4091, HS 2144/2916/1414, AB 4280/4794 và bắt các mức vượt câu sách; đã sửa theo. Còn trình chủ dự án: Đà La đắc địa trong engine (dosang.ts:51, Thìn Tuất Sửu Mùi) lệch NLTT 455/458 (Dần Thân Tỵ Hợi).</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX(CEL-178): luan giai v3 duong doc dem lo pb/model ra trinh duyet
Duong 'du cau trong dem' tra cauDem thang, quen anNoiBo. Them test offline goi
xuLyLuanGiaiV3 voi moi truong gia (do truoc khi sua) + buoc CI.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -27855,7 +27855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F191"/>
+  <dimension ref="A1:F192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33977,6 +33977,38 @@
         </is>
       </c>
       <c r="F191" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>CEL-178</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Sửa lib/rag/v3/xu-ly.ts:403: đường 'đủ câu trong đệm' giờ gỡ pb / model bằng anNoiBo như hai đường vừa viết. Thêm scripts/test-an-noi-bo-v3.ts (gọi xuLyLuanGiaiV3 với môi trường giả, offline) + bước CI.</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>CEL-178 cất pb / model vào đệm cho trang chấm bài của quản trị và đặt anNoiBo để không gửi ra trình duyệt, nhưng chỉ gỡ ở hai đường vừa viết; đường đọc đệm (lượt xem thứ hai trở đi, tức phần lớn lượt) trả thẳng nên tên model lộ trong JSON, trái luật mặt trước không lộ tên model. Lọt vì không bài CI nào gọi xuLyLuanGiaiV3. Bài mới đỏ trước khi sửa (2/6 ca), xanh sau. Chủ dự án bảo sửa trong nhánh này 18/10/2026.</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT(CEL-200): luat quan he — Da La dac tu mo khop engine, cach Da ham Dan Than Ty Hoi, Nhat Nguyet Ky Suu Mui lat
- SAT_DUNG_KINH_DA: Da dac o Thin Tuat Suu Mui theo dosang.ts (chu du an chot 19/10/2026), nguon KL 2618/2481/2482
- Them DA_DAN_THAN_VCD, DA_HAM_GAP_QUYEN, NHAT_NGUYET_KY_HONG_CACH (43 luat)
- NHAT_NGUYET_SUU_MUI_DUNG_KY len lat/cao (TH 4091 la cau thu hep, khong phai cau bac); TT_NHAT_NGUYET_SUU_MUI len nang
- Test doi chieu luat dung sat voi engine

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16859,7 +16859,7 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>18/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -27829,7 +27829,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>lib/tuvi/luat-quan-he.ts: LUAT_QUAN_HE 40 luật (B1 phá cách, B2 Tử Phủ, B3 Thiên Tướng, B4 sát đắc hợp mệnh / Đồng Cơ Lương, B5 Hóa Kỵ / Khoa / Thiên Giải / Nguyệt Đức, E Vũ Khúc / Nhật Nguyệt / Tam hoá). Mỗi luật: sao chủ động, sao bị tác động (có trừ), vị trí đồng cung / tam phương / cung hạn, điều kiện cung, độ sáng, cần kèm, ngưỡng, biến đổi, hành mệnh, mức (lat / chan / giam / giam-luat / thu-hep...), độ bền, uuTien, ngoaiLeCua, câu nghĩa, nguồn + nguồn ngược, chắc chắn, linhVuc tuỳ chọn. TUAN_TRIET: luật chung (phạm vi không lan cung khác, cường độ Triệt mạnh đến 30 tuổi, đảo chiều với sao hãm, cung Kim Mộc chỉ tăng cường độ, vô chính diệu, chặn đầu) + 13 dòng theo sao. doSangHieuDung đổi bậc sáng khi gặp Tuần/Triệt.</t>
+          <t>lib/tuvi/luat-quan-he.ts: LUAT_QUAN_HE 43 luật (B1 phá cách, B2 Tử Phủ, B3 Thiên Tướng, B4 sát đắc hợp mệnh / Đồng Cơ Lương, B5 Hóa Kỵ / Khoa / Thiên Giải / Nguyệt Đức, E Vũ Khúc / Nhật Nguyệt / Tam hoá, cách Đà La hãm ở Dần Thân Tỵ Hợi). Mỗi luật: sao chủ động, sao bị tác động (có trừ), vị trí đồng cung / tam phương / cung hạn, điều kiện cung, độ sáng, cần kèm, ngưỡng, biến đổi, hành mệnh, mức (lat / chan / giam / giam-luat / thu-hep...), độ bền, uuTien, ngoaiLeCua, câu nghĩa, nguồn + nguồn ngược, chắc chắn, linhVuc tuỳ chọn. Kình Đà đắc ở tứ mộ theo dosang.ts (chủ dự án chốt 19/10/2026); test đối chiếu luật dùng sát với engine. TUAN_TRIET: luật chung (phạm vi không lan cung khác, cường độ Triệt mạnh đến 30 tuổi, đảo chiều với sao hãm, cung Kim Mộc chỉ tăng cường độ, vô chính diệu, chặn đầu) + 13 dòng theo sao. doSangHieuDung đổi bậc sáng khi gặp Tuần/Triệt.</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -27855,7 +27855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F192"/>
+  <dimension ref="A1:F193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34009,6 +34009,38 @@
         </is>
       </c>
       <c r="F192" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>lib/tuvi/luat-quan-he.ts: SAT_DUNG_KINH_DA lấy Đà đắc ở tứ mộ (khớp dosang.ts), nguồn chính KL 2618/2481/2482. Thêm DA_DAN_THAN_VCD (Đà Dần Thân ở Mệnh vô chính diệu thành cách, Tuần Triệt làm giảm), DA_HAM_GAP_QUYEN (Đà hãm Dần Thân Tỵ Hợi gặp Quyền + Lộc/Lực Sĩ), NHAT_NGUYET_KY_HONG_CACH (Kình Đà / Không Kiếp đồng cung làm hỏng cách). NHAT_NGUYET_SUU_MUI_DUNG_KY lên lat / cao, bỏ nguonNguoc; TT_NHAT_NGUYET_SUU_MUI lên nang. 43 luật. Test thêm ca đối chiếu engine.</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Chủ dự án chốt 19/10/2026: Đà La đắc ở Thìn Tuất Sửu Mùi (Đà hành Kim, tứ mộ Thổ sinh Kim) — engine đã đúng, mệnh bàn không đổi; bảng luật đang theo NLTT 458 (phía thiểu số, Dần Thân Tỵ Hợi) nên sửa cho khớp. chuyen-gia-tu-vi soát: Đà ở Dần Thân Tỵ Hợi tuy hãm vẫn có cách riêng trong sách (TH 2541/3287, KL 1874, KL 1867, TD 548) nên thêm luật thay vì đổi độ sáng. Nhật Nguyệt Sửu Mùi gặp Kỵ trước bị hạ 'giam' vì đọc nhầm TH 4091 là câu bác; thật ra là câu thu hẹp (hại mắt), còn HS 2916/1653, KL 2131/2461, TH 4092, CK 1135 đều nói Kỵ làm sáng, Tuần Triệt thành cách lớn. Chưa nối engine/prompt, không đổi hành vi.</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT(CEL-200): xet cung theo thu tu sach (C-C) - xetLaSo chay bang luat quan he + Tuan Triet, ra 4 danh sach; Tu Phu che chi o Dan Than
Sua theo chuyen-gia-tu-vi: Tuan Triet chan sao chieu vao, sat ham khong len dac,
luat DUNG xet do sang goc, theo-chung = giam, cung han dung Triet manh theo tuoi,
tran 'chat vat' / 'che khong vung'. Chua noi engine/prompt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16844,7 +16844,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, lib/tuvi/tu-hoa-han.ts, lib/tuvi/luat-to-hop.ts, lib/tuvi/ho-so-cung.ts, lib/tuvi/luat-quan-he.ts</t>
+          <t>lib/rag/nghieng-ve.ts, lib/rag/boi-canh-la-so.ts, lib/rag/tra-loi.ts, lib/tuvi/tu-hoa-han.ts, lib/tuvi/luat-to-hop.ts, lib/tuvi/ho-so-cung.ts, lib/tuvi/luat-quan-he.ts, lib/tuvi/xet-cung.ts</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -16854,7 +16854,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Phân bố đo offline (60 lá × 2024–2030 × 4 chủ đề): cũ thuận rõ 42.8% / cản rõ 1.7% / đủ hai mặt 93.6%; lớp hạn thuận rõ 23.4% / cản rõ 24.9% / đủ hai mặt 81.6%. Ngưỡng chấp nhận (L3) chờ chủ dự án duyệt; cần tách theo chủ đề (sức khỏe, tình cảm) trước khi bật. Rủi ro celes-domain nêu: hệ số tam phương 0.5 và ngưỡng huongTu chưa có cơ sở sách; nhãn 'rõ' tính theo tỉ lệ nên một mục chiếu tam phương đứng một mình vẫn ra 'cản rõ'; Lưu Kỵ ở Mệnh lên phía cản của mọi chủ đề chiếu tới Mệnh. Focused chưa nhận cờ (3b). Kiểm cặp (hoá, sao) ở STANDARD chỉ dựa vào prompt.</t>
+          <t>Xét cung (C-C) còn hoãn: trọng số tọa thủ/chiếu và viTri 'giap' riêng cho cách giáp; tách tiền/hậu vận cho Triệt khi đọc lá gốc; Tuần Triệt ở cung của bên bị tác động; sát đắc đi với bộ không dụng được vẫn có hại; thứ tự Phúc/Mệnh chưa truyền kết quả nền sang cung hỏi; Kỵ gốc và Kỵ lưu gộp tên khi đếm. C-D chờ 3b máy 2; C-E kế tiếp.</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -17355,7 +17355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G287"/>
+  <dimension ref="A1:G288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27843,6 +27843,43 @@
         </is>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Xét cung theo thứ tự sách (3a' bản 7, bước C-C): chạy bảng luật quan hệ trên hồ sơ cung, ra bốn danh sách</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>lib/tuvi/xet-cung.ts xetLaSo(laSo, {cungHoi?, namXem?}): thứ tự Phúc Đức → Mệnh → Thân → cung hỏi (không trùng). Mỗi cung: (a) địa lợi từ hoSoCung; (b) chính tinh độ sáng gốc → hiệu dụng (doSangHieuDung, Triệt mạnh khi tuổi âm &lt; 30, không năm xem coi là mạnh); sao hung KHÔNG lên bậc khi gặp Tuần Triệt (giữ hãm, chỉ ghi giảm); (c) nhanDangCachCuc; (d)(e) khopLuat: dong-cung = cả hai tọa thủ, tam-phuong = tọa thủ/xung/tam hợp (giáp, nhị hợp không tính), cung-han chỉ ở cung hạn (bên bị tác động lấy sao gốc tam phương Mệnh, dùng trietConManh theo năm xem). Luật DUNG mở cửa theo độ sáng GỐC. Tuần Triệt ở cung đang xét chắn sao chiếu vào (xung/tam hợp): cung vô chính diệu gặp Triệt chắn cả, gặp Tuần chắn sao hung; cung có chính tinh chắn bớt (ghi giảm). bienDoi theo-chung = giảm. dieuKienLa: mệnh-cục tương sinh / âm dương thuận lý thiếu thì luật CHẾ/GIẢI vẫn khớp với trạng thái 'khong-vung'. phanXu: ngoại lệ trước (giam-luat chỉ làm yếu), rồi ưu tiên khi hai luật ngược chiều chạm cùng sao; bên thắng luật PHÁ ghi thangPha. Đầu ra không nhãn tốt/xấu: (i) cachThanh/cachPha; (ii) hungKhongCuu (sao hung hãm trong tam phương + Hóa Kỵ, bỏ sao bị chắn cả, cờ giam khi có Tuần/Triệt/chắn) + catBiPha; (iii) tranMuc (khong-ben, một nhóm tác giả, Tuần Triệt giảm, hành mệnh giảm, giam-luat, chắc chắn thấp, hãm gặp Triệt trần ngang đắc, thắng chật vật, chế không vững); (iv) có năm xem: cung đại vận / lưu niên / tiểu hạn, khopGoc và khopHan (chỉ khớp nhờ sao lưu có độ sáng / tứ hoá hạn).</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Hàm thuần, không import lib/rag (app đọc qua @tuvi/*). Chưa nối vào engine/prompt: không đổi hành vi đang chạy. Kình Đà giáp Lộc Tồn KHÔNG phải gặp sát. Tử Phủ cùng chế (TU_PHU_CHE_TU_SAT) chỉ khi Thiên Phủ ở Dần/Thân (Tử Phủ chỉ đồng cung ở đó, TH 4077); để viTri tam-phuong vì phạm vi áp chung cho cả sát. Quét 204.480 lá: không lá nào Tử Phủ Dần Thân gặp đủ 4 sát, nên không có ca test cho tổ hợp đó. Test quét 5760 lá thật, mỗi ca chuyên gia phải gặp ít nhất một lần, không thì đỏ.</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>lib/tuvi/xet-cung.ts, scripts/test-xet-cung.ts, lib/tuvi/luat-quan-he.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27855,7 +27892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F193"/>
+  <dimension ref="A1:F194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34041,6 +34078,38 @@
         </is>
       </c>
       <c r="F193" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Thêm lib/tuvi/xet-cung.ts (xetLaSo, khopLuat, phanXu): chạy 43 luật quan hệ + khối Tuần Triệt trên hồ sơ cung theo thứ tự Phúc → Mệnh → Thân → cung hỏi, ra bốn danh sách (cách thành/phá, hung không được cứu + cát bị phá, trần mức, cung hạn). TU_PHU_CHE_TU_SAT thêm dieuKienCung Thiên Phủ ở Dần/Thân. Test scripts/test-xet-cung.ts vào CI.</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Bước C-C của phương án 3a bản 7 (chủ dự án duyệt 18/10/2026): bảng luật (C-B) mới là dữ liệu, cần bộ chạy đúng thứ tự sách (Tử Vi hàm số 446–456: Phúc, Mệnh, Thân trước; Tuần Triệt xét trước mọi luật) để C-D, C-E đọc kết quả thay vì đếm sao. Đầu ra cố ý không nhãn tốt/xấu vì chiều lớp hạn do engine tính ở chỗ cũ (C1 bản 4). chuyen-gia-tu-vi soát bản đầu nêu 5 lỗi, đã sửa: Tuần Triệt chắn sao chiếu vào (CK 1238); sát hãm gặp Triệt không thành đắc, luật DUNG xét độ sáng gốc (TH 4095, KL 2670); theo-chung = giảm; cung hạn dùng Triệt mạnh theo tuổi; Tử Phủ chỉ đồng cung Dần Thân, thắng luật phá thì trần 'chật vật', thiếu điều kiện cả lá thì 'chế không vững'. Thêm Hóa Kỵ vào danh sách hung, sao lưu có độ sáng. Các điểm chưa tối ưu còn lại ghi ở cột Việc còn lại. Chưa nối engine/prompt, không đổi hành vi.</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT(CEL-200): C-E bo luat ep hai mat cua phep can lop han
- dauMoc lay 6 moc nang nhat, khong chen moc phia thieu
- luat 2 prompt khoiTheoLopHan: co can cu thi neu, khong co thi khong them cho du;
  ghi ro thay cho chi dan "can ca hai mat" / "noi luon phan chua chac"
- cam them "quyet chieu", "lat chieu", "dan chung"
- PHIEN_BAN_NGHIENG_LOP_HAN 2026.10.1 -> 2026.10.2 (chu du an da duyet)
- test-lop-han-chat: kiem khong con luat hai mat, kiem khong chen (dot bien do)
- docs/bay/ai-rag: luat khong ep hai mat; sua quy-tac-luan-giai doi PHIEN_BAN_CHU

Dao quyet dinh 16/10 theo C3/Q2. Chi duong co CELES_LOP_HAN; co tat khong doi byte.
Chua sua quy-tac-luan-giai.ts:76 (doi hash khoa dem moi be mat) - cho chu du an.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -27892,7 +27892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F194"/>
+  <dimension ref="A1:F195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34110,6 +34110,38 @@
         </is>
       </c>
       <c r="F194" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-lop-han)</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>C-E: phép cân lớp hạn bỏ luật 'luôn nói hai mặt'. dauMoc = 6 mốc nặng nhất, không chèn mốc phía thiếu; luật 2 prompt khoiTheoLopHan thành 'có căn cứ thì nêu, không có thì không thêm cho đủ', ghi rõ thay cho 'cân cả hai mặt' / 'nói luôn phần chưa chắc' với câu hỏi thời gian; cấm thêm 'quyết chiều', 'lật chiều', 'dẫn chứng'. PHIEN_BAN_NGHIENG_LOP_HAN 2026.10.1 → 2026.10.2. Chỉ đường cờ CELES_LOP_HAN (chat STANDARD); cờ tắt không đổi byte; Focused không đi qua.</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Đảo quyết định 'luôn nói hai mặt' ngày 16/10 theo C3/Q2 của chủ dự án: ép hai mặt bắt model dựng ý ngược chiều khi năm nghiêng hẳn một phía (đo 60 lá × 7 năm × 4 chủ đề: 6 ca top mốc bị chèn phía kia). CHƯA sửa luật 4 'Cân cả hai mặt' ở quy-tac-luan-giai.ts:76 vì sửa sẽ đổi PHIEN_BAN_CHU — hash khoá đệm mọi bề mặt, toàn bộ bài đệm sinh lại; chờ chủ dự án quyết.</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: backlog cuoi vong K1/K2/K3 + don tai lieu tro ma cu
- Backlog: CEL-143 (K1), CEL-138/142/119 (K2), CEL-186 (K3); go mo ta nut Tao ban moi o CEL-142/147/161/175, L27; NHAN_CACH_CELES, NET_CHINH_TINH -> ten hien hanh.
- HUONG-DAN/AGENTS/bien-tap-vi: tro dung CHUAN_NGON_NGU_CELES, NET_VI/NET_EN; ghi K3 hoi thang.
- TRANG-THAI: tra ve ban main (dong trang thai chi ghi tren main).
- X1 (CEL-148) KHONG ghi o day: ma nam o viec/han-muc-token, ghi backlog cung nhanh do.

Vi sao: soat-tai-lieu bat backlog mo ta ma khong co tren nhanh va tai lieu tro hang da xoa.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -3979,7 +3979,7 @@
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>NHAN_CACH_CELES trong lib/ai/prompt.ts + CHUAN_NGON_NGU_CELES trong lib/rag/chuan-ngon-ngu.ts. Cả prompt chat lẫn prompt bài dài đều nhúng.</t>
+          <t>CHUAN_NGON_NGU_CELES trong lib/rag/chuan-ngon-ngu.ts (NHAN_CACH_CELES ở lib/ai/prompt.ts đã bỏ). Cả prompt chat lẫn prompt bài dài đều nhúng.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="N37" s="8" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O37" s="8" t="inlineStr">
@@ -10540,21 +10540,17 @@
       </c>
       <c r="M119" s="8" t="inlineStr">
         <is>
-          <t>Lần đầu một lá số: nhóm tổng quan 11 câu mất ~47s (đo trên máy) — sát trần 60s nên route đặt hạn chót 52s và bỏ vòng sửa khi còn &lt;20s. Khách mở lá số mới là 11+ lượt gọi model (không hạn mức, theo quyết định). Chưa làm: chuyên gia duyệt trọng số chấm Mạnh/Bình/Cần gắng; lưu Hồng Loan/Thiên Hỷ theo năm; bản tiếng Anh. Điểm đo phần lớn do luna tự chấm (gemini 429).
-CẬP NHẬT 24/09/2026 (giao diện): ba thẻ đầu /la-so lấy từ TQ02/TQ03/TQ08 của v3 (thẻ khuôn cũ chỉ còn là đường lùi khi v3 hỏng); câu đã lên thẻ không lặp ở danh sách; danh sách tổng quan thành thẻ đánh số. Nút chính "Đọc luận giải chuyên sâu" → /luan-giai/sau; link phụ "Khám phá từng chủ đề" → /luan-giai. Bỏ dòng hạn mức (LuotBaiSau) và nhãn "Độ rõ". /luan-giai/sau: tag năm xem nổi bật, bỏ mô tả, mục lục thẻ có số + số câu + "Đã đọc x/14" (điện thoại: chip cuộn ngang), cuối bài "← Đọc lại: chủ đề trước" + "Đọc tiếp".
-ĐÃ LÊN PROD 24/09/2026 (nhánh viec/chong-lap-chuyen-sau, trước đó chờ credit): chống lặp ý giữa các câu chuyên sâu + chặn chữ lạ (production có "აღარ" ở TQ02). Chờ OpenAI nạp credit để Celes chạy đo lại — đổi phiên bản prompt/dữ kiện làm mọi bài đệm phải sinh lại.
-SỰ CỐ 24/09/2026 (ĐÃ XỬ LÝ — chủ dự án nạp credit): OpenAI báo hết credit — gpt-5.6-luna và embedding RAG đều hỏng; bài chưa đệm sẽ lỗi hoặc lùi về bảng cũ.
-CHỐNG LẶP Ý (24/09/2026): câu không hỏi thời điểm thì dữ kiện không kèm mốc tuổi; mỗi câu chuyên sâu biết các câu cùng chủ đề lo phần nào; bộ kiểm chặn mốc tuổi ở câu không hỏi thời điểm, chặn chữ không phải tiếng Việt, chặn bài chuyên sâu không có lời khuyên ở đoạn cuối. Đo lá số A, 19 câu chuyên sâu: câu gắn mốc tuổi sai chỗ 7 → 0, "trước 30 tuổi" 8 → 3 câu, "25–34 tuổi" 10 → 4 câu; giám khảo 4,06 → 4,15. Đổi phiên bản prompt/dữ kiện → mọi bài đệm sinh lại lần đầu.</t>
+          <t>K2 (22/10/2026): luật 7 prompt-v3 — câu khép ý dán sang lá số nào cũng đúng thì bỏ, kết bằng ý cuối của phần luận. Bài cũ chỉ viết lại khi dấu lg (logic) đổi; đổi luật giọng này không tự viết lại bài đã có.</t>
         </is>
       </c>
       <c r="N119" s="8" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O119" s="8" t="inlineStr">
         <is>
-          <t>chong-lap-chuyen-sau</t>
+          <t>2d845f4</t>
         </is>
       </c>
     </row>
@@ -12086,17 +12082,17 @@
       </c>
       <c r="M138" s="8" t="inlineStr">
         <is>
-          <t>Sổ ý và Bức tranh lớn đọc theo tiền tố khoá MỚI: lá số giờ chẵn chỉ thấy các chủ đề đã mở lại sau 26/09 (mở lại chủ đề là tự chuyển khoá). Nút "Tạo bản mới" (thay cho việc tăng thế hệ) vẫn chờ làm.</t>
+          <t>K2 (22/10/2026, CELES-31): khoá đệm tách giọng khỏi logic. PHIEN_BAN_CHU băm các phiên bản logic + XA_DEM_CO_CHU_DICH; sửa giọng văn không làm bài sinh lại. Mỗi câu V3 cất dấu lg (LOGIC_V3): lệch dấu thì câu coi như thiếu và viết lại khi mở, bản cũ hiện tạm; khách hết lượt vẫn được bài cũ thay vì 429. Lúc deploy: đệm 6 bề mặt mất hiệu lực một lần (chủ dự án đã biết). Ngoại lệ lg theo quyết định 10.19 C.</t>
         </is>
       </c>
       <c r="N138" s="8" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O138" s="8" t="inlineStr">
         <is>
-          <t>dem-da-thiet-bi-gioi-han-khach</t>
+          <t>2d845f4</t>
         </is>
       </c>
     </row>
@@ -12363,15 +12359,12 @@
       </c>
       <c r="E142" s="8" t="inlineStr">
         <is>
-          <t>1. phienBanKho(): dấu vân tay các tài liệu đang xuất bản (id, bản xuất bản, mức tin cậy, loại nguồn)
-2. Mỗi câu cất kèm kho; bài cũ không dấu coi như kho 40749bb09806 (đo lúc deploy) để nút không bật hàng loạt
-3. /api/luan-giai-v3 taoMoi: cần đăng nhập (401 cho khách), chỉ viết lại câu viết với kho cũ; tóm lại / bức tranh lớn cũng viết lại theo kho
-4. Nút ở cuối tổng quan (/la-so) và cuối mỗi chủ đề (/luan-giai/sau), chỉ hiện khi có câu viết với kho cũ</t>
+          <t>Đã gỡ 22/10/2026 (K2). Thay bằng dấu lg trên từng câu V3 (CEL-138): đọc đệm thấy lệch dấu logic thì câu coi như thiếu và được viết lại khi mở; chưa viết lại được thì hiện bản cũ. Dấu kho vẫn ghi kèm câu để đo, không còn bật nút nào. Không còn taoMoi ở /api/luan-giai-v3.</t>
         </is>
       </c>
       <c r="F142" s="9" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Tạm dừng</t>
         </is>
       </c>
       <c r="G142" s="8" t="inlineStr">
@@ -12406,17 +12399,17 @@
       </c>
       <c r="M142" s="8" t="inlineStr">
         <is>
-          <t>Mọi thay đổi kho (xuất bản, lưu trữ, đổi mức tin cậy) đều bật nút cho MỌI lá số — gom thay đổi kho thành đợt. Đã kiểm bằng server thật: khách 401, bài cũ banMoi=false. CHƯA kiểm được luồng viết lại khi đã đăng nhập bằng trình duyệt (cần tài khoản thật).</t>
+          <t>Gỡ 22/10/2026 (K2, CELES-31): nút 'Tạo bản mới' và taoMoi ở route V3 đã bỏ. Thay bằng dấu lg trên từng câu (CEL-138): logic đổi thì câu tự viết lại khi mở, người dùng không phải bấm.</t>
         </is>
       </c>
       <c r="N142" s="8" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O142" s="8" t="inlineStr">
         <is>
-          <t>rag-tin-cay</t>
+          <t>2d845f4</t>
         </is>
       </c>
     </row>
@@ -12486,17 +12479,17 @@
       </c>
       <c r="M143" s="8" t="inlineStr">
         <is>
-          <t>KẾT QUẢ LƯỢT 1: 1.091 mục (741 tổ hợp) từ 997 đoạn, 74% ứng viên qua kiểm tất định, tốn 0,64 tr token vào / 0,37 tr ra. Tiêu chí: #1 ghép bỏ qua 0,4% ĐẠT · #2 ý có nguồn 51% → 78% ĐẠT · #3 độ phủ 100% ĐẠT · #5 p95 30,2 → 22,4 giây ĐẠT · #4 so mù ~47% (luna 48/42, gpt-4o-mini 50/46) TRƯỢT → không bật (QĐ-15). Chỉ gọi được 2 model giám khảo khác nhau. Chẩn đoán: văn ngang nhau, thư viện tăng độ có căn cứ nhưng giám khảo máy không chấm độ đúng. Độ đúng trích ~80% trên 40 mẫu, lỗi chính: bỏ sót điều kiện cung; ~6,5 cặp ngược chiều mỗi bài. Chủ dự án chọn hướng: tự đọc mù chấm độ đúng / sửa khâu trích rồi đo lại / đổi ngưỡng. || 26/09: bộ đo độ đúng (CEL-144) cũng không thấy B đúng hơn A → giữ tắt.</t>
+          <t>K1 (22/10/2026, CELES-26): khối T### chỉ nhận mục nặng ĐÃ duyệt (cờ CELES_THU_VIEN_MANH_CHUA_DUYET=1 mở lại); mục bị lật bởi quan hệ ĐÃ xác minh thì bỏ trước trần 18; quan hệ do máy gán thì giữ cả hai, ghi 'chưa xác minh', không dẫn theo bên nào; bỏ dòng 'cân cả hai'. Câu V3 mới lưu canCu = toàn bộ tập đã cấp (thư viện: id + đợt + dấu sha1; nguồn: documentId + versionId + chunkId), không ra trình duyệt. Còn lại: X3 dùng canCu để thu hồi bài khi một mục bị gỡ.</t>
         </is>
       </c>
       <c r="N143" s="8" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O143" s="8" t="inlineStr">
         <is>
-          <t>thu-vien-su-nghiep</t>
+          <t>57fc633</t>
         </is>
       </c>
     </row>
@@ -12805,12 +12798,12 @@
       </c>
       <c r="M147" s="8" t="inlineStr">
         <is>
-          <t>OpenAI đang HẾT CREDIT — chưa sinh được bài mới nào cho tới khi nạp. Cách tắt: xoá mã câu khỏi CAU_THU_VIEN. Máy đo trước đó: kiến thức +1 điểm, cách viết ngang — chủ dự án tự đánh giá. Lá số đã có bài Sự nghiệp: bấm "Tạo bản mới" ở cuối chủ đề để xem bản có thư viện (mỗi lá một lần).</t>
+          <t>OpenAI đang HẾT CREDIT — chưa sinh được bài mới nào cho tới khi nạp. Cách tắt: xoá mã câu khỏi CAU_THU_VIEN. Máy đo trước đó: kiến thức +1 điểm, cách viết ngang — chủ dự án tự đánh giá. Nút 'Tạo bản mới' đã gỡ 22/10/2026 (K2): bài cũ chỉ viết lại khi dấu logic đổi, không theo dấu kho.</t>
         </is>
       </c>
       <c r="N147" s="8" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O147" s="8" t="inlineStr">
@@ -14402,12 +14395,12 @@
       </c>
       <c r="M167" s="8" t="inlineStr">
         <is>
-          <t>Bài chỉ viết bằng tiếng Việt; giao diện EN có dòng báo. Chưa có nút Tạo bản mới và xuất bài như web. Chưa chạy thật: production chưa nhận Bearer (chờ merge viec/app-gd1).</t>
+          <t>Bài chỉ viết bằng tiếng Việt; giao diện EN có dòng báo. Chưa có xuất bài như web (nút Tạo bản mới web đã gỡ 22/10/2026). Chưa chạy thật: production chưa nhận Bearer (chờ merge viec/app-gd1).</t>
         </is>
       </c>
       <c r="N167" s="8" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O167" s="8" t="inlineStr">
@@ -15119,12 +15112,12 @@
       </c>
       <c r="M176" s="8" t="inlineStr">
         <is>
-          <t>Chưa đo mù chất lượng bài như Sự nghiệp (so-sanh-v3). Tỉ lệ qua kiểm tất định 53–74% (Con cái thấp nhất). Câu có hỏi thời điểm (TD02, TB03, TB05, SK02, CC01, RN01, TC01, GD03) chưa dùng thư viện. Bài đã viết của các câu vừa bật sẽ hiện "Tạo bản mới"</t>
+          <t>Chưa đo mù chất lượng bài như Sự nghiệp (so-sanh-v3). Tỉ lệ qua kiểm tất định 53–74% (Con cái thấp nhất). Câu có hỏi thời điểm (TD02, TB03, TB05, SK02, CC01, RN01, TC01, GD03) chưa dùng thư viện. Bài đã viết của các câu vừa bật giữ nguyên (nút Tạo bản mới đã gỡ 22/10/2026); chỉ viết lại khi dấu logic đổi.</t>
         </is>
       </c>
       <c r="N176" s="8" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O176" s="8" t="inlineStr">
@@ -15906,18 +15899,17 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>Đã push 4fb4ce9, CI xanh (run 37307475844). CHƯA GỘP main, chờ chủ dự án duyệt. Thêm commit sửa log y_dinh (retrieval_runs) trên cùng nhánh. Việc nối tiếp: CEL-191 (spec xong, chờ gộp), CEL-192 (discovery).
-Eval I5 (05/10/2026, 155 lượt, model ghim): 23/30 flow đạt; 502 3/155 (flow 28 đã sửa ở 738430e, đo lại 0/20); viết lại 14/155; p50/p95 11,5/19,8 s. Eval mù: Barnum 100%, 502 0/24. CHỜ CHỦ DỰ ÁN QUYẾT: flow 2 (trọng yếu, 'Tháng 10 tôi tìm việc được không?') khuôn A chỉ 2/5 vì planner luật không nhận 'tìm việc' → model phân loại ghi đè ý định — sửa cần luật mới hoặc đụng planner chung; flow 18 (EN 'this year') khuôn G vì planner không đọc 'this year' — đụng planner chung; flow 22/22.5 kỳ vọng tong-quan trong spec đã lỗi thời (planner giờ ra gia-dao); flow 29 eval đòi chip 'Sang năm' có mặt, thiết kế chỉ thêm từ tháng 9 âm. Nợ: chip A/B (tachHaiVe), flow 17 bịa 'hai lần', trẻ dưới 1 tuổi bị luận như đã đi học, chip đoán giới tính, KHONG_CAN_CU 502 ~1%. CỔNG TRƯỚC PRODUCTION: 502 ≤ 1%; lỗi chặn dữ kiện = 0; flow trọng yếu 100%; p95 chốt theo mốc đo; CEL-190; thân bài + chip EN; app di động (Q7).</t>
+          <t>K3 (22/10/2026, CELES-34): hỏi một tháng thì nói theo độ tin, mã chặn THANG_CHAC_CAO; PHIEN_BAN_FOCUSED focused-2026.10.22 (hội thoại đang dở lúc deploy mất meta lượt trước một lần). Chưa đo tỉ lệ viết lại bằng model thật. Đường B + so mù A/B: chờ chủ dự án quyết ngân sách (CELES-38).</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
         <is>
-          <t>05/10/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O186" s="8" t="inlineStr">
         <is>
-          <t>(nhánh viec/cel-186-focused-chat)</t>
+          <t>c2e58ff</t>
         </is>
       </c>
     </row>
@@ -17348,7 +17340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G278"/>
+  <dimension ref="A1:G286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -19903,7 +19895,7 @@
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>quick-read.ts đọc THẲNG từ dữ liệu lá số ra ba góc nhìn: một chính, hai phụ. Lời văn lấy từ kho NET_CHINH_TINH (14 chính tinh) và bảng chủ đề 12 cung.</t>
+          <t>quick-read.ts đọc THẲNG từ dữ liệu lá số ra ba góc nhìn: một chính, hai phụ. Lời văn lấy từ NET_VI / NET_EN trong lib/tuvi/quick-read-noi-dung.ts (14 chính tinh) và bảng chủ đề 12 cung.</t>
         </is>
       </c>
       <c r="F73" s="32" t="inlineStr">
@@ -23728,7 +23720,7 @@
       </c>
       <c r="F176" s="32" t="inlineStr">
         <is>
-          <t>Chỉ thêm chủ đề khi gói đợt đã có trong Supabase — thêm trước là dấu kho đổi, nút "Tạo bản mới" hiện mà viết lại không có gì mới. Sự nghiệp giữ nguyên dấu sn-2,sn-2b.</t>
+          <t>Chỉ thêm chủ đề khi gói đợt đã có trong Supabase — thêm trước là dấu kho đổi mà thư viện rỗng. Từ K2 (22/10/2026) dấu kho chỉ ghi để đo, không bật viết lại; viết lại theo dấu lg. Sự nghiệp giữ nguyên dấu sn-2,sn-2b.</t>
         </is>
       </c>
       <c r="G176" s="8" t="inlineStr">
@@ -27500,6 +27492,302 @@
       <c r="G278" t="inlineStr">
         <is>
           <t>app/api/admin/can-duyet/route.ts, app/admin/can-duyet/page.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Thư viện → prompt V3</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>K1-1</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Lọc mục nặng chưa duyệt</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>cho-prompt.ts: mục có mức nặng mà chưa ai duyệt không vào khối T###; khopHet vẫn giữ đủ để đo. Cờ CELES_THU_VIEN_MANH_CHUA_DUYET=1 mở lại.</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Nghĩa sách nặng chưa ai duyệt không được tự quyết nội dung bài (QĐ 10.15).</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/cho-prompt.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Thư viện → prompt V3</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>K1-2</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Bỏ mục bị lật</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Quan hệ lật/hoá giải ĐÃ duyệt cùng cung: bỏ mục đích TRƯỚC trần 18, xếp mục lật lên đầu, miễn hạn mức bỏ sao. Quan hệ máy gán: giữ cả hai, chú thích 'chưa xác minh', không dẫn theo bên nào.</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Chỉ quan hệ đã xác minh mới được xoá một mục khỏi prompt (ghi chú kỹ thuật 1 của chủ dự án).</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-vien/cho-prompt.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Luận giải V3</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>K1-3</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Lưu căn cứ mỗi câu</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Câu V3 mới cất canCu = toàn bộ tập đã cấp cho câu đó. anNoiBo gỡ canCu (và pb, tên model ở đường trả từ đệm) trước khi trả trình duyệt.</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Nguồn RAG và tên model không ra trình duyệt; trước K1 đường trả từ đệm từng lộ pb + tên model.</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts, scripts/test-thu-vien-prompt.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>CEL-138</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Đệm V3</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>K2-1</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Khoá giọng tách khoá logic</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>PHIEN_BAN_CHU = băm (các PHIEN_BAN_* logic + XA_DEM_CO_CHU_DICH). Chuẩn giọng không vào khoá.</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Sửa giọng từng làm mọi lá số sinh lại (đổi THE_HE_DEM); test-focused kiểm DAU_VAO_PHIEN_BAN_CHU.</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>lib/rag/phien-ban-chu.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>CEL-138</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Đệm V3</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>K2-2</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Dấu lg từng câu</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Câu, tóm lại, bức tranh lớn cất lg = LOGIC_V3 (thiếu dấu = LG_TRUOC_DAU). Đọc đệm: lệch dấu = thiếu → viết lại; chưa viết lại được thì hiện bản cũ; tóm lại lệch dấu mà câu chưa viết lại thì giữ tóm lại cũ, không ghép từ câu logic cũ. lg không ra trình duyệt.</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Khách hết lượt không được nhận 429 khi đã có bài cũ.</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts, scripts/test-dau-logic-v3.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>CEL-119</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Prompt V3</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>K2-3</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Câu khép ý mang ý riêng</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Luật 7 prompt-v3: câu khép ý dán sang lá số nào cũng đúng thì bỏ, kết bằng ý cuối của phần luận.</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Câu kết chung chung lặp ở mọi bài (khảo sát v4).</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/prompt-v3.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Focused — hỏi một tháng</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>K3-1</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Nói theo độ tin</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Có thoiGian.thang: mô tả hướng thuan-ro / can-ro đổi sang nói rõ chiều nhưng theo độ tin (MO_TA_HUONG_THANG); khối thời gian thêm dòng ĐỘ TIN (độ tin khác độ nặng, tháng vướng nặng vẫn nói nặng). Guard tên đọc cùng chữ (hoiThang).</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Không thêm luật đứng trên MO_TA_HUONG trái với nó: đổi chính mô tả. Độ tin thấp không được thành nói nhẹ đi (C1 bản 4).</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/prompt.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Focused — validator</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>K3-2</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>THANG_CHAC_CAO (tầng B)</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Hỏi một tháng: câu nào có 'chắc chắn / chắc luôn / chắc như đinh / trăm phần trăm' thì viết lại; tha khi cùng vế có không/chưa/chẳng/khó/đâu hoặc lời dặn hãy/cần/nếu. CHAC_CHAN_GIA bắt trước thì không báo trùng.</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Không bắt 'nhất định' đứng một mình ('ở một mức nhất định'). Tầng B sai hai lần là 502 — danh sách giữ hẹp.</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>lib/rag/focused/kiem.ts, lib/rag/focused/hop-dong.ts, scripts/test-thang-chac-thap.ts</t>
         </is>
       </c>
     </row>
@@ -27515,7 +27803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F184"/>
+  <dimension ref="A1:F188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33413,6 +33701,134 @@
         </is>
       </c>
       <c r="F184" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>57fc633 (nhánh viec/kho-toi-thieu, gộp vào viec/khoa-dem-giong)</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>CEL-143, CELES-26</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>K1 kho tối thiểu: chặn mục nặng chưa duyệt, bỏ mục bị lật đã xác minh, bỏ 'cân cả hai', lưu căn cứ câu V3, vá lộ pb/tên model ở đường đệm.</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Quyết định 10.15 kho tri thức: nghĩa nặng chưa ai duyệt và nhãn lật do máy gán đã được đưa thẳng vào bài luận mà không ai kiểm. Cần căn cứ để X3 truy được bài nào dùng mục nào khi phải thu hồi.</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>0b4c50d, 2e40bc1, e912738, 2d845f4 (nhánh viec/khoa-dem-giong)</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>CEL-138, CEL-142, CEL-119, CELES-31</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>K2: tách khoá đệm giọng khỏi logic, dấu lg trên từng câu V3, gỡ nút 'Tạo bản mới', câu khép ý V3 phải mang ý riêng.</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Mỗi lần sửa giọng là mọi bài sinh lại (tốn tiền, người dùng thấy bài đổi), còn sửa logic thì bài cũ sai vẫn nằm đó tới khi người dùng tự bấm nút. Dấu lg cho bài sai tự viết lại, bài chỉ khác giọng thì giữ.</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>(commit này, nhánh viec/so-mu-cach-viet)</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>CEL-036, CEL-142, CEL-147, CEL-161, CEL-175, L12, L27</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Dọn mô tả còn trỏ nút 'Tạo bản mới' đã gỡ và mã đã đổi tên (NHAN_CACH_CELES, NET_CHINH_TINH).</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>soat-tai-lieu bắt được: backlog còn tả luồng không còn chạy, người đọc sau sẽ tin nút vẫn còn.</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>c2e58ff (nhánh viec/so-mu-cach-viet)</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>CEL-186, CELES-34</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>K3 phần tháng: Focused hỏi một tháng nói theo độ tin, validator chặn nói chắc ở tầng tháng.</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Vận một tháng là lớp mỏng nhất của lá số, nói 'chắc chắn' ở tầng này là vượt dữ kiện. Phần A/B của K3 tách ra vì chạy A/B cần model trả phí hoặc Groq miễn phí không đủ sức (prompt V3 ~5,8k token + 6k trả lời &gt; 8k TPM).</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: backlog CEL-186 duong B + so mu A/B; script nhan --env cho worktree (CELES-38)
Da sinh 24 cap so mu tren model that (~0,27 USD, B dat 24/24, A 23/24, B dat ~1,6 lan).
Ket qua va cach cham: D:/Celestia/so-mu-ab-2026-10-22/BAO-CAO.md.

Vi sao: worktree khong co .env.local rieng; backlog phai mo ta duong B va nguong
dua vao san pham truoc khi cham mu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -15899,7 +15899,7 @@
       </c>
       <c r="M186" s="8" t="inlineStr">
         <is>
-          <t>K3 (22/10/2026, CELES-34): hỏi một tháng thì nói theo độ tin, mã chặn THANG_CHAC_CAO; PHIEN_BAN_FOCUSED focused-2026.10.22 (hội thoại đang dở lúc deploy mất meta lượt trước một lần). Chưa đo tỉ lệ viết lại bằng model thật. Đường B + so mù A/B: chờ chủ dự án quyết ngân sách (CELES-38).</t>
+          <t>K3 (22/10/2026, CELES-34): hỏi một tháng thì nói theo độ tin, mã chặn THANG_CHAC_CAO; PHIEN_BAN_FOCUSED focused-2026.10.22 (hội thoại đang dở lúc deploy mất meta lượt trước một lần). Chưa đo tỉ lệ viết lại bằng model thật. Đường B (CELES-38, 22/10): đã viết sau cờ thuNghiem.duongB (chỉ script), đã sinh 24 cặp so mù trên model thật (~0,27 USD; B đắt ~1,6 lần A, lọc ý chỉ bỏ 2/90 ý). Chờ chấm mù (CELES-35); ngưỡng đưa vào sản phẩm: B thắng ≥14/24, không thua vì an toàn. Kết quả: D:/Celestia/so-mu-ab-2026-10-22/BAO-CAO.md.</t>
         </is>
       </c>
       <c r="N186" s="8" t="inlineStr">
@@ -17340,7 +17340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G286"/>
+  <dimension ref="A1:G287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27791,6 +27791,43 @@
         </is>
       </c>
     </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>CEL-186</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Luận giải V3 — đường B (thử nghiệm)</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>K3-3</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Lập ý → lọc → diễn đạt</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Chỉ khi thuNghiem.duongB: lượt 1 (SYSTEM_LAP_Y = luật căn cứ + luật an toàn) trả ý kèm mã + mức chắc; kiemDanY bỏ ý không mã / mã lạ / sao ngoài dữ kiện, chỉ HẠ mức chắc theo loại căn cứ (mạnh cần F + nguồn không bổ trợ; cung chính / cách cục sàn vừa); lượt 2 dùng system sản phẩm, chỉ diễn đạt ý đã giữ; sao được nêu ở 'vì sao' = sao của ý + F được dẫn + xung chiếu/tam hợp của các cung ấy. Hỏng lượt 1 hoặc 0 ý thì lùi đường A.</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Sản phẩm không có đường bật duongB (test-duong-b-v3 quét app/lib/components). Ý mạnh vẫn phải nói bằng lời xu hướng (celes-domain bắt 'nói chắc' trái luật an toàn).</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/duong-b.ts, lib/rag/v3/index.ts, scripts/sinh-cap-ab-v3.ts, scripts/test-duong-b-v3.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27803,7 +27840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F188"/>
+  <dimension ref="A1:F189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33829,6 +33866,38 @@
         </is>
       </c>
       <c r="F188" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>cc0e871 + commit này (nhánh viec/duong-b-ab)</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>CEL-186, CELES-38</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Đường B luận giải V3 sau cờ thử nghiệm + script sinh 24 cặp so mù A/B trên model thật, trần cứng 1 USD.</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Chủ dự án đổi quyết định 22/10/2026: cho test mất phí, chỉ việc thật cần. Cần số đo xem tách lập ý khỏi diễn đạt có đáng gấp 1,6 lần chi phí không trước khi đụng sản phẩm.</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: backlog dot 1 - X1, X2 nguyet han Cach 1, G1-G3, ngoai le co phi, T-02..T-05
Vi sao: ghi mot lan cho ca dot tich hop (CELES-36); X2 chon cach thong dung ba sach cung noi (QD 10.23, Q5), X3 chua gop cho Q-X3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1364,7 +1364,7 @@
         <is>
           <t>1. cungDaiVan() theo tuổi âm tại năm xem
 2. cungTieuHan() theo năm
-3. cungNguyetHan() theo tháng ÂM (không phải tháng dương)</t>
+3. cungNguyetHan() theo tháng ÂM. Từ cung tiểu hạn năm xem (kể là tháng 1) đếm NGHỊCH tới tháng sinh âm; tại đó kể giờ Tý, đếm THUẬN tới chi giờ sinh: cung dừng lại là tháng Giêng. Tháng xem m: thuận (m−1) cung từ tháng Giêng. Tháng nhuận dùng cung của tháng chính.</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
@@ -1404,17 +1404,18 @@
       </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
-          <t>Lớp NGÀY chưa có — xem CEL-071. Bẫy đã trả giá: nguyệt hạn phải nhận tháng ÂM.</t>
+          <t>Lớp NGÀY chưa có — xem CEL-071. Bẫy đã trả giá: nguyệt hạn phải nhận tháng ÂM.
+X2 (22/10/2026): nguyệt hạn theo Cách 1, PHUONG_PHAP.phienBan 2026.10.2. Bài đệm cũ hết hạn: 6 bề mặt có |v: sinh lại khi mở; câu V3 có dữ kiện nguyệt hạn viết lại khi mở và không lùi về bài thế hệ trước. Đếm số bài sẽ viết lại: scripts/dem-bai-dem-dot-1.ts (chủ dự án chạy). App phải build lại sau khi lên production.</t>
         </is>
       </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O4" s="8" t="inlineStr">
         <is>
-          <t>a04efc7</t>
+          <t>9d89e40</t>
         </is>
       </c>
     </row>
@@ -12879,17 +12880,18 @@
       </c>
       <c r="M148" s="8" t="inlineStr">
         <is>
-          <t>Số đo nền (60 câu): mỗi câu 1,25 lượt, 11.678 vào (41% đệm), 1.429 ra; token ra ~61% tiền, vòng sửa 22% token ra (30/37 ca lỗi một câu). Ước giảm ~20–25% mỗi câu (9 nghìn → ~7 nghìn / lá đọc trọn) — CHƯA đo được vì OpenAI hết credit; đo lại bằng 6 câu (~0,1 tr token). Test: một vòng A/B nghiệm thu ~3 tr → ~0,5 tr token (~0,25 tr với Batch). Sửa cục bộ chưa chạy thật với model — có đường lùi về sửa cả bài.</t>
+          <t>Số đo nền (60 câu): mỗi câu 1,25 lượt, 11.678 vào (41% đệm), 1.429 ra; token ra ~61% tiền, vòng sửa 22% token ra (30/37 ca lỗi một câu). Ước giảm ~20–25% mỗi câu (9 nghìn → ~7 nghìn / lá đọc trọn) — CHƯA đo được vì OpenAI hết credit; đo lại bằng 6 câu (~0,1 tr token). Test: một vòng A/B nghiệm thu ~3 tr → ~0,5 tr token (~0,25 tr với Batch). Sửa cục bộ chưa chạy thật với model — có đường lùi về sửa cả bài.
+X1 (22/10/2026, Codex máy 2, commit f7495ca nhánh viec/han-muc-token, đã gộp vào viec/tich-hop-dot-1 (000b19d)): cổng chi phí đặt TRƯỚC lời gọi provider, phủ cả gọi trực tiếp lẫn fallback. Bốn trần: token Groq/ngày, token thử/ngày, số lượt thử/ngày, ngân sách tiến trình; lượt thử chỉ được ba model Groq, chặn fallback sang model trả phí. Lỗi mạng/timeout giữ dấu đối soát, khởi động lại vẫn chặn; embedding sống và OpenAI batch bị chặn trong context thử. Vận hành: docs/quy-trinh/X1-han-muc-thu-nghiem.md. Rủi ro: trần dựa sổ ứng dụng + ước lượng token, không giữ chỗ quota đa máy; script thử cũ thiếu cấu hình mới sẽ dừng.</t>
         </is>
       </c>
       <c r="N148" s="8" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>22/10/2026</t>
         </is>
       </c>
       <c r="O148" s="8" t="inlineStr">
         <is>
-          <t>giam-chi-phi-token</t>
+          <t>000b19d</t>
         </is>
       </c>
     </row>
@@ -17340,7 +17342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G287"/>
+  <dimension ref="A1:G291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27828,6 +27830,154 @@
         </is>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>CEL-148</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Cổng chi phí thử nghiệm (X1)</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>X1-1</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Nhận diện và chặn trước HTTP</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Nhận diện context thử kể cả cờ sai/rỗng; đọc đầy đủ sổ theo ngày UTC; cộng lượt sắp gọi rồi mới so trần; tạo dấu trước HTTP; chốt usage một lần; lỗi chưa rõ giữ dấu. Không đổi cấu hình model, không gian embedding, engine hay prompt.</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Đếm sau khi gọi và chỉ chặn tại fallback không bảo vệ được script gọi trực tiếp hay embedding trả phí.</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>lib/ai/ngan-sach-thu.ts, docs/quy-trinh/X1-han-muc-thu-nghiem.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>CEL-003</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Nguyệt hạn (X2)</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>X2-1</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>An cung nguyệt hạn tháng xem</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Từ cung tiểu hạn năm xem (kể là tháng 1) đếm NGHỊCH tới tháng sinh âm; tại đó kể giờ Tý, đếm THUẬN tới chi giờ sinh: cung dừng lại là tháng Giêng. Tháng xem m: thuận (m−1) cung từ tháng Giêng. Tháng nhuận dùng cung của tháng chính. Công thức: thangGieng = tieuHan − (thangSinh − 1) + chiGio.</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Đổi quy tắc vận hạn phải tăng PHUONG_PHAP.phienBan trong cùng đợt (không thì đệm phát bài cũ). Vân tay mẫu đóng băng test-ansao-chuan nay gồm cả tiểu hạn, nguyệt hạn, lưu tinh (T-03) nên đổi quy tắc mà quên cập nhật mẫu là CI đỏ. Bất biến kiểm trên 60 lá số và 300 ca đối chiếu với cung Mệnh (test-nguyet-han).</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>lib/tuvi/ansao.ts, lib/tuvi/phuong-phap.ts, scripts/test-nguyet-han.ts, scripts/test-ansao-chuan.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>CEL-003</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Nguyệt hạn (X2)</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>X2-2</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Bài V3 cũ có nguyệt hạn</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>locBaiTheHeTruoc: đường lùi về bài thế hệ trước chỉ nhận câu có dấu lg đúng, hoặc câu không mang dữ kiện nguyệt hạn (q.van chứa 'nguyet').</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Còn một đường: banCu (bài cũ hiện tạm khi viết lại lỗi) vẫn có thể hiện nguyệt hạn cũ cho tới lần viết lại thành công.</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts, scripts/test-dau-logic-v3.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>CEL-148</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Cổng chi phí thử nghiệm (X1)</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>X1-2</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Ngoại lệ có phí hẹp cho lượt thử</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Lượt thử (so mù, cổng chất lượng) chỉ được gọi model trả phí khi đủ cả bốn biến: AI_GHIM_MODEL (đúng một provider|model), AI_TRAN_USD (trần cứng), AI_GIA_VAO_USD, AI_GIA_RA_USD. Cộng chi phí ước trước mỗi lời gọi, vượt trần thì dừng. Thiếu một biến là quay về luật X1 (chỉ Groq).</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Không bao giờ đổi ai_model_configs để thử. Chạy --dem trước để biết số lượt. Không có ngoại lệ nào cho đường người dùng thật.</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>lib/ai/ngan-sach-thu.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27840,7 +27990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F189"/>
+  <dimension ref="A1:F193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33898,6 +34048,134 @@
         </is>
       </c>
       <c r="F189" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>f7495ca (gộp 000b19d, nhánh viec/tich-hop-dot-1)</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>CEL-148, CELES-30</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Thêm cổng chi phí X1 cho lượt thử nghiệm: bốn trần, chỉ ba model Groq, chặn fallback trả phí, giữ dấu lỗi qua khởi động lại.</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Đếm sau khi gọi và chỉ chặn tại fallback không bảo vệ được script gọi trực tiếp hoặc embedding trả phí; luật Ngân sách = 0 cần một cổng cứng trước provider.</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Codex (máy 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>18bc889, 77d6190 (gộp 10dbed6), 9d89e40, e8629cf, 079c8d0 (nhánh viec/tich-hop-dot-1)</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>CEL-003, CELES-28</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Nguyệt hạn tính theo Cách 1 (từ cung tiểu hạn đếm nghịch tới tháng sinh, kể giờ Tý thuận tới giờ sinh ra tháng Giêng); tăng phienBan 2026.10.2; đường lùi V3 không trả bài logic cũ cho câu có nguyệt hạn; vân tay mẫu đóng băng thêm vận hạn (T-03, T-05).</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Chủ dự án duyệt Cách 1 (Q5, 22/10/2026, theo quyết định 10.23): chọn cách thông dụng mà ba sách cùng nói (Tử Vi hàm số tr.26 dòng 325, Hà Thúc Hồng dòng 981/1681, Ảo Bí dòng 1904), để Celes thống nhất một chuẩn. Cách trước (tháng Giêng tại cung tiểu hạn) là Cách 2 có nguồn ở Ảo Bí dòng 1905, một phương pháp khác được sách ghi nhận; ghi lại trong docs/chien-luoc/X2-nguyet-han-phuong-an.md. Sáu đáp án đếm tay được chuyên gia kiểm độc lập. Tăng phiên bản ngay (Q6 A) để bài đệm đổi theo cách đã chọn.</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Codex (máy 2) + Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>d53071e, 0bf3829 (gộp 000b19d), b2b687f (nhánh viec/tich-hop-dot-1)</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>CEL-196, CEL-197, CELES-24, CELES-33, CELES-35</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Gộp các công cụ đo đợt 1: G1 script đếm kho tri thức thật + bộ 100 mục đáp án; G2 script hiệu chuẩn model miễn phí (Groq, Gemini) cho việc tiền lọc mục kho; cổng 10.22: script sinh 24 cặp so mù sách thô với bài có thư viện (đã sinh, chờ chấm mù).</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Kế hoạch kho tri thức đợt 1 (duyệt 21/10/2026) cần số đo trước khi quyết bước sau. G1 (22/10): kho 7.883 mục, 0 mục đã duyệt, 2.430 mục nặng nay bị K1 chặn; 701 nhóm gộp ≥2 căn cứ; 98 cặp mâu thuẫn cát/hung cùng chủ đề; tỉ lệ thiếu căn cứ trên 60 lá × 8 chủ đề = 0% cả trước và sau K1. G2: một model đơn lẻ chưa đủ (kiemMuc 53%, gpt-oss-120b 73%); cặp hai model Groq bắt 29/30 lỗi cài sẵn; phần so với chủ dự án duyệt chưa có dữ liệu nên CHƯA cho AI tự duyệt thay người, chỉ tiền lọc. Cổng 10.22 sinh 24 cặp với trần 0,5 USD (Q3), tốn ~0,123 USD. Báo cáo: D:\Celestia\BAO-CAO-G1-dem-kho-tri-thuc-2026-10-22.md, BAO-CAO-G2-hieu-chuan-model-2026-10-22.md.</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Codex (máy 2) + Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>03e1321, e8629cf, 079c8d0, d0635f3, 684f301 (nhánh viec/tich-hop-dot-1)</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>CEL-148, CEL-142, CEL-186, CEL-003, CELES-36</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Ngoại lệ có phí hẹp cho lượt thử (ghim một model, trần USD cứng). Bốn máy canh vào CI: T-02 (không còn nút 'Tạo bản mới', vietLai người thường 403, taoMoi bị bỏ qua), T-03 (vân tay mẫu đóng băng gồm vận hạn), T-04 (cờ đường B tắt thì luận giải V3 y như cũ), T-05 (đường lùi không trả nguyệt hạn cũ). Script đếm bài đệm sẽ viết lại sau đợt 1 (chỉ đọc DB). X3 (cổng thu hồi) CHƯA gộp: chờ chủ dự án trả lời Q-X3-1..6.</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Chủ dự án cho phép test có phí khi thật cần, trần 0,5 USD, chạy --dem trước (Q3, 22/10/2026); X1 chặn mọi model trả phí nên cần một lối hẹp, có trần, không chạm cấu hình model. Bốn máy canh chặn các lỗi đã có giá: nút xả đệm quay lại; đổi quy tắc vận hạn lần 2 mà mẫu đóng băng không bắt (bài học 22/10/2026); bật nhầm đường B; bài nguyệt hạn cũ lọt qua đường lùi. Mỗi máy canh đã thử đột biến cho đỏ. Script đếm để chủ dự án ước lượt model trước khi lên production (Q7).</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FIX: che phan thang cua bai V3 cu dang hien tam (lo hong so 6, X2)
Moi duong con hien ban cu (khach het luot, viet lai loi lui banCu, giu tom lai cu,
buc tranh cu, bai the he truoc) di qua cheThangBanCu: ban khac phienBan thi bo cau
noi thang cu the / nguyet han, them cau "Phan nhip tung thang tam an o ban nay."
Dem giu nguyen ban goc. Test nhom 7 trong test-dau-logic-v3 (da o CI).

Vi sao: X2 tang phienBan nen moi bai V3 phai viet lai; cham tran token thi bai loi
lui ve ban cu con nguyet han tinh theo cach cu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -27927,12 +27927,12 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>locBaiTheHeTruoc: đường lùi về bài thế hệ trước chỉ nhận câu có dấu lg đúng, hoặc câu không mang dữ kiện nguyệt hạn (q.van chứa 'nguyet').</t>
+          <t>locBaiTheHeTruoc: đường lùi về bài thế hệ trước chỉ nhận câu có dấu lg đúng nếu câu đó mang dữ kiện nguyệt hạn. Mọi đường còn hiện bản cũ (khách hết lượt, viết lại lỗi lùi banCu, giữ tóm lại cũ, bức tranh cũ, bài thế hệ trước) đi qua cheThangBanCu: bản có phienBan khác hiện hành thì bỏ các câu / ý chính / gợi ý nói tới tháng cụ thể hoặc nguyệt hạn, thêm câu 'Phần nhịp từng tháng tạm ẩn ở bản này.', phần khác giữ nguyên. Chỉ đổi thứ trả ra, đệm giữ bản gốc để lần viết lại sau thay hẳn.</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>Còn một đường: banCu (bài cũ hiện tạm khi viết lại lỗi) vẫn có thể hiện nguyệt hạn cũ cho tới lần viết lại thành công.</t>
+          <t>Bản cũ khác phienBan không bao giờ được hiện câu nhịp tháng tính theo quy tắc cũ, kể cả khi hết trần token và viết lại lỗi. Máy canh: nhóm 7 scripts/test-dau-logic-v3.ts (CI).</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
@@ -27990,7 +27990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F193"/>
+  <dimension ref="A1:F194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34176,6 +34176,38 @@
         </is>
       </c>
       <c r="F193" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>(nhánh viec/tich-hop-dot-1)</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>CEL-003</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Che phần tháng của bài V3 cũ đang hiện tạm (cheThangBanCu trong lib/rag/v3/xu-ly.ts) + test nhóm 7.</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Lỗ hổng số 6 do điều phối chỉ ra 22/10/2026: X2 tăng phienBan nên mọi bài V3 đã lưu phải viết lại; sau deploy dễ chạm trần token, bài viết lỗi lùi về bản cũ còn nguyệt hạn tính theo cách cũ. Ẩn câu tháng thay vì chặn cả bài để người dùng vẫn đọc được phần năm và phần khác.</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
DOCS: backlog X3 cong thu hoi (CEL-143, CELES-27)
Ghi CEL-143: viec con lai, tep chinh, dieu kien bat; 6 buoc Logic X3-1..X3-6; nhat ky gop 5c7b17a, 8d089c7.
Vi sao: X3 da gop vao nhanh tich hop, backlog phai mo ta dung luong thu hoi dang chay.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -12470,27 +12470,28 @@
       </c>
       <c r="K143" s="8" t="inlineStr">
         <is>
-          <t>KIEN-TRUC-LUAN-GIAI.md, lib/rag/thu-vien/*, lib/rag/v3/index.ts, lib/rag/v3/kiem-v3.ts, lib/rag/v3/truy-hoi-v3.ts, app/api/luan-giai-v3/route.ts, scripts/dung-thu-vien.ts, scripts/do-thu-vien.ts, scripts/test-thu-vien.ts, scripts/so-sanh-v3.ts</t>
+          <t>KIEN-TRUC-LUAN-GIAI.md, lib/rag/thu-vien/*, lib/rag/v3/index.ts, lib/rag/v3/kiem-v3.ts, lib/rag/v3/truy-hoi-v3.ts, app/api/luan-giai-v3/route.ts, scripts/dung-thu-vien.ts, scripts/do-thu-vien.ts, scripts/test-thu-vien.ts, scripts/so-sanh-v3.ts, lib/rag/thu-hoi/cong.ts, lib/rag/thu-hoi/kho.ts, lib/rag/thu-vien/dau.ts, scripts/thu-hoi-muc.ts, supabase/va-thu-hoi-muc.sql</t>
         </is>
       </c>
       <c r="L143" s="8" t="inlineStr">
         <is>
-          <t>Tắt (CAU_THU_VIEN rỗng)</t>
+          <t>Tắt (CAU_THU_VIEN rỗng). Cổng X3: CELES_CONG_THU_HOI=1 và đã chạy va-thu-hoi-muc.sql.</t>
         </is>
       </c>
       <c r="M143" s="8" t="inlineStr">
         <is>
-          <t>K1 (22/10/2026, CELES-26): khối T### chỉ nhận mục nặng ĐÃ duyệt (cờ CELES_THU_VIEN_MANH_CHUA_DUYET=1 mở lại); mục bị lật bởi quan hệ ĐÃ xác minh thì bỏ trước trần 18; quan hệ do máy gán thì giữ cả hai, ghi 'chưa xác minh', không dẫn theo bên nào; bỏ dòng 'cân cả hai'. Câu V3 mới lưu canCu = toàn bộ tập đã cấp (thư viện: id + đợt + dấu sha1; nguồn: documentId + versionId + chunkId), không ra trình duyệt. Còn lại: X3 dùng canCu để thu hồi bài khi một mục bị gỡ.</t>
+          <t>K1 (22/10/2026, CELES-26): khối T### chỉ nhận mục nặng ĐÃ duyệt (cờ CELES_THU_VIEN_MANH_CHUA_DUYET=1 mở lại); mục bị lật bởi quan hệ ĐÃ xác minh thì bỏ trước trần 18; quan hệ do máy gán thì giữ cả hai, ghi 'chưa xác minh', không dẫn theo bên nào; bỏ dòng 'cân cả hai'. Câu V3 mới lưu canCu = toàn bộ tập đã cấp (thư viện: id + đợt + dấu sha1; nguồn: documentId + versionId + chunkId), không ra trình duyệt.
+X3 (23/10/2026, CELES-27): cổng thu hồi mục thư viện. Bảng thu_hoi_muc_thu_vien ghi dấu mục đã thu hồi; máy chủ đọc 60 giây một lần sau cờ CELES_CONG_THU_HOI=1. Câu V3 đã lưu dựa vào mục đó thì được viết lại đúng câu ấy khi có người mở (tính như sinh thường, trong hạn mức X1). Viết hỏng thì hiện câu chờ, đệm giữ bản gốc. Tóm lại, bức tranh, sổ ý và Sổ kết luận cũng được lọc. Đoạn SÁCH thu hồi bằng knowledge_chunks.trang_thai='loai_tru', không qua bảng. Rủi ro: câu viết trước K1 không có căn cứ nên cổng không thấy; lỗi đọc bảng thì cổng mở. Còn lại: chủ dự án chạy supabase/va-thu-hoi-muc.sql, bật cờ trên Preview và đo độ trễ (3a) trước khi bật Production; chữ câu chờ EN/app/PDF ở CELES-39.</t>
         </is>
       </c>
       <c r="N143" s="8" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="O143" s="8" t="inlineStr">
         <is>
-          <t>57fc633</t>
+          <t>5c7b17a, 8d089c7</t>
         </is>
       </c>
     </row>
@@ -17342,7 +17343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G291"/>
+  <dimension ref="A1:G297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27978,6 +27979,228 @@
         </is>
       </c>
     </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Cổng thu hồi (X3)</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>X3-1</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Đọc tập dấu thu hồi</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Cờ CELES_CONG_THU_HOI khác 1 thì tập rỗng, không có truy vấn nào. Bật thì đọc thu_hoi_muc_thu_vien (cột dau, huy_luc is null). Production chỉ đọc phạm vi all; Preview đọc all cộng phạm vi phamViDem của chính máy chủ. Giữ trong RAM 60 giây.</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Lỗi đọc tạm thời: thử lại 1 lần, sau đó dùng tập tốt gần nhất (tối đa 30 phút) hoặc tập rỗng. Cổng MỞ, ghi log [thu-hoi] mo-cong-do-loi, không bao giờ làm hỏng trang. Chưa có bảng hoặc thiếu khoá service-role thì cổng tắt và nhớ trạng thái 10 phút.</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-hoi/kho.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Cổng thu hồi (X3)</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>X3-2</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Nhận câu dính</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Câu dính khi canCu.thuVien[].dau (dấu HIỆN TẠI của mục đã vào prompt) giao với tập thu hồi. thayThuHoi (dấu lịch sử) chỉ dùng để nhận ra tóm lại hoặc bức tranh cũ ghép từ câu đã viết lại.</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Dấu là sha1(ý + điều kiện), 8 hex, tính trong thu-vien/dau.ts. Câu viết trước K1 không có canCu nên là điểm mù đã biết.</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>lib/rag/thu-hoi/cong.ts, lib/rag/thu-vien/dau.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Cổng thu hồi (X3)</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>X3-3</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Viết lại đúng câu dính</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Câu dính coi như thiếu và chỉ câu đó được viết lại khi có người mở. Lượt viết nhận tập thu hồi nên khối thư viện bỏ mục đó. Bản mới mang thayThuHoi. Lần mở sau đọc thẳng đệm, 0 lượt model.</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Tính như sinh thường, trong hạn mức X1. Mục thu hồi vẫn tính trong biLat, nên mục nó đã gỡ vẫn bị gỡ (5a). Lượt song song ghi câu dính thì không được gộp.</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts, lib/rag/thu-vien/cho-prompt.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Cổng thu hồi (X3)</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>X3-4</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Viết hỏng → câu chờ</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Viết lại hỏng hoặc khách hết lượt thì trả câu chờ (tamAn), dựng MỚI chỉ từ id, câu hỏi và độ rõ. HTTP 200. Đệm giữ bản gốc để hoàn tác thu hồi vẫn còn bài. Không lùi về bản cũ hay thế hệ trước.</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Hai lớp che cùng sống: câu dính được xét TRƯỚC (vào biThuHoi, không vào banCu) nên câu chờ không bao giờ đi qua cheThangBanCu và không mang chữ bản cũ. Câu chỉ khác phienBan vẫn được che phần tháng. Câu chờ không hứa lúc nào có bài.</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts, components/luangiai/CauTraLoiV3.tsx, components/luangiai/TongQuanV3.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Cổng thu hồi (X3)</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>X3-5</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Lọc tóm lại, bức tranh, sổ ý, Sổ kết luận</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Tóm lại hoặc bức tranh có dauTV dính thì không trả và không giữ làm bản cũ. Nếu không có dauTV thì soát qua câu nguồn. Bản mới ghi dauTV. Sổ ý bỏ ý của câu dính. soKetLuanV3 lọc tóm lại và ý tổng quan dính.</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Phạm vi 6a: bài V3 đã lưu và Sổ kết luận. Chat STANDARD/Focused và kho nghiệm lý nằm ngoài phạm vi.</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>lib/rag/v3/xu-ly.ts, lib/rag/v3/so-ket-luan.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Cổng thu hồi (X3)</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>X3-6</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Lệnh vận hành</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>scripts/thu-hoi-muc.ts có các lệnh xem / thu-hoi / hoan-tac, theo --dau, --id --chu-de hoặc --theo-chunk. Mặc định chạy khô và in số câu đệm bị ảnh hưởng. Ghi thật cần --ap-dung và --ly-do. Hoàn tác là điền huy_luc, không xoá hàng.</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Ghi phạm vi all (production) bắt buộc có --ghi-production. Thử trên Preview lấy phạm vi qua /api/phien-ban của chính URL Preview. KHÔNG bao giờ bật loai_tru để thử, vì nó ăn ngay trên production (database dùng chung).</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>scripts/thu-hoi-muc.ts, supabase/va-thu-hoi-muc.sql</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27990,7 +28213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F194"/>
+  <dimension ref="A1:F195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34208,6 +34431,38 @@
         </is>
       </c>
       <c r="F194" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>5c7b17a, 8d089c7 (nhánh viec/cong-thu-hoi)</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>CEL-143, CELES-27</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>X3 cổng thu hồi tri thức: một bảng thu_hoi_muc_thu_vien (chỉ thêm, RLS, chỉ service-role); câu V3 đã lưu dựa vào mục thư viện đã thu hồi được viết lại đúng câu khi có người mở, viết hỏng thì hiện câu chờ; lọc tóm lại, bức tranh, sổ ý và Sổ kết luận; script vận hành mặc định chạy khô; test offline test-cong-thu-hoi (86 ca) vào CI. Gộp với abcad96 giữ cả hai lớp che (câu dính xét trước phần tháng).</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Gỡ một mục sai khỏi thư viện thì không sửa được bài đã lưu: bài V3 trong đệm và Sổ kết luận vẫn hiện nguyên lời dựa vào mục đó. Chủ dự án quyết 22/10/2026 (1a, 2 có, 3a, 4a, 5a, 6a): đoạn sách thu hồi bằng loai_tru, bảng chỉ cho mục thư viện; viết lại đúng câu dính trong hạn mức thay vì xoá cả bài; câu chờ không hứa hẹn; đo độ trễ trên Preview trước khi bật.</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: go dau giao dien AI theo Hallmark + may canh CI (CEL-207)
- Eyebrow cau thuong, font than bai, khong gian chu; bo eyebrow lap tieu de
- Bo gach / mui ten trang tri; EN bo em dash
- KhoiGuong theo .dark-band; 👍👎 -> icon SVG; token spacing / mau; thanh scaleX
- scripts/kiem-dau-ai.mjs: sloplint Hallmark (MIT, vendored) tang floor, danh sach nen 5 dau menh ban

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -1083,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O205"/>
+  <dimension ref="A1:O206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5611,7 +5611,7 @@
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>Token màu, kiểu chữ, bo góc tập trung ở globals.css. Hồng #df37a7 chỉ cho nút hành động chính, mỗi khung nhìn đúng một cái. Vàng kim #D4AF37 chỉ cho dấu thương hiệu. Từ 16/10/2026 mang 'chất liệu' của Your Best Version: chữ Be Vietnam Pro (tiêu đề đậm 800, khít chữ), thẻ bo 22px + bóng mềm, nút viên thuốc, ô nhập/ô chọn bo 12px, nền ngày ngả tím nhạt #f6f3f7, nhãn eyebrow chữ đậm nhỏ (không còn mono). Bảng màu, bố cục, linh vật, dấu thương hiệu giữ nguyên.</t>
+          <t>Token màu, kiểu chữ, bo góc tập trung ở globals.css. Hồng #df37a7 chỉ cho nút hành động chính, mỗi khung nhìn đúng một cái. Vàng kim #D4AF37 chỉ cho dấu thương hiệu. Từ 16/10/2026 mang 'chất liệu' của Your Best Version: chữ Be Vietnam Pro (tiêu đề đậm 800, khít chữ), thẻ bo 22px + bóng mềm, nút viên thuốc, ô nhập/ô chọn bo 12px, nền ngày ngả tím nhạt #f6f3f7, nhãn eyebrow chữ đậm nhỏ, câu thường (không mono, không HOA từ 25/10/2026, CEL-207). Bảng màu, bố cục, linh vật, dấu thương hiệu giữ nguyên.</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -17331,6 +17331,83 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>CEL-207</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>G. Trải nghiệm &amp; giao diện</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Gỡ dấu 'giao diện AI làm' + máy canh Hallmark</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Gỡ các dấu quen của web do AI sinh theo bộ luật Hallmark (sloplint, MIT): eyebrow thành nhãn câu thường, font thân bài 13px/600, không giãn chữ (bỏ rule eyebrow trùng ở khối YBV); bỏ eyebrow lặp tiêu đề (/tai-khoan); bỏ gạch trang trí trong option và mũi tên '→' dính cuối nhãn (giữ mũi tên trong nội dung luận; nút mở lại khối chuyển đổi dùng IconMuiTenPhai); bản EN bỏ toàn bộ em dash, tiếng Việt giữ gạch trong văn xuôi; KhoiGuong dùng .dark-band + viền --line + --accent-chu riêng của dải (#f58fd0, 8,3:1); 👍👎 ở PhanHoiLuot thành icon SVG IconHuuIch/IconKhongDung, nút ≥44px; số thô → token --space-*, màu thô → token (SoDoBonChang, MucDeepSection); thanh BanDoManhYeu đổi transition width → scaleX; thêm ::selection theo accent.</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>CI chạy node scripts/kiem-dau-ai.mjs: sloplint tầng floor trên app/ + components/ (trừ quản trị), so với danh sách nền scripts/hallmark/nen.json; dấu mới → đỏ.</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Chờ nghiệm thu</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>GIAO DIỆN</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Mọi người</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Toàn hệ thống</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>app/globals.css, lib/i18n/vi.ts, lib/i18n/en.ts, components/luangiai/KhoiGuong.tsx, components/PhanHoiLuot.tsx, components/ui/icons.tsx, scripts/kiem-dau-ai.mjs, scripts/hallmark/ (sloplint.mjs, LICENSE, nen.json), .github/workflows/kiem-tra.yml</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>Nền còn 5 dấu ở mệnh bàn (chữ HOA 8–10px PalaceCell, VoidMarkers; '›' TuViChart) — việc riêng. Gate 54 (eyebrow lặp tiêu đề) soát bằng mắt khi review vì sloplint bắt theo tên class. App di động có eyebrow riêng, chưa đồng bộ. Lỗi vùng chạm &lt;44px ở header/btn-sm/pill-tag có từ trước (test-man-hinh), không do việc này. Trùng tệp với nhánh tích hợp ở app/luan-giai/sau/page.tsx.</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>(nhánh viec/go-dau-ai-giao-dien)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O97"/>
   <dataValidations count="1">
@@ -17348,7 +17425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G278"/>
+  <dimension ref="A1:G280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27503,6 +27580,80 @@
         </is>
       </c>
     </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>CEL-207</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Máy canh dấu AI</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Chạy sloplint tầng floor</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>scripts/kiem-dau-ai.mjs gọi scripts/hallmark/sloplint.mjs app components --scope app --tier floor --json; lọc trang/component quản trị, gate 19/20/34/54, và gate 48/7a/39a ở app/globals.css (tệp token). Thêm kiểm riêng em dash trong lib/i18n/en.ts (bỏ dòng chú thích).</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Floor của sloplint không ghi ngoại lệ được nên cổng phải là danh sách nền. Gate 54 bắt theo TÊN class eyebrow, không theo nội dung — không bật. Đường dẫn finding là tương đối, regex phải có (^|[\\/]) mới khớp.</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>scripts/kiem-dau-ai.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>CEL-207</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Máy canh dấu AI</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>So với danh sách nền</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Dấu vân = '[gate] tệp bằng-chứng' (không theo số dòng). Dấu ngoài scripts/hallmark/nen.json → in MỚI, thoát 1. Sửa hết dấu cũ thì chạy --cap-nhat để rút khỏi nền.</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Nền chỉ được BỚT, không thêm dấu mới vào nền. Dấu EN mang tiền tố './lib/i18n/en.ts'.</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>scripts/hallmark/nen.json, .github/workflows/kiem-tra.yml, scripts/kiem-nhanh.mjs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27515,7 +27666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F184"/>
+  <dimension ref="A1:F185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33413,6 +33564,38 @@
         </is>
       </c>
       <c r="F184" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>(nhánh viec/go-dau-ai-giao-dien)</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>CEL-207, CEL-057</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Gỡ dấu giao diện AI theo Hallmark: eyebrow câu thường, bỏ gạch/mũi tên trang trí, EN bỏ em dash, KhoiGuong theo .dark-band, emoji 👍👎 → icon, token spacing/màu, thanh scaleX; thêm máy canh CI kiem-dau-ai (sloplint vendored MIT, tầng floor, danh sách nền 5 dấu).</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Chủ dự án 25/10/2026 đưa Hallmark (github.com/Nutlope/hallmark) để Celes không trông như giao diện AI làm. Audit (D:\Celestia\dot\hallmark\BAO-CAO-audit.md) đo 104 dấu tầng floor; chủ dự án duyệt 4 điểm: giữ eyebrow nhưng câu thường, gạch chỉ gỡ ở EN và chỗ trang trí (tiếng Việt dùng gạch là văn phong thường), CI chỉ chặn tầng floor không thêm dịch vụ, hook chặn push main. Sau sửa còn 5 dấu ở mệnh bàn để thành việc riêng. Máy canh dùng danh sách nền theo dấu vân thay cho mốc đếm vì phan-bien chỉ ra mốc đếm cho phép đổi một dấu cũ lấy một dấu mới.</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
PERF: cong thu hoi tra ngay tap cu, doc lai DB o nen (CEL-143)
Vi sao: do tren Preview 31/10 moi lan doc bang thu hoi mat 851-1394 ms; it nguoi dung
thi luot nao cung qua 60 giay, mo lai bai da luu tu 1,6 s thanh ~3 s. Chu du an duyet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -28079,7 +28079,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Cờ CELES_CONG_THU_HOI khác 1 thì tập rỗng, không có truy vấn nào. Bật thì đọc thu_hoi_muc_thu_vien (cột dau, huy_luc is null). Production chỉ đọc phạm vi all; Preview đọc all cộng phạm vi phamViDem của chính máy chủ. Giữ trong RAM 60 giây.</t>
+          <t>Cờ CELES_CONG_THU_HOI khác 1 thì tập rỗng, không có truy vấn nào. Bật thì đọc thu_hoi_muc_thu_vien (cột dau, huy_luc is null). Production chỉ đọc phạm vi all; Preview đọc all cộng phạm vi phamViDem của chính máy chủ. Giữ trong RAM 60 giây. Hết 60 giây mà lần đọc trước tốt và tập tốt gần nhất chưa quá 30 phút: trả NGAY tập cũ, đọc lại DB ở nền (after(), một lượt đọc nền tại một thời điểm). Quá 30 phút hoặc lần trước lỗi / tắt thì chờ đọc như cũ.</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -28364,7 +28364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F196"/>
+  <dimension ref="A1:F197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34646,6 +34646,38 @@
         </is>
       </c>
       <c r="F196" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>(nhánh viec/tich-hop-dot-1)</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>CEL-143</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Cổng thu hồi: hết 60 giây thì trả ngay tập cũ và đọc lại DB ở nền thay vì bắt lượt đang chờ.</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Đo trên Preview 31/10/2026: mỗi lần đọc bảng thu hồi mất 851–1394 ms (5 lần), không chỉ lúc khởi động; ít người dùng thì gần như lượt nào cũng quá 60 giây nên mở lại bài đã lưu từ 1,6 s thành ~3 s. Chủ dự án duyệt 31/10, chấp nhận mục vừa thu hồi có thể lọt thêm một lượt.</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: bat lop van han mac dinh; sach tu hoa chi lam nguon cho cau van han (CEL-200)
Chu du an quyet 31/10/2026:
- Lop van han (luu tu hoa) BAT mac dinh; CELES_LOP_HAN=0 la cong tac tat.
- 4 sach tu hoa chi vao cau van han / cau nhac tu hoa (lib/rag/nguon-tu-hoa.ts).
  truyHoi mac dinh loai chung (lay du 10 ung vien roi loc truoc RRF).
  Chat + Focused theo tin hieu thoi gian nguoi hoi noi ra; Hanh trinh luon;
  v3 chi cau thoiDiem='co'; khoa dem DEM_CHUNG co them quyen.
- NHOM_NGUON them 4 sach (hai tap Tu Hoa Phai chung mot nhom).
- PHIEN_BAN_TRUY_HOI 2026.10.1; snapshot 3b ghi lai chi vi so phien ban nay.
- Bai moi test-nguon-tu-hoa (CI); ba bai kiem duong tat ghim CELES_LOP_HAN=0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16850,13 +16850,12 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>Cờ server CELES_LOP_HAN=1 (chung với CEL-199), mặc định tắt</t>
+          <t>BẬT mặc định từ 31/10/2026 (chủ dự án: bỏ chặn lưu tứ hoá). Tắt khẩn cấp: CELES_LOP_HAN=0 (đường cũ).</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Máy 2 xong 3b (17a9ab3) và Commit 4 phần mã. Toàn tính năng vẫn Đang phát triển: chờ 3a' C1/C3 máy 1, kho và Hành trình; chưa bật cờ/tăng đệm. Chưa đo model thật, chi phí/502/độ trễ; chủ dự án chạy eval-chat-quyet-dinh sau tích hợp. Vòng 2 việc1–2 xong mã, B4 không tăng đệm nên bài đã lưu vẫn có thể chứa câu cũ; việc3 bộ ca đáp án chờ push được chủ dự án bảo rồi nhánh riêng.
-Xét cung (C-C) còn hoãn: trọng số tọa thủ/chiếu và viTri 'giap' riêng cho cách giáp; tách tiền/hậu vận cho Triệt khi đọc lá gốc; Tuần Triệt ở cung của bên bị tác động; sát đắc đi với bộ không dụng được vẫn có hại; thứ tự Phúc/Mệnh chưa truyền kết quả nền sang cung hỏi; Kỵ gốc và Kỵ lưu gộp tên khi đếm. C-D chờ 3b máy 2; C-E kế tiếp.</t>
+          <t>Đã bật cờ khi CHƯA đo phân bố hai phía offline và chưa đo model thật (chi phí, 502, độ trễ) — chủ dự án chọn bỏ rào cản 31/10. Bật cờ đổi prompt bài dài / bảng lĩnh vực (chuNguonLopHan) và chat câu thời điểm; bài v3 đã đệm trước đó vẫn trả tới khi hết hạn. Sách tứ hoá chỉ vào câu vận hạn / câu nhắc tứ hoá (lib/rag/nguon-tu-hoa.ts). Còn chờ chủ dự án: bảng luật tổ hợp đợt 2 (D:\Celestia\BANG-LUAT-TO-HOP-dot-2-2026-10-27.md).</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -16866,7 +16865,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>(nhánh viec/van-han-3b, gộp van-han-lop-han 31/10)</t>
+          <t>(nhánh viec/van-han-3b)</t>
         </is>
       </c>
     </row>
@@ -17434,7 +17433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G293"/>
+  <dimension ref="A1:G294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -28144,6 +28143,43 @@
         </is>
       </c>
     </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Sách tứ hoá chỉ làm nguồn cho câu vận hạn (truy hồi 2026.10.1)</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>truyHoi nhận cauHinh.nguonTuHoa (mặc định false). Tắt thì lấy dư 10 ứng viên ở cả nhánh vector và từ khoá rồi bỏ đoạn của sách có tiêu đề chứa 'Tứ Hóa Phái' / 'Tinh Thành' / 'Phi Tinh Lương Phái' TRƯỚC khi gộp RRF. Bật khi: chat STANDARD + Focused — choNguonTuHoaTheoKeHoach: người hỏi nói mốc thời gian (phamViThoiGian khác khong-ro, namMucTieu, thangMucTieu), gọi tên đại vận / lưu niên / nguyệt hạn, hỏi 'khi nào', hoặc câu nhắc tứ hoá / Hóa Lộc-Quyền-Khoa-Kỵ / phi hoá; Hành trình — luôn; bài v3 — câu khung hỏi THẲNG thời điểm (thoiDiem='co'; 'phu' không tính vì trọng tâm vẫn là lá gốc) hoặc câu nhắc tứ hoá, khoá đệm DEM_CHUNG có thêm quyền; phòng thử truy hồi admin — bật, ghi đè được. Bài dài, bảng lĩnh vực, bản đọc sâu, bề mặt ngắn, kết nối: không.</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>KHÔNG dựa vào keHoach.lopHan: planner tự thêm lưu niên cho cả câu không mốc thời gian ('tính tôi thế nào'), test-nguon-tu-hoa bắt được. Nhận sách theo TIÊU ĐỀ, không theo he_phai. Hai tập Tứ Hóa Phái cùng nhóm nguồn 'tu-hoa-phai' trong NHOM_NGUON: không tự đứng làm hai nguồn cho một luật tổ hợp.</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>lib/rag/nguon-tu-hoa.ts, lib/rag/truy-hoi.ts, lib/rag/tra-loi.ts, lib/rag/focused/tra-loi-focused.ts, lib/rag/moc-hanh-trinh.ts, lib/rag/v3/index.ts, lib/rag/v3/truy-hoi-v3.ts, lib/tuvi/luat-to-hop.ts, scripts/test-nguon-tu-hoa.ts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28156,7 +28192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F199"/>
+  <dimension ref="A1:F200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34534,6 +34570,38 @@
         </is>
       </c>
       <c r="F199" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-3b)</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Bật lớp vận hạn mặc định (CELES_LOP_HAN=0 để tắt). Bốn sách tứ hoá thành nguồn chỉ cho câu vận hạn / câu nhắc tứ hoá; luận lá gốc không lấy đoạn từ chúng. Thêm 4 sách vào NHOM_NGUON (3 nhóm). PHIEN_BAN_TRUY_HOI 2026.10.1. Ba bài kiểm đường tắt ghim CELES_LOP_HAN=0; snapshot 3b ghi lại chỉ vì số phiên bản truy hồi.</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Chủ dự án quyết 31/10/2026: '1. nghiệm thu 3b và push 2. bỏ chặn lưu tứ hoá 3. bỏ rào cản 4. nhận 4 sách làm nguồn, tuy nhiên sách tứ hoá chỉ ghi nhận làm nguồn cho câu hỏi liên quan vận hạn, tránh luận giải bình thường cũng lấy dữ liệu từ sách tứ hoá, trừ trường hợp cần trích dữ liệu liên quan tứ hoá'. Bốn sách nạp 26/10 (4.634 đoạn) chiếm khoảng một phần ba kho; để chung là lấn sách luận lá gốc ở mọi bề mặt. Bước đo phân bố offline trước khi bật cờ bị bỏ theo lệnh 'bỏ rào cản'.</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>

<commit_message>
FEAT: lop van han - nguon tu hoa chi cho cau van han, cau noi nhan moc, tu ghi lop hoa (CEL-200)
- Sach tu hoa chi lam nguon cho cau van han (ke ca "co nen..." khong noi moc) va cau nhac tu hoa
- Cau noi trong chat nhan moc thoi gian cua cau truoc (keThuaVanHan)
- Cau con pham luat sau khi sua: luot sua thu hai, bo rieng cau, chi chan ca luot khi cau rao pham
- ghiLopHoa: Hoa khong ghi lop ma chi khop mot lop thi tu ghi "luu" / "dai van" / "goc"
- Thu hep hai luat bat nham cua loiHoaLopHan (dai van noi ve sao khac; sao di kem khong nhan hoa)
- Do model that 2 la x 12 cau: 23/24 rong -> 2/24 rong, Hoa thieu lop 36/67 -> 0/82

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRODUCT-BACKLOG.xlsx
+++ b/PRODUCT-BACKLOG.xlsx
@@ -16855,7 +16855,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Đã bật cờ khi CHƯA đo phân bố hai phía offline và chưa đo model thật (chi phí, 502, độ trễ) — chủ dự án chọn bỏ rào cản 31/10. Bật cờ đổi prompt bài dài / bảng lĩnh vực (chuNguonLopHan) và chat câu thời điểm; bài v3 đã đệm trước đó vẫn trả tới khi hết hạn. Sách tứ hoá chỉ vào câu vận hạn / câu nhắc tứ hoá (lib/rag/nguon-tu-hoa.ts). Còn chờ chủ dự án: bảng luật tổ hợp đợt 2 (D:\Celestia\BANG-LUAT-TO-HOP-dot-2-2026-10-27.md).</t>
+          <t>Đo model thật 31/10 (scripts/do-lop-han-that.ts, lá 24/8/2000 giờ Tuất nam + 3/11/1985 giờ Hợi nữ, 12 câu mỗi lá, bật cờ): trước sửa 23/24 lượt rỗng; lần 7 (bản commit) 2/24 rỗng (cả hai là câu rào còn phạm luật, chặn có chủ đích), 0/82 lần nhắc Hóa thiếu lớp (lần 4: 36/67), trung bình ~29,5s/lượt so với ~26s khi tắt cờ. Mọi câu vận hạn lấy 1–4 đoạn sách tứ hoá; 'Tính cách tôi thế nào?' lấy 0. Đường Focused (đang tắt) chưa nối ghiLopHoa. Còn chờ chủ dự án: bảng luật tổ hợp đợt 2 (D:\Celestia\BANG-LUAT-TO-HOP-dot-2-2026-10-27.md), Q0.</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -17433,7 +17433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G294"/>
+  <dimension ref="A1:G297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -28166,17 +28166,128 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>truyHoi nhận cauHinh.nguonTuHoa (mặc định false). Tắt thì lấy dư 10 ứng viên ở cả nhánh vector và từ khoá rồi bỏ đoạn của sách có tiêu đề chứa 'Tứ Hóa Phái' / 'Tinh Thành' / 'Phi Tinh Lương Phái' TRƯỚC khi gộp RRF. Bật khi: chat STANDARD + Focused — choNguonTuHoaTheoKeHoach: người hỏi nói mốc thời gian (phamViThoiGian khác khong-ro, namMucTieu, thangMucTieu), gọi tên đại vận / lưu niên / nguyệt hạn, hỏi 'khi nào', hoặc câu nhắc tứ hoá / Hóa Lộc-Quyền-Khoa-Kỵ / phi hoá; Hành trình — luôn; bài v3 — câu khung hỏi THẲNG thời điểm (thoiDiem='co'; 'phu' không tính vì trọng tâm vẫn là lá gốc) hoặc câu nhắc tứ hoá, khoá đệm DEM_CHUNG có thêm quyền; phòng thử truy hồi admin — bật, ghi đè được. Bài dài, bảng lĩnh vực, bản đọc sâu, bề mặt ngắn, kết nối: không.</t>
+          <t>truyHoi nhận cauHinh.nguonTuHoa (mặc định false). Tắt thì lấy dư 10 ứng viên ở cả nhánh vector và từ khoá rồi bỏ đoạn của sách có tiêu đề chứa 'Tứ Hóa Phái' / 'Tinh Thành' / 'Phi Tinh Lương Phái' TRƯỚC khi gộp RRF. Bật khi: chat STANDARD + Focused — choNguonTuHoaTheoKeHoach: coTinHieuThoiGian (phamViThoiGian khác khong-ro, yDinh thoi-diem, namMucTieu, thangMucTieu, thực thể đại vận / lưu niên / nguyệt hạn) HOẶC hoiLucNay (yDinh quyet-dinh 'có nên…'; yDinh co-khong không có thực thể sao/cung/cách cục/hoá/dấu và không hỏi bản tính / độ hợp / duyên) HOẶC câu nhắc tứ hoá; Hành trình — luôn; bài v3 — câu khung hỏi THẲNG thời điểm hoặc nhắc tứ hoá; phòng thử truy hồi admin — bật. Bài dài, bảng lĩnh vực, bản đọc sâu, bề mặt ngắn, kết nối: không.</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>KHÔNG dựa vào keHoach.lopHan: planner tự thêm lưu niên cho cả câu không mốc thời gian ('tính tôi thế nào'), test-nguon-tu-hoa bắt được. Nhận sách theo TIÊU ĐỀ, không theo he_phai. Hai tập Tứ Hóa Phái cùng nhóm nguồn 'tu-hoa-phai' trong NHOM_NGUON: không tự đứng làm hai nguồn cho một luật tổ hợp.</t>
+          <t>KHÔNG dựa vào keHoach.lopHan: planner tự thêm lưu niên cho cả câu không mốc thời gian ('tính tôi thế nào'). Nhận sách theo TIÊU ĐỀ, không theo he_phai. Hai tập Tứ Hóa Phái cùng nhóm nguồn 'tu-hoa-phai'.</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>lib/rag/nguon-tu-hoa.ts, lib/rag/truy-hoi.ts, lib/rag/tra-loi.ts, lib/rag/focused/tra-loi-focused.ts, lib/rag/moc-hanh-trinh.ts, lib/rag/v3/index.ts, lib/rag/v3/truy-hoi-v3.ts, lib/tuvi/luat-to-hop.ts, scripts/test-nguon-tu-hoa.ts</t>
+          <t>lib/rag/nguon-tu-hoa.ts, lib/rag/van-han-qua-luot.ts, lib/rag/truy-hoi.ts, lib/rag/tra-loi.ts, lib/rag/focused/tra-loi-focused.ts, lib/rag/moc-hanh-trinh.ts, lib/rag/v3/index.ts, lib/rag/v3/truy-hoi-v3.ts, lib/tuvi/luat-to-hop.ts, scripts/test-nguon-tu-hoa.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Câu nối trong chat nhận mốc thời gian của câu trước (keThuaVanHan)</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Sau khi planner lập kế hoạch, ở cả STANDARD và Focused: câu hiện tại KHÔNG có tín hiệu thời gian VÀ là câu nối rõ ràng (mở bằng 'vậy còn / thế còn / vậy thì / còn …', hoặc kết bằng '… thì sao?') thì lùi tối đa 4 câu người dùng trước. Gặp câu có tín hiệu thời gian thì nhận lopHan, phamViThoiGian, namMucTieu, thangMucTieu của câu đó (và yDinh nếu câu hiện tại chỉ là mo-ta); gặp câu không phải câu nối thì dừng. Không kế thừa khi câu nối có chủ đề tong-quan hoặc hỏi bản tính / độ hợp / duyên (HOI_BAN_TINH), và không chạy khi CELES_LOP_HAN=0. Ví dụ: 'Năm 2027 công việc tôi thế nào?' → 'Vậy còn tình cảm?' được luận cho 2027.</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>KHÔNG dùng laCauNoiTiep (coi mọi câu ≤5 chữ là nối tiếp → 'Tính tôi thế nào?' bị luận theo 2027). Không dò 'con ' không dấu ('Con tôi học thế nào?' là câu mới). Không nâng PHIEN_BAN_PLANNER (nằm trong PHIEN_BAN_CHU, nâng là xả đệm).</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>lib/rag/van-han-qua-luot.ts, lib/rag/tra-loi.ts, lib/rag/focused/tra-loi-focused.ts, scripts/test-nguon-tu-hoa.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Câu còn phạm luật chữ / gắn hoá sau khi sửa: bỏ riêng câu, không xoá trắng lượt</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>suaCauTiengLong sửa cả tiêu đề ý khi phạm luật lớp hạn; prompt sửa nêu rõ chữ cấm (nền, nhịp, phần nổi…) và luật 'mỗi Hóa kèm tên sao nhận hoá'. Còn câu phạm thì có lượt sửa thứ hai (chỉ khi cần): văn chính sửa lại một lần; mọi chuỗi còn phạm trong bản cấu trúc (kể cả cachNoi / canNhac / buocTiepTheo, vốn không nằm trong văn nên lượt đầu không chạm, và câu dongBo không chép được vì model đổi số câu) gộp vào MỘT lượt gọi. Sau đó boCauPham bỏ riêng câu vẫn phạm ở văn và ở bản cấu trúc (ý chính rỗng thì bỏ ý; trường phụ ở phần 'vì sao' còn câu rào phạm thì bỏ cả trường). Câu phạm mà là câu RÀO (tuy, nhưng, nếu, chưa, khó, không nên, đừng, Kỵ…) thì KHÔNG bỏ lẻ: chặn cả lượt, vì bỏ nó là để lại vế lạc quan trơ trọi. Lượt chỉ rỗng khi câu rào phạm hoặc không còn câu nào. loiChuLopHan không bắt 'nền tảng' (từ thường; doiTenCung sinh 'phần chỗ ở và nền tảng'). Prompt lớp hạn (nghieng-ve.ts) thêm cấm 'nền/nhịp' nghĩa bóng kể cả khi dữ kiện cách cục viết 'dựng nền', và 'không rõ sao nhận hoá thì đừng nêu Hóa đó'. loiHoaLopHan nhận tên lớp chen giữa hoá và sao ('Hóa Quyền đại vận vào Thái Âm'). Cảnh báo '[lop-han] chặn lượt chat' in kèm tối đa 3 câu bị bắt để theo dõi.</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Đo model thật 31/10: xoá trắng cả lượt vì một chữ 'nhịp' / 'nền' / một Hóa thiếu tên sao làm 23/24 lượt chat rỗng (người dùng thấy báo lỗi). Nguồn chữ 'nền' nằm ngay trong mã: lib/tuvi/cach-cuc.ts:106 ('dựng nền lâu dài') và doiTenCung (Điền Trạch). Không sửa câu cách cục trong engine vì bộ đóng băng boi-canh-dong-bang.json ghim nó. Đo lần 3–4: thêm chốt câu rào thì rỗng lại 4/11 rồi 6/24 — gốc là (a) bản cấu trúc không được sửa khi model đổi số câu, (b) bộ kiểm hoá bắt nhầm 'Hóa X đại vận vào Sao' (đúng dữ kiện lá 3/11/1985). Bộ kiểm hoá vẫn bắt đúng câu trộn lớp thật: lá 24/8/2000 giờ Tuất có lưu Hóa Kỵ 2026 vào Liêm Trinh (Mệnh) và Hóa Kỵ gốc vào Thiên Đồng (Điền Trạch); câu 'Hóa Kỵ vào Liêm Trinh và Điền Trạch' gộp hai lớp làm một nên bị chặn đúng. Lần 5 (sau nới): 2/24 rỗng, cả hai do câu rào còn chữ 'nhịp' hoặc 'Lưu Hóa Kỵ' không kèm tên sao — chặn đúng luật.</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>lib/rag/sua-chua.ts, lib/rag/tra-loi.ts, lib/rag/kiem-lop-han.ts, lib/rag/nghieng-ve.ts, scripts/test-lop-han-3b.ts, scripts/do-lop-han-that.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Lớp hạn (vận hạn)</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Tự ghi lớp cho Hóa không nói rõ lớp (ghiLopHoa)</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Ở chat STANDARD khi lớp hạn bật: sau khi model trả lời và sau mỗi lượt sửa, ghiLopHoa đọc từng Hóa đã kèm tên sao trong văn và mọi chuỗi của bản cấu trúc. Nếu Hóa + sao đó (và cung nếu câu có ghi) chỉ khớp ĐÚNG MỘT lớp trong bảng hoá của engine (gốc / lưu năm đang xem / đại vận) thì chèn chữ lớp: 'lưu Hóa Kỵ' (đầu câu viết hoa 'Lưu'), 'Hóa Quyền đại vận', 'Hóa Lộc gốc'. Hóa đã ghi lớp, khớp nhiều lớp, không có tên sao, hay một Hóa đi với nhiều sao thì để nguyên. Prompt lớp hạn (nghieng-ve.ts) cũng dặn model ghi lớp. Đường Focused (đang tắt) chưa nối. Cùng đợt, thu hẹp hai luật của loiHoaLopHan vốn bắt nhầm câu đúng: (a) 'lưu hoá lẫn đại vận' chỉ bắt khi chữ 'đại vận' đứng SÁT hoá ('lưu Hóa Kỵ đại vận'), không bắt khi 'đại vận' nói về sao khác trong cùng câu; (b) 'một hoá gắn nhiều sao' bỏ qua sao đứng sau 'cùng / gặp / với' mà không nhận hoá nào trong bảng ('lưu Hóa Kỵ vào Liêm Trinh cùng Kình Dương'). 'X và Tử Vi', 'X, Thiên Cơ' vẫn bị bắt.</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Đo model thật 31/10 lần 4: 27/64 lần nhắc Hóa không ghi lớp — 'Hóa Quyền vào Vũ Khúc' (gốc), 'Hóa Kỵ vào Liêm Trinh' (lưu 2026), 'Hóa Kỵ vào Thiên Cơ' (đại vận) đứng cạnh nhau, người đọc tưởng cùng một lớp. Chủ dự án yêu cầu lưu tứ hoá / đại vận phân biệt rõ với tứ hoá gốc. Không chèn khi khớp nhiều lớp (đoán sai lớp còn tệ hơn không ghi). Mã phân biệt theo LỚP, không theo phái. Đo lần 6: 5/24 lượt rỗng; soát từng câu bị chặn thì 2 lượt chặn đúng (lá 1985: 'Quyền đại vận vào Thiên Cơ' sai — Quyền đại vận ở Thái Âm; 'Hóa Quyền năm nay vào phần tiền bạc' sai cung), 3 lượt bắt nhầm do hai luật (a), (b).</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>lib/rag/kiem-lop-han.ts, lib/rag/tra-loi.ts, lib/rag/nghieng-ve.ts, scripts/test-lop-han-3b.ts</t>
         </is>
       </c>
     </row>
@@ -28192,7 +28303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F200"/>
+  <dimension ref="A1:F201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34602,6 +34713,38 @@
         </is>
       </c>
       <c r="F200" t="inlineStr">
+        <is>
+          <t>Claude (máy 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>(nhánh viec/van-han-3b)</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>CEL-200</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Bật lớp vận hạn mặc định (CELES_LOP_HAN=0 để tắt). Bốn sách tứ hoá chỉ làm nguồn cho câu vận hạn (kể cả câu 'có nên…' không nói mốc, câu có/không về chuyện đời) và câu nhắc tứ hoá. Câu nối trong chat nhận mốc của câu trước. Câu còn phạm luật lớp hạn sau khi sửa bị bỏ riêng, không xoá trắng cả lượt. Thêm bài đo model thật scripts/do-lop-han-that.ts. PHIEN_BAN_TRUY_HOI 2026.10.1. Hóa không ghi lớp mà chỉ khớp một lớp thì tự ghi 'lưu' / 'đại vận' / 'gốc'.</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Chủ dự án quyết 31/10/2026: bỏ chặn lưu tứ hoá, bỏ rào cản, nhận 4 sách nhưng chỉ cho câu vận hạn; câu 'Có nên đổi việc không?' phải tự hiểu là hỏi lúc này; câu trong chat liên quan vận hạn phải luận theo vận hạn; không fix cứng danh sách câu. Chủ dự án yêu cầu test thực tế trước khi chốt: đo model thật 2 lá số × 12 câu thì bật cờ ban đầu 23/24 lượt rỗng (lý do: chữ 'nhịp', 'nền' do chính mã đưa vào prompt, và Hóa thiếu tên sao); sau sửa 24/24 có trả lời, độ dài ngang cờ tắt, chậm thêm ~7s/lượt. Chủ dự án yêu cầu lưu tứ hoá / tứ hoá đại vận phân biệt rõ với tứ hoá gốc khi RAG: đo lần 4 có 36/67 lần nhắc Hóa không ghi lớp; sau ghiLopHoa + luật prompt, lần 7 còn 0/82, 2/24 lượt rỗng (chặn đúng câu rào phạm luật).</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
         <is>
           <t>Claude (máy 1)</t>
         </is>

</xml_diff>